<commit_message>
Build hackathon archive from SQLite
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sayyid/Documents/hackathon/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3728205-E47B-A342-A642-B620187BAF0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9FC6D66-1044-6D41-8E4A-A435353DC7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17840" xr2:uid="{9DF71BD7-8522-F64A-9F16-BDAC1601D549}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17800" xr2:uid="{9DF71BD7-8522-F64A-9F16-BDAC1601D549}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="968" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="555">
   <si>
     <t>#</t>
   </si>
@@ -1636,6 +1636,69 @@
   </si>
   <si>
     <t>Agentic AI + VR - Talk to the movie characters</t>
+  </si>
+  <si>
+    <t>https://luma.com/r6v3evdi?tk=BuCFqn</t>
+  </si>
+  <si>
+    <t>amber.ac</t>
+  </si>
+  <si>
+    <t>Kingdom Of PAL</t>
+  </si>
+  <si>
+    <t>sayyid,bruce</t>
+  </si>
+  <si>
+    <t>kingdom of pal: 7 dwarfs and a shiekh, a tool to help maange one person community biz</t>
+  </si>
+  <si>
+    <t>4.5K AWS Credits</t>
+  </si>
+  <si>
+    <t>BUIDL_OPC_Hackathon_SG</t>
+  </si>
+  <si>
+    <t>https://luma.com/68nouvl9?tk=yuORah</t>
+  </si>
+  <si>
+    <t>https://github.com/sayyidkhan/alien-homecoming</t>
+  </si>
+  <si>
+    <t>Terra Loft</t>
+  </si>
+  <si>
+    <t>Folly</t>
+  </si>
+  <si>
+    <t>Alien Homecoming</t>
+  </si>
+  <si>
+    <t>An adventure game where an alien is trying to find its way home, each map is ai rendered</t>
+  </si>
+  <si>
+    <t>18/7/2026</t>
+  </si>
+  <si>
+    <t>Whackathon 2026</t>
+  </si>
+  <si>
+    <t>Zo Computer Jul 2026 Build Challenge (Kill your SaaS)</t>
+  </si>
+  <si>
+    <t>15 Jul - 25 Jul 2026</t>
+  </si>
+  <si>
+    <t>Infra</t>
+  </si>
+  <si>
+    <t>clone google drive together with other commonly used infra features</t>
+  </si>
+  <si>
+    <t>Zo Drive</t>
+  </si>
+  <si>
+    <t>https://github.com/sayyidkhan/zo-drive</t>
   </si>
 </sst>
 </file>
@@ -2013,7 +2076,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E31B418-2D71-AD42-B07B-AEB5ED36DC01}">
-  <dimension ref="A1:P71"/>
+  <dimension ref="A1:P74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="53.1640625" bestFit="1" customWidth="1"/>
@@ -5510,7 +5573,7 @@
         <v>501</v>
       </c>
       <c r="L70" t="s">
-        <v>21</v>
+        <v>504</v>
       </c>
       <c r="M70" t="s">
         <v>500</v>
@@ -5573,6 +5636,156 @@
       </c>
       <c r="P71" t="s">
         <v>489</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>540</v>
+      </c>
+      <c r="C72" t="s">
+        <v>535</v>
+      </c>
+      <c r="D72" s="5">
+        <v>46363</v>
+      </c>
+      <c r="E72">
+        <v>1</v>
+      </c>
+      <c r="F72" t="s">
+        <v>306</v>
+      </c>
+      <c r="G72" t="s">
+        <v>539</v>
+      </c>
+      <c r="H72" t="s">
+        <v>230</v>
+      </c>
+      <c r="I72" t="s">
+        <v>538</v>
+      </c>
+      <c r="J72" t="s">
+        <v>537</v>
+      </c>
+      <c r="K72" t="s">
+        <v>536</v>
+      </c>
+      <c r="L72" t="s">
+        <v>535</v>
+      </c>
+      <c r="M72" t="s">
+        <v>287</v>
+      </c>
+      <c r="N72" t="s">
+        <v>29</v>
+      </c>
+      <c r="O72" t="s">
+        <v>21</v>
+      </c>
+      <c r="P72" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>548</v>
+      </c>
+      <c r="C73" t="s">
+        <v>544</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="E73">
+        <v>1</v>
+      </c>
+      <c r="F73" t="s">
+        <v>306</v>
+      </c>
+      <c r="G73" t="s">
+        <v>21</v>
+      </c>
+      <c r="H73" t="s">
+        <v>476</v>
+      </c>
+      <c r="I73" t="s">
+        <v>546</v>
+      </c>
+      <c r="J73" t="s">
+        <v>295</v>
+      </c>
+      <c r="K73" t="s">
+        <v>545</v>
+      </c>
+      <c r="L73" t="s">
+        <v>544</v>
+      </c>
+      <c r="M73" t="s">
+        <v>287</v>
+      </c>
+      <c r="N73" t="s">
+        <v>543</v>
+      </c>
+      <c r="O73" t="s">
+        <v>542</v>
+      </c>
+      <c r="P73" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>549</v>
+      </c>
+      <c r="C74" t="s">
+        <v>504</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="E74">
+        <v>10</v>
+      </c>
+      <c r="F74" t="s">
+        <v>306</v>
+      </c>
+      <c r="G74" t="s">
+        <v>21</v>
+      </c>
+      <c r="H74" t="s">
+        <v>551</v>
+      </c>
+      <c r="I74" t="s">
+        <v>552</v>
+      </c>
+      <c r="J74" t="s">
+        <v>295</v>
+      </c>
+      <c r="K74" t="s">
+        <v>553</v>
+      </c>
+      <c r="L74" t="s">
+        <v>504</v>
+      </c>
+      <c r="M74" t="s">
+        <v>500</v>
+      </c>
+      <c r="N74" t="s">
+        <v>319</v>
+      </c>
+      <c r="O74" t="s">
+        <v>554</v>
+      </c>
+      <c r="P74" t="s">
+        <v>498</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update hackathon social links workbook
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R7828600880c74791"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R0b560ad46e134790"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rc19c9d3b1df04ca2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rbf276a3e885d4d81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R42df29894e6c4d83"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1686,12 +1687,252 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="20">
+  <x:fills count="68">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -1819,7 +2060,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="82">
+  <x:cellXfs count="274">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1986,6 +2227,358 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="25" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="28" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="28" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="28" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="31" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="31" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="31" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="34" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="34" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="34" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="37" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="37" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="37" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="40" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="40" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="40" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="43" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="46" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="46" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="46" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="49" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="52" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="52" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="52" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="55" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="55" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="55" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="58" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="58" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="58" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="61" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="64" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="64" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="64" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="67" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="67" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="67" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2021,7 +2614,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PeopleDirectory" displayName="PeopleDirectory" ref="A4:E97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="PeopleDirectory" displayName="PeopleDirectory" ref="A4:E97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:E97"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Person ID"/>
@@ -2029,6 +2622,19 @@
     <x:tableColumn id="3" name="Hackathon #s"/>
     <x:tableColumn id="4" name="Builds Together"/>
     <x:tableColumn id="5" name="LinkedIn URL"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="HackathonSocials" displayName="HackathonSocials" ref="A4:D78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:D78"/>
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="Hackathon #"/>
+    <x:tableColumn id="2" name="LinkedIn"/>
+    <x:tableColumn id="3" name="Instagram"/>
+    <x:tableColumn id="4" name="Facebook"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -5940,8 +6546,8 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R8016dd5737b44859"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Ra149db7c5d904487"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R3125aaa772464745"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rde171be31a8b4499"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5963,37 +6569,37 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="72" t="str">
+      <x:c r="A1" s="264" t="str">
         <x:v>People &amp; LinkedIn Directory</x:v>
       </x:c>
-      <x:c r="B1" s="72"/>
-      <x:c r="C1" s="72"/>
-      <x:c r="D1" s="72"/>
-      <x:c r="E1" s="72"/>
+      <x:c r="B1" s="264"/>
+      <x:c r="C1" s="264"/>
+      <x:c r="D1" s="264"/>
+      <x:c r="E1" s="264"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="76" t="str">
+      <x:c r="A2" s="268" t="str">
         <x:v>One person per row. LinkedIn URLs are added only after the profile has been verified against the hackathon context.</x:v>
       </x:c>
-      <x:c r="B2" s="76"/>
-      <x:c r="C2" s="76"/>
-      <x:c r="D2" s="76"/>
-      <x:c r="E2" s="76"/>
+      <x:c r="B2" s="268"/>
+      <x:c r="C2" s="268"/>
+      <x:c r="D2" s="268"/>
+      <x:c r="E2" s="268"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="81" t="str">
+      <x:c r="A4" s="273" t="str">
         <x:v>Person ID</x:v>
       </x:c>
-      <x:c r="B4" s="81" t="str">
+      <x:c r="B4" s="273" t="str">
         <x:v>Name</x:v>
       </x:c>
-      <x:c r="C4" s="81" t="str">
+      <x:c r="C4" s="273" t="str">
         <x:v>Hackathon #s</x:v>
       </x:c>
-      <x:c r="D4" s="81" t="str">
+      <x:c r="D4" s="273" t="str">
         <x:v>Builds Together</x:v>
       </x:c>
-      <x:c r="E4" s="81" t="str">
+      <x:c r="E4" s="273" t="str">
         <x:v>LinkedIn URL</x:v>
       </x:c>
     </x:row>
@@ -7508,12 +8114,690 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R45bd2c53e7074db0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rcbc3366266394a6c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R88f217f5678d49e9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rc5d39091b8554c39"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf77f56bc5fa3424d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0d479790cd04231"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="56" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="56" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="56" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="264" t="str">
+        <x:v>Socials by Hackathon</x:v>
+      </x:c>
+      <x:c r="B1" s="264"/>
+      <x:c r="C1" s="264"/>
+      <x:c r="D1" s="264"/>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="268" t="str">
+        <x:v>One row per numbered hackathon. Add only posts that clearly document the relevant build or event.</x:v>
+      </x:c>
+      <x:c r="B2" s="268"/>
+      <x:c r="C2" s="268"/>
+      <x:c r="D2" s="268"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="273" t="str">
+        <x:v>Hackathon #</x:v>
+      </x:c>
+      <x:c r="B4" s="273" t="str">
+        <x:v>LinkedIn</x:v>
+      </x:c>
+      <x:c r="C4" s="273" t="str">
+        <x:v>Instagram</x:v>
+      </x:c>
+      <x:c r="D4" s="273" t="str">
+        <x:v>Facebook</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="A5" s="31" t="str">
+        <x:v>#001</x:v>
+      </x:c>
+      <x:c r="B5" s="33"/>
+      <x:c r="C5" s="33"/>
+      <x:c r="D5" s="33"/>
+    </x:row>
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="A6" s="31" t="str">
+        <x:v>#002</x:v>
+      </x:c>
+      <x:c r="B6" s="33"/>
+      <x:c r="C6" s="33"/>
+      <x:c r="D6" s="33"/>
+    </x:row>
+    <x:row r="7" ht="28" customHeight="1">
+      <x:c r="A7" s="31" t="str">
+        <x:v>#003</x:v>
+      </x:c>
+      <x:c r="B7" s="33"/>
+      <x:c r="C7" s="33"/>
+      <x:c r="D7" s="33"/>
+    </x:row>
+    <x:row r="8" ht="28" customHeight="1">
+      <x:c r="A8" s="31" t="str">
+        <x:v>#004</x:v>
+      </x:c>
+      <x:c r="B8" s="33"/>
+      <x:c r="C8" s="33"/>
+      <x:c r="D8" s="33"/>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="A9" s="31" t="str">
+        <x:v>#005</x:v>
+      </x:c>
+      <x:c r="B9" s="33"/>
+      <x:c r="C9" s="33"/>
+      <x:c r="D9" s="33"/>
+    </x:row>
+    <x:row r="10" ht="28" customHeight="1">
+      <x:c r="A10" s="31" t="str">
+        <x:v>#006</x:v>
+      </x:c>
+      <x:c r="B10" s="33"/>
+      <x:c r="C10" s="33"/>
+      <x:c r="D10" s="33"/>
+    </x:row>
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="A11" s="31" t="str">
+        <x:v>#007</x:v>
+      </x:c>
+      <x:c r="B11" s="33"/>
+      <x:c r="C11" s="33"/>
+      <x:c r="D11" s="33"/>
+    </x:row>
+    <x:row r="12" ht="28" customHeight="1">
+      <x:c r="A12" s="31" t="str">
+        <x:v>#008</x:v>
+      </x:c>
+      <x:c r="B12" s="33"/>
+      <x:c r="C12" s="33"/>
+      <x:c r="D12" s="33"/>
+    </x:row>
+    <x:row r="13" ht="28" customHeight="1">
+      <x:c r="A13" s="31" t="str">
+        <x:v>#009</x:v>
+      </x:c>
+      <x:c r="B13" s="33"/>
+      <x:c r="C13" s="33"/>
+      <x:c r="D13" s="33"/>
+    </x:row>
+    <x:row r="14" ht="28" customHeight="1">
+      <x:c r="A14" s="31" t="str">
+        <x:v>#010</x:v>
+      </x:c>
+      <x:c r="B14" s="33"/>
+      <x:c r="C14" s="33"/>
+      <x:c r="D14" s="33"/>
+    </x:row>
+    <x:row r="15" ht="28" customHeight="1">
+      <x:c r="A15" s="31" t="str">
+        <x:v>#011</x:v>
+      </x:c>
+      <x:c r="B15" s="33"/>
+      <x:c r="C15" s="33"/>
+      <x:c r="D15" s="33"/>
+    </x:row>
+    <x:row r="16" ht="28" customHeight="1">
+      <x:c r="A16" s="31" t="str">
+        <x:v>#012</x:v>
+      </x:c>
+      <x:c r="B16" s="33"/>
+      <x:c r="C16" s="33"/>
+      <x:c r="D16" s="33"/>
+    </x:row>
+    <x:row r="17" ht="28" customHeight="1">
+      <x:c r="A17" s="31" t="str">
+        <x:v>#013</x:v>
+      </x:c>
+      <x:c r="B17" s="33"/>
+      <x:c r="C17" s="33"/>
+      <x:c r="D17" s="33"/>
+    </x:row>
+    <x:row r="18" ht="28" customHeight="1">
+      <x:c r="A18" s="31" t="str">
+        <x:v>#014</x:v>
+      </x:c>
+      <x:c r="B18" s="33"/>
+      <x:c r="C18" s="33"/>
+      <x:c r="D18" s="33"/>
+    </x:row>
+    <x:row r="19" ht="28" customHeight="1">
+      <x:c r="A19" s="31" t="str">
+        <x:v>#015</x:v>
+      </x:c>
+      <x:c r="B19" s="33"/>
+      <x:c r="C19" s="33"/>
+      <x:c r="D19" s="33"/>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="A20" s="31" t="str">
+        <x:v>#016</x:v>
+      </x:c>
+      <x:c r="B20" s="33"/>
+      <x:c r="C20" s="33"/>
+      <x:c r="D20" s="33"/>
+    </x:row>
+    <x:row r="21" ht="28" customHeight="1">
+      <x:c r="A21" s="31" t="str">
+        <x:v>#017</x:v>
+      </x:c>
+      <x:c r="B21" s="33"/>
+      <x:c r="C21" s="33"/>
+      <x:c r="D21" s="33"/>
+    </x:row>
+    <x:row r="22" ht="28" customHeight="1">
+      <x:c r="A22" s="31" t="str">
+        <x:v>#018</x:v>
+      </x:c>
+      <x:c r="B22" s="33"/>
+      <x:c r="C22" s="33"/>
+      <x:c r="D22" s="33"/>
+    </x:row>
+    <x:row r="23" ht="28" customHeight="1">
+      <x:c r="A23" s="31" t="str">
+        <x:v>#019</x:v>
+      </x:c>
+      <x:c r="B23" s="33"/>
+      <x:c r="C23" s="33"/>
+      <x:c r="D23" s="33"/>
+    </x:row>
+    <x:row r="24" ht="28" customHeight="1">
+      <x:c r="A24" s="31" t="str">
+        <x:v>#020</x:v>
+      </x:c>
+      <x:c r="B24" s="33"/>
+      <x:c r="C24" s="33"/>
+      <x:c r="D24" s="33"/>
+    </x:row>
+    <x:row r="25" ht="28" customHeight="1">
+      <x:c r="A25" s="31" t="str">
+        <x:v>#021</x:v>
+      </x:c>
+      <x:c r="B25" s="33"/>
+      <x:c r="C25" s="33"/>
+      <x:c r="D25" s="33"/>
+    </x:row>
+    <x:row r="26" ht="28" customHeight="1">
+      <x:c r="A26" s="31" t="str">
+        <x:v>#022</x:v>
+      </x:c>
+      <x:c r="B26" s="33"/>
+      <x:c r="C26" s="33"/>
+      <x:c r="D26" s="33"/>
+    </x:row>
+    <x:row r="27" ht="28" customHeight="1">
+      <x:c r="A27" s="31" t="str">
+        <x:v>#023</x:v>
+      </x:c>
+      <x:c r="B27" s="33"/>
+      <x:c r="C27" s="33"/>
+      <x:c r="D27" s="33"/>
+    </x:row>
+    <x:row r="28" ht="28" customHeight="1">
+      <x:c r="A28" s="31" t="str">
+        <x:v>#024</x:v>
+      </x:c>
+      <x:c r="B28" s="33"/>
+      <x:c r="C28" s="33"/>
+      <x:c r="D28" s="33"/>
+    </x:row>
+    <x:row r="29" ht="28" customHeight="1">
+      <x:c r="A29" s="31" t="str">
+        <x:v>#025</x:v>
+      </x:c>
+      <x:c r="B29" s="33"/>
+      <x:c r="C29" s="33"/>
+      <x:c r="D29" s="33"/>
+    </x:row>
+    <x:row r="30" ht="28" customHeight="1">
+      <x:c r="A30" s="31" t="str">
+        <x:v>#026</x:v>
+      </x:c>
+      <x:c r="B30" s="33"/>
+      <x:c r="C30" s="33"/>
+      <x:c r="D30" s="33"/>
+    </x:row>
+    <x:row r="31" ht="28" customHeight="1">
+      <x:c r="A31" s="31" t="str">
+        <x:v>#027</x:v>
+      </x:c>
+      <x:c r="B31" s="33"/>
+      <x:c r="C31" s="33"/>
+      <x:c r="D31" s="33"/>
+    </x:row>
+    <x:row r="32" ht="28" customHeight="1">
+      <x:c r="A32" s="31" t="str">
+        <x:v>#028</x:v>
+      </x:c>
+      <x:c r="B32" s="33"/>
+      <x:c r="C32" s="33"/>
+      <x:c r="D32" s="33"/>
+    </x:row>
+    <x:row r="33" ht="28" customHeight="1">
+      <x:c r="A33" s="31" t="str">
+        <x:v>#029</x:v>
+      </x:c>
+      <x:c r="B33" s="33"/>
+      <x:c r="C33" s="33"/>
+      <x:c r="D33" s="33"/>
+    </x:row>
+    <x:row r="34" ht="28" customHeight="1">
+      <x:c r="A34" s="31" t="str">
+        <x:v>#030</x:v>
+      </x:c>
+      <x:c r="B34" s="33"/>
+      <x:c r="C34" s="33"/>
+      <x:c r="D34" s="33"/>
+    </x:row>
+    <x:row r="35" ht="28" customHeight="1">
+      <x:c r="A35" s="31" t="str">
+        <x:v>#031</x:v>
+      </x:c>
+      <x:c r="B35" s="33"/>
+      <x:c r="C35" s="33"/>
+      <x:c r="D35" s="33"/>
+    </x:row>
+    <x:row r="36" ht="28" customHeight="1">
+      <x:c r="A36" s="31" t="str">
+        <x:v>#032</x:v>
+      </x:c>
+      <x:c r="B36" s="33"/>
+      <x:c r="C36" s="33"/>
+      <x:c r="D36" s="33"/>
+    </x:row>
+    <x:row r="37" ht="28" customHeight="1">
+      <x:c r="A37" s="31" t="str">
+        <x:v>#033</x:v>
+      </x:c>
+      <x:c r="B37" s="33"/>
+      <x:c r="C37" s="33"/>
+      <x:c r="D37" s="33"/>
+    </x:row>
+    <x:row r="38" ht="28" customHeight="1">
+      <x:c r="A38" s="31" t="str">
+        <x:v>#034</x:v>
+      </x:c>
+      <x:c r="B38" s="33"/>
+      <x:c r="C38" s="33"/>
+      <x:c r="D38" s="33"/>
+    </x:row>
+    <x:row r="39" ht="28" customHeight="1">
+      <x:c r="A39" s="31" t="str">
+        <x:v>#035</x:v>
+      </x:c>
+      <x:c r="B39" s="33"/>
+      <x:c r="C39" s="33"/>
+      <x:c r="D39" s="33"/>
+    </x:row>
+    <x:row r="40" ht="28" customHeight="1">
+      <x:c r="A40" s="31" t="str">
+        <x:v>#036</x:v>
+      </x:c>
+      <x:c r="B40" s="33"/>
+      <x:c r="C40" s="33"/>
+      <x:c r="D40" s="33"/>
+    </x:row>
+    <x:row r="41" ht="28" customHeight="1">
+      <x:c r="A41" s="31" t="str">
+        <x:v>#037</x:v>
+      </x:c>
+      <x:c r="B41" s="33"/>
+      <x:c r="C41" s="33"/>
+      <x:c r="D41" s="33"/>
+    </x:row>
+    <x:row r="42" ht="28" customHeight="1">
+      <x:c r="A42" s="31" t="str">
+        <x:v>#038</x:v>
+      </x:c>
+      <x:c r="B42" s="33"/>
+      <x:c r="C42" s="33"/>
+      <x:c r="D42" s="33"/>
+    </x:row>
+    <x:row r="43" ht="28" customHeight="1">
+      <x:c r="A43" s="31" t="str">
+        <x:v>#039</x:v>
+      </x:c>
+      <x:c r="B43" s="33"/>
+      <x:c r="C43" s="33"/>
+      <x:c r="D43" s="33"/>
+    </x:row>
+    <x:row r="44" ht="28" customHeight="1">
+      <x:c r="A44" s="31" t="str">
+        <x:v>#040</x:v>
+      </x:c>
+      <x:c r="B44" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7373307701516427264/</x:v>
+      </x:c>
+      <x:c r="C44" s="33"/>
+      <x:c r="D44" s="33"/>
+    </x:row>
+    <x:row r="45" ht="28" customHeight="1">
+      <x:c r="A45" s="31" t="str">
+        <x:v>#041</x:v>
+      </x:c>
+      <x:c r="B45" s="33"/>
+      <x:c r="C45" s="33"/>
+      <x:c r="D45" s="33"/>
+    </x:row>
+    <x:row r="46" ht="28" customHeight="1">
+      <x:c r="A46" s="31" t="str">
+        <x:v>#042</x:v>
+      </x:c>
+      <x:c r="B46" s="33"/>
+      <x:c r="C46" s="33"/>
+      <x:c r="D46" s="33"/>
+    </x:row>
+    <x:row r="47" ht="28" customHeight="1">
+      <x:c r="A47" s="31" t="str">
+        <x:v>#043</x:v>
+      </x:c>
+      <x:c r="B47" s="33"/>
+      <x:c r="C47" s="33"/>
+      <x:c r="D47" s="33"/>
+    </x:row>
+    <x:row r="48" ht="28" customHeight="1">
+      <x:c r="A48" s="31" t="str">
+        <x:v>#044</x:v>
+      </x:c>
+      <x:c r="B48" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7387523389042843648/</x:v>
+      </x:c>
+      <x:c r="C48" s="33"/>
+      <x:c r="D48" s="33"/>
+    </x:row>
+    <x:row r="49" ht="28" customHeight="1">
+      <x:c r="A49" s="31" t="str">
+        <x:v>#045</x:v>
+      </x:c>
+      <x:c r="B49" s="33"/>
+      <x:c r="C49" s="33"/>
+      <x:c r="D49" s="33"/>
+    </x:row>
+    <x:row r="50" ht="28" customHeight="1">
+      <x:c r="A50" s="31" t="str">
+        <x:v>#046</x:v>
+      </x:c>
+      <x:c r="B50" s="33"/>
+      <x:c r="C50" s="33"/>
+      <x:c r="D50" s="33"/>
+    </x:row>
+    <x:row r="51" ht="28" customHeight="1">
+      <x:c r="A51" s="31" t="str">
+        <x:v>#047</x:v>
+      </x:c>
+      <x:c r="B51" s="33"/>
+      <x:c r="C51" s="33"/>
+      <x:c r="D51" s="33"/>
+    </x:row>
+    <x:row r="52" ht="28" customHeight="1">
+      <x:c r="A52" s="31" t="str">
+        <x:v>#048</x:v>
+      </x:c>
+      <x:c r="B52" s="33"/>
+      <x:c r="C52" s="33"/>
+      <x:c r="D52" s="33"/>
+    </x:row>
+    <x:row r="53" ht="28" customHeight="1">
+      <x:c r="A53" s="31" t="str">
+        <x:v>#049</x:v>
+      </x:c>
+      <x:c r="B53" s="33"/>
+      <x:c r="C53" s="33"/>
+      <x:c r="D53" s="33"/>
+    </x:row>
+    <x:row r="54" ht="28" customHeight="1">
+      <x:c r="A54" s="31" t="str">
+        <x:v>#050</x:v>
+      </x:c>
+      <x:c r="B54" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7425889935137837056/</x:v>
+      </x:c>
+      <x:c r="C54" s="33"/>
+      <x:c r="D54" s="33"/>
+    </x:row>
+    <x:row r="55" ht="28" customHeight="1">
+      <x:c r="A55" s="31" t="str">
+        <x:v>#051</x:v>
+      </x:c>
+      <x:c r="B55" s="33"/>
+      <x:c r="C55" s="33"/>
+      <x:c r="D55" s="33"/>
+    </x:row>
+    <x:row r="56" ht="28" customHeight="1">
+      <x:c r="A56" s="31" t="str">
+        <x:v>#052</x:v>
+      </x:c>
+      <x:c r="B56" s="33"/>
+      <x:c r="C56" s="33"/>
+      <x:c r="D56" s="33"/>
+    </x:row>
+    <x:row r="57" ht="28" customHeight="1">
+      <x:c r="A57" s="31" t="str">
+        <x:v>#053</x:v>
+      </x:c>
+      <x:c r="B57" s="33"/>
+      <x:c r="C57" s="33"/>
+      <x:c r="D57" s="33"/>
+    </x:row>
+    <x:row r="58" ht="28" customHeight="1">
+      <x:c r="A58" s="31" t="str">
+        <x:v>#054</x:v>
+      </x:c>
+      <x:c r="B58" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7438474540781006848/</x:v>
+      </x:c>
+      <x:c r="C58" s="33"/>
+      <x:c r="D58" s="33"/>
+    </x:row>
+    <x:row r="59" ht="28" customHeight="1">
+      <x:c r="A59" s="31" t="str">
+        <x:v>#055</x:v>
+      </x:c>
+      <x:c r="B59" s="33"/>
+      <x:c r="C59" s="33"/>
+      <x:c r="D59" s="33"/>
+    </x:row>
+    <x:row r="60" ht="28" customHeight="1">
+      <x:c r="A60" s="31" t="str">
+        <x:v>#056</x:v>
+      </x:c>
+      <x:c r="B60" s="33"/>
+      <x:c r="C60" s="33"/>
+      <x:c r="D60" s="33"/>
+    </x:row>
+    <x:row r="61" ht="28" customHeight="1">
+      <x:c r="A61" s="31" t="str">
+        <x:v>#057</x:v>
+      </x:c>
+      <x:c r="B61" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7448758050586521600/</x:v>
+      </x:c>
+      <x:c r="C61" s="33"/>
+      <x:c r="D61" s="33"/>
+    </x:row>
+    <x:row r="62" ht="28" customHeight="1">
+      <x:c r="A62" s="31" t="str">
+        <x:v>#058</x:v>
+      </x:c>
+      <x:c r="B62" s="33"/>
+      <x:c r="C62" s="33"/>
+      <x:c r="D62" s="33"/>
+    </x:row>
+    <x:row r="63" ht="28" customHeight="1">
+      <x:c r="A63" s="31" t="str">
+        <x:v>#059</x:v>
+      </x:c>
+      <x:c r="B63" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7455961388025389056/</x:v>
+      </x:c>
+      <x:c r="C63" s="33"/>
+      <x:c r="D63" s="33"/>
+    </x:row>
+    <x:row r="64" ht="28" customHeight="1">
+      <x:c r="A64" s="31" t="str">
+        <x:v>#060</x:v>
+      </x:c>
+      <x:c r="B64" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7455961388025389056/</x:v>
+      </x:c>
+      <x:c r="C64" s="33"/>
+      <x:c r="D64" s="33"/>
+    </x:row>
+    <x:row r="65" ht="28" customHeight="1">
+      <x:c r="A65" s="31" t="str">
+        <x:v>#061</x:v>
+      </x:c>
+      <x:c r="B65" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7455961388025389056/</x:v>
+      </x:c>
+      <x:c r="C65" s="33"/>
+      <x:c r="D65" s="33"/>
+    </x:row>
+    <x:row r="66" ht="28" customHeight="1">
+      <x:c r="A66" s="31" t="str">
+        <x:v>#062</x:v>
+      </x:c>
+      <x:c r="B66" s="33"/>
+      <x:c r="C66" s="33"/>
+      <x:c r="D66" s="33"/>
+    </x:row>
+    <x:row r="67" ht="28" customHeight="1">
+      <x:c r="A67" s="31" t="str">
+        <x:v>#063</x:v>
+      </x:c>
+      <x:c r="B67" s="33"/>
+      <x:c r="C67" s="33"/>
+      <x:c r="D67" s="33"/>
+    </x:row>
+    <x:row r="68" ht="28" customHeight="1">
+      <x:c r="A68" s="31" t="str">
+        <x:v>#064</x:v>
+      </x:c>
+      <x:c r="B68" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7459414332150534144/</x:v>
+      </x:c>
+      <x:c r="C68" s="33"/>
+      <x:c r="D68" s="33"/>
+    </x:row>
+    <x:row r="69" ht="28" customHeight="1">
+      <x:c r="A69" s="31" t="str">
+        <x:v>#065</x:v>
+      </x:c>
+      <x:c r="B69" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7462661884056416256/</x:v>
+      </x:c>
+      <x:c r="C69" s="33"/>
+      <x:c r="D69" s="33"/>
+    </x:row>
+    <x:row r="70" ht="28" customHeight="1">
+      <x:c r="A70" s="31" t="str">
+        <x:v>#066</x:v>
+      </x:c>
+      <x:c r="B70" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7471043781799178240/</x:v>
+      </x:c>
+      <x:c r="C70" s="33"/>
+      <x:c r="D70" s="33"/>
+    </x:row>
+    <x:row r="71" ht="28" customHeight="1">
+      <x:c r="A71" s="31" t="str">
+        <x:v>#067</x:v>
+      </x:c>
+      <x:c r="B71" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7472197868632571905/</x:v>
+      </x:c>
+      <x:c r="C71" s="33"/>
+      <x:c r="D71" s="33"/>
+    </x:row>
+    <x:row r="72" ht="28" customHeight="1">
+      <x:c r="A72" s="31" t="str">
+        <x:v>#068</x:v>
+      </x:c>
+      <x:c r="B72" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7480285163512418306/</x:v>
+      </x:c>
+      <x:c r="C72" s="33"/>
+      <x:c r="D72" s="33"/>
+    </x:row>
+    <x:row r="73" ht="28" customHeight="1">
+      <x:c r="A73" s="31" t="str">
+        <x:v>#069</x:v>
+      </x:c>
+      <x:c r="B73" s="33"/>
+      <x:c r="C73" s="33"/>
+      <x:c r="D73" s="33"/>
+    </x:row>
+    <x:row r="74" ht="28" customHeight="1">
+      <x:c r="A74" s="31" t="str">
+        <x:v>#070</x:v>
+      </x:c>
+      <x:c r="B74" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7477508615239585792/</x:v>
+      </x:c>
+      <x:c r="C74" s="33"/>
+      <x:c r="D74" s="33"/>
+    </x:row>
+    <x:row r="75" ht="28" customHeight="1">
+      <x:c r="A75" s="31" t="str">
+        <x:v>#071</x:v>
+      </x:c>
+      <x:c r="B75" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7482072463900835840/</x:v>
+      </x:c>
+      <x:c r="C75" s="33"/>
+      <x:c r="D75" s="33"/>
+    </x:row>
+    <x:row r="76" ht="28" customHeight="1">
+      <x:c r="A76" s="31" t="str">
+        <x:v>#072</x:v>
+      </x:c>
+      <x:c r="B76" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7486774772140474368/</x:v>
+      </x:c>
+      <x:c r="C76" s="33"/>
+      <x:c r="D76" s="33"/>
+    </x:row>
+    <x:row r="77" ht="28" customHeight="1">
+      <x:c r="A77" s="31" t="str">
+        <x:v>#073</x:v>
+      </x:c>
+      <x:c r="B77" s="33"/>
+      <x:c r="C77" s="33"/>
+      <x:c r="D77" s="33"/>
+    </x:row>
+    <x:row r="78" ht="28" customHeight="1">
+      <x:c r="A78" s="31" t="str">
+        <x:v>#074</x:v>
+      </x:c>
+      <x:c r="B78" s="33" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7490764342309855232/</x:v>
+      </x:c>
+      <x:c r="C78" s="33"/>
+      <x:c r="D78" s="33"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A2:D2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbcab74682574abe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
data: add verified Instagram social links
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Raa580b2d22704c99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R52b5067bfad74239"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R15748b08699e4984"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R7c2bf57a340d4397"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rd065917edd194156"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rb4aa76b357a949be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1687,12 +1687,72 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="71">
+  <x:fills count="83">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -2075,7 +2135,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="286">
+  <x:cellXfs count="334">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2616,6 +2676,94 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="70" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="76" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="76" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="76" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="79" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="79" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="79" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="79" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="79" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="82" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="82" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="82" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2651,7 +2799,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="PeopleDirectory" displayName="PeopleDirectory" ref="A4:E97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="PeopleDirectory" displayName="PeopleDirectory" ref="A4:E97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:E97"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Person ID"/>
@@ -2665,7 +2813,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="HackathonSocials" displayName="HackathonSocials" ref="A4:D78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="HackathonSocials" displayName="HackathonSocials" ref="A4:D78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:D78"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Hackathon #"/>
@@ -6583,8 +6731,8 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rdb908968ce9e4eca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R53c9e167c902416c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R1b3ae87c4d7b46fe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R6938c3b897514945"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6606,37 +6754,37 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="276" t="str">
+      <x:c r="A1" s="324" t="str">
         <x:v>People &amp; LinkedIn Directory</x:v>
       </x:c>
-      <x:c r="B1" s="276"/>
-      <x:c r="C1" s="276"/>
-      <x:c r="D1" s="276"/>
-      <x:c r="E1" s="276"/>
+      <x:c r="B1" s="324"/>
+      <x:c r="C1" s="324"/>
+      <x:c r="D1" s="324"/>
+      <x:c r="E1" s="324"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="280" t="str">
+      <x:c r="A2" s="328" t="str">
         <x:v>One person per row. LinkedIn URLs are added only after the profile has been verified against the hackathon context.</x:v>
       </x:c>
-      <x:c r="B2" s="280"/>
-      <x:c r="C2" s="280"/>
-      <x:c r="D2" s="280"/>
-      <x:c r="E2" s="280"/>
+      <x:c r="B2" s="328"/>
+      <x:c r="C2" s="328"/>
+      <x:c r="D2" s="328"/>
+      <x:c r="E2" s="328"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="285" t="str">
+      <x:c r="A4" s="333" t="str">
         <x:v>Person ID</x:v>
       </x:c>
-      <x:c r="B4" s="285" t="str">
+      <x:c r="B4" s="333" t="str">
         <x:v>Name</x:v>
       </x:c>
-      <x:c r="C4" s="285" t="str">
+      <x:c r="C4" s="333" t="str">
         <x:v>Hackathon #s</x:v>
       </x:c>
-      <x:c r="D4" s="285" t="str">
+      <x:c r="D4" s="333" t="str">
         <x:v>Builds Together</x:v>
       </x:c>
-      <x:c r="E4" s="285" t="str">
+      <x:c r="E4" s="333" t="str">
         <x:v>LinkedIn URL</x:v>
       </x:c>
     </x:row>
@@ -8151,12 +8299,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R9cab7809317048d4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R8b303ccf99714314"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R3b3d8b41fc4740ea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rb6dfd90f61dc42d3"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53edaf8e007c441a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cc9331619654673"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8172,32 +8320,32 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="276" t="str">
+      <x:c r="A1" s="324" t="str">
         <x:v>Socials by Hackathon</x:v>
       </x:c>
-      <x:c r="B1" s="276"/>
-      <x:c r="C1" s="276"/>
-      <x:c r="D1" s="276"/>
+      <x:c r="B1" s="324"/>
+      <x:c r="C1" s="324"/>
+      <x:c r="D1" s="324"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="280" t="str">
+      <x:c r="A2" s="328" t="str">
         <x:v>One row per numbered hackathon. Add only posts that clearly document the relevant build or event.</x:v>
       </x:c>
-      <x:c r="B2" s="280"/>
-      <x:c r="C2" s="280"/>
-      <x:c r="D2" s="280"/>
+      <x:c r="B2" s="328"/>
+      <x:c r="C2" s="328"/>
+      <x:c r="D2" s="328"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="285" t="str">
+      <x:c r="A4" s="333" t="str">
         <x:v>Hackathon #</x:v>
       </x:c>
-      <x:c r="B4" s="285" t="str">
+      <x:c r="B4" s="333" t="str">
         <x:v>LinkedIn</x:v>
       </x:c>
-      <x:c r="C4" s="285" t="str">
+      <x:c r="C4" s="333" t="str">
         <x:v>Instagram</x:v>
       </x:c>
-      <x:c r="D4" s="285" t="str">
+      <x:c r="D4" s="333" t="str">
         <x:v>Facebook</x:v>
       </x:c>
     </x:row>
@@ -8286,7 +8434,9 @@
         <x:v>#011</x:v>
       </x:c>
       <x:c r="B15" s="33"/>
-      <x:c r="C15" s="33"/>
+      <x:c r="C15" s="33" t="str">
+        <x:v>https://www.instagram.com/p/BZsdBDyAuNk/</x:v>
+      </x:c>
       <x:c r="D15" s="33"/>
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
@@ -8310,7 +8460,9 @@
         <x:v>#014</x:v>
       </x:c>
       <x:c r="B18" s="33"/>
-      <x:c r="C18" s="33"/>
+      <x:c r="C18" s="33" t="str">
+        <x:v>https://www.instagram.com/p/BgWUFk4FOSa/</x:v>
+      </x:c>
       <x:c r="D18" s="33"/>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
@@ -8318,7 +8470,9 @@
         <x:v>#015</x:v>
       </x:c>
       <x:c r="B19" s="33"/>
-      <x:c r="C19" s="33"/>
+      <x:c r="C19" s="33" t="str">
+        <x:v>https://www.instagram.com/p/Bgvs2dLAeue/</x:v>
+      </x:c>
       <x:c r="D19" s="33"/>
     </x:row>
     <x:row r="20" ht="28" customHeight="1">
@@ -8334,7 +8488,9 @@
         <x:v>#017</x:v>
       </x:c>
       <x:c r="B21" s="33"/>
-      <x:c r="C21" s="33"/>
+      <x:c r="C21" s="33" t="str">
+        <x:v>https://www.instagram.com/p/BjogOfOA6tG/</x:v>
+      </x:c>
       <x:c r="D21" s="33"/>
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
@@ -8342,7 +8498,10 @@
         <x:v>#018</x:v>
       </x:c>
       <x:c r="B22" s="33"/>
-      <x:c r="C22" s="33"/>
+      <x:c r="C22" s="33" t="str">
+        <x:v>https://www.instagram.com/p/BngqOFTggiI/
+https://www.instagram.com/p/Bngpa4igs3o/</x:v>
+      </x:c>
       <x:c r="D22" s="33"/>
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
@@ -8350,7 +8509,9 @@
         <x:v>#019</x:v>
       </x:c>
       <x:c r="B23" s="33"/>
-      <x:c r="C23" s="33"/>
+      <x:c r="C23" s="33" t="str">
+        <x:v>https://www.instagram.com/p/Bo6FW7zg0Zj/</x:v>
+      </x:c>
       <x:c r="D23" s="33"/>
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
@@ -8358,7 +8519,10 @@
         <x:v>#020</x:v>
       </x:c>
       <x:c r="B24" s="33"/>
-      <x:c r="C24" s="33"/>
+      <x:c r="C24" s="33" t="str">
+        <x:v>https://www.instagram.com/p/BpMd-mignvt/
+https://www.instagram.com/p/BpMRvP0g435/</x:v>
+      </x:c>
       <x:c r="D24" s="33"/>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
@@ -8366,7 +8530,9 @@
         <x:v>#021</x:v>
       </x:c>
       <x:c r="B25" s="33"/>
-      <x:c r="C25" s="33"/>
+      <x:c r="C25" s="33" t="str">
+        <x:v>https://www.instagram.com/p/BqADJkbAn8x/</x:v>
+      </x:c>
       <x:c r="D25" s="33"/>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
@@ -8382,7 +8548,9 @@
         <x:v>#023</x:v>
       </x:c>
       <x:c r="B27" s="33"/>
-      <x:c r="C27" s="33"/>
+      <x:c r="C27" s="33" t="str">
+        <x:v>https://www.instagram.com/p/Bs2f8FHHXNo/</x:v>
+      </x:c>
       <x:c r="D27" s="33"/>
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
@@ -8398,7 +8566,9 @@
         <x:v>#025</x:v>
       </x:c>
       <x:c r="B29" s="33"/>
-      <x:c r="C29" s="33"/>
+      <x:c r="C29" s="33" t="str">
+        <x:v>https://www.instagram.com/p/Bxo5Ka1FLrR/</x:v>
+      </x:c>
       <x:c r="D29" s="33"/>
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
@@ -8422,7 +8592,10 @@
         <x:v>#028</x:v>
       </x:c>
       <x:c r="B32" s="33"/>
-      <x:c r="C32" s="33"/>
+      <x:c r="C32" s="33" t="str">
+        <x:v>https://www.instagram.com/p/B2EYk1KluTZ/
+https://www.instagram.com/p/B2JzcFglegx/</x:v>
+      </x:c>
       <x:c r="D32" s="33"/>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
@@ -8446,7 +8619,9 @@
         <x:v>#031</x:v>
       </x:c>
       <x:c r="B35" s="33"/>
-      <x:c r="C35" s="33"/>
+      <x:c r="C35" s="33" t="str">
+        <x:v>https://www.instagram.com/p/CrGJq7JvfYS/</x:v>
+      </x:c>
       <x:c r="D35" s="33"/>
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
@@ -8454,7 +8629,9 @@
         <x:v>#032</x:v>
       </x:c>
       <x:c r="B36" s="33"/>
-      <x:c r="C36" s="33"/>
+      <x:c r="C36" s="33" t="str">
+        <x:v>https://www.instagram.com/p/C0_xx0zRc1u/</x:v>
+      </x:c>
       <x:c r="D36" s="33"/>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
@@ -8462,7 +8639,9 @@
         <x:v>#033</x:v>
       </x:c>
       <x:c r="B37" s="33"/>
-      <x:c r="C37" s="33"/>
+      <x:c r="C37" s="33" t="str">
+        <x:v>https://www.instagram.com/p/C1E93kNxOjM/</x:v>
+      </x:c>
       <x:c r="D37" s="33"/>
     </x:row>
     <x:row r="38" ht="28" customHeight="1">
@@ -8470,7 +8649,9 @@
         <x:v>#034</x:v>
       </x:c>
       <x:c r="B38" s="33"/>
-      <x:c r="C38" s="33"/>
+      <x:c r="C38" s="33" t="str">
+        <x:v>https://www.instagram.com/p/C8MapmzSGnB/</x:v>
+      </x:c>
       <x:c r="D38" s="33"/>
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
@@ -8478,7 +8659,10 @@
         <x:v>#035</x:v>
       </x:c>
       <x:c r="B39" s="33"/>
-      <x:c r="C39" s="33"/>
+      <x:c r="C39" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DHlaIwwz9Qg/
+https://www.instagram.com/p/DHlZp4wTHze/</x:v>
+      </x:c>
       <x:c r="D39" s="33"/>
     </x:row>
     <x:row r="40" ht="28" customHeight="1">
@@ -8486,7 +8670,12 @@
         <x:v>#036</x:v>
       </x:c>
       <x:c r="B40" s="33"/>
-      <x:c r="C40" s="33"/>
+      <x:c r="C40" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DLBb3yoT412/
+https://www.instagram.com/p/DLFWtVrx0_O/
+https://www.instagram.com/reel/DLEZ4_LRK_G/
+https://www.instagram.com/reel/DLEGXTsTe1y/</x:v>
+      </x:c>
       <x:c r="D40" s="33"/>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
@@ -8494,7 +8683,9 @@
         <x:v>#037</x:v>
       </x:c>
       <x:c r="B41" s="33"/>
-      <x:c r="C41" s="33"/>
+      <x:c r="C41" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DLcXTxAxUgg/</x:v>
+      </x:c>
       <x:c r="D41" s="33"/>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
@@ -8510,7 +8701,9 @@
         <x:v>#039</x:v>
       </x:c>
       <x:c r="B43" s="33"/>
-      <x:c r="C43" s="33"/>
+      <x:c r="C43" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DNLa9r_xO3o/</x:v>
+      </x:c>
       <x:c r="D43" s="33"/>
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
@@ -8521,7 +8714,9 @@
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7373307701516427264/</x:v>
       </x:c>
       <x:c r="C44" s="33" t="str">
-        <x:v>https://www.instagram.com/reel/DOVLDxsE37O/
+        <x:v>https://www.instagram.com/p/DOQcqfMk4Wk/
+https://www.instagram.com/p/DOVACxLE9PW/
+https://www.instagram.com/reel/DOVLDxsE37O/
 https://www.instagram.com/reel/DOQFqH8kfeT/</x:v>
       </x:c>
       <x:c r="D44" s="33"/>
@@ -8531,7 +8726,9 @@
         <x:v>#041</x:v>
       </x:c>
       <x:c r="B45" s="33"/>
-      <x:c r="C45" s="33"/>
+      <x:c r="C45" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DO0q1KYky3H/</x:v>
+      </x:c>
       <x:c r="D45" s="33"/>
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
@@ -8539,7 +8736,9 @@
         <x:v>#042</x:v>
       </x:c>
       <x:c r="B46" s="33"/>
-      <x:c r="C46" s="33"/>
+      <x:c r="C46" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DPOUBvaE3GR/</x:v>
+      </x:c>
       <x:c r="D46" s="33"/>
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
@@ -8547,7 +8746,9 @@
         <x:v>#043</x:v>
       </x:c>
       <x:c r="B47" s="33"/>
-      <x:c r="C47" s="33"/>
+      <x:c r="C47" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DPbGjobkxFW/</x:v>
+      </x:c>
       <x:c r="D47" s="33"/>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
@@ -8557,7 +8758,9 @@
       <x:c r="B48" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7387523389042843648/</x:v>
       </x:c>
-      <x:c r="C48" s="33"/>
+      <x:c r="C48" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DP-pSUWjPCS/</x:v>
+      </x:c>
       <x:c r="D48" s="33"/>
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
@@ -8601,7 +8804,9 @@
         <x:v>#049</x:v>
       </x:c>
       <x:c r="B53" s="33"/>
-      <x:c r="C53" s="33"/>
+      <x:c r="C53" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DT49z3cE84y/</x:v>
+      </x:c>
       <x:c r="D53" s="33"/>
     </x:row>
     <x:row r="54" ht="28" customHeight="1">
@@ -8611,7 +8816,9 @@
       <x:c r="B54" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7425889935137837056/</x:v>
       </x:c>
-      <x:c r="C54" s="33"/>
+      <x:c r="C54" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DUdGe1jk_Wh/</x:v>
+      </x:c>
       <x:c r="D54" s="33"/>
     </x:row>
     <x:row r="55" ht="28" customHeight="1">
@@ -8627,7 +8834,9 @@
         <x:v>#052</x:v>
       </x:c>
       <x:c r="B56" s="33"/>
-      <x:c r="C56" s="33"/>
+      <x:c r="C56" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DVTWt5qE6QA/</x:v>
+      </x:c>
       <x:c r="D56" s="33"/>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
@@ -8635,7 +8844,9 @@
         <x:v>#053</x:v>
       </x:c>
       <x:c r="B57" s="33"/>
-      <x:c r="C57" s="33"/>
+      <x:c r="C57" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DVTWt5qE6QA/</x:v>
+      </x:c>
       <x:c r="D57" s="33"/>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
@@ -8645,7 +8856,9 @@
       <x:c r="B58" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7438474540781006848/</x:v>
       </x:c>
-      <x:c r="C58" s="33"/>
+      <x:c r="C58" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DV0x7PoE18a/</x:v>
+      </x:c>
       <x:c r="D58" s="33"/>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
@@ -8653,7 +8866,9 @@
         <x:v>#055</x:v>
       </x:c>
       <x:c r="B59" s="33"/>
-      <x:c r="C59" s="33"/>
+      <x:c r="C59" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DWd1UjUkwSf/</x:v>
+      </x:c>
       <x:c r="D59" s="33"/>
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
@@ -8671,7 +8886,10 @@
       <x:c r="B61" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7448758050586521600/</x:v>
       </x:c>
-      <x:c r="C61" s="33"/>
+      <x:c r="C61" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DW9CxfwE6Ln/
+https://www.instagram.com/p/DW_vFeIk0-2/</x:v>
+      </x:c>
       <x:c r="D61" s="33"/>
     </x:row>
     <x:row r="62" ht="28" customHeight="1">
@@ -8679,7 +8897,9 @@
         <x:v>#058</x:v>
       </x:c>
       <x:c r="B62" s="33"/>
-      <x:c r="C62" s="33"/>
+      <x:c r="C62" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DXRahaqk28d/</x:v>
+      </x:c>
       <x:c r="D62" s="33"/>
     </x:row>
     <x:row r="63" ht="28" customHeight="1">
@@ -8689,7 +8909,9 @@
       <x:c r="B63" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7455961388025389056/</x:v>
       </x:c>
-      <x:c r="C63" s="33"/>
+      <x:c r="C63" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DXg-YyWE5r6/</x:v>
+      </x:c>
       <x:c r="D63" s="33"/>
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
@@ -8699,7 +8921,9 @@
       <x:c r="B64" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7455961388025389056/</x:v>
       </x:c>
-      <x:c r="C64" s="33"/>
+      <x:c r="C64" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DXwnu_3E2dI/</x:v>
+      </x:c>
       <x:c r="D64" s="33"/>
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
@@ -8710,7 +8934,8 @@
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7455961388025389056/</x:v>
       </x:c>
       <x:c r="C65" s="33" t="str">
-        <x:v>https://www.instagram.com/reel/DXykZomTmXD/</x:v>
+        <x:v>https://www.instagram.com/p/DXwqrEOkwoB/
+https://www.instagram.com/reel/DXykZomTmXD/</x:v>
       </x:c>
       <x:c r="D65" s="33"/>
     </x:row>
@@ -8719,7 +8944,9 @@
         <x:v>#062</x:v>
       </x:c>
       <x:c r="B66" s="33"/>
-      <x:c r="C66" s="33"/>
+      <x:c r="C66" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DX4HAVzE9WO/</x:v>
+      </x:c>
       <x:c r="D66" s="33"/>
     </x:row>
     <x:row r="67" ht="28" customHeight="1">
@@ -8737,7 +8964,9 @@
       <x:c r="B68" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7459414332150534144/</x:v>
       </x:c>
-      <x:c r="C68" s="33"/>
+      <x:c r="C68" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DYLfGwuk3Xc/</x:v>
+      </x:c>
       <x:c r="D68" s="33"/>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
@@ -8747,7 +8976,9 @@
       <x:c r="B69" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7462661884056416256/</x:v>
       </x:c>
-      <x:c r="C69" s="33"/>
+      <x:c r="C69" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DYe1dlpE7Af/</x:v>
+      </x:c>
       <x:c r="D69" s="33"/>
     </x:row>
     <x:row r="70" ht="28" customHeight="1">
@@ -8808,6 +9039,7 @@
       </x:c>
       <x:c r="C74" s="33" t="str">
         <x:v>https://www.instagram.com/p/DaFSqK7k2ce/
+https://www.instagram.com/p/DaFSaYHkwPC/
 https://www.instagram.com/reel/DaFm4k2zifY/</x:v>
       </x:c>
       <x:c r="D74" s="33"/>
@@ -8865,7 +9097,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10e5c17c0bbe49e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4b0574c63c6488f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add verified Facebook hackathon posts
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R7c2bf57a340d4397"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rd065917edd194156"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rb4aa76b357a949be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R9aa34ef47d804ffb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Reb5da65a08cb43e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R0d0eafa1c156406f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1687,12 +1687,27 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="83">
+  <x:fills count="86">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -2135,7 +2150,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="334">
+  <x:cellXfs count="346">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2764,6 +2779,28 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="82" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="85" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="85" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="85" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2799,7 +2836,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="PeopleDirectory" displayName="PeopleDirectory" ref="A4:E97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="PeopleDirectory" displayName="PeopleDirectory" ref="A4:E97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:E97"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Person ID"/>
@@ -2813,7 +2850,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="HackathonSocials" displayName="HackathonSocials" ref="A4:D78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="HackathonSocials" displayName="HackathonSocials" ref="A4:D78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:D78"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Hackathon #"/>
@@ -6731,8 +6768,8 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R1b3ae87c4d7b46fe"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R6938c3b897514945"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rb6075c084f8c45f3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Ra245c1e0d8674d83"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6754,37 +6791,37 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="324" t="str">
+      <x:c r="A1" s="336" t="str">
         <x:v>People &amp; LinkedIn Directory</x:v>
       </x:c>
-      <x:c r="B1" s="324"/>
-      <x:c r="C1" s="324"/>
-      <x:c r="D1" s="324"/>
-      <x:c r="E1" s="324"/>
+      <x:c r="B1" s="336"/>
+      <x:c r="C1" s="336"/>
+      <x:c r="D1" s="336"/>
+      <x:c r="E1" s="336"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="328" t="str">
+      <x:c r="A2" s="340" t="str">
         <x:v>One person per row. LinkedIn URLs are added only after the profile has been verified against the hackathon context.</x:v>
       </x:c>
-      <x:c r="B2" s="328"/>
-      <x:c r="C2" s="328"/>
-      <x:c r="D2" s="328"/>
-      <x:c r="E2" s="328"/>
+      <x:c r="B2" s="340"/>
+      <x:c r="C2" s="340"/>
+      <x:c r="D2" s="340"/>
+      <x:c r="E2" s="340"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="333" t="str">
+      <x:c r="A4" s="345" t="str">
         <x:v>Person ID</x:v>
       </x:c>
-      <x:c r="B4" s="333" t="str">
+      <x:c r="B4" s="345" t="str">
         <x:v>Name</x:v>
       </x:c>
-      <x:c r="C4" s="333" t="str">
+      <x:c r="C4" s="345" t="str">
         <x:v>Hackathon #s</x:v>
       </x:c>
-      <x:c r="D4" s="333" t="str">
+      <x:c r="D4" s="345" t="str">
         <x:v>Builds Together</x:v>
       </x:c>
-      <x:c r="E4" s="333" t="str">
+      <x:c r="E4" s="345" t="str">
         <x:v>LinkedIn URL</x:v>
       </x:c>
     </x:row>
@@ -8299,12 +8336,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R3b3d8b41fc4740ea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rb6dfd90f61dc42d3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R7ab314a0fed54074"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R1f6be82af4b84a01"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cc9331619654673"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7bad1ff2b1047cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8320,32 +8357,32 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="324" t="str">
+      <x:c r="A1" s="336" t="str">
         <x:v>Socials by Hackathon</x:v>
       </x:c>
-      <x:c r="B1" s="324"/>
-      <x:c r="C1" s="324"/>
-      <x:c r="D1" s="324"/>
+      <x:c r="B1" s="336"/>
+      <x:c r="C1" s="336"/>
+      <x:c r="D1" s="336"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="328" t="str">
+      <x:c r="A2" s="340" t="str">
         <x:v>One row per numbered hackathon. Add only posts that clearly document the relevant build or event.</x:v>
       </x:c>
-      <x:c r="B2" s="328"/>
-      <x:c r="C2" s="328"/>
-      <x:c r="D2" s="328"/>
+      <x:c r="B2" s="340"/>
+      <x:c r="C2" s="340"/>
+      <x:c r="D2" s="340"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="333" t="str">
+      <x:c r="A4" s="345" t="str">
         <x:v>Hackathon #</x:v>
       </x:c>
-      <x:c r="B4" s="333" t="str">
+      <x:c r="B4" s="345" t="str">
         <x:v>LinkedIn</x:v>
       </x:c>
-      <x:c r="C4" s="333" t="str">
+      <x:c r="C4" s="345" t="str">
         <x:v>Instagram</x:v>
       </x:c>
-      <x:c r="D4" s="333" t="str">
+      <x:c r="D4" s="345" t="str">
         <x:v>Facebook</x:v>
       </x:c>
     </x:row>
@@ -8596,7 +8633,10 @@
         <x:v>https://www.instagram.com/p/B2EYk1KluTZ/
 https://www.instagram.com/p/B2JzcFglegx/</x:v>
       </x:c>
-      <x:c r="D32" s="33"/>
+      <x:c r="D32" s="33" t="str">
+        <x:v>https://www.facebook.com/sayyid.iskandar/posts/pfbid0rxHXvZDwNWumGZdXFgUnJiu12SW3FUwyTueeejHBw8a6tAGgyLHUFeZB8n2iNhmfl
+https://www.facebook.com/sayyid.iskandar/posts/pfbid02YSrksK2xzkZUh8uifPrWYxk6VHt7aMVfcef6vc1AXoauq9GTCUGQQpLDQpbUUAUyl</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="31" t="str">
@@ -8604,7 +8644,9 @@
       </x:c>
       <x:c r="B33" s="33"/>
       <x:c r="C33" s="33"/>
-      <x:c r="D33" s="33"/>
+      <x:c r="D33" s="33" t="str">
+        <x:v>https://www.facebook.com/sayyid.iskandar/posts/pfbid02HTKxyfqPKL2uR4n9zFFxAzkXbE7FYNjkzzuQpqRpEgeCBzYnqvfko88xe9nDPD4kl</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
       <x:c r="A34" s="31" t="str">
@@ -8612,7 +8654,9 @@
       </x:c>
       <x:c r="B34" s="33"/>
       <x:c r="C34" s="33"/>
-      <x:c r="D34" s="33"/>
+      <x:c r="D34" s="33" t="str">
+        <x:v>https://www.facebook.com/sayyid.iskandar/posts/pfbid02T7TywvEM5ypGy8vVEQyJVS1ZAzQns7CGz483NQGZX5CKf1DaCw8P6VbcAFdQmqczl</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
       <x:c r="A35" s="31" t="str">
@@ -9097,7 +9141,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4b0574c63c6488f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20f0bc675f6a4498"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Facebook links for early hackathons
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R9aa34ef47d804ffb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Reb5da65a08cb43e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R0d0eafa1c156406f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R28e005c0099e4b40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R6705015e69934533"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R1595edbff3bf4d76"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1687,12 +1687,57 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="86">
+  <x:fills count="95">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -2150,7 +2195,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="346">
+  <x:cellXfs count="382">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2801,6 +2846,72 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="85" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="88" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="88" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="88" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="90" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="90" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="90" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="90" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="91" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="91" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="91" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="91" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="91" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="92" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="92" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="92" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="93" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="93" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="93" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="93" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="94" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="94" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="94" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="94" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="94" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2836,7 +2947,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="PeopleDirectory" displayName="PeopleDirectory" ref="A4:E97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="PeopleDirectory" displayName="PeopleDirectory" ref="A4:E97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:E97"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Person ID"/>
@@ -2850,7 +2961,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="HackathonSocials" displayName="HackathonSocials" ref="A4:D78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="HackathonSocials" displayName="HackathonSocials" ref="A4:D78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:D78"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Hackathon #"/>
@@ -6768,8 +6879,8 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rb6075c084f8c45f3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Ra245c1e0d8674d83"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rd1d6895ee3984d3d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R575e2953fed6448a"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6791,37 +6902,37 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="336" t="str">
+      <x:c r="A1" s="372" t="str">
         <x:v>People &amp; LinkedIn Directory</x:v>
       </x:c>
-      <x:c r="B1" s="336"/>
-      <x:c r="C1" s="336"/>
-      <x:c r="D1" s="336"/>
-      <x:c r="E1" s="336"/>
+      <x:c r="B1" s="372"/>
+      <x:c r="C1" s="372"/>
+      <x:c r="D1" s="372"/>
+      <x:c r="E1" s="372"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="340" t="str">
+      <x:c r="A2" s="376" t="str">
         <x:v>One person per row. LinkedIn URLs are added only after the profile has been verified against the hackathon context.</x:v>
       </x:c>
-      <x:c r="B2" s="340"/>
-      <x:c r="C2" s="340"/>
-      <x:c r="D2" s="340"/>
-      <x:c r="E2" s="340"/>
+      <x:c r="B2" s="376"/>
+      <x:c r="C2" s="376"/>
+      <x:c r="D2" s="376"/>
+      <x:c r="E2" s="376"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="345" t="str">
+      <x:c r="A4" s="381" t="str">
         <x:v>Person ID</x:v>
       </x:c>
-      <x:c r="B4" s="345" t="str">
+      <x:c r="B4" s="381" t="str">
         <x:v>Name</x:v>
       </x:c>
-      <x:c r="C4" s="345" t="str">
+      <x:c r="C4" s="381" t="str">
         <x:v>Hackathon #s</x:v>
       </x:c>
-      <x:c r="D4" s="345" t="str">
+      <x:c r="D4" s="381" t="str">
         <x:v>Builds Together</x:v>
       </x:c>
-      <x:c r="E4" s="345" t="str">
+      <x:c r="E4" s="381" t="str">
         <x:v>LinkedIn URL</x:v>
       </x:c>
     </x:row>
@@ -8336,12 +8447,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R7ab314a0fed54074"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R1f6be82af4b84a01"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R4ee87c5572dc4665"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R7d80b928feb14ef1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7bad1ff2b1047cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b0067a011d6440a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8357,32 +8468,32 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="336" t="str">
+      <x:c r="A1" s="372" t="str">
         <x:v>Socials by Hackathon</x:v>
       </x:c>
-      <x:c r="B1" s="336"/>
-      <x:c r="C1" s="336"/>
-      <x:c r="D1" s="336"/>
+      <x:c r="B1" s="372"/>
+      <x:c r="C1" s="372"/>
+      <x:c r="D1" s="372"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="340" t="str">
+      <x:c r="A2" s="376" t="str">
         <x:v>One row per numbered hackathon. Add only posts that clearly document the relevant build or event.</x:v>
       </x:c>
-      <x:c r="B2" s="340"/>
-      <x:c r="C2" s="340"/>
-      <x:c r="D2" s="340"/>
+      <x:c r="B2" s="376"/>
+      <x:c r="C2" s="376"/>
+      <x:c r="D2" s="376"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="345" t="str">
+      <x:c r="A4" s="381" t="str">
         <x:v>Hackathon #</x:v>
       </x:c>
-      <x:c r="B4" s="345" t="str">
+      <x:c r="B4" s="381" t="str">
         <x:v>LinkedIn</x:v>
       </x:c>
-      <x:c r="C4" s="345" t="str">
+      <x:c r="C4" s="381" t="str">
         <x:v>Instagram</x:v>
       </x:c>
-      <x:c r="D4" s="345" t="str">
+      <x:c r="D4" s="381" t="str">
         <x:v>Facebook</x:v>
       </x:c>
     </x:row>
@@ -8614,7 +8725,9 @@
       </x:c>
       <x:c r="B30" s="33"/>
       <x:c r="C30" s="33"/>
-      <x:c r="D30" s="33"/>
+      <x:c r="D30" s="33" t="str">
+        <x:v>https://www.facebook.com/share/p/18y8TAM2dB/</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="31" t="str">
@@ -8622,7 +8735,9 @@
       </x:c>
       <x:c r="B31" s="33"/>
       <x:c r="C31" s="33"/>
-      <x:c r="D31" s="33"/>
+      <x:c r="D31" s="33" t="str">
+        <x:v>https://www.facebook.com/share/p/1F5LDVBjUj/</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="28" customHeight="1">
       <x:c r="A32" s="31" t="str">
@@ -8635,7 +8750,10 @@
       </x:c>
       <x:c r="D32" s="33" t="str">
         <x:v>https://www.facebook.com/sayyid.iskandar/posts/pfbid0rxHXvZDwNWumGZdXFgUnJiu12SW3FUwyTueeejHBw8a6tAGgyLHUFeZB8n2iNhmfl
-https://www.facebook.com/sayyid.iskandar/posts/pfbid02YSrksK2xzkZUh8uifPrWYxk6VHt7aMVfcef6vc1AXoauq9GTCUGQQpLDQpbUUAUyl</x:v>
+https://www.facebook.com/sayyid.iskandar/posts/pfbid02YSrksK2xzkZUh8uifPrWYxk6VHt7aMVfcef6vc1AXoauq9GTCUGQQpLDQpbUUAUyl
+https://www.facebook.com/share/p/1DSDV99DjY/
+https://www.facebook.com/share/p/1HXZcYB6ew/
+https://www.facebook.com/share/p/1BiUy52YeW/</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
@@ -9141,7 +9259,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20f0bc675f6a4498"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d0182c10172441c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add hackathon 76 and collaboration details
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rc307e89d2d8945f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rbf64d9745936415f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rc1207e026d3c4b46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R7590d383b6dd40f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R47a7aa279be44f0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Ra285abd31123409f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rf13838d95dd94a59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R55b80483501b4af8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7292,12 +7292,62 @@
         <x:v>571</x:v>
       </x:c>
     </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>Build with Gemini Hackathon 2026</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>65labs, Google, Lorong AI</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>22/08/2026</x:v>
+      </x:c>
+      <x:c r="E77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>Days</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>Agentic AI</x:v>
+      </x:c>
+      <x:c r="I77" t="str">
+        <x:v>A local-first city-management game where players govern Innovation City with Gemma as an on-device chief of staff for incident triage, guardrails, and scenario stress-testing.</x:v>
+      </x:c>
+      <x:c r="J77" t="str">
+        <x:v>sayyid</x:v>
+      </x:c>
+      <x:c r="K77" t="str">
+        <x:v>Agrim Tycoon</x:v>
+      </x:c>
+      <x:c r="L77" t="str">
+        <x:v>Google DeepMind</x:v>
+      </x:c>
+      <x:c r="M77" t="str">
+        <x:v>Singapore</x:v>
+      </x:c>
+      <x:c r="N77" t="str">
+        <x:v>Lorong AI @ One-North</x:v>
+      </x:c>
+      <x:c r="O77" t="str">
+        <x:v>https://github.com/sayyidkhan/agrim-tycoon</x:v>
+      </x:c>
+      <x:c r="P77" t="str">
+        <x:v>https://luma.com/deepmind-v4ci?tk=LBgGrm</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R5ce0b09602644e1a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R2612d25b05e44e0f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R93ba604481784592"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R6237d52b96ac4461"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rddee6565c28d489e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rb7fffae7adad4e63"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rce319407610248f0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R5d0ef9dfd39b4ace"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -8861,12 +8911,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R8c264dd3ab834c7c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R5046b6121afd4088"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rabfaedd31cb64952"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R2b59ec15417f4146"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71f7a03c310f4897"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8ade021bdd34bf9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9648,7 +9698,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fa66f0023ba45ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d2de7b73dcf4834"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Refine journey map and footer
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R47a7aa279be44f0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Ra285abd31123409f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rf13838d95dd94a59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R55b80483501b4af8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R13ccbd733d274525"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rfb48c492052f4390"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rd62f055ce8ed4efc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Rbcb6ded8cc804028"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7315,7 +7315,7 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H77" t="str">
-        <x:v>Agentic AI</x:v>
+        <x:v>Embedded Models</x:v>
       </x:c>
       <x:c r="I77" t="str">
         <x:v>A local-first city-management game where players govern Innovation City with Gemma as an on-device chief of staff for incident triage, guardrails, and scenario stress-testing.</x:v>
@@ -7344,10 +7344,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rddee6565c28d489e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rb7fffae7adad4e63"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rce319407610248f0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R5d0ef9dfd39b4ace"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rd3e82a7fec9144ca"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rc54ffb4d38ac4894"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rf2087b1b0ceb4224"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R470feb4815b94eaf"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -8911,12 +8911,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rabfaedd31cb64952"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R2b59ec15417f4146"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rd92cf0cbb7d54c00"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R115843bb66dd4914"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8ade021bdd34bf9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re614aaef33704e48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9698,7 +9698,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d2de7b73dcf4834"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60cd9b5ecd9c446b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10181,6 +10181,17 @@
       </x:c>
       <x:c r="C52" s="33" t="str"/>
     </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>Embedded Models</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>Agentic AI</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>On-device and local model builds</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:C1"/>

</xml_diff>

<commit_message>
Update journey presentation and hackathon data
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R13ccbd733d274525"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rfb48c492052f4390"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rd62f055ce8ed4efc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Rbcb6ded8cc804028"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R5aef58ba89bb4aca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Ra3575d456bb843c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R08eb509b6f0a4f78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R0898d9c4d973478f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2690,16 +2690,6 @@
   <x:si>
     <x:t xml:space="preserve">https://www.instagram.com/p/B2EYk1KluTZ/
 https://www.instagram.com/p/B2JzcFglegx/</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://www.facebook.com/sayyid.iskandar/posts/pfbid0rxHXvZDwNWumGZdXFgUnJiu12SW3FUwyTueeejHBw8a6tAGgyLHUFeZB8n2iNhmfl
-https://www.facebook.com/sayyid.iskandar/posts/pfbid02YSrksK2xzkZUh8uifPrWYxk6VHt7aMVfcef6vc1AXoauq9GTCUGQQpLDQpbUUAUyl
-https://www.facebook.com/share/p/1DSDV99DjY/
-https://www.facebook.com/share/p/1HXZcYB6ew/
-https://www.facebook.com/share/p/1BiUy52YeW/</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://www.facebook.com/sayyid.iskandar/posts/pfbid02HTKxyfqPKL2uR4n9zFFxAzkXbE7FYNjkzzuQpqRpEgeCBzYnqvfko88xe9nDPD4kl</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">https://www.facebook.com/sayyid.iskandar/posts/pfbid02T7TywvEM5ypGy8vVEQyJVS1ZAzQns7CGz483NQGZX5CKf1DaCw8P6VbcAFdQmqczl</x:t>
@@ -7344,10 +7334,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rd3e82a7fec9144ca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rc54ffb4d38ac4894"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rf2087b1b0ceb4224"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R470feb4815b94eaf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R1e41c0594f8946b7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R51f60dac8f4e4a9f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Ra9252408299f4de2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R6dc63dc5b4d044c4"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -8911,12 +8901,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rd92cf0cbb7d54c00"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R115843bb66dd4914"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rca8e5dbfdd8e41b7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R2a1ff2ed907d4b5d"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re614aaef33704e48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b535532c5694e97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9207,8 +9197,18 @@
       <x:c r="C32" s="10" t="s">
         <x:v>891</x:v>
       </x:c>
-      <x:c r="D32" s="10" t="s">
-        <x:v>892</x:v>
+      <x:c r="D32" s="10" t="str">
+        <x:v>https://www.facebook.com/sayyid.iskandar/posts/pfbid0rxHXvZDwNWumGZdXFgUnJiu12SW3FUwyTueeejHBw8a6tAGgyLHUFeZB8n2iNhmfl
+https://www.facebook.com/sayyid.iskandar/posts/pfbid02YSrksK2xzkZUh8uifPrWYxk6VHt7aMVfcef6vc1AXoauq9GTCUGQQpLDQpbUUAUyl
+https://www.facebook.com/share/p/1DSDV99DjY/
+https://www.facebook.com/share/p/1HXZcYB6ew/
+https://www.facebook.com/share/p/1BiUy52YeW/
+https://www.facebook.com/share/p/1QzGUmEibA/
+https://www.facebook.com/share/p/19Thtkbyvq/
+https://www.facebook.com/share/p/182DHiJcRd/
+https://www.facebook.com/share/p/1DeRrdfhWH/
+https://www.facebook.com/share/p/1HYmuCRfuP/
+https://www.facebook.com/share/p/1JmrdD1Bb7/</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
@@ -9217,8 +9217,9 @@
       </x:c>
       <x:c r="B33" s="10"/>
       <x:c r="C33" s="10"/>
-      <x:c r="D33" s="10" t="s">
-        <x:v>893</x:v>
+      <x:c r="D33" s="10" t="str">
+        <x:v>https://www.facebook.com/sayyid.iskandar/posts/pfbid02HTKxyfqPKL2uR4n9zFFxAzkXbE7FYNjkzzuQpqRpEgeCBzYnqvfko88xe9nDPD4kl
+https://www.facebook.com/share/v/1BNrHxPRHz/</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
@@ -9228,7 +9229,7 @@
       <x:c r="B34" s="10"/>
       <x:c r="C34" s="10"/>
       <x:c r="D34" s="10" t="s">
-        <x:v>894</x:v>
+        <x:v>892</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
@@ -9237,17 +9238,17 @@
       </x:c>
       <x:c r="B35" s="10"/>
       <x:c r="C35" s="10" t="s">
-        <x:v>895</x:v>
+        <x:v>893</x:v>
       </x:c>
       <x:c r="D35" s="10"/>
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
       <x:c r="A36" s="8" t="s">
-        <x:v>896</x:v>
+        <x:v>894</x:v>
       </x:c>
       <x:c r="B36" s="10"/>
       <x:c r="C36" s="10" t="s">
-        <x:v>897</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="D36" s="10"/>
     </x:row>
@@ -9257,7 +9258,7 @@
       </x:c>
       <x:c r="B37" s="10"/>
       <x:c r="C37" s="10" t="s">
-        <x:v>898</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="D37" s="10"/>
     </x:row>
@@ -9267,7 +9268,7 @@
       </x:c>
       <x:c r="B38" s="10"/>
       <x:c r="C38" s="10" t="s">
-        <x:v>899</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="D38" s="10"/>
     </x:row>
@@ -9277,33 +9278,33 @@
       </x:c>
       <x:c r="B39" s="10"/>
       <x:c r="C39" s="10" t="s">
-        <x:v>900</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="D39" s="10"/>
     </x:row>
     <x:row r="40" ht="28" customHeight="1">
       <x:c r="A40" s="8" t="s">
-        <x:v>901</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="B40" s="10"/>
       <x:c r="C40" s="10" t="s">
-        <x:v>902</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="D40" s="10"/>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="8" t="s">
-        <x:v>903</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="B41" s="10"/>
       <x:c r="C41" s="10" t="s">
-        <x:v>904</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="D41" s="10"/>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
       <x:c r="A42" s="8" t="s">
-        <x:v>905</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="B42" s="10"/>
       <x:c r="C42" s="10"/>
@@ -9315,61 +9316,61 @@
       </x:c>
       <x:c r="B43" s="10"/>
       <x:c r="C43" s="10" t="s">
-        <x:v>906</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="D43" s="10"/>
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="8" t="s">
+        <x:v>905</x:v>
+      </x:c>
+      <x:c r="B44" s="10" t="s">
+        <x:v>906</x:v>
+      </x:c>
+      <x:c r="C44" s="10" t="s">
         <x:v>907</x:v>
-      </x:c>
-      <x:c r="B44" s="10" t="s">
-        <x:v>908</x:v>
-      </x:c>
-      <x:c r="C44" s="10" t="s">
-        <x:v>909</x:v>
       </x:c>
       <x:c r="D44" s="10"/>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
       <x:c r="A45" s="8" t="s">
-        <x:v>910</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="B45" s="10"/>
       <x:c r="C45" s="10" t="s">
-        <x:v>911</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="D45" s="10"/>
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
       <x:c r="A46" s="8" t="s">
-        <x:v>912</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="B46" s="10"/>
       <x:c r="C46" s="10" t="s">
-        <x:v>913</x:v>
+        <x:v>911</x:v>
       </x:c>
       <x:c r="D46" s="10"/>
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
       <x:c r="A47" s="8" t="s">
-        <x:v>914</x:v>
+        <x:v>912</x:v>
       </x:c>
       <x:c r="B47" s="10"/>
       <x:c r="C47" s="10" t="s">
-        <x:v>915</x:v>
+        <x:v>913</x:v>
       </x:c>
       <x:c r="D47" s="10"/>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
       <x:c r="A48" s="8" t="s">
+        <x:v>914</x:v>
+      </x:c>
+      <x:c r="B48" s="10" t="s">
+        <x:v>915</x:v>
+      </x:c>
+      <x:c r="C48" s="10" t="s">
         <x:v>916</x:v>
-      </x:c>
-      <x:c r="B48" s="10" t="s">
-        <x:v>917</x:v>
-      </x:c>
-      <x:c r="C48" s="10" t="s">
-        <x:v>918</x:v>
       </x:c>
       <x:c r="D48" s="10"/>
     </x:row>
@@ -9379,7 +9380,7 @@
       </x:c>
       <x:c r="B49" s="10"/>
       <x:c r="C49" s="10" t="s">
-        <x:v>919</x:v>
+        <x:v>917</x:v>
       </x:c>
       <x:c r="D49" s="10"/>
     </x:row>
@@ -9389,13 +9390,13 @@
       </x:c>
       <x:c r="B50" s="10"/>
       <x:c r="C50" s="10" t="s">
-        <x:v>920</x:v>
+        <x:v>918</x:v>
       </x:c>
       <x:c r="D50" s="10"/>
     </x:row>
     <x:row r="51" ht="28" customHeight="1">
       <x:c r="A51" s="8" t="s">
-        <x:v>921</x:v>
+        <x:v>919</x:v>
       </x:c>
       <x:c r="B51" s="10"/>
       <x:c r="C51" s="10"/>
@@ -9411,29 +9412,29 @@
     </x:row>
     <x:row r="53" ht="28" customHeight="1">
       <x:c r="A53" s="8" t="s">
-        <x:v>922</x:v>
+        <x:v>920</x:v>
       </x:c>
       <x:c r="B53" s="10"/>
       <x:c r="C53" s="10" t="s">
-        <x:v>923</x:v>
+        <x:v>921</x:v>
       </x:c>
       <x:c r="D53" s="10"/>
     </x:row>
     <x:row r="54" ht="28" customHeight="1">
       <x:c r="A54" s="8" t="s">
+        <x:v>922</x:v>
+      </x:c>
+      <x:c r="B54" s="10" t="s">
+        <x:v>923</x:v>
+      </x:c>
+      <x:c r="C54" s="10" t="s">
         <x:v>924</x:v>
-      </x:c>
-      <x:c r="B54" s="10" t="s">
-        <x:v>925</x:v>
-      </x:c>
-      <x:c r="C54" s="10" t="s">
-        <x:v>926</x:v>
       </x:c>
       <x:c r="D54" s="10"/>
     </x:row>
     <x:row r="55" ht="28" customHeight="1">
       <x:c r="A55" s="8" t="s">
-        <x:v>927</x:v>
+        <x:v>925</x:v>
       </x:c>
       <x:c r="B55" s="10"/>
       <x:c r="C55" s="10"/>
@@ -9441,49 +9442,49 @@
     </x:row>
     <x:row r="56" ht="28" customHeight="1">
       <x:c r="A56" s="8" t="s">
-        <x:v>928</x:v>
+        <x:v>926</x:v>
       </x:c>
       <x:c r="B56" s="10"/>
       <x:c r="C56" s="10" t="s">
-        <x:v>929</x:v>
+        <x:v>927</x:v>
       </x:c>
       <x:c r="D56" s="10"/>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
       <x:c r="A57" s="8" t="s">
-        <x:v>930</x:v>
+        <x:v>928</x:v>
       </x:c>
       <x:c r="B57" s="10"/>
       <x:c r="C57" s="10" t="s">
-        <x:v>929</x:v>
+        <x:v>927</x:v>
       </x:c>
       <x:c r="D57" s="10"/>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
       <x:c r="A58" s="8" t="s">
+        <x:v>929</x:v>
+      </x:c>
+      <x:c r="B58" s="10" t="s">
+        <x:v>930</x:v>
+      </x:c>
+      <x:c r="C58" s="10" t="s">
         <x:v>931</x:v>
-      </x:c>
-      <x:c r="B58" s="10" t="s">
-        <x:v>932</x:v>
-      </x:c>
-      <x:c r="C58" s="10" t="s">
-        <x:v>933</x:v>
       </x:c>
       <x:c r="D58" s="10"/>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
       <x:c r="A59" s="8" t="s">
-        <x:v>934</x:v>
+        <x:v>932</x:v>
       </x:c>
       <x:c r="B59" s="10"/>
       <x:c r="C59" s="10" t="s">
-        <x:v>935</x:v>
+        <x:v>933</x:v>
       </x:c>
       <x:c r="D59" s="10"/>
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
       <x:c r="A60" s="8" t="s">
-        <x:v>936</x:v>
+        <x:v>934</x:v>
       </x:c>
       <x:c r="B60" s="10"/>
       <x:c r="C60" s="10"/>
@@ -9491,13 +9492,13 @@
     </x:row>
     <x:row r="61" ht="28" customHeight="1">
       <x:c r="A61" s="8" t="s">
+        <x:v>935</x:v>
+      </x:c>
+      <x:c r="B61" s="10" t="s">
+        <x:v>936</x:v>
+      </x:c>
+      <x:c r="C61" s="10" t="s">
         <x:v>937</x:v>
-      </x:c>
-      <x:c r="B61" s="10" t="s">
-        <x:v>938</x:v>
-      </x:c>
-      <x:c r="C61" s="10" t="s">
-        <x:v>939</x:v>
       </x:c>
       <x:c r="D61" s="10"/>
     </x:row>
@@ -9507,7 +9508,7 @@
       </x:c>
       <x:c r="B62" s="10"/>
       <x:c r="C62" s="10" t="s">
-        <x:v>940</x:v>
+        <x:v>938</x:v>
       </x:c>
       <x:c r="D62" s="10"/>
     </x:row>
@@ -9516,50 +9517,50 @@
         <x:v>815</x:v>
       </x:c>
       <x:c r="B63" s="10" t="s">
-        <x:v>941</x:v>
+        <x:v>939</x:v>
       </x:c>
       <x:c r="C63" s="10" t="s">
-        <x:v>942</x:v>
+        <x:v>940</x:v>
       </x:c>
       <x:c r="D63" s="10"/>
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
       <x:c r="A64" s="8" t="s">
-        <x:v>943</x:v>
+        <x:v>941</x:v>
       </x:c>
       <x:c r="B64" s="10" t="s">
-        <x:v>941</x:v>
+        <x:v>939</x:v>
       </x:c>
       <x:c r="C64" s="10" t="s">
-        <x:v>944</x:v>
+        <x:v>942</x:v>
       </x:c>
       <x:c r="D64" s="10"/>
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
       <x:c r="A65" s="8" t="s">
-        <x:v>945</x:v>
+        <x:v>943</x:v>
       </x:c>
       <x:c r="B65" s="10" t="s">
-        <x:v>941</x:v>
+        <x:v>939</x:v>
       </x:c>
       <x:c r="C65" s="10" t="s">
-        <x:v>946</x:v>
+        <x:v>944</x:v>
       </x:c>
       <x:c r="D65" s="10"/>
     </x:row>
     <x:row r="66" ht="28" customHeight="1">
       <x:c r="A66" s="8" t="s">
-        <x:v>947</x:v>
+        <x:v>945</x:v>
       </x:c>
       <x:c r="B66" s="10"/>
       <x:c r="C66" s="10" t="s">
-        <x:v>948</x:v>
+        <x:v>946</x:v>
       </x:c>
       <x:c r="D66" s="10"/>
     </x:row>
     <x:row r="67" ht="28" customHeight="1">
       <x:c r="A67" s="8" t="s">
-        <x:v>949</x:v>
+        <x:v>947</x:v>
       </x:c>
       <x:c r="B67" s="10"/>
       <x:c r="C67" s="10"/>
@@ -9570,34 +9571,34 @@
         <x:v>743</x:v>
       </x:c>
       <x:c r="B68" s="10" t="s">
-        <x:v>950</x:v>
+        <x:v>948</x:v>
       </x:c>
       <x:c r="C68" s="10" t="s">
-        <x:v>951</x:v>
+        <x:v>949</x:v>
       </x:c>
       <x:c r="D68" s="10"/>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
       <x:c r="A69" s="8" t="s">
+        <x:v>950</x:v>
+      </x:c>
+      <x:c r="B69" s="10" t="s">
+        <x:v>951</x:v>
+      </x:c>
+      <x:c r="C69" s="10" t="s">
         <x:v>952</x:v>
-      </x:c>
-      <x:c r="B69" s="10" t="s">
-        <x:v>953</x:v>
-      </x:c>
-      <x:c r="C69" s="10" t="s">
-        <x:v>954</x:v>
       </x:c>
       <x:c r="D69" s="10"/>
     </x:row>
     <x:row r="70" ht="28" customHeight="1">
       <x:c r="A70" s="8" t="s">
+        <x:v>953</x:v>
+      </x:c>
+      <x:c r="B70" s="10" t="s">
+        <x:v>954</x:v>
+      </x:c>
+      <x:c r="C70" s="10" t="s">
         <x:v>955</x:v>
-      </x:c>
-      <x:c r="B70" s="10" t="s">
-        <x:v>956</x:v>
-      </x:c>
-      <x:c r="C70" s="10" t="s">
-        <x:v>957</x:v>
       </x:c>
       <x:c r="D70" s="10"/>
     </x:row>
@@ -9606,22 +9607,22 @@
         <x:v>592</x:v>
       </x:c>
       <x:c r="B71" s="10" t="s">
-        <x:v>958</x:v>
+        <x:v>956</x:v>
       </x:c>
       <x:c r="C71" s="10" t="s">
-        <x:v>959</x:v>
+        <x:v>957</x:v>
       </x:c>
       <x:c r="D71" s="10"/>
     </x:row>
     <x:row r="72" ht="28" customHeight="1">
       <x:c r="A72" s="8" t="s">
+        <x:v>958</x:v>
+      </x:c>
+      <x:c r="B72" s="10" t="s">
+        <x:v>959</x:v>
+      </x:c>
+      <x:c r="C72" s="10" t="s">
         <x:v>960</x:v>
-      </x:c>
-      <x:c r="B72" s="10" t="s">
-        <x:v>961</x:v>
-      </x:c>
-      <x:c r="C72" s="10" t="s">
-        <x:v>962</x:v>
       </x:c>
       <x:c r="D72" s="10"/>
     </x:row>
@@ -9631,62 +9632,62 @@
       </x:c>
       <x:c r="B73" s="10"/>
       <x:c r="C73" s="10" t="s">
-        <x:v>963</x:v>
+        <x:v>961</x:v>
       </x:c>
       <x:c r="D73" s="10"/>
     </x:row>
     <x:row r="74" ht="28" customHeight="1">
       <x:c r="A74" s="8" t="s">
+        <x:v>962</x:v>
+      </x:c>
+      <x:c r="B74" s="10" t="s">
+        <x:v>963</x:v>
+      </x:c>
+      <x:c r="C74" s="10" t="s">
         <x:v>964</x:v>
-      </x:c>
-      <x:c r="B74" s="10" t="s">
-        <x:v>965</x:v>
-      </x:c>
-      <x:c r="C74" s="10" t="s">
-        <x:v>966</x:v>
       </x:c>
       <x:c r="D74" s="10"/>
     </x:row>
     <x:row r="75" ht="28" customHeight="1">
       <x:c r="A75" s="8" t="s">
+        <x:v>965</x:v>
+      </x:c>
+      <x:c r="B75" s="10" t="s">
+        <x:v>966</x:v>
+      </x:c>
+      <x:c r="C75" s="10" t="s">
         <x:v>967</x:v>
-      </x:c>
-      <x:c r="B75" s="10" t="s">
-        <x:v>968</x:v>
-      </x:c>
-      <x:c r="C75" s="10" t="s">
-        <x:v>969</x:v>
       </x:c>
       <x:c r="D75" s="10"/>
     </x:row>
     <x:row r="76" ht="28" customHeight="1">
       <x:c r="A76" s="8" t="s">
+        <x:v>968</x:v>
+      </x:c>
+      <x:c r="B76" s="10" t="s">
+        <x:v>969</x:v>
+      </x:c>
+      <x:c r="C76" s="10" t="s">
         <x:v>970</x:v>
-      </x:c>
-      <x:c r="B76" s="10" t="s">
-        <x:v>971</x:v>
-      </x:c>
-      <x:c r="C76" s="10" t="s">
-        <x:v>972</x:v>
       </x:c>
       <x:c r="D76" s="10"/>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
       <x:c r="A77" s="8" t="s">
-        <x:v>973</x:v>
+        <x:v>971</x:v>
       </x:c>
       <x:c r="B77" s="10"/>
       <x:c r="C77" s="10" t="s">
-        <x:v>974</x:v>
+        <x:v>972</x:v>
       </x:c>
       <x:c r="D77" s="10"/>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
       <x:c r="A78" s="8" t="s">
-        <x:v>975</x:v>
+        <x:v>973</x:v>
       </x:c>
       <x:c r="B78" s="10" t="s">
-        <x:v>976</x:v>
+        <x:v>974</x:v>
       </x:c>
       <x:c r="C78" s="10"/>
       <x:c r="D78" s="10"/>
@@ -9698,7 +9699,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60cd9b5ecd9c446b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49d9dc0e01324f10"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Sync hackathon Instagram posts
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rdae371fc9853439f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R32dc23d35cb246d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Red74c1c8c23c4880"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R88a09f4364824f65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R09ff87e5489142d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rf791c9765f454829"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rab145a6692b240b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R2256eac61144484b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7368,10 +7368,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R8d8b8ae947ec4e43"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R3e84531356534562"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R1912646e4e834534"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R15b2ef1c5c85484c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rcce5d34c3f9641de"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rf3366dbc6f514fdb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R7759f302a5e2463c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R65193c3d7467496f"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -8949,12 +8949,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R8f490b2be0c942ed"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R4b7b8507b5f84684"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R7a8778c8e54f4990"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R456ae07b45e14c70"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b5bcdcbf09d4b87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b8b3a7920794003"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9756,7 +9756,9 @@
       <x:c r="B77" s="10" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7490764342309855232/</x:v>
       </x:c>
-      <x:c r="C77" s="10"/>
+      <x:c r="C77" s="10" t="str">
+        <x:v>https://www.instagram.com/p/Db50W3FHYuM/</x:v>
+      </x:c>
       <x:c r="D77" s="10"/>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
@@ -9766,41 +9768,76 @@
       <x:c r="B78" s="10" t="str">
         <x:v>https://www.linkedin.com/posts/sayyidkhan92_hackathon-singapore-ai-activity-7495846654978478080-lNv7?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAABzB85UB8iZMlY6hoj9K3g7MfcRKsCZOvqw</x:v>
       </x:c>
-      <x:c r="C78" s="10"/>
+      <x:c r="C78" s="10" t="str">
+        <x:v>https://www.instagram.com/p/DcOZh7DHVFE/</x:v>
+      </x:c>
       <x:c r="D78" s="10"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" t="str">
-        <x:v>#077</x:v>
-      </x:c>
-      <x:c r="B79" t="str">
-        <x:v>https://www.linkedin.com/posts/sayyidkhan92_hackathon-singapore-ai-activity-7498397192852779008-CO54?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAABzB85UB8iZMlY6hoj9K3g7MfcRKsCZOvqw</x:v>
-      </x:c>
-      <x:c r="C79"/>
+        <x:v>#076</x:v>
+      </x:c>
+      <x:c r="B79"/>
+      <x:c r="C79" t="str">
+        <x:v>https://www.instagram.com/reel/Dcgk8b_RELZ/
+https://www.instagram.com/p/DcghI50ncWn/</x:v>
+      </x:c>
       <x:c r="D79"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" t="str">
+        <x:v>#077</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>https://www.linkedin.com/posts/sayyidkhan92_hackathon-singapore-ai-activity-7498397192852779008-CO54?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAABzB85UB8iZMlY6hoj9K3g7MfcRKsCZOvqw</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>https://www.instagram.com/p/Dcxszh0nbh6/</x:v>
+      </x:c>
+      <x:c r="D80"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>#078</x:v>
+      </x:c>
+      <x:c r="B81"/>
+      <x:c r="C81" t="str">
+        <x:v>https://www.instagram.com/p/Dc5Nkd-nU1B/</x:v>
+      </x:c>
+      <x:c r="D81"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
         <x:v>#079</x:v>
       </x:c>
-      <x:c r="B80" t="str">
+      <x:c r="B82" t="str">
         <x:v>https://www.linkedin.com/posts/sayyidkhan92_hackathon-ai-sarawak-activity-7502243111935307776-MYar?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAABzB85UB8iZMlY6hoj9K3g7MfcRKsCZOvqw
 https://www.linkedin.com/posts/sohwanwei_saiyan-saiyanbuilders-singaporesarawak-ugcPost-7502187273908596737-4La9?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAABzB85UB8iZMlY6hoj9K3g7MfcRKsCZOvqw</x:v>
       </x:c>
-      <x:c r="C80" t="str">
+      <x:c r="C82" t="str">
         <x:v>https://www.instagram.com/p/Dc5QhzbmxIE/?utm_source=ig_web_copy_link&amp;stkn=MzRlODBiNWFlZA==
 https://www.instagram.com/reel/Dc5TWF8TcSt/?utm_source=ig_web_copy_link&amp;stkn=MzRlODBiNWFlZA==
 https://www.instagram.com/reel/Dc5ksn1xwM_/?utm_source=ig_web_copy_link&amp;stkn=MzRlODBiNWFlZA==
 https://www.instagram.com/p/Dc7j6K9k9Rn/?utm_source=ig_web_copy_link&amp;stkn=MzRlODBiNWFlZA==
-https://www.instagram.com/p/DdEa6eRHUJq/?utm_source=ig_web_copy_link&amp;stkn=MzRlODBiNWFlZA==</x:v>
-      </x:c>
-      <x:c r="D80"/>
-    </x:row>
-    <x:row r="81">
-      <x:c r="A81"/>
-      <x:c r="B81"/>
-      <x:c r="C81"/>
-      <x:c r="D81"/>
+https://www.instagram.com/p/DdEa6eRHUJq/?utm_source=ig_web_copy_link&amp;stkn=MzRlODBiNWFlZA==
+https://www.instagram.com/reel/Dc8Mz_8z325/
+https://www.instagram.com/reel/Dc5UiWhxVXR/</x:v>
+      </x:c>
+      <x:c r="D82"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="str">
+        <x:v>#080</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>https://www.linkedin.com/posts/sayyidkhan92_hackathon-astra-ai-activity-7506342725504557056-ifQj?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAABzB85UB8iZMlY6hoj9K3g7MfcRKsCZOvqw
+https://www.linkedin.com/posts/sayyidkhan92_hackathon-astra-ai-activity-7504873783019597824-0MLK?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAABzB85UB8iZMlY6hoj9K3g7MfcRKsCZOvqw</x:v>
+      </x:c>
+      <x:c r="C83" t="str">
+        <x:v>https://www.instagram.com/reel/DdOiYzlxNim/?utm_source=ig_web_copy_link&amp;stkn=MzRlODBiNWFlZA==
+https://www.instagram.com/p/DdY81t8k9G8/?utm_source=ig_web_copy_link&amp;stkn=MzRlODBiNWFlZA==</x:v>
+      </x:c>
+      <x:c r="D83"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -9809,7 +9846,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f903c8d7d0c4d12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdab94895611c405e"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Update hackathon records through 81
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R09ff87e5489142d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rf791c9765f454829"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rab145a6692b240b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R2256eac61144484b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rf0b0ffea8a0c45ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R35079b4ce08146ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R5241c6ec257c4f20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Ra032356c03114601"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2002,9 +2002,6 @@
     <x:t xml:space="preserve">Bruce Chua</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">#069, #071</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://www.linkedin.com/in/bruce-chua-28832a414/</x:t>
   </x:si>
   <x:si>
@@ -2032,21 +2029,12 @@
     <x:t xml:space="preserve">Clarence Chan</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">#054, #055, #056, #062, #066, #068</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://www.linkedin.com/in/clarencechanxy/</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">P021</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">clement</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">#050, #051</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://www.linkedin.com/in/clement-lork/</x:t>
   </x:si>
   <x:si>
@@ -2543,9 +2531,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">P077</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">#001, #002, #003, #004, #005, #006, #007, #008, #009, #010, #011, #012, #013, #014, #015, #017, #018, #019, #020, #021, #022, #023, #024, #025, #026, #027, #028, #029, #030, #031, #032, #033, #034, #035, #036, #037, #038, #039, #041, #042, #043, #044, #045, #046, #047, #048, #049, #050, #051, #052, #053, #054, #055, #056, #057, #058, #059, #060, #061, #062, #063, #064, #065, #066, #067, #068, #069, #070, #071, #072, #073</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">https://www.linkedin.com/in/sayyidkhan92/</x:t>
@@ -7297,12 +7282,14 @@
         <x:v>A bilingual digital visitor experience for Long Taa, a Sebup longhouse village in Sarawak, with trip planning and a Kimi-powered visitor assistant.</x:v>
       </x:c>
       <x:c r="J80" t="str">
-        <x:v>sayyid</x:v>
+        <x:v>sayyid, Hao Ming, Bruce</x:v>
       </x:c>
       <x:c r="K80" t="str">
         <x:v>Long Taa Borneo Eco Stay</x:v>
       </x:c>
-      <x:c r="L80"/>
+      <x:c r="L80" t="str">
+        <x:v>Longtaa Borneo</x:v>
+      </x:c>
       <x:c r="M80" t="str">
         <x:v>Malaysia</x:v>
       </x:c>
@@ -7345,7 +7332,7 @@
         <x:v>Explore a real 3D city with a flying crow, then generate AI travel scenes of yourself at your destination.</x:v>
       </x:c>
       <x:c r="J81" t="str">
-        <x:v>sayyid</x:v>
+        <x:v>sayyid, Clement Lork</x:v>
       </x:c>
       <x:c r="K81" t="str">
         <x:v>Itachi's Crow</x:v>
@@ -7366,12 +7353,60 @@
         <x:v>https://luma.com/fdzbrq5b?tk=QX3FM2</x:v>
       </x:c>
     </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="n">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>Anti-Drug Jam 2026</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>SCOGA, Esports Academy, National Council Against Drug Abuse (NCADA)</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>19 Sep 2026</x:v>
+      </x:c>
+      <x:c r="E82" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F82" t="str">
+        <x:v>Days</x:v>
+      </x:c>
+      <x:c r="G82"/>
+      <x:c r="H82" t="str">
+        <x:v>Anti Drugs</x:v>
+      </x:c>
+      <x:c r="I82" t="str">
+        <x:v>An illustrated storybook adventure where you sketch solutions to help Bob navigate peer pressure and find his safe way home.</x:v>
+      </x:c>
+      <x:c r="J82" t="str">
+        <x:v>sayyid</x:v>
+      </x:c>
+      <x:c r="K82" t="str">
+        <x:v>The Next 8 Seconds: Draw Your Way Home</x:v>
+      </x:c>
+      <x:c r="L82" t="str">
+        <x:v>SCOGA × NCADA</x:v>
+      </x:c>
+      <x:c r="M82" t="str">
+        <x:v>Singapore</x:v>
+      </x:c>
+      <x:c r="N82" t="str">
+        <x:v>*SCAPE Ground Theatre</x:v>
+      </x:c>
+      <x:c r="O82" t="str">
+        <x:v>https://github.com/sayyidkhan/8-mins</x:v>
+      </x:c>
+      <x:c r="P82" t="str">
+        <x:v>https://scoga-anti-drug-jam-2026.ai.studio/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rcce5d34c3f9641de"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rf3366dbc6f514fdb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R7759f302a5e2463c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R65193c3d7467496f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R3f95f9f804ab4a8f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R8b0af0f376454f2b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R880109457c7f4454"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Rb55064a177d348af"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7694,25 +7729,25 @@
       <x:c r="B21" s="7" t="s">
         <x:v>662</x:v>
       </x:c>
-      <x:c r="C21" s="7" t="s">
+      <x:c r="C21" s="7" t="str">
+        <x:v>#069, #071, #079</x:v>
+      </x:c>
+      <x:c r="D21" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E21" s="10" t="s">
         <x:v>663</x:v>
-      </x:c>
-      <x:c r="D21" s="9">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E21" s="10" t="s">
-        <x:v>664</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
       <x:c r="A22" s="8" t="s">
+        <x:v>664</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="s">
         <x:v>665</x:v>
       </x:c>
-      <x:c r="B22" s="7" t="s">
+      <x:c r="C22" s="7" t="s">
         <x:v>666</x:v>
-      </x:c>
-      <x:c r="C22" s="7" t="s">
-        <x:v>667</x:v>
       </x:c>
       <x:c r="D22" s="9">
         <x:v>1</x:v>
@@ -7721,13 +7756,13 @@
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
       <x:c r="A23" s="8" t="s">
+        <x:v>667</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="s">
         <x:v>668</x:v>
       </x:c>
-      <x:c r="B23" s="7" t="s">
+      <x:c r="C23" s="7" t="s">
         <x:v>669</x:v>
-      </x:c>
-      <x:c r="C23" s="7" t="s">
-        <x:v>670</x:v>
       </x:c>
       <x:c r="D23" s="9">
         <x:v>1</x:v>
@@ -7736,44 +7771,44 @@
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
       <x:c r="A24" s="8" t="s">
+        <x:v>670</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="s">
         <x:v>671</x:v>
       </x:c>
-      <x:c r="B24" s="7" t="s">
+      <x:c r="C24" s="7" t="str">
+        <x:v>#054, #055, #056, #062, #066, #068, #075</x:v>
+      </x:c>
+      <x:c r="D24" s="9" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E24" s="10" t="s">
         <x:v>672</x:v>
-      </x:c>
-      <x:c r="C24" s="7" t="s">
-        <x:v>673</x:v>
-      </x:c>
-      <x:c r="D24" s="9">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E24" s="10" t="s">
-        <x:v>674</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
       <x:c r="A25" s="8" t="s">
-        <x:v>675</x:v>
-      </x:c>
-      <x:c r="B25" s="7" t="s">
-        <x:v>676</x:v>
-      </x:c>
-      <x:c r="C25" s="7" t="s">
-        <x:v>677</x:v>
-      </x:c>
-      <x:c r="D25" s="9">
-        <x:v>2</x:v>
+        <x:v>673</x:v>
+      </x:c>
+      <x:c r="B25" s="7" t="str">
+        <x:v>Clement Lork</x:v>
+      </x:c>
+      <x:c r="C25" s="7" t="str">
+        <x:v>#050, #051, #080</x:v>
+      </x:c>
+      <x:c r="D25" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E25" s="10" t="s">
-        <x:v>678</x:v>
+        <x:v>674</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="8" t="s">
-        <x:v>679</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="B26" s="7" t="s">
-        <x:v>680</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="C26" s="7" t="s">
         <x:v>615</x:v>
@@ -7785,13 +7820,13 @@
     </x:row>
     <x:row r="27" ht="28" customHeight="1">
       <x:c r="A27" s="8" t="s">
-        <x:v>681</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="B27" s="7" t="s">
-        <x:v>682</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="C27" s="7" t="s">
-        <x:v>683</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="D27" s="9">
         <x:v>1</x:v>
@@ -7800,13 +7835,13 @@
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
       <x:c r="A28" s="8" t="s">
-        <x:v>684</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="B28" s="7" t="s">
-        <x:v>685</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="C28" s="7" t="s">
-        <x:v>686</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="D28" s="9">
         <x:v>2</x:v>
@@ -7815,13 +7850,13 @@
     </x:row>
     <x:row r="29" ht="28" customHeight="1">
       <x:c r="A29" s="8" t="s">
-        <x:v>687</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="B29" s="7" t="s">
-        <x:v>688</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="C29" s="7" t="s">
-        <x:v>689</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="D29" s="9">
         <x:v>4</x:v>
@@ -7830,13 +7865,13 @@
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
       <x:c r="A30" s="8" t="s">
-        <x:v>690</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="B30" s="7" t="s">
-        <x:v>691</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="C30" s="7" t="s">
-        <x:v>683</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="D30" s="9">
         <x:v>1</x:v>
@@ -7845,10 +7880,10 @@
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="8" t="s">
-        <x:v>692</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="B31" s="7" t="s">
-        <x:v>693</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="C31" s="7" t="s">
         <x:v>628</x:v>
@@ -7857,35 +7892,35 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E31" s="10" t="s">
-        <x:v>694</x:v>
+        <x:v>690</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="28" customHeight="1">
       <x:c r="A32" s="8" t="s">
-        <x:v>695</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="B32" s="7" t="s">
-        <x:v>696</x:v>
+        <x:v>692</x:v>
       </x:c>
       <x:c r="C32" s="7" t="s">
-        <x:v>697</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="D32" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E32" s="10" t="s">
-        <x:v>698</x:v>
+        <x:v>694</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="8" t="s">
-        <x:v>699</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="B33" s="7" t="s">
-        <x:v>700</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="C33" s="7" t="s">
-        <x:v>667</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="D33" s="9">
         <x:v>1</x:v>
@@ -7894,13 +7929,13 @@
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
       <x:c r="A34" s="8" t="s">
-        <x:v>701</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="B34" s="7" t="s">
-        <x:v>702</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="C34" s="7" t="s">
-        <x:v>703</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="D34" s="9">
         <x:v>1</x:v>
@@ -7909,47 +7944,47 @@
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
       <x:c r="A35" s="8" t="s">
-        <x:v>704</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="B35" s="7" t="s">
-        <x:v>705</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="C35" s="7" t="s">
-        <x:v>706</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="D35" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E35" s="10" t="s">
-        <x:v>707</x:v>
+        <x:v>703</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
       <x:c r="A36" s="8" t="s">
-        <x:v>708</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="B36" s="7" t="s">
-        <x:v>709</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="C36" s="7" t="s">
-        <x:v>710</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="D36" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E36" s="10" t="s">
-        <x:v>711</x:v>
+        <x:v>707</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
       <x:c r="A37" s="8" t="s">
-        <x:v>712</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="B37" s="7" t="s">
-        <x:v>713</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="C37" s="7" t="s">
-        <x:v>714</x:v>
+        <x:v>710</x:v>
       </x:c>
       <x:c r="D37" s="9">
         <x:v>1</x:v>
@@ -7958,10 +7993,10 @@
     </x:row>
     <x:row r="38" ht="28" customHeight="1">
       <x:c r="A38" s="8" t="s">
-        <x:v>715</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="B38" s="7" t="s">
-        <x:v>716</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="C38" s="7" t="s">
         <x:v>649</x:v>
@@ -7973,13 +8008,13 @@
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
       <x:c r="A39" s="8" t="s">
-        <x:v>717</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="B39" s="7" t="s">
-        <x:v>718</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="C39" s="7" t="s">
-        <x:v>719</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="D39" s="9">
         <x:v>3</x:v>
@@ -7988,47 +8023,47 @@
     </x:row>
     <x:row r="40" ht="28" customHeight="1">
       <x:c r="A40" s="8" t="s">
-        <x:v>720</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="B40" s="7" t="s">
-        <x:v>721</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="C40" s="7" t="s">
-        <x:v>722</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="D40" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E40" s="10" t="s">
-        <x:v>723</x:v>
+        <x:v>719</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="8" t="s">
-        <x:v>724</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="B41" s="7" t="s">
-        <x:v>725</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="C41" s="7" t="s">
+        <x:v>718</x:v>
+      </x:c>
+      <x:c r="D41" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E41" s="10" t="s">
         <x:v>722</x:v>
-      </x:c>
-      <x:c r="D41" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E41" s="10" t="s">
-        <x:v>726</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
       <x:c r="A42" s="8" t="s">
-        <x:v>727</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="B42" s="7" t="s">
-        <x:v>728</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="C42" s="7" t="s">
-        <x:v>729</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="D42" s="9">
         <x:v>1</x:v>
@@ -8037,45 +8072,45 @@
     </x:row>
     <x:row r="43" ht="28" customHeight="1">
       <x:c r="A43" s="8" t="s">
-        <x:v>730</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="B43" s="7" t="s">
-        <x:v>731</x:v>
-      </x:c>
-      <x:c r="C43" s="7" t="s">
-        <x:v>645</x:v>
-      </x:c>
-      <x:c r="D43" s="9">
-        <x:v>1</x:v>
+        <x:v>727</x:v>
+      </x:c>
+      <x:c r="C43" s="7" t="str">
+        <x:v>#069, #079</x:v>
+      </x:c>
+      <x:c r="D43" s="9" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E43" s="10"/>
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="8" t="s">
-        <x:v>732</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="B44" s="7" t="s">
-        <x:v>733</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="C44" s="7" t="s">
-        <x:v>686</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="D44" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E44" s="10" t="s">
-        <x:v>734</x:v>
+        <x:v>730</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
       <x:c r="A45" s="8" t="s">
-        <x:v>735</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="B45" s="7" t="s">
-        <x:v>736</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="C45" s="7" t="s">
-        <x:v>737</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="D45" s="9">
         <x:v>1</x:v>
@@ -8084,13 +8119,13 @@
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
       <x:c r="A46" s="8" t="s">
-        <x:v>738</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="B46" s="7" t="s">
-        <x:v>739</x:v>
+        <x:v>735</x:v>
       </x:c>
       <x:c r="C46" s="7" t="s">
-        <x:v>703</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="D46" s="9">
         <x:v>1</x:v>
@@ -8099,10 +8134,10 @@
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
       <x:c r="A47" s="8" t="s">
-        <x:v>740</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="B47" s="7" t="s">
-        <x:v>741</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="C47" s="7" t="s">
         <x:v>611</x:v>
@@ -8111,35 +8146,35 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E47" s="10" t="s">
-        <x:v>742</x:v>
+        <x:v>738</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
       <x:c r="A48" s="8" t="s">
-        <x:v>743</x:v>
+        <x:v>739</x:v>
       </x:c>
       <x:c r="B48" s="7" t="s">
-        <x:v>744</x:v>
+        <x:v>740</x:v>
       </x:c>
       <x:c r="C48" s="7" t="s">
-        <x:v>745</x:v>
+        <x:v>741</x:v>
       </x:c>
       <x:c r="D48" s="9">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="10" t="s">
-        <x:v>746</x:v>
+        <x:v>742</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
       <x:c r="A49" s="8" t="s">
-        <x:v>747</x:v>
+        <x:v>743</x:v>
       </x:c>
       <x:c r="B49" s="7" t="s">
-        <x:v>748</x:v>
+        <x:v>744</x:v>
       </x:c>
       <x:c r="C49" s="7" t="s">
-        <x:v>749</x:v>
+        <x:v>745</x:v>
       </x:c>
       <x:c r="D49" s="9">
         <x:v>1</x:v>
@@ -8148,13 +8183,13 @@
     </x:row>
     <x:row r="50" ht="28" customHeight="1">
       <x:c r="A50" s="8" t="s">
-        <x:v>750</x:v>
+        <x:v>746</x:v>
       </x:c>
       <x:c r="B50" s="7" t="s">
-        <x:v>751</x:v>
+        <x:v>747</x:v>
       </x:c>
       <x:c r="C50" s="7" t="s">
-        <x:v>714</x:v>
+        <x:v>710</x:v>
       </x:c>
       <x:c r="D50" s="9">
         <x:v>1</x:v>
@@ -8163,64 +8198,64 @@
     </x:row>
     <x:row r="51" ht="28" customHeight="1">
       <x:c r="A51" s="8" t="s">
-        <x:v>752</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="B51" s="7" t="s">
-        <x:v>753</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="C51" s="7" t="s">
-        <x:v>754</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="D51" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E51" s="10" t="s">
-        <x:v>755</x:v>
+        <x:v>751</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="28" customHeight="1">
       <x:c r="A52" s="8" t="s">
-        <x:v>756</x:v>
+        <x:v>752</x:v>
       </x:c>
       <x:c r="B52" s="7" t="s">
-        <x:v>757</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="C52" s="7" t="s">
-        <x:v>758</x:v>
+        <x:v>754</x:v>
       </x:c>
       <x:c r="D52" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E52" s="10" t="s">
-        <x:v>759</x:v>
+        <x:v>755</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="28" customHeight="1">
       <x:c r="A53" s="8" t="s">
-        <x:v>760</x:v>
+        <x:v>756</x:v>
       </x:c>
       <x:c r="B53" s="7" t="s">
-        <x:v>761</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="C53" s="7" t="s">
-        <x:v>762</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="D53" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E53" s="10" t="s">
-        <x:v>763</x:v>
+        <x:v>759</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="28" customHeight="1">
       <x:c r="A54" s="8" t="s">
-        <x:v>764</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="B54" s="7" t="s">
-        <x:v>765</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="C54" s="7" t="s">
-        <x:v>766</x:v>
+        <x:v>762</x:v>
       </x:c>
       <x:c r="D54" s="9">
         <x:v>1</x:v>
@@ -8229,78 +8264,78 @@
     </x:row>
     <x:row r="55" ht="28" customHeight="1">
       <x:c r="A55" s="8" t="s">
-        <x:v>767</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="B55" s="7" t="s">
-        <x:v>768</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="C55" s="7" t="s">
-        <x:v>769</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="D55" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E55" s="10" t="s">
-        <x:v>770</x:v>
+        <x:v>766</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="28" customHeight="1">
       <x:c r="A56" s="8" t="s">
-        <x:v>771</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="B56" s="7" t="s">
-        <x:v>772</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="C56" s="7" t="s">
-        <x:v>773</x:v>
+        <x:v>769</x:v>
       </x:c>
       <x:c r="D56" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E56" s="10" t="s">
-        <x:v>774</x:v>
+        <x:v>770</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
       <x:c r="A57" s="8" t="s">
-        <x:v>775</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="B57" s="7" t="s">
-        <x:v>776</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="C57" s="7" t="s">
-        <x:v>777</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="D57" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E57" s="10" t="s">
-        <x:v>778</x:v>
+        <x:v>774</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
       <x:c r="A58" s="8" t="s">
-        <x:v>779</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="B58" s="7" t="s">
-        <x:v>780</x:v>
+        <x:v>776</x:v>
       </x:c>
       <x:c r="C58" s="7" t="s">
-        <x:v>781</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="D58" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E58" s="10" t="s">
-        <x:v>782</x:v>
+        <x:v>778</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
       <x:c r="A59" s="8" t="s">
-        <x:v>783</x:v>
+        <x:v>779</x:v>
       </x:c>
       <x:c r="B59" s="7" t="s">
-        <x:v>784</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="C59" s="7" t="s">
         <x:v>615</x:v>
@@ -8312,10 +8347,10 @@
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
       <x:c r="A60" s="8" t="s">
-        <x:v>785</x:v>
+        <x:v>781</x:v>
       </x:c>
       <x:c r="B60" s="7" t="s">
-        <x:v>786</x:v>
+        <x:v>782</x:v>
       </x:c>
       <x:c r="C60" s="7" t="s">
         <x:v>652</x:v>
@@ -8327,10 +8362,10 @@
     </x:row>
     <x:row r="61" ht="28" customHeight="1">
       <x:c r="A61" s="8" t="s">
-        <x:v>787</x:v>
+        <x:v>783</x:v>
       </x:c>
       <x:c r="B61" s="7" t="s">
-        <x:v>788</x:v>
+        <x:v>784</x:v>
       </x:c>
       <x:c r="C61" s="7" t="s">
         <x:v>636</x:v>
@@ -8342,10 +8377,10 @@
     </x:row>
     <x:row r="62" ht="28" customHeight="1">
       <x:c r="A62" s="8" t="s">
-        <x:v>789</x:v>
+        <x:v>785</x:v>
       </x:c>
       <x:c r="B62" s="7" t="s">
-        <x:v>790</x:v>
+        <x:v>786</x:v>
       </x:c>
       <x:c r="C62" s="7" t="s">
         <x:v>642</x:v>
@@ -8354,15 +8389,15 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E62" s="10" t="s">
-        <x:v>791</x:v>
+        <x:v>787</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="28" customHeight="1">
       <x:c r="A63" s="8" t="s">
-        <x:v>792</x:v>
+        <x:v>788</x:v>
       </x:c>
       <x:c r="B63" s="7" t="s">
-        <x:v>793</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="C63" s="7" t="s">
         <x:v>636</x:v>
@@ -8374,13 +8409,13 @@
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
       <x:c r="A64" s="8" t="s">
-        <x:v>794</x:v>
+        <x:v>790</x:v>
       </x:c>
       <x:c r="B64" s="7" t="s">
-        <x:v>795</x:v>
+        <x:v>791</x:v>
       </x:c>
       <x:c r="C64" s="7" t="s">
-        <x:v>796</x:v>
+        <x:v>792</x:v>
       </x:c>
       <x:c r="D64" s="9">
         <x:v>1</x:v>
@@ -8389,13 +8424,13 @@
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
       <x:c r="A65" s="8" t="s">
-        <x:v>797</x:v>
+        <x:v>793</x:v>
       </x:c>
       <x:c r="B65" s="7" t="s">
-        <x:v>798</x:v>
+        <x:v>794</x:v>
       </x:c>
       <x:c r="C65" s="7" t="s">
-        <x:v>799</x:v>
+        <x:v>795</x:v>
       </x:c>
       <x:c r="D65" s="9">
         <x:v>1</x:v>
@@ -8404,10 +8439,10 @@
     </x:row>
     <x:row r="66" ht="28" customHeight="1">
       <x:c r="A66" s="8" t="s">
-        <x:v>800</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="B66" s="7" t="s">
-        <x:v>801</x:v>
+        <x:v>797</x:v>
       </x:c>
       <x:c r="C66" s="7" t="s">
         <x:v>625</x:v>
@@ -8419,27 +8454,27 @@
     </x:row>
     <x:row r="67" ht="28" customHeight="1">
       <x:c r="A67" s="8" t="s">
-        <x:v>802</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="B67" s="7" t="s">
-        <x:v>803</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="C67" s="7" t="s">
-        <x:v>781</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="D67" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E67" s="10" t="s">
-        <x:v>804</x:v>
+        <x:v>800</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="28" customHeight="1">
       <x:c r="A68" s="8" t="s">
-        <x:v>805</x:v>
+        <x:v>801</x:v>
       </x:c>
       <x:c r="B68" s="7" t="s">
-        <x:v>806</x:v>
+        <x:v>802</x:v>
       </x:c>
       <x:c r="C68" s="7" t="s">
         <x:v>652</x:v>
@@ -8448,15 +8483,15 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E68" s="10" t="s">
-        <x:v>807</x:v>
+        <x:v>803</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
       <x:c r="A69" s="8" t="s">
-        <x:v>808</x:v>
+        <x:v>804</x:v>
       </x:c>
       <x:c r="B69" s="7" t="s">
-        <x:v>809</x:v>
+        <x:v>805</x:v>
       </x:c>
       <x:c r="C69" s="7" t="s">
         <x:v>632</x:v>
@@ -8468,10 +8503,10 @@
     </x:row>
     <x:row r="70" ht="28" customHeight="1">
       <x:c r="A70" s="8" t="s">
-        <x:v>810</x:v>
+        <x:v>806</x:v>
       </x:c>
       <x:c r="B70" s="7" t="s">
-        <x:v>811</x:v>
+        <x:v>807</x:v>
       </x:c>
       <x:c r="C70" s="7" t="s">
         <x:v>660</x:v>
@@ -8483,13 +8518,13 @@
     </x:row>
     <x:row r="71" ht="28" customHeight="1">
       <x:c r="A71" s="8" t="s">
-        <x:v>812</x:v>
+        <x:v>808</x:v>
       </x:c>
       <x:c r="B71" s="7" t="s">
-        <x:v>813</x:v>
+        <x:v>809</x:v>
       </x:c>
       <x:c r="C71" s="7" t="s">
-        <x:v>814</x:v>
+        <x:v>810</x:v>
       </x:c>
       <x:c r="D71" s="9">
         <x:v>1</x:v>
@@ -8498,44 +8533,44 @@
     </x:row>
     <x:row r="72" ht="28" customHeight="1">
       <x:c r="A72" s="8" t="s">
-        <x:v>815</x:v>
+        <x:v>811</x:v>
       </x:c>
       <x:c r="B72" s="7" t="s">
-        <x:v>816</x:v>
+        <x:v>812</x:v>
       </x:c>
       <x:c r="C72" s="7" t="s">
-        <x:v>817</x:v>
+        <x:v>813</x:v>
       </x:c>
       <x:c r="D72" s="9">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E72" s="10" t="s">
-        <x:v>818</x:v>
+        <x:v>814</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="28" customHeight="1">
       <x:c r="A73" s="8" t="s">
-        <x:v>819</x:v>
+        <x:v>815</x:v>
       </x:c>
       <x:c r="B73" s="7" t="s">
-        <x:v>820</x:v>
+        <x:v>816</x:v>
       </x:c>
       <x:c r="C73" s="7" t="s">
-        <x:v>821</x:v>
+        <x:v>817</x:v>
       </x:c>
       <x:c r="D73" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E73" s="10" t="s">
-        <x:v>822</x:v>
+        <x:v>818</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="28" customHeight="1">
       <x:c r="A74" s="8" t="s">
-        <x:v>823</x:v>
+        <x:v>819</x:v>
       </x:c>
       <x:c r="B74" s="7" t="s">
-        <x:v>824</x:v>
+        <x:v>820</x:v>
       </x:c>
       <x:c r="C74" s="7" t="s">
         <x:v>618</x:v>
@@ -8544,18 +8579,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E74" s="10" t="s">
-        <x:v>825</x:v>
+        <x:v>821</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="28" customHeight="1">
       <x:c r="A75" s="8" t="s">
-        <x:v>826</x:v>
+        <x:v>822</x:v>
       </x:c>
       <x:c r="B75" s="7" t="s">
-        <x:v>827</x:v>
+        <x:v>823</x:v>
       </x:c>
       <x:c r="C75" s="7" t="s">
-        <x:v>737</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="D75" s="9">
         <x:v>1</x:v>
@@ -8564,44 +8599,44 @@
     </x:row>
     <x:row r="76" ht="28" customHeight="1">
       <x:c r="A76" s="8" t="s">
-        <x:v>828</x:v>
+        <x:v>824</x:v>
       </x:c>
       <x:c r="B76" s="7" t="s">
-        <x:v>829</x:v>
+        <x:v>825</x:v>
       </x:c>
       <x:c r="C76" s="7" t="s">
-        <x:v>706</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="D76" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E76" s="10" t="s">
-        <x:v>830</x:v>
+        <x:v>826</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
       <x:c r="A77" s="8" t="s">
-        <x:v>831</x:v>
+        <x:v>827</x:v>
       </x:c>
       <x:c r="B77" s="7" t="s">
-        <x:v>832</x:v>
+        <x:v>828</x:v>
       </x:c>
       <x:c r="C77" s="7" t="s">
-        <x:v>814</x:v>
+        <x:v>810</x:v>
       </x:c>
       <x:c r="D77" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E77" s="10" t="s">
-        <x:v>833</x:v>
+        <x:v>829</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
       <x:c r="A78" s="8" t="s">
-        <x:v>834</x:v>
+        <x:v>830</x:v>
       </x:c>
       <x:c r="B78" s="7" t="s">
-        <x:v>835</x:v>
+        <x:v>831</x:v>
       </x:c>
       <x:c r="C78" s="7" t="s">
         <x:v>607</x:v>
@@ -8610,18 +8645,18 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E78" s="10" t="s">
-        <x:v>836</x:v>
+        <x:v>832</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="28" customHeight="1">
       <x:c r="A79" s="8" t="s">
-        <x:v>837</x:v>
+        <x:v>833</x:v>
       </x:c>
       <x:c r="B79" s="7" t="s">
-        <x:v>838</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="C79" s="7" t="s">
-        <x:v>706</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="D79" s="9">
         <x:v>1</x:v>
@@ -8630,61 +8665,61 @@
     </x:row>
     <x:row r="80" ht="28" customHeight="1">
       <x:c r="A80" s="8" t="s">
-        <x:v>839</x:v>
+        <x:v>835</x:v>
       </x:c>
       <x:c r="B80" s="7" t="s">
-        <x:v>840</x:v>
+        <x:v>836</x:v>
       </x:c>
       <x:c r="C80" s="7" t="s">
-        <x:v>841</x:v>
+        <x:v>837</x:v>
       </x:c>
       <x:c r="D80" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E80" s="10" t="s">
-        <x:v>842</x:v>
+        <x:v>838</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="28" customHeight="1">
       <x:c r="A81" s="8" t="s">
-        <x:v>843</x:v>
+        <x:v>839</x:v>
       </x:c>
       <x:c r="B81" s="7" t="s">
         <x:v>172</x:v>
       </x:c>
-      <x:c r="C81" s="7" t="s">
-        <x:v>844</x:v>
-      </x:c>
-      <x:c r="D81" s="9">
-        <x:v>71</x:v>
+      <x:c r="C81" s="7" t="str">
+        <x:v>#001, #002, #003, #004, #005, #006, #007, #008, #009, #010, #011, #012, #013, #014, #015, #017, #018, #019, #020, #021, #022, #023, #024, #025, #026, #027, #028, #029, #030, #031, #032, #033, #034, #035, #036, #037, #038, #039, #041, #042, #043, #044, #045, #046, #047, #048, #049, #050, #051, #052, #053, #054, #055, #056, #057, #058, #059, #060, #061, #062, #063, #064, #065, #066, #067, #068, #069, #070, #071, #072, #073, #074, #075, #076, #077, #078, #079, #080, #081</x:v>
+      </x:c>
+      <x:c r="D81" s="9" t="n">
+        <x:v>79</x:v>
       </x:c>
       <x:c r="E81" s="10" t="s">
-        <x:v>845</x:v>
+        <x:v>840</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="28" customHeight="1">
       <x:c r="A82" s="8" t="s">
-        <x:v>846</x:v>
+        <x:v>841</x:v>
       </x:c>
       <x:c r="B82" s="7" t="s">
-        <x:v>847</x:v>
+        <x:v>842</x:v>
       </x:c>
       <x:c r="C82" s="7" t="s">
-        <x:v>848</x:v>
+        <x:v>843</x:v>
       </x:c>
       <x:c r="D82" s="9">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E82" s="10" t="s">
-        <x:v>849</x:v>
+        <x:v>844</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="28" customHeight="1">
       <x:c r="A83" s="8" t="s">
-        <x:v>850</x:v>
+        <x:v>845</x:v>
       </x:c>
       <x:c r="B83" s="7" t="s">
-        <x:v>851</x:v>
+        <x:v>846</x:v>
       </x:c>
       <x:c r="C83" s="7" t="s">
         <x:v>625</x:v>
@@ -8696,13 +8731,13 @@
     </x:row>
     <x:row r="84" ht="28" customHeight="1">
       <x:c r="A84" s="8" t="s">
-        <x:v>852</x:v>
+        <x:v>847</x:v>
       </x:c>
       <x:c r="B84" s="7" t="s">
-        <x:v>853</x:v>
+        <x:v>848</x:v>
       </x:c>
       <x:c r="C84" s="7" t="s">
-        <x:v>854</x:v>
+        <x:v>849</x:v>
       </x:c>
       <x:c r="D84" s="9">
         <x:v>1</x:v>
@@ -8711,10 +8746,10 @@
     </x:row>
     <x:row r="85" ht="28" customHeight="1">
       <x:c r="A85" s="8" t="s">
-        <x:v>855</x:v>
+        <x:v>850</x:v>
       </x:c>
       <x:c r="B85" s="7" t="s">
-        <x:v>856</x:v>
+        <x:v>851</x:v>
       </x:c>
       <x:c r="C85" s="7" t="s">
         <x:v>628</x:v>
@@ -8723,52 +8758,52 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E85" s="10" t="s">
-        <x:v>857</x:v>
+        <x:v>852</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="28" customHeight="1">
       <x:c r="A86" s="8" t="s">
-        <x:v>858</x:v>
+        <x:v>853</x:v>
       </x:c>
       <x:c r="B86" s="7" t="s">
-        <x:v>859</x:v>
+        <x:v>854</x:v>
       </x:c>
       <x:c r="C86" s="7" t="s">
-        <x:v>860</x:v>
+        <x:v>855</x:v>
       </x:c>
       <x:c r="D86" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E86" s="10" t="s">
-        <x:v>861</x:v>
+        <x:v>856</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="28" customHeight="1">
       <x:c r="A87" s="8" t="s">
-        <x:v>862</x:v>
+        <x:v>857</x:v>
       </x:c>
       <x:c r="B87" s="7" t="s">
-        <x:v>863</x:v>
+        <x:v>858</x:v>
       </x:c>
       <x:c r="C87" s="7" t="s">
-        <x:v>864</x:v>
+        <x:v>859</x:v>
       </x:c>
       <x:c r="D87" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E87" s="10" t="s">
-        <x:v>865</x:v>
+        <x:v>860</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="28" customHeight="1">
       <x:c r="A88" s="8" t="s">
-        <x:v>866</x:v>
+        <x:v>861</x:v>
       </x:c>
       <x:c r="B88" s="7" t="s">
-        <x:v>867</x:v>
+        <x:v>862</x:v>
       </x:c>
       <x:c r="C88" s="7" t="s">
-        <x:v>737</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="D88" s="9">
         <x:v>1</x:v>
@@ -8777,10 +8812,10 @@
     </x:row>
     <x:row r="89" ht="28" customHeight="1">
       <x:c r="A89" s="8" t="s">
-        <x:v>868</x:v>
+        <x:v>863</x:v>
       </x:c>
       <x:c r="B89" s="7" t="s">
-        <x:v>869</x:v>
+        <x:v>864</x:v>
       </x:c>
       <x:c r="C89" s="7" t="s">
         <x:v>649</x:v>
@@ -8792,30 +8827,30 @@
     </x:row>
     <x:row r="90" ht="28" customHeight="1">
       <x:c r="A90" s="8" t="s">
-        <x:v>870</x:v>
+        <x:v>865</x:v>
       </x:c>
       <x:c r="B90" s="7" t="s">
-        <x:v>871</x:v>
+        <x:v>866</x:v>
       </x:c>
       <x:c r="C90" s="7" t="s">
-        <x:v>781</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="D90" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E90" s="10" t="s">
-        <x:v>872</x:v>
+        <x:v>867</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="28" customHeight="1">
       <x:c r="A91" s="8" t="s">
-        <x:v>873</x:v>
+        <x:v>868</x:v>
       </x:c>
       <x:c r="B91" s="7" t="s">
-        <x:v>874</x:v>
+        <x:v>869</x:v>
       </x:c>
       <x:c r="C91" s="7" t="s">
-        <x:v>875</x:v>
+        <x:v>870</x:v>
       </x:c>
       <x:c r="D91" s="9">
         <x:v>1</x:v>
@@ -8824,30 +8859,30 @@
     </x:row>
     <x:row r="92" ht="28" customHeight="1">
       <x:c r="A92" s="8" t="s">
-        <x:v>876</x:v>
+        <x:v>871</x:v>
       </x:c>
       <x:c r="B92" s="7" t="s">
-        <x:v>877</x:v>
+        <x:v>872</x:v>
       </x:c>
       <x:c r="C92" s="7" t="s">
-        <x:v>878</x:v>
+        <x:v>873</x:v>
       </x:c>
       <x:c r="D92" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E92" s="10" t="s">
-        <x:v>879</x:v>
+        <x:v>874</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="28" customHeight="1">
       <x:c r="A93" s="8" t="s">
-        <x:v>880</x:v>
+        <x:v>875</x:v>
       </x:c>
       <x:c r="B93" s="7" t="s">
-        <x:v>881</x:v>
+        <x:v>876</x:v>
       </x:c>
       <x:c r="C93" s="7" t="s">
-        <x:v>814</x:v>
+        <x:v>810</x:v>
       </x:c>
       <x:c r="D93" s="9">
         <x:v>1</x:v>
@@ -8856,30 +8891,30 @@
     </x:row>
     <x:row r="94" ht="28" customHeight="1">
       <x:c r="A94" s="8" t="s">
-        <x:v>882</x:v>
+        <x:v>877</x:v>
       </x:c>
       <x:c r="B94" s="7" t="s">
-        <x:v>883</x:v>
+        <x:v>878</x:v>
       </x:c>
       <x:c r="C94" s="7" t="s">
-        <x:v>706</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="D94" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E94" s="10" t="s">
-        <x:v>884</x:v>
+        <x:v>879</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="28" customHeight="1">
       <x:c r="A95" s="8" t="s">
-        <x:v>885</x:v>
+        <x:v>880</x:v>
       </x:c>
       <x:c r="B95" s="7" t="s">
-        <x:v>886</x:v>
+        <x:v>881</x:v>
       </x:c>
       <x:c r="C95" s="7" t="s">
-        <x:v>703</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="D95" s="9">
         <x:v>1</x:v>
@@ -8888,47 +8923,47 @@
     </x:row>
     <x:row r="96" ht="28" customHeight="1">
       <x:c r="A96" s="8" t="s">
-        <x:v>887</x:v>
+        <x:v>882</x:v>
       </x:c>
       <x:c r="B96" s="7" t="s">
-        <x:v>888</x:v>
+        <x:v>883</x:v>
       </x:c>
       <x:c r="C96" s="7" t="s">
-        <x:v>889</x:v>
+        <x:v>884</x:v>
       </x:c>
       <x:c r="D96" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E96" s="10" t="s">
-        <x:v>890</x:v>
+        <x:v>885</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="28" customHeight="1">
       <x:c r="A97" s="8" t="s">
-        <x:v>891</x:v>
+        <x:v>886</x:v>
       </x:c>
       <x:c r="B97" s="7" t="s">
-        <x:v>892</x:v>
+        <x:v>887</x:v>
       </x:c>
       <x:c r="C97" s="7" t="s">
-        <x:v>854</x:v>
+        <x:v>849</x:v>
       </x:c>
       <x:c r="D97" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E97" s="10" t="s">
-        <x:v>893</x:v>
+        <x:v>888</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="s">
-        <x:v>894</x:v>
+        <x:v>889</x:v>
       </x:c>
       <x:c r="B98" t="s">
-        <x:v>895</x:v>
+        <x:v>890</x:v>
       </x:c>
       <x:c r="C98" t="s">
-        <x:v>896</x:v>
+        <x:v>891</x:v>
       </x:c>
       <x:c r="D98">
         <x:v>1</x:v>
@@ -8949,12 +8984,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R7a8778c8e54f4990"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R456ae07b45e14c70"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R8ed7b0a6feba43dd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R81b3acfc33184b12"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b8b3a7920794003"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22c89ca492d24a21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8969,7 +9004,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>897</x:v>
+        <x:v>892</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -9777,7 +9812,9 @@
       <x:c r="A79" t="str">
         <x:v>#076</x:v>
       </x:c>
-      <x:c r="B79"/>
+      <x:c r="B79" t="str">
+        <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7498397192852779008/</x:v>
+      </x:c>
       <x:c r="C79" t="str">
         <x:v>https://www.instagram.com/reel/Dcgk8b_RELZ/
 https://www.instagram.com/p/DcghI50ncWn/</x:v>
@@ -9788,9 +9825,7 @@
       <x:c r="A80" t="str">
         <x:v>#077</x:v>
       </x:c>
-      <x:c r="B80" t="str">
-        <x:v>https://www.linkedin.com/posts/sayyidkhan92_hackathon-singapore-ai-activity-7498397192852779008-CO54?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAABzB85UB8iZMlY6hoj9K3g7MfcRKsCZOvqw</x:v>
-      </x:c>
+      <x:c r="B80"/>
       <x:c r="C80" t="str">
         <x:v>https://www.instagram.com/p/Dcxszh0nbh6/</x:v>
       </x:c>
@@ -9831,13 +9866,24 @@
       </x:c>
       <x:c r="B83" t="str">
         <x:v>https://www.linkedin.com/posts/sayyidkhan92_hackathon-astra-ai-activity-7506342725504557056-ifQj?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAABzB85UB8iZMlY6hoj9K3g7MfcRKsCZOvqw
-https://www.linkedin.com/posts/sayyidkhan92_hackathon-astra-ai-activity-7504873783019597824-0MLK?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAABzB85UB8iZMlY6hoj9K3g7MfcRKsCZOvqw</x:v>
+https://www.linkedin.com/posts/sayyidkhan92_hackathon-astra-ai-activity-7504873783019597824-0MLK?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAABzB85UB8iZMlY6hoj9K3g7MfcRKsCZOvqw
+https://www.linkedin.com/feed/update/urn:li:activity:7505062754270175232/</x:v>
       </x:c>
       <x:c r="C83" t="str">
         <x:v>https://www.instagram.com/reel/DdOiYzlxNim/?utm_source=ig_web_copy_link&amp;stkn=MzRlODBiNWFlZA==
 https://www.instagram.com/p/DdY81t8k9G8/?utm_source=ig_web_copy_link&amp;stkn=MzRlODBiNWFlZA==</x:v>
       </x:c>
       <x:c r="D83"/>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>#081</x:v>
+      </x:c>
+      <x:c r="B84"/>
+      <x:c r="C84" t="str">
+        <x:v>https://www.instagram.com/p/Dddoi71EyhB/?utm_source=ig_web_copy_link&amp;stkn=MzRlODBiNWFlZA==</x:v>
+      </x:c>
+      <x:c r="D84"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -9846,7 +9892,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdab94895611c405e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R416a1ce653a64a9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9862,27 +9908,27 @@
   <x:sheetData>
     <x:row r="1" ht="34.75" customHeight="1">
       <x:c r="A1" s="20" t="s">
-        <x:v>898</x:v>
+        <x:v>893</x:v>
       </x:c>
       <x:c r="B1" s="20"/>
       <x:c r="C1" s="20"/>
     </x:row>
     <x:row r="2" ht="45.25" customHeight="1">
       <x:c r="A2" s="21" t="s">
-        <x:v>899</x:v>
+        <x:v>894</x:v>
       </x:c>
       <x:c r="B2" s="21"/>
       <x:c r="C2" s="21"/>
     </x:row>
     <x:row r="4" ht="29.25" customHeight="1">
       <x:c r="A4" s="15" t="s">
-        <x:v>900</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="B4" s="15" t="s">
-        <x:v>901</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C4" s="15" t="s">
-        <x:v>902</x:v>
+        <x:v>897</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.75" customHeight="1">
@@ -9890,7 +9936,7 @@
         <x:v>311</x:v>
       </x:c>
       <x:c r="B5" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="C5" s="17"/>
     </x:row>
@@ -9899,7 +9945,7 @@
         <x:v>170</x:v>
       </x:c>
       <x:c r="B6" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C6" s="17"/>
     </x:row>
@@ -9908,7 +9954,7 @@
         <x:v>380</x:v>
       </x:c>
       <x:c r="B7" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C7" s="17"/>
     </x:row>
@@ -9917,7 +9963,7 @@
         <x:v>457</x:v>
       </x:c>
       <x:c r="B8" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C8" s="17"/>
     </x:row>
@@ -9926,7 +9972,7 @@
         <x:v>348</x:v>
       </x:c>
       <x:c r="B9" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C9" s="17"/>
     </x:row>
@@ -9935,27 +9981,27 @@
         <x:v>369</x:v>
       </x:c>
       <x:c r="B10" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C10" s="17" t="s">
-        <x:v>908</x:v>
+        <x:v>903</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.75" customHeight="1">
       <x:c r="A11" s="16" t="s">
-        <x:v>909</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="B11" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C11" s="17"/>
     </x:row>
     <x:row r="12" ht="26.75" customHeight="1">
       <x:c r="A12" s="16" t="s">
-        <x:v>910</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="B12" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C12" s="17"/>
     </x:row>
@@ -9964,25 +10010,25 @@
         <x:v>304</x:v>
       </x:c>
       <x:c r="B13" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C13" s="17"/>
     </x:row>
     <x:row r="14" ht="26.75" customHeight="1">
       <x:c r="A14" s="16" t="s">
-        <x:v>912</x:v>
+        <x:v>907</x:v>
       </x:c>
       <x:c r="B14" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C14" s="17"/>
     </x:row>
     <x:row r="15" ht="26.75" customHeight="1">
       <x:c r="A15" s="16" t="s">
-        <x:v>914</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="B15" s="16" t="s">
-        <x:v>915</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="C15" s="17"/>
     </x:row>
@@ -9991,7 +10037,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B16" s="16" t="s">
-        <x:v>916</x:v>
+        <x:v>911</x:v>
       </x:c>
       <x:c r="C16" s="17"/>
     </x:row>
@@ -10000,7 +10046,7 @@
         <x:v>198</x:v>
       </x:c>
       <x:c r="B17" s="16" t="s">
-        <x:v>916</x:v>
+        <x:v>911</x:v>
       </x:c>
       <x:c r="C17" s="17"/>
     </x:row>
@@ -10009,7 +10055,7 @@
         <x:v>406</x:v>
       </x:c>
       <x:c r="B18" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C18" s="17"/>
     </x:row>
@@ -10018,7 +10064,7 @@
         <x:v>261</x:v>
       </x:c>
       <x:c r="B19" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="C19" s="17"/>
     </x:row>
@@ -10027,16 +10073,16 @@
         <x:v>565</x:v>
       </x:c>
       <x:c r="B20" s="16" t="s">
-        <x:v>915</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="C20" s="17"/>
     </x:row>
     <x:row r="21" ht="26.75" customHeight="1">
       <x:c r="A21" s="16" t="s">
-        <x:v>917</x:v>
+        <x:v>912</x:v>
       </x:c>
       <x:c r="B21" s="16" t="s">
-        <x:v>915</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="C21" s="17"/>
     </x:row>
@@ -10045,25 +10091,25 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B22" s="16" t="s">
-        <x:v>915</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="C22" s="17"/>
     </x:row>
     <x:row r="23" ht="26.75" customHeight="1">
       <x:c r="A23" s="16" t="s">
-        <x:v>918</x:v>
+        <x:v>913</x:v>
       </x:c>
       <x:c r="B23" s="16" t="s">
-        <x:v>919</x:v>
+        <x:v>914</x:v>
       </x:c>
       <x:c r="C23" s="17"/>
     </x:row>
     <x:row r="24" ht="26.75" customHeight="1">
       <x:c r="A24" s="16" t="s">
-        <x:v>920</x:v>
+        <x:v>915</x:v>
       </x:c>
       <x:c r="B24" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
     </x:row>
@@ -10072,7 +10118,7 @@
         <x:v>326</x:v>
       </x:c>
       <x:c r="B25" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
     </x:row>
@@ -10081,7 +10127,7 @@
         <x:v>467</x:v>
       </x:c>
       <x:c r="B26" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
     </x:row>
@@ -10090,18 +10136,18 @@
         <x:v>557</x:v>
       </x:c>
       <x:c r="B27" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C27" s="17" t="s">
-        <x:v>921</x:v>
+        <x:v>916</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="26.75" customHeight="1">
       <x:c r="A28" s="16" t="s">
-        <x:v>922</x:v>
+        <x:v>917</x:v>
       </x:c>
       <x:c r="B28" s="16" t="s">
-        <x:v>919</x:v>
+        <x:v>914</x:v>
       </x:c>
       <x:c r="C28" s="17"/>
     </x:row>
@@ -10110,7 +10156,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B29" s="16" t="s">
-        <x:v>919</x:v>
+        <x:v>914</x:v>
       </x:c>
       <x:c r="C29" s="17"/>
     </x:row>
@@ -10119,7 +10165,7 @@
         <x:v>191</x:v>
       </x:c>
       <x:c r="B30" s="16" t="s">
-        <x:v>919</x:v>
+        <x:v>914</x:v>
       </x:c>
       <x:c r="C30" s="17"/>
     </x:row>
@@ -10128,7 +10174,7 @@
         <x:v>141</x:v>
       </x:c>
       <x:c r="B31" s="16" t="s">
-        <x:v>916</x:v>
+        <x:v>911</x:v>
       </x:c>
       <x:c r="C31" s="17"/>
     </x:row>
@@ -10137,16 +10183,16 @@
         <x:v>552</x:v>
       </x:c>
       <x:c r="B32" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C32" s="17"/>
     </x:row>
     <x:row r="33" ht="26.75" customHeight="1">
       <x:c r="A33" s="16" t="s">
-        <x:v>923</x:v>
+        <x:v>918</x:v>
       </x:c>
       <x:c r="B33" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C33" s="17"/>
     </x:row>
@@ -10155,7 +10201,7 @@
         <x:v>319</x:v>
       </x:c>
       <x:c r="B34" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C34" s="17"/>
     </x:row>
@@ -10164,7 +10210,7 @@
         <x:v>507</x:v>
       </x:c>
       <x:c r="B35" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C35" s="17"/>
     </x:row>
@@ -10173,18 +10219,18 @@
         <x:v>269</x:v>
       </x:c>
       <x:c r="B36" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C36" s="17" t="s">
-        <x:v>908</x:v>
+        <x:v>903</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="26.75" customHeight="1">
       <x:c r="A37" s="16" t="s">
-        <x:v>924</x:v>
+        <x:v>919</x:v>
       </x:c>
       <x:c r="B37" s="16" t="s">
-        <x:v>916</x:v>
+        <x:v>911</x:v>
       </x:c>
       <x:c r="C37" s="17"/>
     </x:row>
@@ -10193,7 +10239,7 @@
         <x:v>177</x:v>
       </x:c>
       <x:c r="B38" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C38" s="17"/>
     </x:row>
@@ -10202,10 +10248,10 @@
         <x:v>240</x:v>
       </x:c>
       <x:c r="B39" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C39" s="17" t="s">
-        <x:v>925</x:v>
+        <x:v>920</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="26.75" customHeight="1">
@@ -10213,25 +10259,25 @@
         <x:v>446</x:v>
       </x:c>
       <x:c r="B40" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C40" s="17"/>
     </x:row>
     <x:row r="41" ht="26.75" customHeight="1">
       <x:c r="A41" s="16" t="s">
-        <x:v>926</x:v>
+        <x:v>921</x:v>
       </x:c>
       <x:c r="B41" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C41" s="17"/>
     </x:row>
     <x:row r="42" ht="26.75" customHeight="1">
       <x:c r="A42" s="16" t="s">
-        <x:v>927</x:v>
+        <x:v>922</x:v>
       </x:c>
       <x:c r="B42" s="16" t="s">
-        <x:v>915</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="C42" s="17"/>
     </x:row>
@@ -10240,10 +10286,10 @@
         <x:v>224</x:v>
       </x:c>
       <x:c r="B43" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C43" s="17" t="s">
-        <x:v>908</x:v>
+        <x:v>903</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="26.75" customHeight="1">
@@ -10251,7 +10297,7 @@
         <x:v>182</x:v>
       </x:c>
       <x:c r="B44" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C44" s="17"/>
     </x:row>
@@ -10260,16 +10306,16 @@
         <x:v>162</x:v>
       </x:c>
       <x:c r="B45" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C45" s="17"/>
     </x:row>
     <x:row r="46" ht="26.75" customHeight="1">
       <x:c r="A46" s="16" t="s">
-        <x:v>928</x:v>
+        <x:v>923</x:v>
       </x:c>
       <x:c r="B46" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C46" s="17"/>
     </x:row>
@@ -10278,19 +10324,19 @@
         <x:v>156</x:v>
       </x:c>
       <x:c r="B47" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C47" s="17"/>
     </x:row>
     <x:row r="48" ht="26.75" customHeight="1">
       <x:c r="A48" s="16" t="s">
-        <x:v>929</x:v>
+        <x:v>924</x:v>
       </x:c>
       <x:c r="B48" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C48" s="17" t="s">
-        <x:v>930</x:v>
+        <x:v>925</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="26.75" customHeight="1">
@@ -10298,7 +10344,7 @@
         <x:v>287</x:v>
       </x:c>
       <x:c r="B49" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C49" s="17"/>
     </x:row>
@@ -10307,16 +10353,16 @@
         <x:v>212</x:v>
       </x:c>
       <x:c r="B50" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C50" s="17"/>
     </x:row>
     <x:row r="51" ht="26.75" customHeight="1">
       <x:c r="A51" s="16" t="s">
-        <x:v>931</x:v>
+        <x:v>926</x:v>
       </x:c>
       <x:c r="B51" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C51" s="17"/>
     </x:row>
@@ -10325,7 +10371,7 @@
         <x:v>232</x:v>
       </x:c>
       <x:c r="B52" s="16" t="s">
-        <x:v>919</x:v>
+        <x:v>914</x:v>
       </x:c>
       <x:c r="C52" s="17"/>
     </x:row>
@@ -10337,7 +10383,7 @@
         <x:v>380</x:v>
       </x:c>
       <x:c r="C53" t="s">
-        <x:v>932</x:v>
+        <x:v>927</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -10345,7 +10391,7 @@
         <x:v>584</x:v>
       </x:c>
       <x:c r="B54" t="s">
-        <x:v>907</x:v>
+        <x:v>902</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -10353,10 +10399,10 @@
         <x:v>591</x:v>
       </x:c>
       <x:c r="B55" t="s">
-        <x:v>905</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C55" t="s">
-        <x:v>933</x:v>
+        <x:v>928</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -10379,6 +10425,17 @@
       </x:c>
       <x:c r="C57" t="str">
         <x:v>Small-business digital experiences and commerce tools</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="str">
+        <x:v>Anti Drugs</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>Smart Nation / Social Good</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>Interactive anti-drug and youth-wellbeing builds</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Correct Speechmatics credit value
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R920a35f0fb9c4f03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R8e5c2df39bce417e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R4b7d632abb7c45b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R371e977b97b2497d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Re0c04f97a6f84395"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R92026aed3fc64568"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rfed7be8c2c3543cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Rc24012c213284865"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1376,9 +1376,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">29/4/2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">2K Speechmatics Credits</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Agentic AI (Voice)</x:t>
@@ -6320,20 +6317,20 @@
       <x:c r="F61" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="G61" t="s">
+      <x:c r="G61" t="str">
+        <x:v>2K USD Speechmatics Credits</x:v>
+      </x:c>
+      <x:c r="H61" t="s">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="H61" t="s">
+      <x:c r="I61" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="I61" t="s">
-        <x:v>457</x:v>
       </x:c>
       <x:c r="J61" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K61" t="s">
-        <x:v>458</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="L61" t="s">
         <x:v>25</x:v>
@@ -6342,13 +6339,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N61" t="s">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="O61" t="s">
         <x:v>459</x:v>
       </x:c>
-      <x:c r="O61" t="s">
+      <x:c r="P61" s="1" t="s">
         <x:v>460</x:v>
-      </x:c>
-      <x:c r="P61" s="1" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -6356,13 +6353,13 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="B62" t="s">
+        <x:v>461</x:v>
+      </x:c>
+      <x:c r="C62" t="s">
         <x:v>462</x:v>
       </x:c>
-      <x:c r="C62" t="s">
+      <x:c r="D62" s="2" t="s">
         <x:v>463</x:v>
-      </x:c>
-      <x:c r="D62" s="2" t="s">
-        <x:v>464</x:v>
       </x:c>
       <x:c r="E62">
         <x:v>1</x:v>
@@ -6371,19 +6368,19 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="G62" t="s">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="H62" t="s">
         <x:v>465</x:v>
       </x:c>
-      <x:c r="H62" t="s">
+      <x:c r="I62" t="s">
         <x:v>466</x:v>
-      </x:c>
-      <x:c r="I62" t="s">
-        <x:v>467</x:v>
       </x:c>
       <x:c r="J62" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K62" t="s">
-        <x:v>468</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="L62" t="s">
         <x:v>25</x:v>
@@ -6398,7 +6395,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="P62" s="1" t="s">
-        <x:v>469</x:v>
+        <x:v>468</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -6406,10 +6403,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="B63" t="s">
+        <x:v>469</x:v>
+      </x:c>
+      <x:c r="C63" t="s">
         <x:v>470</x:v>
-      </x:c>
-      <x:c r="C63" t="s">
-        <x:v>471</x:v>
       </x:c>
       <x:c r="D63" s="5">
         <x:v>46085</x:v>
@@ -6418,7 +6415,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F63" t="s">
-        <x:v>472</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="G63" t="s">
         <x:v>25</x:v>
@@ -6427,13 +6424,13 @@
         <x:v>405</x:v>
       </x:c>
       <x:c r="I63" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="J63" t="s">
         <x:v>407</x:v>
       </x:c>
       <x:c r="K63" t="s">
-        <x:v>474</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="L63" t="s">
         <x:v>25</x:v>
@@ -6442,13 +6439,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N63" t="s">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="O63" t="s">
         <x:v>475</x:v>
       </x:c>
-      <x:c r="O63" t="s">
+      <x:c r="P63" t="s">
         <x:v>476</x:v>
-      </x:c>
-      <x:c r="P63" t="s">
-        <x:v>477</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -6456,10 +6453,10 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="B64" t="s">
-        <x:v>478</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="C64" t="s">
-        <x:v>463</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="D64" s="5">
         <x:v>46116</x:v>
@@ -6474,16 +6471,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H64" t="s">
-        <x:v>466</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="I64" t="s">
-        <x:v>479</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="J64" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K64" t="s">
-        <x:v>480</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="L64" t="s">
         <x:v>25</x:v>
@@ -6495,10 +6492,10 @@
         <x:v>359</x:v>
       </x:c>
       <x:c r="O64" t="s">
+        <x:v>480</x:v>
+      </x:c>
+      <x:c r="P64" t="s">
         <x:v>481</x:v>
-      </x:c>
-      <x:c r="P64" t="s">
-        <x:v>482</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -6506,10 +6503,10 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="B65" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="C65" t="s">
         <x:v>483</x:v>
-      </x:c>
-      <x:c r="C65" t="s">
-        <x:v>484</x:v>
       </x:c>
       <x:c r="D65" s="5">
         <x:v>46270</x:v>
@@ -6524,16 +6521,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H65" t="s">
-        <x:v>466</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="I65" t="s">
+        <x:v>484</x:v>
+      </x:c>
+      <x:c r="J65" t="s">
         <x:v>485</x:v>
       </x:c>
-      <x:c r="J65" t="s">
+      <x:c r="K65" t="s">
         <x:v>486</x:v>
-      </x:c>
-      <x:c r="K65" t="s">
-        <x:v>487</x:v>
       </x:c>
       <x:c r="L65" t="s">
         <x:v>25</x:v>
@@ -6545,10 +6542,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="O65" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="P65" t="s">
         <x:v>488</x:v>
-      </x:c>
-      <x:c r="P65" t="s">
-        <x:v>489</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -6556,13 +6553,13 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B66" t="s">
+        <x:v>489</x:v>
+      </x:c>
+      <x:c r="C66" t="s">
         <x:v>490</x:v>
       </x:c>
-      <x:c r="C66" t="s">
+      <x:c r="D66" s="2" t="s">
         <x:v>491</x:v>
-      </x:c>
-      <x:c r="D66" s="2" t="s">
-        <x:v>492</x:v>
       </x:c>
       <x:c r="E66">
         <x:v>1</x:v>
@@ -6577,13 +6574,13 @@
         <x:v>379</x:v>
       </x:c>
       <x:c r="I66" t="s">
-        <x:v>493</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="J66" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K66" t="s">
-        <x:v>494</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="L66" t="s">
         <x:v>25</x:v>
@@ -6592,13 +6589,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N66" t="s">
+        <x:v>494</x:v>
+      </x:c>
+      <x:c r="O66" t="s">
         <x:v>495</x:v>
       </x:c>
-      <x:c r="O66" t="s">
+      <x:c r="P66" t="s">
         <x:v>496</x:v>
-      </x:c>
-      <x:c r="P66" t="s">
-        <x:v>497</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -6606,13 +6603,13 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B67" t="s">
+        <x:v>497</x:v>
+      </x:c>
+      <x:c r="C67" t="s">
         <x:v>498</x:v>
       </x:c>
-      <x:c r="C67" t="s">
+      <x:c r="D67" s="2" t="s">
         <x:v>499</x:v>
-      </x:c>
-      <x:c r="D67" s="2" t="s">
-        <x:v>500</x:v>
       </x:c>
       <x:c r="E67">
         <x:v>1</x:v>
@@ -6621,7 +6618,7 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="G67" t="s">
-        <x:v>501</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="H67" t="s">
         <x:v>405</x:v>
@@ -6630,10 +6627,10 @@
         <x:v>414</x:v>
       </x:c>
       <x:c r="J67" t="s">
+        <x:v>501</x:v>
+      </x:c>
+      <x:c r="K67" t="s">
         <x:v>502</x:v>
-      </x:c>
-      <x:c r="K67" t="s">
-        <x:v>503</x:v>
       </x:c>
       <x:c r="L67" t="s">
         <x:v>25</x:v>
@@ -6656,13 +6653,13 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B68" t="s">
-        <x:v>504</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="C68" t="s">
         <x:v>266</x:v>
       </x:c>
       <x:c r="D68" s="2" t="s">
-        <x:v>505</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="E68">
         <x:v>3</x:v>
@@ -6674,19 +6671,19 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H68" t="s">
+        <x:v>505</x:v>
+      </x:c>
+      <x:c r="I68" t="s">
         <x:v>506</x:v>
       </x:c>
-      <x:c r="I68" t="s">
+      <x:c r="J68" t="s">
         <x:v>507</x:v>
       </x:c>
-      <x:c r="J68" t="s">
+      <x:c r="K68" t="s">
         <x:v>508</x:v>
       </x:c>
-      <x:c r="K68" t="s">
+      <x:c r="L68" t="s">
         <x:v>509</x:v>
-      </x:c>
-      <x:c r="L68" t="s">
-        <x:v>510</x:v>
       </x:c>
       <x:c r="M68" t="s">
         <x:v>26</x:v>
@@ -6695,7 +6692,7 @@
         <x:v>273</x:v>
       </x:c>
       <x:c r="O68" t="s">
-        <x:v>511</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="P68" t="s">
         <x:v>25</x:v>
@@ -6706,13 +6703,13 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B69" t="s">
+        <x:v>511</x:v>
+      </x:c>
+      <x:c r="C69" t="s">
+        <x:v>498</x:v>
+      </x:c>
+      <x:c r="D69" s="2" t="s">
         <x:v>512</x:v>
-      </x:c>
-      <x:c r="C69" t="s">
-        <x:v>499</x:v>
-      </x:c>
-      <x:c r="D69" s="2" t="s">
-        <x:v>513</x:v>
       </x:c>
       <x:c r="E69">
         <x:v>1</x:v>
@@ -6730,10 +6727,10 @@
         <x:v>414</x:v>
       </x:c>
       <x:c r="J69" t="s">
-        <x:v>502</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="K69" t="s">
-        <x:v>514</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="L69" t="s">
         <x:v>25</x:v>
@@ -6742,13 +6739,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N69" t="s">
+        <x:v>514</x:v>
+      </x:c>
+      <x:c r="O69" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="P69" t="s">
         <x:v>515</x:v>
-      </x:c>
-      <x:c r="O69" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="P69" t="s">
-        <x:v>516</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -6756,13 +6753,13 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="B70" t="s">
+        <x:v>516</x:v>
+      </x:c>
+      <x:c r="C70" t="s">
         <x:v>517</x:v>
       </x:c>
-      <x:c r="C70" t="s">
+      <x:c r="D70" s="2" t="s">
         <x:v>518</x:v>
-      </x:c>
-      <x:c r="D70" s="2" t="s">
-        <x:v>519</x:v>
       </x:c>
       <x:c r="E70">
         <x:v>2</x:v>
@@ -6771,31 +6768,31 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="H70" t="s">
+        <x:v>519</x:v>
+      </x:c>
+      <x:c r="I70" t="s">
         <x:v>520</x:v>
       </x:c>
-      <x:c r="I70" t="s">
+      <x:c r="J70" t="s">
         <x:v>521</x:v>
       </x:c>
-      <x:c r="J70" t="s">
+      <x:c r="K70" t="s">
         <x:v>522</x:v>
       </x:c>
-      <x:c r="K70" t="s">
+      <x:c r="L70" t="s">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="M70" t="s">
         <x:v>523</x:v>
-      </x:c>
-      <x:c r="L70" t="s">
-        <x:v>518</x:v>
-      </x:c>
-      <x:c r="M70" t="s">
-        <x:v>524</x:v>
       </x:c>
       <x:c r="N70" t="s">
         <x:v>359</x:v>
       </x:c>
       <x:c r="O70" t="s">
+        <x:v>524</x:v>
+      </x:c>
+      <x:c r="P70" t="s">
         <x:v>525</x:v>
-      </x:c>
-      <x:c r="P70" t="s">
-        <x:v>526</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -6803,13 +6800,13 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="B71" t="s">
+        <x:v>526</x:v>
+      </x:c>
+      <x:c r="C71" t="s">
         <x:v>527</x:v>
       </x:c>
-      <x:c r="C71" t="s">
+      <x:c r="D71" s="5" t="s">
         <x:v>528</x:v>
-      </x:c>
-      <x:c r="D71" s="5" t="s">
-        <x:v>529</x:v>
       </x:c>
       <x:c r="E71">
         <x:v>1</x:v>
@@ -6821,31 +6818,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H71" t="s">
-        <x:v>520</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="I71" t="s">
-        <x:v>530</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="J71" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K71" t="s">
-        <x:v>531</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="L71" t="s">
-        <x:v>528</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="M71" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N71" t="s">
-        <x:v>495</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="O71" t="s">
+        <x:v>531</x:v>
+      </x:c>
+      <x:c r="P71" t="s">
         <x:v>532</x:v>
-      </x:c>
-      <x:c r="P71" t="s">
-        <x:v>533</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -6853,10 +6850,10 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B72" t="s">
+        <x:v>533</x:v>
+      </x:c>
+      <x:c r="C72" t="s">
         <x:v>534</x:v>
-      </x:c>
-      <x:c r="C72" t="s">
-        <x:v>535</x:v>
       </x:c>
       <x:c r="D72" s="5">
         <x:v>46363</x:v>
@@ -6868,22 +6865,22 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="G72" t="s">
-        <x:v>536</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="H72" t="s">
         <x:v>239</x:v>
       </x:c>
       <x:c r="I72" t="s">
+        <x:v>536</x:v>
+      </x:c>
+      <x:c r="J72" t="s">
         <x:v>537</x:v>
       </x:c>
-      <x:c r="J72" t="s">
+      <x:c r="K72" t="s">
         <x:v>538</x:v>
       </x:c>
-      <x:c r="K72" t="s">
-        <x:v>539</x:v>
-      </x:c>
       <x:c r="L72" t="s">
-        <x:v>535</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="M72" t="s">
         <x:v>26</x:v>
@@ -6895,7 +6892,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="P72" t="s">
-        <x:v>540</x:v>
+        <x:v>539</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -6903,13 +6900,13 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B73" t="s">
+        <x:v>540</x:v>
+      </x:c>
+      <x:c r="C73" t="s">
         <x:v>541</x:v>
       </x:c>
-      <x:c r="C73" t="s">
+      <x:c r="D73" s="2" t="s">
         <x:v>542</x:v>
-      </x:c>
-      <x:c r="D73" s="2" t="s">
-        <x:v>543</x:v>
       </x:c>
       <x:c r="E73">
         <x:v>1</x:v>
@@ -6921,31 +6918,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H73" t="s">
-        <x:v>466</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="I73" t="s">
-        <x:v>544</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="J73" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K73" t="s">
-        <x:v>545</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="L73" t="s">
-        <x:v>542</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="M73" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N73" t="s">
+        <x:v>545</x:v>
+      </x:c>
+      <x:c r="O73" t="s">
         <x:v>546</x:v>
       </x:c>
-      <x:c r="O73" t="s">
+      <x:c r="P73" t="s">
         <x:v>547</x:v>
-      </x:c>
-      <x:c r="P73" t="s">
-        <x:v>548</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -6953,13 +6950,13 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B74" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="C74" t="s">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="D74" s="2" t="s">
         <x:v>549</x:v>
-      </x:c>
-      <x:c r="C74" t="s">
-        <x:v>518</x:v>
-      </x:c>
-      <x:c r="D74" s="2" t="s">
-        <x:v>550</x:v>
       </x:c>
       <x:c r="E74">
         <x:v>10</x:v>
@@ -6971,31 +6968,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H74" t="s">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="I74" t="s">
         <x:v>551</x:v>
-      </x:c>
-      <x:c r="I74" t="s">
-        <x:v>552</x:v>
       </x:c>
       <x:c r="J74" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K74" t="s">
-        <x:v>553</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="L74" t="s">
-        <x:v>518</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="M74" t="s">
-        <x:v>524</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="N74" t="s">
         <x:v>359</x:v>
       </x:c>
       <x:c r="O74" t="s">
-        <x:v>554</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="P74" t="s">
-        <x:v>526</x:v>
+        <x:v>525</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="34">
@@ -7003,10 +7000,10 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B75" s="12" t="s">
+        <x:v>554</x:v>
+      </x:c>
+      <x:c r="C75" s="12" t="s">
         <x:v>555</x:v>
-      </x:c>
-      <x:c r="C75" s="12" t="s">
-        <x:v>556</x:v>
       </x:c>
       <x:c r="D75" s="5">
         <x:v>46150</x:v>
@@ -7021,19 +7018,19 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H75" s="12" t="s">
+        <x:v>555</x:v>
+      </x:c>
+      <x:c r="I75" s="14" t="s">
         <x:v>556</x:v>
-      </x:c>
-      <x:c r="I75" s="14" t="s">
-        <x:v>557</x:v>
       </x:c>
       <x:c r="J75" s="12" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K75" s="12" t="s">
-        <x:v>558</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="L75" s="12" t="s">
-        <x:v>556</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="M75" s="12" t="s">
         <x:v>26</x:v>
@@ -7042,7 +7039,7 @@
         <x:v>273</x:v>
       </x:c>
       <x:c r="O75" t="s">
-        <x:v>559</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="P75" s="12" t="s">
         <x:v>25</x:v>
@@ -7053,13 +7050,13 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B76" s="12" t="s">
+        <x:v>559</x:v>
+      </x:c>
+      <x:c r="C76" s="12" t="s">
         <x:v>560</x:v>
       </x:c>
-      <x:c r="C76" s="12" t="s">
+      <x:c r="D76" s="13" t="s">
         <x:v>561</x:v>
-      </x:c>
-      <x:c r="D76" s="13" t="s">
-        <x:v>562</x:v>
       </x:c>
       <x:c r="E76">
         <x:v>1</x:v>
@@ -7068,34 +7065,34 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="G76" s="12" t="s">
+        <x:v>562</x:v>
+      </x:c>
+      <x:c r="H76" s="12" t="s">
         <x:v>563</x:v>
       </x:c>
-      <x:c r="H76" s="12" t="s">
+      <x:c r="I76" s="12" t="s">
         <x:v>564</x:v>
       </x:c>
-      <x:c r="I76" s="12" t="s">
+      <x:c r="J76" s="12" t="s">
         <x:v>565</x:v>
       </x:c>
-      <x:c r="J76" s="12" t="s">
+      <x:c r="K76" s="12" t="s">
         <x:v>566</x:v>
       </x:c>
-      <x:c r="K76" s="12" t="s">
-        <x:v>567</x:v>
-      </x:c>
       <x:c r="L76" s="12" t="s">
-        <x:v>561</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="M76" s="12" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N76" s="12" t="s">
+        <x:v>567</x:v>
+      </x:c>
+      <x:c r="O76" s="1" t="s">
         <x:v>568</x:v>
       </x:c>
-      <x:c r="O76" s="1" t="s">
+      <x:c r="P76" t="s">
         <x:v>569</x:v>
-      </x:c>
-      <x:c r="P76" t="s">
-        <x:v>570</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -7103,13 +7100,13 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B77" t="s">
+        <x:v>570</x:v>
+      </x:c>
+      <x:c r="C77" t="s">
         <x:v>571</x:v>
       </x:c>
-      <x:c r="C77" t="s">
+      <x:c r="D77" t="s">
         <x:v>572</x:v>
-      </x:c>
-      <x:c r="D77" t="s">
-        <x:v>573</x:v>
       </x:c>
       <x:c r="E77">
         <x:v>1</x:v>
@@ -7121,31 +7118,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H77" t="s">
+        <x:v>573</x:v>
+      </x:c>
+      <x:c r="I77" t="s">
         <x:v>574</x:v>
-      </x:c>
-      <x:c r="I77" t="s">
-        <x:v>575</x:v>
       </x:c>
       <x:c r="J77" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K77" t="s">
+        <x:v>575</x:v>
+      </x:c>
+      <x:c r="L77" t="s">
         <x:v>576</x:v>
-      </x:c>
-      <x:c r="L77" t="s">
-        <x:v>577</x:v>
       </x:c>
       <x:c r="M77" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N77" t="s">
+        <x:v>577</x:v>
+      </x:c>
+      <x:c r="O77" t="s">
         <x:v>578</x:v>
       </x:c>
-      <x:c r="O77" t="s">
+      <x:c r="P77" t="s">
         <x:v>579</x:v>
-      </x:c>
-      <x:c r="P77" t="s">
-        <x:v>580</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -7153,13 +7150,13 @@
         <x:v>77</x:v>
       </x:c>
       <x:c r="B78" t="s">
+        <x:v>580</x:v>
+      </x:c>
+      <x:c r="C78" t="s">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="D78" t="s">
         <x:v>581</x:v>
-      </x:c>
-      <x:c r="C78" t="s">
-        <x:v>518</x:v>
-      </x:c>
-      <x:c r="D78" t="s">
-        <x:v>582</x:v>
       </x:c>
       <x:c r="E78">
         <x:v>1</x:v>
@@ -7171,31 +7168,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H78" t="s">
+        <x:v>582</x:v>
+      </x:c>
+      <x:c r="I78" t="s">
         <x:v>583</x:v>
-      </x:c>
-      <x:c r="I78" t="s">
-        <x:v>584</x:v>
       </x:c>
       <x:c r="J78" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K78" t="s">
-        <x:v>585</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="L78" t="s">
-        <x:v>518</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="M78" t="s">
-        <x:v>524</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="N78" t="s">
         <x:v>359</x:v>
       </x:c>
       <x:c r="O78" t="s">
-        <x:v>586</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="P78" t="s">
-        <x:v>526</x:v>
+        <x:v>525</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -7203,37 +7200,37 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="B79" t="s">
+        <x:v>586</x:v>
+      </x:c>
+      <x:c r="C79" t="s">
         <x:v>587</x:v>
       </x:c>
-      <x:c r="C79" t="s">
+      <x:c r="D79" t="s">
         <x:v>588</x:v>
-      </x:c>
-      <x:c r="D79" t="s">
-        <x:v>589</x:v>
       </x:c>
       <x:c r="E79">
         <x:v>4</x:v>
       </x:c>
       <x:c r="F79" t="s">
-        <x:v>472</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="G79" t="s">
         <x:v>25</x:v>
       </x:c>
       <x:c r="H79" t="s">
+        <x:v>589</x:v>
+      </x:c>
+      <x:c r="I79" t="s">
         <x:v>590</x:v>
       </x:c>
-      <x:c r="I79" t="s">
+      <x:c r="J79" t="s">
         <x:v>591</x:v>
       </x:c>
-      <x:c r="J79" t="s">
+      <x:c r="K79" t="s">
         <x:v>592</x:v>
       </x:c>
-      <x:c r="K79" t="s">
+      <x:c r="L79" t="s">
         <x:v>593</x:v>
-      </x:c>
-      <x:c r="L79" t="s">
-        <x:v>594</x:v>
       </x:c>
       <x:c r="M79" t="s">
         <x:v>26</x:v>
@@ -7242,10 +7239,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="O79" t="s">
+        <x:v>594</x:v>
+      </x:c>
+      <x:c r="P79" t="s">
         <x:v>595</x:v>
-      </x:c>
-      <x:c r="P79" t="s">
-        <x:v>596</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -7398,10 +7395,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Ra38df73f9d8a4298"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R1ba6eb9af55c4083"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rbe6ab65a94c74f27"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R57d8a03b3c984837"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rfd28d8fbb5354157"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R7e5644dcb48e4150"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Ra1dcce16a7064cf6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R7c13ec40084d41f0"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7424,7 +7421,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>597</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -7433,7 +7430,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="19" t="s">
-        <x:v>598</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="B2" s="19"/>
       <x:c r="C2" s="19"/>
@@ -7442,64 +7439,64 @@
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="11" t="s">
+        <x:v>598</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="s">
         <x:v>599</x:v>
       </x:c>
-      <x:c r="B4" s="11" t="s">
+      <x:c r="C4" s="11" t="s">
         <x:v>600</x:v>
       </x:c>
-      <x:c r="C4" s="11" t="s">
+      <x:c r="D4" s="11" t="s">
         <x:v>601</x:v>
       </x:c>
-      <x:c r="D4" s="11" t="s">
+      <x:c r="E4" s="11" t="s">
         <x:v>602</x:v>
-      </x:c>
-      <x:c r="E4" s="11" t="s">
-        <x:v>603</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="8" t="s">
+        <x:v>603</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="s">
         <x:v>604</x:v>
       </x:c>
-      <x:c r="B5" s="7" t="s">
+      <x:c r="C5" s="7" t="s">
         <x:v>605</x:v>
-      </x:c>
-      <x:c r="C5" s="7" t="s">
-        <x:v>606</x:v>
       </x:c>
       <x:c r="D5" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E5" s="10" t="s">
-        <x:v>607</x:v>
+        <x:v>606</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="8" t="s">
+        <x:v>607</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>608</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="s">
+      <x:c r="C6" s="7" t="s">
         <x:v>609</x:v>
       </x:c>
-      <x:c r="C6" s="7" t="s">
+      <x:c r="D6" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="s">
         <x:v>610</x:v>
-      </x:c>
-      <x:c r="D6" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E6" s="10" t="s">
-        <x:v>611</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="8" t="s">
+        <x:v>611</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
         <x:v>612</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="s">
+      <x:c r="C7" s="7" t="s">
         <x:v>613</x:v>
-      </x:c>
-      <x:c r="C7" s="7" t="s">
-        <x:v>614</x:v>
       </x:c>
       <x:c r="D7" s="9">
         <x:v>1</x:v>
@@ -7508,47 +7505,47 @@
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
       <x:c r="A8" s="8" t="s">
+        <x:v>614</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
         <x:v>615</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="s">
+      <x:c r="C8" s="7" t="s">
         <x:v>616</x:v>
       </x:c>
-      <x:c r="C8" s="7" t="s">
+      <x:c r="D8" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="s">
         <x:v>617</x:v>
-      </x:c>
-      <x:c r="D8" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E8" s="10" t="s">
-        <x:v>618</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" s="8" t="s">
+        <x:v>618</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
         <x:v>619</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="s">
+      <x:c r="C9" s="7" t="s">
+        <x:v>609</x:v>
+      </x:c>
+      <x:c r="D9" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="s">
         <x:v>620</x:v>
-      </x:c>
-      <x:c r="C9" s="7" t="s">
-        <x:v>610</x:v>
-      </x:c>
-      <x:c r="D9" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E9" s="10" t="s">
-        <x:v>621</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
       <x:c r="A10" s="8" t="s">
+        <x:v>621</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="s">
         <x:v>622</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="s">
+      <x:c r="C10" s="7" t="s">
         <x:v>623</x:v>
-      </x:c>
-      <x:c r="C10" s="7" t="s">
-        <x:v>624</x:v>
       </x:c>
       <x:c r="D10" s="9">
         <x:v>1</x:v>
@@ -7557,47 +7554,47 @@
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
       <x:c r="A11" s="8" t="s">
+        <x:v>624</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="s">
         <x:v>625</x:v>
       </x:c>
-      <x:c r="B11" s="7" t="s">
+      <x:c r="C11" s="7" t="s">
         <x:v>626</x:v>
       </x:c>
-      <x:c r="C11" s="7" t="s">
+      <x:c r="D11" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="10" t="s">
         <x:v>627</x:v>
-      </x:c>
-      <x:c r="D11" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E11" s="10" t="s">
-        <x:v>628</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
       <x:c r="A12" s="8" t="s">
+        <x:v>628</x:v>
+      </x:c>
+      <x:c r="B12" s="7" t="s">
         <x:v>629</x:v>
       </x:c>
-      <x:c r="B12" s="7" t="s">
+      <x:c r="C12" s="7" t="s">
         <x:v>630</x:v>
       </x:c>
-      <x:c r="C12" s="7" t="s">
+      <x:c r="D12" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="s">
         <x:v>631</x:v>
-      </x:c>
-      <x:c r="D12" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E12" s="10" t="s">
-        <x:v>632</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
       <x:c r="A13" s="8" t="s">
+        <x:v>632</x:v>
+      </x:c>
+      <x:c r="B13" s="7" t="s">
         <x:v>633</x:v>
       </x:c>
-      <x:c r="B13" s="7" t="s">
+      <x:c r="C13" s="7" t="s">
         <x:v>634</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="s">
-        <x:v>635</x:v>
       </x:c>
       <x:c r="D13" s="9">
         <x:v>1</x:v>
@@ -7606,30 +7603,30 @@
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
       <x:c r="A14" s="8" t="s">
+        <x:v>635</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="s">
         <x:v>636</x:v>
       </x:c>
-      <x:c r="B14" s="7" t="s">
+      <x:c r="C14" s="7" t="s">
+        <x:v>634</x:v>
+      </x:c>
+      <x:c r="D14" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="s">
         <x:v>637</x:v>
-      </x:c>
-      <x:c r="C14" s="7" t="s">
-        <x:v>635</x:v>
-      </x:c>
-      <x:c r="D14" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E14" s="10" t="s">
-        <x:v>638</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
       <x:c r="A15" s="8" t="s">
+        <x:v>638</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="s">
         <x:v>639</x:v>
       </x:c>
-      <x:c r="B15" s="7" t="s">
+      <x:c r="C15" s="7" t="s">
         <x:v>640</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="s">
-        <x:v>641</x:v>
       </x:c>
       <x:c r="D15" s="9">
         <x:v>1</x:v>
@@ -7638,30 +7635,30 @@
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
       <x:c r="A16" s="8" t="s">
+        <x:v>641</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="s">
         <x:v>642</x:v>
       </x:c>
-      <x:c r="B16" s="7" t="s">
+      <x:c r="C16" s="7" t="s">
         <x:v>643</x:v>
       </x:c>
-      <x:c r="C16" s="7" t="s">
+      <x:c r="D16" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="s">
         <x:v>644</x:v>
-      </x:c>
-      <x:c r="D16" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E16" s="10" t="s">
-        <x:v>645</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
       <x:c r="A17" s="8" t="s">
+        <x:v>645</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="s">
         <x:v>646</x:v>
       </x:c>
-      <x:c r="B17" s="7" t="s">
+      <x:c r="C17" s="7" t="s">
         <x:v>647</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="s">
-        <x:v>648</x:v>
       </x:c>
       <x:c r="D17" s="9">
         <x:v>1</x:v>
@@ -7670,47 +7667,47 @@
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
       <x:c r="A18" s="8" t="s">
+        <x:v>648</x:v>
+      </x:c>
+      <x:c r="B18" s="7" t="s">
         <x:v>649</x:v>
       </x:c>
-      <x:c r="B18" s="7" t="s">
+      <x:c r="C18" s="7" t="s">
         <x:v>650</x:v>
       </x:c>
-      <x:c r="C18" s="7" t="s">
+      <x:c r="D18" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="s">
         <x:v>651</x:v>
-      </x:c>
-      <x:c r="D18" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E18" s="10" t="s">
-        <x:v>652</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
       <x:c r="A19" s="8" t="s">
+        <x:v>652</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="s">
         <x:v>653</x:v>
       </x:c>
-      <x:c r="B19" s="7" t="s">
+      <x:c r="C19" s="7" t="s">
         <x:v>654</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="s">
-        <x:v>655</x:v>
       </x:c>
       <x:c r="D19" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E19" s="10" t="s">
-        <x:v>656</x:v>
+        <x:v>655</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28" customHeight="1">
       <x:c r="A20" s="8" t="s">
+        <x:v>656</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="s">
         <x:v>657</x:v>
       </x:c>
-      <x:c r="B20" s="7" t="s">
+      <x:c r="C20" s="7" t="s">
         <x:v>658</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>659</x:v>
       </x:c>
       <x:c r="D20" s="9">
         <x:v>1</x:v>
@@ -7719,10 +7716,10 @@
     </x:row>
     <x:row r="21" ht="28" customHeight="1">
       <x:c r="A21" s="8" t="s">
+        <x:v>659</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="s">
         <x:v>660</x:v>
-      </x:c>
-      <x:c r="B21" s="7" t="s">
-        <x:v>661</x:v>
       </x:c>
       <x:c r="C21" s="7" t="str">
         <x:v>#069, #071, #079</x:v>
@@ -7731,18 +7728,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E21" s="10" t="s">
-        <x:v>662</x:v>
+        <x:v>661</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
       <x:c r="A22" s="8" t="s">
+        <x:v>662</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="s">
         <x:v>663</x:v>
       </x:c>
-      <x:c r="B22" s="7" t="s">
+      <x:c r="C22" s="7" t="s">
         <x:v>664</x:v>
-      </x:c>
-      <x:c r="C22" s="7" t="s">
-        <x:v>665</x:v>
       </x:c>
       <x:c r="D22" s="9">
         <x:v>1</x:v>
@@ -7751,13 +7748,13 @@
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
       <x:c r="A23" s="8" t="s">
+        <x:v>665</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="s">
         <x:v>666</x:v>
       </x:c>
-      <x:c r="B23" s="7" t="s">
+      <x:c r="C23" s="7" t="s">
         <x:v>667</x:v>
-      </x:c>
-      <x:c r="C23" s="7" t="s">
-        <x:v>668</x:v>
       </x:c>
       <x:c r="D23" s="9">
         <x:v>1</x:v>
@@ -7766,10 +7763,10 @@
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
       <x:c r="A24" s="8" t="s">
+        <x:v>668</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="s">
         <x:v>669</x:v>
-      </x:c>
-      <x:c r="B24" s="7" t="s">
-        <x:v>670</x:v>
       </x:c>
       <x:c r="C24" s="7" t="str">
         <x:v>#054, #055, #056, #062, #066, #068, #075</x:v>
@@ -7778,12 +7775,12 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E24" s="10" t="s">
-        <x:v>671</x:v>
+        <x:v>670</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
       <x:c r="A25" s="8" t="s">
-        <x:v>672</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
         <x:v>Clement Lork</x:v>
@@ -7795,18 +7792,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E25" s="10" t="s">
-        <x:v>673</x:v>
+        <x:v>672</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="8" t="s">
+        <x:v>673</x:v>
+      </x:c>
+      <x:c r="B26" s="7" t="s">
         <x:v>674</x:v>
       </x:c>
-      <x:c r="B26" s="7" t="s">
-        <x:v>675</x:v>
-      </x:c>
       <x:c r="C26" s="7" t="s">
-        <x:v>614</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="D26" s="9">
         <x:v>1</x:v>
@@ -7815,13 +7812,13 @@
     </x:row>
     <x:row r="27" ht="28" customHeight="1">
       <x:c r="A27" s="8" t="s">
+        <x:v>675</x:v>
+      </x:c>
+      <x:c r="B27" s="7" t="s">
         <x:v>676</x:v>
       </x:c>
-      <x:c r="B27" s="7" t="s">
+      <x:c r="C27" s="7" t="s">
         <x:v>677</x:v>
-      </x:c>
-      <x:c r="C27" s="7" t="s">
-        <x:v>678</x:v>
       </x:c>
       <x:c r="D27" s="9">
         <x:v>1</x:v>
@@ -7830,13 +7827,13 @@
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
       <x:c r="A28" s="8" t="s">
+        <x:v>678</x:v>
+      </x:c>
+      <x:c r="B28" s="7" t="s">
         <x:v>679</x:v>
       </x:c>
-      <x:c r="B28" s="7" t="s">
+      <x:c r="C28" s="7" t="s">
         <x:v>680</x:v>
-      </x:c>
-      <x:c r="C28" s="7" t="s">
-        <x:v>681</x:v>
       </x:c>
       <x:c r="D28" s="9">
         <x:v>2</x:v>
@@ -7845,13 +7842,13 @@
     </x:row>
     <x:row r="29" ht="28" customHeight="1">
       <x:c r="A29" s="8" t="s">
+        <x:v>681</x:v>
+      </x:c>
+      <x:c r="B29" s="7" t="s">
         <x:v>682</x:v>
       </x:c>
-      <x:c r="B29" s="7" t="s">
+      <x:c r="C29" s="7" t="s">
         <x:v>683</x:v>
-      </x:c>
-      <x:c r="C29" s="7" t="s">
-        <x:v>684</x:v>
       </x:c>
       <x:c r="D29" s="9">
         <x:v>4</x:v>
@@ -7860,13 +7857,13 @@
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
       <x:c r="A30" s="8" t="s">
+        <x:v>684</x:v>
+      </x:c>
+      <x:c r="B30" s="7" t="s">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="B30" s="7" t="s">
-        <x:v>686</x:v>
-      </x:c>
       <x:c r="C30" s="7" t="s">
-        <x:v>678</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="D30" s="9">
         <x:v>1</x:v>
@@ -7875,47 +7872,47 @@
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="8" t="s">
+        <x:v>686</x:v>
+      </x:c>
+      <x:c r="B31" s="7" t="s">
         <x:v>687</x:v>
       </x:c>
-      <x:c r="B31" s="7" t="s">
+      <x:c r="C31" s="7" t="s">
+        <x:v>626</x:v>
+      </x:c>
+      <x:c r="D31" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E31" s="10" t="s">
         <x:v>688</x:v>
-      </x:c>
-      <x:c r="C31" s="7" t="s">
-        <x:v>627</x:v>
-      </x:c>
-      <x:c r="D31" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E31" s="10" t="s">
-        <x:v>689</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="28" customHeight="1">
       <x:c r="A32" s="8" t="s">
+        <x:v>689</x:v>
+      </x:c>
+      <x:c r="B32" s="7" t="s">
         <x:v>690</x:v>
       </x:c>
-      <x:c r="B32" s="7" t="s">
+      <x:c r="C32" s="7" t="s">
         <x:v>691</x:v>
       </x:c>
-      <x:c r="C32" s="7" t="s">
+      <x:c r="D32" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E32" s="10" t="s">
         <x:v>692</x:v>
-      </x:c>
-      <x:c r="D32" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E32" s="10" t="s">
-        <x:v>693</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="8" t="s">
+        <x:v>693</x:v>
+      </x:c>
+      <x:c r="B33" s="7" t="s">
         <x:v>694</x:v>
       </x:c>
-      <x:c r="B33" s="7" t="s">
-        <x:v>695</x:v>
-      </x:c>
       <x:c r="C33" s="7" t="s">
-        <x:v>665</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="D33" s="9">
         <x:v>1</x:v>
@@ -7924,13 +7921,13 @@
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
       <x:c r="A34" s="8" t="s">
+        <x:v>695</x:v>
+      </x:c>
+      <x:c r="B34" s="7" t="s">
         <x:v>696</x:v>
       </x:c>
-      <x:c r="B34" s="7" t="s">
+      <x:c r="C34" s="7" t="s">
         <x:v>697</x:v>
-      </x:c>
-      <x:c r="C34" s="7" t="s">
-        <x:v>698</x:v>
       </x:c>
       <x:c r="D34" s="9">
         <x:v>1</x:v>
@@ -7939,47 +7936,47 @@
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
       <x:c r="A35" s="8" t="s">
+        <x:v>698</x:v>
+      </x:c>
+      <x:c r="B35" s="7" t="s">
         <x:v>699</x:v>
       </x:c>
-      <x:c r="B35" s="7" t="s">
+      <x:c r="C35" s="7" t="s">
         <x:v>700</x:v>
       </x:c>
-      <x:c r="C35" s="7" t="s">
+      <x:c r="D35" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E35" s="10" t="s">
         <x:v>701</x:v>
-      </x:c>
-      <x:c r="D35" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E35" s="10" t="s">
-        <x:v>702</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
       <x:c r="A36" s="8" t="s">
+        <x:v>702</x:v>
+      </x:c>
+      <x:c r="B36" s="7" t="s">
         <x:v>703</x:v>
       </x:c>
-      <x:c r="B36" s="7" t="s">
+      <x:c r="C36" s="7" t="s">
         <x:v>704</x:v>
       </x:c>
-      <x:c r="C36" s="7" t="s">
+      <x:c r="D36" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E36" s="10" t="s">
         <x:v>705</x:v>
-      </x:c>
-      <x:c r="D36" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E36" s="10" t="s">
-        <x:v>706</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
       <x:c r="A37" s="8" t="s">
+        <x:v>706</x:v>
+      </x:c>
+      <x:c r="B37" s="7" t="s">
         <x:v>707</x:v>
       </x:c>
-      <x:c r="B37" s="7" t="s">
+      <x:c r="C37" s="7" t="s">
         <x:v>708</x:v>
-      </x:c>
-      <x:c r="C37" s="7" t="s">
-        <x:v>709</x:v>
       </x:c>
       <x:c r="D37" s="9">
         <x:v>1</x:v>
@@ -7988,13 +7985,13 @@
     </x:row>
     <x:row r="38" ht="28" customHeight="1">
       <x:c r="A38" s="8" t="s">
+        <x:v>709</x:v>
+      </x:c>
+      <x:c r="B38" s="7" t="s">
         <x:v>710</x:v>
       </x:c>
-      <x:c r="B38" s="7" t="s">
-        <x:v>711</x:v>
-      </x:c>
       <x:c r="C38" s="7" t="s">
-        <x:v>648</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="D38" s="9">
         <x:v>1</x:v>
@@ -8003,13 +8000,13 @@
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
       <x:c r="A39" s="8" t="s">
+        <x:v>711</x:v>
+      </x:c>
+      <x:c r="B39" s="7" t="s">
         <x:v>712</x:v>
       </x:c>
-      <x:c r="B39" s="7" t="s">
+      <x:c r="C39" s="7" t="s">
         <x:v>713</x:v>
-      </x:c>
-      <x:c r="C39" s="7" t="s">
-        <x:v>714</x:v>
       </x:c>
       <x:c r="D39" s="9">
         <x:v>3</x:v>
@@ -8018,47 +8015,47 @@
     </x:row>
     <x:row r="40" ht="28" customHeight="1">
       <x:c r="A40" s="8" t="s">
+        <x:v>714</x:v>
+      </x:c>
+      <x:c r="B40" s="7" t="s">
         <x:v>715</x:v>
       </x:c>
-      <x:c r="B40" s="7" t="s">
+      <x:c r="C40" s="7" t="s">
         <x:v>716</x:v>
       </x:c>
-      <x:c r="C40" s="7" t="s">
+      <x:c r="D40" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E40" s="10" t="s">
         <x:v>717</x:v>
-      </x:c>
-      <x:c r="D40" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E40" s="10" t="s">
-        <x:v>718</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="8" t="s">
+        <x:v>718</x:v>
+      </x:c>
+      <x:c r="B41" s="7" t="s">
         <x:v>719</x:v>
       </x:c>
-      <x:c r="B41" s="7" t="s">
+      <x:c r="C41" s="7" t="s">
+        <x:v>716</x:v>
+      </x:c>
+      <x:c r="D41" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E41" s="10" t="s">
         <x:v>720</x:v>
-      </x:c>
-      <x:c r="C41" s="7" t="s">
-        <x:v>717</x:v>
-      </x:c>
-      <x:c r="D41" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E41" s="10" t="s">
-        <x:v>721</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
       <x:c r="A42" s="8" t="s">
+        <x:v>721</x:v>
+      </x:c>
+      <x:c r="B42" s="7" t="s">
         <x:v>722</x:v>
       </x:c>
-      <x:c r="B42" s="7" t="s">
+      <x:c r="C42" s="7" t="s">
         <x:v>723</x:v>
-      </x:c>
-      <x:c r="C42" s="7" t="s">
-        <x:v>724</x:v>
       </x:c>
       <x:c r="D42" s="9">
         <x:v>1</x:v>
@@ -8067,10 +8064,10 @@
     </x:row>
     <x:row r="43" ht="28" customHeight="1">
       <x:c r="A43" s="8" t="s">
+        <x:v>724</x:v>
+      </x:c>
+      <x:c r="B43" s="7" t="s">
         <x:v>725</x:v>
-      </x:c>
-      <x:c r="B43" s="7" t="s">
-        <x:v>726</x:v>
       </x:c>
       <x:c r="C43" s="7" t="str">
         <x:v>#069, #079</x:v>
@@ -8082,30 +8079,30 @@
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="8" t="s">
+        <x:v>726</x:v>
+      </x:c>
+      <x:c r="B44" s="7" t="s">
         <x:v>727</x:v>
       </x:c>
-      <x:c r="B44" s="7" t="s">
-        <x:v>728</x:v>
-      </x:c>
       <x:c r="C44" s="7" t="s">
-        <x:v>681</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="D44" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E44" s="10" t="s">
-        <x:v>729</x:v>
+        <x:v>728</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
       <x:c r="A45" s="8" t="s">
+        <x:v>729</x:v>
+      </x:c>
+      <x:c r="B45" s="7" t="s">
         <x:v>730</x:v>
       </x:c>
-      <x:c r="B45" s="7" t="s">
+      <x:c r="C45" s="7" t="s">
         <x:v>731</x:v>
-      </x:c>
-      <x:c r="C45" s="7" t="s">
-        <x:v>732</x:v>
       </x:c>
       <x:c r="D45" s="9">
         <x:v>1</x:v>
@@ -8114,13 +8111,13 @@
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
       <x:c r="A46" s="8" t="s">
+        <x:v>732</x:v>
+      </x:c>
+      <x:c r="B46" s="7" t="s">
         <x:v>733</x:v>
       </x:c>
-      <x:c r="B46" s="7" t="s">
-        <x:v>734</x:v>
-      </x:c>
       <x:c r="C46" s="7" t="s">
-        <x:v>698</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="D46" s="9">
         <x:v>1</x:v>
@@ -8129,47 +8126,47 @@
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
       <x:c r="A47" s="8" t="s">
+        <x:v>734</x:v>
+      </x:c>
+      <x:c r="B47" s="7" t="s">
         <x:v>735</x:v>
       </x:c>
-      <x:c r="B47" s="7" t="s">
+      <x:c r="C47" s="7" t="s">
+        <x:v>609</x:v>
+      </x:c>
+      <x:c r="D47" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E47" s="10" t="s">
         <x:v>736</x:v>
-      </x:c>
-      <x:c r="C47" s="7" t="s">
-        <x:v>610</x:v>
-      </x:c>
-      <x:c r="D47" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E47" s="10" t="s">
-        <x:v>737</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
       <x:c r="A48" s="8" t="s">
+        <x:v>737</x:v>
+      </x:c>
+      <x:c r="B48" s="7" t="s">
         <x:v>738</x:v>
       </x:c>
-      <x:c r="B48" s="7" t="s">
+      <x:c r="C48" s="7" t="s">
         <x:v>739</x:v>
-      </x:c>
-      <x:c r="C48" s="7" t="s">
-        <x:v>740</x:v>
       </x:c>
       <x:c r="D48" s="9">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="10" t="s">
-        <x:v>741</x:v>
+        <x:v>740</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
       <x:c r="A49" s="8" t="s">
+        <x:v>741</x:v>
+      </x:c>
+      <x:c r="B49" s="7" t="s">
         <x:v>742</x:v>
       </x:c>
-      <x:c r="B49" s="7" t="s">
+      <x:c r="C49" s="7" t="s">
         <x:v>743</x:v>
-      </x:c>
-      <x:c r="C49" s="7" t="s">
-        <x:v>744</x:v>
       </x:c>
       <x:c r="D49" s="9">
         <x:v>1</x:v>
@@ -8178,13 +8175,13 @@
     </x:row>
     <x:row r="50" ht="28" customHeight="1">
       <x:c r="A50" s="8" t="s">
+        <x:v>744</x:v>
+      </x:c>
+      <x:c r="B50" s="7" t="s">
         <x:v>745</x:v>
       </x:c>
-      <x:c r="B50" s="7" t="s">
-        <x:v>746</x:v>
-      </x:c>
       <x:c r="C50" s="7" t="s">
-        <x:v>709</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="D50" s="9">
         <x:v>1</x:v>
@@ -8193,64 +8190,64 @@
     </x:row>
     <x:row r="51" ht="28" customHeight="1">
       <x:c r="A51" s="8" t="s">
+        <x:v>746</x:v>
+      </x:c>
+      <x:c r="B51" s="7" t="s">
         <x:v>747</x:v>
       </x:c>
-      <x:c r="B51" s="7" t="s">
+      <x:c r="C51" s="7" t="s">
         <x:v>748</x:v>
-      </x:c>
-      <x:c r="C51" s="7" t="s">
-        <x:v>749</x:v>
       </x:c>
       <x:c r="D51" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E51" s="10" t="s">
-        <x:v>750</x:v>
+        <x:v>749</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="28" customHeight="1">
       <x:c r="A52" s="8" t="s">
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="B52" s="7" t="s">
         <x:v>751</x:v>
       </x:c>
-      <x:c r="B52" s="7" t="s">
+      <x:c r="C52" s="7" t="s">
         <x:v>752</x:v>
       </x:c>
-      <x:c r="C52" s="7" t="s">
+      <x:c r="D52" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E52" s="10" t="s">
         <x:v>753</x:v>
-      </x:c>
-      <x:c r="D52" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E52" s="10" t="s">
-        <x:v>754</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="28" customHeight="1">
       <x:c r="A53" s="8" t="s">
+        <x:v>754</x:v>
+      </x:c>
+      <x:c r="B53" s="7" t="s">
         <x:v>755</x:v>
       </x:c>
-      <x:c r="B53" s="7" t="s">
+      <x:c r="C53" s="7" t="s">
         <x:v>756</x:v>
-      </x:c>
-      <x:c r="C53" s="7" t="s">
-        <x:v>757</x:v>
       </x:c>
       <x:c r="D53" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E53" s="10" t="s">
-        <x:v>758</x:v>
+        <x:v>757</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="28" customHeight="1">
       <x:c r="A54" s="8" t="s">
+        <x:v>758</x:v>
+      </x:c>
+      <x:c r="B54" s="7" t="s">
         <x:v>759</x:v>
       </x:c>
-      <x:c r="B54" s="7" t="s">
+      <x:c r="C54" s="7" t="s">
         <x:v>760</x:v>
-      </x:c>
-      <x:c r="C54" s="7" t="s">
-        <x:v>761</x:v>
       </x:c>
       <x:c r="D54" s="9">
         <x:v>1</x:v>
@@ -8259,81 +8256,81 @@
     </x:row>
     <x:row r="55" ht="28" customHeight="1">
       <x:c r="A55" s="8" t="s">
+        <x:v>761</x:v>
+      </x:c>
+      <x:c r="B55" s="7" t="s">
         <x:v>762</x:v>
       </x:c>
-      <x:c r="B55" s="7" t="s">
+      <x:c r="C55" s="7" t="s">
         <x:v>763</x:v>
       </x:c>
-      <x:c r="C55" s="7" t="s">
+      <x:c r="D55" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E55" s="10" t="s">
         <x:v>764</x:v>
-      </x:c>
-      <x:c r="D55" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E55" s="10" t="s">
-        <x:v>765</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="28" customHeight="1">
       <x:c r="A56" s="8" t="s">
+        <x:v>765</x:v>
+      </x:c>
+      <x:c r="B56" s="7" t="s">
         <x:v>766</x:v>
       </x:c>
-      <x:c r="B56" s="7" t="s">
+      <x:c r="C56" s="7" t="s">
         <x:v>767</x:v>
       </x:c>
-      <x:c r="C56" s="7" t="s">
+      <x:c r="D56" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E56" s="10" t="s">
         <x:v>768</x:v>
-      </x:c>
-      <x:c r="D56" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E56" s="10" t="s">
-        <x:v>769</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
       <x:c r="A57" s="8" t="s">
+        <x:v>769</x:v>
+      </x:c>
+      <x:c r="B57" s="7" t="s">
         <x:v>770</x:v>
       </x:c>
-      <x:c r="B57" s="7" t="s">
+      <x:c r="C57" s="7" t="s">
         <x:v>771</x:v>
       </x:c>
-      <x:c r="C57" s="7" t="s">
+      <x:c r="D57" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E57" s="10" t="s">
         <x:v>772</x:v>
-      </x:c>
-      <x:c r="D57" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E57" s="10" t="s">
-        <x:v>773</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
       <x:c r="A58" s="8" t="s">
+        <x:v>773</x:v>
+      </x:c>
+      <x:c r="B58" s="7" t="s">
         <x:v>774</x:v>
       </x:c>
-      <x:c r="B58" s="7" t="s">
+      <x:c r="C58" s="7" t="s">
         <x:v>775</x:v>
-      </x:c>
-      <x:c r="C58" s="7" t="s">
-        <x:v>776</x:v>
       </x:c>
       <x:c r="D58" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E58" s="10" t="s">
-        <x:v>777</x:v>
+        <x:v>776</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
       <x:c r="A59" s="8" t="s">
+        <x:v>777</x:v>
+      </x:c>
+      <x:c r="B59" s="7" t="s">
         <x:v>778</x:v>
       </x:c>
-      <x:c r="B59" s="7" t="s">
-        <x:v>779</x:v>
-      </x:c>
       <x:c r="C59" s="7" t="s">
-        <x:v>614</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="D59" s="9">
         <x:v>1</x:v>
@@ -8342,13 +8339,13 @@
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
       <x:c r="A60" s="8" t="s">
+        <x:v>779</x:v>
+      </x:c>
+      <x:c r="B60" s="7" t="s">
         <x:v>780</x:v>
       </x:c>
-      <x:c r="B60" s="7" t="s">
-        <x:v>781</x:v>
-      </x:c>
       <x:c r="C60" s="7" t="s">
-        <x:v>651</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="D60" s="9">
         <x:v>1</x:v>
@@ -8357,13 +8354,13 @@
     </x:row>
     <x:row r="61" ht="28" customHeight="1">
       <x:c r="A61" s="8" t="s">
+        <x:v>781</x:v>
+      </x:c>
+      <x:c r="B61" s="7" t="s">
         <x:v>782</x:v>
       </x:c>
-      <x:c r="B61" s="7" t="s">
-        <x:v>783</x:v>
-      </x:c>
       <x:c r="C61" s="7" t="s">
-        <x:v>635</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="D61" s="9">
         <x:v>1</x:v>
@@ -8372,30 +8369,30 @@
     </x:row>
     <x:row r="62" ht="28" customHeight="1">
       <x:c r="A62" s="8" t="s">
+        <x:v>783</x:v>
+      </x:c>
+      <x:c r="B62" s="7" t="s">
         <x:v>784</x:v>
       </x:c>
-      <x:c r="B62" s="7" t="s">
+      <x:c r="C62" s="7" t="s">
+        <x:v>640</x:v>
+      </x:c>
+      <x:c r="D62" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E62" s="10" t="s">
         <x:v>785</x:v>
-      </x:c>
-      <x:c r="C62" s="7" t="s">
-        <x:v>641</x:v>
-      </x:c>
-      <x:c r="D62" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E62" s="10" t="s">
-        <x:v>786</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="28" customHeight="1">
       <x:c r="A63" s="8" t="s">
+        <x:v>786</x:v>
+      </x:c>
+      <x:c r="B63" s="7" t="s">
         <x:v>787</x:v>
       </x:c>
-      <x:c r="B63" s="7" t="s">
-        <x:v>788</x:v>
-      </x:c>
       <x:c r="C63" s="7" t="s">
-        <x:v>635</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="D63" s="9">
         <x:v>1</x:v>
@@ -8404,13 +8401,13 @@
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
       <x:c r="A64" s="8" t="s">
+        <x:v>788</x:v>
+      </x:c>
+      <x:c r="B64" s="7" t="s">
         <x:v>789</x:v>
       </x:c>
-      <x:c r="B64" s="7" t="s">
+      <x:c r="C64" s="7" t="s">
         <x:v>790</x:v>
-      </x:c>
-      <x:c r="C64" s="7" t="s">
-        <x:v>791</x:v>
       </x:c>
       <x:c r="D64" s="9">
         <x:v>1</x:v>
@@ -8419,13 +8416,13 @@
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
       <x:c r="A65" s="8" t="s">
+        <x:v>791</x:v>
+      </x:c>
+      <x:c r="B65" s="7" t="s">
         <x:v>792</x:v>
       </x:c>
-      <x:c r="B65" s="7" t="s">
+      <x:c r="C65" s="7" t="s">
         <x:v>793</x:v>
-      </x:c>
-      <x:c r="C65" s="7" t="s">
-        <x:v>794</x:v>
       </x:c>
       <x:c r="D65" s="9">
         <x:v>1</x:v>
@@ -8434,13 +8431,13 @@
     </x:row>
     <x:row r="66" ht="28" customHeight="1">
       <x:c r="A66" s="8" t="s">
+        <x:v>794</x:v>
+      </x:c>
+      <x:c r="B66" s="7" t="s">
         <x:v>795</x:v>
       </x:c>
-      <x:c r="B66" s="7" t="s">
-        <x:v>796</x:v>
-      </x:c>
       <x:c r="C66" s="7" t="s">
-        <x:v>624</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="D66" s="9">
         <x:v>1</x:v>
@@ -8449,47 +8446,47 @@
     </x:row>
     <x:row r="67" ht="28" customHeight="1">
       <x:c r="A67" s="8" t="s">
+        <x:v>796</x:v>
+      </x:c>
+      <x:c r="B67" s="7" t="s">
         <x:v>797</x:v>
       </x:c>
-      <x:c r="B67" s="7" t="s">
-        <x:v>798</x:v>
-      </x:c>
       <x:c r="C67" s="7" t="s">
-        <x:v>776</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="D67" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E67" s="10" t="s">
-        <x:v>799</x:v>
+        <x:v>798</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="28" customHeight="1">
       <x:c r="A68" s="8" t="s">
+        <x:v>799</x:v>
+      </x:c>
+      <x:c r="B68" s="7" t="s">
         <x:v>800</x:v>
       </x:c>
-      <x:c r="B68" s="7" t="s">
+      <x:c r="C68" s="7" t="s">
+        <x:v>650</x:v>
+      </x:c>
+      <x:c r="D68" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E68" s="10" t="s">
         <x:v>801</x:v>
-      </x:c>
-      <x:c r="C68" s="7" t="s">
-        <x:v>651</x:v>
-      </x:c>
-      <x:c r="D68" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E68" s="10" t="s">
-        <x:v>802</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
       <x:c r="A69" s="8" t="s">
+        <x:v>802</x:v>
+      </x:c>
+      <x:c r="B69" s="7" t="s">
         <x:v>803</x:v>
       </x:c>
-      <x:c r="B69" s="7" t="s">
-        <x:v>804</x:v>
-      </x:c>
       <x:c r="C69" s="7" t="s">
-        <x:v>631</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="D69" s="9">
         <x:v>1</x:v>
@@ -8498,13 +8495,13 @@
     </x:row>
     <x:row r="70" ht="28" customHeight="1">
       <x:c r="A70" s="8" t="s">
+        <x:v>804</x:v>
+      </x:c>
+      <x:c r="B70" s="7" t="s">
         <x:v>805</x:v>
       </x:c>
-      <x:c r="B70" s="7" t="s">
-        <x:v>806</x:v>
-      </x:c>
       <x:c r="C70" s="7" t="s">
-        <x:v>659</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="D70" s="9">
         <x:v>1</x:v>
@@ -8513,13 +8510,13 @@
     </x:row>
     <x:row r="71" ht="28" customHeight="1">
       <x:c r="A71" s="8" t="s">
+        <x:v>806</x:v>
+      </x:c>
+      <x:c r="B71" s="7" t="s">
         <x:v>807</x:v>
       </x:c>
-      <x:c r="B71" s="7" t="s">
+      <x:c r="C71" s="7" t="s">
         <x:v>808</x:v>
-      </x:c>
-      <x:c r="C71" s="7" t="s">
-        <x:v>809</x:v>
       </x:c>
       <x:c r="D71" s="9">
         <x:v>1</x:v>
@@ -8528,64 +8525,64 @@
     </x:row>
     <x:row r="72" ht="28" customHeight="1">
       <x:c r="A72" s="8" t="s">
+        <x:v>809</x:v>
+      </x:c>
+      <x:c r="B72" s="7" t="s">
         <x:v>810</x:v>
       </x:c>
-      <x:c r="B72" s="7" t="s">
+      <x:c r="C72" s="7" t="s">
         <x:v>811</x:v>
-      </x:c>
-      <x:c r="C72" s="7" t="s">
-        <x:v>812</x:v>
       </x:c>
       <x:c r="D72" s="9">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E72" s="10" t="s">
-        <x:v>813</x:v>
+        <x:v>812</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="28" customHeight="1">
       <x:c r="A73" s="8" t="s">
+        <x:v>813</x:v>
+      </x:c>
+      <x:c r="B73" s="7" t="s">
         <x:v>814</x:v>
       </x:c>
-      <x:c r="B73" s="7" t="s">
+      <x:c r="C73" s="7" t="s">
         <x:v>815</x:v>
       </x:c>
-      <x:c r="C73" s="7" t="s">
+      <x:c r="D73" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E73" s="10" t="s">
         <x:v>816</x:v>
-      </x:c>
-      <x:c r="D73" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E73" s="10" t="s">
-        <x:v>817</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="28" customHeight="1">
       <x:c r="A74" s="8" t="s">
+        <x:v>817</x:v>
+      </x:c>
+      <x:c r="B74" s="7" t="s">
         <x:v>818</x:v>
       </x:c>
-      <x:c r="B74" s="7" t="s">
+      <x:c r="C74" s="7" t="s">
+        <x:v>616</x:v>
+      </x:c>
+      <x:c r="D74" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E74" s="10" t="s">
         <x:v>819</x:v>
-      </x:c>
-      <x:c r="C74" s="7" t="s">
-        <x:v>617</x:v>
-      </x:c>
-      <x:c r="D74" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E74" s="10" t="s">
-        <x:v>820</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="28" customHeight="1">
       <x:c r="A75" s="8" t="s">
+        <x:v>820</x:v>
+      </x:c>
+      <x:c r="B75" s="7" t="s">
         <x:v>821</x:v>
       </x:c>
-      <x:c r="B75" s="7" t="s">
-        <x:v>822</x:v>
-      </x:c>
       <x:c r="C75" s="7" t="s">
-        <x:v>732</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="D75" s="9">
         <x:v>1</x:v>
@@ -8594,64 +8591,64 @@
     </x:row>
     <x:row r="76" ht="28" customHeight="1">
       <x:c r="A76" s="8" t="s">
+        <x:v>822</x:v>
+      </x:c>
+      <x:c r="B76" s="7" t="s">
         <x:v>823</x:v>
       </x:c>
-      <x:c r="B76" s="7" t="s">
+      <x:c r="C76" s="7" t="s">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="D76" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E76" s="10" t="s">
         <x:v>824</x:v>
-      </x:c>
-      <x:c r="C76" s="7" t="s">
-        <x:v>701</x:v>
-      </x:c>
-      <x:c r="D76" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E76" s="10" t="s">
-        <x:v>825</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
       <x:c r="A77" s="8" t="s">
+        <x:v>825</x:v>
+      </x:c>
+      <x:c r="B77" s="7" t="s">
         <x:v>826</x:v>
       </x:c>
-      <x:c r="B77" s="7" t="s">
+      <x:c r="C77" s="7" t="s">
+        <x:v>808</x:v>
+      </x:c>
+      <x:c r="D77" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E77" s="10" t="s">
         <x:v>827</x:v>
-      </x:c>
-      <x:c r="C77" s="7" t="s">
-        <x:v>809</x:v>
-      </x:c>
-      <x:c r="D77" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E77" s="10" t="s">
-        <x:v>828</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
       <x:c r="A78" s="8" t="s">
+        <x:v>828</x:v>
+      </x:c>
+      <x:c r="B78" s="7" t="s">
         <x:v>829</x:v>
       </x:c>
-      <x:c r="B78" s="7" t="s">
-        <x:v>830</x:v>
-      </x:c>
       <x:c r="C78" s="7" t="s">
-        <x:v>606</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="D78" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E78" s="10" t="s">
-        <x:v>831</x:v>
+        <x:v>830</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="28" customHeight="1">
       <x:c r="A79" s="8" t="s">
+        <x:v>831</x:v>
+      </x:c>
+      <x:c r="B79" s="7" t="s">
         <x:v>832</x:v>
       </x:c>
-      <x:c r="B79" s="7" t="s">
-        <x:v>833</x:v>
-      </x:c>
       <x:c r="C79" s="7" t="s">
-        <x:v>701</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="D79" s="9">
         <x:v>1</x:v>
@@ -8660,24 +8657,24 @@
     </x:row>
     <x:row r="80" ht="28" customHeight="1">
       <x:c r="A80" s="8" t="s">
+        <x:v>833</x:v>
+      </x:c>
+      <x:c r="B80" s="7" t="s">
         <x:v>834</x:v>
       </x:c>
-      <x:c r="B80" s="7" t="s">
+      <x:c r="C80" s="7" t="s">
         <x:v>835</x:v>
       </x:c>
-      <x:c r="C80" s="7" t="s">
+      <x:c r="D80" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E80" s="10" t="s">
         <x:v>836</x:v>
-      </x:c>
-      <x:c r="D80" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E80" s="10" t="s">
-        <x:v>837</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="28" customHeight="1">
       <x:c r="A81" s="8" t="s">
-        <x:v>838</x:v>
+        <x:v>837</x:v>
       </x:c>
       <x:c r="B81" s="7" t="s">
         <x:v>172</x:v>
@@ -8689,35 +8686,35 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="E81" s="10" t="s">
-        <x:v>839</x:v>
+        <x:v>838</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="28" customHeight="1">
       <x:c r="A82" s="8" t="s">
+        <x:v>839</x:v>
+      </x:c>
+      <x:c r="B82" s="7" t="s">
         <x:v>840</x:v>
       </x:c>
-      <x:c r="B82" s="7" t="s">
+      <x:c r="C82" s="7" t="s">
         <x:v>841</x:v>
-      </x:c>
-      <x:c r="C82" s="7" t="s">
-        <x:v>842</x:v>
       </x:c>
       <x:c r="D82" s="9">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E82" s="10" t="s">
-        <x:v>843</x:v>
+        <x:v>842</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="28" customHeight="1">
       <x:c r="A83" s="8" t="s">
+        <x:v>843</x:v>
+      </x:c>
+      <x:c r="B83" s="7" t="s">
         <x:v>844</x:v>
       </x:c>
-      <x:c r="B83" s="7" t="s">
-        <x:v>845</x:v>
-      </x:c>
       <x:c r="C83" s="7" t="s">
-        <x:v>624</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="D83" s="9">
         <x:v>1</x:v>
@@ -8726,13 +8723,13 @@
     </x:row>
     <x:row r="84" ht="28" customHeight="1">
       <x:c r="A84" s="8" t="s">
+        <x:v>845</x:v>
+      </x:c>
+      <x:c r="B84" s="7" t="s">
         <x:v>846</x:v>
       </x:c>
-      <x:c r="B84" s="7" t="s">
+      <x:c r="C84" s="7" t="s">
         <x:v>847</x:v>
-      </x:c>
-      <x:c r="C84" s="7" t="s">
-        <x:v>848</x:v>
       </x:c>
       <x:c r="D84" s="9">
         <x:v>1</x:v>
@@ -8741,64 +8738,64 @@
     </x:row>
     <x:row r="85" ht="28" customHeight="1">
       <x:c r="A85" s="8" t="s">
+        <x:v>848</x:v>
+      </x:c>
+      <x:c r="B85" s="7" t="s">
         <x:v>849</x:v>
       </x:c>
-      <x:c r="B85" s="7" t="s">
+      <x:c r="C85" s="7" t="s">
+        <x:v>626</x:v>
+      </x:c>
+      <x:c r="D85" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E85" s="10" t="s">
         <x:v>850</x:v>
-      </x:c>
-      <x:c r="C85" s="7" t="s">
-        <x:v>627</x:v>
-      </x:c>
-      <x:c r="D85" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E85" s="10" t="s">
-        <x:v>851</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="28" customHeight="1">
       <x:c r="A86" s="8" t="s">
+        <x:v>851</x:v>
+      </x:c>
+      <x:c r="B86" s="7" t="s">
         <x:v>852</x:v>
       </x:c>
-      <x:c r="B86" s="7" t="s">
+      <x:c r="C86" s="7" t="s">
         <x:v>853</x:v>
       </x:c>
-      <x:c r="C86" s="7" t="s">
+      <x:c r="D86" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E86" s="10" t="s">
         <x:v>854</x:v>
-      </x:c>
-      <x:c r="D86" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E86" s="10" t="s">
-        <x:v>855</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="28" customHeight="1">
       <x:c r="A87" s="8" t="s">
+        <x:v>855</x:v>
+      </x:c>
+      <x:c r="B87" s="7" t="s">
         <x:v>856</x:v>
       </x:c>
-      <x:c r="B87" s="7" t="s">
+      <x:c r="C87" s="7" t="s">
         <x:v>857</x:v>
       </x:c>
-      <x:c r="C87" s="7" t="s">
+      <x:c r="D87" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E87" s="10" t="s">
         <x:v>858</x:v>
-      </x:c>
-      <x:c r="D87" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E87" s="10" t="s">
-        <x:v>859</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="28" customHeight="1">
       <x:c r="A88" s="8" t="s">
+        <x:v>859</x:v>
+      </x:c>
+      <x:c r="B88" s="7" t="s">
         <x:v>860</x:v>
       </x:c>
-      <x:c r="B88" s="7" t="s">
-        <x:v>861</x:v>
-      </x:c>
       <x:c r="C88" s="7" t="s">
-        <x:v>732</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="D88" s="9">
         <x:v>1</x:v>
@@ -8807,13 +8804,13 @@
     </x:row>
     <x:row r="89" ht="28" customHeight="1">
       <x:c r="A89" s="8" t="s">
+        <x:v>861</x:v>
+      </x:c>
+      <x:c r="B89" s="7" t="s">
         <x:v>862</x:v>
       </x:c>
-      <x:c r="B89" s="7" t="s">
-        <x:v>863</x:v>
-      </x:c>
       <x:c r="C89" s="7" t="s">
-        <x:v>648</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="D89" s="9">
         <x:v>1</x:v>
@@ -8822,30 +8819,30 @@
     </x:row>
     <x:row r="90" ht="28" customHeight="1">
       <x:c r="A90" s="8" t="s">
+        <x:v>863</x:v>
+      </x:c>
+      <x:c r="B90" s="7" t="s">
         <x:v>864</x:v>
       </x:c>
-      <x:c r="B90" s="7" t="s">
-        <x:v>865</x:v>
-      </x:c>
       <x:c r="C90" s="7" t="s">
-        <x:v>776</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="D90" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E90" s="10" t="s">
-        <x:v>866</x:v>
+        <x:v>865</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="28" customHeight="1">
       <x:c r="A91" s="8" t="s">
+        <x:v>866</x:v>
+      </x:c>
+      <x:c r="B91" s="7" t="s">
         <x:v>867</x:v>
       </x:c>
-      <x:c r="B91" s="7" t="s">
+      <x:c r="C91" s="7" t="s">
         <x:v>868</x:v>
-      </x:c>
-      <x:c r="C91" s="7" t="s">
-        <x:v>869</x:v>
       </x:c>
       <x:c r="D91" s="9">
         <x:v>1</x:v>
@@ -8854,30 +8851,30 @@
     </x:row>
     <x:row r="92" ht="28" customHeight="1">
       <x:c r="A92" s="8" t="s">
+        <x:v>869</x:v>
+      </x:c>
+      <x:c r="B92" s="7" t="s">
         <x:v>870</x:v>
       </x:c>
-      <x:c r="B92" s="7" t="s">
+      <x:c r="C92" s="7" t="s">
         <x:v>871</x:v>
-      </x:c>
-      <x:c r="C92" s="7" t="s">
-        <x:v>872</x:v>
       </x:c>
       <x:c r="D92" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E92" s="10" t="s">
-        <x:v>873</x:v>
+        <x:v>872</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="28" customHeight="1">
       <x:c r="A93" s="8" t="s">
+        <x:v>873</x:v>
+      </x:c>
+      <x:c r="B93" s="7" t="s">
         <x:v>874</x:v>
       </x:c>
-      <x:c r="B93" s="7" t="s">
-        <x:v>875</x:v>
-      </x:c>
       <x:c r="C93" s="7" t="s">
-        <x:v>809</x:v>
+        <x:v>808</x:v>
       </x:c>
       <x:c r="D93" s="9">
         <x:v>1</x:v>
@@ -8886,30 +8883,30 @@
     </x:row>
     <x:row r="94" ht="28" customHeight="1">
       <x:c r="A94" s="8" t="s">
+        <x:v>875</x:v>
+      </x:c>
+      <x:c r="B94" s="7" t="s">
         <x:v>876</x:v>
       </x:c>
-      <x:c r="B94" s="7" t="s">
+      <x:c r="C94" s="7" t="s">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="D94" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E94" s="10" t="s">
         <x:v>877</x:v>
-      </x:c>
-      <x:c r="C94" s="7" t="s">
-        <x:v>701</x:v>
-      </x:c>
-      <x:c r="D94" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E94" s="10" t="s">
-        <x:v>878</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="28" customHeight="1">
       <x:c r="A95" s="8" t="s">
+        <x:v>878</x:v>
+      </x:c>
+      <x:c r="B95" s="7" t="s">
         <x:v>879</x:v>
       </x:c>
-      <x:c r="B95" s="7" t="s">
-        <x:v>880</x:v>
-      </x:c>
       <x:c r="C95" s="7" t="s">
-        <x:v>698</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="D95" s="9">
         <x:v>1</x:v>
@@ -8918,47 +8915,47 @@
     </x:row>
     <x:row r="96" ht="28" customHeight="1">
       <x:c r="A96" s="8" t="s">
+        <x:v>880</x:v>
+      </x:c>
+      <x:c r="B96" s="7" t="s">
         <x:v>881</x:v>
       </x:c>
-      <x:c r="B96" s="7" t="s">
+      <x:c r="C96" s="7" t="s">
         <x:v>882</x:v>
-      </x:c>
-      <x:c r="C96" s="7" t="s">
-        <x:v>883</x:v>
       </x:c>
       <x:c r="D96" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E96" s="10" t="s">
-        <x:v>884</x:v>
+        <x:v>883</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="28" customHeight="1">
       <x:c r="A97" s="8" t="s">
+        <x:v>884</x:v>
+      </x:c>
+      <x:c r="B97" s="7" t="s">
         <x:v>885</x:v>
       </x:c>
-      <x:c r="B97" s="7" t="s">
+      <x:c r="C97" s="7" t="s">
+        <x:v>847</x:v>
+      </x:c>
+      <x:c r="D97" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E97" s="10" t="s">
         <x:v>886</x:v>
-      </x:c>
-      <x:c r="C97" s="7" t="s">
-        <x:v>848</x:v>
-      </x:c>
-      <x:c r="D97" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E97" s="10" t="s">
-        <x:v>887</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="s">
+        <x:v>887</x:v>
+      </x:c>
+      <x:c r="B98" t="s">
         <x:v>888</x:v>
       </x:c>
-      <x:c r="B98" t="s">
+      <x:c r="C98" t="s">
         <x:v>889</x:v>
-      </x:c>
-      <x:c r="C98" t="s">
-        <x:v>890</x:v>
       </x:c>
       <x:c r="D98">
         <x:v>1</x:v>
@@ -8979,12 +8976,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rca388b157f0d4b07"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R36702bf93f504345"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R44a0218bf92e4dfd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Re5a6ec2bcb9b49f6"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31018f881d3d4df5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R352cf6a99b764d67"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8999,7 +8996,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>891</x:v>
+        <x:v>890</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -9887,7 +9884,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c515df95d5343e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1be11ad109a04c6b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9903,27 +9900,27 @@
   <x:sheetData>
     <x:row r="1" ht="34.75" customHeight="1">
       <x:c r="A1" s="20" t="s">
-        <x:v>892</x:v>
+        <x:v>891</x:v>
       </x:c>
       <x:c r="B1" s="20"/>
       <x:c r="C1" s="20"/>
     </x:row>
     <x:row r="2" ht="45.25" customHeight="1">
       <x:c r="A2" s="21" t="s">
-        <x:v>893</x:v>
+        <x:v>892</x:v>
       </x:c>
       <x:c r="B2" s="21"/>
       <x:c r="C2" s="21"/>
     </x:row>
     <x:row r="4" ht="29.25" customHeight="1">
       <x:c r="A4" s="15" t="s">
+        <x:v>893</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="s">
         <x:v>894</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="s">
+      <x:c r="C4" s="15" t="s">
         <x:v>895</x:v>
-      </x:c>
-      <x:c r="C4" s="15" t="s">
-        <x:v>896</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.75" customHeight="1">
@@ -9931,7 +9928,7 @@
         <x:v>310</x:v>
       </x:c>
       <x:c r="B5" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C5" s="17"/>
     </x:row>
@@ -9940,7 +9937,7 @@
         <x:v>170</x:v>
       </x:c>
       <x:c r="B6" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C6" s="17"/>
     </x:row>
@@ -9949,16 +9946,16 @@
         <x:v>379</x:v>
       </x:c>
       <x:c r="B7" s="16" t="s">
-        <x:v>899</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="C7" s="17"/>
     </x:row>
     <x:row r="8" ht="26.75" customHeight="1">
       <x:c r="A8" s="16" t="s">
-        <x:v>456</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="B8" s="16" t="s">
-        <x:v>899</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="C8" s="17"/>
     </x:row>
@@ -9967,7 +9964,7 @@
         <x:v>347</x:v>
       </x:c>
       <x:c r="B9" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C9" s="17"/>
     </x:row>
@@ -9976,27 +9973,27 @@
         <x:v>368</x:v>
       </x:c>
       <x:c r="B10" s="16" t="s">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="s">
         <x:v>901</x:v>
-      </x:c>
-      <x:c r="C10" s="17" t="s">
-        <x:v>902</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.75" customHeight="1">
       <x:c r="A11" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="B11" s="16" t="s">
-        <x:v>899</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="C11" s="17"/>
     </x:row>
     <x:row r="12" ht="26.75" customHeight="1">
       <x:c r="A12" s="16" t="s">
+        <x:v>903</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="s">
         <x:v>904</x:v>
-      </x:c>
-      <x:c r="B12" s="16" t="s">
-        <x:v>905</x:v>
       </x:c>
       <x:c r="C12" s="17"/>
     </x:row>
@@ -10005,25 +10002,25 @@
         <x:v>303</x:v>
       </x:c>
       <x:c r="B13" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C13" s="17"/>
     </x:row>
     <x:row r="14" ht="26.75" customHeight="1">
       <x:c r="A14" s="16" t="s">
+        <x:v>905</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="s">
         <x:v>906</x:v>
-      </x:c>
-      <x:c r="B14" s="16" t="s">
-        <x:v>907</x:v>
       </x:c>
       <x:c r="C14" s="17"/>
     </x:row>
     <x:row r="15" ht="26.75" customHeight="1">
       <x:c r="A15" s="16" t="s">
+        <x:v>907</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="s">
         <x:v>908</x:v>
-      </x:c>
-      <x:c r="B15" s="16" t="s">
-        <x:v>909</x:v>
       </x:c>
       <x:c r="C15" s="17"/>
     </x:row>
@@ -10032,7 +10029,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B16" s="16" t="s">
-        <x:v>910</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="C16" s="17"/>
     </x:row>
@@ -10041,7 +10038,7 @@
         <x:v>198</x:v>
       </x:c>
       <x:c r="B17" s="16" t="s">
-        <x:v>910</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="C17" s="17"/>
     </x:row>
@@ -10050,7 +10047,7 @@
         <x:v>405</x:v>
       </x:c>
       <x:c r="B18" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="C18" s="17"/>
     </x:row>
@@ -10059,25 +10056,25 @@
         <x:v>260</x:v>
       </x:c>
       <x:c r="B19" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C19" s="17"/>
     </x:row>
     <x:row r="20" ht="26.75" customHeight="1">
       <x:c r="A20" s="16" t="s">
-        <x:v>564</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="B20" s="16" t="s">
-        <x:v>909</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C20" s="17"/>
     </x:row>
     <x:row r="21" ht="26.75" customHeight="1">
       <x:c r="A21" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="B21" s="16" t="s">
-        <x:v>909</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C21" s="17"/>
     </x:row>
@@ -10086,25 +10083,25 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B22" s="16" t="s">
-        <x:v>909</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C22" s="17"/>
     </x:row>
     <x:row r="23" ht="26.75" customHeight="1">
       <x:c r="A23" s="16" t="s">
+        <x:v>911</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="s">
         <x:v>912</x:v>
-      </x:c>
-      <x:c r="B23" s="16" t="s">
-        <x:v>913</x:v>
       </x:c>
       <x:c r="C23" s="17"/>
     </x:row>
     <x:row r="24" ht="26.75" customHeight="1">
       <x:c r="A24" s="16" t="s">
-        <x:v>914</x:v>
+        <x:v>913</x:v>
       </x:c>
       <x:c r="B24" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
     </x:row>
@@ -10113,36 +10110,36 @@
         <x:v>325</x:v>
       </x:c>
       <x:c r="B25" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
     </x:row>
     <x:row r="26" ht="26.75" customHeight="1">
       <x:c r="A26" s="16" t="s">
-        <x:v>466</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="B26" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
     </x:row>
     <x:row r="27" ht="26.75" customHeight="1">
       <x:c r="A27" s="16" t="s">
-        <x:v>556</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="B27" s="16" t="s">
-        <x:v>901</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C27" s="17" t="s">
-        <x:v>915</x:v>
+        <x:v>914</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="26.75" customHeight="1">
       <x:c r="A28" s="16" t="s">
-        <x:v>916</x:v>
+        <x:v>915</x:v>
       </x:c>
       <x:c r="B28" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>912</x:v>
       </x:c>
       <x:c r="C28" s="17"/>
     </x:row>
@@ -10151,7 +10148,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B29" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>912</x:v>
       </x:c>
       <x:c r="C29" s="17"/>
     </x:row>
@@ -10160,7 +10157,7 @@
         <x:v>191</x:v>
       </x:c>
       <x:c r="B30" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>912</x:v>
       </x:c>
       <x:c r="C30" s="17"/>
     </x:row>
@@ -10169,25 +10166,25 @@
         <x:v>141</x:v>
       </x:c>
       <x:c r="B31" s="16" t="s">
-        <x:v>910</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="C31" s="17"/>
     </x:row>
     <x:row r="32" ht="26.75" customHeight="1">
       <x:c r="A32" s="16" t="s">
-        <x:v>551</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="B32" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="C32" s="17"/>
     </x:row>
     <x:row r="33" ht="26.75" customHeight="1">
       <x:c r="A33" s="16" t="s">
-        <x:v>917</x:v>
+        <x:v>916</x:v>
       </x:c>
       <x:c r="B33" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="C33" s="17"/>
     </x:row>
@@ -10196,16 +10193,16 @@
         <x:v>318</x:v>
       </x:c>
       <x:c r="B34" s="16" t="s">
-        <x:v>899</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="C34" s="17"/>
     </x:row>
     <x:row r="35" ht="26.75" customHeight="1">
       <x:c r="A35" s="16" t="s">
-        <x:v>506</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="B35" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C35" s="17"/>
     </x:row>
@@ -10214,18 +10211,18 @@
         <x:v>268</x:v>
       </x:c>
       <x:c r="B36" s="16" t="s">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C36" s="17" t="s">
         <x:v>901</x:v>
-      </x:c>
-      <x:c r="C36" s="17" t="s">
-        <x:v>902</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="26.75" customHeight="1">
       <x:c r="A37" s="16" t="s">
-        <x:v>918</x:v>
+        <x:v>917</x:v>
       </x:c>
       <x:c r="B37" s="16" t="s">
-        <x:v>910</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="C37" s="17"/>
     </x:row>
@@ -10234,7 +10231,7 @@
         <x:v>177</x:v>
       </x:c>
       <x:c r="B38" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C38" s="17"/>
     </x:row>
@@ -10243,10 +10240,10 @@
         <x:v>239</x:v>
       </x:c>
       <x:c r="B39" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="C39" s="17" t="s">
-        <x:v>919</x:v>
+        <x:v>918</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="26.75" customHeight="1">
@@ -10254,25 +10251,25 @@
         <x:v>445</x:v>
       </x:c>
       <x:c r="B40" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="C40" s="17"/>
     </x:row>
     <x:row r="41" ht="26.75" customHeight="1">
       <x:c r="A41" s="16" t="s">
-        <x:v>920</x:v>
+        <x:v>919</x:v>
       </x:c>
       <x:c r="B41" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="C41" s="17"/>
     </x:row>
     <x:row r="42" ht="26.75" customHeight="1">
       <x:c r="A42" s="16" t="s">
-        <x:v>921</x:v>
+        <x:v>920</x:v>
       </x:c>
       <x:c r="B42" s="16" t="s">
-        <x:v>909</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C42" s="17"/>
     </x:row>
@@ -10281,10 +10278,10 @@
         <x:v>224</x:v>
       </x:c>
       <x:c r="B43" s="16" t="s">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C43" s="17" t="s">
         <x:v>901</x:v>
-      </x:c>
-      <x:c r="C43" s="17" t="s">
-        <x:v>902</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="26.75" customHeight="1">
@@ -10292,7 +10289,7 @@
         <x:v>182</x:v>
       </x:c>
       <x:c r="B44" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C44" s="17"/>
     </x:row>
@@ -10301,16 +10298,16 @@
         <x:v>162</x:v>
       </x:c>
       <x:c r="B45" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C45" s="17"/>
     </x:row>
     <x:row r="46" ht="26.75" customHeight="1">
       <x:c r="A46" s="16" t="s">
-        <x:v>922</x:v>
+        <x:v>921</x:v>
       </x:c>
       <x:c r="B46" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C46" s="17"/>
     </x:row>
@@ -10319,19 +10316,19 @@
         <x:v>156</x:v>
       </x:c>
       <x:c r="B47" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C47" s="17"/>
     </x:row>
     <x:row r="48" ht="26.75" customHeight="1">
       <x:c r="A48" s="16" t="s">
+        <x:v>922</x:v>
+      </x:c>
+      <x:c r="B48" s="16" t="s">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C48" s="17" t="s">
         <x:v>923</x:v>
-      </x:c>
-      <x:c r="B48" s="16" t="s">
-        <x:v>901</x:v>
-      </x:c>
-      <x:c r="C48" s="17" t="s">
-        <x:v>924</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="26.75" customHeight="1">
@@ -10339,7 +10336,7 @@
         <x:v>286</x:v>
       </x:c>
       <x:c r="B49" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C49" s="17"/>
     </x:row>
@@ -10348,16 +10345,16 @@
         <x:v>212</x:v>
       </x:c>
       <x:c r="B50" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C50" s="17"/>
     </x:row>
     <x:row r="51" ht="26.75" customHeight="1">
       <x:c r="A51" s="16" t="s">
-        <x:v>925</x:v>
+        <x:v>924</x:v>
       </x:c>
       <x:c r="B51" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C51" s="17"/>
     </x:row>
@@ -10366,38 +10363,38 @@
         <x:v>232</x:v>
       </x:c>
       <x:c r="B52" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>912</x:v>
       </x:c>
       <x:c r="C52" s="17"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" t="s">
-        <x:v>574</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="B53" t="s">
         <x:v>379</x:v>
       </x:c>
       <x:c r="C53" t="s">
-        <x:v>926</x:v>
+        <x:v>925</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" t="s">
-        <x:v>583</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="B54" t="s">
-        <x:v>901</x:v>
+        <x:v>900</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" t="s">
-        <x:v>590</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="B55" t="s">
-        <x:v>899</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="C55" t="s">
-        <x:v>927</x:v>
+        <x:v>926</x:v>
       </x:c>
     </x:row>
     <x:row r="56">

</xml_diff>

<commit_message>
Clarify Cybrdeck credit award value
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Re0c04f97a6f84395"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R92026aed3fc64568"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rfed7be8c2c3543cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Rc24012c213284865"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R00c80d8725c847ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R7bbd9a769e0a4101"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R6d2dd8a32ce94e28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R51a7f1b3aea84553"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1697,9 +1697,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">15/08/2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Best Vertical Solution (Family Office Track), 25USD + 2000 in app credits worth of Cybrdeck API credits</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Family Office</x:t>
@@ -7064,20 +7061,20 @@
       <x:c r="F76" s="12" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="G76" s="12" t="s">
+      <x:c r="G76" s="12" t="str">
+        <x:v>Best Vertical Solution (Family Office Track), 2,000 Cybrdeck API credits (worth US$25)</x:v>
+      </x:c>
+      <x:c r="H76" s="12" t="s">
         <x:v>562</x:v>
       </x:c>
-      <x:c r="H76" s="12" t="s">
+      <x:c r="I76" s="12" t="s">
         <x:v>563</x:v>
       </x:c>
-      <x:c r="I76" s="12" t="s">
+      <x:c r="J76" s="12" t="s">
         <x:v>564</x:v>
       </x:c>
-      <x:c r="J76" s="12" t="s">
+      <x:c r="K76" s="12" t="s">
         <x:v>565</x:v>
-      </x:c>
-      <x:c r="K76" s="12" t="s">
-        <x:v>566</x:v>
       </x:c>
       <x:c r="L76" s="12" t="s">
         <x:v>560</x:v>
@@ -7086,13 +7083,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N76" s="12" t="s">
+        <x:v>566</x:v>
+      </x:c>
+      <x:c r="O76" s="1" t="s">
         <x:v>567</x:v>
       </x:c>
-      <x:c r="O76" s="1" t="s">
+      <x:c r="P76" t="s">
         <x:v>568</x:v>
-      </x:c>
-      <x:c r="P76" t="s">
-        <x:v>569</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -7100,13 +7097,13 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B77" t="s">
+        <x:v>569</x:v>
+      </x:c>
+      <x:c r="C77" t="s">
         <x:v>570</x:v>
       </x:c>
-      <x:c r="C77" t="s">
+      <x:c r="D77" t="s">
         <x:v>571</x:v>
-      </x:c>
-      <x:c r="D77" t="s">
-        <x:v>572</x:v>
       </x:c>
       <x:c r="E77">
         <x:v>1</x:v>
@@ -7118,31 +7115,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H77" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="I77" t="s">
         <x:v>573</x:v>
-      </x:c>
-      <x:c r="I77" t="s">
-        <x:v>574</x:v>
       </x:c>
       <x:c r="J77" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K77" t="s">
+        <x:v>574</x:v>
+      </x:c>
+      <x:c r="L77" t="s">
         <x:v>575</x:v>
-      </x:c>
-      <x:c r="L77" t="s">
-        <x:v>576</x:v>
       </x:c>
       <x:c r="M77" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N77" t="s">
+        <x:v>576</x:v>
+      </x:c>
+      <x:c r="O77" t="s">
         <x:v>577</x:v>
       </x:c>
-      <x:c r="O77" t="s">
+      <x:c r="P77" t="s">
         <x:v>578</x:v>
-      </x:c>
-      <x:c r="P77" t="s">
-        <x:v>579</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -7150,13 +7147,13 @@
         <x:v>77</x:v>
       </x:c>
       <x:c r="B78" t="s">
-        <x:v>580</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="C78" t="s">
         <x:v>517</x:v>
       </x:c>
       <x:c r="D78" t="s">
-        <x:v>581</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="E78">
         <x:v>1</x:v>
@@ -7168,16 +7165,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H78" t="s">
+        <x:v>581</x:v>
+      </x:c>
+      <x:c r="I78" t="s">
         <x:v>582</x:v>
-      </x:c>
-      <x:c r="I78" t="s">
-        <x:v>583</x:v>
       </x:c>
       <x:c r="J78" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K78" t="s">
-        <x:v>584</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="L78" t="s">
         <x:v>517</x:v>
@@ -7189,7 +7186,7 @@
         <x:v>359</x:v>
       </x:c>
       <x:c r="O78" t="s">
-        <x:v>585</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="P78" t="s">
         <x:v>525</x:v>
@@ -7200,13 +7197,13 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="B79" t="s">
+        <x:v>585</x:v>
+      </x:c>
+      <x:c r="C79" t="s">
         <x:v>586</x:v>
       </x:c>
-      <x:c r="C79" t="s">
+      <x:c r="D79" t="s">
         <x:v>587</x:v>
-      </x:c>
-      <x:c r="D79" t="s">
-        <x:v>588</x:v>
       </x:c>
       <x:c r="E79">
         <x:v>4</x:v>
@@ -7218,19 +7215,19 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H79" t="s">
+        <x:v>588</x:v>
+      </x:c>
+      <x:c r="I79" t="s">
         <x:v>589</x:v>
       </x:c>
-      <x:c r="I79" t="s">
+      <x:c r="J79" t="s">
         <x:v>590</x:v>
       </x:c>
-      <x:c r="J79" t="s">
+      <x:c r="K79" t="s">
         <x:v>591</x:v>
       </x:c>
-      <x:c r="K79" t="s">
+      <x:c r="L79" t="s">
         <x:v>592</x:v>
-      </x:c>
-      <x:c r="L79" t="s">
-        <x:v>593</x:v>
       </x:c>
       <x:c r="M79" t="s">
         <x:v>26</x:v>
@@ -7239,10 +7236,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="O79" t="s">
+        <x:v>593</x:v>
+      </x:c>
+      <x:c r="P79" t="s">
         <x:v>594</x:v>
-      </x:c>
-      <x:c r="P79" t="s">
-        <x:v>595</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -7395,10 +7392,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rfd28d8fbb5354157"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R7e5644dcb48e4150"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Ra1dcce16a7064cf6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R7c13ec40084d41f0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Re26bd447967545c1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R2d1af01fc7934f9e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Raf810d0659c449d2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Reac6b8f89afe446f"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7421,7 +7418,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>596</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -7430,7 +7427,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="19" t="s">
-        <x:v>597</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="B2" s="19"/>
       <x:c r="C2" s="19"/>
@@ -7439,64 +7436,64 @@
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="11" t="s">
+        <x:v>597</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="s">
         <x:v>598</x:v>
       </x:c>
-      <x:c r="B4" s="11" t="s">
+      <x:c r="C4" s="11" t="s">
         <x:v>599</x:v>
       </x:c>
-      <x:c r="C4" s="11" t="s">
+      <x:c r="D4" s="11" t="s">
         <x:v>600</x:v>
       </x:c>
-      <x:c r="D4" s="11" t="s">
+      <x:c r="E4" s="11" t="s">
         <x:v>601</x:v>
-      </x:c>
-      <x:c r="E4" s="11" t="s">
-        <x:v>602</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="8" t="s">
+        <x:v>602</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="s">
         <x:v>603</x:v>
       </x:c>
-      <x:c r="B5" s="7" t="s">
+      <x:c r="C5" s="7" t="s">
         <x:v>604</x:v>
-      </x:c>
-      <x:c r="C5" s="7" t="s">
-        <x:v>605</x:v>
       </x:c>
       <x:c r="D5" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E5" s="10" t="s">
-        <x:v>606</x:v>
+        <x:v>605</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="8" t="s">
+        <x:v>606</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>607</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="s">
+      <x:c r="C6" s="7" t="s">
         <x:v>608</x:v>
       </x:c>
-      <x:c r="C6" s="7" t="s">
+      <x:c r="D6" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="s">
         <x:v>609</x:v>
-      </x:c>
-      <x:c r="D6" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E6" s="10" t="s">
-        <x:v>610</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="8" t="s">
+        <x:v>610</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
         <x:v>611</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="s">
+      <x:c r="C7" s="7" t="s">
         <x:v>612</x:v>
-      </x:c>
-      <x:c r="C7" s="7" t="s">
-        <x:v>613</x:v>
       </x:c>
       <x:c r="D7" s="9">
         <x:v>1</x:v>
@@ -7505,47 +7502,47 @@
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
       <x:c r="A8" s="8" t="s">
+        <x:v>613</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
         <x:v>614</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="s">
+      <x:c r="C8" s="7" t="s">
         <x:v>615</x:v>
       </x:c>
-      <x:c r="C8" s="7" t="s">
+      <x:c r="D8" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="s">
         <x:v>616</x:v>
-      </x:c>
-      <x:c r="D8" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E8" s="10" t="s">
-        <x:v>617</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" s="8" t="s">
+        <x:v>617</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
         <x:v>618</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="s">
+      <x:c r="C9" s="7" t="s">
+        <x:v>608</x:v>
+      </x:c>
+      <x:c r="D9" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="s">
         <x:v>619</x:v>
-      </x:c>
-      <x:c r="C9" s="7" t="s">
-        <x:v>609</x:v>
-      </x:c>
-      <x:c r="D9" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E9" s="10" t="s">
-        <x:v>620</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
       <x:c r="A10" s="8" t="s">
+        <x:v>620</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="s">
         <x:v>621</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="s">
+      <x:c r="C10" s="7" t="s">
         <x:v>622</x:v>
-      </x:c>
-      <x:c r="C10" s="7" t="s">
-        <x:v>623</x:v>
       </x:c>
       <x:c r="D10" s="9">
         <x:v>1</x:v>
@@ -7554,47 +7551,47 @@
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
       <x:c r="A11" s="8" t="s">
+        <x:v>623</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="s">
         <x:v>624</x:v>
       </x:c>
-      <x:c r="B11" s="7" t="s">
+      <x:c r="C11" s="7" t="s">
         <x:v>625</x:v>
       </x:c>
-      <x:c r="C11" s="7" t="s">
+      <x:c r="D11" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="10" t="s">
         <x:v>626</x:v>
-      </x:c>
-      <x:c r="D11" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E11" s="10" t="s">
-        <x:v>627</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
       <x:c r="A12" s="8" t="s">
+        <x:v>627</x:v>
+      </x:c>
+      <x:c r="B12" s="7" t="s">
         <x:v>628</x:v>
       </x:c>
-      <x:c r="B12" s="7" t="s">
+      <x:c r="C12" s="7" t="s">
         <x:v>629</x:v>
       </x:c>
-      <x:c r="C12" s="7" t="s">
+      <x:c r="D12" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="s">
         <x:v>630</x:v>
-      </x:c>
-      <x:c r="D12" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E12" s="10" t="s">
-        <x:v>631</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
       <x:c r="A13" s="8" t="s">
+        <x:v>631</x:v>
+      </x:c>
+      <x:c r="B13" s="7" t="s">
         <x:v>632</x:v>
       </x:c>
-      <x:c r="B13" s="7" t="s">
+      <x:c r="C13" s="7" t="s">
         <x:v>633</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="s">
-        <x:v>634</x:v>
       </x:c>
       <x:c r="D13" s="9">
         <x:v>1</x:v>
@@ -7603,30 +7600,30 @@
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
       <x:c r="A14" s="8" t="s">
+        <x:v>634</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="s">
         <x:v>635</x:v>
       </x:c>
-      <x:c r="B14" s="7" t="s">
+      <x:c r="C14" s="7" t="s">
+        <x:v>633</x:v>
+      </x:c>
+      <x:c r="D14" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="s">
         <x:v>636</x:v>
-      </x:c>
-      <x:c r="C14" s="7" t="s">
-        <x:v>634</x:v>
-      </x:c>
-      <x:c r="D14" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E14" s="10" t="s">
-        <x:v>637</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
       <x:c r="A15" s="8" t="s">
+        <x:v>637</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="s">
         <x:v>638</x:v>
       </x:c>
-      <x:c r="B15" s="7" t="s">
+      <x:c r="C15" s="7" t="s">
         <x:v>639</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="s">
-        <x:v>640</x:v>
       </x:c>
       <x:c r="D15" s="9">
         <x:v>1</x:v>
@@ -7635,30 +7632,30 @@
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
       <x:c r="A16" s="8" t="s">
+        <x:v>640</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="s">
         <x:v>641</x:v>
       </x:c>
-      <x:c r="B16" s="7" t="s">
+      <x:c r="C16" s="7" t="s">
         <x:v>642</x:v>
       </x:c>
-      <x:c r="C16" s="7" t="s">
+      <x:c r="D16" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="s">
         <x:v>643</x:v>
-      </x:c>
-      <x:c r="D16" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E16" s="10" t="s">
-        <x:v>644</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
       <x:c r="A17" s="8" t="s">
+        <x:v>644</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="s">
         <x:v>645</x:v>
       </x:c>
-      <x:c r="B17" s="7" t="s">
+      <x:c r="C17" s="7" t="s">
         <x:v>646</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="s">
-        <x:v>647</x:v>
       </x:c>
       <x:c r="D17" s="9">
         <x:v>1</x:v>
@@ -7667,47 +7664,47 @@
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
       <x:c r="A18" s="8" t="s">
+        <x:v>647</x:v>
+      </x:c>
+      <x:c r="B18" s="7" t="s">
         <x:v>648</x:v>
       </x:c>
-      <x:c r="B18" s="7" t="s">
+      <x:c r="C18" s="7" t="s">
         <x:v>649</x:v>
       </x:c>
-      <x:c r="C18" s="7" t="s">
+      <x:c r="D18" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="s">
         <x:v>650</x:v>
-      </x:c>
-      <x:c r="D18" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E18" s="10" t="s">
-        <x:v>651</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
       <x:c r="A19" s="8" t="s">
+        <x:v>651</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="s">
         <x:v>652</x:v>
       </x:c>
-      <x:c r="B19" s="7" t="s">
+      <x:c r="C19" s="7" t="s">
         <x:v>653</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="s">
-        <x:v>654</x:v>
       </x:c>
       <x:c r="D19" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E19" s="10" t="s">
-        <x:v>655</x:v>
+        <x:v>654</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28" customHeight="1">
       <x:c r="A20" s="8" t="s">
+        <x:v>655</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="s">
         <x:v>656</x:v>
       </x:c>
-      <x:c r="B20" s="7" t="s">
+      <x:c r="C20" s="7" t="s">
         <x:v>657</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>658</x:v>
       </x:c>
       <x:c r="D20" s="9">
         <x:v>1</x:v>
@@ -7716,10 +7713,10 @@
     </x:row>
     <x:row r="21" ht="28" customHeight="1">
       <x:c r="A21" s="8" t="s">
+        <x:v>658</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="s">
         <x:v>659</x:v>
-      </x:c>
-      <x:c r="B21" s="7" t="s">
-        <x:v>660</x:v>
       </x:c>
       <x:c r="C21" s="7" t="str">
         <x:v>#069, #071, #079</x:v>
@@ -7728,18 +7725,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E21" s="10" t="s">
-        <x:v>661</x:v>
+        <x:v>660</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
       <x:c r="A22" s="8" t="s">
+        <x:v>661</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="s">
         <x:v>662</x:v>
       </x:c>
-      <x:c r="B22" s="7" t="s">
+      <x:c r="C22" s="7" t="s">
         <x:v>663</x:v>
-      </x:c>
-      <x:c r="C22" s="7" t="s">
-        <x:v>664</x:v>
       </x:c>
       <x:c r="D22" s="9">
         <x:v>1</x:v>
@@ -7748,13 +7745,13 @@
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
       <x:c r="A23" s="8" t="s">
+        <x:v>664</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="s">
         <x:v>665</x:v>
       </x:c>
-      <x:c r="B23" s="7" t="s">
+      <x:c r="C23" s="7" t="s">
         <x:v>666</x:v>
-      </x:c>
-      <x:c r="C23" s="7" t="s">
-        <x:v>667</x:v>
       </x:c>
       <x:c r="D23" s="9">
         <x:v>1</x:v>
@@ -7763,10 +7760,10 @@
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
       <x:c r="A24" s="8" t="s">
+        <x:v>667</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="s">
         <x:v>668</x:v>
-      </x:c>
-      <x:c r="B24" s="7" t="s">
-        <x:v>669</x:v>
       </x:c>
       <x:c r="C24" s="7" t="str">
         <x:v>#054, #055, #056, #062, #066, #068, #075</x:v>
@@ -7775,12 +7772,12 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E24" s="10" t="s">
-        <x:v>670</x:v>
+        <x:v>669</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
       <x:c r="A25" s="8" t="s">
-        <x:v>671</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
         <x:v>Clement Lork</x:v>
@@ -7792,18 +7789,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E25" s="10" t="s">
-        <x:v>672</x:v>
+        <x:v>671</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="8" t="s">
+        <x:v>672</x:v>
+      </x:c>
+      <x:c r="B26" s="7" t="s">
         <x:v>673</x:v>
       </x:c>
-      <x:c r="B26" s="7" t="s">
-        <x:v>674</x:v>
-      </x:c>
       <x:c r="C26" s="7" t="s">
-        <x:v>613</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="D26" s="9">
         <x:v>1</x:v>
@@ -7812,13 +7809,13 @@
     </x:row>
     <x:row r="27" ht="28" customHeight="1">
       <x:c r="A27" s="8" t="s">
+        <x:v>674</x:v>
+      </x:c>
+      <x:c r="B27" s="7" t="s">
         <x:v>675</x:v>
       </x:c>
-      <x:c r="B27" s="7" t="s">
+      <x:c r="C27" s="7" t="s">
         <x:v>676</x:v>
-      </x:c>
-      <x:c r="C27" s="7" t="s">
-        <x:v>677</x:v>
       </x:c>
       <x:c r="D27" s="9">
         <x:v>1</x:v>
@@ -7827,13 +7824,13 @@
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
       <x:c r="A28" s="8" t="s">
+        <x:v>677</x:v>
+      </x:c>
+      <x:c r="B28" s="7" t="s">
         <x:v>678</x:v>
       </x:c>
-      <x:c r="B28" s="7" t="s">
+      <x:c r="C28" s="7" t="s">
         <x:v>679</x:v>
-      </x:c>
-      <x:c r="C28" s="7" t="s">
-        <x:v>680</x:v>
       </x:c>
       <x:c r="D28" s="9">
         <x:v>2</x:v>
@@ -7842,13 +7839,13 @@
     </x:row>
     <x:row r="29" ht="28" customHeight="1">
       <x:c r="A29" s="8" t="s">
+        <x:v>680</x:v>
+      </x:c>
+      <x:c r="B29" s="7" t="s">
         <x:v>681</x:v>
       </x:c>
-      <x:c r="B29" s="7" t="s">
+      <x:c r="C29" s="7" t="s">
         <x:v>682</x:v>
-      </x:c>
-      <x:c r="C29" s="7" t="s">
-        <x:v>683</x:v>
       </x:c>
       <x:c r="D29" s="9">
         <x:v>4</x:v>
@@ -7857,13 +7854,13 @@
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
       <x:c r="A30" s="8" t="s">
+        <x:v>683</x:v>
+      </x:c>
+      <x:c r="B30" s="7" t="s">
         <x:v>684</x:v>
       </x:c>
-      <x:c r="B30" s="7" t="s">
-        <x:v>685</x:v>
-      </x:c>
       <x:c r="C30" s="7" t="s">
-        <x:v>677</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="D30" s="9">
         <x:v>1</x:v>
@@ -7872,47 +7869,47 @@
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="8" t="s">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="B31" s="7" t="s">
         <x:v>686</x:v>
       </x:c>
-      <x:c r="B31" s="7" t="s">
+      <x:c r="C31" s="7" t="s">
+        <x:v>625</x:v>
+      </x:c>
+      <x:c r="D31" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E31" s="10" t="s">
         <x:v>687</x:v>
-      </x:c>
-      <x:c r="C31" s="7" t="s">
-        <x:v>626</x:v>
-      </x:c>
-      <x:c r="D31" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E31" s="10" t="s">
-        <x:v>688</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="28" customHeight="1">
       <x:c r="A32" s="8" t="s">
+        <x:v>688</x:v>
+      </x:c>
+      <x:c r="B32" s="7" t="s">
         <x:v>689</x:v>
       </x:c>
-      <x:c r="B32" s="7" t="s">
+      <x:c r="C32" s="7" t="s">
         <x:v>690</x:v>
       </x:c>
-      <x:c r="C32" s="7" t="s">
+      <x:c r="D32" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E32" s="10" t="s">
         <x:v>691</x:v>
-      </x:c>
-      <x:c r="D32" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E32" s="10" t="s">
-        <x:v>692</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="8" t="s">
+        <x:v>692</x:v>
+      </x:c>
+      <x:c r="B33" s="7" t="s">
         <x:v>693</x:v>
       </x:c>
-      <x:c r="B33" s="7" t="s">
-        <x:v>694</x:v>
-      </x:c>
       <x:c r="C33" s="7" t="s">
-        <x:v>664</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="D33" s="9">
         <x:v>1</x:v>
@@ -7921,13 +7918,13 @@
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
       <x:c r="A34" s="8" t="s">
+        <x:v>694</x:v>
+      </x:c>
+      <x:c r="B34" s="7" t="s">
         <x:v>695</x:v>
       </x:c>
-      <x:c r="B34" s="7" t="s">
+      <x:c r="C34" s="7" t="s">
         <x:v>696</x:v>
-      </x:c>
-      <x:c r="C34" s="7" t="s">
-        <x:v>697</x:v>
       </x:c>
       <x:c r="D34" s="9">
         <x:v>1</x:v>
@@ -7936,47 +7933,47 @@
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
       <x:c r="A35" s="8" t="s">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="B35" s="7" t="s">
         <x:v>698</x:v>
       </x:c>
-      <x:c r="B35" s="7" t="s">
+      <x:c r="C35" s="7" t="s">
         <x:v>699</x:v>
       </x:c>
-      <x:c r="C35" s="7" t="s">
+      <x:c r="D35" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E35" s="10" t="s">
         <x:v>700</x:v>
-      </x:c>
-      <x:c r="D35" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E35" s="10" t="s">
-        <x:v>701</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
       <x:c r="A36" s="8" t="s">
+        <x:v>701</x:v>
+      </x:c>
+      <x:c r="B36" s="7" t="s">
         <x:v>702</x:v>
       </x:c>
-      <x:c r="B36" s="7" t="s">
+      <x:c r="C36" s="7" t="s">
         <x:v>703</x:v>
       </x:c>
-      <x:c r="C36" s="7" t="s">
+      <x:c r="D36" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E36" s="10" t="s">
         <x:v>704</x:v>
-      </x:c>
-      <x:c r="D36" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E36" s="10" t="s">
-        <x:v>705</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
       <x:c r="A37" s="8" t="s">
+        <x:v>705</x:v>
+      </x:c>
+      <x:c r="B37" s="7" t="s">
         <x:v>706</x:v>
       </x:c>
-      <x:c r="B37" s="7" t="s">
+      <x:c r="C37" s="7" t="s">
         <x:v>707</x:v>
-      </x:c>
-      <x:c r="C37" s="7" t="s">
-        <x:v>708</x:v>
       </x:c>
       <x:c r="D37" s="9">
         <x:v>1</x:v>
@@ -7985,13 +7982,13 @@
     </x:row>
     <x:row r="38" ht="28" customHeight="1">
       <x:c r="A38" s="8" t="s">
+        <x:v>708</x:v>
+      </x:c>
+      <x:c r="B38" s="7" t="s">
         <x:v>709</x:v>
       </x:c>
-      <x:c r="B38" s="7" t="s">
-        <x:v>710</x:v>
-      </x:c>
       <x:c r="C38" s="7" t="s">
-        <x:v>647</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="D38" s="9">
         <x:v>1</x:v>
@@ -8000,13 +7997,13 @@
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
       <x:c r="A39" s="8" t="s">
+        <x:v>710</x:v>
+      </x:c>
+      <x:c r="B39" s="7" t="s">
         <x:v>711</x:v>
       </x:c>
-      <x:c r="B39" s="7" t="s">
+      <x:c r="C39" s="7" t="s">
         <x:v>712</x:v>
-      </x:c>
-      <x:c r="C39" s="7" t="s">
-        <x:v>713</x:v>
       </x:c>
       <x:c r="D39" s="9">
         <x:v>3</x:v>
@@ -8015,47 +8012,47 @@
     </x:row>
     <x:row r="40" ht="28" customHeight="1">
       <x:c r="A40" s="8" t="s">
+        <x:v>713</x:v>
+      </x:c>
+      <x:c r="B40" s="7" t="s">
         <x:v>714</x:v>
       </x:c>
-      <x:c r="B40" s="7" t="s">
+      <x:c r="C40" s="7" t="s">
         <x:v>715</x:v>
       </x:c>
-      <x:c r="C40" s="7" t="s">
+      <x:c r="D40" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E40" s="10" t="s">
         <x:v>716</x:v>
-      </x:c>
-      <x:c r="D40" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E40" s="10" t="s">
-        <x:v>717</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="8" t="s">
+        <x:v>717</x:v>
+      </x:c>
+      <x:c r="B41" s="7" t="s">
         <x:v>718</x:v>
       </x:c>
-      <x:c r="B41" s="7" t="s">
+      <x:c r="C41" s="7" t="s">
+        <x:v>715</x:v>
+      </x:c>
+      <x:c r="D41" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E41" s="10" t="s">
         <x:v>719</x:v>
-      </x:c>
-      <x:c r="C41" s="7" t="s">
-        <x:v>716</x:v>
-      </x:c>
-      <x:c r="D41" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E41" s="10" t="s">
-        <x:v>720</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
       <x:c r="A42" s="8" t="s">
+        <x:v>720</x:v>
+      </x:c>
+      <x:c r="B42" s="7" t="s">
         <x:v>721</x:v>
       </x:c>
-      <x:c r="B42" s="7" t="s">
+      <x:c r="C42" s="7" t="s">
         <x:v>722</x:v>
-      </x:c>
-      <x:c r="C42" s="7" t="s">
-        <x:v>723</x:v>
       </x:c>
       <x:c r="D42" s="9">
         <x:v>1</x:v>
@@ -8064,10 +8061,10 @@
     </x:row>
     <x:row r="43" ht="28" customHeight="1">
       <x:c r="A43" s="8" t="s">
+        <x:v>723</x:v>
+      </x:c>
+      <x:c r="B43" s="7" t="s">
         <x:v>724</x:v>
-      </x:c>
-      <x:c r="B43" s="7" t="s">
-        <x:v>725</x:v>
       </x:c>
       <x:c r="C43" s="7" t="str">
         <x:v>#069, #079</x:v>
@@ -8079,30 +8076,30 @@
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="8" t="s">
+        <x:v>725</x:v>
+      </x:c>
+      <x:c r="B44" s="7" t="s">
         <x:v>726</x:v>
       </x:c>
-      <x:c r="B44" s="7" t="s">
-        <x:v>727</x:v>
-      </x:c>
       <x:c r="C44" s="7" t="s">
-        <x:v>680</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="D44" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E44" s="10" t="s">
-        <x:v>728</x:v>
+        <x:v>727</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
       <x:c r="A45" s="8" t="s">
+        <x:v>728</x:v>
+      </x:c>
+      <x:c r="B45" s="7" t="s">
         <x:v>729</x:v>
       </x:c>
-      <x:c r="B45" s="7" t="s">
+      <x:c r="C45" s="7" t="s">
         <x:v>730</x:v>
-      </x:c>
-      <x:c r="C45" s="7" t="s">
-        <x:v>731</x:v>
       </x:c>
       <x:c r="D45" s="9">
         <x:v>1</x:v>
@@ -8111,13 +8108,13 @@
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
       <x:c r="A46" s="8" t="s">
+        <x:v>731</x:v>
+      </x:c>
+      <x:c r="B46" s="7" t="s">
         <x:v>732</x:v>
       </x:c>
-      <x:c r="B46" s="7" t="s">
-        <x:v>733</x:v>
-      </x:c>
       <x:c r="C46" s="7" t="s">
-        <x:v>697</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="D46" s="9">
         <x:v>1</x:v>
@@ -8126,47 +8123,47 @@
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
       <x:c r="A47" s="8" t="s">
+        <x:v>733</x:v>
+      </x:c>
+      <x:c r="B47" s="7" t="s">
         <x:v>734</x:v>
       </x:c>
-      <x:c r="B47" s="7" t="s">
+      <x:c r="C47" s="7" t="s">
+        <x:v>608</x:v>
+      </x:c>
+      <x:c r="D47" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E47" s="10" t="s">
         <x:v>735</x:v>
-      </x:c>
-      <x:c r="C47" s="7" t="s">
-        <x:v>609</x:v>
-      </x:c>
-      <x:c r="D47" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E47" s="10" t="s">
-        <x:v>736</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
       <x:c r="A48" s="8" t="s">
+        <x:v>736</x:v>
+      </x:c>
+      <x:c r="B48" s="7" t="s">
         <x:v>737</x:v>
       </x:c>
-      <x:c r="B48" s="7" t="s">
+      <x:c r="C48" s="7" t="s">
         <x:v>738</x:v>
-      </x:c>
-      <x:c r="C48" s="7" t="s">
-        <x:v>739</x:v>
       </x:c>
       <x:c r="D48" s="9">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="10" t="s">
-        <x:v>740</x:v>
+        <x:v>739</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
       <x:c r="A49" s="8" t="s">
+        <x:v>740</x:v>
+      </x:c>
+      <x:c r="B49" s="7" t="s">
         <x:v>741</x:v>
       </x:c>
-      <x:c r="B49" s="7" t="s">
+      <x:c r="C49" s="7" t="s">
         <x:v>742</x:v>
-      </x:c>
-      <x:c r="C49" s="7" t="s">
-        <x:v>743</x:v>
       </x:c>
       <x:c r="D49" s="9">
         <x:v>1</x:v>
@@ -8175,13 +8172,13 @@
     </x:row>
     <x:row r="50" ht="28" customHeight="1">
       <x:c r="A50" s="8" t="s">
+        <x:v>743</x:v>
+      </x:c>
+      <x:c r="B50" s="7" t="s">
         <x:v>744</x:v>
       </x:c>
-      <x:c r="B50" s="7" t="s">
-        <x:v>745</x:v>
-      </x:c>
       <x:c r="C50" s="7" t="s">
-        <x:v>708</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="D50" s="9">
         <x:v>1</x:v>
@@ -8190,64 +8187,64 @@
     </x:row>
     <x:row r="51" ht="28" customHeight="1">
       <x:c r="A51" s="8" t="s">
+        <x:v>745</x:v>
+      </x:c>
+      <x:c r="B51" s="7" t="s">
         <x:v>746</x:v>
       </x:c>
-      <x:c r="B51" s="7" t="s">
+      <x:c r="C51" s="7" t="s">
         <x:v>747</x:v>
-      </x:c>
-      <x:c r="C51" s="7" t="s">
-        <x:v>748</x:v>
       </x:c>
       <x:c r="D51" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E51" s="10" t="s">
-        <x:v>749</x:v>
+        <x:v>748</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="28" customHeight="1">
       <x:c r="A52" s="8" t="s">
+        <x:v>749</x:v>
+      </x:c>
+      <x:c r="B52" s="7" t="s">
         <x:v>750</x:v>
       </x:c>
-      <x:c r="B52" s="7" t="s">
+      <x:c r="C52" s="7" t="s">
         <x:v>751</x:v>
       </x:c>
-      <x:c r="C52" s="7" t="s">
+      <x:c r="D52" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E52" s="10" t="s">
         <x:v>752</x:v>
-      </x:c>
-      <x:c r="D52" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E52" s="10" t="s">
-        <x:v>753</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="28" customHeight="1">
       <x:c r="A53" s="8" t="s">
+        <x:v>753</x:v>
+      </x:c>
+      <x:c r="B53" s="7" t="s">
         <x:v>754</x:v>
       </x:c>
-      <x:c r="B53" s="7" t="s">
+      <x:c r="C53" s="7" t="s">
         <x:v>755</x:v>
-      </x:c>
-      <x:c r="C53" s="7" t="s">
-        <x:v>756</x:v>
       </x:c>
       <x:c r="D53" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E53" s="10" t="s">
-        <x:v>757</x:v>
+        <x:v>756</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="28" customHeight="1">
       <x:c r="A54" s="8" t="s">
+        <x:v>757</x:v>
+      </x:c>
+      <x:c r="B54" s="7" t="s">
         <x:v>758</x:v>
       </x:c>
-      <x:c r="B54" s="7" t="s">
+      <x:c r="C54" s="7" t="s">
         <x:v>759</x:v>
-      </x:c>
-      <x:c r="C54" s="7" t="s">
-        <x:v>760</x:v>
       </x:c>
       <x:c r="D54" s="9">
         <x:v>1</x:v>
@@ -8256,81 +8253,81 @@
     </x:row>
     <x:row r="55" ht="28" customHeight="1">
       <x:c r="A55" s="8" t="s">
+        <x:v>760</x:v>
+      </x:c>
+      <x:c r="B55" s="7" t="s">
         <x:v>761</x:v>
       </x:c>
-      <x:c r="B55" s="7" t="s">
+      <x:c r="C55" s="7" t="s">
         <x:v>762</x:v>
       </x:c>
-      <x:c r="C55" s="7" t="s">
+      <x:c r="D55" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E55" s="10" t="s">
         <x:v>763</x:v>
-      </x:c>
-      <x:c r="D55" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E55" s="10" t="s">
-        <x:v>764</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="28" customHeight="1">
       <x:c r="A56" s="8" t="s">
+        <x:v>764</x:v>
+      </x:c>
+      <x:c r="B56" s="7" t="s">
         <x:v>765</x:v>
       </x:c>
-      <x:c r="B56" s="7" t="s">
+      <x:c r="C56" s="7" t="s">
         <x:v>766</x:v>
       </x:c>
-      <x:c r="C56" s="7" t="s">
+      <x:c r="D56" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E56" s="10" t="s">
         <x:v>767</x:v>
-      </x:c>
-      <x:c r="D56" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E56" s="10" t="s">
-        <x:v>768</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
       <x:c r="A57" s="8" t="s">
+        <x:v>768</x:v>
+      </x:c>
+      <x:c r="B57" s="7" t="s">
         <x:v>769</x:v>
       </x:c>
-      <x:c r="B57" s="7" t="s">
+      <x:c r="C57" s="7" t="s">
         <x:v>770</x:v>
       </x:c>
-      <x:c r="C57" s="7" t="s">
+      <x:c r="D57" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E57" s="10" t="s">
         <x:v>771</x:v>
-      </x:c>
-      <x:c r="D57" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E57" s="10" t="s">
-        <x:v>772</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
       <x:c r="A58" s="8" t="s">
+        <x:v>772</x:v>
+      </x:c>
+      <x:c r="B58" s="7" t="s">
         <x:v>773</x:v>
       </x:c>
-      <x:c r="B58" s="7" t="s">
+      <x:c r="C58" s="7" t="s">
         <x:v>774</x:v>
-      </x:c>
-      <x:c r="C58" s="7" t="s">
-        <x:v>775</x:v>
       </x:c>
       <x:c r="D58" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E58" s="10" t="s">
-        <x:v>776</x:v>
+        <x:v>775</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
       <x:c r="A59" s="8" t="s">
+        <x:v>776</x:v>
+      </x:c>
+      <x:c r="B59" s="7" t="s">
         <x:v>777</x:v>
       </x:c>
-      <x:c r="B59" s="7" t="s">
-        <x:v>778</x:v>
-      </x:c>
       <x:c r="C59" s="7" t="s">
-        <x:v>613</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="D59" s="9">
         <x:v>1</x:v>
@@ -8339,13 +8336,13 @@
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
       <x:c r="A60" s="8" t="s">
+        <x:v>778</x:v>
+      </x:c>
+      <x:c r="B60" s="7" t="s">
         <x:v>779</x:v>
       </x:c>
-      <x:c r="B60" s="7" t="s">
-        <x:v>780</x:v>
-      </x:c>
       <x:c r="C60" s="7" t="s">
-        <x:v>650</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="D60" s="9">
         <x:v>1</x:v>
@@ -8354,13 +8351,13 @@
     </x:row>
     <x:row r="61" ht="28" customHeight="1">
       <x:c r="A61" s="8" t="s">
+        <x:v>780</x:v>
+      </x:c>
+      <x:c r="B61" s="7" t="s">
         <x:v>781</x:v>
       </x:c>
-      <x:c r="B61" s="7" t="s">
-        <x:v>782</x:v>
-      </x:c>
       <x:c r="C61" s="7" t="s">
-        <x:v>634</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="D61" s="9">
         <x:v>1</x:v>
@@ -8369,30 +8366,30 @@
     </x:row>
     <x:row r="62" ht="28" customHeight="1">
       <x:c r="A62" s="8" t="s">
+        <x:v>782</x:v>
+      </x:c>
+      <x:c r="B62" s="7" t="s">
         <x:v>783</x:v>
       </x:c>
-      <x:c r="B62" s="7" t="s">
+      <x:c r="C62" s="7" t="s">
+        <x:v>639</x:v>
+      </x:c>
+      <x:c r="D62" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E62" s="10" t="s">
         <x:v>784</x:v>
-      </x:c>
-      <x:c r="C62" s="7" t="s">
-        <x:v>640</x:v>
-      </x:c>
-      <x:c r="D62" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E62" s="10" t="s">
-        <x:v>785</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="28" customHeight="1">
       <x:c r="A63" s="8" t="s">
+        <x:v>785</x:v>
+      </x:c>
+      <x:c r="B63" s="7" t="s">
         <x:v>786</x:v>
       </x:c>
-      <x:c r="B63" s="7" t="s">
-        <x:v>787</x:v>
-      </x:c>
       <x:c r="C63" s="7" t="s">
-        <x:v>634</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="D63" s="9">
         <x:v>1</x:v>
@@ -8401,13 +8398,13 @@
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
       <x:c r="A64" s="8" t="s">
+        <x:v>787</x:v>
+      </x:c>
+      <x:c r="B64" s="7" t="s">
         <x:v>788</x:v>
       </x:c>
-      <x:c r="B64" s="7" t="s">
+      <x:c r="C64" s="7" t="s">
         <x:v>789</x:v>
-      </x:c>
-      <x:c r="C64" s="7" t="s">
-        <x:v>790</x:v>
       </x:c>
       <x:c r="D64" s="9">
         <x:v>1</x:v>
@@ -8416,13 +8413,13 @@
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
       <x:c r="A65" s="8" t="s">
+        <x:v>790</x:v>
+      </x:c>
+      <x:c r="B65" s="7" t="s">
         <x:v>791</x:v>
       </x:c>
-      <x:c r="B65" s="7" t="s">
+      <x:c r="C65" s="7" t="s">
         <x:v>792</x:v>
-      </x:c>
-      <x:c r="C65" s="7" t="s">
-        <x:v>793</x:v>
       </x:c>
       <x:c r="D65" s="9">
         <x:v>1</x:v>
@@ -8431,13 +8428,13 @@
     </x:row>
     <x:row r="66" ht="28" customHeight="1">
       <x:c r="A66" s="8" t="s">
+        <x:v>793</x:v>
+      </x:c>
+      <x:c r="B66" s="7" t="s">
         <x:v>794</x:v>
       </x:c>
-      <x:c r="B66" s="7" t="s">
-        <x:v>795</x:v>
-      </x:c>
       <x:c r="C66" s="7" t="s">
-        <x:v>623</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="D66" s="9">
         <x:v>1</x:v>
@@ -8446,47 +8443,47 @@
     </x:row>
     <x:row r="67" ht="28" customHeight="1">
       <x:c r="A67" s="8" t="s">
+        <x:v>795</x:v>
+      </x:c>
+      <x:c r="B67" s="7" t="s">
         <x:v>796</x:v>
       </x:c>
-      <x:c r="B67" s="7" t="s">
-        <x:v>797</x:v>
-      </x:c>
       <x:c r="C67" s="7" t="s">
-        <x:v>775</x:v>
+        <x:v>774</x:v>
       </x:c>
       <x:c r="D67" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E67" s="10" t="s">
-        <x:v>798</x:v>
+        <x:v>797</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="28" customHeight="1">
       <x:c r="A68" s="8" t="s">
+        <x:v>798</x:v>
+      </x:c>
+      <x:c r="B68" s="7" t="s">
         <x:v>799</x:v>
       </x:c>
-      <x:c r="B68" s="7" t="s">
+      <x:c r="C68" s="7" t="s">
+        <x:v>649</x:v>
+      </x:c>
+      <x:c r="D68" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E68" s="10" t="s">
         <x:v>800</x:v>
-      </x:c>
-      <x:c r="C68" s="7" t="s">
-        <x:v>650</x:v>
-      </x:c>
-      <x:c r="D68" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E68" s="10" t="s">
-        <x:v>801</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
       <x:c r="A69" s="8" t="s">
+        <x:v>801</x:v>
+      </x:c>
+      <x:c r="B69" s="7" t="s">
         <x:v>802</x:v>
       </x:c>
-      <x:c r="B69" s="7" t="s">
-        <x:v>803</x:v>
-      </x:c>
       <x:c r="C69" s="7" t="s">
-        <x:v>630</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="D69" s="9">
         <x:v>1</x:v>
@@ -8495,13 +8492,13 @@
     </x:row>
     <x:row r="70" ht="28" customHeight="1">
       <x:c r="A70" s="8" t="s">
+        <x:v>803</x:v>
+      </x:c>
+      <x:c r="B70" s="7" t="s">
         <x:v>804</x:v>
       </x:c>
-      <x:c r="B70" s="7" t="s">
-        <x:v>805</x:v>
-      </x:c>
       <x:c r="C70" s="7" t="s">
-        <x:v>658</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="D70" s="9">
         <x:v>1</x:v>
@@ -8510,13 +8507,13 @@
     </x:row>
     <x:row r="71" ht="28" customHeight="1">
       <x:c r="A71" s="8" t="s">
+        <x:v>805</x:v>
+      </x:c>
+      <x:c r="B71" s="7" t="s">
         <x:v>806</x:v>
       </x:c>
-      <x:c r="B71" s="7" t="s">
+      <x:c r="C71" s="7" t="s">
         <x:v>807</x:v>
-      </x:c>
-      <x:c r="C71" s="7" t="s">
-        <x:v>808</x:v>
       </x:c>
       <x:c r="D71" s="9">
         <x:v>1</x:v>
@@ -8525,64 +8522,64 @@
     </x:row>
     <x:row r="72" ht="28" customHeight="1">
       <x:c r="A72" s="8" t="s">
+        <x:v>808</x:v>
+      </x:c>
+      <x:c r="B72" s="7" t="s">
         <x:v>809</x:v>
       </x:c>
-      <x:c r="B72" s="7" t="s">
+      <x:c r="C72" s="7" t="s">
         <x:v>810</x:v>
-      </x:c>
-      <x:c r="C72" s="7" t="s">
-        <x:v>811</x:v>
       </x:c>
       <x:c r="D72" s="9">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E72" s="10" t="s">
-        <x:v>812</x:v>
+        <x:v>811</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="28" customHeight="1">
       <x:c r="A73" s="8" t="s">
+        <x:v>812</x:v>
+      </x:c>
+      <x:c r="B73" s="7" t="s">
         <x:v>813</x:v>
       </x:c>
-      <x:c r="B73" s="7" t="s">
+      <x:c r="C73" s="7" t="s">
         <x:v>814</x:v>
       </x:c>
-      <x:c r="C73" s="7" t="s">
+      <x:c r="D73" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E73" s="10" t="s">
         <x:v>815</x:v>
-      </x:c>
-      <x:c r="D73" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E73" s="10" t="s">
-        <x:v>816</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="28" customHeight="1">
       <x:c r="A74" s="8" t="s">
+        <x:v>816</x:v>
+      </x:c>
+      <x:c r="B74" s="7" t="s">
         <x:v>817</x:v>
       </x:c>
-      <x:c r="B74" s="7" t="s">
+      <x:c r="C74" s="7" t="s">
+        <x:v>615</x:v>
+      </x:c>
+      <x:c r="D74" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E74" s="10" t="s">
         <x:v>818</x:v>
-      </x:c>
-      <x:c r="C74" s="7" t="s">
-        <x:v>616</x:v>
-      </x:c>
-      <x:c r="D74" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E74" s="10" t="s">
-        <x:v>819</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="28" customHeight="1">
       <x:c r="A75" s="8" t="s">
+        <x:v>819</x:v>
+      </x:c>
+      <x:c r="B75" s="7" t="s">
         <x:v>820</x:v>
       </x:c>
-      <x:c r="B75" s="7" t="s">
-        <x:v>821</x:v>
-      </x:c>
       <x:c r="C75" s="7" t="s">
-        <x:v>731</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="D75" s="9">
         <x:v>1</x:v>
@@ -8591,64 +8588,64 @@
     </x:row>
     <x:row r="76" ht="28" customHeight="1">
       <x:c r="A76" s="8" t="s">
+        <x:v>821</x:v>
+      </x:c>
+      <x:c r="B76" s="7" t="s">
         <x:v>822</x:v>
       </x:c>
-      <x:c r="B76" s="7" t="s">
+      <x:c r="C76" s="7" t="s">
+        <x:v>699</x:v>
+      </x:c>
+      <x:c r="D76" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E76" s="10" t="s">
         <x:v>823</x:v>
-      </x:c>
-      <x:c r="C76" s="7" t="s">
-        <x:v>700</x:v>
-      </x:c>
-      <x:c r="D76" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E76" s="10" t="s">
-        <x:v>824</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
       <x:c r="A77" s="8" t="s">
+        <x:v>824</x:v>
+      </x:c>
+      <x:c r="B77" s="7" t="s">
         <x:v>825</x:v>
       </x:c>
-      <x:c r="B77" s="7" t="s">
+      <x:c r="C77" s="7" t="s">
+        <x:v>807</x:v>
+      </x:c>
+      <x:c r="D77" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E77" s="10" t="s">
         <x:v>826</x:v>
-      </x:c>
-      <x:c r="C77" s="7" t="s">
-        <x:v>808</x:v>
-      </x:c>
-      <x:c r="D77" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E77" s="10" t="s">
-        <x:v>827</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
       <x:c r="A78" s="8" t="s">
+        <x:v>827</x:v>
+      </x:c>
+      <x:c r="B78" s="7" t="s">
         <x:v>828</x:v>
       </x:c>
-      <x:c r="B78" s="7" t="s">
-        <x:v>829</x:v>
-      </x:c>
       <x:c r="C78" s="7" t="s">
-        <x:v>605</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="D78" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E78" s="10" t="s">
-        <x:v>830</x:v>
+        <x:v>829</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="28" customHeight="1">
       <x:c r="A79" s="8" t="s">
+        <x:v>830</x:v>
+      </x:c>
+      <x:c r="B79" s="7" t="s">
         <x:v>831</x:v>
       </x:c>
-      <x:c r="B79" s="7" t="s">
-        <x:v>832</x:v>
-      </x:c>
       <x:c r="C79" s="7" t="s">
-        <x:v>700</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="D79" s="9">
         <x:v>1</x:v>
@@ -8657,24 +8654,24 @@
     </x:row>
     <x:row r="80" ht="28" customHeight="1">
       <x:c r="A80" s="8" t="s">
+        <x:v>832</x:v>
+      </x:c>
+      <x:c r="B80" s="7" t="s">
         <x:v>833</x:v>
       </x:c>
-      <x:c r="B80" s="7" t="s">
+      <x:c r="C80" s="7" t="s">
         <x:v>834</x:v>
       </x:c>
-      <x:c r="C80" s="7" t="s">
+      <x:c r="D80" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E80" s="10" t="s">
         <x:v>835</x:v>
-      </x:c>
-      <x:c r="D80" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E80" s="10" t="s">
-        <x:v>836</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="28" customHeight="1">
       <x:c r="A81" s="8" t="s">
-        <x:v>837</x:v>
+        <x:v>836</x:v>
       </x:c>
       <x:c r="B81" s="7" t="s">
         <x:v>172</x:v>
@@ -8686,35 +8683,35 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="E81" s="10" t="s">
-        <x:v>838</x:v>
+        <x:v>837</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="28" customHeight="1">
       <x:c r="A82" s="8" t="s">
+        <x:v>838</x:v>
+      </x:c>
+      <x:c r="B82" s="7" t="s">
         <x:v>839</x:v>
       </x:c>
-      <x:c r="B82" s="7" t="s">
+      <x:c r="C82" s="7" t="s">
         <x:v>840</x:v>
-      </x:c>
-      <x:c r="C82" s="7" t="s">
-        <x:v>841</x:v>
       </x:c>
       <x:c r="D82" s="9">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E82" s="10" t="s">
-        <x:v>842</x:v>
+        <x:v>841</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="28" customHeight="1">
       <x:c r="A83" s="8" t="s">
+        <x:v>842</x:v>
+      </x:c>
+      <x:c r="B83" s="7" t="s">
         <x:v>843</x:v>
       </x:c>
-      <x:c r="B83" s="7" t="s">
-        <x:v>844</x:v>
-      </x:c>
       <x:c r="C83" s="7" t="s">
-        <x:v>623</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="D83" s="9">
         <x:v>1</x:v>
@@ -8723,13 +8720,13 @@
     </x:row>
     <x:row r="84" ht="28" customHeight="1">
       <x:c r="A84" s="8" t="s">
+        <x:v>844</x:v>
+      </x:c>
+      <x:c r="B84" s="7" t="s">
         <x:v>845</x:v>
       </x:c>
-      <x:c r="B84" s="7" t="s">
+      <x:c r="C84" s="7" t="s">
         <x:v>846</x:v>
-      </x:c>
-      <x:c r="C84" s="7" t="s">
-        <x:v>847</x:v>
       </x:c>
       <x:c r="D84" s="9">
         <x:v>1</x:v>
@@ -8738,64 +8735,64 @@
     </x:row>
     <x:row r="85" ht="28" customHeight="1">
       <x:c r="A85" s="8" t="s">
+        <x:v>847</x:v>
+      </x:c>
+      <x:c r="B85" s="7" t="s">
         <x:v>848</x:v>
       </x:c>
-      <x:c r="B85" s="7" t="s">
+      <x:c r="C85" s="7" t="s">
+        <x:v>625</x:v>
+      </x:c>
+      <x:c r="D85" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E85" s="10" t="s">
         <x:v>849</x:v>
-      </x:c>
-      <x:c r="C85" s="7" t="s">
-        <x:v>626</x:v>
-      </x:c>
-      <x:c r="D85" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E85" s="10" t="s">
-        <x:v>850</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="28" customHeight="1">
       <x:c r="A86" s="8" t="s">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="B86" s="7" t="s">
         <x:v>851</x:v>
       </x:c>
-      <x:c r="B86" s="7" t="s">
+      <x:c r="C86" s="7" t="s">
         <x:v>852</x:v>
       </x:c>
-      <x:c r="C86" s="7" t="s">
+      <x:c r="D86" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E86" s="10" t="s">
         <x:v>853</x:v>
-      </x:c>
-      <x:c r="D86" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E86" s="10" t="s">
-        <x:v>854</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="28" customHeight="1">
       <x:c r="A87" s="8" t="s">
+        <x:v>854</x:v>
+      </x:c>
+      <x:c r="B87" s="7" t="s">
         <x:v>855</x:v>
       </x:c>
-      <x:c r="B87" s="7" t="s">
+      <x:c r="C87" s="7" t="s">
         <x:v>856</x:v>
       </x:c>
-      <x:c r="C87" s="7" t="s">
+      <x:c r="D87" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E87" s="10" t="s">
         <x:v>857</x:v>
-      </x:c>
-      <x:c r="D87" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E87" s="10" t="s">
-        <x:v>858</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="28" customHeight="1">
       <x:c r="A88" s="8" t="s">
+        <x:v>858</x:v>
+      </x:c>
+      <x:c r="B88" s="7" t="s">
         <x:v>859</x:v>
       </x:c>
-      <x:c r="B88" s="7" t="s">
-        <x:v>860</x:v>
-      </x:c>
       <x:c r="C88" s="7" t="s">
-        <x:v>731</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="D88" s="9">
         <x:v>1</x:v>
@@ -8804,13 +8801,13 @@
     </x:row>
     <x:row r="89" ht="28" customHeight="1">
       <x:c r="A89" s="8" t="s">
+        <x:v>860</x:v>
+      </x:c>
+      <x:c r="B89" s="7" t="s">
         <x:v>861</x:v>
       </x:c>
-      <x:c r="B89" s="7" t="s">
-        <x:v>862</x:v>
-      </x:c>
       <x:c r="C89" s="7" t="s">
-        <x:v>647</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="D89" s="9">
         <x:v>1</x:v>
@@ -8819,30 +8816,30 @@
     </x:row>
     <x:row r="90" ht="28" customHeight="1">
       <x:c r="A90" s="8" t="s">
+        <x:v>862</x:v>
+      </x:c>
+      <x:c r="B90" s="7" t="s">
         <x:v>863</x:v>
       </x:c>
-      <x:c r="B90" s="7" t="s">
-        <x:v>864</x:v>
-      </x:c>
       <x:c r="C90" s="7" t="s">
-        <x:v>775</x:v>
+        <x:v>774</x:v>
       </x:c>
       <x:c r="D90" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E90" s="10" t="s">
-        <x:v>865</x:v>
+        <x:v>864</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="28" customHeight="1">
       <x:c r="A91" s="8" t="s">
+        <x:v>865</x:v>
+      </x:c>
+      <x:c r="B91" s="7" t="s">
         <x:v>866</x:v>
       </x:c>
-      <x:c r="B91" s="7" t="s">
+      <x:c r="C91" s="7" t="s">
         <x:v>867</x:v>
-      </x:c>
-      <x:c r="C91" s="7" t="s">
-        <x:v>868</x:v>
       </x:c>
       <x:c r="D91" s="9">
         <x:v>1</x:v>
@@ -8851,30 +8848,30 @@
     </x:row>
     <x:row r="92" ht="28" customHeight="1">
       <x:c r="A92" s="8" t="s">
+        <x:v>868</x:v>
+      </x:c>
+      <x:c r="B92" s="7" t="s">
         <x:v>869</x:v>
       </x:c>
-      <x:c r="B92" s="7" t="s">
+      <x:c r="C92" s="7" t="s">
         <x:v>870</x:v>
-      </x:c>
-      <x:c r="C92" s="7" t="s">
-        <x:v>871</x:v>
       </x:c>
       <x:c r="D92" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E92" s="10" t="s">
-        <x:v>872</x:v>
+        <x:v>871</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="28" customHeight="1">
       <x:c r="A93" s="8" t="s">
+        <x:v>872</x:v>
+      </x:c>
+      <x:c r="B93" s="7" t="s">
         <x:v>873</x:v>
       </x:c>
-      <x:c r="B93" s="7" t="s">
-        <x:v>874</x:v>
-      </x:c>
       <x:c r="C93" s="7" t="s">
-        <x:v>808</x:v>
+        <x:v>807</x:v>
       </x:c>
       <x:c r="D93" s="9">
         <x:v>1</x:v>
@@ -8883,30 +8880,30 @@
     </x:row>
     <x:row r="94" ht="28" customHeight="1">
       <x:c r="A94" s="8" t="s">
+        <x:v>874</x:v>
+      </x:c>
+      <x:c r="B94" s="7" t="s">
         <x:v>875</x:v>
       </x:c>
-      <x:c r="B94" s="7" t="s">
+      <x:c r="C94" s="7" t="s">
+        <x:v>699</x:v>
+      </x:c>
+      <x:c r="D94" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E94" s="10" t="s">
         <x:v>876</x:v>
-      </x:c>
-      <x:c r="C94" s="7" t="s">
-        <x:v>700</x:v>
-      </x:c>
-      <x:c r="D94" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E94" s="10" t="s">
-        <x:v>877</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="28" customHeight="1">
       <x:c r="A95" s="8" t="s">
+        <x:v>877</x:v>
+      </x:c>
+      <x:c r="B95" s="7" t="s">
         <x:v>878</x:v>
       </x:c>
-      <x:c r="B95" s="7" t="s">
-        <x:v>879</x:v>
-      </x:c>
       <x:c r="C95" s="7" t="s">
-        <x:v>697</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="D95" s="9">
         <x:v>1</x:v>
@@ -8915,47 +8912,47 @@
     </x:row>
     <x:row r="96" ht="28" customHeight="1">
       <x:c r="A96" s="8" t="s">
+        <x:v>879</x:v>
+      </x:c>
+      <x:c r="B96" s="7" t="s">
         <x:v>880</x:v>
       </x:c>
-      <x:c r="B96" s="7" t="s">
+      <x:c r="C96" s="7" t="s">
         <x:v>881</x:v>
-      </x:c>
-      <x:c r="C96" s="7" t="s">
-        <x:v>882</x:v>
       </x:c>
       <x:c r="D96" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E96" s="10" t="s">
-        <x:v>883</x:v>
+        <x:v>882</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="28" customHeight="1">
       <x:c r="A97" s="8" t="s">
+        <x:v>883</x:v>
+      </x:c>
+      <x:c r="B97" s="7" t="s">
         <x:v>884</x:v>
       </x:c>
-      <x:c r="B97" s="7" t="s">
+      <x:c r="C97" s="7" t="s">
+        <x:v>846</x:v>
+      </x:c>
+      <x:c r="D97" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E97" s="10" t="s">
         <x:v>885</x:v>
-      </x:c>
-      <x:c r="C97" s="7" t="s">
-        <x:v>847</x:v>
-      </x:c>
-      <x:c r="D97" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E97" s="10" t="s">
-        <x:v>886</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="s">
+        <x:v>886</x:v>
+      </x:c>
+      <x:c r="B98" t="s">
         <x:v>887</x:v>
       </x:c>
-      <x:c r="B98" t="s">
+      <x:c r="C98" t="s">
         <x:v>888</x:v>
-      </x:c>
-      <x:c r="C98" t="s">
-        <x:v>889</x:v>
       </x:c>
       <x:c r="D98">
         <x:v>1</x:v>
@@ -8976,12 +8973,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R44a0218bf92e4dfd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Re5a6ec2bcb9b49f6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rb3c9d81df03a4817"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R917ea9851b8b4f4f"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R352cf6a99b764d67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3efb391343944b07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8996,7 +8993,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>890</x:v>
+        <x:v>889</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -9884,7 +9881,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1be11ad109a04c6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0396aacf4b0747cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9900,27 +9897,27 @@
   <x:sheetData>
     <x:row r="1" ht="34.75" customHeight="1">
       <x:c r="A1" s="20" t="s">
-        <x:v>891</x:v>
+        <x:v>890</x:v>
       </x:c>
       <x:c r="B1" s="20"/>
       <x:c r="C1" s="20"/>
     </x:row>
     <x:row r="2" ht="45.25" customHeight="1">
       <x:c r="A2" s="21" t="s">
-        <x:v>892</x:v>
+        <x:v>891</x:v>
       </x:c>
       <x:c r="B2" s="21"/>
       <x:c r="C2" s="21"/>
     </x:row>
     <x:row r="4" ht="29.25" customHeight="1">
       <x:c r="A4" s="15" t="s">
+        <x:v>892</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="s">
         <x:v>893</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="s">
+      <x:c r="C4" s="15" t="s">
         <x:v>894</x:v>
-      </x:c>
-      <x:c r="C4" s="15" t="s">
-        <x:v>895</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.75" customHeight="1">
@@ -9928,7 +9925,7 @@
         <x:v>310</x:v>
       </x:c>
       <x:c r="B5" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C5" s="17"/>
     </x:row>
@@ -9937,7 +9934,7 @@
         <x:v>170</x:v>
       </x:c>
       <x:c r="B6" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C6" s="17"/>
     </x:row>
@@ -9946,7 +9943,7 @@
         <x:v>379</x:v>
       </x:c>
       <x:c r="B7" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C7" s="17"/>
     </x:row>
@@ -9955,7 +9952,7 @@
         <x:v>455</x:v>
       </x:c>
       <x:c r="B8" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C8" s="17"/>
     </x:row>
@@ -9964,7 +9961,7 @@
         <x:v>347</x:v>
       </x:c>
       <x:c r="B9" s="16" t="s">
-        <x:v>899</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="C9" s="17"/>
     </x:row>
@@ -9973,27 +9970,27 @@
         <x:v>368</x:v>
       </x:c>
       <x:c r="B10" s="16" t="s">
+        <x:v>899</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="s">
         <x:v>900</x:v>
-      </x:c>
-      <x:c r="C10" s="17" t="s">
-        <x:v>901</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.75" customHeight="1">
       <x:c r="A11" s="16" t="s">
-        <x:v>902</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="B11" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C11" s="17"/>
     </x:row>
     <x:row r="12" ht="26.75" customHeight="1">
       <x:c r="A12" s="16" t="s">
+        <x:v>902</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="s">
         <x:v>903</x:v>
-      </x:c>
-      <x:c r="B12" s="16" t="s">
-        <x:v>904</x:v>
       </x:c>
       <x:c r="C12" s="17"/>
     </x:row>
@@ -10002,25 +9999,25 @@
         <x:v>303</x:v>
       </x:c>
       <x:c r="B13" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C13" s="17"/>
     </x:row>
     <x:row r="14" ht="26.75" customHeight="1">
       <x:c r="A14" s="16" t="s">
+        <x:v>904</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="s">
         <x:v>905</x:v>
-      </x:c>
-      <x:c r="B14" s="16" t="s">
-        <x:v>906</x:v>
       </x:c>
       <x:c r="C14" s="17"/>
     </x:row>
     <x:row r="15" ht="26.75" customHeight="1">
       <x:c r="A15" s="16" t="s">
+        <x:v>906</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="s">
         <x:v>907</x:v>
-      </x:c>
-      <x:c r="B15" s="16" t="s">
-        <x:v>908</x:v>
       </x:c>
       <x:c r="C15" s="17"/>
     </x:row>
@@ -10029,7 +10026,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B16" s="16" t="s">
-        <x:v>909</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C16" s="17"/>
     </x:row>
@@ -10038,7 +10035,7 @@
         <x:v>198</x:v>
       </x:c>
       <x:c r="B17" s="16" t="s">
-        <x:v>909</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C17" s="17"/>
     </x:row>
@@ -10047,7 +10044,7 @@
         <x:v>405</x:v>
       </x:c>
       <x:c r="B18" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C18" s="17"/>
     </x:row>
@@ -10056,25 +10053,25 @@
         <x:v>260</x:v>
       </x:c>
       <x:c r="B19" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C19" s="17"/>
     </x:row>
     <x:row r="20" ht="26.75" customHeight="1">
       <x:c r="A20" s="16" t="s">
-        <x:v>563</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="B20" s="16" t="s">
-        <x:v>908</x:v>
+        <x:v>907</x:v>
       </x:c>
       <x:c r="C20" s="17"/>
     </x:row>
     <x:row r="21" ht="26.75" customHeight="1">
       <x:c r="A21" s="16" t="s">
-        <x:v>910</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="B21" s="16" t="s">
-        <x:v>908</x:v>
+        <x:v>907</x:v>
       </x:c>
       <x:c r="C21" s="17"/>
     </x:row>
@@ -10083,25 +10080,25 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B22" s="16" t="s">
-        <x:v>908</x:v>
+        <x:v>907</x:v>
       </x:c>
       <x:c r="C22" s="17"/>
     </x:row>
     <x:row r="23" ht="26.75" customHeight="1">
       <x:c r="A23" s="16" t="s">
+        <x:v>910</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="s">
         <x:v>911</x:v>
-      </x:c>
-      <x:c r="B23" s="16" t="s">
-        <x:v>912</x:v>
       </x:c>
       <x:c r="C23" s="17"/>
     </x:row>
     <x:row r="24" ht="26.75" customHeight="1">
       <x:c r="A24" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>912</x:v>
       </x:c>
       <x:c r="B24" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
     </x:row>
@@ -10110,7 +10107,7 @@
         <x:v>325</x:v>
       </x:c>
       <x:c r="B25" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
     </x:row>
@@ -10119,7 +10116,7 @@
         <x:v>465</x:v>
       </x:c>
       <x:c r="B26" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
     </x:row>
@@ -10128,18 +10125,18 @@
         <x:v>555</x:v>
       </x:c>
       <x:c r="B27" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C27" s="17" t="s">
-        <x:v>914</x:v>
+        <x:v>913</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="26.75" customHeight="1">
       <x:c r="A28" s="16" t="s">
-        <x:v>915</x:v>
+        <x:v>914</x:v>
       </x:c>
       <x:c r="B28" s="16" t="s">
-        <x:v>912</x:v>
+        <x:v>911</x:v>
       </x:c>
       <x:c r="C28" s="17"/>
     </x:row>
@@ -10148,7 +10145,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B29" s="16" t="s">
-        <x:v>912</x:v>
+        <x:v>911</x:v>
       </x:c>
       <x:c r="C29" s="17"/>
     </x:row>
@@ -10157,7 +10154,7 @@
         <x:v>191</x:v>
       </x:c>
       <x:c r="B30" s="16" t="s">
-        <x:v>912</x:v>
+        <x:v>911</x:v>
       </x:c>
       <x:c r="C30" s="17"/>
     </x:row>
@@ -10166,7 +10163,7 @@
         <x:v>141</x:v>
       </x:c>
       <x:c r="B31" s="16" t="s">
-        <x:v>909</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C31" s="17"/>
     </x:row>
@@ -10175,16 +10172,16 @@
         <x:v>550</x:v>
       </x:c>
       <x:c r="B32" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C32" s="17"/>
     </x:row>
     <x:row r="33" ht="26.75" customHeight="1">
       <x:c r="A33" s="16" t="s">
-        <x:v>916</x:v>
+        <x:v>915</x:v>
       </x:c>
       <x:c r="B33" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C33" s="17"/>
     </x:row>
@@ -10193,7 +10190,7 @@
         <x:v>318</x:v>
       </x:c>
       <x:c r="B34" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C34" s="17"/>
     </x:row>
@@ -10202,7 +10199,7 @@
         <x:v>505</x:v>
       </x:c>
       <x:c r="B35" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C35" s="17"/>
     </x:row>
@@ -10211,18 +10208,18 @@
         <x:v>268</x:v>
       </x:c>
       <x:c r="B36" s="16" t="s">
+        <x:v>899</x:v>
+      </x:c>
+      <x:c r="C36" s="17" t="s">
         <x:v>900</x:v>
-      </x:c>
-      <x:c r="C36" s="17" t="s">
-        <x:v>901</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="26.75" customHeight="1">
       <x:c r="A37" s="16" t="s">
-        <x:v>917</x:v>
+        <x:v>916</x:v>
       </x:c>
       <x:c r="B37" s="16" t="s">
-        <x:v>909</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="C37" s="17"/>
     </x:row>
@@ -10231,7 +10228,7 @@
         <x:v>177</x:v>
       </x:c>
       <x:c r="B38" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C38" s="17"/>
     </x:row>
@@ -10240,10 +10237,10 @@
         <x:v>239</x:v>
       </x:c>
       <x:c r="B39" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C39" s="17" t="s">
-        <x:v>918</x:v>
+        <x:v>917</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="26.75" customHeight="1">
@@ -10251,25 +10248,25 @@
         <x:v>445</x:v>
       </x:c>
       <x:c r="B40" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C40" s="17"/>
     </x:row>
     <x:row r="41" ht="26.75" customHeight="1">
       <x:c r="A41" s="16" t="s">
-        <x:v>919</x:v>
+        <x:v>918</x:v>
       </x:c>
       <x:c r="B41" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C41" s="17"/>
     </x:row>
     <x:row r="42" ht="26.75" customHeight="1">
       <x:c r="A42" s="16" t="s">
-        <x:v>920</x:v>
+        <x:v>919</x:v>
       </x:c>
       <x:c r="B42" s="16" t="s">
-        <x:v>908</x:v>
+        <x:v>907</x:v>
       </x:c>
       <x:c r="C42" s="17"/>
     </x:row>
@@ -10278,10 +10275,10 @@
         <x:v>224</x:v>
       </x:c>
       <x:c r="B43" s="16" t="s">
+        <x:v>899</x:v>
+      </x:c>
+      <x:c r="C43" s="17" t="s">
         <x:v>900</x:v>
-      </x:c>
-      <x:c r="C43" s="17" t="s">
-        <x:v>901</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="26.75" customHeight="1">
@@ -10289,7 +10286,7 @@
         <x:v>182</x:v>
       </x:c>
       <x:c r="B44" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C44" s="17"/>
     </x:row>
@@ -10298,16 +10295,16 @@
         <x:v>162</x:v>
       </x:c>
       <x:c r="B45" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C45" s="17"/>
     </x:row>
     <x:row r="46" ht="26.75" customHeight="1">
       <x:c r="A46" s="16" t="s">
-        <x:v>921</x:v>
+        <x:v>920</x:v>
       </x:c>
       <x:c r="B46" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C46" s="17"/>
     </x:row>
@@ -10316,19 +10313,19 @@
         <x:v>156</x:v>
       </x:c>
       <x:c r="B47" s="16" t="s">
-        <x:v>899</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="C47" s="17"/>
     </x:row>
     <x:row r="48" ht="26.75" customHeight="1">
       <x:c r="A48" s="16" t="s">
+        <x:v>921</x:v>
+      </x:c>
+      <x:c r="B48" s="16" t="s">
+        <x:v>899</x:v>
+      </x:c>
+      <x:c r="C48" s="17" t="s">
         <x:v>922</x:v>
-      </x:c>
-      <x:c r="B48" s="16" t="s">
-        <x:v>900</x:v>
-      </x:c>
-      <x:c r="C48" s="17" t="s">
-        <x:v>923</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="26.75" customHeight="1">
@@ -10336,7 +10333,7 @@
         <x:v>286</x:v>
       </x:c>
       <x:c r="B49" s="16" t="s">
-        <x:v>899</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="C49" s="17"/>
     </x:row>
@@ -10345,16 +10342,16 @@
         <x:v>212</x:v>
       </x:c>
       <x:c r="B50" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C50" s="17"/>
     </x:row>
     <x:row r="51" ht="26.75" customHeight="1">
       <x:c r="A51" s="16" t="s">
-        <x:v>924</x:v>
+        <x:v>923</x:v>
       </x:c>
       <x:c r="B51" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C51" s="17"/>
     </x:row>
@@ -10363,38 +10360,38 @@
         <x:v>232</x:v>
       </x:c>
       <x:c r="B52" s="16" t="s">
-        <x:v>912</x:v>
+        <x:v>911</x:v>
       </x:c>
       <x:c r="C52" s="17"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" t="s">
-        <x:v>573</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="B53" t="s">
         <x:v>379</x:v>
       </x:c>
       <x:c r="C53" t="s">
-        <x:v>925</x:v>
+        <x:v>924</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" t="s">
-        <x:v>582</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="B54" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" t="s">
-        <x:v>589</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="B55" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C55" t="s">
-        <x:v>926</x:v>
+        <x:v>925</x:v>
       </x:c>
     </x:row>
     <x:row r="56">

</xml_diff>

<commit_message>
Correct AWS credit value
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R00c80d8725c847ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R7bbd9a769e0a4101"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R6d2dd8a32ce94e28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R51a7f1b3aea84553"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R0c56dd53672e4b09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rf09d13ae9b374812"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R9f337570e15a4110"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R3a60d2e62ca749a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1616,9 +1616,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">amber.ac</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">4.5K AWS Credits</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">kingdom of pal: 7 dwarfs and a shiekh, a tool to help maange one person community biz</x:t>
@@ -6861,20 +6858,20 @@
       <x:c r="F72" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="G72" t="s">
-        <x:v>535</x:v>
+      <x:c r="G72" t="str">
+        <x:v>4.5K USD AWS Credits</x:v>
       </x:c>
       <x:c r="H72" t="s">
         <x:v>239</x:v>
       </x:c>
       <x:c r="I72" t="s">
+        <x:v>535</x:v>
+      </x:c>
+      <x:c r="J72" t="s">
         <x:v>536</x:v>
       </x:c>
-      <x:c r="J72" t="s">
+      <x:c r="K72" t="s">
         <x:v>537</x:v>
-      </x:c>
-      <x:c r="K72" t="s">
-        <x:v>538</x:v>
       </x:c>
       <x:c r="L72" t="s">
         <x:v>534</x:v>
@@ -6889,7 +6886,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="P72" t="s">
-        <x:v>539</x:v>
+        <x:v>538</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -6897,13 +6894,13 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B73" t="s">
+        <x:v>539</x:v>
+      </x:c>
+      <x:c r="C73" t="s">
         <x:v>540</x:v>
       </x:c>
-      <x:c r="C73" t="s">
+      <x:c r="D73" s="2" t="s">
         <x:v>541</x:v>
-      </x:c>
-      <x:c r="D73" s="2" t="s">
-        <x:v>542</x:v>
       </x:c>
       <x:c r="E73">
         <x:v>1</x:v>
@@ -6918,28 +6915,28 @@
         <x:v>465</x:v>
       </x:c>
       <x:c r="I73" t="s">
-        <x:v>543</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="J73" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K73" t="s">
-        <x:v>544</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="L73" t="s">
-        <x:v>541</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="M73" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N73" t="s">
+        <x:v>544</x:v>
+      </x:c>
+      <x:c r="O73" t="s">
         <x:v>545</x:v>
       </x:c>
-      <x:c r="O73" t="s">
+      <x:c r="P73" t="s">
         <x:v>546</x:v>
-      </x:c>
-      <x:c r="P73" t="s">
-        <x:v>547</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -6947,13 +6944,13 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B74" t="s">
-        <x:v>548</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="C74" t="s">
         <x:v>517</x:v>
       </x:c>
       <x:c r="D74" s="2" t="s">
-        <x:v>549</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="E74">
         <x:v>10</x:v>
@@ -6965,16 +6962,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H74" t="s">
+        <x:v>549</x:v>
+      </x:c>
+      <x:c r="I74" t="s">
         <x:v>550</x:v>
-      </x:c>
-      <x:c r="I74" t="s">
-        <x:v>551</x:v>
       </x:c>
       <x:c r="J74" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K74" t="s">
-        <x:v>552</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="L74" t="s">
         <x:v>517</x:v>
@@ -6986,7 +6983,7 @@
         <x:v>359</x:v>
       </x:c>
       <x:c r="O74" t="s">
-        <x:v>553</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="P74" t="s">
         <x:v>525</x:v>
@@ -6997,10 +6994,10 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B75" s="12" t="s">
+        <x:v>553</x:v>
+      </x:c>
+      <x:c r="C75" s="12" t="s">
         <x:v>554</x:v>
-      </x:c>
-      <x:c r="C75" s="12" t="s">
-        <x:v>555</x:v>
       </x:c>
       <x:c r="D75" s="5">
         <x:v>46150</x:v>
@@ -7015,19 +7012,19 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H75" s="12" t="s">
+        <x:v>554</x:v>
+      </x:c>
+      <x:c r="I75" s="14" t="s">
         <x:v>555</x:v>
-      </x:c>
-      <x:c r="I75" s="14" t="s">
-        <x:v>556</x:v>
       </x:c>
       <x:c r="J75" s="12" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K75" s="12" t="s">
-        <x:v>557</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="L75" s="12" t="s">
-        <x:v>555</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="M75" s="12" t="s">
         <x:v>26</x:v>
@@ -7036,7 +7033,7 @@
         <x:v>273</x:v>
       </x:c>
       <x:c r="O75" t="s">
-        <x:v>558</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="P75" s="12" t="s">
         <x:v>25</x:v>
@@ -7047,13 +7044,13 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B76" s="12" t="s">
+        <x:v>558</x:v>
+      </x:c>
+      <x:c r="C76" s="12" t="s">
         <x:v>559</x:v>
       </x:c>
-      <x:c r="C76" s="12" t="s">
+      <x:c r="D76" s="13" t="s">
         <x:v>560</x:v>
-      </x:c>
-      <x:c r="D76" s="13" t="s">
-        <x:v>561</x:v>
       </x:c>
       <x:c r="E76">
         <x:v>1</x:v>
@@ -7065,31 +7062,31 @@
         <x:v>Best Vertical Solution (Family Office Track), 2,000 Cybrdeck API credits (worth US$25)</x:v>
       </x:c>
       <x:c r="H76" s="12" t="s">
+        <x:v>561</x:v>
+      </x:c>
+      <x:c r="I76" s="12" t="s">
         <x:v>562</x:v>
       </x:c>
-      <x:c r="I76" s="12" t="s">
+      <x:c r="J76" s="12" t="s">
         <x:v>563</x:v>
       </x:c>
-      <x:c r="J76" s="12" t="s">
+      <x:c r="K76" s="12" t="s">
         <x:v>564</x:v>
       </x:c>
-      <x:c r="K76" s="12" t="s">
-        <x:v>565</x:v>
-      </x:c>
       <x:c r="L76" s="12" t="s">
-        <x:v>560</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="M76" s="12" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N76" s="12" t="s">
+        <x:v>565</x:v>
+      </x:c>
+      <x:c r="O76" s="1" t="s">
         <x:v>566</x:v>
       </x:c>
-      <x:c r="O76" s="1" t="s">
+      <x:c r="P76" t="s">
         <x:v>567</x:v>
-      </x:c>
-      <x:c r="P76" t="s">
-        <x:v>568</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -7097,13 +7094,13 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B77" t="s">
+        <x:v>568</x:v>
+      </x:c>
+      <x:c r="C77" t="s">
         <x:v>569</x:v>
       </x:c>
-      <x:c r="C77" t="s">
+      <x:c r="D77" t="s">
         <x:v>570</x:v>
-      </x:c>
-      <x:c r="D77" t="s">
-        <x:v>571</x:v>
       </x:c>
       <x:c r="E77">
         <x:v>1</x:v>
@@ -7115,31 +7112,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H77" t="s">
+        <x:v>571</x:v>
+      </x:c>
+      <x:c r="I77" t="s">
         <x:v>572</x:v>
-      </x:c>
-      <x:c r="I77" t="s">
-        <x:v>573</x:v>
       </x:c>
       <x:c r="J77" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K77" t="s">
+        <x:v>573</x:v>
+      </x:c>
+      <x:c r="L77" t="s">
         <x:v>574</x:v>
-      </x:c>
-      <x:c r="L77" t="s">
-        <x:v>575</x:v>
       </x:c>
       <x:c r="M77" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N77" t="s">
+        <x:v>575</x:v>
+      </x:c>
+      <x:c r="O77" t="s">
         <x:v>576</x:v>
       </x:c>
-      <x:c r="O77" t="s">
+      <x:c r="P77" t="s">
         <x:v>577</x:v>
-      </x:c>
-      <x:c r="P77" t="s">
-        <x:v>578</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -7147,13 +7144,13 @@
         <x:v>77</x:v>
       </x:c>
       <x:c r="B78" t="s">
-        <x:v>579</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="C78" t="s">
         <x:v>517</x:v>
       </x:c>
       <x:c r="D78" t="s">
-        <x:v>580</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="E78">
         <x:v>1</x:v>
@@ -7165,16 +7162,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H78" t="s">
+        <x:v>580</x:v>
+      </x:c>
+      <x:c r="I78" t="s">
         <x:v>581</x:v>
-      </x:c>
-      <x:c r="I78" t="s">
-        <x:v>582</x:v>
       </x:c>
       <x:c r="J78" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K78" t="s">
-        <x:v>583</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="L78" t="s">
         <x:v>517</x:v>
@@ -7186,7 +7183,7 @@
         <x:v>359</x:v>
       </x:c>
       <x:c r="O78" t="s">
-        <x:v>584</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="P78" t="s">
         <x:v>525</x:v>
@@ -7197,13 +7194,13 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="B79" t="s">
+        <x:v>584</x:v>
+      </x:c>
+      <x:c r="C79" t="s">
         <x:v>585</x:v>
       </x:c>
-      <x:c r="C79" t="s">
+      <x:c r="D79" t="s">
         <x:v>586</x:v>
-      </x:c>
-      <x:c r="D79" t="s">
-        <x:v>587</x:v>
       </x:c>
       <x:c r="E79">
         <x:v>4</x:v>
@@ -7215,19 +7212,19 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H79" t="s">
+        <x:v>587</x:v>
+      </x:c>
+      <x:c r="I79" t="s">
         <x:v>588</x:v>
       </x:c>
-      <x:c r="I79" t="s">
+      <x:c r="J79" t="s">
         <x:v>589</x:v>
       </x:c>
-      <x:c r="J79" t="s">
+      <x:c r="K79" t="s">
         <x:v>590</x:v>
       </x:c>
-      <x:c r="K79" t="s">
+      <x:c r="L79" t="s">
         <x:v>591</x:v>
-      </x:c>
-      <x:c r="L79" t="s">
-        <x:v>592</x:v>
       </x:c>
       <x:c r="M79" t="s">
         <x:v>26</x:v>
@@ -7236,10 +7233,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="O79" t="s">
+        <x:v>592</x:v>
+      </x:c>
+      <x:c r="P79" t="s">
         <x:v>593</x:v>
-      </x:c>
-      <x:c r="P79" t="s">
-        <x:v>594</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -7392,10 +7389,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Re26bd447967545c1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R2d1af01fc7934f9e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Raf810d0659c449d2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Reac6b8f89afe446f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rd3c0acdaa85c4abe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R8c3340ff6dff4df1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rf9320db7364943e0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Ree5ca64eaaba4361"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7418,7 +7415,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>595</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -7427,7 +7424,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="19" t="s">
-        <x:v>596</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="B2" s="19"/>
       <x:c r="C2" s="19"/>
@@ -7436,64 +7433,64 @@
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="11" t="s">
+        <x:v>596</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="s">
         <x:v>597</x:v>
       </x:c>
-      <x:c r="B4" s="11" t="s">
+      <x:c r="C4" s="11" t="s">
         <x:v>598</x:v>
       </x:c>
-      <x:c r="C4" s="11" t="s">
+      <x:c r="D4" s="11" t="s">
         <x:v>599</x:v>
       </x:c>
-      <x:c r="D4" s="11" t="s">
+      <x:c r="E4" s="11" t="s">
         <x:v>600</x:v>
-      </x:c>
-      <x:c r="E4" s="11" t="s">
-        <x:v>601</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="8" t="s">
+        <x:v>601</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="s">
         <x:v>602</x:v>
       </x:c>
-      <x:c r="B5" s="7" t="s">
+      <x:c r="C5" s="7" t="s">
         <x:v>603</x:v>
-      </x:c>
-      <x:c r="C5" s="7" t="s">
-        <x:v>604</x:v>
       </x:c>
       <x:c r="D5" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E5" s="10" t="s">
-        <x:v>605</x:v>
+        <x:v>604</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="8" t="s">
+        <x:v>605</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>606</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="s">
+      <x:c r="C6" s="7" t="s">
         <x:v>607</x:v>
       </x:c>
-      <x:c r="C6" s="7" t="s">
+      <x:c r="D6" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="s">
         <x:v>608</x:v>
-      </x:c>
-      <x:c r="D6" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E6" s="10" t="s">
-        <x:v>609</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="8" t="s">
+        <x:v>609</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
         <x:v>610</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="s">
+      <x:c r="C7" s="7" t="s">
         <x:v>611</x:v>
-      </x:c>
-      <x:c r="C7" s="7" t="s">
-        <x:v>612</x:v>
       </x:c>
       <x:c r="D7" s="9">
         <x:v>1</x:v>
@@ -7502,47 +7499,47 @@
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
       <x:c r="A8" s="8" t="s">
+        <x:v>612</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
         <x:v>613</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="s">
+      <x:c r="C8" s="7" t="s">
         <x:v>614</x:v>
       </x:c>
-      <x:c r="C8" s="7" t="s">
+      <x:c r="D8" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="s">
         <x:v>615</x:v>
-      </x:c>
-      <x:c r="D8" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E8" s="10" t="s">
-        <x:v>616</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" s="8" t="s">
+        <x:v>616</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
         <x:v>617</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="s">
+      <x:c r="C9" s="7" t="s">
+        <x:v>607</x:v>
+      </x:c>
+      <x:c r="D9" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="s">
         <x:v>618</x:v>
-      </x:c>
-      <x:c r="C9" s="7" t="s">
-        <x:v>608</x:v>
-      </x:c>
-      <x:c r="D9" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E9" s="10" t="s">
-        <x:v>619</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
       <x:c r="A10" s="8" t="s">
+        <x:v>619</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="s">
         <x:v>620</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="s">
+      <x:c r="C10" s="7" t="s">
         <x:v>621</x:v>
-      </x:c>
-      <x:c r="C10" s="7" t="s">
-        <x:v>622</x:v>
       </x:c>
       <x:c r="D10" s="9">
         <x:v>1</x:v>
@@ -7551,47 +7548,47 @@
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
       <x:c r="A11" s="8" t="s">
+        <x:v>622</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="s">
         <x:v>623</x:v>
       </x:c>
-      <x:c r="B11" s="7" t="s">
+      <x:c r="C11" s="7" t="s">
         <x:v>624</x:v>
       </x:c>
-      <x:c r="C11" s="7" t="s">
+      <x:c r="D11" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="10" t="s">
         <x:v>625</x:v>
-      </x:c>
-      <x:c r="D11" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E11" s="10" t="s">
-        <x:v>626</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
       <x:c r="A12" s="8" t="s">
+        <x:v>626</x:v>
+      </x:c>
+      <x:c r="B12" s="7" t="s">
         <x:v>627</x:v>
       </x:c>
-      <x:c r="B12" s="7" t="s">
+      <x:c r="C12" s="7" t="s">
         <x:v>628</x:v>
       </x:c>
-      <x:c r="C12" s="7" t="s">
+      <x:c r="D12" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="s">
         <x:v>629</x:v>
-      </x:c>
-      <x:c r="D12" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E12" s="10" t="s">
-        <x:v>630</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
       <x:c r="A13" s="8" t="s">
+        <x:v>630</x:v>
+      </x:c>
+      <x:c r="B13" s="7" t="s">
         <x:v>631</x:v>
       </x:c>
-      <x:c r="B13" s="7" t="s">
+      <x:c r="C13" s="7" t="s">
         <x:v>632</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="s">
-        <x:v>633</x:v>
       </x:c>
       <x:c r="D13" s="9">
         <x:v>1</x:v>
@@ -7600,30 +7597,30 @@
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
       <x:c r="A14" s="8" t="s">
+        <x:v>633</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="s">
         <x:v>634</x:v>
       </x:c>
-      <x:c r="B14" s="7" t="s">
+      <x:c r="C14" s="7" t="s">
+        <x:v>632</x:v>
+      </x:c>
+      <x:c r="D14" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="s">
         <x:v>635</x:v>
-      </x:c>
-      <x:c r="C14" s="7" t="s">
-        <x:v>633</x:v>
-      </x:c>
-      <x:c r="D14" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E14" s="10" t="s">
-        <x:v>636</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
       <x:c r="A15" s="8" t="s">
+        <x:v>636</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="s">
         <x:v>637</x:v>
       </x:c>
-      <x:c r="B15" s="7" t="s">
+      <x:c r="C15" s="7" t="s">
         <x:v>638</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="s">
-        <x:v>639</x:v>
       </x:c>
       <x:c r="D15" s="9">
         <x:v>1</x:v>
@@ -7632,30 +7629,30 @@
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
       <x:c r="A16" s="8" t="s">
+        <x:v>639</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="s">
         <x:v>640</x:v>
       </x:c>
-      <x:c r="B16" s="7" t="s">
+      <x:c r="C16" s="7" t="s">
         <x:v>641</x:v>
       </x:c>
-      <x:c r="C16" s="7" t="s">
+      <x:c r="D16" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="s">
         <x:v>642</x:v>
-      </x:c>
-      <x:c r="D16" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E16" s="10" t="s">
-        <x:v>643</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
       <x:c r="A17" s="8" t="s">
+        <x:v>643</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="s">
         <x:v>644</x:v>
       </x:c>
-      <x:c r="B17" s="7" t="s">
+      <x:c r="C17" s="7" t="s">
         <x:v>645</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="s">
-        <x:v>646</x:v>
       </x:c>
       <x:c r="D17" s="9">
         <x:v>1</x:v>
@@ -7664,47 +7661,47 @@
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
       <x:c r="A18" s="8" t="s">
+        <x:v>646</x:v>
+      </x:c>
+      <x:c r="B18" s="7" t="s">
         <x:v>647</x:v>
       </x:c>
-      <x:c r="B18" s="7" t="s">
+      <x:c r="C18" s="7" t="s">
         <x:v>648</x:v>
       </x:c>
-      <x:c r="C18" s="7" t="s">
+      <x:c r="D18" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="s">
         <x:v>649</x:v>
-      </x:c>
-      <x:c r="D18" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E18" s="10" t="s">
-        <x:v>650</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
       <x:c r="A19" s="8" t="s">
+        <x:v>650</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="s">
         <x:v>651</x:v>
       </x:c>
-      <x:c r="B19" s="7" t="s">
+      <x:c r="C19" s="7" t="s">
         <x:v>652</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="s">
-        <x:v>653</x:v>
       </x:c>
       <x:c r="D19" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E19" s="10" t="s">
-        <x:v>654</x:v>
+        <x:v>653</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28" customHeight="1">
       <x:c r="A20" s="8" t="s">
+        <x:v>654</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="s">
         <x:v>655</x:v>
       </x:c>
-      <x:c r="B20" s="7" t="s">
+      <x:c r="C20" s="7" t="s">
         <x:v>656</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>657</x:v>
       </x:c>
       <x:c r="D20" s="9">
         <x:v>1</x:v>
@@ -7713,10 +7710,10 @@
     </x:row>
     <x:row r="21" ht="28" customHeight="1">
       <x:c r="A21" s="8" t="s">
+        <x:v>657</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="s">
         <x:v>658</x:v>
-      </x:c>
-      <x:c r="B21" s="7" t="s">
-        <x:v>659</x:v>
       </x:c>
       <x:c r="C21" s="7" t="str">
         <x:v>#069, #071, #079</x:v>
@@ -7725,18 +7722,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E21" s="10" t="s">
-        <x:v>660</x:v>
+        <x:v>659</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
       <x:c r="A22" s="8" t="s">
+        <x:v>660</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="s">
         <x:v>661</x:v>
       </x:c>
-      <x:c r="B22" s="7" t="s">
+      <x:c r="C22" s="7" t="s">
         <x:v>662</x:v>
-      </x:c>
-      <x:c r="C22" s="7" t="s">
-        <x:v>663</x:v>
       </x:c>
       <x:c r="D22" s="9">
         <x:v>1</x:v>
@@ -7745,13 +7742,13 @@
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
       <x:c r="A23" s="8" t="s">
+        <x:v>663</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="s">
         <x:v>664</x:v>
       </x:c>
-      <x:c r="B23" s="7" t="s">
+      <x:c r="C23" s="7" t="s">
         <x:v>665</x:v>
-      </x:c>
-      <x:c r="C23" s="7" t="s">
-        <x:v>666</x:v>
       </x:c>
       <x:c r="D23" s="9">
         <x:v>1</x:v>
@@ -7760,10 +7757,10 @@
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
       <x:c r="A24" s="8" t="s">
+        <x:v>666</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="s">
         <x:v>667</x:v>
-      </x:c>
-      <x:c r="B24" s="7" t="s">
-        <x:v>668</x:v>
       </x:c>
       <x:c r="C24" s="7" t="str">
         <x:v>#054, #055, #056, #062, #066, #068, #075</x:v>
@@ -7772,12 +7769,12 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E24" s="10" t="s">
-        <x:v>669</x:v>
+        <x:v>668</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
       <x:c r="A25" s="8" t="s">
-        <x:v>670</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
         <x:v>Clement Lork</x:v>
@@ -7789,18 +7786,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E25" s="10" t="s">
-        <x:v>671</x:v>
+        <x:v>670</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="8" t="s">
+        <x:v>671</x:v>
+      </x:c>
+      <x:c r="B26" s="7" t="s">
         <x:v>672</x:v>
       </x:c>
-      <x:c r="B26" s="7" t="s">
-        <x:v>673</x:v>
-      </x:c>
       <x:c r="C26" s="7" t="s">
-        <x:v>612</x:v>
+        <x:v>611</x:v>
       </x:c>
       <x:c r="D26" s="9">
         <x:v>1</x:v>
@@ -7809,13 +7806,13 @@
     </x:row>
     <x:row r="27" ht="28" customHeight="1">
       <x:c r="A27" s="8" t="s">
+        <x:v>673</x:v>
+      </x:c>
+      <x:c r="B27" s="7" t="s">
         <x:v>674</x:v>
       </x:c>
-      <x:c r="B27" s="7" t="s">
+      <x:c r="C27" s="7" t="s">
         <x:v>675</x:v>
-      </x:c>
-      <x:c r="C27" s="7" t="s">
-        <x:v>676</x:v>
       </x:c>
       <x:c r="D27" s="9">
         <x:v>1</x:v>
@@ -7824,13 +7821,13 @@
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
       <x:c r="A28" s="8" t="s">
+        <x:v>676</x:v>
+      </x:c>
+      <x:c r="B28" s="7" t="s">
         <x:v>677</x:v>
       </x:c>
-      <x:c r="B28" s="7" t="s">
+      <x:c r="C28" s="7" t="s">
         <x:v>678</x:v>
-      </x:c>
-      <x:c r="C28" s="7" t="s">
-        <x:v>679</x:v>
       </x:c>
       <x:c r="D28" s="9">
         <x:v>2</x:v>
@@ -7839,13 +7836,13 @@
     </x:row>
     <x:row r="29" ht="28" customHeight="1">
       <x:c r="A29" s="8" t="s">
+        <x:v>679</x:v>
+      </x:c>
+      <x:c r="B29" s="7" t="s">
         <x:v>680</x:v>
       </x:c>
-      <x:c r="B29" s="7" t="s">
+      <x:c r="C29" s="7" t="s">
         <x:v>681</x:v>
-      </x:c>
-      <x:c r="C29" s="7" t="s">
-        <x:v>682</x:v>
       </x:c>
       <x:c r="D29" s="9">
         <x:v>4</x:v>
@@ -7854,13 +7851,13 @@
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
       <x:c r="A30" s="8" t="s">
+        <x:v>682</x:v>
+      </x:c>
+      <x:c r="B30" s="7" t="s">
         <x:v>683</x:v>
       </x:c>
-      <x:c r="B30" s="7" t="s">
-        <x:v>684</x:v>
-      </x:c>
       <x:c r="C30" s="7" t="s">
-        <x:v>676</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="D30" s="9">
         <x:v>1</x:v>
@@ -7869,47 +7866,47 @@
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="8" t="s">
+        <x:v>684</x:v>
+      </x:c>
+      <x:c r="B31" s="7" t="s">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="B31" s="7" t="s">
+      <x:c r="C31" s="7" t="s">
+        <x:v>624</x:v>
+      </x:c>
+      <x:c r="D31" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E31" s="10" t="s">
         <x:v>686</x:v>
-      </x:c>
-      <x:c r="C31" s="7" t="s">
-        <x:v>625</x:v>
-      </x:c>
-      <x:c r="D31" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E31" s="10" t="s">
-        <x:v>687</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="28" customHeight="1">
       <x:c r="A32" s="8" t="s">
+        <x:v>687</x:v>
+      </x:c>
+      <x:c r="B32" s="7" t="s">
         <x:v>688</x:v>
       </x:c>
-      <x:c r="B32" s="7" t="s">
+      <x:c r="C32" s="7" t="s">
         <x:v>689</x:v>
       </x:c>
-      <x:c r="C32" s="7" t="s">
+      <x:c r="D32" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E32" s="10" t="s">
         <x:v>690</x:v>
-      </x:c>
-      <x:c r="D32" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E32" s="10" t="s">
-        <x:v>691</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="8" t="s">
+        <x:v>691</x:v>
+      </x:c>
+      <x:c r="B33" s="7" t="s">
         <x:v>692</x:v>
       </x:c>
-      <x:c r="B33" s="7" t="s">
-        <x:v>693</x:v>
-      </x:c>
       <x:c r="C33" s="7" t="s">
-        <x:v>663</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="D33" s="9">
         <x:v>1</x:v>
@@ -7918,13 +7915,13 @@
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
       <x:c r="A34" s="8" t="s">
+        <x:v>693</x:v>
+      </x:c>
+      <x:c r="B34" s="7" t="s">
         <x:v>694</x:v>
       </x:c>
-      <x:c r="B34" s="7" t="s">
+      <x:c r="C34" s="7" t="s">
         <x:v>695</x:v>
-      </x:c>
-      <x:c r="C34" s="7" t="s">
-        <x:v>696</x:v>
       </x:c>
       <x:c r="D34" s="9">
         <x:v>1</x:v>
@@ -7933,47 +7930,47 @@
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
       <x:c r="A35" s="8" t="s">
+        <x:v>696</x:v>
+      </x:c>
+      <x:c r="B35" s="7" t="s">
         <x:v>697</x:v>
       </x:c>
-      <x:c r="B35" s="7" t="s">
+      <x:c r="C35" s="7" t="s">
         <x:v>698</x:v>
       </x:c>
-      <x:c r="C35" s="7" t="s">
+      <x:c r="D35" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E35" s="10" t="s">
         <x:v>699</x:v>
-      </x:c>
-      <x:c r="D35" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E35" s="10" t="s">
-        <x:v>700</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
       <x:c r="A36" s="8" t="s">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="B36" s="7" t="s">
         <x:v>701</x:v>
       </x:c>
-      <x:c r="B36" s="7" t="s">
+      <x:c r="C36" s="7" t="s">
         <x:v>702</x:v>
       </x:c>
-      <x:c r="C36" s="7" t="s">
+      <x:c r="D36" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E36" s="10" t="s">
         <x:v>703</x:v>
-      </x:c>
-      <x:c r="D36" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E36" s="10" t="s">
-        <x:v>704</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
       <x:c r="A37" s="8" t="s">
+        <x:v>704</x:v>
+      </x:c>
+      <x:c r="B37" s="7" t="s">
         <x:v>705</x:v>
       </x:c>
-      <x:c r="B37" s="7" t="s">
+      <x:c r="C37" s="7" t="s">
         <x:v>706</x:v>
-      </x:c>
-      <x:c r="C37" s="7" t="s">
-        <x:v>707</x:v>
       </x:c>
       <x:c r="D37" s="9">
         <x:v>1</x:v>
@@ -7982,13 +7979,13 @@
     </x:row>
     <x:row r="38" ht="28" customHeight="1">
       <x:c r="A38" s="8" t="s">
+        <x:v>707</x:v>
+      </x:c>
+      <x:c r="B38" s="7" t="s">
         <x:v>708</x:v>
       </x:c>
-      <x:c r="B38" s="7" t="s">
-        <x:v>709</x:v>
-      </x:c>
       <x:c r="C38" s="7" t="s">
-        <x:v>646</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="D38" s="9">
         <x:v>1</x:v>
@@ -7997,13 +7994,13 @@
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
       <x:c r="A39" s="8" t="s">
+        <x:v>709</x:v>
+      </x:c>
+      <x:c r="B39" s="7" t="s">
         <x:v>710</x:v>
       </x:c>
-      <x:c r="B39" s="7" t="s">
+      <x:c r="C39" s="7" t="s">
         <x:v>711</x:v>
-      </x:c>
-      <x:c r="C39" s="7" t="s">
-        <x:v>712</x:v>
       </x:c>
       <x:c r="D39" s="9">
         <x:v>3</x:v>
@@ -8012,47 +8009,47 @@
     </x:row>
     <x:row r="40" ht="28" customHeight="1">
       <x:c r="A40" s="8" t="s">
+        <x:v>712</x:v>
+      </x:c>
+      <x:c r="B40" s="7" t="s">
         <x:v>713</x:v>
       </x:c>
-      <x:c r="B40" s="7" t="s">
+      <x:c r="C40" s="7" t="s">
         <x:v>714</x:v>
       </x:c>
-      <x:c r="C40" s="7" t="s">
+      <x:c r="D40" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E40" s="10" t="s">
         <x:v>715</x:v>
-      </x:c>
-      <x:c r="D40" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E40" s="10" t="s">
-        <x:v>716</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="8" t="s">
+        <x:v>716</x:v>
+      </x:c>
+      <x:c r="B41" s="7" t="s">
         <x:v>717</x:v>
       </x:c>
-      <x:c r="B41" s="7" t="s">
+      <x:c r="C41" s="7" t="s">
+        <x:v>714</x:v>
+      </x:c>
+      <x:c r="D41" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E41" s="10" t="s">
         <x:v>718</x:v>
-      </x:c>
-      <x:c r="C41" s="7" t="s">
-        <x:v>715</x:v>
-      </x:c>
-      <x:c r="D41" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E41" s="10" t="s">
-        <x:v>719</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
       <x:c r="A42" s="8" t="s">
+        <x:v>719</x:v>
+      </x:c>
+      <x:c r="B42" s="7" t="s">
         <x:v>720</x:v>
       </x:c>
-      <x:c r="B42" s="7" t="s">
+      <x:c r="C42" s="7" t="s">
         <x:v>721</x:v>
-      </x:c>
-      <x:c r="C42" s="7" t="s">
-        <x:v>722</x:v>
       </x:c>
       <x:c r="D42" s="9">
         <x:v>1</x:v>
@@ -8061,10 +8058,10 @@
     </x:row>
     <x:row r="43" ht="28" customHeight="1">
       <x:c r="A43" s="8" t="s">
+        <x:v>722</x:v>
+      </x:c>
+      <x:c r="B43" s="7" t="s">
         <x:v>723</x:v>
-      </x:c>
-      <x:c r="B43" s="7" t="s">
-        <x:v>724</x:v>
       </x:c>
       <x:c r="C43" s="7" t="str">
         <x:v>#069, #079</x:v>
@@ -8076,30 +8073,30 @@
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="8" t="s">
+        <x:v>724</x:v>
+      </x:c>
+      <x:c r="B44" s="7" t="s">
         <x:v>725</x:v>
       </x:c>
-      <x:c r="B44" s="7" t="s">
-        <x:v>726</x:v>
-      </x:c>
       <x:c r="C44" s="7" t="s">
-        <x:v>679</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="D44" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E44" s="10" t="s">
-        <x:v>727</x:v>
+        <x:v>726</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
       <x:c r="A45" s="8" t="s">
+        <x:v>727</x:v>
+      </x:c>
+      <x:c r="B45" s="7" t="s">
         <x:v>728</x:v>
       </x:c>
-      <x:c r="B45" s="7" t="s">
+      <x:c r="C45" s="7" t="s">
         <x:v>729</x:v>
-      </x:c>
-      <x:c r="C45" s="7" t="s">
-        <x:v>730</x:v>
       </x:c>
       <x:c r="D45" s="9">
         <x:v>1</x:v>
@@ -8108,13 +8105,13 @@
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
       <x:c r="A46" s="8" t="s">
+        <x:v>730</x:v>
+      </x:c>
+      <x:c r="B46" s="7" t="s">
         <x:v>731</x:v>
       </x:c>
-      <x:c r="B46" s="7" t="s">
-        <x:v>732</x:v>
-      </x:c>
       <x:c r="C46" s="7" t="s">
-        <x:v>696</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="D46" s="9">
         <x:v>1</x:v>
@@ -8123,47 +8120,47 @@
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
       <x:c r="A47" s="8" t="s">
+        <x:v>732</x:v>
+      </x:c>
+      <x:c r="B47" s="7" t="s">
         <x:v>733</x:v>
       </x:c>
-      <x:c r="B47" s="7" t="s">
+      <x:c r="C47" s="7" t="s">
+        <x:v>607</x:v>
+      </x:c>
+      <x:c r="D47" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E47" s="10" t="s">
         <x:v>734</x:v>
-      </x:c>
-      <x:c r="C47" s="7" t="s">
-        <x:v>608</x:v>
-      </x:c>
-      <x:c r="D47" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E47" s="10" t="s">
-        <x:v>735</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
       <x:c r="A48" s="8" t="s">
+        <x:v>735</x:v>
+      </x:c>
+      <x:c r="B48" s="7" t="s">
         <x:v>736</x:v>
       </x:c>
-      <x:c r="B48" s="7" t="s">
+      <x:c r="C48" s="7" t="s">
         <x:v>737</x:v>
-      </x:c>
-      <x:c r="C48" s="7" t="s">
-        <x:v>738</x:v>
       </x:c>
       <x:c r="D48" s="9">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="10" t="s">
-        <x:v>739</x:v>
+        <x:v>738</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
       <x:c r="A49" s="8" t="s">
+        <x:v>739</x:v>
+      </x:c>
+      <x:c r="B49" s="7" t="s">
         <x:v>740</x:v>
       </x:c>
-      <x:c r="B49" s="7" t="s">
+      <x:c r="C49" s="7" t="s">
         <x:v>741</x:v>
-      </x:c>
-      <x:c r="C49" s="7" t="s">
-        <x:v>742</x:v>
       </x:c>
       <x:c r="D49" s="9">
         <x:v>1</x:v>
@@ -8172,13 +8169,13 @@
     </x:row>
     <x:row r="50" ht="28" customHeight="1">
       <x:c r="A50" s="8" t="s">
+        <x:v>742</x:v>
+      </x:c>
+      <x:c r="B50" s="7" t="s">
         <x:v>743</x:v>
       </x:c>
-      <x:c r="B50" s="7" t="s">
-        <x:v>744</x:v>
-      </x:c>
       <x:c r="C50" s="7" t="s">
-        <x:v>707</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="D50" s="9">
         <x:v>1</x:v>
@@ -8187,64 +8184,64 @@
     </x:row>
     <x:row r="51" ht="28" customHeight="1">
       <x:c r="A51" s="8" t="s">
+        <x:v>744</x:v>
+      </x:c>
+      <x:c r="B51" s="7" t="s">
         <x:v>745</x:v>
       </x:c>
-      <x:c r="B51" s="7" t="s">
+      <x:c r="C51" s="7" t="s">
         <x:v>746</x:v>
-      </x:c>
-      <x:c r="C51" s="7" t="s">
-        <x:v>747</x:v>
       </x:c>
       <x:c r="D51" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E51" s="10" t="s">
-        <x:v>748</x:v>
+        <x:v>747</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="28" customHeight="1">
       <x:c r="A52" s="8" t="s">
+        <x:v>748</x:v>
+      </x:c>
+      <x:c r="B52" s="7" t="s">
         <x:v>749</x:v>
       </x:c>
-      <x:c r="B52" s="7" t="s">
+      <x:c r="C52" s="7" t="s">
         <x:v>750</x:v>
       </x:c>
-      <x:c r="C52" s="7" t="s">
+      <x:c r="D52" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E52" s="10" t="s">
         <x:v>751</x:v>
-      </x:c>
-      <x:c r="D52" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E52" s="10" t="s">
-        <x:v>752</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="28" customHeight="1">
       <x:c r="A53" s="8" t="s">
+        <x:v>752</x:v>
+      </x:c>
+      <x:c r="B53" s="7" t="s">
         <x:v>753</x:v>
       </x:c>
-      <x:c r="B53" s="7" t="s">
+      <x:c r="C53" s="7" t="s">
         <x:v>754</x:v>
-      </x:c>
-      <x:c r="C53" s="7" t="s">
-        <x:v>755</x:v>
       </x:c>
       <x:c r="D53" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E53" s="10" t="s">
-        <x:v>756</x:v>
+        <x:v>755</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="28" customHeight="1">
       <x:c r="A54" s="8" t="s">
+        <x:v>756</x:v>
+      </x:c>
+      <x:c r="B54" s="7" t="s">
         <x:v>757</x:v>
       </x:c>
-      <x:c r="B54" s="7" t="s">
+      <x:c r="C54" s="7" t="s">
         <x:v>758</x:v>
-      </x:c>
-      <x:c r="C54" s="7" t="s">
-        <x:v>759</x:v>
       </x:c>
       <x:c r="D54" s="9">
         <x:v>1</x:v>
@@ -8253,81 +8250,81 @@
     </x:row>
     <x:row r="55" ht="28" customHeight="1">
       <x:c r="A55" s="8" t="s">
+        <x:v>759</x:v>
+      </x:c>
+      <x:c r="B55" s="7" t="s">
         <x:v>760</x:v>
       </x:c>
-      <x:c r="B55" s="7" t="s">
+      <x:c r="C55" s="7" t="s">
         <x:v>761</x:v>
       </x:c>
-      <x:c r="C55" s="7" t="s">
+      <x:c r="D55" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E55" s="10" t="s">
         <x:v>762</x:v>
-      </x:c>
-      <x:c r="D55" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E55" s="10" t="s">
-        <x:v>763</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="28" customHeight="1">
       <x:c r="A56" s="8" t="s">
+        <x:v>763</x:v>
+      </x:c>
+      <x:c r="B56" s="7" t="s">
         <x:v>764</x:v>
       </x:c>
-      <x:c r="B56" s="7" t="s">
+      <x:c r="C56" s="7" t="s">
         <x:v>765</x:v>
       </x:c>
-      <x:c r="C56" s="7" t="s">
+      <x:c r="D56" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E56" s="10" t="s">
         <x:v>766</x:v>
-      </x:c>
-      <x:c r="D56" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E56" s="10" t="s">
-        <x:v>767</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
       <x:c r="A57" s="8" t="s">
+        <x:v>767</x:v>
+      </x:c>
+      <x:c r="B57" s="7" t="s">
         <x:v>768</x:v>
       </x:c>
-      <x:c r="B57" s="7" t="s">
+      <x:c r="C57" s="7" t="s">
         <x:v>769</x:v>
       </x:c>
-      <x:c r="C57" s="7" t="s">
+      <x:c r="D57" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E57" s="10" t="s">
         <x:v>770</x:v>
-      </x:c>
-      <x:c r="D57" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E57" s="10" t="s">
-        <x:v>771</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
       <x:c r="A58" s="8" t="s">
+        <x:v>771</x:v>
+      </x:c>
+      <x:c r="B58" s="7" t="s">
         <x:v>772</x:v>
       </x:c>
-      <x:c r="B58" s="7" t="s">
+      <x:c r="C58" s="7" t="s">
         <x:v>773</x:v>
-      </x:c>
-      <x:c r="C58" s="7" t="s">
-        <x:v>774</x:v>
       </x:c>
       <x:c r="D58" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E58" s="10" t="s">
-        <x:v>775</x:v>
+        <x:v>774</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
       <x:c r="A59" s="8" t="s">
+        <x:v>775</x:v>
+      </x:c>
+      <x:c r="B59" s="7" t="s">
         <x:v>776</x:v>
       </x:c>
-      <x:c r="B59" s="7" t="s">
-        <x:v>777</x:v>
-      </x:c>
       <x:c r="C59" s="7" t="s">
-        <x:v>612</x:v>
+        <x:v>611</x:v>
       </x:c>
       <x:c r="D59" s="9">
         <x:v>1</x:v>
@@ -8336,13 +8333,13 @@
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
       <x:c r="A60" s="8" t="s">
+        <x:v>777</x:v>
+      </x:c>
+      <x:c r="B60" s="7" t="s">
         <x:v>778</x:v>
       </x:c>
-      <x:c r="B60" s="7" t="s">
-        <x:v>779</x:v>
-      </x:c>
       <x:c r="C60" s="7" t="s">
-        <x:v>649</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="D60" s="9">
         <x:v>1</x:v>
@@ -8351,13 +8348,13 @@
     </x:row>
     <x:row r="61" ht="28" customHeight="1">
       <x:c r="A61" s="8" t="s">
+        <x:v>779</x:v>
+      </x:c>
+      <x:c r="B61" s="7" t="s">
         <x:v>780</x:v>
       </x:c>
-      <x:c r="B61" s="7" t="s">
-        <x:v>781</x:v>
-      </x:c>
       <x:c r="C61" s="7" t="s">
-        <x:v>633</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="D61" s="9">
         <x:v>1</x:v>
@@ -8366,30 +8363,30 @@
     </x:row>
     <x:row r="62" ht="28" customHeight="1">
       <x:c r="A62" s="8" t="s">
+        <x:v>781</x:v>
+      </x:c>
+      <x:c r="B62" s="7" t="s">
         <x:v>782</x:v>
       </x:c>
-      <x:c r="B62" s="7" t="s">
+      <x:c r="C62" s="7" t="s">
+        <x:v>638</x:v>
+      </x:c>
+      <x:c r="D62" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E62" s="10" t="s">
         <x:v>783</x:v>
-      </x:c>
-      <x:c r="C62" s="7" t="s">
-        <x:v>639</x:v>
-      </x:c>
-      <x:c r="D62" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E62" s="10" t="s">
-        <x:v>784</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="28" customHeight="1">
       <x:c r="A63" s="8" t="s">
+        <x:v>784</x:v>
+      </x:c>
+      <x:c r="B63" s="7" t="s">
         <x:v>785</x:v>
       </x:c>
-      <x:c r="B63" s="7" t="s">
-        <x:v>786</x:v>
-      </x:c>
       <x:c r="C63" s="7" t="s">
-        <x:v>633</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="D63" s="9">
         <x:v>1</x:v>
@@ -8398,13 +8395,13 @@
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
       <x:c r="A64" s="8" t="s">
+        <x:v>786</x:v>
+      </x:c>
+      <x:c r="B64" s="7" t="s">
         <x:v>787</x:v>
       </x:c>
-      <x:c r="B64" s="7" t="s">
+      <x:c r="C64" s="7" t="s">
         <x:v>788</x:v>
-      </x:c>
-      <x:c r="C64" s="7" t="s">
-        <x:v>789</x:v>
       </x:c>
       <x:c r="D64" s="9">
         <x:v>1</x:v>
@@ -8413,13 +8410,13 @@
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
       <x:c r="A65" s="8" t="s">
+        <x:v>789</x:v>
+      </x:c>
+      <x:c r="B65" s="7" t="s">
         <x:v>790</x:v>
       </x:c>
-      <x:c r="B65" s="7" t="s">
+      <x:c r="C65" s="7" t="s">
         <x:v>791</x:v>
-      </x:c>
-      <x:c r="C65" s="7" t="s">
-        <x:v>792</x:v>
       </x:c>
       <x:c r="D65" s="9">
         <x:v>1</x:v>
@@ -8428,13 +8425,13 @@
     </x:row>
     <x:row r="66" ht="28" customHeight="1">
       <x:c r="A66" s="8" t="s">
+        <x:v>792</x:v>
+      </x:c>
+      <x:c r="B66" s="7" t="s">
         <x:v>793</x:v>
       </x:c>
-      <x:c r="B66" s="7" t="s">
-        <x:v>794</x:v>
-      </x:c>
       <x:c r="C66" s="7" t="s">
-        <x:v>622</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="D66" s="9">
         <x:v>1</x:v>
@@ -8443,47 +8440,47 @@
     </x:row>
     <x:row r="67" ht="28" customHeight="1">
       <x:c r="A67" s="8" t="s">
+        <x:v>794</x:v>
+      </x:c>
+      <x:c r="B67" s="7" t="s">
         <x:v>795</x:v>
       </x:c>
-      <x:c r="B67" s="7" t="s">
-        <x:v>796</x:v>
-      </x:c>
       <x:c r="C67" s="7" t="s">
-        <x:v>774</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="D67" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E67" s="10" t="s">
-        <x:v>797</x:v>
+        <x:v>796</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="28" customHeight="1">
       <x:c r="A68" s="8" t="s">
+        <x:v>797</x:v>
+      </x:c>
+      <x:c r="B68" s="7" t="s">
         <x:v>798</x:v>
       </x:c>
-      <x:c r="B68" s="7" t="s">
+      <x:c r="C68" s="7" t="s">
+        <x:v>648</x:v>
+      </x:c>
+      <x:c r="D68" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E68" s="10" t="s">
         <x:v>799</x:v>
-      </x:c>
-      <x:c r="C68" s="7" t="s">
-        <x:v>649</x:v>
-      </x:c>
-      <x:c r="D68" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E68" s="10" t="s">
-        <x:v>800</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
       <x:c r="A69" s="8" t="s">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="B69" s="7" t="s">
         <x:v>801</x:v>
       </x:c>
-      <x:c r="B69" s="7" t="s">
-        <x:v>802</x:v>
-      </x:c>
       <x:c r="C69" s="7" t="s">
-        <x:v>629</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="D69" s="9">
         <x:v>1</x:v>
@@ -8492,13 +8489,13 @@
     </x:row>
     <x:row r="70" ht="28" customHeight="1">
       <x:c r="A70" s="8" t="s">
+        <x:v>802</x:v>
+      </x:c>
+      <x:c r="B70" s="7" t="s">
         <x:v>803</x:v>
       </x:c>
-      <x:c r="B70" s="7" t="s">
-        <x:v>804</x:v>
-      </x:c>
       <x:c r="C70" s="7" t="s">
-        <x:v>657</x:v>
+        <x:v>656</x:v>
       </x:c>
       <x:c r="D70" s="9">
         <x:v>1</x:v>
@@ -8507,13 +8504,13 @@
     </x:row>
     <x:row r="71" ht="28" customHeight="1">
       <x:c r="A71" s="8" t="s">
+        <x:v>804</x:v>
+      </x:c>
+      <x:c r="B71" s="7" t="s">
         <x:v>805</x:v>
       </x:c>
-      <x:c r="B71" s="7" t="s">
+      <x:c r="C71" s="7" t="s">
         <x:v>806</x:v>
-      </x:c>
-      <x:c r="C71" s="7" t="s">
-        <x:v>807</x:v>
       </x:c>
       <x:c r="D71" s="9">
         <x:v>1</x:v>
@@ -8522,64 +8519,64 @@
     </x:row>
     <x:row r="72" ht="28" customHeight="1">
       <x:c r="A72" s="8" t="s">
+        <x:v>807</x:v>
+      </x:c>
+      <x:c r="B72" s="7" t="s">
         <x:v>808</x:v>
       </x:c>
-      <x:c r="B72" s="7" t="s">
+      <x:c r="C72" s="7" t="s">
         <x:v>809</x:v>
-      </x:c>
-      <x:c r="C72" s="7" t="s">
-        <x:v>810</x:v>
       </x:c>
       <x:c r="D72" s="9">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E72" s="10" t="s">
-        <x:v>811</x:v>
+        <x:v>810</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="28" customHeight="1">
       <x:c r="A73" s="8" t="s">
+        <x:v>811</x:v>
+      </x:c>
+      <x:c r="B73" s="7" t="s">
         <x:v>812</x:v>
       </x:c>
-      <x:c r="B73" s="7" t="s">
+      <x:c r="C73" s="7" t="s">
         <x:v>813</x:v>
       </x:c>
-      <x:c r="C73" s="7" t="s">
+      <x:c r="D73" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E73" s="10" t="s">
         <x:v>814</x:v>
-      </x:c>
-      <x:c r="D73" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E73" s="10" t="s">
-        <x:v>815</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="28" customHeight="1">
       <x:c r="A74" s="8" t="s">
+        <x:v>815</x:v>
+      </x:c>
+      <x:c r="B74" s="7" t="s">
         <x:v>816</x:v>
       </x:c>
-      <x:c r="B74" s="7" t="s">
+      <x:c r="C74" s="7" t="s">
+        <x:v>614</x:v>
+      </x:c>
+      <x:c r="D74" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E74" s="10" t="s">
         <x:v>817</x:v>
-      </x:c>
-      <x:c r="C74" s="7" t="s">
-        <x:v>615</x:v>
-      </x:c>
-      <x:c r="D74" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E74" s="10" t="s">
-        <x:v>818</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="28" customHeight="1">
       <x:c r="A75" s="8" t="s">
+        <x:v>818</x:v>
+      </x:c>
+      <x:c r="B75" s="7" t="s">
         <x:v>819</x:v>
       </x:c>
-      <x:c r="B75" s="7" t="s">
-        <x:v>820</x:v>
-      </x:c>
       <x:c r="C75" s="7" t="s">
-        <x:v>730</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="D75" s="9">
         <x:v>1</x:v>
@@ -8588,64 +8585,64 @@
     </x:row>
     <x:row r="76" ht="28" customHeight="1">
       <x:c r="A76" s="8" t="s">
+        <x:v>820</x:v>
+      </x:c>
+      <x:c r="B76" s="7" t="s">
         <x:v>821</x:v>
       </x:c>
-      <x:c r="B76" s="7" t="s">
+      <x:c r="C76" s="7" t="s">
+        <x:v>698</x:v>
+      </x:c>
+      <x:c r="D76" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E76" s="10" t="s">
         <x:v>822</x:v>
-      </x:c>
-      <x:c r="C76" s="7" t="s">
-        <x:v>699</x:v>
-      </x:c>
-      <x:c r="D76" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E76" s="10" t="s">
-        <x:v>823</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
       <x:c r="A77" s="8" t="s">
+        <x:v>823</x:v>
+      </x:c>
+      <x:c r="B77" s="7" t="s">
         <x:v>824</x:v>
       </x:c>
-      <x:c r="B77" s="7" t="s">
+      <x:c r="C77" s="7" t="s">
+        <x:v>806</x:v>
+      </x:c>
+      <x:c r="D77" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E77" s="10" t="s">
         <x:v>825</x:v>
-      </x:c>
-      <x:c r="C77" s="7" t="s">
-        <x:v>807</x:v>
-      </x:c>
-      <x:c r="D77" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E77" s="10" t="s">
-        <x:v>826</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
       <x:c r="A78" s="8" t="s">
+        <x:v>826</x:v>
+      </x:c>
+      <x:c r="B78" s="7" t="s">
         <x:v>827</x:v>
       </x:c>
-      <x:c r="B78" s="7" t="s">
-        <x:v>828</x:v>
-      </x:c>
       <x:c r="C78" s="7" t="s">
-        <x:v>604</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="D78" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E78" s="10" t="s">
-        <x:v>829</x:v>
+        <x:v>828</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="28" customHeight="1">
       <x:c r="A79" s="8" t="s">
+        <x:v>829</x:v>
+      </x:c>
+      <x:c r="B79" s="7" t="s">
         <x:v>830</x:v>
       </x:c>
-      <x:c r="B79" s="7" t="s">
-        <x:v>831</x:v>
-      </x:c>
       <x:c r="C79" s="7" t="s">
-        <x:v>699</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="D79" s="9">
         <x:v>1</x:v>
@@ -8654,24 +8651,24 @@
     </x:row>
     <x:row r="80" ht="28" customHeight="1">
       <x:c r="A80" s="8" t="s">
+        <x:v>831</x:v>
+      </x:c>
+      <x:c r="B80" s="7" t="s">
         <x:v>832</x:v>
       </x:c>
-      <x:c r="B80" s="7" t="s">
+      <x:c r="C80" s="7" t="s">
         <x:v>833</x:v>
       </x:c>
-      <x:c r="C80" s="7" t="s">
+      <x:c r="D80" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E80" s="10" t="s">
         <x:v>834</x:v>
-      </x:c>
-      <x:c r="D80" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E80" s="10" t="s">
-        <x:v>835</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="28" customHeight="1">
       <x:c r="A81" s="8" t="s">
-        <x:v>836</x:v>
+        <x:v>835</x:v>
       </x:c>
       <x:c r="B81" s="7" t="s">
         <x:v>172</x:v>
@@ -8683,35 +8680,35 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="E81" s="10" t="s">
-        <x:v>837</x:v>
+        <x:v>836</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="28" customHeight="1">
       <x:c r="A82" s="8" t="s">
+        <x:v>837</x:v>
+      </x:c>
+      <x:c r="B82" s="7" t="s">
         <x:v>838</x:v>
       </x:c>
-      <x:c r="B82" s="7" t="s">
+      <x:c r="C82" s="7" t="s">
         <x:v>839</x:v>
-      </x:c>
-      <x:c r="C82" s="7" t="s">
-        <x:v>840</x:v>
       </x:c>
       <x:c r="D82" s="9">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E82" s="10" t="s">
-        <x:v>841</x:v>
+        <x:v>840</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="28" customHeight="1">
       <x:c r="A83" s="8" t="s">
+        <x:v>841</x:v>
+      </x:c>
+      <x:c r="B83" s="7" t="s">
         <x:v>842</x:v>
       </x:c>
-      <x:c r="B83" s="7" t="s">
-        <x:v>843</x:v>
-      </x:c>
       <x:c r="C83" s="7" t="s">
-        <x:v>622</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="D83" s="9">
         <x:v>1</x:v>
@@ -8720,13 +8717,13 @@
     </x:row>
     <x:row r="84" ht="28" customHeight="1">
       <x:c r="A84" s="8" t="s">
+        <x:v>843</x:v>
+      </x:c>
+      <x:c r="B84" s="7" t="s">
         <x:v>844</x:v>
       </x:c>
-      <x:c r="B84" s="7" t="s">
+      <x:c r="C84" s="7" t="s">
         <x:v>845</x:v>
-      </x:c>
-      <x:c r="C84" s="7" t="s">
-        <x:v>846</x:v>
       </x:c>
       <x:c r="D84" s="9">
         <x:v>1</x:v>
@@ -8735,64 +8732,64 @@
     </x:row>
     <x:row r="85" ht="28" customHeight="1">
       <x:c r="A85" s="8" t="s">
+        <x:v>846</x:v>
+      </x:c>
+      <x:c r="B85" s="7" t="s">
         <x:v>847</x:v>
       </x:c>
-      <x:c r="B85" s="7" t="s">
+      <x:c r="C85" s="7" t="s">
+        <x:v>624</x:v>
+      </x:c>
+      <x:c r="D85" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E85" s="10" t="s">
         <x:v>848</x:v>
-      </x:c>
-      <x:c r="C85" s="7" t="s">
-        <x:v>625</x:v>
-      </x:c>
-      <x:c r="D85" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E85" s="10" t="s">
-        <x:v>849</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="28" customHeight="1">
       <x:c r="A86" s="8" t="s">
+        <x:v>849</x:v>
+      </x:c>
+      <x:c r="B86" s="7" t="s">
         <x:v>850</x:v>
       </x:c>
-      <x:c r="B86" s="7" t="s">
+      <x:c r="C86" s="7" t="s">
         <x:v>851</x:v>
       </x:c>
-      <x:c r="C86" s="7" t="s">
+      <x:c r="D86" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E86" s="10" t="s">
         <x:v>852</x:v>
-      </x:c>
-      <x:c r="D86" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E86" s="10" t="s">
-        <x:v>853</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="28" customHeight="1">
       <x:c r="A87" s="8" t="s">
+        <x:v>853</x:v>
+      </x:c>
+      <x:c r="B87" s="7" t="s">
         <x:v>854</x:v>
       </x:c>
-      <x:c r="B87" s="7" t="s">
+      <x:c r="C87" s="7" t="s">
         <x:v>855</x:v>
       </x:c>
-      <x:c r="C87" s="7" t="s">
+      <x:c r="D87" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E87" s="10" t="s">
         <x:v>856</x:v>
-      </x:c>
-      <x:c r="D87" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E87" s="10" t="s">
-        <x:v>857</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="28" customHeight="1">
       <x:c r="A88" s="8" t="s">
+        <x:v>857</x:v>
+      </x:c>
+      <x:c r="B88" s="7" t="s">
         <x:v>858</x:v>
       </x:c>
-      <x:c r="B88" s="7" t="s">
-        <x:v>859</x:v>
-      </x:c>
       <x:c r="C88" s="7" t="s">
-        <x:v>730</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="D88" s="9">
         <x:v>1</x:v>
@@ -8801,13 +8798,13 @@
     </x:row>
     <x:row r="89" ht="28" customHeight="1">
       <x:c r="A89" s="8" t="s">
+        <x:v>859</x:v>
+      </x:c>
+      <x:c r="B89" s="7" t="s">
         <x:v>860</x:v>
       </x:c>
-      <x:c r="B89" s="7" t="s">
-        <x:v>861</x:v>
-      </x:c>
       <x:c r="C89" s="7" t="s">
-        <x:v>646</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="D89" s="9">
         <x:v>1</x:v>
@@ -8816,30 +8813,30 @@
     </x:row>
     <x:row r="90" ht="28" customHeight="1">
       <x:c r="A90" s="8" t="s">
+        <x:v>861</x:v>
+      </x:c>
+      <x:c r="B90" s="7" t="s">
         <x:v>862</x:v>
       </x:c>
-      <x:c r="B90" s="7" t="s">
-        <x:v>863</x:v>
-      </x:c>
       <x:c r="C90" s="7" t="s">
-        <x:v>774</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="D90" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E90" s="10" t="s">
-        <x:v>864</x:v>
+        <x:v>863</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="28" customHeight="1">
       <x:c r="A91" s="8" t="s">
+        <x:v>864</x:v>
+      </x:c>
+      <x:c r="B91" s="7" t="s">
         <x:v>865</x:v>
       </x:c>
-      <x:c r="B91" s="7" t="s">
+      <x:c r="C91" s="7" t="s">
         <x:v>866</x:v>
-      </x:c>
-      <x:c r="C91" s="7" t="s">
-        <x:v>867</x:v>
       </x:c>
       <x:c r="D91" s="9">
         <x:v>1</x:v>
@@ -8848,30 +8845,30 @@
     </x:row>
     <x:row r="92" ht="28" customHeight="1">
       <x:c r="A92" s="8" t="s">
+        <x:v>867</x:v>
+      </x:c>
+      <x:c r="B92" s="7" t="s">
         <x:v>868</x:v>
       </x:c>
-      <x:c r="B92" s="7" t="s">
+      <x:c r="C92" s="7" t="s">
         <x:v>869</x:v>
-      </x:c>
-      <x:c r="C92" s="7" t="s">
-        <x:v>870</x:v>
       </x:c>
       <x:c r="D92" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E92" s="10" t="s">
-        <x:v>871</x:v>
+        <x:v>870</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="28" customHeight="1">
       <x:c r="A93" s="8" t="s">
+        <x:v>871</x:v>
+      </x:c>
+      <x:c r="B93" s="7" t="s">
         <x:v>872</x:v>
       </x:c>
-      <x:c r="B93" s="7" t="s">
-        <x:v>873</x:v>
-      </x:c>
       <x:c r="C93" s="7" t="s">
-        <x:v>807</x:v>
+        <x:v>806</x:v>
       </x:c>
       <x:c r="D93" s="9">
         <x:v>1</x:v>
@@ -8880,30 +8877,30 @@
     </x:row>
     <x:row r="94" ht="28" customHeight="1">
       <x:c r="A94" s="8" t="s">
+        <x:v>873</x:v>
+      </x:c>
+      <x:c r="B94" s="7" t="s">
         <x:v>874</x:v>
       </x:c>
-      <x:c r="B94" s="7" t="s">
+      <x:c r="C94" s="7" t="s">
+        <x:v>698</x:v>
+      </x:c>
+      <x:c r="D94" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E94" s="10" t="s">
         <x:v>875</x:v>
-      </x:c>
-      <x:c r="C94" s="7" t="s">
-        <x:v>699</x:v>
-      </x:c>
-      <x:c r="D94" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E94" s="10" t="s">
-        <x:v>876</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="28" customHeight="1">
       <x:c r="A95" s="8" t="s">
+        <x:v>876</x:v>
+      </x:c>
+      <x:c r="B95" s="7" t="s">
         <x:v>877</x:v>
       </x:c>
-      <x:c r="B95" s="7" t="s">
-        <x:v>878</x:v>
-      </x:c>
       <x:c r="C95" s="7" t="s">
-        <x:v>696</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="D95" s="9">
         <x:v>1</x:v>
@@ -8912,47 +8909,47 @@
     </x:row>
     <x:row r="96" ht="28" customHeight="1">
       <x:c r="A96" s="8" t="s">
+        <x:v>878</x:v>
+      </x:c>
+      <x:c r="B96" s="7" t="s">
         <x:v>879</x:v>
       </x:c>
-      <x:c r="B96" s="7" t="s">
+      <x:c r="C96" s="7" t="s">
         <x:v>880</x:v>
-      </x:c>
-      <x:c r="C96" s="7" t="s">
-        <x:v>881</x:v>
       </x:c>
       <x:c r="D96" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E96" s="10" t="s">
-        <x:v>882</x:v>
+        <x:v>881</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="28" customHeight="1">
       <x:c r="A97" s="8" t="s">
+        <x:v>882</x:v>
+      </x:c>
+      <x:c r="B97" s="7" t="s">
         <x:v>883</x:v>
       </x:c>
-      <x:c r="B97" s="7" t="s">
+      <x:c r="C97" s="7" t="s">
+        <x:v>845</x:v>
+      </x:c>
+      <x:c r="D97" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E97" s="10" t="s">
         <x:v>884</x:v>
-      </x:c>
-      <x:c r="C97" s="7" t="s">
-        <x:v>846</x:v>
-      </x:c>
-      <x:c r="D97" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E97" s="10" t="s">
-        <x:v>885</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="s">
+        <x:v>885</x:v>
+      </x:c>
+      <x:c r="B98" t="s">
         <x:v>886</x:v>
       </x:c>
-      <x:c r="B98" t="s">
+      <x:c r="C98" t="s">
         <x:v>887</x:v>
-      </x:c>
-      <x:c r="C98" t="s">
-        <x:v>888</x:v>
       </x:c>
       <x:c r="D98">
         <x:v>1</x:v>
@@ -8973,12 +8970,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rb3c9d81df03a4817"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R917ea9851b8b4f4f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rb8b900f310034500"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R580474e253304ace"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3efb391343944b07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1597c1ac4fd45ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8993,7 +8990,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>889</x:v>
+        <x:v>888</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -9881,7 +9878,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0396aacf4b0747cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re650d76b22f74a1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9897,27 +9894,27 @@
   <x:sheetData>
     <x:row r="1" ht="34.75" customHeight="1">
       <x:c r="A1" s="20" t="s">
-        <x:v>890</x:v>
+        <x:v>889</x:v>
       </x:c>
       <x:c r="B1" s="20"/>
       <x:c r="C1" s="20"/>
     </x:row>
     <x:row r="2" ht="45.25" customHeight="1">
       <x:c r="A2" s="21" t="s">
-        <x:v>891</x:v>
+        <x:v>890</x:v>
       </x:c>
       <x:c r="B2" s="21"/>
       <x:c r="C2" s="21"/>
     </x:row>
     <x:row r="4" ht="29.25" customHeight="1">
       <x:c r="A4" s="15" t="s">
+        <x:v>891</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="s">
         <x:v>892</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="s">
+      <x:c r="C4" s="15" t="s">
         <x:v>893</x:v>
-      </x:c>
-      <x:c r="C4" s="15" t="s">
-        <x:v>894</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.75" customHeight="1">
@@ -9925,7 +9922,7 @@
         <x:v>310</x:v>
       </x:c>
       <x:c r="B5" s="16" t="s">
-        <x:v>895</x:v>
+        <x:v>894</x:v>
       </x:c>
       <x:c r="C5" s="17"/>
     </x:row>
@@ -9934,7 +9931,7 @@
         <x:v>170</x:v>
       </x:c>
       <x:c r="B6" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C6" s="17"/>
     </x:row>
@@ -9943,7 +9940,7 @@
         <x:v>379</x:v>
       </x:c>
       <x:c r="B7" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C7" s="17"/>
     </x:row>
@@ -9952,7 +9949,7 @@
         <x:v>455</x:v>
       </x:c>
       <x:c r="B8" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C8" s="17"/>
     </x:row>
@@ -9961,7 +9958,7 @@
         <x:v>347</x:v>
       </x:c>
       <x:c r="B9" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C9" s="17"/>
     </x:row>
@@ -9970,27 +9967,27 @@
         <x:v>368</x:v>
       </x:c>
       <x:c r="B10" s="16" t="s">
+        <x:v>898</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="s">
         <x:v>899</x:v>
-      </x:c>
-      <x:c r="C10" s="17" t="s">
-        <x:v>900</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.75" customHeight="1">
       <x:c r="A11" s="16" t="s">
-        <x:v>901</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="B11" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C11" s="17"/>
     </x:row>
     <x:row r="12" ht="26.75" customHeight="1">
       <x:c r="A12" s="16" t="s">
+        <x:v>901</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="s">
         <x:v>902</x:v>
-      </x:c>
-      <x:c r="B12" s="16" t="s">
-        <x:v>903</x:v>
       </x:c>
       <x:c r="C12" s="17"/>
     </x:row>
@@ -9999,25 +9996,25 @@
         <x:v>303</x:v>
       </x:c>
       <x:c r="B13" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C13" s="17"/>
     </x:row>
     <x:row r="14" ht="26.75" customHeight="1">
       <x:c r="A14" s="16" t="s">
+        <x:v>903</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="s">
         <x:v>904</x:v>
-      </x:c>
-      <x:c r="B14" s="16" t="s">
-        <x:v>905</x:v>
       </x:c>
       <x:c r="C14" s="17"/>
     </x:row>
     <x:row r="15" ht="26.75" customHeight="1">
       <x:c r="A15" s="16" t="s">
+        <x:v>905</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="s">
         <x:v>906</x:v>
-      </x:c>
-      <x:c r="B15" s="16" t="s">
-        <x:v>907</x:v>
       </x:c>
       <x:c r="C15" s="17"/>
     </x:row>
@@ -10026,7 +10023,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B16" s="16" t="s">
-        <x:v>908</x:v>
+        <x:v>907</x:v>
       </x:c>
       <x:c r="C16" s="17"/>
     </x:row>
@@ -10035,7 +10032,7 @@
         <x:v>198</x:v>
       </x:c>
       <x:c r="B17" s="16" t="s">
-        <x:v>908</x:v>
+        <x:v>907</x:v>
       </x:c>
       <x:c r="C17" s="17"/>
     </x:row>
@@ -10044,7 +10041,7 @@
         <x:v>405</x:v>
       </x:c>
       <x:c r="B18" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C18" s="17"/>
     </x:row>
@@ -10053,25 +10050,25 @@
         <x:v>260</x:v>
       </x:c>
       <x:c r="B19" s="16" t="s">
-        <x:v>895</x:v>
+        <x:v>894</x:v>
       </x:c>
       <x:c r="C19" s="17"/>
     </x:row>
     <x:row r="20" ht="26.75" customHeight="1">
       <x:c r="A20" s="16" t="s">
-        <x:v>562</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="B20" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C20" s="17"/>
     </x:row>
     <x:row r="21" ht="26.75" customHeight="1">
       <x:c r="A21" s="16" t="s">
-        <x:v>909</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="B21" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C21" s="17"/>
     </x:row>
@@ -10080,25 +10077,25 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B22" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C22" s="17"/>
     </x:row>
     <x:row r="23" ht="26.75" customHeight="1">
       <x:c r="A23" s="16" t="s">
+        <x:v>909</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="s">
         <x:v>910</x:v>
-      </x:c>
-      <x:c r="B23" s="16" t="s">
-        <x:v>911</x:v>
       </x:c>
       <x:c r="C23" s="17"/>
     </x:row>
     <x:row r="24" ht="26.75" customHeight="1">
       <x:c r="A24" s="16" t="s">
-        <x:v>912</x:v>
+        <x:v>911</x:v>
       </x:c>
       <x:c r="B24" s="16" t="s">
-        <x:v>895</x:v>
+        <x:v>894</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
     </x:row>
@@ -10107,7 +10104,7 @@
         <x:v>325</x:v>
       </x:c>
       <x:c r="B25" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
     </x:row>
@@ -10116,27 +10113,27 @@
         <x:v>465</x:v>
       </x:c>
       <x:c r="B26" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
     </x:row>
     <x:row r="27" ht="26.75" customHeight="1">
       <x:c r="A27" s="16" t="s">
-        <x:v>555</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="B27" s="16" t="s">
-        <x:v>899</x:v>
+        <x:v>898</x:v>
       </x:c>
       <x:c r="C27" s="17" t="s">
-        <x:v>913</x:v>
+        <x:v>912</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="26.75" customHeight="1">
       <x:c r="A28" s="16" t="s">
-        <x:v>914</x:v>
+        <x:v>913</x:v>
       </x:c>
       <x:c r="B28" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="C28" s="17"/>
     </x:row>
@@ -10145,7 +10142,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B29" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="C29" s="17"/>
     </x:row>
@@ -10154,7 +10151,7 @@
         <x:v>191</x:v>
       </x:c>
       <x:c r="B30" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="C30" s="17"/>
     </x:row>
@@ -10163,25 +10160,25 @@
         <x:v>141</x:v>
       </x:c>
       <x:c r="B31" s="16" t="s">
-        <x:v>908</x:v>
+        <x:v>907</x:v>
       </x:c>
       <x:c r="C31" s="17"/>
     </x:row>
     <x:row r="32" ht="26.75" customHeight="1">
       <x:c r="A32" s="16" t="s">
-        <x:v>550</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="B32" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C32" s="17"/>
     </x:row>
     <x:row r="33" ht="26.75" customHeight="1">
       <x:c r="A33" s="16" t="s">
-        <x:v>915</x:v>
+        <x:v>914</x:v>
       </x:c>
       <x:c r="B33" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C33" s="17"/>
     </x:row>
@@ -10190,7 +10187,7 @@
         <x:v>318</x:v>
       </x:c>
       <x:c r="B34" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C34" s="17"/>
     </x:row>
@@ -10199,7 +10196,7 @@
         <x:v>505</x:v>
       </x:c>
       <x:c r="B35" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C35" s="17"/>
     </x:row>
@@ -10208,18 +10205,18 @@
         <x:v>268</x:v>
       </x:c>
       <x:c r="B36" s="16" t="s">
+        <x:v>898</x:v>
+      </x:c>
+      <x:c r="C36" s="17" t="s">
         <x:v>899</x:v>
-      </x:c>
-      <x:c r="C36" s="17" t="s">
-        <x:v>900</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="26.75" customHeight="1">
       <x:c r="A37" s="16" t="s">
-        <x:v>916</x:v>
+        <x:v>915</x:v>
       </x:c>
       <x:c r="B37" s="16" t="s">
-        <x:v>908</x:v>
+        <x:v>907</x:v>
       </x:c>
       <x:c r="C37" s="17"/>
     </x:row>
@@ -10228,7 +10225,7 @@
         <x:v>177</x:v>
       </x:c>
       <x:c r="B38" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="C38" s="17"/>
     </x:row>
@@ -10237,10 +10234,10 @@
         <x:v>239</x:v>
       </x:c>
       <x:c r="B39" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C39" s="17" t="s">
-        <x:v>917</x:v>
+        <x:v>916</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="26.75" customHeight="1">
@@ -10248,25 +10245,25 @@
         <x:v>445</x:v>
       </x:c>
       <x:c r="B40" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C40" s="17"/>
     </x:row>
     <x:row r="41" ht="26.75" customHeight="1">
       <x:c r="A41" s="16" t="s">
-        <x:v>918</x:v>
+        <x:v>917</x:v>
       </x:c>
       <x:c r="B41" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C41" s="17"/>
     </x:row>
     <x:row r="42" ht="26.75" customHeight="1">
       <x:c r="A42" s="16" t="s">
-        <x:v>919</x:v>
+        <x:v>918</x:v>
       </x:c>
       <x:c r="B42" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C42" s="17"/>
     </x:row>
@@ -10275,10 +10272,10 @@
         <x:v>224</x:v>
       </x:c>
       <x:c r="B43" s="16" t="s">
+        <x:v>898</x:v>
+      </x:c>
+      <x:c r="C43" s="17" t="s">
         <x:v>899</x:v>
-      </x:c>
-      <x:c r="C43" s="17" t="s">
-        <x:v>900</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="26.75" customHeight="1">
@@ -10286,7 +10283,7 @@
         <x:v>182</x:v>
       </x:c>
       <x:c r="B44" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="C44" s="17"/>
     </x:row>
@@ -10295,16 +10292,16 @@
         <x:v>162</x:v>
       </x:c>
       <x:c r="B45" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="C45" s="17"/>
     </x:row>
     <x:row r="46" ht="26.75" customHeight="1">
       <x:c r="A46" s="16" t="s">
-        <x:v>920</x:v>
+        <x:v>919</x:v>
       </x:c>
       <x:c r="B46" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="C46" s="17"/>
     </x:row>
@@ -10313,19 +10310,19 @@
         <x:v>156</x:v>
       </x:c>
       <x:c r="B47" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C47" s="17"/>
     </x:row>
     <x:row r="48" ht="26.75" customHeight="1">
       <x:c r="A48" s="16" t="s">
+        <x:v>920</x:v>
+      </x:c>
+      <x:c r="B48" s="16" t="s">
+        <x:v>898</x:v>
+      </x:c>
+      <x:c r="C48" s="17" t="s">
         <x:v>921</x:v>
-      </x:c>
-      <x:c r="B48" s="16" t="s">
-        <x:v>899</x:v>
-      </x:c>
-      <x:c r="C48" s="17" t="s">
-        <x:v>922</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="26.75" customHeight="1">
@@ -10333,7 +10330,7 @@
         <x:v>286</x:v>
       </x:c>
       <x:c r="B49" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C49" s="17"/>
     </x:row>
@@ -10342,16 +10339,16 @@
         <x:v>212</x:v>
       </x:c>
       <x:c r="B50" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="C50" s="17"/>
     </x:row>
     <x:row r="51" ht="26.75" customHeight="1">
       <x:c r="A51" s="16" t="s">
-        <x:v>923</x:v>
+        <x:v>922</x:v>
       </x:c>
       <x:c r="B51" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="C51" s="17"/>
     </x:row>
@@ -10360,38 +10357,38 @@
         <x:v>232</x:v>
       </x:c>
       <x:c r="B52" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="C52" s="17"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" t="s">
-        <x:v>572</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="B53" t="s">
         <x:v>379</x:v>
       </x:c>
       <x:c r="C53" t="s">
-        <x:v>924</x:v>
+        <x:v>923</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" t="s">
-        <x:v>581</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="B54" t="s">
-        <x:v>899</x:v>
+        <x:v>898</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" t="s">
-        <x:v>588</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="B55" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C55" t="s">
-        <x:v>925</x:v>
+        <x:v>924</x:v>
       </x:c>
     </x:row>
     <x:row r="56">

</xml_diff>

<commit_message>
Clarify Agora API credit award
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R0c56dd53672e4b09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rf09d13ae9b374812"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R9f337570e15a4110"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R3a60d2e62ca749a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Re85e6d5eea674bdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rc33f3faf2b4f46a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rd65b798ac75e4ea0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R58e526986d784a6c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1289,9 +1289,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Agora.io</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">3rd Prize: S$ 300 Cash, and S$ 385 worth of Credits</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Agentic AI (Voice), Healthcare</x:t>
@@ -6161,20 +6158,20 @@
       <x:c r="F58" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="G58" t="s">
+      <x:c r="G58" t="str">
+        <x:v>3rd Prize: S$300 Cash and S$385 worth of API Credits</x:v>
+      </x:c>
+      <x:c r="H58" t="s">
         <x:v>426</x:v>
       </x:c>
-      <x:c r="H58" t="s">
+      <x:c r="I58" t="s">
         <x:v>427</x:v>
-      </x:c>
-      <x:c r="I58" t="s">
-        <x:v>428</x:v>
       </x:c>
       <x:c r="J58" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K58" t="s">
-        <x:v>429</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="L58" t="s">
         <x:v>25</x:v>
@@ -6183,13 +6180,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N58" t="s">
+        <x:v>429</x:v>
+      </x:c>
+      <x:c r="O58" t="s">
         <x:v>430</x:v>
       </x:c>
-      <x:c r="O58" t="s">
+      <x:c r="P58" t="s">
         <x:v>431</x:v>
-      </x:c>
-      <x:c r="P58" t="s">
-        <x:v>432</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -6197,13 +6194,13 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="B59" t="s">
+        <x:v>432</x:v>
+      </x:c>
+      <x:c r="C59" t="s">
         <x:v>433</x:v>
       </x:c>
-      <x:c r="C59" t="s">
+      <x:c r="D59" s="2" t="s">
         <x:v>434</x:v>
-      </x:c>
-      <x:c r="D59" s="2" t="s">
-        <x:v>435</x:v>
       </x:c>
       <x:c r="E59">
         <x:v>1</x:v>
@@ -6218,16 +6215,16 @@
         <x:v>141</x:v>
       </x:c>
       <x:c r="I59" t="s">
+        <x:v>435</x:v>
+      </x:c>
+      <x:c r="J59" t="s">
         <x:v>436</x:v>
       </x:c>
-      <x:c r="J59" t="s">
+      <x:c r="K59" t="s">
         <x:v>437</x:v>
       </x:c>
-      <x:c r="K59" t="s">
+      <x:c r="L59" t="s">
         <x:v>438</x:v>
-      </x:c>
-      <x:c r="L59" t="s">
-        <x:v>439</x:v>
       </x:c>
       <x:c r="M59" t="s">
         <x:v>26</x:v>
@@ -6236,10 +6233,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="O59" t="s">
+        <x:v>439</x:v>
+      </x:c>
+      <x:c r="P59" t="s">
         <x:v>440</x:v>
-      </x:c>
-      <x:c r="P59" t="s">
-        <x:v>441</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -6247,13 +6244,13 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B60" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="C60" t="s">
         <x:v>442</x:v>
       </x:c>
-      <x:c r="C60" t="s">
+      <x:c r="D60" s="2" t="s">
         <x:v>443</x:v>
-      </x:c>
-      <x:c r="D60" s="2" t="s">
-        <x:v>444</x:v>
       </x:c>
       <x:c r="E60">
         <x:v>1</x:v>
@@ -6265,16 +6262,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H60" t="s">
+        <x:v>444</x:v>
+      </x:c>
+      <x:c r="I60" t="s">
         <x:v>445</x:v>
       </x:c>
-      <x:c r="I60" t="s">
+      <x:c r="J60" t="s">
         <x:v>446</x:v>
       </x:c>
-      <x:c r="J60" t="s">
+      <x:c r="K60" t="s">
         <x:v>447</x:v>
-      </x:c>
-      <x:c r="K60" t="s">
-        <x:v>448</x:v>
       </x:c>
       <x:c r="L60" t="s">
         <x:v>25</x:v>
@@ -6283,13 +6280,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N60" t="s">
+        <x:v>448</x:v>
+      </x:c>
+      <x:c r="O60" t="s">
         <x:v>449</x:v>
       </x:c>
-      <x:c r="O60" t="s">
+      <x:c r="P60" t="s">
         <x:v>450</x:v>
-      </x:c>
-      <x:c r="P60" t="s">
-        <x:v>451</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -6297,13 +6294,13 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="B61" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C61" t="s">
         <x:v>452</x:v>
       </x:c>
-      <x:c r="C61" t="s">
+      <x:c r="D61" s="2" t="s">
         <x:v>453</x:v>
-      </x:c>
-      <x:c r="D61" s="2" t="s">
-        <x:v>454</x:v>
       </x:c>
       <x:c r="E61">
         <x:v>1</x:v>
@@ -6315,16 +6312,16 @@
         <x:v>2K USD Speechmatics Credits</x:v>
       </x:c>
       <x:c r="H61" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="I61" t="s">
         <x:v>455</x:v>
-      </x:c>
-      <x:c r="I61" t="s">
-        <x:v>456</x:v>
       </x:c>
       <x:c r="J61" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K61" t="s">
-        <x:v>457</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="L61" t="s">
         <x:v>25</x:v>
@@ -6333,13 +6330,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N61" t="s">
+        <x:v>457</x:v>
+      </x:c>
+      <x:c r="O61" t="s">
         <x:v>458</x:v>
       </x:c>
-      <x:c r="O61" t="s">
+      <x:c r="P61" s="1" t="s">
         <x:v>459</x:v>
-      </x:c>
-      <x:c r="P61" s="1" t="s">
-        <x:v>460</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -6347,13 +6344,13 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="B62" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="C62" t="s">
         <x:v>461</x:v>
       </x:c>
-      <x:c r="C62" t="s">
+      <x:c r="D62" s="2" t="s">
         <x:v>462</x:v>
-      </x:c>
-      <x:c r="D62" s="2" t="s">
-        <x:v>463</x:v>
       </x:c>
       <x:c r="E62">
         <x:v>1</x:v>
@@ -6362,19 +6359,19 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="G62" t="s">
+        <x:v>463</x:v>
+      </x:c>
+      <x:c r="H62" t="s">
         <x:v>464</x:v>
       </x:c>
-      <x:c r="H62" t="s">
+      <x:c r="I62" t="s">
         <x:v>465</x:v>
-      </x:c>
-      <x:c r="I62" t="s">
-        <x:v>466</x:v>
       </x:c>
       <x:c r="J62" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K62" t="s">
-        <x:v>467</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="L62" t="s">
         <x:v>25</x:v>
@@ -6389,7 +6386,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="P62" s="1" t="s">
-        <x:v>468</x:v>
+        <x:v>467</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -6397,10 +6394,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="B63" t="s">
+        <x:v>468</x:v>
+      </x:c>
+      <x:c r="C63" t="s">
         <x:v>469</x:v>
-      </x:c>
-      <x:c r="C63" t="s">
-        <x:v>470</x:v>
       </x:c>
       <x:c r="D63" s="5">
         <x:v>46085</x:v>
@@ -6409,7 +6406,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F63" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="G63" t="s">
         <x:v>25</x:v>
@@ -6418,13 +6415,13 @@
         <x:v>405</x:v>
       </x:c>
       <x:c r="I63" t="s">
-        <x:v>472</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="J63" t="s">
         <x:v>407</x:v>
       </x:c>
       <x:c r="K63" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="L63" t="s">
         <x:v>25</x:v>
@@ -6433,13 +6430,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N63" t="s">
+        <x:v>473</x:v>
+      </x:c>
+      <x:c r="O63" t="s">
         <x:v>474</x:v>
       </x:c>
-      <x:c r="O63" t="s">
+      <x:c r="P63" t="s">
         <x:v>475</x:v>
-      </x:c>
-      <x:c r="P63" t="s">
-        <x:v>476</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -6447,10 +6444,10 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="B64" t="s">
-        <x:v>477</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="C64" t="s">
-        <x:v>462</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="D64" s="5">
         <x:v>46116</x:v>
@@ -6465,16 +6462,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H64" t="s">
-        <x:v>465</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="I64" t="s">
-        <x:v>478</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="J64" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K64" t="s">
-        <x:v>479</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="L64" t="s">
         <x:v>25</x:v>
@@ -6486,10 +6483,10 @@
         <x:v>359</x:v>
       </x:c>
       <x:c r="O64" t="s">
+        <x:v>479</x:v>
+      </x:c>
+      <x:c r="P64" t="s">
         <x:v>480</x:v>
-      </x:c>
-      <x:c r="P64" t="s">
-        <x:v>481</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -6497,10 +6494,10 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="B65" t="s">
+        <x:v>481</x:v>
+      </x:c>
+      <x:c r="C65" t="s">
         <x:v>482</x:v>
-      </x:c>
-      <x:c r="C65" t="s">
-        <x:v>483</x:v>
       </x:c>
       <x:c r="D65" s="5">
         <x:v>46270</x:v>
@@ -6515,16 +6512,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H65" t="s">
-        <x:v>465</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="I65" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="J65" t="s">
         <x:v>484</x:v>
       </x:c>
-      <x:c r="J65" t="s">
+      <x:c r="K65" t="s">
         <x:v>485</x:v>
-      </x:c>
-      <x:c r="K65" t="s">
-        <x:v>486</x:v>
       </x:c>
       <x:c r="L65" t="s">
         <x:v>25</x:v>
@@ -6536,10 +6533,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="O65" t="s">
+        <x:v>486</x:v>
+      </x:c>
+      <x:c r="P65" t="s">
         <x:v>487</x:v>
-      </x:c>
-      <x:c r="P65" t="s">
-        <x:v>488</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -6547,13 +6544,13 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B66" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="C66" t="s">
         <x:v>489</x:v>
       </x:c>
-      <x:c r="C66" t="s">
+      <x:c r="D66" s="2" t="s">
         <x:v>490</x:v>
-      </x:c>
-      <x:c r="D66" s="2" t="s">
-        <x:v>491</x:v>
       </x:c>
       <x:c r="E66">
         <x:v>1</x:v>
@@ -6568,13 +6565,13 @@
         <x:v>379</x:v>
       </x:c>
       <x:c r="I66" t="s">
-        <x:v>492</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="J66" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K66" t="s">
-        <x:v>493</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="L66" t="s">
         <x:v>25</x:v>
@@ -6583,13 +6580,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N66" t="s">
+        <x:v>493</x:v>
+      </x:c>
+      <x:c r="O66" t="s">
         <x:v>494</x:v>
       </x:c>
-      <x:c r="O66" t="s">
+      <x:c r="P66" t="s">
         <x:v>495</x:v>
-      </x:c>
-      <x:c r="P66" t="s">
-        <x:v>496</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -6597,13 +6594,13 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B67" t="s">
+        <x:v>496</x:v>
+      </x:c>
+      <x:c r="C67" t="s">
         <x:v>497</x:v>
       </x:c>
-      <x:c r="C67" t="s">
+      <x:c r="D67" s="2" t="s">
         <x:v>498</x:v>
-      </x:c>
-      <x:c r="D67" s="2" t="s">
-        <x:v>499</x:v>
       </x:c>
       <x:c r="E67">
         <x:v>1</x:v>
@@ -6612,7 +6609,7 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="G67" t="s">
-        <x:v>500</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="H67" t="s">
         <x:v>405</x:v>
@@ -6621,10 +6618,10 @@
         <x:v>414</x:v>
       </x:c>
       <x:c r="J67" t="s">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="K67" t="s">
         <x:v>501</x:v>
-      </x:c>
-      <x:c r="K67" t="s">
-        <x:v>502</x:v>
       </x:c>
       <x:c r="L67" t="s">
         <x:v>25</x:v>
@@ -6647,13 +6644,13 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B68" t="s">
-        <x:v>503</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="C68" t="s">
         <x:v>266</x:v>
       </x:c>
       <x:c r="D68" s="2" t="s">
-        <x:v>504</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="E68">
         <x:v>3</x:v>
@@ -6665,19 +6662,19 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H68" t="s">
+        <x:v>504</x:v>
+      </x:c>
+      <x:c r="I68" t="s">
         <x:v>505</x:v>
       </x:c>
-      <x:c r="I68" t="s">
+      <x:c r="J68" t="s">
         <x:v>506</x:v>
       </x:c>
-      <x:c r="J68" t="s">
+      <x:c r="K68" t="s">
         <x:v>507</x:v>
       </x:c>
-      <x:c r="K68" t="s">
+      <x:c r="L68" t="s">
         <x:v>508</x:v>
-      </x:c>
-      <x:c r="L68" t="s">
-        <x:v>509</x:v>
       </x:c>
       <x:c r="M68" t="s">
         <x:v>26</x:v>
@@ -6686,7 +6683,7 @@
         <x:v>273</x:v>
       </x:c>
       <x:c r="O68" t="s">
-        <x:v>510</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="P68" t="s">
         <x:v>25</x:v>
@@ -6697,13 +6694,13 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B69" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="C69" t="s">
+        <x:v>497</x:v>
+      </x:c>
+      <x:c r="D69" s="2" t="s">
         <x:v>511</x:v>
-      </x:c>
-      <x:c r="C69" t="s">
-        <x:v>498</x:v>
-      </x:c>
-      <x:c r="D69" s="2" t="s">
-        <x:v>512</x:v>
       </x:c>
       <x:c r="E69">
         <x:v>1</x:v>
@@ -6721,10 +6718,10 @@
         <x:v>414</x:v>
       </x:c>
       <x:c r="J69" t="s">
-        <x:v>501</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="K69" t="s">
-        <x:v>513</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="L69" t="s">
         <x:v>25</x:v>
@@ -6733,13 +6730,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N69" t="s">
+        <x:v>513</x:v>
+      </x:c>
+      <x:c r="O69" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="P69" t="s">
         <x:v>514</x:v>
-      </x:c>
-      <x:c r="O69" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="P69" t="s">
-        <x:v>515</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -6747,13 +6744,13 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="B70" t="s">
+        <x:v>515</x:v>
+      </x:c>
+      <x:c r="C70" t="s">
         <x:v>516</x:v>
       </x:c>
-      <x:c r="C70" t="s">
+      <x:c r="D70" s="2" t="s">
         <x:v>517</x:v>
-      </x:c>
-      <x:c r="D70" s="2" t="s">
-        <x:v>518</x:v>
       </x:c>
       <x:c r="E70">
         <x:v>2</x:v>
@@ -6762,31 +6759,31 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="H70" t="s">
+        <x:v>518</x:v>
+      </x:c>
+      <x:c r="I70" t="s">
         <x:v>519</x:v>
       </x:c>
-      <x:c r="I70" t="s">
+      <x:c r="J70" t="s">
         <x:v>520</x:v>
       </x:c>
-      <x:c r="J70" t="s">
+      <x:c r="K70" t="s">
         <x:v>521</x:v>
       </x:c>
-      <x:c r="K70" t="s">
+      <x:c r="L70" t="s">
+        <x:v>516</x:v>
+      </x:c>
+      <x:c r="M70" t="s">
         <x:v>522</x:v>
-      </x:c>
-      <x:c r="L70" t="s">
-        <x:v>517</x:v>
-      </x:c>
-      <x:c r="M70" t="s">
-        <x:v>523</x:v>
       </x:c>
       <x:c r="N70" t="s">
         <x:v>359</x:v>
       </x:c>
       <x:c r="O70" t="s">
+        <x:v>523</x:v>
+      </x:c>
+      <x:c r="P70" t="s">
         <x:v>524</x:v>
-      </x:c>
-      <x:c r="P70" t="s">
-        <x:v>525</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -6794,13 +6791,13 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="B71" t="s">
+        <x:v>525</x:v>
+      </x:c>
+      <x:c r="C71" t="s">
         <x:v>526</x:v>
       </x:c>
-      <x:c r="C71" t="s">
+      <x:c r="D71" s="5" t="s">
         <x:v>527</x:v>
-      </x:c>
-      <x:c r="D71" s="5" t="s">
-        <x:v>528</x:v>
       </x:c>
       <x:c r="E71">
         <x:v>1</x:v>
@@ -6812,31 +6809,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H71" t="s">
-        <x:v>519</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="I71" t="s">
-        <x:v>529</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="J71" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K71" t="s">
-        <x:v>530</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="L71" t="s">
-        <x:v>527</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="M71" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N71" t="s">
-        <x:v>494</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="O71" t="s">
+        <x:v>530</x:v>
+      </x:c>
+      <x:c r="P71" t="s">
         <x:v>531</x:v>
-      </x:c>
-      <x:c r="P71" t="s">
-        <x:v>532</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -6844,10 +6841,10 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B72" t="s">
+        <x:v>532</x:v>
+      </x:c>
+      <x:c r="C72" t="s">
         <x:v>533</x:v>
-      </x:c>
-      <x:c r="C72" t="s">
-        <x:v>534</x:v>
       </x:c>
       <x:c r="D72" s="5">
         <x:v>46363</x:v>
@@ -6865,16 +6862,16 @@
         <x:v>239</x:v>
       </x:c>
       <x:c r="I72" t="s">
+        <x:v>534</x:v>
+      </x:c>
+      <x:c r="J72" t="s">
         <x:v>535</x:v>
       </x:c>
-      <x:c r="J72" t="s">
+      <x:c r="K72" t="s">
         <x:v>536</x:v>
       </x:c>
-      <x:c r="K72" t="s">
-        <x:v>537</x:v>
-      </x:c>
       <x:c r="L72" t="s">
-        <x:v>534</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="M72" t="s">
         <x:v>26</x:v>
@@ -6886,7 +6883,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="P72" t="s">
-        <x:v>538</x:v>
+        <x:v>537</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -6894,13 +6891,13 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B73" t="s">
+        <x:v>538</x:v>
+      </x:c>
+      <x:c r="C73" t="s">
         <x:v>539</x:v>
       </x:c>
-      <x:c r="C73" t="s">
+      <x:c r="D73" s="2" t="s">
         <x:v>540</x:v>
-      </x:c>
-      <x:c r="D73" s="2" t="s">
-        <x:v>541</x:v>
       </x:c>
       <x:c r="E73">
         <x:v>1</x:v>
@@ -6912,31 +6909,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H73" t="s">
-        <x:v>465</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="I73" t="s">
-        <x:v>542</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="J73" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K73" t="s">
-        <x:v>543</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="L73" t="s">
-        <x:v>540</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="M73" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N73" t="s">
+        <x:v>543</x:v>
+      </x:c>
+      <x:c r="O73" t="s">
         <x:v>544</x:v>
       </x:c>
-      <x:c r="O73" t="s">
+      <x:c r="P73" t="s">
         <x:v>545</x:v>
-      </x:c>
-      <x:c r="P73" t="s">
-        <x:v>546</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -6944,13 +6941,13 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B74" t="s">
+        <x:v>546</x:v>
+      </x:c>
+      <x:c r="C74" t="s">
+        <x:v>516</x:v>
+      </x:c>
+      <x:c r="D74" s="2" t="s">
         <x:v>547</x:v>
-      </x:c>
-      <x:c r="C74" t="s">
-        <x:v>517</x:v>
-      </x:c>
-      <x:c r="D74" s="2" t="s">
-        <x:v>548</x:v>
       </x:c>
       <x:c r="E74">
         <x:v>10</x:v>
@@ -6962,31 +6959,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H74" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="I74" t="s">
         <x:v>549</x:v>
-      </x:c>
-      <x:c r="I74" t="s">
-        <x:v>550</x:v>
       </x:c>
       <x:c r="J74" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K74" t="s">
-        <x:v>551</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="L74" t="s">
-        <x:v>517</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="M74" t="s">
-        <x:v>523</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="N74" t="s">
         <x:v>359</x:v>
       </x:c>
       <x:c r="O74" t="s">
-        <x:v>552</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="P74" t="s">
-        <x:v>525</x:v>
+        <x:v>524</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="34">
@@ -6994,10 +6991,10 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B75" s="12" t="s">
+        <x:v>552</x:v>
+      </x:c>
+      <x:c r="C75" s="12" t="s">
         <x:v>553</x:v>
-      </x:c>
-      <x:c r="C75" s="12" t="s">
-        <x:v>554</x:v>
       </x:c>
       <x:c r="D75" s="5">
         <x:v>46150</x:v>
@@ -7012,19 +7009,19 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H75" s="12" t="s">
+        <x:v>553</x:v>
+      </x:c>
+      <x:c r="I75" s="14" t="s">
         <x:v>554</x:v>
-      </x:c>
-      <x:c r="I75" s="14" t="s">
-        <x:v>555</x:v>
       </x:c>
       <x:c r="J75" s="12" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K75" s="12" t="s">
-        <x:v>556</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="L75" s="12" t="s">
-        <x:v>554</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="M75" s="12" t="s">
         <x:v>26</x:v>
@@ -7033,7 +7030,7 @@
         <x:v>273</x:v>
       </x:c>
       <x:c r="O75" t="s">
-        <x:v>557</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="P75" s="12" t="s">
         <x:v>25</x:v>
@@ -7044,13 +7041,13 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B76" s="12" t="s">
+        <x:v>557</x:v>
+      </x:c>
+      <x:c r="C76" s="12" t="s">
         <x:v>558</x:v>
       </x:c>
-      <x:c r="C76" s="12" t="s">
+      <x:c r="D76" s="13" t="s">
         <x:v>559</x:v>
-      </x:c>
-      <x:c r="D76" s="13" t="s">
-        <x:v>560</x:v>
       </x:c>
       <x:c r="E76">
         <x:v>1</x:v>
@@ -7062,31 +7059,31 @@
         <x:v>Best Vertical Solution (Family Office Track), 2,000 Cybrdeck API credits (worth US$25)</x:v>
       </x:c>
       <x:c r="H76" s="12" t="s">
+        <x:v>560</x:v>
+      </x:c>
+      <x:c r="I76" s="12" t="s">
         <x:v>561</x:v>
       </x:c>
-      <x:c r="I76" s="12" t="s">
+      <x:c r="J76" s="12" t="s">
         <x:v>562</x:v>
       </x:c>
-      <x:c r="J76" s="12" t="s">
+      <x:c r="K76" s="12" t="s">
         <x:v>563</x:v>
       </x:c>
-      <x:c r="K76" s="12" t="s">
-        <x:v>564</x:v>
-      </x:c>
       <x:c r="L76" s="12" t="s">
-        <x:v>559</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="M76" s="12" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N76" s="12" t="s">
+        <x:v>564</x:v>
+      </x:c>
+      <x:c r="O76" s="1" t="s">
         <x:v>565</x:v>
       </x:c>
-      <x:c r="O76" s="1" t="s">
+      <x:c r="P76" t="s">
         <x:v>566</x:v>
-      </x:c>
-      <x:c r="P76" t="s">
-        <x:v>567</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -7094,13 +7091,13 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B77" t="s">
+        <x:v>567</x:v>
+      </x:c>
+      <x:c r="C77" t="s">
         <x:v>568</x:v>
       </x:c>
-      <x:c r="C77" t="s">
+      <x:c r="D77" t="s">
         <x:v>569</x:v>
-      </x:c>
-      <x:c r="D77" t="s">
-        <x:v>570</x:v>
       </x:c>
       <x:c r="E77">
         <x:v>1</x:v>
@@ -7112,31 +7109,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H77" t="s">
+        <x:v>570</x:v>
+      </x:c>
+      <x:c r="I77" t="s">
         <x:v>571</x:v>
-      </x:c>
-      <x:c r="I77" t="s">
-        <x:v>572</x:v>
       </x:c>
       <x:c r="J77" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K77" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="L77" t="s">
         <x:v>573</x:v>
-      </x:c>
-      <x:c r="L77" t="s">
-        <x:v>574</x:v>
       </x:c>
       <x:c r="M77" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N77" t="s">
+        <x:v>574</x:v>
+      </x:c>
+      <x:c r="O77" t="s">
         <x:v>575</x:v>
       </x:c>
-      <x:c r="O77" t="s">
+      <x:c r="P77" t="s">
         <x:v>576</x:v>
-      </x:c>
-      <x:c r="P77" t="s">
-        <x:v>577</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -7144,13 +7141,13 @@
         <x:v>77</x:v>
       </x:c>
       <x:c r="B78" t="s">
+        <x:v>577</x:v>
+      </x:c>
+      <x:c r="C78" t="s">
+        <x:v>516</x:v>
+      </x:c>
+      <x:c r="D78" t="s">
         <x:v>578</x:v>
-      </x:c>
-      <x:c r="C78" t="s">
-        <x:v>517</x:v>
-      </x:c>
-      <x:c r="D78" t="s">
-        <x:v>579</x:v>
       </x:c>
       <x:c r="E78">
         <x:v>1</x:v>
@@ -7162,31 +7159,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H78" t="s">
+        <x:v>579</x:v>
+      </x:c>
+      <x:c r="I78" t="s">
         <x:v>580</x:v>
-      </x:c>
-      <x:c r="I78" t="s">
-        <x:v>581</x:v>
       </x:c>
       <x:c r="J78" t="s">
         <x:v>312</x:v>
       </x:c>
       <x:c r="K78" t="s">
-        <x:v>582</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="L78" t="s">
-        <x:v>517</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="M78" t="s">
-        <x:v>523</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="N78" t="s">
         <x:v>359</x:v>
       </x:c>
       <x:c r="O78" t="s">
-        <x:v>583</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="P78" t="s">
-        <x:v>525</x:v>
+        <x:v>524</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -7194,37 +7191,37 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="B79" t="s">
+        <x:v>583</x:v>
+      </x:c>
+      <x:c r="C79" t="s">
         <x:v>584</x:v>
       </x:c>
-      <x:c r="C79" t="s">
+      <x:c r="D79" t="s">
         <x:v>585</x:v>
-      </x:c>
-      <x:c r="D79" t="s">
-        <x:v>586</x:v>
       </x:c>
       <x:c r="E79">
         <x:v>4</x:v>
       </x:c>
       <x:c r="F79" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="G79" t="s">
         <x:v>25</x:v>
       </x:c>
       <x:c r="H79" t="s">
+        <x:v>586</x:v>
+      </x:c>
+      <x:c r="I79" t="s">
         <x:v>587</x:v>
       </x:c>
-      <x:c r="I79" t="s">
+      <x:c r="J79" t="s">
         <x:v>588</x:v>
       </x:c>
-      <x:c r="J79" t="s">
+      <x:c r="K79" t="s">
         <x:v>589</x:v>
       </x:c>
-      <x:c r="K79" t="s">
+      <x:c r="L79" t="s">
         <x:v>590</x:v>
-      </x:c>
-      <x:c r="L79" t="s">
-        <x:v>591</x:v>
       </x:c>
       <x:c r="M79" t="s">
         <x:v>26</x:v>
@@ -7233,10 +7230,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="O79" t="s">
+        <x:v>591</x:v>
+      </x:c>
+      <x:c r="P79" t="s">
         <x:v>592</x:v>
-      </x:c>
-      <x:c r="P79" t="s">
-        <x:v>593</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -7389,10 +7386,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rd3c0acdaa85c4abe"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R8c3340ff6dff4df1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rf9320db7364943e0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Ree5ca64eaaba4361"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rcf02be9cb02e4fb8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R72131753d7d1444d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Ra6cf2c842bf747cc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R25389dc8659d4e98"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7415,7 +7412,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>594</x:v>
+        <x:v>593</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -7424,7 +7421,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="19" t="s">
-        <x:v>595</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="B2" s="19"/>
       <x:c r="C2" s="19"/>
@@ -7433,64 +7430,64 @@
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="11" t="s">
+        <x:v>595</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="s">
         <x:v>596</x:v>
       </x:c>
-      <x:c r="B4" s="11" t="s">
+      <x:c r="C4" s="11" t="s">
         <x:v>597</x:v>
       </x:c>
-      <x:c r="C4" s="11" t="s">
+      <x:c r="D4" s="11" t="s">
         <x:v>598</x:v>
       </x:c>
-      <x:c r="D4" s="11" t="s">
+      <x:c r="E4" s="11" t="s">
         <x:v>599</x:v>
-      </x:c>
-      <x:c r="E4" s="11" t="s">
-        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="8" t="s">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="s">
         <x:v>601</x:v>
       </x:c>
-      <x:c r="B5" s="7" t="s">
+      <x:c r="C5" s="7" t="s">
         <x:v>602</x:v>
-      </x:c>
-      <x:c r="C5" s="7" t="s">
-        <x:v>603</x:v>
       </x:c>
       <x:c r="D5" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E5" s="10" t="s">
-        <x:v>604</x:v>
+        <x:v>603</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="8" t="s">
+        <x:v>604</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>605</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="s">
+      <x:c r="C6" s="7" t="s">
         <x:v>606</x:v>
       </x:c>
-      <x:c r="C6" s="7" t="s">
+      <x:c r="D6" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="s">
         <x:v>607</x:v>
-      </x:c>
-      <x:c r="D6" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E6" s="10" t="s">
-        <x:v>608</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="8" t="s">
+        <x:v>608</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
         <x:v>609</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="s">
+      <x:c r="C7" s="7" t="s">
         <x:v>610</x:v>
-      </x:c>
-      <x:c r="C7" s="7" t="s">
-        <x:v>611</x:v>
       </x:c>
       <x:c r="D7" s="9">
         <x:v>1</x:v>
@@ -7499,47 +7496,47 @@
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
       <x:c r="A8" s="8" t="s">
+        <x:v>611</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
         <x:v>612</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="s">
+      <x:c r="C8" s="7" t="s">
         <x:v>613</x:v>
       </x:c>
-      <x:c r="C8" s="7" t="s">
+      <x:c r="D8" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="s">
         <x:v>614</x:v>
-      </x:c>
-      <x:c r="D8" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E8" s="10" t="s">
-        <x:v>615</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" s="8" t="s">
+        <x:v>615</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
         <x:v>616</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="s">
+      <x:c r="C9" s="7" t="s">
+        <x:v>606</x:v>
+      </x:c>
+      <x:c r="D9" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="s">
         <x:v>617</x:v>
-      </x:c>
-      <x:c r="C9" s="7" t="s">
-        <x:v>607</x:v>
-      </x:c>
-      <x:c r="D9" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E9" s="10" t="s">
-        <x:v>618</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
       <x:c r="A10" s="8" t="s">
+        <x:v>618</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="s">
         <x:v>619</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="s">
+      <x:c r="C10" s="7" t="s">
         <x:v>620</x:v>
-      </x:c>
-      <x:c r="C10" s="7" t="s">
-        <x:v>621</x:v>
       </x:c>
       <x:c r="D10" s="9">
         <x:v>1</x:v>
@@ -7548,47 +7545,47 @@
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
       <x:c r="A11" s="8" t="s">
+        <x:v>621</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="s">
         <x:v>622</x:v>
       </x:c>
-      <x:c r="B11" s="7" t="s">
+      <x:c r="C11" s="7" t="s">
         <x:v>623</x:v>
       </x:c>
-      <x:c r="C11" s="7" t="s">
+      <x:c r="D11" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="10" t="s">
         <x:v>624</x:v>
-      </x:c>
-      <x:c r="D11" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E11" s="10" t="s">
-        <x:v>625</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
       <x:c r="A12" s="8" t="s">
+        <x:v>625</x:v>
+      </x:c>
+      <x:c r="B12" s="7" t="s">
         <x:v>626</x:v>
       </x:c>
-      <x:c r="B12" s="7" t="s">
+      <x:c r="C12" s="7" t="s">
         <x:v>627</x:v>
       </x:c>
-      <x:c r="C12" s="7" t="s">
+      <x:c r="D12" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="s">
         <x:v>628</x:v>
-      </x:c>
-      <x:c r="D12" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E12" s="10" t="s">
-        <x:v>629</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
       <x:c r="A13" s="8" t="s">
+        <x:v>629</x:v>
+      </x:c>
+      <x:c r="B13" s="7" t="s">
         <x:v>630</x:v>
       </x:c>
-      <x:c r="B13" s="7" t="s">
+      <x:c r="C13" s="7" t="s">
         <x:v>631</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="s">
-        <x:v>632</x:v>
       </x:c>
       <x:c r="D13" s="9">
         <x:v>1</x:v>
@@ -7597,30 +7594,30 @@
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
       <x:c r="A14" s="8" t="s">
+        <x:v>632</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="s">
         <x:v>633</x:v>
       </x:c>
-      <x:c r="B14" s="7" t="s">
+      <x:c r="C14" s="7" t="s">
+        <x:v>631</x:v>
+      </x:c>
+      <x:c r="D14" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="s">
         <x:v>634</x:v>
-      </x:c>
-      <x:c r="C14" s="7" t="s">
-        <x:v>632</x:v>
-      </x:c>
-      <x:c r="D14" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E14" s="10" t="s">
-        <x:v>635</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
       <x:c r="A15" s="8" t="s">
+        <x:v>635</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="s">
         <x:v>636</x:v>
       </x:c>
-      <x:c r="B15" s="7" t="s">
+      <x:c r="C15" s="7" t="s">
         <x:v>637</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="s">
-        <x:v>638</x:v>
       </x:c>
       <x:c r="D15" s="9">
         <x:v>1</x:v>
@@ -7629,30 +7626,30 @@
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
       <x:c r="A16" s="8" t="s">
+        <x:v>638</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="s">
         <x:v>639</x:v>
       </x:c>
-      <x:c r="B16" s="7" t="s">
+      <x:c r="C16" s="7" t="s">
         <x:v>640</x:v>
       </x:c>
-      <x:c r="C16" s="7" t="s">
+      <x:c r="D16" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="s">
         <x:v>641</x:v>
-      </x:c>
-      <x:c r="D16" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E16" s="10" t="s">
-        <x:v>642</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
       <x:c r="A17" s="8" t="s">
+        <x:v>642</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="s">
         <x:v>643</x:v>
       </x:c>
-      <x:c r="B17" s="7" t="s">
+      <x:c r="C17" s="7" t="s">
         <x:v>644</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="s">
-        <x:v>645</x:v>
       </x:c>
       <x:c r="D17" s="9">
         <x:v>1</x:v>
@@ -7661,47 +7658,47 @@
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
       <x:c r="A18" s="8" t="s">
+        <x:v>645</x:v>
+      </x:c>
+      <x:c r="B18" s="7" t="s">
         <x:v>646</x:v>
       </x:c>
-      <x:c r="B18" s="7" t="s">
+      <x:c r="C18" s="7" t="s">
         <x:v>647</x:v>
       </x:c>
-      <x:c r="C18" s="7" t="s">
+      <x:c r="D18" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="s">
         <x:v>648</x:v>
-      </x:c>
-      <x:c r="D18" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E18" s="10" t="s">
-        <x:v>649</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
       <x:c r="A19" s="8" t="s">
+        <x:v>649</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="s">
         <x:v>650</x:v>
       </x:c>
-      <x:c r="B19" s="7" t="s">
+      <x:c r="C19" s="7" t="s">
         <x:v>651</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="s">
-        <x:v>652</x:v>
       </x:c>
       <x:c r="D19" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E19" s="10" t="s">
-        <x:v>653</x:v>
+        <x:v>652</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28" customHeight="1">
       <x:c r="A20" s="8" t="s">
+        <x:v>653</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="s">
         <x:v>654</x:v>
       </x:c>
-      <x:c r="B20" s="7" t="s">
+      <x:c r="C20" s="7" t="s">
         <x:v>655</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>656</x:v>
       </x:c>
       <x:c r="D20" s="9">
         <x:v>1</x:v>
@@ -7710,10 +7707,10 @@
     </x:row>
     <x:row r="21" ht="28" customHeight="1">
       <x:c r="A21" s="8" t="s">
+        <x:v>656</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="s">
         <x:v>657</x:v>
-      </x:c>
-      <x:c r="B21" s="7" t="s">
-        <x:v>658</x:v>
       </x:c>
       <x:c r="C21" s="7" t="str">
         <x:v>#069, #071, #079</x:v>
@@ -7722,18 +7719,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E21" s="10" t="s">
-        <x:v>659</x:v>
+        <x:v>658</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
       <x:c r="A22" s="8" t="s">
+        <x:v>659</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="s">
         <x:v>660</x:v>
       </x:c>
-      <x:c r="B22" s="7" t="s">
+      <x:c r="C22" s="7" t="s">
         <x:v>661</x:v>
-      </x:c>
-      <x:c r="C22" s="7" t="s">
-        <x:v>662</x:v>
       </x:c>
       <x:c r="D22" s="9">
         <x:v>1</x:v>
@@ -7742,13 +7739,13 @@
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
       <x:c r="A23" s="8" t="s">
+        <x:v>662</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="s">
         <x:v>663</x:v>
       </x:c>
-      <x:c r="B23" s="7" t="s">
+      <x:c r="C23" s="7" t="s">
         <x:v>664</x:v>
-      </x:c>
-      <x:c r="C23" s="7" t="s">
-        <x:v>665</x:v>
       </x:c>
       <x:c r="D23" s="9">
         <x:v>1</x:v>
@@ -7757,10 +7754,10 @@
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
       <x:c r="A24" s="8" t="s">
+        <x:v>665</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="s">
         <x:v>666</x:v>
-      </x:c>
-      <x:c r="B24" s="7" t="s">
-        <x:v>667</x:v>
       </x:c>
       <x:c r="C24" s="7" t="str">
         <x:v>#054, #055, #056, #062, #066, #068, #075</x:v>
@@ -7769,12 +7766,12 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E24" s="10" t="s">
-        <x:v>668</x:v>
+        <x:v>667</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
       <x:c r="A25" s="8" t="s">
-        <x:v>669</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
         <x:v>Clement Lork</x:v>
@@ -7786,18 +7783,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E25" s="10" t="s">
-        <x:v>670</x:v>
+        <x:v>669</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="8" t="s">
+        <x:v>670</x:v>
+      </x:c>
+      <x:c r="B26" s="7" t="s">
         <x:v>671</x:v>
       </x:c>
-      <x:c r="B26" s="7" t="s">
-        <x:v>672</x:v>
-      </x:c>
       <x:c r="C26" s="7" t="s">
-        <x:v>611</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="D26" s="9">
         <x:v>1</x:v>
@@ -7806,13 +7803,13 @@
     </x:row>
     <x:row r="27" ht="28" customHeight="1">
       <x:c r="A27" s="8" t="s">
+        <x:v>672</x:v>
+      </x:c>
+      <x:c r="B27" s="7" t="s">
         <x:v>673</x:v>
       </x:c>
-      <x:c r="B27" s="7" t="s">
+      <x:c r="C27" s="7" t="s">
         <x:v>674</x:v>
-      </x:c>
-      <x:c r="C27" s="7" t="s">
-        <x:v>675</x:v>
       </x:c>
       <x:c r="D27" s="9">
         <x:v>1</x:v>
@@ -7821,13 +7818,13 @@
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
       <x:c r="A28" s="8" t="s">
+        <x:v>675</x:v>
+      </x:c>
+      <x:c r="B28" s="7" t="s">
         <x:v>676</x:v>
       </x:c>
-      <x:c r="B28" s="7" t="s">
+      <x:c r="C28" s="7" t="s">
         <x:v>677</x:v>
-      </x:c>
-      <x:c r="C28" s="7" t="s">
-        <x:v>678</x:v>
       </x:c>
       <x:c r="D28" s="9">
         <x:v>2</x:v>
@@ -7836,13 +7833,13 @@
     </x:row>
     <x:row r="29" ht="28" customHeight="1">
       <x:c r="A29" s="8" t="s">
+        <x:v>678</x:v>
+      </x:c>
+      <x:c r="B29" s="7" t="s">
         <x:v>679</x:v>
       </x:c>
-      <x:c r="B29" s="7" t="s">
+      <x:c r="C29" s="7" t="s">
         <x:v>680</x:v>
-      </x:c>
-      <x:c r="C29" s="7" t="s">
-        <x:v>681</x:v>
       </x:c>
       <x:c r="D29" s="9">
         <x:v>4</x:v>
@@ -7851,13 +7848,13 @@
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
       <x:c r="A30" s="8" t="s">
+        <x:v>681</x:v>
+      </x:c>
+      <x:c r="B30" s="7" t="s">
         <x:v>682</x:v>
       </x:c>
-      <x:c r="B30" s="7" t="s">
-        <x:v>683</x:v>
-      </x:c>
       <x:c r="C30" s="7" t="s">
-        <x:v>675</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="D30" s="9">
         <x:v>1</x:v>
@@ -7866,47 +7863,47 @@
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="8" t="s">
+        <x:v>683</x:v>
+      </x:c>
+      <x:c r="B31" s="7" t="s">
         <x:v>684</x:v>
       </x:c>
-      <x:c r="B31" s="7" t="s">
+      <x:c r="C31" s="7" t="s">
+        <x:v>623</x:v>
+      </x:c>
+      <x:c r="D31" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E31" s="10" t="s">
         <x:v>685</x:v>
-      </x:c>
-      <x:c r="C31" s="7" t="s">
-        <x:v>624</x:v>
-      </x:c>
-      <x:c r="D31" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E31" s="10" t="s">
-        <x:v>686</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="28" customHeight="1">
       <x:c r="A32" s="8" t="s">
+        <x:v>686</x:v>
+      </x:c>
+      <x:c r="B32" s="7" t="s">
         <x:v>687</x:v>
       </x:c>
-      <x:c r="B32" s="7" t="s">
+      <x:c r="C32" s="7" t="s">
         <x:v>688</x:v>
       </x:c>
-      <x:c r="C32" s="7" t="s">
+      <x:c r="D32" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E32" s="10" t="s">
         <x:v>689</x:v>
-      </x:c>
-      <x:c r="D32" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E32" s="10" t="s">
-        <x:v>690</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="8" t="s">
+        <x:v>690</x:v>
+      </x:c>
+      <x:c r="B33" s="7" t="s">
         <x:v>691</x:v>
       </x:c>
-      <x:c r="B33" s="7" t="s">
-        <x:v>692</x:v>
-      </x:c>
       <x:c r="C33" s="7" t="s">
-        <x:v>662</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="D33" s="9">
         <x:v>1</x:v>
@@ -7915,13 +7912,13 @@
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
       <x:c r="A34" s="8" t="s">
+        <x:v>692</x:v>
+      </x:c>
+      <x:c r="B34" s="7" t="s">
         <x:v>693</x:v>
       </x:c>
-      <x:c r="B34" s="7" t="s">
+      <x:c r="C34" s="7" t="s">
         <x:v>694</x:v>
-      </x:c>
-      <x:c r="C34" s="7" t="s">
-        <x:v>695</x:v>
       </x:c>
       <x:c r="D34" s="9">
         <x:v>1</x:v>
@@ -7930,47 +7927,47 @@
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
       <x:c r="A35" s="8" t="s">
+        <x:v>695</x:v>
+      </x:c>
+      <x:c r="B35" s="7" t="s">
         <x:v>696</x:v>
       </x:c>
-      <x:c r="B35" s="7" t="s">
+      <x:c r="C35" s="7" t="s">
         <x:v>697</x:v>
       </x:c>
-      <x:c r="C35" s="7" t="s">
+      <x:c r="D35" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E35" s="10" t="s">
         <x:v>698</x:v>
-      </x:c>
-      <x:c r="D35" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E35" s="10" t="s">
-        <x:v>699</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
       <x:c r="A36" s="8" t="s">
+        <x:v>699</x:v>
+      </x:c>
+      <x:c r="B36" s="7" t="s">
         <x:v>700</x:v>
       </x:c>
-      <x:c r="B36" s="7" t="s">
+      <x:c r="C36" s="7" t="s">
         <x:v>701</x:v>
       </x:c>
-      <x:c r="C36" s="7" t="s">
+      <x:c r="D36" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E36" s="10" t="s">
         <x:v>702</x:v>
-      </x:c>
-      <x:c r="D36" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E36" s="10" t="s">
-        <x:v>703</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
       <x:c r="A37" s="8" t="s">
+        <x:v>703</x:v>
+      </x:c>
+      <x:c r="B37" s="7" t="s">
         <x:v>704</x:v>
       </x:c>
-      <x:c r="B37" s="7" t="s">
+      <x:c r="C37" s="7" t="s">
         <x:v>705</x:v>
-      </x:c>
-      <x:c r="C37" s="7" t="s">
-        <x:v>706</x:v>
       </x:c>
       <x:c r="D37" s="9">
         <x:v>1</x:v>
@@ -7979,13 +7976,13 @@
     </x:row>
     <x:row r="38" ht="28" customHeight="1">
       <x:c r="A38" s="8" t="s">
+        <x:v>706</x:v>
+      </x:c>
+      <x:c r="B38" s="7" t="s">
         <x:v>707</x:v>
       </x:c>
-      <x:c r="B38" s="7" t="s">
-        <x:v>708</x:v>
-      </x:c>
       <x:c r="C38" s="7" t="s">
-        <x:v>645</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="D38" s="9">
         <x:v>1</x:v>
@@ -7994,13 +7991,13 @@
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
       <x:c r="A39" s="8" t="s">
+        <x:v>708</x:v>
+      </x:c>
+      <x:c r="B39" s="7" t="s">
         <x:v>709</x:v>
       </x:c>
-      <x:c r="B39" s="7" t="s">
+      <x:c r="C39" s="7" t="s">
         <x:v>710</x:v>
-      </x:c>
-      <x:c r="C39" s="7" t="s">
-        <x:v>711</x:v>
       </x:c>
       <x:c r="D39" s="9">
         <x:v>3</x:v>
@@ -8009,47 +8006,47 @@
     </x:row>
     <x:row r="40" ht="28" customHeight="1">
       <x:c r="A40" s="8" t="s">
+        <x:v>711</x:v>
+      </x:c>
+      <x:c r="B40" s="7" t="s">
         <x:v>712</x:v>
       </x:c>
-      <x:c r="B40" s="7" t="s">
+      <x:c r="C40" s="7" t="s">
         <x:v>713</x:v>
       </x:c>
-      <x:c r="C40" s="7" t="s">
+      <x:c r="D40" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E40" s="10" t="s">
         <x:v>714</x:v>
-      </x:c>
-      <x:c r="D40" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E40" s="10" t="s">
-        <x:v>715</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="8" t="s">
+        <x:v>715</x:v>
+      </x:c>
+      <x:c r="B41" s="7" t="s">
         <x:v>716</x:v>
       </x:c>
-      <x:c r="B41" s="7" t="s">
+      <x:c r="C41" s="7" t="s">
+        <x:v>713</x:v>
+      </x:c>
+      <x:c r="D41" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E41" s="10" t="s">
         <x:v>717</x:v>
-      </x:c>
-      <x:c r="C41" s="7" t="s">
-        <x:v>714</x:v>
-      </x:c>
-      <x:c r="D41" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E41" s="10" t="s">
-        <x:v>718</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
       <x:c r="A42" s="8" t="s">
+        <x:v>718</x:v>
+      </x:c>
+      <x:c r="B42" s="7" t="s">
         <x:v>719</x:v>
       </x:c>
-      <x:c r="B42" s="7" t="s">
+      <x:c r="C42" s="7" t="s">
         <x:v>720</x:v>
-      </x:c>
-      <x:c r="C42" s="7" t="s">
-        <x:v>721</x:v>
       </x:c>
       <x:c r="D42" s="9">
         <x:v>1</x:v>
@@ -8058,10 +8055,10 @@
     </x:row>
     <x:row r="43" ht="28" customHeight="1">
       <x:c r="A43" s="8" t="s">
+        <x:v>721</x:v>
+      </x:c>
+      <x:c r="B43" s="7" t="s">
         <x:v>722</x:v>
-      </x:c>
-      <x:c r="B43" s="7" t="s">
-        <x:v>723</x:v>
       </x:c>
       <x:c r="C43" s="7" t="str">
         <x:v>#069, #079</x:v>
@@ -8073,30 +8070,30 @@
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="8" t="s">
+        <x:v>723</x:v>
+      </x:c>
+      <x:c r="B44" s="7" t="s">
         <x:v>724</x:v>
       </x:c>
-      <x:c r="B44" s="7" t="s">
-        <x:v>725</x:v>
-      </x:c>
       <x:c r="C44" s="7" t="s">
-        <x:v>678</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="D44" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E44" s="10" t="s">
-        <x:v>726</x:v>
+        <x:v>725</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
       <x:c r="A45" s="8" t="s">
+        <x:v>726</x:v>
+      </x:c>
+      <x:c r="B45" s="7" t="s">
         <x:v>727</x:v>
       </x:c>
-      <x:c r="B45" s="7" t="s">
+      <x:c r="C45" s="7" t="s">
         <x:v>728</x:v>
-      </x:c>
-      <x:c r="C45" s="7" t="s">
-        <x:v>729</x:v>
       </x:c>
       <x:c r="D45" s="9">
         <x:v>1</x:v>
@@ -8105,13 +8102,13 @@
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
       <x:c r="A46" s="8" t="s">
+        <x:v>729</x:v>
+      </x:c>
+      <x:c r="B46" s="7" t="s">
         <x:v>730</x:v>
       </x:c>
-      <x:c r="B46" s="7" t="s">
-        <x:v>731</x:v>
-      </x:c>
       <x:c r="C46" s="7" t="s">
-        <x:v>695</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="D46" s="9">
         <x:v>1</x:v>
@@ -8120,47 +8117,47 @@
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
       <x:c r="A47" s="8" t="s">
+        <x:v>731</x:v>
+      </x:c>
+      <x:c r="B47" s="7" t="s">
         <x:v>732</x:v>
       </x:c>
-      <x:c r="B47" s="7" t="s">
+      <x:c r="C47" s="7" t="s">
+        <x:v>606</x:v>
+      </x:c>
+      <x:c r="D47" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E47" s="10" t="s">
         <x:v>733</x:v>
-      </x:c>
-      <x:c r="C47" s="7" t="s">
-        <x:v>607</x:v>
-      </x:c>
-      <x:c r="D47" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E47" s="10" t="s">
-        <x:v>734</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
       <x:c r="A48" s="8" t="s">
+        <x:v>734</x:v>
+      </x:c>
+      <x:c r="B48" s="7" t="s">
         <x:v>735</x:v>
       </x:c>
-      <x:c r="B48" s="7" t="s">
+      <x:c r="C48" s="7" t="s">
         <x:v>736</x:v>
-      </x:c>
-      <x:c r="C48" s="7" t="s">
-        <x:v>737</x:v>
       </x:c>
       <x:c r="D48" s="9">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="10" t="s">
-        <x:v>738</x:v>
+        <x:v>737</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
       <x:c r="A49" s="8" t="s">
+        <x:v>738</x:v>
+      </x:c>
+      <x:c r="B49" s="7" t="s">
         <x:v>739</x:v>
       </x:c>
-      <x:c r="B49" s="7" t="s">
+      <x:c r="C49" s="7" t="s">
         <x:v>740</x:v>
-      </x:c>
-      <x:c r="C49" s="7" t="s">
-        <x:v>741</x:v>
       </x:c>
       <x:c r="D49" s="9">
         <x:v>1</x:v>
@@ -8169,13 +8166,13 @@
     </x:row>
     <x:row r="50" ht="28" customHeight="1">
       <x:c r="A50" s="8" t="s">
+        <x:v>741</x:v>
+      </x:c>
+      <x:c r="B50" s="7" t="s">
         <x:v>742</x:v>
       </x:c>
-      <x:c r="B50" s="7" t="s">
-        <x:v>743</x:v>
-      </x:c>
       <x:c r="C50" s="7" t="s">
-        <x:v>706</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="D50" s="9">
         <x:v>1</x:v>
@@ -8184,64 +8181,64 @@
     </x:row>
     <x:row r="51" ht="28" customHeight="1">
       <x:c r="A51" s="8" t="s">
+        <x:v>743</x:v>
+      </x:c>
+      <x:c r="B51" s="7" t="s">
         <x:v>744</x:v>
       </x:c>
-      <x:c r="B51" s="7" t="s">
+      <x:c r="C51" s="7" t="s">
         <x:v>745</x:v>
-      </x:c>
-      <x:c r="C51" s="7" t="s">
-        <x:v>746</x:v>
       </x:c>
       <x:c r="D51" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E51" s="10" t="s">
-        <x:v>747</x:v>
+        <x:v>746</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="28" customHeight="1">
       <x:c r="A52" s="8" t="s">
+        <x:v>747</x:v>
+      </x:c>
+      <x:c r="B52" s="7" t="s">
         <x:v>748</x:v>
       </x:c>
-      <x:c r="B52" s="7" t="s">
+      <x:c r="C52" s="7" t="s">
         <x:v>749</x:v>
       </x:c>
-      <x:c r="C52" s="7" t="s">
+      <x:c r="D52" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E52" s="10" t="s">
         <x:v>750</x:v>
-      </x:c>
-      <x:c r="D52" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E52" s="10" t="s">
-        <x:v>751</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="28" customHeight="1">
       <x:c r="A53" s="8" t="s">
+        <x:v>751</x:v>
+      </x:c>
+      <x:c r="B53" s="7" t="s">
         <x:v>752</x:v>
       </x:c>
-      <x:c r="B53" s="7" t="s">
+      <x:c r="C53" s="7" t="s">
         <x:v>753</x:v>
-      </x:c>
-      <x:c r="C53" s="7" t="s">
-        <x:v>754</x:v>
       </x:c>
       <x:c r="D53" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E53" s="10" t="s">
-        <x:v>755</x:v>
+        <x:v>754</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="28" customHeight="1">
       <x:c r="A54" s="8" t="s">
+        <x:v>755</x:v>
+      </x:c>
+      <x:c r="B54" s="7" t="s">
         <x:v>756</x:v>
       </x:c>
-      <x:c r="B54" s="7" t="s">
+      <x:c r="C54" s="7" t="s">
         <x:v>757</x:v>
-      </x:c>
-      <x:c r="C54" s="7" t="s">
-        <x:v>758</x:v>
       </x:c>
       <x:c r="D54" s="9">
         <x:v>1</x:v>
@@ -8250,81 +8247,81 @@
     </x:row>
     <x:row r="55" ht="28" customHeight="1">
       <x:c r="A55" s="8" t="s">
+        <x:v>758</x:v>
+      </x:c>
+      <x:c r="B55" s="7" t="s">
         <x:v>759</x:v>
       </x:c>
-      <x:c r="B55" s="7" t="s">
+      <x:c r="C55" s="7" t="s">
         <x:v>760</x:v>
       </x:c>
-      <x:c r="C55" s="7" t="s">
+      <x:c r="D55" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E55" s="10" t="s">
         <x:v>761</x:v>
-      </x:c>
-      <x:c r="D55" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E55" s="10" t="s">
-        <x:v>762</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="28" customHeight="1">
       <x:c r="A56" s="8" t="s">
+        <x:v>762</x:v>
+      </x:c>
+      <x:c r="B56" s="7" t="s">
         <x:v>763</x:v>
       </x:c>
-      <x:c r="B56" s="7" t="s">
+      <x:c r="C56" s="7" t="s">
         <x:v>764</x:v>
       </x:c>
-      <x:c r="C56" s="7" t="s">
+      <x:c r="D56" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E56" s="10" t="s">
         <x:v>765</x:v>
-      </x:c>
-      <x:c r="D56" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E56" s="10" t="s">
-        <x:v>766</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
       <x:c r="A57" s="8" t="s">
+        <x:v>766</x:v>
+      </x:c>
+      <x:c r="B57" s="7" t="s">
         <x:v>767</x:v>
       </x:c>
-      <x:c r="B57" s="7" t="s">
+      <x:c r="C57" s="7" t="s">
         <x:v>768</x:v>
       </x:c>
-      <x:c r="C57" s="7" t="s">
+      <x:c r="D57" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E57" s="10" t="s">
         <x:v>769</x:v>
-      </x:c>
-      <x:c r="D57" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E57" s="10" t="s">
-        <x:v>770</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
       <x:c r="A58" s="8" t="s">
+        <x:v>770</x:v>
+      </x:c>
+      <x:c r="B58" s="7" t="s">
         <x:v>771</x:v>
       </x:c>
-      <x:c r="B58" s="7" t="s">
+      <x:c r="C58" s="7" t="s">
         <x:v>772</x:v>
-      </x:c>
-      <x:c r="C58" s="7" t="s">
-        <x:v>773</x:v>
       </x:c>
       <x:c r="D58" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E58" s="10" t="s">
-        <x:v>774</x:v>
+        <x:v>773</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
       <x:c r="A59" s="8" t="s">
+        <x:v>774</x:v>
+      </x:c>
+      <x:c r="B59" s="7" t="s">
         <x:v>775</x:v>
       </x:c>
-      <x:c r="B59" s="7" t="s">
-        <x:v>776</x:v>
-      </x:c>
       <x:c r="C59" s="7" t="s">
-        <x:v>611</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="D59" s="9">
         <x:v>1</x:v>
@@ -8333,13 +8330,13 @@
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
       <x:c r="A60" s="8" t="s">
+        <x:v>776</x:v>
+      </x:c>
+      <x:c r="B60" s="7" t="s">
         <x:v>777</x:v>
       </x:c>
-      <x:c r="B60" s="7" t="s">
-        <x:v>778</x:v>
-      </x:c>
       <x:c r="C60" s="7" t="s">
-        <x:v>648</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="D60" s="9">
         <x:v>1</x:v>
@@ -8348,13 +8345,13 @@
     </x:row>
     <x:row r="61" ht="28" customHeight="1">
       <x:c r="A61" s="8" t="s">
+        <x:v>778</x:v>
+      </x:c>
+      <x:c r="B61" s="7" t="s">
         <x:v>779</x:v>
       </x:c>
-      <x:c r="B61" s="7" t="s">
-        <x:v>780</x:v>
-      </x:c>
       <x:c r="C61" s="7" t="s">
-        <x:v>632</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="D61" s="9">
         <x:v>1</x:v>
@@ -8363,30 +8360,30 @@
     </x:row>
     <x:row r="62" ht="28" customHeight="1">
       <x:c r="A62" s="8" t="s">
+        <x:v>780</x:v>
+      </x:c>
+      <x:c r="B62" s="7" t="s">
         <x:v>781</x:v>
       </x:c>
-      <x:c r="B62" s="7" t="s">
+      <x:c r="C62" s="7" t="s">
+        <x:v>637</x:v>
+      </x:c>
+      <x:c r="D62" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E62" s="10" t="s">
         <x:v>782</x:v>
-      </x:c>
-      <x:c r="C62" s="7" t="s">
-        <x:v>638</x:v>
-      </x:c>
-      <x:c r="D62" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E62" s="10" t="s">
-        <x:v>783</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="28" customHeight="1">
       <x:c r="A63" s="8" t="s">
+        <x:v>783</x:v>
+      </x:c>
+      <x:c r="B63" s="7" t="s">
         <x:v>784</x:v>
       </x:c>
-      <x:c r="B63" s="7" t="s">
-        <x:v>785</x:v>
-      </x:c>
       <x:c r="C63" s="7" t="s">
-        <x:v>632</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="D63" s="9">
         <x:v>1</x:v>
@@ -8395,13 +8392,13 @@
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
       <x:c r="A64" s="8" t="s">
+        <x:v>785</x:v>
+      </x:c>
+      <x:c r="B64" s="7" t="s">
         <x:v>786</x:v>
       </x:c>
-      <x:c r="B64" s="7" t="s">
+      <x:c r="C64" s="7" t="s">
         <x:v>787</x:v>
-      </x:c>
-      <x:c r="C64" s="7" t="s">
-        <x:v>788</x:v>
       </x:c>
       <x:c r="D64" s="9">
         <x:v>1</x:v>
@@ -8410,13 +8407,13 @@
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
       <x:c r="A65" s="8" t="s">
+        <x:v>788</x:v>
+      </x:c>
+      <x:c r="B65" s="7" t="s">
         <x:v>789</x:v>
       </x:c>
-      <x:c r="B65" s="7" t="s">
+      <x:c r="C65" s="7" t="s">
         <x:v>790</x:v>
-      </x:c>
-      <x:c r="C65" s="7" t="s">
-        <x:v>791</x:v>
       </x:c>
       <x:c r="D65" s="9">
         <x:v>1</x:v>
@@ -8425,13 +8422,13 @@
     </x:row>
     <x:row r="66" ht="28" customHeight="1">
       <x:c r="A66" s="8" t="s">
+        <x:v>791</x:v>
+      </x:c>
+      <x:c r="B66" s="7" t="s">
         <x:v>792</x:v>
       </x:c>
-      <x:c r="B66" s="7" t="s">
-        <x:v>793</x:v>
-      </x:c>
       <x:c r="C66" s="7" t="s">
-        <x:v>621</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="D66" s="9">
         <x:v>1</x:v>
@@ -8440,47 +8437,47 @@
     </x:row>
     <x:row r="67" ht="28" customHeight="1">
       <x:c r="A67" s="8" t="s">
+        <x:v>793</x:v>
+      </x:c>
+      <x:c r="B67" s="7" t="s">
         <x:v>794</x:v>
       </x:c>
-      <x:c r="B67" s="7" t="s">
-        <x:v>795</x:v>
-      </x:c>
       <x:c r="C67" s="7" t="s">
-        <x:v>773</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="D67" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E67" s="10" t="s">
-        <x:v>796</x:v>
+        <x:v>795</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="28" customHeight="1">
       <x:c r="A68" s="8" t="s">
+        <x:v>796</x:v>
+      </x:c>
+      <x:c r="B68" s="7" t="s">
         <x:v>797</x:v>
       </x:c>
-      <x:c r="B68" s="7" t="s">
+      <x:c r="C68" s="7" t="s">
+        <x:v>647</x:v>
+      </x:c>
+      <x:c r="D68" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E68" s="10" t="s">
         <x:v>798</x:v>
-      </x:c>
-      <x:c r="C68" s="7" t="s">
-        <x:v>648</x:v>
-      </x:c>
-      <x:c r="D68" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E68" s="10" t="s">
-        <x:v>799</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
       <x:c r="A69" s="8" t="s">
+        <x:v>799</x:v>
+      </x:c>
+      <x:c r="B69" s="7" t="s">
         <x:v>800</x:v>
       </x:c>
-      <x:c r="B69" s="7" t="s">
-        <x:v>801</x:v>
-      </x:c>
       <x:c r="C69" s="7" t="s">
-        <x:v>628</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="D69" s="9">
         <x:v>1</x:v>
@@ -8489,13 +8486,13 @@
     </x:row>
     <x:row r="70" ht="28" customHeight="1">
       <x:c r="A70" s="8" t="s">
+        <x:v>801</x:v>
+      </x:c>
+      <x:c r="B70" s="7" t="s">
         <x:v>802</x:v>
       </x:c>
-      <x:c r="B70" s="7" t="s">
-        <x:v>803</x:v>
-      </x:c>
       <x:c r="C70" s="7" t="s">
-        <x:v>656</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="D70" s="9">
         <x:v>1</x:v>
@@ -8504,13 +8501,13 @@
     </x:row>
     <x:row r="71" ht="28" customHeight="1">
       <x:c r="A71" s="8" t="s">
+        <x:v>803</x:v>
+      </x:c>
+      <x:c r="B71" s="7" t="s">
         <x:v>804</x:v>
       </x:c>
-      <x:c r="B71" s="7" t="s">
+      <x:c r="C71" s="7" t="s">
         <x:v>805</x:v>
-      </x:c>
-      <x:c r="C71" s="7" t="s">
-        <x:v>806</x:v>
       </x:c>
       <x:c r="D71" s="9">
         <x:v>1</x:v>
@@ -8519,64 +8516,64 @@
     </x:row>
     <x:row r="72" ht="28" customHeight="1">
       <x:c r="A72" s="8" t="s">
+        <x:v>806</x:v>
+      </x:c>
+      <x:c r="B72" s="7" t="s">
         <x:v>807</x:v>
       </x:c>
-      <x:c r="B72" s="7" t="s">
+      <x:c r="C72" s="7" t="s">
         <x:v>808</x:v>
-      </x:c>
-      <x:c r="C72" s="7" t="s">
-        <x:v>809</x:v>
       </x:c>
       <x:c r="D72" s="9">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E72" s="10" t="s">
-        <x:v>810</x:v>
+        <x:v>809</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="28" customHeight="1">
       <x:c r="A73" s="8" t="s">
+        <x:v>810</x:v>
+      </x:c>
+      <x:c r="B73" s="7" t="s">
         <x:v>811</x:v>
       </x:c>
-      <x:c r="B73" s="7" t="s">
+      <x:c r="C73" s="7" t="s">
         <x:v>812</x:v>
       </x:c>
-      <x:c r="C73" s="7" t="s">
+      <x:c r="D73" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E73" s="10" t="s">
         <x:v>813</x:v>
-      </x:c>
-      <x:c r="D73" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E73" s="10" t="s">
-        <x:v>814</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="28" customHeight="1">
       <x:c r="A74" s="8" t="s">
+        <x:v>814</x:v>
+      </x:c>
+      <x:c r="B74" s="7" t="s">
         <x:v>815</x:v>
       </x:c>
-      <x:c r="B74" s="7" t="s">
+      <x:c r="C74" s="7" t="s">
+        <x:v>613</x:v>
+      </x:c>
+      <x:c r="D74" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E74" s="10" t="s">
         <x:v>816</x:v>
-      </x:c>
-      <x:c r="C74" s="7" t="s">
-        <x:v>614</x:v>
-      </x:c>
-      <x:c r="D74" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E74" s="10" t="s">
-        <x:v>817</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="28" customHeight="1">
       <x:c r="A75" s="8" t="s">
+        <x:v>817</x:v>
+      </x:c>
+      <x:c r="B75" s="7" t="s">
         <x:v>818</x:v>
       </x:c>
-      <x:c r="B75" s="7" t="s">
-        <x:v>819</x:v>
-      </x:c>
       <x:c r="C75" s="7" t="s">
-        <x:v>729</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="D75" s="9">
         <x:v>1</x:v>
@@ -8585,64 +8582,64 @@
     </x:row>
     <x:row r="76" ht="28" customHeight="1">
       <x:c r="A76" s="8" t="s">
+        <x:v>819</x:v>
+      </x:c>
+      <x:c r="B76" s="7" t="s">
         <x:v>820</x:v>
       </x:c>
-      <x:c r="B76" s="7" t="s">
+      <x:c r="C76" s="7" t="s">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="D76" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E76" s="10" t="s">
         <x:v>821</x:v>
-      </x:c>
-      <x:c r="C76" s="7" t="s">
-        <x:v>698</x:v>
-      </x:c>
-      <x:c r="D76" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E76" s="10" t="s">
-        <x:v>822</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
       <x:c r="A77" s="8" t="s">
+        <x:v>822</x:v>
+      </x:c>
+      <x:c r="B77" s="7" t="s">
         <x:v>823</x:v>
       </x:c>
-      <x:c r="B77" s="7" t="s">
+      <x:c r="C77" s="7" t="s">
+        <x:v>805</x:v>
+      </x:c>
+      <x:c r="D77" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E77" s="10" t="s">
         <x:v>824</x:v>
-      </x:c>
-      <x:c r="C77" s="7" t="s">
-        <x:v>806</x:v>
-      </x:c>
-      <x:c r="D77" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E77" s="10" t="s">
-        <x:v>825</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
       <x:c r="A78" s="8" t="s">
+        <x:v>825</x:v>
+      </x:c>
+      <x:c r="B78" s="7" t="s">
         <x:v>826</x:v>
       </x:c>
-      <x:c r="B78" s="7" t="s">
-        <x:v>827</x:v>
-      </x:c>
       <x:c r="C78" s="7" t="s">
-        <x:v>603</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="D78" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E78" s="10" t="s">
-        <x:v>828</x:v>
+        <x:v>827</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="28" customHeight="1">
       <x:c r="A79" s="8" t="s">
+        <x:v>828</x:v>
+      </x:c>
+      <x:c r="B79" s="7" t="s">
         <x:v>829</x:v>
       </x:c>
-      <x:c r="B79" s="7" t="s">
-        <x:v>830</x:v>
-      </x:c>
       <x:c r="C79" s="7" t="s">
-        <x:v>698</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="D79" s="9">
         <x:v>1</x:v>
@@ -8651,24 +8648,24 @@
     </x:row>
     <x:row r="80" ht="28" customHeight="1">
       <x:c r="A80" s="8" t="s">
+        <x:v>830</x:v>
+      </x:c>
+      <x:c r="B80" s="7" t="s">
         <x:v>831</x:v>
       </x:c>
-      <x:c r="B80" s="7" t="s">
+      <x:c r="C80" s="7" t="s">
         <x:v>832</x:v>
       </x:c>
-      <x:c r="C80" s="7" t="s">
+      <x:c r="D80" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E80" s="10" t="s">
         <x:v>833</x:v>
-      </x:c>
-      <x:c r="D80" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E80" s="10" t="s">
-        <x:v>834</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="28" customHeight="1">
       <x:c r="A81" s="8" t="s">
-        <x:v>835</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="B81" s="7" t="s">
         <x:v>172</x:v>
@@ -8680,35 +8677,35 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="E81" s="10" t="s">
-        <x:v>836</x:v>
+        <x:v>835</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="28" customHeight="1">
       <x:c r="A82" s="8" t="s">
+        <x:v>836</x:v>
+      </x:c>
+      <x:c r="B82" s="7" t="s">
         <x:v>837</x:v>
       </x:c>
-      <x:c r="B82" s="7" t="s">
+      <x:c r="C82" s="7" t="s">
         <x:v>838</x:v>
-      </x:c>
-      <x:c r="C82" s="7" t="s">
-        <x:v>839</x:v>
       </x:c>
       <x:c r="D82" s="9">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E82" s="10" t="s">
-        <x:v>840</x:v>
+        <x:v>839</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="28" customHeight="1">
       <x:c r="A83" s="8" t="s">
+        <x:v>840</x:v>
+      </x:c>
+      <x:c r="B83" s="7" t="s">
         <x:v>841</x:v>
       </x:c>
-      <x:c r="B83" s="7" t="s">
-        <x:v>842</x:v>
-      </x:c>
       <x:c r="C83" s="7" t="s">
-        <x:v>621</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="D83" s="9">
         <x:v>1</x:v>
@@ -8717,13 +8714,13 @@
     </x:row>
     <x:row r="84" ht="28" customHeight="1">
       <x:c r="A84" s="8" t="s">
+        <x:v>842</x:v>
+      </x:c>
+      <x:c r="B84" s="7" t="s">
         <x:v>843</x:v>
       </x:c>
-      <x:c r="B84" s="7" t="s">
+      <x:c r="C84" s="7" t="s">
         <x:v>844</x:v>
-      </x:c>
-      <x:c r="C84" s="7" t="s">
-        <x:v>845</x:v>
       </x:c>
       <x:c r="D84" s="9">
         <x:v>1</x:v>
@@ -8732,64 +8729,64 @@
     </x:row>
     <x:row r="85" ht="28" customHeight="1">
       <x:c r="A85" s="8" t="s">
+        <x:v>845</x:v>
+      </x:c>
+      <x:c r="B85" s="7" t="s">
         <x:v>846</x:v>
       </x:c>
-      <x:c r="B85" s="7" t="s">
+      <x:c r="C85" s="7" t="s">
+        <x:v>623</x:v>
+      </x:c>
+      <x:c r="D85" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E85" s="10" t="s">
         <x:v>847</x:v>
-      </x:c>
-      <x:c r="C85" s="7" t="s">
-        <x:v>624</x:v>
-      </x:c>
-      <x:c r="D85" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E85" s="10" t="s">
-        <x:v>848</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="28" customHeight="1">
       <x:c r="A86" s="8" t="s">
+        <x:v>848</x:v>
+      </x:c>
+      <x:c r="B86" s="7" t="s">
         <x:v>849</x:v>
       </x:c>
-      <x:c r="B86" s="7" t="s">
+      <x:c r="C86" s="7" t="s">
         <x:v>850</x:v>
       </x:c>
-      <x:c r="C86" s="7" t="s">
+      <x:c r="D86" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E86" s="10" t="s">
         <x:v>851</x:v>
-      </x:c>
-      <x:c r="D86" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E86" s="10" t="s">
-        <x:v>852</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="28" customHeight="1">
       <x:c r="A87" s="8" t="s">
+        <x:v>852</x:v>
+      </x:c>
+      <x:c r="B87" s="7" t="s">
         <x:v>853</x:v>
       </x:c>
-      <x:c r="B87" s="7" t="s">
+      <x:c r="C87" s="7" t="s">
         <x:v>854</x:v>
       </x:c>
-      <x:c r="C87" s="7" t="s">
+      <x:c r="D87" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E87" s="10" t="s">
         <x:v>855</x:v>
-      </x:c>
-      <x:c r="D87" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E87" s="10" t="s">
-        <x:v>856</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="28" customHeight="1">
       <x:c r="A88" s="8" t="s">
+        <x:v>856</x:v>
+      </x:c>
+      <x:c r="B88" s="7" t="s">
         <x:v>857</x:v>
       </x:c>
-      <x:c r="B88" s="7" t="s">
-        <x:v>858</x:v>
-      </x:c>
       <x:c r="C88" s="7" t="s">
-        <x:v>729</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="D88" s="9">
         <x:v>1</x:v>
@@ -8798,13 +8795,13 @@
     </x:row>
     <x:row r="89" ht="28" customHeight="1">
       <x:c r="A89" s="8" t="s">
+        <x:v>858</x:v>
+      </x:c>
+      <x:c r="B89" s="7" t="s">
         <x:v>859</x:v>
       </x:c>
-      <x:c r="B89" s="7" t="s">
-        <x:v>860</x:v>
-      </x:c>
       <x:c r="C89" s="7" t="s">
-        <x:v>645</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="D89" s="9">
         <x:v>1</x:v>
@@ -8813,30 +8810,30 @@
     </x:row>
     <x:row r="90" ht="28" customHeight="1">
       <x:c r="A90" s="8" t="s">
+        <x:v>860</x:v>
+      </x:c>
+      <x:c r="B90" s="7" t="s">
         <x:v>861</x:v>
       </x:c>
-      <x:c r="B90" s="7" t="s">
-        <x:v>862</x:v>
-      </x:c>
       <x:c r="C90" s="7" t="s">
-        <x:v>773</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="D90" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E90" s="10" t="s">
-        <x:v>863</x:v>
+        <x:v>862</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="28" customHeight="1">
       <x:c r="A91" s="8" t="s">
+        <x:v>863</x:v>
+      </x:c>
+      <x:c r="B91" s="7" t="s">
         <x:v>864</x:v>
       </x:c>
-      <x:c r="B91" s="7" t="s">
+      <x:c r="C91" s="7" t="s">
         <x:v>865</x:v>
-      </x:c>
-      <x:c r="C91" s="7" t="s">
-        <x:v>866</x:v>
       </x:c>
       <x:c r="D91" s="9">
         <x:v>1</x:v>
@@ -8845,30 +8842,30 @@
     </x:row>
     <x:row r="92" ht="28" customHeight="1">
       <x:c r="A92" s="8" t="s">
+        <x:v>866</x:v>
+      </x:c>
+      <x:c r="B92" s="7" t="s">
         <x:v>867</x:v>
       </x:c>
-      <x:c r="B92" s="7" t="s">
+      <x:c r="C92" s="7" t="s">
         <x:v>868</x:v>
-      </x:c>
-      <x:c r="C92" s="7" t="s">
-        <x:v>869</x:v>
       </x:c>
       <x:c r="D92" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E92" s="10" t="s">
-        <x:v>870</x:v>
+        <x:v>869</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="28" customHeight="1">
       <x:c r="A93" s="8" t="s">
+        <x:v>870</x:v>
+      </x:c>
+      <x:c r="B93" s="7" t="s">
         <x:v>871</x:v>
       </x:c>
-      <x:c r="B93" s="7" t="s">
-        <x:v>872</x:v>
-      </x:c>
       <x:c r="C93" s="7" t="s">
-        <x:v>806</x:v>
+        <x:v>805</x:v>
       </x:c>
       <x:c r="D93" s="9">
         <x:v>1</x:v>
@@ -8877,30 +8874,30 @@
     </x:row>
     <x:row r="94" ht="28" customHeight="1">
       <x:c r="A94" s="8" t="s">
+        <x:v>872</x:v>
+      </x:c>
+      <x:c r="B94" s="7" t="s">
         <x:v>873</x:v>
       </x:c>
-      <x:c r="B94" s="7" t="s">
+      <x:c r="C94" s="7" t="s">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="D94" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E94" s="10" t="s">
         <x:v>874</x:v>
-      </x:c>
-      <x:c r="C94" s="7" t="s">
-        <x:v>698</x:v>
-      </x:c>
-      <x:c r="D94" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E94" s="10" t="s">
-        <x:v>875</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="28" customHeight="1">
       <x:c r="A95" s="8" t="s">
+        <x:v>875</x:v>
+      </x:c>
+      <x:c r="B95" s="7" t="s">
         <x:v>876</x:v>
       </x:c>
-      <x:c r="B95" s="7" t="s">
-        <x:v>877</x:v>
-      </x:c>
       <x:c r="C95" s="7" t="s">
-        <x:v>695</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="D95" s="9">
         <x:v>1</x:v>
@@ -8909,47 +8906,47 @@
     </x:row>
     <x:row r="96" ht="28" customHeight="1">
       <x:c r="A96" s="8" t="s">
+        <x:v>877</x:v>
+      </x:c>
+      <x:c r="B96" s="7" t="s">
         <x:v>878</x:v>
       </x:c>
-      <x:c r="B96" s="7" t="s">
+      <x:c r="C96" s="7" t="s">
         <x:v>879</x:v>
-      </x:c>
-      <x:c r="C96" s="7" t="s">
-        <x:v>880</x:v>
       </x:c>
       <x:c r="D96" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E96" s="10" t="s">
-        <x:v>881</x:v>
+        <x:v>880</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="28" customHeight="1">
       <x:c r="A97" s="8" t="s">
+        <x:v>881</x:v>
+      </x:c>
+      <x:c r="B97" s="7" t="s">
         <x:v>882</x:v>
       </x:c>
-      <x:c r="B97" s="7" t="s">
+      <x:c r="C97" s="7" t="s">
+        <x:v>844</x:v>
+      </x:c>
+      <x:c r="D97" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E97" s="10" t="s">
         <x:v>883</x:v>
-      </x:c>
-      <x:c r="C97" s="7" t="s">
-        <x:v>845</x:v>
-      </x:c>
-      <x:c r="D97" s="9">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E97" s="10" t="s">
-        <x:v>884</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="s">
+        <x:v>884</x:v>
+      </x:c>
+      <x:c r="B98" t="s">
         <x:v>885</x:v>
       </x:c>
-      <x:c r="B98" t="s">
+      <x:c r="C98" t="s">
         <x:v>886</x:v>
-      </x:c>
-      <x:c r="C98" t="s">
-        <x:v>887</x:v>
       </x:c>
       <x:c r="D98">
         <x:v>1</x:v>
@@ -8970,12 +8967,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rb8b900f310034500"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R580474e253304ace"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R4692635d88174a6d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R5c0c6bf84136459a"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1597c1ac4fd45ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4409329e81d242a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8990,7 +8987,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>888</x:v>
+        <x:v>887</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -9878,7 +9875,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re650d76b22f74a1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e63e02f1f5d42d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9894,27 +9891,27 @@
   <x:sheetData>
     <x:row r="1" ht="34.75" customHeight="1">
       <x:c r="A1" s="20" t="s">
-        <x:v>889</x:v>
+        <x:v>888</x:v>
       </x:c>
       <x:c r="B1" s="20"/>
       <x:c r="C1" s="20"/>
     </x:row>
     <x:row r="2" ht="45.25" customHeight="1">
       <x:c r="A2" s="21" t="s">
-        <x:v>890</x:v>
+        <x:v>889</x:v>
       </x:c>
       <x:c r="B2" s="21"/>
       <x:c r="C2" s="21"/>
     </x:row>
     <x:row r="4" ht="29.25" customHeight="1">
       <x:c r="A4" s="15" t="s">
+        <x:v>890</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="s">
         <x:v>891</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="s">
+      <x:c r="C4" s="15" t="s">
         <x:v>892</x:v>
-      </x:c>
-      <x:c r="C4" s="15" t="s">
-        <x:v>893</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.75" customHeight="1">
@@ -9922,7 +9919,7 @@
         <x:v>310</x:v>
       </x:c>
       <x:c r="B5" s="16" t="s">
-        <x:v>894</x:v>
+        <x:v>893</x:v>
       </x:c>
       <x:c r="C5" s="17"/>
     </x:row>
@@ -9931,7 +9928,7 @@
         <x:v>170</x:v>
       </x:c>
       <x:c r="B6" s="16" t="s">
-        <x:v>895</x:v>
+        <x:v>894</x:v>
       </x:c>
       <x:c r="C6" s="17"/>
     </x:row>
@@ -9940,16 +9937,16 @@
         <x:v>379</x:v>
       </x:c>
       <x:c r="B7" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C7" s="17"/>
     </x:row>
     <x:row r="8" ht="26.75" customHeight="1">
       <x:c r="A8" s="16" t="s">
-        <x:v>455</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="B8" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C8" s="17"/>
     </x:row>
@@ -9958,7 +9955,7 @@
         <x:v>347</x:v>
       </x:c>
       <x:c r="B9" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C9" s="17"/>
     </x:row>
@@ -9967,27 +9964,27 @@
         <x:v>368</x:v>
       </x:c>
       <x:c r="B10" s="16" t="s">
+        <x:v>897</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="s">
         <x:v>898</x:v>
-      </x:c>
-      <x:c r="C10" s="17" t="s">
-        <x:v>899</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.75" customHeight="1">
       <x:c r="A11" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="B11" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C11" s="17"/>
     </x:row>
     <x:row r="12" ht="26.75" customHeight="1">
       <x:c r="A12" s="16" t="s">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="s">
         <x:v>901</x:v>
-      </x:c>
-      <x:c r="B12" s="16" t="s">
-        <x:v>902</x:v>
       </x:c>
       <x:c r="C12" s="17"/>
     </x:row>
@@ -9996,25 +9993,25 @@
         <x:v>303</x:v>
       </x:c>
       <x:c r="B13" s="16" t="s">
-        <x:v>895</x:v>
+        <x:v>894</x:v>
       </x:c>
       <x:c r="C13" s="17"/>
     </x:row>
     <x:row r="14" ht="26.75" customHeight="1">
       <x:c r="A14" s="16" t="s">
+        <x:v>902</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="s">
         <x:v>903</x:v>
-      </x:c>
-      <x:c r="B14" s="16" t="s">
-        <x:v>904</x:v>
       </x:c>
       <x:c r="C14" s="17"/>
     </x:row>
     <x:row r="15" ht="26.75" customHeight="1">
       <x:c r="A15" s="16" t="s">
+        <x:v>904</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="s">
         <x:v>905</x:v>
-      </x:c>
-      <x:c r="B15" s="16" t="s">
-        <x:v>906</x:v>
       </x:c>
       <x:c r="C15" s="17"/>
     </x:row>
@@ -10023,7 +10020,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B16" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C16" s="17"/>
     </x:row>
@@ -10032,7 +10029,7 @@
         <x:v>198</x:v>
       </x:c>
       <x:c r="B17" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C17" s="17"/>
     </x:row>
@@ -10041,7 +10038,7 @@
         <x:v>405</x:v>
       </x:c>
       <x:c r="B18" s="16" t="s">
-        <x:v>902</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C18" s="17"/>
     </x:row>
@@ -10050,25 +10047,25 @@
         <x:v>260</x:v>
       </x:c>
       <x:c r="B19" s="16" t="s">
-        <x:v>894</x:v>
+        <x:v>893</x:v>
       </x:c>
       <x:c r="C19" s="17"/>
     </x:row>
     <x:row r="20" ht="26.75" customHeight="1">
       <x:c r="A20" s="16" t="s">
-        <x:v>561</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="B20" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C20" s="17"/>
     </x:row>
     <x:row r="21" ht="26.75" customHeight="1">
       <x:c r="A21" s="16" t="s">
-        <x:v>908</x:v>
+        <x:v>907</x:v>
       </x:c>
       <x:c r="B21" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C21" s="17"/>
     </x:row>
@@ -10077,25 +10074,25 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B22" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C22" s="17"/>
     </x:row>
     <x:row r="23" ht="26.75" customHeight="1">
       <x:c r="A23" s="16" t="s">
+        <x:v>908</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="s">
         <x:v>909</x:v>
-      </x:c>
-      <x:c r="B23" s="16" t="s">
-        <x:v>910</x:v>
       </x:c>
       <x:c r="C23" s="17"/>
     </x:row>
     <x:row r="24" ht="26.75" customHeight="1">
       <x:c r="A24" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="B24" s="16" t="s">
-        <x:v>894</x:v>
+        <x:v>893</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
     </x:row>
@@ -10104,36 +10101,36 @@
         <x:v>325</x:v>
       </x:c>
       <x:c r="B25" s="16" t="s">
-        <x:v>895</x:v>
+        <x:v>894</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
     </x:row>
     <x:row r="26" ht="26.75" customHeight="1">
       <x:c r="A26" s="16" t="s">
-        <x:v>465</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="B26" s="16" t="s">
-        <x:v>895</x:v>
+        <x:v>894</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
     </x:row>
     <x:row r="27" ht="26.75" customHeight="1">
       <x:c r="A27" s="16" t="s">
-        <x:v>554</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="B27" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C27" s="17" t="s">
-        <x:v>912</x:v>
+        <x:v>911</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="26.75" customHeight="1">
       <x:c r="A28" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>912</x:v>
       </x:c>
       <x:c r="B28" s="16" t="s">
-        <x:v>910</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="C28" s="17"/>
     </x:row>
@@ -10142,7 +10139,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B29" s="16" t="s">
-        <x:v>910</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="C29" s="17"/>
     </x:row>
@@ -10151,7 +10148,7 @@
         <x:v>191</x:v>
       </x:c>
       <x:c r="B30" s="16" t="s">
-        <x:v>910</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="C30" s="17"/>
     </x:row>
@@ -10160,25 +10157,25 @@
         <x:v>141</x:v>
       </x:c>
       <x:c r="B31" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C31" s="17"/>
     </x:row>
     <x:row r="32" ht="26.75" customHeight="1">
       <x:c r="A32" s="16" t="s">
-        <x:v>549</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="B32" s="16" t="s">
-        <x:v>902</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C32" s="17"/>
     </x:row>
     <x:row r="33" ht="26.75" customHeight="1">
       <x:c r="A33" s="16" t="s">
-        <x:v>914</x:v>
+        <x:v>913</x:v>
       </x:c>
       <x:c r="B33" s="16" t="s">
-        <x:v>902</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C33" s="17"/>
     </x:row>
@@ -10187,16 +10184,16 @@
         <x:v>318</x:v>
       </x:c>
       <x:c r="B34" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C34" s="17"/>
     </x:row>
     <x:row r="35" ht="26.75" customHeight="1">
       <x:c r="A35" s="16" t="s">
-        <x:v>505</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="B35" s="16" t="s">
-        <x:v>895</x:v>
+        <x:v>894</x:v>
       </x:c>
       <x:c r="C35" s="17"/>
     </x:row>
@@ -10205,18 +10202,18 @@
         <x:v>268</x:v>
       </x:c>
       <x:c r="B36" s="16" t="s">
+        <x:v>897</x:v>
+      </x:c>
+      <x:c r="C36" s="17" t="s">
         <x:v>898</x:v>
-      </x:c>
-      <x:c r="C36" s="17" t="s">
-        <x:v>899</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="26.75" customHeight="1">
       <x:c r="A37" s="16" t="s">
-        <x:v>915</x:v>
+        <x:v>914</x:v>
       </x:c>
       <x:c r="B37" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="C37" s="17"/>
     </x:row>
@@ -10225,7 +10222,7 @@
         <x:v>177</x:v>
       </x:c>
       <x:c r="B38" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C38" s="17"/>
     </x:row>
@@ -10234,36 +10231,36 @@
         <x:v>239</x:v>
       </x:c>
       <x:c r="B39" s="16" t="s">
-        <x:v>902</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C39" s="17" t="s">
-        <x:v>916</x:v>
+        <x:v>915</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="26.75" customHeight="1">
       <x:c r="A40" s="16" t="s">
-        <x:v>445</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="B40" s="16" t="s">
-        <x:v>902</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C40" s="17"/>
     </x:row>
     <x:row r="41" ht="26.75" customHeight="1">
       <x:c r="A41" s="16" t="s">
-        <x:v>917</x:v>
+        <x:v>916</x:v>
       </x:c>
       <x:c r="B41" s="16" t="s">
-        <x:v>902</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C41" s="17"/>
     </x:row>
     <x:row r="42" ht="26.75" customHeight="1">
       <x:c r="A42" s="16" t="s">
-        <x:v>918</x:v>
+        <x:v>917</x:v>
       </x:c>
       <x:c r="B42" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C42" s="17"/>
     </x:row>
@@ -10272,10 +10269,10 @@
         <x:v>224</x:v>
       </x:c>
       <x:c r="B43" s="16" t="s">
+        <x:v>897</x:v>
+      </x:c>
+      <x:c r="C43" s="17" t="s">
         <x:v>898</x:v>
-      </x:c>
-      <x:c r="C43" s="17" t="s">
-        <x:v>899</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="26.75" customHeight="1">
@@ -10283,7 +10280,7 @@
         <x:v>182</x:v>
       </x:c>
       <x:c r="B44" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C44" s="17"/>
     </x:row>
@@ -10292,16 +10289,16 @@
         <x:v>162</x:v>
       </x:c>
       <x:c r="B45" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C45" s="17"/>
     </x:row>
     <x:row r="46" ht="26.75" customHeight="1">
       <x:c r="A46" s="16" t="s">
-        <x:v>919</x:v>
+        <x:v>918</x:v>
       </x:c>
       <x:c r="B46" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C46" s="17"/>
     </x:row>
@@ -10310,19 +10307,19 @@
         <x:v>156</x:v>
       </x:c>
       <x:c r="B47" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C47" s="17"/>
     </x:row>
     <x:row r="48" ht="26.75" customHeight="1">
       <x:c r="A48" s="16" t="s">
+        <x:v>919</x:v>
+      </x:c>
+      <x:c r="B48" s="16" t="s">
+        <x:v>897</x:v>
+      </x:c>
+      <x:c r="C48" s="17" t="s">
         <x:v>920</x:v>
-      </x:c>
-      <x:c r="B48" s="16" t="s">
-        <x:v>898</x:v>
-      </x:c>
-      <x:c r="C48" s="17" t="s">
-        <x:v>921</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="26.75" customHeight="1">
@@ -10330,7 +10327,7 @@
         <x:v>286</x:v>
       </x:c>
       <x:c r="B49" s="16" t="s">
-        <x:v>897</x:v>
+        <x:v>896</x:v>
       </x:c>
       <x:c r="C49" s="17"/>
     </x:row>
@@ -10339,16 +10336,16 @@
         <x:v>212</x:v>
       </x:c>
       <x:c r="B50" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C50" s="17"/>
     </x:row>
     <x:row r="51" ht="26.75" customHeight="1">
       <x:c r="A51" s="16" t="s">
-        <x:v>922</x:v>
+        <x:v>921</x:v>
       </x:c>
       <x:c r="B51" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C51" s="17"/>
     </x:row>
@@ -10357,38 +10354,38 @@
         <x:v>232</x:v>
       </x:c>
       <x:c r="B52" s="16" t="s">
-        <x:v>910</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="C52" s="17"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" t="s">
-        <x:v>571</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="B53" t="s">
         <x:v>379</x:v>
       </x:c>
       <x:c r="C53" t="s">
-        <x:v>923</x:v>
+        <x:v>922</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" t="s">
-        <x:v>580</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="B54" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" t="s">
-        <x:v>587</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="B55" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C55" t="s">
-        <x:v>924</x:v>
+        <x:v>923</x:v>
       </x:c>
     </x:row>
     <x:row r="56">

</xml_diff>

<commit_message>
Add structured award tracking to source workbook
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rc222a9472e3344dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R2c9bb016314a477d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R9465833a97b243a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Rb2db0512aa28459e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R4e84b1532c424402"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rd2dd75fc65884b43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rbebb77c9a0d749d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Rbfb085d9a3b840a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2780,7 +2780,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="14">
+  <x:numFmts count="2">
+    <x:numFmt numFmtId="200" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="201" formatCode="#,##0"/>
+  </x:numFmts>
+  <x:fonts count="15">
     <x:font>
       <x:sz val="12"/>
       <x:color theme="1"/>
@@ -2858,8 +2862,14 @@
       <x:color rgb="FF5F6368"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -2889,6 +2899,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE8E7E2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -2955,7 +2975,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="22">
+  <x:cellXfs count="41">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3014,6 +3034,51 @@
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -3285,10 +3350,25 @@
     <x:col min="14" max="14" width="45.5" customWidth="1"/>
     <x:col min="15" max="15" width="62.1640625" customWidth="1"/>
     <x:col min="16" max="16" width="49.1640625" customWidth="1"/>
-    <x:col min="17" max="17" width="11.1640625" customWidth="1"/>
+    <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="28" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="18" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="20" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="16" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="22" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="16" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="18" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="20" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="32" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="20" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="14" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="16" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="18" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="22" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="32" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -3336,6 +3416,54 @@
       </x:c>
       <x:c r="P1" t="s">
         <x:v>15</x:v>
+      </x:c>
+      <x:c r="Q1" s="26" t="str">
+        <x:v>Award Type</x:v>
+      </x:c>
+      <x:c r="R1" s="26" t="str">
+        <x:v>Additional Info</x:v>
+      </x:c>
+      <x:c r="S1" s="26" t="str">
+        <x:v>Cash-equivalent Amount</x:v>
+      </x:c>
+      <x:c r="T1" s="26" t="str">
+        <x:v>Cash-equivalent Currency</x:v>
+      </x:c>
+      <x:c r="U1" s="26" t="str">
+        <x:v>Credit Amount</x:v>
+      </x:c>
+      <x:c r="V1" s="26" t="str">
+        <x:v>Credit Currency / Units</x:v>
+      </x:c>
+      <x:c r="W1" s="26" t="str">
+        <x:v>Subscription Count</x:v>
+      </x:c>
+      <x:c r="X1" s="26" t="str">
+        <x:v>Subscription Amount</x:v>
+      </x:c>
+      <x:c r="Y1" s="26" t="str">
+        <x:v>Subscription Currency</x:v>
+      </x:c>
+      <x:c r="Z1" s="26" t="str">
+        <x:v>Other Non-cash Prize</x:v>
+      </x:c>
+      <x:c r="AA1" s="26" t="str">
+        <x:v>Physical Asset</x:v>
+      </x:c>
+      <x:c r="AB1" s="26" t="str">
+        <x:v>Trophy Count</x:v>
+      </x:c>
+      <x:c r="AC1" s="26" t="str">
+        <x:v>Funding Amount</x:v>
+      </x:c>
+      <x:c r="AD1" s="26" t="str">
+        <x:v>Funding Currency</x:v>
+      </x:c>
+      <x:c r="AE1" s="26" t="str">
+        <x:v>Cash-equivalent Treatment</x:v>
+      </x:c>
+      <x:c r="AF1" s="26" t="str">
+        <x:v>Review Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -3387,6 +3515,32 @@
       <x:c r="P2" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q2" s="36" t="str">
+        <x:v>1st Place</x:v>
+      </x:c>
+      <x:c r="R2" s="36"/>
+      <x:c r="S2" s="37"/>
+      <x:c r="T2" s="38"/>
+      <x:c r="U2" s="37"/>
+      <x:c r="V2" s="38"/>
+      <x:c r="W2" s="38"/>
+      <x:c r="X2" s="37"/>
+      <x:c r="Y2" s="38"/>
+      <x:c r="Z2" s="36"/>
+      <x:c r="AA2" s="36"/>
+      <x:c r="AB2" s="39"/>
+      <x:c r="AC2" s="40" t="n">
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="AD2" s="36" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="AE2" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF2" s="38" t="str">
+        <x:v>Funding, not a cash prize</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3">
@@ -3437,6 +3591,22 @@
       <x:c r="P3" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q3" s="36"/>
+      <x:c r="R3" s="36"/>
+      <x:c r="S3" s="37"/>
+      <x:c r="T3" s="38"/>
+      <x:c r="U3" s="37"/>
+      <x:c r="V3" s="38"/>
+      <x:c r="W3" s="38"/>
+      <x:c r="X3" s="37"/>
+      <x:c r="Y3" s="38"/>
+      <x:c r="Z3" s="36"/>
+      <x:c r="AA3" s="36"/>
+      <x:c r="AB3" s="39"/>
+      <x:c r="AC3" s="40"/>
+      <x:c r="AD3" s="36"/>
+      <x:c r="AE3" s="38"/>
+      <x:c r="AF3" s="38"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4">
@@ -3487,6 +3657,30 @@
       <x:c r="P4" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q4" s="36" t="str">
+        <x:v>Best Project</x:v>
+      </x:c>
+      <x:c r="R4" s="36" t="str">
+        <x:v>Rated best project</x:v>
+      </x:c>
+      <x:c r="S4" s="37"/>
+      <x:c r="T4" s="38"/>
+      <x:c r="U4" s="37"/>
+      <x:c r="V4" s="38"/>
+      <x:c r="W4" s="38"/>
+      <x:c r="X4" s="37"/>
+      <x:c r="Y4" s="38"/>
+      <x:c r="Z4" s="36"/>
+      <x:c r="AA4" s="36"/>
+      <x:c r="AB4" s="39"/>
+      <x:c r="AC4" s="40"/>
+      <x:c r="AD4" s="36"/>
+      <x:c r="AE4" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF4" s="38" t="str">
+        <x:v>Recognition only</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5">
@@ -3537,6 +3731,40 @@
       <x:c r="P5" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q5" s="36" t="str">
+        <x:v>1st Place</x:v>
+      </x:c>
+      <x:c r="R5" s="36" t="str">
+        <x:v>Best Use of IBM Bluemix</x:v>
+      </x:c>
+      <x:c r="S5" s="37"/>
+      <x:c r="T5" s="38"/>
+      <x:c r="U5" s="37" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="V5" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="W5" s="38"/>
+      <x:c r="X5" s="37"/>
+      <x:c r="Y5" s="38"/>
+      <x:c r="Z5" s="36" t="str">
+        <x:v>IBM Bluemix credits; SmartWatch</x:v>
+      </x:c>
+      <x:c r="AA5" s="36" t="str">
+        <x:v>SmartWatch</x:v>
+      </x:c>
+      <x:c r="AB5" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AC5" s="40"/>
+      <x:c r="AD5" s="36"/>
+      <x:c r="AE5" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF5" s="38" t="str">
+        <x:v>US$100,000 IBM Bluemix credit value</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6">
@@ -3587,6 +3815,22 @@
       <x:c r="P6" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q6" s="36"/>
+      <x:c r="R6" s="36"/>
+      <x:c r="S6" s="37"/>
+      <x:c r="T6" s="38"/>
+      <x:c r="U6" s="37"/>
+      <x:c r="V6" s="38"/>
+      <x:c r="W6" s="38"/>
+      <x:c r="X6" s="37"/>
+      <x:c r="Y6" s="38"/>
+      <x:c r="Z6" s="36"/>
+      <x:c r="AA6" s="36"/>
+      <x:c r="AB6" s="39"/>
+      <x:c r="AC6" s="40"/>
+      <x:c r="AD6" s="36"/>
+      <x:c r="AE6" s="38"/>
+      <x:c r="AF6" s="38"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7">
@@ -3637,6 +3881,28 @@
       <x:c r="P7" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q7" s="36" t="str">
+        <x:v>Top 10</x:v>
+      </x:c>
+      <x:c r="R7" s="36"/>
+      <x:c r="S7" s="37"/>
+      <x:c r="T7" s="38"/>
+      <x:c r="U7" s="37"/>
+      <x:c r="V7" s="38"/>
+      <x:c r="W7" s="38"/>
+      <x:c r="X7" s="37"/>
+      <x:c r="Y7" s="38"/>
+      <x:c r="Z7" s="36"/>
+      <x:c r="AA7" s="36"/>
+      <x:c r="AB7" s="39"/>
+      <x:c r="AC7" s="40"/>
+      <x:c r="AD7" s="36"/>
+      <x:c r="AE7" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF7" s="38" t="str">
+        <x:v>Recognition only</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8">
@@ -3687,6 +3953,22 @@
       <x:c r="P8" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q8" s="36"/>
+      <x:c r="R8" s="36"/>
+      <x:c r="S8" s="37"/>
+      <x:c r="T8" s="38"/>
+      <x:c r="U8" s="37"/>
+      <x:c r="V8" s="38"/>
+      <x:c r="W8" s="38"/>
+      <x:c r="X8" s="37"/>
+      <x:c r="Y8" s="38"/>
+      <x:c r="Z8" s="36"/>
+      <x:c r="AA8" s="36"/>
+      <x:c r="AB8" s="39"/>
+      <x:c r="AC8" s="40"/>
+      <x:c r="AD8" s="36"/>
+      <x:c r="AE8" s="38"/>
+      <x:c r="AF8" s="38"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9">
@@ -3737,6 +4019,22 @@
       <x:c r="P9" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q9" s="36"/>
+      <x:c r="R9" s="36"/>
+      <x:c r="S9" s="37"/>
+      <x:c r="T9" s="38"/>
+      <x:c r="U9" s="37"/>
+      <x:c r="V9" s="38"/>
+      <x:c r="W9" s="38"/>
+      <x:c r="X9" s="37"/>
+      <x:c r="Y9" s="38"/>
+      <x:c r="Z9" s="36"/>
+      <x:c r="AA9" s="36"/>
+      <x:c r="AB9" s="39"/>
+      <x:c r="AC9" s="40"/>
+      <x:c r="AD9" s="36"/>
+      <x:c r="AE9" s="38"/>
+      <x:c r="AF9" s="38"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10">
@@ -3787,6 +4085,22 @@
       <x:c r="P10" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q10" s="36"/>
+      <x:c r="R10" s="36"/>
+      <x:c r="S10" s="37"/>
+      <x:c r="T10" s="38"/>
+      <x:c r="U10" s="37"/>
+      <x:c r="V10" s="38"/>
+      <x:c r="W10" s="38"/>
+      <x:c r="X10" s="37"/>
+      <x:c r="Y10" s="38"/>
+      <x:c r="Z10" s="36"/>
+      <x:c r="AA10" s="36"/>
+      <x:c r="AB10" s="39"/>
+      <x:c r="AC10" s="40"/>
+      <x:c r="AD10" s="36"/>
+      <x:c r="AE10" s="38"/>
+      <x:c r="AF10" s="38"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11">
@@ -3837,6 +4151,30 @@
       <x:c r="P11" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q11" s="36" t="str">
+        <x:v>Best Project</x:v>
+      </x:c>
+      <x:c r="R11" s="36" t="str">
+        <x:v>Rated best project</x:v>
+      </x:c>
+      <x:c r="S11" s="37"/>
+      <x:c r="T11" s="38"/>
+      <x:c r="U11" s="37"/>
+      <x:c r="V11" s="38"/>
+      <x:c r="W11" s="38"/>
+      <x:c r="X11" s="37"/>
+      <x:c r="Y11" s="38"/>
+      <x:c r="Z11" s="36"/>
+      <x:c r="AA11" s="36"/>
+      <x:c r="AB11" s="39"/>
+      <x:c r="AC11" s="40"/>
+      <x:c r="AD11" s="36"/>
+      <x:c r="AE11" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF11" s="38" t="str">
+        <x:v>Recognition only</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12">
@@ -3887,6 +4225,22 @@
       <x:c r="P12" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q12" s="36"/>
+      <x:c r="R12" s="36"/>
+      <x:c r="S12" s="37"/>
+      <x:c r="T12" s="38"/>
+      <x:c r="U12" s="37"/>
+      <x:c r="V12" s="38"/>
+      <x:c r="W12" s="38"/>
+      <x:c r="X12" s="37"/>
+      <x:c r="Y12" s="38"/>
+      <x:c r="Z12" s="36"/>
+      <x:c r="AA12" s="36"/>
+      <x:c r="AB12" s="39"/>
+      <x:c r="AC12" s="40"/>
+      <x:c r="AD12" s="36"/>
+      <x:c r="AE12" s="38"/>
+      <x:c r="AF12" s="38"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13">
@@ -3937,6 +4291,22 @@
       <x:c r="P13" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q13" s="36"/>
+      <x:c r="R13" s="36"/>
+      <x:c r="S13" s="37"/>
+      <x:c r="T13" s="38"/>
+      <x:c r="U13" s="37"/>
+      <x:c r="V13" s="38"/>
+      <x:c r="W13" s="38"/>
+      <x:c r="X13" s="37"/>
+      <x:c r="Y13" s="38"/>
+      <x:c r="Z13" s="36"/>
+      <x:c r="AA13" s="36"/>
+      <x:c r="AB13" s="39"/>
+      <x:c r="AC13" s="40"/>
+      <x:c r="AD13" s="36"/>
+      <x:c r="AE13" s="38"/>
+      <x:c r="AF13" s="38"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14">
@@ -3987,6 +4357,22 @@
       <x:c r="P14" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q14" s="36"/>
+      <x:c r="R14" s="36"/>
+      <x:c r="S14" s="37"/>
+      <x:c r="T14" s="38"/>
+      <x:c r="U14" s="37"/>
+      <x:c r="V14" s="38"/>
+      <x:c r="W14" s="38"/>
+      <x:c r="X14" s="37"/>
+      <x:c r="Y14" s="38"/>
+      <x:c r="Z14" s="36"/>
+      <x:c r="AA14" s="36"/>
+      <x:c r="AB14" s="39"/>
+      <x:c r="AC14" s="40"/>
+      <x:c r="AD14" s="36"/>
+      <x:c r="AE14" s="38"/>
+      <x:c r="AF14" s="38"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15">
@@ -4037,6 +4423,34 @@
       <x:c r="P15" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q15" s="36" t="str">
+        <x:v>3rd Place</x:v>
+      </x:c>
+      <x:c r="R15" s="36"/>
+      <x:c r="S15" s="37" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="T15" s="38" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="U15" s="37"/>
+      <x:c r="V15" s="38"/>
+      <x:c r="W15" s="38"/>
+      <x:c r="X15" s="37"/>
+      <x:c r="Y15" s="38"/>
+      <x:c r="Z15" s="36" t="str">
+        <x:v>S$100 Capitaland voucher</x:v>
+      </x:c>
+      <x:c r="AA15" s="36"/>
+      <x:c r="AB15" s="39"/>
+      <x:c r="AC15" s="40"/>
+      <x:c r="AD15" s="36"/>
+      <x:c r="AE15" s="38" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AF15" s="38" t="str">
+        <x:v>Voucher counted as cash equivalent</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16">
@@ -4087,6 +4501,22 @@
       <x:c r="P16" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q16" s="36"/>
+      <x:c r="R16" s="36"/>
+      <x:c r="S16" s="37"/>
+      <x:c r="T16" s="38"/>
+      <x:c r="U16" s="37"/>
+      <x:c r="V16" s="38"/>
+      <x:c r="W16" s="38"/>
+      <x:c r="X16" s="37"/>
+      <x:c r="Y16" s="38"/>
+      <x:c r="Z16" s="36"/>
+      <x:c r="AA16" s="36"/>
+      <x:c r="AB16" s="39"/>
+      <x:c r="AC16" s="40"/>
+      <x:c r="AD16" s="36"/>
+      <x:c r="AE16" s="38"/>
+      <x:c r="AF16" s="38"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17">
@@ -4137,6 +4567,22 @@
       <x:c r="P17" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q17" s="36"/>
+      <x:c r="R17" s="36"/>
+      <x:c r="S17" s="37"/>
+      <x:c r="T17" s="38"/>
+      <x:c r="U17" s="37"/>
+      <x:c r="V17" s="38"/>
+      <x:c r="W17" s="38"/>
+      <x:c r="X17" s="37"/>
+      <x:c r="Y17" s="38"/>
+      <x:c r="Z17" s="36"/>
+      <x:c r="AA17" s="36"/>
+      <x:c r="AB17" s="39"/>
+      <x:c r="AC17" s="40"/>
+      <x:c r="AD17" s="36"/>
+      <x:c r="AE17" s="38"/>
+      <x:c r="AF17" s="38"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18">
@@ -4187,6 +4633,32 @@
       <x:c r="P18" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q18" s="36" t="str">
+        <x:v>2nd Place</x:v>
+      </x:c>
+      <x:c r="R18" s="36"/>
+      <x:c r="S18" s="37" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="T18" s="38" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="U18" s="37"/>
+      <x:c r="V18" s="38"/>
+      <x:c r="W18" s="38"/>
+      <x:c r="X18" s="37"/>
+      <x:c r="Y18" s="38"/>
+      <x:c r="Z18" s="36"/>
+      <x:c r="AA18" s="36"/>
+      <x:c r="AB18" s="39"/>
+      <x:c r="AC18" s="40"/>
+      <x:c r="AD18" s="36"/>
+      <x:c r="AE18" s="38" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AF18" s="38" t="str">
+        <x:v>Explicit cash</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19">
@@ -4237,6 +4709,22 @@
       <x:c r="P19" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q19" s="36"/>
+      <x:c r="R19" s="36"/>
+      <x:c r="S19" s="37"/>
+      <x:c r="T19" s="38"/>
+      <x:c r="U19" s="37"/>
+      <x:c r="V19" s="38"/>
+      <x:c r="W19" s="38"/>
+      <x:c r="X19" s="37"/>
+      <x:c r="Y19" s="38"/>
+      <x:c r="Z19" s="36"/>
+      <x:c r="AA19" s="36"/>
+      <x:c r="AB19" s="39"/>
+      <x:c r="AC19" s="40"/>
+      <x:c r="AD19" s="36"/>
+      <x:c r="AE19" s="38"/>
+      <x:c r="AF19" s="38"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20">
@@ -4287,6 +4775,22 @@
       <x:c r="P20" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q20" s="36"/>
+      <x:c r="R20" s="36"/>
+      <x:c r="S20" s="37"/>
+      <x:c r="T20" s="38"/>
+      <x:c r="U20" s="37"/>
+      <x:c r="V20" s="38"/>
+      <x:c r="W20" s="38"/>
+      <x:c r="X20" s="37"/>
+      <x:c r="Y20" s="38"/>
+      <x:c r="Z20" s="36"/>
+      <x:c r="AA20" s="36"/>
+      <x:c r="AB20" s="39"/>
+      <x:c r="AC20" s="40"/>
+      <x:c r="AD20" s="36"/>
+      <x:c r="AE20" s="38"/>
+      <x:c r="AF20" s="38"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21">
@@ -4337,6 +4841,22 @@
       <x:c r="P21" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q21" s="36"/>
+      <x:c r="R21" s="36"/>
+      <x:c r="S21" s="37"/>
+      <x:c r="T21" s="38"/>
+      <x:c r="U21" s="37"/>
+      <x:c r="V21" s="38"/>
+      <x:c r="W21" s="38"/>
+      <x:c r="X21" s="37"/>
+      <x:c r="Y21" s="38"/>
+      <x:c r="Z21" s="36"/>
+      <x:c r="AA21" s="36"/>
+      <x:c r="AB21" s="39"/>
+      <x:c r="AC21" s="40"/>
+      <x:c r="AD21" s="36"/>
+      <x:c r="AE21" s="38"/>
+      <x:c r="AF21" s="38"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22">
@@ -4387,6 +4907,22 @@
       <x:c r="P22" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q22" s="36"/>
+      <x:c r="R22" s="36"/>
+      <x:c r="S22" s="37"/>
+      <x:c r="T22" s="38"/>
+      <x:c r="U22" s="37"/>
+      <x:c r="V22" s="38"/>
+      <x:c r="W22" s="38"/>
+      <x:c r="X22" s="37"/>
+      <x:c r="Y22" s="38"/>
+      <x:c r="Z22" s="36"/>
+      <x:c r="AA22" s="36"/>
+      <x:c r="AB22" s="39"/>
+      <x:c r="AC22" s="40"/>
+      <x:c r="AD22" s="36"/>
+      <x:c r="AE22" s="38"/>
+      <x:c r="AF22" s="38"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23">
@@ -4437,6 +4973,22 @@
       <x:c r="P23" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q23" s="36"/>
+      <x:c r="R23" s="36"/>
+      <x:c r="S23" s="37"/>
+      <x:c r="T23" s="38"/>
+      <x:c r="U23" s="37"/>
+      <x:c r="V23" s="38"/>
+      <x:c r="W23" s="38"/>
+      <x:c r="X23" s="37"/>
+      <x:c r="Y23" s="38"/>
+      <x:c r="Z23" s="36"/>
+      <x:c r="AA23" s="36"/>
+      <x:c r="AB23" s="39"/>
+      <x:c r="AC23" s="40"/>
+      <x:c r="AD23" s="36"/>
+      <x:c r="AE23" s="38"/>
+      <x:c r="AF23" s="38"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24">
@@ -4487,6 +5039,22 @@
       <x:c r="P24" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q24" s="36"/>
+      <x:c r="R24" s="36"/>
+      <x:c r="S24" s="37"/>
+      <x:c r="T24" s="38"/>
+      <x:c r="U24" s="37"/>
+      <x:c r="V24" s="38"/>
+      <x:c r="W24" s="38"/>
+      <x:c r="X24" s="37"/>
+      <x:c r="Y24" s="38"/>
+      <x:c r="Z24" s="36"/>
+      <x:c r="AA24" s="36"/>
+      <x:c r="AB24" s="39"/>
+      <x:c r="AC24" s="40"/>
+      <x:c r="AD24" s="36"/>
+      <x:c r="AE24" s="38"/>
+      <x:c r="AF24" s="38"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25">
@@ -4537,6 +5105,22 @@
       <x:c r="P25" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q25" s="36"/>
+      <x:c r="R25" s="36"/>
+      <x:c r="S25" s="37"/>
+      <x:c r="T25" s="38"/>
+      <x:c r="U25" s="37"/>
+      <x:c r="V25" s="38"/>
+      <x:c r="W25" s="38"/>
+      <x:c r="X25" s="37"/>
+      <x:c r="Y25" s="38"/>
+      <x:c r="Z25" s="36"/>
+      <x:c r="AA25" s="36"/>
+      <x:c r="AB25" s="39"/>
+      <x:c r="AC25" s="40"/>
+      <x:c r="AD25" s="36"/>
+      <x:c r="AE25" s="38"/>
+      <x:c r="AF25" s="38"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26">
@@ -4586,6 +5170,32 @@
       </x:c>
       <x:c r="P26" t="s">
         <x:v>25</x:v>
+      </x:c>
+      <x:c r="Q26" s="36" t="str">
+        <x:v>3rd Place</x:v>
+      </x:c>
+      <x:c r="R26" s="36"/>
+      <x:c r="S26" s="37" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="T26" s="38" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="U26" s="37"/>
+      <x:c r="V26" s="38"/>
+      <x:c r="W26" s="38"/>
+      <x:c r="X26" s="37"/>
+      <x:c r="Y26" s="38"/>
+      <x:c r="Z26" s="36"/>
+      <x:c r="AA26" s="36"/>
+      <x:c r="AB26" s="39"/>
+      <x:c r="AC26" s="40"/>
+      <x:c r="AD26" s="36"/>
+      <x:c r="AE26" s="38" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AF26" s="38" t="str">
+        <x:v>Explicit cash</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -4637,6 +5247,22 @@
       <x:c r="P27" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q27" s="36"/>
+      <x:c r="R27" s="36"/>
+      <x:c r="S27" s="37"/>
+      <x:c r="T27" s="38"/>
+      <x:c r="U27" s="37"/>
+      <x:c r="V27" s="38"/>
+      <x:c r="W27" s="38"/>
+      <x:c r="X27" s="37"/>
+      <x:c r="Y27" s="38"/>
+      <x:c r="Z27" s="36"/>
+      <x:c r="AA27" s="36"/>
+      <x:c r="AB27" s="39"/>
+      <x:c r="AC27" s="40"/>
+      <x:c r="AD27" s="36"/>
+      <x:c r="AE27" s="38"/>
+      <x:c r="AF27" s="38"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28">
@@ -4687,6 +5313,22 @@
       <x:c r="P28" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q28" s="36"/>
+      <x:c r="R28" s="36"/>
+      <x:c r="S28" s="37"/>
+      <x:c r="T28" s="38"/>
+      <x:c r="U28" s="37"/>
+      <x:c r="V28" s="38"/>
+      <x:c r="W28" s="38"/>
+      <x:c r="X28" s="37"/>
+      <x:c r="Y28" s="38"/>
+      <x:c r="Z28" s="36"/>
+      <x:c r="AA28" s="36"/>
+      <x:c r="AB28" s="39"/>
+      <x:c r="AC28" s="40"/>
+      <x:c r="AD28" s="36"/>
+      <x:c r="AE28" s="38"/>
+      <x:c r="AF28" s="38"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29">
@@ -4737,6 +5379,22 @@
       <x:c r="P29" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q29" s="36"/>
+      <x:c r="R29" s="36"/>
+      <x:c r="S29" s="37"/>
+      <x:c r="T29" s="38"/>
+      <x:c r="U29" s="37"/>
+      <x:c r="V29" s="38"/>
+      <x:c r="W29" s="38"/>
+      <x:c r="X29" s="37"/>
+      <x:c r="Y29" s="38"/>
+      <x:c r="Z29" s="36"/>
+      <x:c r="AA29" s="36"/>
+      <x:c r="AB29" s="39"/>
+      <x:c r="AC29" s="40"/>
+      <x:c r="AD29" s="36"/>
+      <x:c r="AE29" s="38"/>
+      <x:c r="AF29" s="38"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30">
@@ -4787,6 +5445,22 @@
       <x:c r="P30" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q30" s="36"/>
+      <x:c r="R30" s="36"/>
+      <x:c r="S30" s="37"/>
+      <x:c r="T30" s="38"/>
+      <x:c r="U30" s="37"/>
+      <x:c r="V30" s="38"/>
+      <x:c r="W30" s="38"/>
+      <x:c r="X30" s="37"/>
+      <x:c r="Y30" s="38"/>
+      <x:c r="Z30" s="36"/>
+      <x:c r="AA30" s="36"/>
+      <x:c r="AB30" s="39"/>
+      <x:c r="AC30" s="40"/>
+      <x:c r="AD30" s="36"/>
+      <x:c r="AE30" s="38"/>
+      <x:c r="AF30" s="38"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31">
@@ -4837,6 +5511,22 @@
       <x:c r="P31" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q31" s="36"/>
+      <x:c r="R31" s="36"/>
+      <x:c r="S31" s="37"/>
+      <x:c r="T31" s="38"/>
+      <x:c r="U31" s="37"/>
+      <x:c r="V31" s="38"/>
+      <x:c r="W31" s="38"/>
+      <x:c r="X31" s="37"/>
+      <x:c r="Y31" s="38"/>
+      <x:c r="Z31" s="36"/>
+      <x:c r="AA31" s="36"/>
+      <x:c r="AB31" s="39"/>
+      <x:c r="AC31" s="40"/>
+      <x:c r="AD31" s="36"/>
+      <x:c r="AE31" s="38"/>
+      <x:c r="AF31" s="38"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32">
@@ -4887,6 +5577,22 @@
       <x:c r="P32" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q32" s="36"/>
+      <x:c r="R32" s="36"/>
+      <x:c r="S32" s="37"/>
+      <x:c r="T32" s="38"/>
+      <x:c r="U32" s="37"/>
+      <x:c r="V32" s="38"/>
+      <x:c r="W32" s="38"/>
+      <x:c r="X32" s="37"/>
+      <x:c r="Y32" s="38"/>
+      <x:c r="Z32" s="36"/>
+      <x:c r="AA32" s="36"/>
+      <x:c r="AB32" s="39"/>
+      <x:c r="AC32" s="40"/>
+      <x:c r="AD32" s="36"/>
+      <x:c r="AE32" s="38"/>
+      <x:c r="AF32" s="38"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33">
@@ -4935,6 +5641,22 @@
       <x:c r="P33" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q33" s="36"/>
+      <x:c r="R33" s="36"/>
+      <x:c r="S33" s="37"/>
+      <x:c r="T33" s="38"/>
+      <x:c r="U33" s="37"/>
+      <x:c r="V33" s="38"/>
+      <x:c r="W33" s="38"/>
+      <x:c r="X33" s="37"/>
+      <x:c r="Y33" s="38"/>
+      <x:c r="Z33" s="36"/>
+      <x:c r="AA33" s="36"/>
+      <x:c r="AB33" s="39"/>
+      <x:c r="AC33" s="40"/>
+      <x:c r="AD33" s="36"/>
+      <x:c r="AE33" s="38"/>
+      <x:c r="AF33" s="38"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34">
@@ -4985,6 +5707,32 @@
       <x:c r="P34" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q34" s="36" t="str">
+        <x:v>3rd Prize</x:v>
+      </x:c>
+      <x:c r="R34" s="36"/>
+      <x:c r="S34" s="37" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="T34" s="38" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="U34" s="37"/>
+      <x:c r="V34" s="38"/>
+      <x:c r="W34" s="38"/>
+      <x:c r="X34" s="37"/>
+      <x:c r="Y34" s="38"/>
+      <x:c r="Z34" s="36"/>
+      <x:c r="AA34" s="36"/>
+      <x:c r="AB34" s="39"/>
+      <x:c r="AC34" s="40"/>
+      <x:c r="AD34" s="36"/>
+      <x:c r="AE34" s="38" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AF34" s="38" t="str">
+        <x:v>Confirmed cash</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35">
@@ -5035,6 +5783,22 @@
       <x:c r="P35" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q35" s="36"/>
+      <x:c r="R35" s="36"/>
+      <x:c r="S35" s="37"/>
+      <x:c r="T35" s="38"/>
+      <x:c r="U35" s="37"/>
+      <x:c r="V35" s="38"/>
+      <x:c r="W35" s="38"/>
+      <x:c r="X35" s="37"/>
+      <x:c r="Y35" s="38"/>
+      <x:c r="Z35" s="36"/>
+      <x:c r="AA35" s="36"/>
+      <x:c r="AB35" s="39"/>
+      <x:c r="AC35" s="40"/>
+      <x:c r="AD35" s="36"/>
+      <x:c r="AE35" s="38"/>
+      <x:c r="AF35" s="38"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36">
@@ -5085,6 +5849,32 @@
       <x:c r="P36" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q36" s="36" t="str">
+        <x:v>2nd Prize</x:v>
+      </x:c>
+      <x:c r="R36" s="36"/>
+      <x:c r="S36" s="37" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="T36" s="38" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="U36" s="37"/>
+      <x:c r="V36" s="38"/>
+      <x:c r="W36" s="38"/>
+      <x:c r="X36" s="37"/>
+      <x:c r="Y36" s="38"/>
+      <x:c r="Z36" s="36"/>
+      <x:c r="AA36" s="36"/>
+      <x:c r="AB36" s="39"/>
+      <x:c r="AC36" s="40"/>
+      <x:c r="AD36" s="36"/>
+      <x:c r="AE36" s="38" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AF36" s="38" t="str">
+        <x:v>Confirmed cash</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37">
@@ -5135,6 +5925,22 @@
       <x:c r="P37" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q37" s="36"/>
+      <x:c r="R37" s="36"/>
+      <x:c r="S37" s="37"/>
+      <x:c r="T37" s="38"/>
+      <x:c r="U37" s="37"/>
+      <x:c r="V37" s="38"/>
+      <x:c r="W37" s="38"/>
+      <x:c r="X37" s="37"/>
+      <x:c r="Y37" s="38"/>
+      <x:c r="Z37" s="36"/>
+      <x:c r="AA37" s="36"/>
+      <x:c r="AB37" s="39"/>
+      <x:c r="AC37" s="40"/>
+      <x:c r="AD37" s="36"/>
+      <x:c r="AE37" s="38"/>
+      <x:c r="AF37" s="38"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38">
@@ -5185,6 +5991,22 @@
       <x:c r="P38" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q38" s="36"/>
+      <x:c r="R38" s="36"/>
+      <x:c r="S38" s="37"/>
+      <x:c r="T38" s="38"/>
+      <x:c r="U38" s="37"/>
+      <x:c r="V38" s="38"/>
+      <x:c r="W38" s="38"/>
+      <x:c r="X38" s="37"/>
+      <x:c r="Y38" s="38"/>
+      <x:c r="Z38" s="36"/>
+      <x:c r="AA38" s="36"/>
+      <x:c r="AB38" s="39"/>
+      <x:c r="AC38" s="40"/>
+      <x:c r="AD38" s="36"/>
+      <x:c r="AE38" s="38"/>
+      <x:c r="AF38" s="38"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39">
@@ -5235,6 +6057,36 @@
       <x:c r="P39" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q39" s="36" t="str">
+        <x:v>2nd Prize</x:v>
+      </x:c>
+      <x:c r="R39" s="36"/>
+      <x:c r="S39" s="37"/>
+      <x:c r="T39" s="38"/>
+      <x:c r="U39" s="37"/>
+      <x:c r="V39" s="38"/>
+      <x:c r="W39" s="38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X39" s="37" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="Y39" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="Z39" s="36" t="str">
+        <x:v>Manus Pro subscription</x:v>
+      </x:c>
+      <x:c r="AA39" s="36"/>
+      <x:c r="AB39" s="39"/>
+      <x:c r="AC39" s="40"/>
+      <x:c r="AD39" s="36"/>
+      <x:c r="AE39" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF39" s="38" t="str">
+        <x:v>US$39 monthly value at award period</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40">
@@ -5285,6 +6137,22 @@
       <x:c r="P40" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q40" s="36"/>
+      <x:c r="R40" s="36"/>
+      <x:c r="S40" s="37"/>
+      <x:c r="T40" s="38"/>
+      <x:c r="U40" s="37"/>
+      <x:c r="V40" s="38"/>
+      <x:c r="W40" s="38"/>
+      <x:c r="X40" s="37"/>
+      <x:c r="Y40" s="38"/>
+      <x:c r="Z40" s="36"/>
+      <x:c r="AA40" s="36"/>
+      <x:c r="AB40" s="39"/>
+      <x:c r="AC40" s="40"/>
+      <x:c r="AD40" s="36"/>
+      <x:c r="AE40" s="38"/>
+      <x:c r="AF40" s="38"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41">
@@ -5332,6 +6200,36 @@
       <x:c r="P41" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q41" s="36" t="str">
+        <x:v>Best Finisher</x:v>
+      </x:c>
+      <x:c r="R41" s="36" t="str">
+        <x:v>Novel Hackathon</x:v>
+      </x:c>
+      <x:c r="S41" s="37"/>
+      <x:c r="T41" s="38"/>
+      <x:c r="U41" s="37"/>
+      <x:c r="V41" s="38"/>
+      <x:c r="W41" s="38"/>
+      <x:c r="X41" s="37"/>
+      <x:c r="Y41" s="38"/>
+      <x:c r="Z41" s="36" t="str">
+        <x:v>Trophy</x:v>
+      </x:c>
+      <x:c r="AA41" s="36" t="str">
+        <x:v>Trophy</x:v>
+      </x:c>
+      <x:c r="AB41" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC41" s="40"/>
+      <x:c r="AD41" s="36"/>
+      <x:c r="AE41" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF41" s="38" t="str">
+        <x:v>Trophy, not cash</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42">
@@ -5379,6 +6277,22 @@
       <x:c r="P42" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q42" s="36"/>
+      <x:c r="R42" s="36"/>
+      <x:c r="S42" s="37"/>
+      <x:c r="T42" s="38"/>
+      <x:c r="U42" s="37"/>
+      <x:c r="V42" s="38"/>
+      <x:c r="W42" s="38"/>
+      <x:c r="X42" s="37"/>
+      <x:c r="Y42" s="38"/>
+      <x:c r="Z42" s="36"/>
+      <x:c r="AA42" s="36"/>
+      <x:c r="AB42" s="39"/>
+      <x:c r="AC42" s="40"/>
+      <x:c r="AD42" s="36"/>
+      <x:c r="AE42" s="38"/>
+      <x:c r="AF42" s="38"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43">
@@ -5429,6 +6343,34 @@
       <x:c r="P43" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q43" s="36" t="str">
+        <x:v>1st Prize</x:v>
+      </x:c>
+      <x:c r="R43" s="36"/>
+      <x:c r="S43" s="37"/>
+      <x:c r="T43" s="38"/>
+      <x:c r="U43" s="37" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="V43" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="W43" s="38"/>
+      <x:c r="X43" s="37"/>
+      <x:c r="Y43" s="38"/>
+      <x:c r="Z43" s="36" t="str">
+        <x:v>Nosana Cloud credit</x:v>
+      </x:c>
+      <x:c r="AA43" s="36"/>
+      <x:c r="AB43" s="39"/>
+      <x:c r="AC43" s="40"/>
+      <x:c r="AD43" s="36"/>
+      <x:c r="AE43" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF43" s="38" t="str">
+        <x:v>Cloud credit, not cash</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44">
@@ -5479,6 +6421,22 @@
       <x:c r="P44" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q44" s="36"/>
+      <x:c r="R44" s="36"/>
+      <x:c r="S44" s="37"/>
+      <x:c r="T44" s="38"/>
+      <x:c r="U44" s="37"/>
+      <x:c r="V44" s="38"/>
+      <x:c r="W44" s="38"/>
+      <x:c r="X44" s="37"/>
+      <x:c r="Y44" s="38"/>
+      <x:c r="Z44" s="36"/>
+      <x:c r="AA44" s="36"/>
+      <x:c r="AB44" s="39"/>
+      <x:c r="AC44" s="40"/>
+      <x:c r="AD44" s="36"/>
+      <x:c r="AE44" s="38"/>
+      <x:c r="AF44" s="38"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45">
@@ -5529,6 +6487,22 @@
       <x:c r="P45" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q45" s="36"/>
+      <x:c r="R45" s="36"/>
+      <x:c r="S45" s="37"/>
+      <x:c r="T45" s="38"/>
+      <x:c r="U45" s="37"/>
+      <x:c r="V45" s="38"/>
+      <x:c r="W45" s="38"/>
+      <x:c r="X45" s="37"/>
+      <x:c r="Y45" s="38"/>
+      <x:c r="Z45" s="36"/>
+      <x:c r="AA45" s="36"/>
+      <x:c r="AB45" s="39"/>
+      <x:c r="AC45" s="40"/>
+      <x:c r="AD45" s="36"/>
+      <x:c r="AE45" s="38"/>
+      <x:c r="AF45" s="38"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46">
@@ -5579,6 +6553,22 @@
       <x:c r="P46" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q46" s="36"/>
+      <x:c r="R46" s="36"/>
+      <x:c r="S46" s="37"/>
+      <x:c r="T46" s="38"/>
+      <x:c r="U46" s="37"/>
+      <x:c r="V46" s="38"/>
+      <x:c r="W46" s="38"/>
+      <x:c r="X46" s="37"/>
+      <x:c r="Y46" s="38"/>
+      <x:c r="Z46" s="36"/>
+      <x:c r="AA46" s="36"/>
+      <x:c r="AB46" s="39"/>
+      <x:c r="AC46" s="40"/>
+      <x:c r="AD46" s="36"/>
+      <x:c r="AE46" s="38"/>
+      <x:c r="AF46" s="38"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47">
@@ -5629,6 +6619,22 @@
       <x:c r="P47" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q47" s="36"/>
+      <x:c r="R47" s="36"/>
+      <x:c r="S47" s="37"/>
+      <x:c r="T47" s="38"/>
+      <x:c r="U47" s="37"/>
+      <x:c r="V47" s="38"/>
+      <x:c r="W47" s="38"/>
+      <x:c r="X47" s="37"/>
+      <x:c r="Y47" s="38"/>
+      <x:c r="Z47" s="36"/>
+      <x:c r="AA47" s="36"/>
+      <x:c r="AB47" s="39"/>
+      <x:c r="AC47" s="40"/>
+      <x:c r="AD47" s="36"/>
+      <x:c r="AE47" s="38"/>
+      <x:c r="AF47" s="38"/>
     </x:row>
     <x:row r="48" ht="49.75" customHeight="1">
       <x:c r="A48">
@@ -5679,6 +6685,22 @@
       <x:c r="P48" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q48" s="36"/>
+      <x:c r="R48" s="36"/>
+      <x:c r="S48" s="37"/>
+      <x:c r="T48" s="38"/>
+      <x:c r="U48" s="37"/>
+      <x:c r="V48" s="38"/>
+      <x:c r="W48" s="38"/>
+      <x:c r="X48" s="37"/>
+      <x:c r="Y48" s="38"/>
+      <x:c r="Z48" s="36"/>
+      <x:c r="AA48" s="36"/>
+      <x:c r="AB48" s="39"/>
+      <x:c r="AC48" s="40"/>
+      <x:c r="AD48" s="36"/>
+      <x:c r="AE48" s="38"/>
+      <x:c r="AF48" s="38"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49">
@@ -5729,6 +6751,22 @@
       <x:c r="P49" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q49" s="36"/>
+      <x:c r="R49" s="36"/>
+      <x:c r="S49" s="37"/>
+      <x:c r="T49" s="38"/>
+      <x:c r="U49" s="37"/>
+      <x:c r="V49" s="38"/>
+      <x:c r="W49" s="38"/>
+      <x:c r="X49" s="37"/>
+      <x:c r="Y49" s="38"/>
+      <x:c r="Z49" s="36"/>
+      <x:c r="AA49" s="36"/>
+      <x:c r="AB49" s="39"/>
+      <x:c r="AC49" s="40"/>
+      <x:c r="AD49" s="36"/>
+      <x:c r="AE49" s="38"/>
+      <x:c r="AF49" s="38"/>
     </x:row>
     <x:row r="50" ht="34">
       <x:c r="A50">
@@ -5779,6 +6817,22 @@
       <x:c r="P50" t="s">
         <x:v>372</x:v>
       </x:c>
+      <x:c r="Q50" s="36"/>
+      <x:c r="R50" s="36"/>
+      <x:c r="S50" s="37"/>
+      <x:c r="T50" s="38"/>
+      <x:c r="U50" s="37"/>
+      <x:c r="V50" s="38"/>
+      <x:c r="W50" s="38"/>
+      <x:c r="X50" s="37"/>
+      <x:c r="Y50" s="38"/>
+      <x:c r="Z50" s="36"/>
+      <x:c r="AA50" s="36"/>
+      <x:c r="AB50" s="39"/>
+      <x:c r="AC50" s="40"/>
+      <x:c r="AD50" s="36"/>
+      <x:c r="AE50" s="38"/>
+      <x:c r="AF50" s="38"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51">
@@ -5829,6 +6883,34 @@
       <x:c r="P51" t="s">
         <x:v>382</x:v>
       </x:c>
+      <x:c r="Q51" s="36" t="str">
+        <x:v>1st Prize</x:v>
+      </x:c>
+      <x:c r="R51" s="36"/>
+      <x:c r="S51" s="37"/>
+      <x:c r="T51" s="38"/>
+      <x:c r="U51" s="37" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="V51" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="W51" s="38"/>
+      <x:c r="X51" s="37"/>
+      <x:c r="Y51" s="38"/>
+      <x:c r="Z51" s="36" t="str">
+        <x:v>OpenRouter credits</x:v>
+      </x:c>
+      <x:c r="AA51" s="36"/>
+      <x:c r="AB51" s="39"/>
+      <x:c r="AC51" s="40"/>
+      <x:c r="AD51" s="36"/>
+      <x:c r="AE51" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF51" s="38" t="str">
+        <x:v>API credits, not cash</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52">
@@ -5879,6 +6961,22 @@
       <x:c r="P52" t="s">
         <x:v>382</x:v>
       </x:c>
+      <x:c r="Q52" s="36"/>
+      <x:c r="R52" s="36"/>
+      <x:c r="S52" s="37"/>
+      <x:c r="T52" s="38"/>
+      <x:c r="U52" s="37"/>
+      <x:c r="V52" s="38"/>
+      <x:c r="W52" s="38"/>
+      <x:c r="X52" s="37"/>
+      <x:c r="Y52" s="38"/>
+      <x:c r="Z52" s="36"/>
+      <x:c r="AA52" s="36"/>
+      <x:c r="AB52" s="39"/>
+      <x:c r="AC52" s="40"/>
+      <x:c r="AD52" s="36"/>
+      <x:c r="AE52" s="38"/>
+      <x:c r="AF52" s="38"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53">
@@ -5929,6 +7027,34 @@
       <x:c r="P53" t="s">
         <x:v>393</x:v>
       </x:c>
+      <x:c r="Q53" s="36" t="str">
+        <x:v>1st Prize</x:v>
+      </x:c>
+      <x:c r="R53" s="36"/>
+      <x:c r="S53" s="37"/>
+      <x:c r="T53" s="38"/>
+      <x:c r="U53" s="37" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="V53" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="W53" s="38"/>
+      <x:c r="X53" s="37"/>
+      <x:c r="Y53" s="38"/>
+      <x:c r="Z53" s="36" t="str">
+        <x:v>API credits</x:v>
+      </x:c>
+      <x:c r="AA53" s="36"/>
+      <x:c r="AB53" s="39"/>
+      <x:c r="AC53" s="40"/>
+      <x:c r="AD53" s="36"/>
+      <x:c r="AE53" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF53" s="38" t="str">
+        <x:v>API credits, not cash</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54">
@@ -5979,6 +7105,34 @@
       <x:c r="P54" t="s">
         <x:v>393</x:v>
       </x:c>
+      <x:c r="Q54" s="36" t="str">
+        <x:v>1st Prize</x:v>
+      </x:c>
+      <x:c r="R54" s="36"/>
+      <x:c r="S54" s="37"/>
+      <x:c r="T54" s="38"/>
+      <x:c r="U54" s="37" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="V54" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="W54" s="38"/>
+      <x:c r="X54" s="37"/>
+      <x:c r="Y54" s="38"/>
+      <x:c r="Z54" s="36" t="str">
+        <x:v>API credits</x:v>
+      </x:c>
+      <x:c r="AA54" s="36"/>
+      <x:c r="AB54" s="39"/>
+      <x:c r="AC54" s="40"/>
+      <x:c r="AD54" s="36"/>
+      <x:c r="AE54" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF54" s="38" t="str">
+        <x:v>API credits, not cash</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="34">
       <x:c r="A55">
@@ -6029,6 +7183,34 @@
       <x:c r="P55" t="s">
         <x:v>407</x:v>
       </x:c>
+      <x:c r="Q55" s="36" t="str">
+        <x:v>1st Prize</x:v>
+      </x:c>
+      <x:c r="R55" s="36"/>
+      <x:c r="S55" s="37"/>
+      <x:c r="T55" s="38"/>
+      <x:c r="U55" s="37" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="V55" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="W55" s="38"/>
+      <x:c r="X55" s="37"/>
+      <x:c r="Y55" s="38"/>
+      <x:c r="Z55" s="36" t="str">
+        <x:v>Wavespeed AI credits</x:v>
+      </x:c>
+      <x:c r="AA55" s="36"/>
+      <x:c r="AB55" s="39"/>
+      <x:c r="AC55" s="40"/>
+      <x:c r="AD55" s="36"/>
+      <x:c r="AE55" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF55" s="38" t="str">
+        <x:v>API credits, not cash</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="17">
       <x:c r="A56">
@@ -6079,6 +7261,22 @@
       <x:c r="P56" t="s">
         <x:v>413</x:v>
       </x:c>
+      <x:c r="Q56" s="36"/>
+      <x:c r="R56" s="36"/>
+      <x:c r="S56" s="37"/>
+      <x:c r="T56" s="38"/>
+      <x:c r="U56" s="37"/>
+      <x:c r="V56" s="38"/>
+      <x:c r="W56" s="38"/>
+      <x:c r="X56" s="37"/>
+      <x:c r="Y56" s="38"/>
+      <x:c r="Z56" s="36"/>
+      <x:c r="AA56" s="36"/>
+      <x:c r="AB56" s="39"/>
+      <x:c r="AC56" s="40"/>
+      <x:c r="AD56" s="36"/>
+      <x:c r="AE56" s="38"/>
+      <x:c r="AF56" s="38"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57">
@@ -6129,6 +7327,22 @@
       <x:c r="P57" t="s">
         <x:v>420</x:v>
       </x:c>
+      <x:c r="Q57" s="36"/>
+      <x:c r="R57" s="36"/>
+      <x:c r="S57" s="37"/>
+      <x:c r="T57" s="38"/>
+      <x:c r="U57" s="37"/>
+      <x:c r="V57" s="38"/>
+      <x:c r="W57" s="38"/>
+      <x:c r="X57" s="37"/>
+      <x:c r="Y57" s="38"/>
+      <x:c r="Z57" s="36"/>
+      <x:c r="AA57" s="36"/>
+      <x:c r="AB57" s="39"/>
+      <x:c r="AC57" s="40"/>
+      <x:c r="AD57" s="36"/>
+      <x:c r="AE57" s="38"/>
+      <x:c r="AF57" s="38"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58">
@@ -6179,6 +7393,38 @@
       <x:c r="P58" t="s">
         <x:v>428</x:v>
       </x:c>
+      <x:c r="Q58" s="36" t="str">
+        <x:v>3rd Prize</x:v>
+      </x:c>
+      <x:c r="R58" s="36"/>
+      <x:c r="S58" s="37" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="T58" s="38" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="U58" s="37" t="n">
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="V58" s="38" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="W58" s="38"/>
+      <x:c r="X58" s="37"/>
+      <x:c r="Y58" s="38"/>
+      <x:c r="Z58" s="36" t="str">
+        <x:v>API credits</x:v>
+      </x:c>
+      <x:c r="AA58" s="36"/>
+      <x:c r="AB58" s="39"/>
+      <x:c r="AC58" s="40"/>
+      <x:c r="AD58" s="36"/>
+      <x:c r="AE58" s="38" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AF58" s="38" t="str">
+        <x:v>Explicit cash; API credit value also tracked</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59">
@@ -6229,6 +7475,22 @@
       <x:c r="P59" t="s">
         <x:v>437</x:v>
       </x:c>
+      <x:c r="Q59" s="36"/>
+      <x:c r="R59" s="36"/>
+      <x:c r="S59" s="37"/>
+      <x:c r="T59" s="38"/>
+      <x:c r="U59" s="37"/>
+      <x:c r="V59" s="38"/>
+      <x:c r="W59" s="38"/>
+      <x:c r="X59" s="37"/>
+      <x:c r="Y59" s="38"/>
+      <x:c r="Z59" s="36"/>
+      <x:c r="AA59" s="36"/>
+      <x:c r="AB59" s="39"/>
+      <x:c r="AC59" s="40"/>
+      <x:c r="AD59" s="36"/>
+      <x:c r="AE59" s="38"/>
+      <x:c r="AF59" s="38"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60">
@@ -6279,6 +7541,22 @@
       <x:c r="P60" t="s">
         <x:v>447</x:v>
       </x:c>
+      <x:c r="Q60" s="36"/>
+      <x:c r="R60" s="36"/>
+      <x:c r="S60" s="37"/>
+      <x:c r="T60" s="38"/>
+      <x:c r="U60" s="37"/>
+      <x:c r="V60" s="38"/>
+      <x:c r="W60" s="38"/>
+      <x:c r="X60" s="37"/>
+      <x:c r="Y60" s="38"/>
+      <x:c r="Z60" s="36"/>
+      <x:c r="AA60" s="36"/>
+      <x:c r="AB60" s="39"/>
+      <x:c r="AC60" s="40"/>
+      <x:c r="AD60" s="36"/>
+      <x:c r="AE60" s="38"/>
+      <x:c r="AF60" s="38"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61">
@@ -6329,6 +7607,36 @@
       <x:c r="P61" s="1" t="s">
         <x:v>456</x:v>
       </x:c>
+      <x:c r="Q61" s="36" t="str">
+        <x:v>Award</x:v>
+      </x:c>
+      <x:c r="R61" s="36" t="str">
+        <x:v>Speechmatics</x:v>
+      </x:c>
+      <x:c r="S61" s="37"/>
+      <x:c r="T61" s="38"/>
+      <x:c r="U61" s="37" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="V61" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="W61" s="38"/>
+      <x:c r="X61" s="37"/>
+      <x:c r="Y61" s="38"/>
+      <x:c r="Z61" s="36" t="str">
+        <x:v>Speechmatics credits</x:v>
+      </x:c>
+      <x:c r="AA61" s="36"/>
+      <x:c r="AB61" s="39"/>
+      <x:c r="AC61" s="40"/>
+      <x:c r="AD61" s="36"/>
+      <x:c r="AE61" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF61" s="38" t="str">
+        <x:v>USD-denominated credit value</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62">
@@ -6379,6 +7687,36 @@
       <x:c r="P62" s="1" t="s">
         <x:v>464</x:v>
       </x:c>
+      <x:c r="Q62" s="36" t="str">
+        <x:v>Award</x:v>
+      </x:c>
+      <x:c r="R62" s="36" t="str">
+        <x:v>v0</x:v>
+      </x:c>
+      <x:c r="S62" s="37"/>
+      <x:c r="T62" s="38"/>
+      <x:c r="U62" s="37"/>
+      <x:c r="V62" s="38"/>
+      <x:c r="W62" s="38"/>
+      <x:c r="X62" s="37"/>
+      <x:c r="Y62" s="38"/>
+      <x:c r="Z62" s="36" t="str">
+        <x:v>v0 Sock</x:v>
+      </x:c>
+      <x:c r="AA62" s="36" t="str">
+        <x:v>v0 Sock</x:v>
+      </x:c>
+      <x:c r="AB62" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AC62" s="40"/>
+      <x:c r="AD62" s="36"/>
+      <x:c r="AE62" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF62" s="38" t="str">
+        <x:v>Physical item, not cash</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63">
@@ -6429,6 +7767,22 @@
       <x:c r="P63" t="s">
         <x:v>472</x:v>
       </x:c>
+      <x:c r="Q63" s="36"/>
+      <x:c r="R63" s="36"/>
+      <x:c r="S63" s="37"/>
+      <x:c r="T63" s="38"/>
+      <x:c r="U63" s="37"/>
+      <x:c r="V63" s="38"/>
+      <x:c r="W63" s="38"/>
+      <x:c r="X63" s="37"/>
+      <x:c r="Y63" s="38"/>
+      <x:c r="Z63" s="36"/>
+      <x:c r="AA63" s="36"/>
+      <x:c r="AB63" s="39"/>
+      <x:c r="AC63" s="40"/>
+      <x:c r="AD63" s="36"/>
+      <x:c r="AE63" s="38"/>
+      <x:c r="AF63" s="38"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64">
@@ -6479,6 +7833,22 @@
       <x:c r="P64" t="s">
         <x:v>477</x:v>
       </x:c>
+      <x:c r="Q64" s="36"/>
+      <x:c r="R64" s="36"/>
+      <x:c r="S64" s="37"/>
+      <x:c r="T64" s="38"/>
+      <x:c r="U64" s="37"/>
+      <x:c r="V64" s="38"/>
+      <x:c r="W64" s="38"/>
+      <x:c r="X64" s="37"/>
+      <x:c r="Y64" s="38"/>
+      <x:c r="Z64" s="36"/>
+      <x:c r="AA64" s="36"/>
+      <x:c r="AB64" s="39"/>
+      <x:c r="AC64" s="40"/>
+      <x:c r="AD64" s="36"/>
+      <x:c r="AE64" s="38"/>
+      <x:c r="AF64" s="38"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65">
@@ -6529,6 +7899,22 @@
       <x:c r="P65" t="s">
         <x:v>484</x:v>
       </x:c>
+      <x:c r="Q65" s="36"/>
+      <x:c r="R65" s="36"/>
+      <x:c r="S65" s="37"/>
+      <x:c r="T65" s="38"/>
+      <x:c r="U65" s="37"/>
+      <x:c r="V65" s="38"/>
+      <x:c r="W65" s="38"/>
+      <x:c r="X65" s="37"/>
+      <x:c r="Y65" s="38"/>
+      <x:c r="Z65" s="36"/>
+      <x:c r="AA65" s="36"/>
+      <x:c r="AB65" s="39"/>
+      <x:c r="AC65" s="40"/>
+      <x:c r="AD65" s="36"/>
+      <x:c r="AE65" s="38"/>
+      <x:c r="AF65" s="38"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66">
@@ -6579,6 +7965,22 @@
       <x:c r="P66" t="s">
         <x:v>492</x:v>
       </x:c>
+      <x:c r="Q66" s="36"/>
+      <x:c r="R66" s="36"/>
+      <x:c r="S66" s="37"/>
+      <x:c r="T66" s="38"/>
+      <x:c r="U66" s="37"/>
+      <x:c r="V66" s="38"/>
+      <x:c r="W66" s="38"/>
+      <x:c r="X66" s="37"/>
+      <x:c r="Y66" s="38"/>
+      <x:c r="Z66" s="36"/>
+      <x:c r="AA66" s="36"/>
+      <x:c r="AB66" s="39"/>
+      <x:c r="AC66" s="40"/>
+      <x:c r="AD66" s="36"/>
+      <x:c r="AE66" s="38"/>
+      <x:c r="AF66" s="38"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67">
@@ -6629,6 +8031,34 @@
       <x:c r="P67" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q67" s="36" t="str">
+        <x:v>Top 20</x:v>
+      </x:c>
+      <x:c r="R67" s="36"/>
+      <x:c r="S67" s="37"/>
+      <x:c r="T67" s="38"/>
+      <x:c r="U67" s="37" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="V67" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="W67" s="38"/>
+      <x:c r="X67" s="37"/>
+      <x:c r="Y67" s="38"/>
+      <x:c r="Z67" s="36" t="str">
+        <x:v>10K OpenAI credits; 2K Gemini Cloud credits</x:v>
+      </x:c>
+      <x:c r="AA67" s="36"/>
+      <x:c r="AB67" s="39"/>
+      <x:c r="AC67" s="40"/>
+      <x:c r="AD67" s="36"/>
+      <x:c r="AE67" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF67" s="38" t="str">
+        <x:v>Credit value total combines two USD-denominated credits</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68">
@@ -6679,6 +8109,22 @@
       <x:c r="P68" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q68" s="36"/>
+      <x:c r="R68" s="36"/>
+      <x:c r="S68" s="37"/>
+      <x:c r="T68" s="38"/>
+      <x:c r="U68" s="37"/>
+      <x:c r="V68" s="38"/>
+      <x:c r="W68" s="38"/>
+      <x:c r="X68" s="37"/>
+      <x:c r="Y68" s="38"/>
+      <x:c r="Z68" s="36"/>
+      <x:c r="AA68" s="36"/>
+      <x:c r="AB68" s="39"/>
+      <x:c r="AC68" s="40"/>
+      <x:c r="AD68" s="36"/>
+      <x:c r="AE68" s="38"/>
+      <x:c r="AF68" s="38"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69">
@@ -6729,6 +8175,22 @@
       <x:c r="P69" t="s">
         <x:v>511</x:v>
       </x:c>
+      <x:c r="Q69" s="36"/>
+      <x:c r="R69" s="36"/>
+      <x:c r="S69" s="37"/>
+      <x:c r="T69" s="38"/>
+      <x:c r="U69" s="37"/>
+      <x:c r="V69" s="38"/>
+      <x:c r="W69" s="38"/>
+      <x:c r="X69" s="37"/>
+      <x:c r="Y69" s="38"/>
+      <x:c r="Z69" s="36"/>
+      <x:c r="AA69" s="36"/>
+      <x:c r="AB69" s="39"/>
+      <x:c r="AC69" s="40"/>
+      <x:c r="AD69" s="36"/>
+      <x:c r="AE69" s="38"/>
+      <x:c r="AF69" s="38"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70">
@@ -6776,6 +8238,22 @@
       <x:c r="P70" t="s">
         <x:v>521</x:v>
       </x:c>
+      <x:c r="Q70" s="36"/>
+      <x:c r="R70" s="36"/>
+      <x:c r="S70" s="37"/>
+      <x:c r="T70" s="38"/>
+      <x:c r="U70" s="37"/>
+      <x:c r="V70" s="38"/>
+      <x:c r="W70" s="38"/>
+      <x:c r="X70" s="37"/>
+      <x:c r="Y70" s="38"/>
+      <x:c r="Z70" s="36"/>
+      <x:c r="AA70" s="36"/>
+      <x:c r="AB70" s="39"/>
+      <x:c r="AC70" s="40"/>
+      <x:c r="AD70" s="36"/>
+      <x:c r="AE70" s="38"/>
+      <x:c r="AF70" s="38"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71">
@@ -6826,6 +8304,22 @@
       <x:c r="P71" t="s">
         <x:v>528</x:v>
       </x:c>
+      <x:c r="Q71" s="36"/>
+      <x:c r="R71" s="36"/>
+      <x:c r="S71" s="37"/>
+      <x:c r="T71" s="38"/>
+      <x:c r="U71" s="37"/>
+      <x:c r="V71" s="38"/>
+      <x:c r="W71" s="38"/>
+      <x:c r="X71" s="37"/>
+      <x:c r="Y71" s="38"/>
+      <x:c r="Z71" s="36"/>
+      <x:c r="AA71" s="36"/>
+      <x:c r="AB71" s="39"/>
+      <x:c r="AC71" s="40"/>
+      <x:c r="AD71" s="36"/>
+      <x:c r="AE71" s="38"/>
+      <x:c r="AF71" s="38"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72">
@@ -6876,6 +8370,36 @@
       <x:c r="P72" t="s">
         <x:v>534</x:v>
       </x:c>
+      <x:c r="Q72" s="36" t="str">
+        <x:v>Award</x:v>
+      </x:c>
+      <x:c r="R72" s="36" t="str">
+        <x:v>AWS</x:v>
+      </x:c>
+      <x:c r="S72" s="37"/>
+      <x:c r="T72" s="38"/>
+      <x:c r="U72" s="37" t="n">
+        <x:v>4500</x:v>
+      </x:c>
+      <x:c r="V72" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="W72" s="38"/>
+      <x:c r="X72" s="37"/>
+      <x:c r="Y72" s="38"/>
+      <x:c r="Z72" s="36" t="str">
+        <x:v>AWS credits</x:v>
+      </x:c>
+      <x:c r="AA72" s="36"/>
+      <x:c r="AB72" s="39"/>
+      <x:c r="AC72" s="40"/>
+      <x:c r="AD72" s="36"/>
+      <x:c r="AE72" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF72" s="38" t="str">
+        <x:v>USD-denominated credit value</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73">
@@ -6926,6 +8450,22 @@
       <x:c r="P73" t="s">
         <x:v>542</x:v>
       </x:c>
+      <x:c r="Q73" s="36"/>
+      <x:c r="R73" s="36"/>
+      <x:c r="S73" s="37"/>
+      <x:c r="T73" s="38"/>
+      <x:c r="U73" s="37"/>
+      <x:c r="V73" s="38"/>
+      <x:c r="W73" s="38"/>
+      <x:c r="X73" s="37"/>
+      <x:c r="Y73" s="38"/>
+      <x:c r="Z73" s="36"/>
+      <x:c r="AA73" s="36"/>
+      <x:c r="AB73" s="39"/>
+      <x:c r="AC73" s="40"/>
+      <x:c r="AD73" s="36"/>
+      <x:c r="AE73" s="38"/>
+      <x:c r="AF73" s="38"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74">
@@ -6976,6 +8516,22 @@
       <x:c r="P74" t="s">
         <x:v>521</x:v>
       </x:c>
+      <x:c r="Q74" s="36"/>
+      <x:c r="R74" s="36"/>
+      <x:c r="S74" s="37"/>
+      <x:c r="T74" s="38"/>
+      <x:c r="U74" s="37"/>
+      <x:c r="V74" s="38"/>
+      <x:c r="W74" s="38"/>
+      <x:c r="X74" s="37"/>
+      <x:c r="Y74" s="38"/>
+      <x:c r="Z74" s="36"/>
+      <x:c r="AA74" s="36"/>
+      <x:c r="AB74" s="39"/>
+      <x:c r="AC74" s="40"/>
+      <x:c r="AD74" s="36"/>
+      <x:c r="AE74" s="38"/>
+      <x:c r="AF74" s="38"/>
     </x:row>
     <x:row r="75" ht="34">
       <x:c r="A75">
@@ -7026,6 +8582,22 @@
       <x:c r="P75" s="12" t="s">
         <x:v>25</x:v>
       </x:c>
+      <x:c r="Q75" s="36"/>
+      <x:c r="R75" s="36"/>
+      <x:c r="S75" s="37"/>
+      <x:c r="T75" s="38"/>
+      <x:c r="U75" s="37"/>
+      <x:c r="V75" s="38"/>
+      <x:c r="W75" s="38"/>
+      <x:c r="X75" s="37"/>
+      <x:c r="Y75" s="38"/>
+      <x:c r="Z75" s="36"/>
+      <x:c r="AA75" s="36"/>
+      <x:c r="AB75" s="39"/>
+      <x:c r="AC75" s="40"/>
+      <x:c r="AD75" s="36"/>
+      <x:c r="AE75" s="38"/>
+      <x:c r="AF75" s="38"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76">
@@ -7076,6 +8648,36 @@
       <x:c r="P76" t="s">
         <x:v>563</x:v>
       </x:c>
+      <x:c r="Q76" s="36" t="str">
+        <x:v>Best Vertical Solution</x:v>
+      </x:c>
+      <x:c r="R76" s="36" t="str">
+        <x:v>Family Office Track</x:v>
+      </x:c>
+      <x:c r="S76" s="37"/>
+      <x:c r="T76" s="38"/>
+      <x:c r="U76" s="37" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="V76" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="W76" s="38"/>
+      <x:c r="X76" s="37"/>
+      <x:c r="Y76" s="38"/>
+      <x:c r="Z76" s="36" t="str">
+        <x:v>2,000 Cybrdeck API credits</x:v>
+      </x:c>
+      <x:c r="AA76" s="36"/>
+      <x:c r="AB76" s="39"/>
+      <x:c r="AC76" s="40"/>
+      <x:c r="AD76" s="36"/>
+      <x:c r="AE76" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF76" s="38" t="str">
+        <x:v>US$25 credit value, not cash</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77">
@@ -7126,6 +8728,22 @@
       <x:c r="P77" t="s">
         <x:v>573</x:v>
       </x:c>
+      <x:c r="Q77" s="36"/>
+      <x:c r="R77" s="36"/>
+      <x:c r="S77" s="37"/>
+      <x:c r="T77" s="38"/>
+      <x:c r="U77" s="37"/>
+      <x:c r="V77" s="38"/>
+      <x:c r="W77" s="38"/>
+      <x:c r="X77" s="37"/>
+      <x:c r="Y77" s="38"/>
+      <x:c r="Z77" s="36"/>
+      <x:c r="AA77" s="36"/>
+      <x:c r="AB77" s="39"/>
+      <x:c r="AC77" s="40"/>
+      <x:c r="AD77" s="36"/>
+      <x:c r="AE77" s="38"/>
+      <x:c r="AF77" s="38"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78">
@@ -7176,6 +8794,22 @@
       <x:c r="P78" t="s">
         <x:v>521</x:v>
       </x:c>
+      <x:c r="Q78" s="36"/>
+      <x:c r="R78" s="36"/>
+      <x:c r="S78" s="37"/>
+      <x:c r="T78" s="38"/>
+      <x:c r="U78" s="37"/>
+      <x:c r="V78" s="38"/>
+      <x:c r="W78" s="38"/>
+      <x:c r="X78" s="37"/>
+      <x:c r="Y78" s="38"/>
+      <x:c r="Z78" s="36"/>
+      <x:c r="AA78" s="36"/>
+      <x:c r="AB78" s="39"/>
+      <x:c r="AC78" s="40"/>
+      <x:c r="AD78" s="36"/>
+      <x:c r="AE78" s="38"/>
+      <x:c r="AF78" s="38"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79">
@@ -7226,6 +8860,22 @@
       <x:c r="P79" t="s">
         <x:v>589</x:v>
       </x:c>
+      <x:c r="Q79" s="36"/>
+      <x:c r="R79" s="36"/>
+      <x:c r="S79" s="37"/>
+      <x:c r="T79" s="38"/>
+      <x:c r="U79" s="37"/>
+      <x:c r="V79" s="38"/>
+      <x:c r="W79" s="38"/>
+      <x:c r="X79" s="37"/>
+      <x:c r="Y79" s="38"/>
+      <x:c r="Z79" s="36"/>
+      <x:c r="AA79" s="36"/>
+      <x:c r="AB79" s="39"/>
+      <x:c r="AC79" s="40"/>
+      <x:c r="AD79" s="36"/>
+      <x:c r="AE79" s="38"/>
+      <x:c r="AF79" s="38"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" t="n">
@@ -7276,6 +8926,40 @@
       <x:c r="P80" t="str">
         <x:v>https://luma.com/n0zkb5w0?tk=OBDQgW</x:v>
       </x:c>
+      <x:c r="Q80" s="36" t="str">
+        <x:v>First Runner Up</x:v>
+      </x:c>
+      <x:c r="R80" s="36" t="str">
+        <x:v>SG × Sarawak AI &amp; Design Hackathon 2026</x:v>
+      </x:c>
+      <x:c r="S80" s="37"/>
+      <x:c r="T80" s="38"/>
+      <x:c r="U80" s="37" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="V80" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="W80" s="38"/>
+      <x:c r="X80" s="37"/>
+      <x:c r="Y80" s="38"/>
+      <x:c r="Z80" s="36" t="str">
+        <x:v>Trophy; Kimi AI credits</x:v>
+      </x:c>
+      <x:c r="AA80" s="36" t="str">
+        <x:v>Trophy</x:v>
+      </x:c>
+      <x:c r="AB80" s="39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC80" s="40"/>
+      <x:c r="AD80" s="36"/>
+      <x:c r="AE80" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF80" s="38" t="str">
+        <x:v>Trophy excluded; credit value tracked</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" t="n">
@@ -7326,6 +9010,36 @@
       <x:c r="P81" t="str">
         <x:v>https://luma.com/fdzbrq5b?tk=QX3FM2</x:v>
       </x:c>
+      <x:c r="Q81" s="36" t="str">
+        <x:v>Best Project</x:v>
+      </x:c>
+      <x:c r="R81" s="36" t="str">
+        <x:v>Best Use of GPT-Image-2.5</x:v>
+      </x:c>
+      <x:c r="S81" s="37"/>
+      <x:c r="T81" s="38"/>
+      <x:c r="U81" s="37" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="V81" s="38" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="W81" s="38"/>
+      <x:c r="X81" s="37"/>
+      <x:c r="Y81" s="38"/>
+      <x:c r="Z81" s="36" t="str">
+        <x:v>OpenAI credits</x:v>
+      </x:c>
+      <x:c r="AA81" s="36"/>
+      <x:c r="AB81" s="39"/>
+      <x:c r="AC81" s="40"/>
+      <x:c r="AD81" s="36"/>
+      <x:c r="AE81" s="38" t="str">
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="AF81" s="38" t="str">
+        <x:v>Credit value tracked</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" t="n">
@@ -7374,13 +9088,29 @@
       <x:c r="P82" t="str">
         <x:v>https://scoga-anti-drug-jam-2026.ai.studio/</x:v>
       </x:c>
+      <x:c r="Q82" s="36"/>
+      <x:c r="R82" s="36"/>
+      <x:c r="S82" s="37"/>
+      <x:c r="T82" s="38"/>
+      <x:c r="U82" s="37"/>
+      <x:c r="V82" s="38"/>
+      <x:c r="W82" s="38"/>
+      <x:c r="X82" s="37"/>
+      <x:c r="Y82" s="38"/>
+      <x:c r="Z82" s="36"/>
+      <x:c r="AA82" s="36"/>
+      <x:c r="AB82" s="39"/>
+      <x:c r="AC82" s="40"/>
+      <x:c r="AD82" s="36"/>
+      <x:c r="AE82" s="38"/>
+      <x:c r="AF82" s="38"/>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rc82893236a504cfa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R7f411480a2ab42da"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rc056577566604ab8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R8a216ef6d3594186"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rabf5a30d1dba4716"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R0f1b817abebf40c3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R5a2d36ecfc3a4c62"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Ra34aeeec271242ae"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -8958,12 +10688,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R7c5259e1379d4be3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R4f3f5084b4da43ea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R92cd4ed292bc47f9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R2a78e24d55824340"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ec03a4b0dc6493a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R873a12a4a2e14e86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9866,7 +11596,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9199a1932c8f4037"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6abdeb321ee6435f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add dynamic prize money dashboard
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R4e84b1532c424402"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rd2dd75fc65884b43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rbebb77c9a0d749d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Rbfb085d9a3b840a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R9124416865754536"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R9a90926175a44f8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R459fc59d6e534022"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R3264dc6ec2614bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R24bf063dedfe4731"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2784,7 +2785,7 @@
     <x:numFmt numFmtId="200" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="15">
+  <x:fonts count="22">
     <x:font>
       <x:sz val="12"/>
       <x:color theme="1"/>
@@ -2868,8 +2869,49 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="20"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF5B6573"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17324D"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF5B6573"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF5B6573"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF17324D"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FF17324D"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -2904,6 +2946,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6F9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F75B5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -2975,7 +3047,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="41">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3081,6 +3153,61 @@
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="20" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="20" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Hyperlink" xfId="1"/>
@@ -9107,10 +9234,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rabf5a30d1dba4716"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R0f1b817abebf40c3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R5a2d36ecfc3a4c62"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Ra34aeeec271242ae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R9118de667af14542"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R107b73507d8849cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R8aab32c703334288"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Rd4cc065d905f4925"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -10688,12 +10815,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R92cd4ed292bc47f9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R2a78e24d55824340"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rc7906072b9014d59"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R789fc1d027354600"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R873a12a4a2e14e86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22566c629c864f5b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11596,7 +11723,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6abdeb321ee6435f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0fd6e8ae1f542aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12149,4 +12276,296 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="4" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="4" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="4" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="4" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="4" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="44" t="str">
+        <x:v>Prize Money &amp; Rewards</x:v>
+      </x:c>
+      <x:c r="B1" s="31"/>
+      <x:c r="C1" s="31"/>
+      <x:c r="D1" s="31"/>
+      <x:c r="E1" s="31"/>
+      <x:c r="F1" s="31"/>
+      <x:c r="G1" s="31"/>
+      <x:c r="H1" s="31"/>
+      <x:c r="I1" s="31"/>
+      <x:c r="J1" s="31"/>
+      <x:c r="K1" s="31"/>
+      <x:c r="L1" s="31"/>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="48" t="str">
+        <x:v>Live summary from the structured award fields on the Hackathons tab. Values refresh when you update the highlighted classification columns there.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="51" t="str">
+        <x:v>Cash-equivalent prizes</x:v>
+      </x:c>
+      <x:c r="B4" s="51"/>
+      <x:c r="C4" s="51"/>
+      <x:c r="D4" s="51"/>
+      <x:c r="E4" s="51"/>
+      <x:c r="F4" s="51"/>
+      <x:c r="H4" s="51" t="str">
+        <x:v>Credits and subscriptions</x:v>
+      </x:c>
+      <x:c r="I4" s="51"/>
+      <x:c r="J4" s="51"/>
+      <x:c r="K4" s="51"/>
+      <x:c r="L4" s="51"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="71" t="str">
+        <x:v>SGD cash + vouchers</x:v>
+      </x:c>
+      <x:c r="B5" s="71"/>
+      <x:c r="C5" s="69" t="n">
+        <x:f>SUMIFS(Hackathons!$S$2:$S$82,Hackathons!$T$2:$T$82,"SGD",Hackathons!$AE$2:$AE$82,"Yes")</x:f>
+        <x:v>2750</x:v>
+      </x:c>
+      <x:c r="D5" s="69"/>
+      <x:c r="H5" s="71" t="str">
+        <x:v>USD credits</x:v>
+      </x:c>
+      <x:c r="I5" s="71"/>
+      <x:c r="J5" s="69" t="n">
+        <x:f>SUMIFS(Hackathons!$U$2:$U$82,Hackathons!$V$2:$V$82,"USD")</x:f>
+        <x:v>126375</x:v>
+      </x:c>
+      <x:c r="K5" s="69"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="71" t="str">
+        <x:v>USD cash + vouchers</x:v>
+      </x:c>
+      <x:c r="B6" s="71"/>
+      <x:c r="C6" s="69" t="n">
+        <x:f>SUMIFS(Hackathons!$S$2:$S$82,Hackathons!$T$2:$T$82,"USD",Hackathons!$AE$2:$AE$82,"Yes")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="69"/>
+      <x:c r="H6" s="71" t="str">
+        <x:v>SGD credits</x:v>
+      </x:c>
+      <x:c r="I6" s="71"/>
+      <x:c r="J6" s="69" t="n">
+        <x:f>SUMIFS(Hackathons!$U$2:$U$82,Hackathons!$V$2:$V$82,"SGD")</x:f>
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="K6" s="69"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="71" t="str">
+        <x:v>Confirmed prize records</x:v>
+      </x:c>
+      <x:c r="B7" s="71"/>
+      <x:c r="C7" s="70" t="n">
+        <x:f>COUNTIFS(Hackathons!$S$2:$S$82,"&gt;0",Hackathons!$AE$2:$AE$82,"Yes")</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D7" s="70"/>
+      <x:c r="H7" s="71" t="str">
+        <x:v>Subscription value (USD)</x:v>
+      </x:c>
+      <x:c r="I7" s="71"/>
+      <x:c r="J7" s="69" t="n">
+        <x:f>SUMIFS(Hackathons!$X$2:$X$82,Hackathons!$Y$2:$Y$82,"USD")</x:f>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="K7" s="69"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="61" t="str">
+        <x:v>Includes vouchers you chose to treat as cash-equivalent. Funding is intentionally excluded.</x:v>
+      </x:c>
+      <x:c r="B8" s="61"/>
+      <x:c r="C8" s="61"/>
+      <x:c r="D8" s="61"/>
+      <x:c r="E8" s="61"/>
+      <x:c r="F8" s="61"/>
+      <x:c r="H8" s="71" t="str">
+        <x:v>Subscriptions collected</x:v>
+      </x:c>
+      <x:c r="I8" s="71"/>
+      <x:c r="J8" s="70" t="n">
+        <x:f>SUM(Hackathons!$W$2:$W$82)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K8" s="70"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="52" t="str">
+        <x:v>Breakdown by currency</x:v>
+      </x:c>
+      <x:c r="B10" s="52"/>
+      <x:c r="C10" s="52"/>
+      <x:c r="D10" s="52"/>
+      <x:c r="E10" s="52"/>
+      <x:c r="F10" s="52"/>
+      <x:c r="G10" s="52"/>
+      <x:c r="H10" s="52"/>
+      <x:c r="I10" s="52"/>
+      <x:c r="J10" s="52"/>
+      <x:c r="K10" s="52"/>
+      <x:c r="L10" s="52"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="63" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="B11" s="63" t="str">
+        <x:v>Currency</x:v>
+      </x:c>
+      <x:c r="C11" s="63" t="str">
+        <x:v>Amount</x:v>
+      </x:c>
+      <x:c r="D11" s="63" t="str">
+        <x:v>How it is calculated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="64" t="str">
+        <x:v>Cash-equivalent prizes</x:v>
+      </x:c>
+      <x:c r="B12" s="64" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="C12" s="67" t="n">
+        <x:f>SUMIFS(Hackathons!$S$2:$S$82,Hackathons!$T$2:$T$82,B12,Hackathons!$AE$2:$AE$82,"Yes")</x:f>
+        <x:v>2750</x:v>
+      </x:c>
+      <x:c r="D12" s="64" t="str">
+        <x:v>Cash and vouchers marked Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="64" t="str">
+        <x:v>Cash-equivalent prizes</x:v>
+      </x:c>
+      <x:c r="B13" s="64" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="C13" s="67" t="n">
+        <x:f>SUMIFS(Hackathons!$S$2:$S$82,Hackathons!$T$2:$T$82,B13,Hackathons!$AE$2:$AE$82,"Yes")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D13" s="64" t="str">
+        <x:v>Cash and vouchers marked Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="64" t="str">
+        <x:v>Credits</x:v>
+      </x:c>
+      <x:c r="B14" s="64" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="C14" s="67" t="n">
+        <x:f>SUMIFS(Hackathons!$U$2:$U$82,Hackathons!$V$2:$V$82,B14)</x:f>
+        <x:v>126375</x:v>
+      </x:c>
+      <x:c r="D14" s="64" t="str">
+        <x:v>Non-cash product / API credits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="64" t="str">
+        <x:v>Credits</x:v>
+      </x:c>
+      <x:c r="B15" s="64" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="C15" s="67" t="n">
+        <x:f>SUMIFS(Hackathons!$U$2:$U$82,Hackathons!$V$2:$V$82,B15)</x:f>
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="D15" s="64" t="str">
+        <x:v>Non-cash product / API credits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="64" t="str">
+        <x:v>Subscriptions</x:v>
+      </x:c>
+      <x:c r="B16" s="64" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="C16" s="67" t="n">
+        <x:f>SUMIFS(Hackathons!$X$2:$X$82,Hackathons!$Y$2:$Y$82,B16)</x:f>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D16" s="64" t="str">
+        <x:v>Known subscription value</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="54" t="str">
+        <x:v>How to maintain this tab</x:v>
+      </x:c>
+      <x:c r="B18" s="54"/>
+      <x:c r="C18" s="54"/>
+      <x:c r="D18" s="54"/>
+      <x:c r="E18" s="54"/>
+      <x:c r="F18" s="54"/>
+      <x:c r="G18" s="54"/>
+      <x:c r="H18" s="54"/>
+      <x:c r="I18" s="54"/>
+      <x:c r="J18" s="54"/>
+      <x:c r="K18" s="54"/>
+      <x:c r="L18" s="54"/>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="57" t="str">
+        <x:v>1. Update the yellow structured fields on Hackathons (columns S–Y and AE).  2. Use Cash-equivalent Treatment = Yes only for prizes you want counted as money.  3. Keep credit and subscription amounts in their original currencies; this dashboard deliberately does not convert currencies.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1"/>
+    <x:row r="21" ht="22" customHeight="1"/>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L2"/>
+    <x:mergeCell ref="A4:F4"/>
+    <x:mergeCell ref="H4:L4"/>
+    <x:mergeCell ref="A5:B5"/>
+    <x:mergeCell ref="C5:D5"/>
+    <x:mergeCell ref="A6:B6"/>
+    <x:mergeCell ref="C6:D6"/>
+    <x:mergeCell ref="A7:B7"/>
+    <x:mergeCell ref="C7:D7"/>
+    <x:mergeCell ref="A8:F8"/>
+    <x:mergeCell ref="H5:I5"/>
+    <x:mergeCell ref="J5:K5"/>
+    <x:mergeCell ref="H6:I6"/>
+    <x:mergeCell ref="J6:K6"/>
+    <x:mergeCell ref="H7:I7"/>
+    <x:mergeCell ref="J7:K7"/>
+    <x:mergeCell ref="H8:I8"/>
+    <x:mergeCell ref="J8:K8"/>
+    <x:mergeCell ref="A10:L10"/>
+    <x:mergeCell ref="A18:L18"/>
+    <x:mergeCell ref="A19:L21"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add linked prize detail breakdown
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R9124416865754536"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R9a90926175a44f8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R459fc59d6e534022"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R3264dc6ec2614bf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R24bf063dedfe4731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R412a67c1d73f4ddb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R7e608036e6544f79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R809ca3189425451b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Rd6fc6ff036414467"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R124a657e538a4d3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R71d217aecd414505"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2785,7 +2786,7 @@
     <x:numFmt numFmtId="200" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="22">
+  <x:fonts count="25">
     <x:font>
       <x:sz val="12"/>
       <x:color theme="1"/>
@@ -2910,8 +2911,26 @@
       <x:color rgb="FF17324D"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="18"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="18"/>
+      <x:color rgb="FF17324D"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="27">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -2983,6 +3002,66 @@
         <x:fgColor rgb="FFFFF4CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6F9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F75B5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6F9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6F9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6F9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -3047,7 +3126,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="72">
+  <x:cellXfs count="107">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3208,6 +3287,85 @@
     <x:xf numFmtId="200" fontId="20" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="20" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="21" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Hyperlink" xfId="1"/>
@@ -3264,6 +3422,34 @@
     <x:tableColumn id="4" name="Facebook"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="PrizeDetailsTable" displayName="PrizeDetailsTable" ref="A4:S29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:S29"/>
+  <x:tableColumns count="19">
+    <x:tableColumn id="1" name="#"/>
+    <x:tableColumn id="2" name="Hackathon"/>
+    <x:tableColumn id="3" name="Original award"/>
+    <x:tableColumn id="4" name="Award type"/>
+    <x:tableColumn id="5" name="Additional info"/>
+    <x:tableColumn id="6" name="Cash-equivalent amount"/>
+    <x:tableColumn id="7" name="Cash currency"/>
+    <x:tableColumn id="8" name="Credit amount"/>
+    <x:tableColumn id="9" name="Credit currency / units"/>
+    <x:tableColumn id="10" name="Subscription count"/>
+    <x:tableColumn id="11" name="Subscription amount"/>
+    <x:tableColumn id="12" name="Subscription currency"/>
+    <x:tableColumn id="13" name="Other non-cash prize"/>
+    <x:tableColumn id="14" name="Physical asset"/>
+    <x:tableColumn id="15" name="Trophy count"/>
+    <x:tableColumn id="16" name="Funding amount"/>
+    <x:tableColumn id="17" name="Funding currency"/>
+    <x:tableColumn id="18" name="Money counted?"/>
+    <x:tableColumn id="19" name="Review note"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -9234,10 +9420,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R9118de667af14542"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R107b73507d8849cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R8aab32c703334288"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Rd4cc065d905f4925"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rbbb3a3ced68d4da4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R11329dca470543b8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R9cc7cdcca01d4159"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R7959174b22c14d3e"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -10815,12 +11001,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rc7906072b9014d59"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R789fc1d027354600"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R924d8bbee39442ca"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R33eefb0e748e46f4"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22566c629c864f5b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e9fee8640894264"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11723,7 +11909,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0fd6e8ae1f542aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b0235f68dc4d45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12568,4 +12754,1828 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF17324D"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="7" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="32" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="14" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="16" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="32" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="105" t="str">
+        <x:v>Prize Money — Detailed Breakdown</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="106" t="str">
+        <x:v>One row per currently classified award or prize record. Each value is linked to the Hackathons tab, so corrections there update this detail view automatically.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="81" t="str">
+        <x:v>Records tracked</x:v>
+      </x:c>
+      <x:c r="B3" s="81"/>
+      <x:c r="C3" s="81"/>
+      <x:c r="D3" s="85" t="n">
+        <x:f>COUNTA(A5:A29)</x:f>
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E3" s="85"/>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="90" t="str">
+        <x:v>#</x:v>
+      </x:c>
+      <x:c r="B4" s="90" t="str">
+        <x:v>Hackathon</x:v>
+      </x:c>
+      <x:c r="C4" s="90" t="str">
+        <x:v>Original award</x:v>
+      </x:c>
+      <x:c r="D4" s="90" t="str">
+        <x:v>Award type</x:v>
+      </x:c>
+      <x:c r="E4" s="90" t="str">
+        <x:v>Additional info</x:v>
+      </x:c>
+      <x:c r="F4" s="90" t="str">
+        <x:v>Cash-equivalent amount</x:v>
+      </x:c>
+      <x:c r="G4" s="90" t="str">
+        <x:v>Cash currency</x:v>
+      </x:c>
+      <x:c r="H4" s="90" t="str">
+        <x:v>Credit amount</x:v>
+      </x:c>
+      <x:c r="I4" s="90" t="str">
+        <x:v>Credit currency / units</x:v>
+      </x:c>
+      <x:c r="J4" s="90" t="str">
+        <x:v>Subscription count</x:v>
+      </x:c>
+      <x:c r="K4" s="90" t="str">
+        <x:v>Subscription amount</x:v>
+      </x:c>
+      <x:c r="L4" s="90" t="str">
+        <x:v>Subscription currency</x:v>
+      </x:c>
+      <x:c r="M4" s="90" t="str">
+        <x:v>Other non-cash prize</x:v>
+      </x:c>
+      <x:c r="N4" s="90" t="str">
+        <x:v>Physical asset</x:v>
+      </x:c>
+      <x:c r="O4" s="90" t="str">
+        <x:v>Trophy count</x:v>
+      </x:c>
+      <x:c r="P4" s="90" t="str">
+        <x:v>Funding amount</x:v>
+      </x:c>
+      <x:c r="Q4" s="90" t="str">
+        <x:v>Funding currency</x:v>
+      </x:c>
+      <x:c r="R4" s="90" t="str">
+        <x:v>Money counted?</x:v>
+      </x:c>
+      <x:c r="S4" s="90" t="str">
+        <x:v>Review note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="36" t="n">
+        <x:f>IF(Hackathons!A2="","",Hackathons!A2)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="36" t="str">
+        <x:f>Hackathons!B2</x:f>
+        <x:v>Education Technology Hackathon</x:v>
+      </x:c>
+      <x:c r="C5" s="36" t="str">
+        <x:f>IF(Hackathons!G2="","",Hackathons!G2)</x:f>
+        <x:v>First Place, 18k SGD seed Funding</x:v>
+      </x:c>
+      <x:c r="D5" s="36" t="str">
+        <x:f>IF(Hackathons!Q2="","",Hackathons!Q2)</x:f>
+        <x:v>1st Place</x:v>
+      </x:c>
+      <x:c r="E5" s="36" t="str">
+        <x:f>IF(Hackathons!R2="","",Hackathons!R2)</x:f>
+      </x:c>
+      <x:c r="F5" s="97" t="str">
+        <x:f>IF(Hackathons!S2="","",Hackathons!S2)</x:f>
+      </x:c>
+      <x:c r="G5" s="98" t="str">
+        <x:f>IF(Hackathons!T2="","",Hackathons!T2)</x:f>
+      </x:c>
+      <x:c r="H5" s="97" t="str">
+        <x:f>IF(Hackathons!U2="","",Hackathons!U2)</x:f>
+      </x:c>
+      <x:c r="I5" s="98" t="str">
+        <x:f>IF(Hackathons!V2="","",Hackathons!V2)</x:f>
+      </x:c>
+      <x:c r="J5" s="99" t="str">
+        <x:f>IF(Hackathons!W2="","",Hackathons!W2)</x:f>
+      </x:c>
+      <x:c r="K5" s="97" t="str">
+        <x:f>IF(Hackathons!X2="","",Hackathons!X2)</x:f>
+      </x:c>
+      <x:c r="L5" s="98" t="str">
+        <x:f>IF(Hackathons!Y2="","",Hackathons!Y2)</x:f>
+      </x:c>
+      <x:c r="M5" s="36" t="str">
+        <x:f>IF(Hackathons!Z2="","",Hackathons!Z2)</x:f>
+      </x:c>
+      <x:c r="N5" s="36" t="str">
+        <x:f>IF(Hackathons!AA2="","",Hackathons!AA2)</x:f>
+      </x:c>
+      <x:c r="O5" s="39" t="str">
+        <x:f>IF(Hackathons!AB2="","",Hackathons!AB2)</x:f>
+      </x:c>
+      <x:c r="P5" s="40" t="n">
+        <x:f>IF(Hackathons!AC2="","",Hackathons!AC2)</x:f>
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="Q5" s="36" t="str">
+        <x:f>IF(Hackathons!AD2="","",Hackathons!AD2)</x:f>
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="R5" s="98" t="str">
+        <x:f>IF(Hackathons!AE2="","",Hackathons!AE2)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S5" s="98" t="str">
+        <x:f>IF(Hackathons!AF2="","",Hackathons!AF2)</x:f>
+        <x:v>Funding, not a cash prize</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="36" t="n">
+        <x:f>IF(Hackathons!A4="","",Hackathons!A4)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="36" t="str">
+        <x:f>Hackathons!B4</x:f>
+        <x:v>DataDriven Hackathon 2016</x:v>
+      </x:c>
+      <x:c r="C6" s="36" t="str">
+        <x:f>IF(Hackathons!G4="","",Hackathons!G4)</x:f>
+        <x:v>*rated best project</x:v>
+      </x:c>
+      <x:c r="D6" s="36" t="str">
+        <x:f>IF(Hackathons!Q4="","",Hackathons!Q4)</x:f>
+        <x:v>Best Project</x:v>
+      </x:c>
+      <x:c r="E6" s="36" t="str">
+        <x:f>IF(Hackathons!R4="","",Hackathons!R4)</x:f>
+        <x:v>Rated best project</x:v>
+      </x:c>
+      <x:c r="F6" s="97" t="str">
+        <x:f>IF(Hackathons!S4="","",Hackathons!S4)</x:f>
+      </x:c>
+      <x:c r="G6" s="98" t="str">
+        <x:f>IF(Hackathons!T4="","",Hackathons!T4)</x:f>
+      </x:c>
+      <x:c r="H6" s="97" t="str">
+        <x:f>IF(Hackathons!U4="","",Hackathons!U4)</x:f>
+      </x:c>
+      <x:c r="I6" s="98" t="str">
+        <x:f>IF(Hackathons!V4="","",Hackathons!V4)</x:f>
+      </x:c>
+      <x:c r="J6" s="99" t="str">
+        <x:f>IF(Hackathons!W4="","",Hackathons!W4)</x:f>
+      </x:c>
+      <x:c r="K6" s="97" t="str">
+        <x:f>IF(Hackathons!X4="","",Hackathons!X4)</x:f>
+      </x:c>
+      <x:c r="L6" s="98" t="str">
+        <x:f>IF(Hackathons!Y4="","",Hackathons!Y4)</x:f>
+      </x:c>
+      <x:c r="M6" s="36" t="str">
+        <x:f>IF(Hackathons!Z4="","",Hackathons!Z4)</x:f>
+      </x:c>
+      <x:c r="N6" s="36" t="str">
+        <x:f>IF(Hackathons!AA4="","",Hackathons!AA4)</x:f>
+      </x:c>
+      <x:c r="O6" s="39" t="str">
+        <x:f>IF(Hackathons!AB4="","",Hackathons!AB4)</x:f>
+      </x:c>
+      <x:c r="P6" s="40" t="str">
+        <x:f>IF(Hackathons!AC4="","",Hackathons!AC4)</x:f>
+      </x:c>
+      <x:c r="Q6" s="36" t="str">
+        <x:f>IF(Hackathons!AD4="","",Hackathons!AD4)</x:f>
+      </x:c>
+      <x:c r="R6" s="98" t="str">
+        <x:f>IF(Hackathons!AE4="","",Hackathons!AE4)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S6" s="98" t="str">
+        <x:f>IF(Hackathons!AF4="","",Hackathons!AF4)</x:f>
+        <x:v>Recognition only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="36" t="n">
+        <x:f>IF(Hackathons!A5="","",Hackathons!A5)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="36" t="str">
+        <x:f>Hackathons!B5</x:f>
+        <x:v>Fintech Festival Hackathon 2016</x:v>
+      </x:c>
+      <x:c r="C7" s="36" t="str">
+        <x:f>IF(Hackathons!G5="","",Hackathons!G5)</x:f>
+        <x:v>1st Place, Best Use of IBM Bluemix, US$100,000 IBM Bluemix Credits, SmartWatch</x:v>
+      </x:c>
+      <x:c r="D7" s="36" t="str">
+        <x:f>IF(Hackathons!Q5="","",Hackathons!Q5)</x:f>
+        <x:v>1st Place</x:v>
+      </x:c>
+      <x:c r="E7" s="36" t="str">
+        <x:f>IF(Hackathons!R5="","",Hackathons!R5)</x:f>
+        <x:v>Best Use of IBM Bluemix</x:v>
+      </x:c>
+      <x:c r="F7" s="97" t="str">
+        <x:f>IF(Hackathons!S5="","",Hackathons!S5)</x:f>
+      </x:c>
+      <x:c r="G7" s="98" t="str">
+        <x:f>IF(Hackathons!T5="","",Hackathons!T5)</x:f>
+      </x:c>
+      <x:c r="H7" s="97" t="n">
+        <x:f>IF(Hackathons!U5="","",Hackathons!U5)</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="I7" s="98" t="str">
+        <x:f>IF(Hackathons!V5="","",Hackathons!V5)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J7" s="99" t="str">
+        <x:f>IF(Hackathons!W5="","",Hackathons!W5)</x:f>
+      </x:c>
+      <x:c r="K7" s="97" t="str">
+        <x:f>IF(Hackathons!X5="","",Hackathons!X5)</x:f>
+      </x:c>
+      <x:c r="L7" s="98" t="str">
+        <x:f>IF(Hackathons!Y5="","",Hackathons!Y5)</x:f>
+      </x:c>
+      <x:c r="M7" s="36" t="str">
+        <x:f>IF(Hackathons!Z5="","",Hackathons!Z5)</x:f>
+        <x:v>IBM Bluemix credits; SmartWatch</x:v>
+      </x:c>
+      <x:c r="N7" s="36" t="str">
+        <x:f>IF(Hackathons!AA5="","",Hackathons!AA5)</x:f>
+        <x:v>SmartWatch</x:v>
+      </x:c>
+      <x:c r="O7" s="39" t="str">
+        <x:f>IF(Hackathons!AB5="","",Hackathons!AB5)</x:f>
+      </x:c>
+      <x:c r="P7" s="40" t="str">
+        <x:f>IF(Hackathons!AC5="","",Hackathons!AC5)</x:f>
+      </x:c>
+      <x:c r="Q7" s="36" t="str">
+        <x:f>IF(Hackathons!AD5="","",Hackathons!AD5)</x:f>
+      </x:c>
+      <x:c r="R7" s="98" t="str">
+        <x:f>IF(Hackathons!AE5="","",Hackathons!AE5)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S7" s="98" t="str">
+        <x:f>IF(Hackathons!AF5="","",Hackathons!AF5)</x:f>
+        <x:v>US$100,000 IBM Bluemix credit value</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="36" t="n">
+        <x:f>IF(Hackathons!A7="","",Hackathons!A7)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B8" s="36" t="str">
+        <x:f>Hackathons!B7</x:f>
+        <x:v>SO.IMPACT Bootcamp 2017</x:v>
+      </x:c>
+      <x:c r="C8" s="36" t="str">
+        <x:f>IF(Hackathons!G7="","",Hackathons!G7)</x:f>
+        <x:v>Shortlisted for top 10</x:v>
+      </x:c>
+      <x:c r="D8" s="36" t="str">
+        <x:f>IF(Hackathons!Q7="","",Hackathons!Q7)</x:f>
+        <x:v>Top 10</x:v>
+      </x:c>
+      <x:c r="E8" s="36" t="str">
+        <x:f>IF(Hackathons!R7="","",Hackathons!R7)</x:f>
+      </x:c>
+      <x:c r="F8" s="97" t="str">
+        <x:f>IF(Hackathons!S7="","",Hackathons!S7)</x:f>
+      </x:c>
+      <x:c r="G8" s="98" t="str">
+        <x:f>IF(Hackathons!T7="","",Hackathons!T7)</x:f>
+      </x:c>
+      <x:c r="H8" s="97" t="str">
+        <x:f>IF(Hackathons!U7="","",Hackathons!U7)</x:f>
+      </x:c>
+      <x:c r="I8" s="98" t="str">
+        <x:f>IF(Hackathons!V7="","",Hackathons!V7)</x:f>
+      </x:c>
+      <x:c r="J8" s="99" t="str">
+        <x:f>IF(Hackathons!W7="","",Hackathons!W7)</x:f>
+      </x:c>
+      <x:c r="K8" s="97" t="str">
+        <x:f>IF(Hackathons!X7="","",Hackathons!X7)</x:f>
+      </x:c>
+      <x:c r="L8" s="98" t="str">
+        <x:f>IF(Hackathons!Y7="","",Hackathons!Y7)</x:f>
+      </x:c>
+      <x:c r="M8" s="36" t="str">
+        <x:f>IF(Hackathons!Z7="","",Hackathons!Z7)</x:f>
+      </x:c>
+      <x:c r="N8" s="36" t="str">
+        <x:f>IF(Hackathons!AA7="","",Hackathons!AA7)</x:f>
+      </x:c>
+      <x:c r="O8" s="39" t="str">
+        <x:f>IF(Hackathons!AB7="","",Hackathons!AB7)</x:f>
+      </x:c>
+      <x:c r="P8" s="40" t="str">
+        <x:f>IF(Hackathons!AC7="","",Hackathons!AC7)</x:f>
+      </x:c>
+      <x:c r="Q8" s="36" t="str">
+        <x:f>IF(Hackathons!AD7="","",Hackathons!AD7)</x:f>
+      </x:c>
+      <x:c r="R8" s="98" t="str">
+        <x:f>IF(Hackathons!AE7="","",Hackathons!AE7)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S8" s="98" t="str">
+        <x:f>IF(Hackathons!AF7="","",Hackathons!AF7)</x:f>
+        <x:v>Recognition only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="36" t="n">
+        <x:f>IF(Hackathons!A11="","",Hackathons!A11)</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B9" s="36" t="str">
+        <x:f>Hackathons!B11</x:f>
+        <x:v>DataDriven Hackathon 2017</x:v>
+      </x:c>
+      <x:c r="C9" s="36" t="str">
+        <x:f>IF(Hackathons!G11="","",Hackathons!G11)</x:f>
+        <x:v>*rated best project </x:v>
+      </x:c>
+      <x:c r="D9" s="36" t="str">
+        <x:f>IF(Hackathons!Q11="","",Hackathons!Q11)</x:f>
+        <x:v>Best Project</x:v>
+      </x:c>
+      <x:c r="E9" s="36" t="str">
+        <x:f>IF(Hackathons!R11="","",Hackathons!R11)</x:f>
+        <x:v>Rated best project</x:v>
+      </x:c>
+      <x:c r="F9" s="97" t="str">
+        <x:f>IF(Hackathons!S11="","",Hackathons!S11)</x:f>
+      </x:c>
+      <x:c r="G9" s="98" t="str">
+        <x:f>IF(Hackathons!T11="","",Hackathons!T11)</x:f>
+      </x:c>
+      <x:c r="H9" s="97" t="str">
+        <x:f>IF(Hackathons!U11="","",Hackathons!U11)</x:f>
+      </x:c>
+      <x:c r="I9" s="98" t="str">
+        <x:f>IF(Hackathons!V11="","",Hackathons!V11)</x:f>
+      </x:c>
+      <x:c r="J9" s="99" t="str">
+        <x:f>IF(Hackathons!W11="","",Hackathons!W11)</x:f>
+      </x:c>
+      <x:c r="K9" s="97" t="str">
+        <x:f>IF(Hackathons!X11="","",Hackathons!X11)</x:f>
+      </x:c>
+      <x:c r="L9" s="98" t="str">
+        <x:f>IF(Hackathons!Y11="","",Hackathons!Y11)</x:f>
+      </x:c>
+      <x:c r="M9" s="36" t="str">
+        <x:f>IF(Hackathons!Z11="","",Hackathons!Z11)</x:f>
+      </x:c>
+      <x:c r="N9" s="36" t="str">
+        <x:f>IF(Hackathons!AA11="","",Hackathons!AA11)</x:f>
+      </x:c>
+      <x:c r="O9" s="39" t="str">
+        <x:f>IF(Hackathons!AB11="","",Hackathons!AB11)</x:f>
+      </x:c>
+      <x:c r="P9" s="40" t="str">
+        <x:f>IF(Hackathons!AC11="","",Hackathons!AC11)</x:f>
+      </x:c>
+      <x:c r="Q9" s="36" t="str">
+        <x:f>IF(Hackathons!AD11="","",Hackathons!AD11)</x:f>
+      </x:c>
+      <x:c r="R9" s="98" t="str">
+        <x:f>IF(Hackathons!AE11="","",Hackathons!AE11)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S9" s="98" t="str">
+        <x:f>IF(Hackathons!AF11="","",Hackathons!AF11)</x:f>
+        <x:v>Recognition only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="36" t="n">
+        <x:f>IF(Hackathons!A15="","",Hackathons!A15)</x:f>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B10" s="36" t="e">
+        <x:f>Hackathons!B15</x:f>
+        <x:v>#SPSEC SP Hackathon 2018</x:v>
+      </x:c>
+      <x:c r="C10" s="36" t="str">
+        <x:f>IF(Hackathons!G15="","",Hackathons!G15)</x:f>
+        <x:v>3rd Place, $100 Capitaland voucher</x:v>
+      </x:c>
+      <x:c r="D10" s="36" t="str">
+        <x:f>IF(Hackathons!Q15="","",Hackathons!Q15)</x:f>
+        <x:v>3rd Place</x:v>
+      </x:c>
+      <x:c r="E10" s="36" t="str">
+        <x:f>IF(Hackathons!R15="","",Hackathons!R15)</x:f>
+      </x:c>
+      <x:c r="F10" s="97" t="n">
+        <x:f>IF(Hackathons!S15="","",Hackathons!S15)</x:f>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G10" s="98" t="str">
+        <x:f>IF(Hackathons!T15="","",Hackathons!T15)</x:f>
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="H10" s="97" t="str">
+        <x:f>IF(Hackathons!U15="","",Hackathons!U15)</x:f>
+      </x:c>
+      <x:c r="I10" s="98" t="str">
+        <x:f>IF(Hackathons!V15="","",Hackathons!V15)</x:f>
+      </x:c>
+      <x:c r="J10" s="99" t="str">
+        <x:f>IF(Hackathons!W15="","",Hackathons!W15)</x:f>
+      </x:c>
+      <x:c r="K10" s="97" t="str">
+        <x:f>IF(Hackathons!X15="","",Hackathons!X15)</x:f>
+      </x:c>
+      <x:c r="L10" s="98" t="str">
+        <x:f>IF(Hackathons!Y15="","",Hackathons!Y15)</x:f>
+      </x:c>
+      <x:c r="M10" s="36" t="str">
+        <x:f>IF(Hackathons!Z15="","",Hackathons!Z15)</x:f>
+        <x:v>S$100 Capitaland voucher</x:v>
+      </x:c>
+      <x:c r="N10" s="36" t="str">
+        <x:f>IF(Hackathons!AA15="","",Hackathons!AA15)</x:f>
+      </x:c>
+      <x:c r="O10" s="39" t="str">
+        <x:f>IF(Hackathons!AB15="","",Hackathons!AB15)</x:f>
+      </x:c>
+      <x:c r="P10" s="40" t="str">
+        <x:f>IF(Hackathons!AC15="","",Hackathons!AC15)</x:f>
+      </x:c>
+      <x:c r="Q10" s="36" t="str">
+        <x:f>IF(Hackathons!AD15="","",Hackathons!AD15)</x:f>
+      </x:c>
+      <x:c r="R10" s="98" t="str">
+        <x:f>IF(Hackathons!AE15="","",Hackathons!AE15)</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="S10" s="98" t="str">
+        <x:f>IF(Hackathons!AF15="","",Hackathons!AF15)</x:f>
+        <x:v>Voucher counted as cash equivalent</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="36" t="n">
+        <x:f>IF(Hackathons!A18="","",Hackathons!A18)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B11" s="36" t="e">
+        <x:f>Hackathons!B18</x:f>
+        <x:v>#Mosque-Tech Challenge 2018</x:v>
+      </x:c>
+      <x:c r="C11" s="36" t="str">
+        <x:f>IF(Hackathons!G18="","",Hackathons!G18)</x:f>
+        <x:v>2nd Place, $600 cash</x:v>
+      </x:c>
+      <x:c r="D11" s="36" t="str">
+        <x:f>IF(Hackathons!Q18="","",Hackathons!Q18)</x:f>
+        <x:v>2nd Place</x:v>
+      </x:c>
+      <x:c r="E11" s="36" t="str">
+        <x:f>IF(Hackathons!R18="","",Hackathons!R18)</x:f>
+      </x:c>
+      <x:c r="F11" s="97" t="n">
+        <x:f>IF(Hackathons!S18="","",Hackathons!S18)</x:f>
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="G11" s="98" t="str">
+        <x:f>IF(Hackathons!T18="","",Hackathons!T18)</x:f>
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="H11" s="97" t="str">
+        <x:f>IF(Hackathons!U18="","",Hackathons!U18)</x:f>
+      </x:c>
+      <x:c r="I11" s="98" t="str">
+        <x:f>IF(Hackathons!V18="","",Hackathons!V18)</x:f>
+      </x:c>
+      <x:c r="J11" s="99" t="str">
+        <x:f>IF(Hackathons!W18="","",Hackathons!W18)</x:f>
+      </x:c>
+      <x:c r="K11" s="97" t="str">
+        <x:f>IF(Hackathons!X18="","",Hackathons!X18)</x:f>
+      </x:c>
+      <x:c r="L11" s="98" t="str">
+        <x:f>IF(Hackathons!Y18="","",Hackathons!Y18)</x:f>
+      </x:c>
+      <x:c r="M11" s="36" t="str">
+        <x:f>IF(Hackathons!Z18="","",Hackathons!Z18)</x:f>
+      </x:c>
+      <x:c r="N11" s="36" t="str">
+        <x:f>IF(Hackathons!AA18="","",Hackathons!AA18)</x:f>
+      </x:c>
+      <x:c r="O11" s="39" t="str">
+        <x:f>IF(Hackathons!AB18="","",Hackathons!AB18)</x:f>
+      </x:c>
+      <x:c r="P11" s="40" t="str">
+        <x:f>IF(Hackathons!AC18="","",Hackathons!AC18)</x:f>
+      </x:c>
+      <x:c r="Q11" s="36" t="str">
+        <x:f>IF(Hackathons!AD18="","",Hackathons!AD18)</x:f>
+      </x:c>
+      <x:c r="R11" s="98" t="str">
+        <x:f>IF(Hackathons!AE18="","",Hackathons!AE18)</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="S11" s="98" t="str">
+        <x:f>IF(Hackathons!AF18="","",Hackathons!AF18)</x:f>
+        <x:v>Explicit cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="36" t="n">
+        <x:f>IF(Hackathons!A26="","",Hackathons!A26)</x:f>
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B12" s="36" t="e">
+        <x:f>Hackathons!B26</x:f>
+        <x:v>#Mosque Hackathon 2019</x:v>
+      </x:c>
+      <x:c r="C12" s="36" t="str">
+        <x:f>IF(Hackathons!G26="","",Hackathons!G26)</x:f>
+        <x:v>3rd Place, $500 SGD cash</x:v>
+      </x:c>
+      <x:c r="D12" s="36" t="str">
+        <x:f>IF(Hackathons!Q26="","",Hackathons!Q26)</x:f>
+        <x:v>3rd Place</x:v>
+      </x:c>
+      <x:c r="E12" s="36" t="str">
+        <x:f>IF(Hackathons!R26="","",Hackathons!R26)</x:f>
+      </x:c>
+      <x:c r="F12" s="97" t="n">
+        <x:f>IF(Hackathons!S26="","",Hackathons!S26)</x:f>
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G12" s="98" t="str">
+        <x:f>IF(Hackathons!T26="","",Hackathons!T26)</x:f>
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="H12" s="97" t="str">
+        <x:f>IF(Hackathons!U26="","",Hackathons!U26)</x:f>
+      </x:c>
+      <x:c r="I12" s="98" t="str">
+        <x:f>IF(Hackathons!V26="","",Hackathons!V26)</x:f>
+      </x:c>
+      <x:c r="J12" s="99" t="str">
+        <x:f>IF(Hackathons!W26="","",Hackathons!W26)</x:f>
+      </x:c>
+      <x:c r="K12" s="97" t="str">
+        <x:f>IF(Hackathons!X26="","",Hackathons!X26)</x:f>
+      </x:c>
+      <x:c r="L12" s="98" t="str">
+        <x:f>IF(Hackathons!Y26="","",Hackathons!Y26)</x:f>
+      </x:c>
+      <x:c r="M12" s="36" t="str">
+        <x:f>IF(Hackathons!Z26="","",Hackathons!Z26)</x:f>
+      </x:c>
+      <x:c r="N12" s="36" t="str">
+        <x:f>IF(Hackathons!AA26="","",Hackathons!AA26)</x:f>
+      </x:c>
+      <x:c r="O12" s="39" t="str">
+        <x:f>IF(Hackathons!AB26="","",Hackathons!AB26)</x:f>
+      </x:c>
+      <x:c r="P12" s="40" t="str">
+        <x:f>IF(Hackathons!AC26="","",Hackathons!AC26)</x:f>
+      </x:c>
+      <x:c r="Q12" s="36" t="str">
+        <x:f>IF(Hackathons!AD26="","",Hackathons!AD26)</x:f>
+      </x:c>
+      <x:c r="R12" s="98" t="str">
+        <x:f>IF(Hackathons!AE26="","",Hackathons!AE26)</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="S12" s="98" t="str">
+        <x:f>IF(Hackathons!AF26="","",Hackathons!AF26)</x:f>
+        <x:v>Explicit cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="36" t="n">
+        <x:f>IF(Hackathons!A34="","",Hackathons!A34)</x:f>
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B13" s="36" t="str">
+        <x:f>Hackathons!B34</x:f>
+        <x:v>ICP Ideathon 2023</x:v>
+      </x:c>
+      <x:c r="C13" s="36" t="str">
+        <x:f>IF(Hackathons!G34="","",Hackathons!G34)</x:f>
+        <x:v>3rd Prize (S$250 Cash)</x:v>
+      </x:c>
+      <x:c r="D13" s="36" t="str">
+        <x:f>IF(Hackathons!Q34="","",Hackathons!Q34)</x:f>
+        <x:v>3rd Prize</x:v>
+      </x:c>
+      <x:c r="E13" s="36" t="str">
+        <x:f>IF(Hackathons!R34="","",Hackathons!R34)</x:f>
+      </x:c>
+      <x:c r="F13" s="97" t="n">
+        <x:f>IF(Hackathons!S34="","",Hackathons!S34)</x:f>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="G13" s="98" t="str">
+        <x:f>IF(Hackathons!T34="","",Hackathons!T34)</x:f>
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="H13" s="97" t="str">
+        <x:f>IF(Hackathons!U34="","",Hackathons!U34)</x:f>
+      </x:c>
+      <x:c r="I13" s="98" t="str">
+        <x:f>IF(Hackathons!V34="","",Hackathons!V34)</x:f>
+      </x:c>
+      <x:c r="J13" s="99" t="str">
+        <x:f>IF(Hackathons!W34="","",Hackathons!W34)</x:f>
+      </x:c>
+      <x:c r="K13" s="97" t="str">
+        <x:f>IF(Hackathons!X34="","",Hackathons!X34)</x:f>
+      </x:c>
+      <x:c r="L13" s="98" t="str">
+        <x:f>IF(Hackathons!Y34="","",Hackathons!Y34)</x:f>
+      </x:c>
+      <x:c r="M13" s="36" t="str">
+        <x:f>IF(Hackathons!Z34="","",Hackathons!Z34)</x:f>
+      </x:c>
+      <x:c r="N13" s="36" t="str">
+        <x:f>IF(Hackathons!AA34="","",Hackathons!AA34)</x:f>
+      </x:c>
+      <x:c r="O13" s="39" t="str">
+        <x:f>IF(Hackathons!AB34="","",Hackathons!AB34)</x:f>
+      </x:c>
+      <x:c r="P13" s="40" t="str">
+        <x:f>IF(Hackathons!AC34="","",Hackathons!AC34)</x:f>
+      </x:c>
+      <x:c r="Q13" s="36" t="str">
+        <x:f>IF(Hackathons!AD34="","",Hackathons!AD34)</x:f>
+      </x:c>
+      <x:c r="R13" s="98" t="str">
+        <x:f>IF(Hackathons!AE34="","",Hackathons!AE34)</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="S13" s="98" t="str">
+        <x:f>IF(Hackathons!AF34="","",Hackathons!AF34)</x:f>
+        <x:v>Confirmed cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="36" t="n">
+        <x:f>IF(Hackathons!A36="","",Hackathons!A36)</x:f>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B14" s="36" t="str">
+        <x:f>Hackathons!B36</x:f>
+        <x:v>Mosque Tech Challenge 2025</x:v>
+      </x:c>
+      <x:c r="C14" s="36" t="str">
+        <x:f>IF(Hackathons!G36="","",Hackathons!G36)</x:f>
+        <x:v>2nd Prize (S$1,000 Cash)</x:v>
+      </x:c>
+      <x:c r="D14" s="36" t="str">
+        <x:f>IF(Hackathons!Q36="","",Hackathons!Q36)</x:f>
+        <x:v>2nd Prize</x:v>
+      </x:c>
+      <x:c r="E14" s="36" t="str">
+        <x:f>IF(Hackathons!R36="","",Hackathons!R36)</x:f>
+      </x:c>
+      <x:c r="F14" s="97" t="n">
+        <x:f>IF(Hackathons!S36="","",Hackathons!S36)</x:f>
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="G14" s="98" t="str">
+        <x:f>IF(Hackathons!T36="","",Hackathons!T36)</x:f>
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="H14" s="97" t="str">
+        <x:f>IF(Hackathons!U36="","",Hackathons!U36)</x:f>
+      </x:c>
+      <x:c r="I14" s="98" t="str">
+        <x:f>IF(Hackathons!V36="","",Hackathons!V36)</x:f>
+      </x:c>
+      <x:c r="J14" s="99" t="str">
+        <x:f>IF(Hackathons!W36="","",Hackathons!W36)</x:f>
+      </x:c>
+      <x:c r="K14" s="97" t="str">
+        <x:f>IF(Hackathons!X36="","",Hackathons!X36)</x:f>
+      </x:c>
+      <x:c r="L14" s="98" t="str">
+        <x:f>IF(Hackathons!Y36="","",Hackathons!Y36)</x:f>
+      </x:c>
+      <x:c r="M14" s="36" t="str">
+        <x:f>IF(Hackathons!Z36="","",Hackathons!Z36)</x:f>
+      </x:c>
+      <x:c r="N14" s="36" t="str">
+        <x:f>IF(Hackathons!AA36="","",Hackathons!AA36)</x:f>
+      </x:c>
+      <x:c r="O14" s="39" t="str">
+        <x:f>IF(Hackathons!AB36="","",Hackathons!AB36)</x:f>
+      </x:c>
+      <x:c r="P14" s="40" t="str">
+        <x:f>IF(Hackathons!AC36="","",Hackathons!AC36)</x:f>
+      </x:c>
+      <x:c r="Q14" s="36" t="str">
+        <x:f>IF(Hackathons!AD36="","",Hackathons!AD36)</x:f>
+      </x:c>
+      <x:c r="R14" s="98" t="str">
+        <x:f>IF(Hackathons!AE36="","",Hackathons!AE36)</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="S14" s="98" t="str">
+        <x:f>IF(Hackathons!AF36="","",Hackathons!AF36)</x:f>
+        <x:v>Confirmed cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="36" t="n">
+        <x:f>IF(Hackathons!A39="","",Hackathons!A39)</x:f>
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B15" s="36" t="str">
+        <x:f>Hackathons!B39</x:f>
+        <x:v>OOJU X Manus.AI Hackathon 2025</x:v>
+      </x:c>
+      <x:c r="C15" s="36" t="str">
+        <x:f>IF(Hackathons!G39="","",Hackathons!G39)</x:f>
+        <x:v>2nd Prize (Manus Pro Subscription)</x:v>
+      </x:c>
+      <x:c r="D15" s="36" t="str">
+        <x:f>IF(Hackathons!Q39="","",Hackathons!Q39)</x:f>
+        <x:v>2nd Prize</x:v>
+      </x:c>
+      <x:c r="E15" s="36" t="str">
+        <x:f>IF(Hackathons!R39="","",Hackathons!R39)</x:f>
+      </x:c>
+      <x:c r="F15" s="97" t="str">
+        <x:f>IF(Hackathons!S39="","",Hackathons!S39)</x:f>
+      </x:c>
+      <x:c r="G15" s="98" t="str">
+        <x:f>IF(Hackathons!T39="","",Hackathons!T39)</x:f>
+      </x:c>
+      <x:c r="H15" s="97" t="str">
+        <x:f>IF(Hackathons!U39="","",Hackathons!U39)</x:f>
+      </x:c>
+      <x:c r="I15" s="98" t="str">
+        <x:f>IF(Hackathons!V39="","",Hackathons!V39)</x:f>
+      </x:c>
+      <x:c r="J15" s="99" t="n">
+        <x:f>IF(Hackathons!W39="","",Hackathons!W39)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K15" s="97" t="n">
+        <x:f>IF(Hackathons!X39="","",Hackathons!X39)</x:f>
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="L15" s="98" t="str">
+        <x:f>IF(Hackathons!Y39="","",Hackathons!Y39)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="M15" s="36" t="str">
+        <x:f>IF(Hackathons!Z39="","",Hackathons!Z39)</x:f>
+        <x:v>Manus Pro subscription</x:v>
+      </x:c>
+      <x:c r="N15" s="36" t="str">
+        <x:f>IF(Hackathons!AA39="","",Hackathons!AA39)</x:f>
+      </x:c>
+      <x:c r="O15" s="39" t="str">
+        <x:f>IF(Hackathons!AB39="","",Hackathons!AB39)</x:f>
+      </x:c>
+      <x:c r="P15" s="40" t="str">
+        <x:f>IF(Hackathons!AC39="","",Hackathons!AC39)</x:f>
+      </x:c>
+      <x:c r="Q15" s="36" t="str">
+        <x:f>IF(Hackathons!AD39="","",Hackathons!AD39)</x:f>
+      </x:c>
+      <x:c r="R15" s="98" t="str">
+        <x:f>IF(Hackathons!AE39="","",Hackathons!AE39)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S15" s="98" t="str">
+        <x:f>IF(Hackathons!AF39="","",Hackathons!AF39)</x:f>
+        <x:v>US$39 monthly value at award period</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="36" t="n">
+        <x:f>IF(Hackathons!A41="","",Hackathons!A41)</x:f>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B16" s="36" t="str">
+        <x:f>Hackathons!B41</x:f>
+        <x:v>Sarawak AI Hackathon 2025</x:v>
+      </x:c>
+      <x:c r="C16" s="36" t="str">
+        <x:f>IF(Hackathons!G41="","",Hackathons!G41)</x:f>
+        <x:v>Throphy, Best Novel Hackathon Finisher</x:v>
+      </x:c>
+      <x:c r="D16" s="36" t="str">
+        <x:f>IF(Hackathons!Q41="","",Hackathons!Q41)</x:f>
+        <x:v>Best Finisher</x:v>
+      </x:c>
+      <x:c r="E16" s="36" t="str">
+        <x:f>IF(Hackathons!R41="","",Hackathons!R41)</x:f>
+        <x:v>Novel Hackathon</x:v>
+      </x:c>
+      <x:c r="F16" s="97" t="str">
+        <x:f>IF(Hackathons!S41="","",Hackathons!S41)</x:f>
+      </x:c>
+      <x:c r="G16" s="98" t="str">
+        <x:f>IF(Hackathons!T41="","",Hackathons!T41)</x:f>
+      </x:c>
+      <x:c r="H16" s="97" t="str">
+        <x:f>IF(Hackathons!U41="","",Hackathons!U41)</x:f>
+      </x:c>
+      <x:c r="I16" s="98" t="str">
+        <x:f>IF(Hackathons!V41="","",Hackathons!V41)</x:f>
+      </x:c>
+      <x:c r="J16" s="99" t="str">
+        <x:f>IF(Hackathons!W41="","",Hackathons!W41)</x:f>
+      </x:c>
+      <x:c r="K16" s="97" t="str">
+        <x:f>IF(Hackathons!X41="","",Hackathons!X41)</x:f>
+      </x:c>
+      <x:c r="L16" s="98" t="str">
+        <x:f>IF(Hackathons!Y41="","",Hackathons!Y41)</x:f>
+      </x:c>
+      <x:c r="M16" s="36" t="str">
+        <x:f>IF(Hackathons!Z41="","",Hackathons!Z41)</x:f>
+        <x:v>Trophy</x:v>
+      </x:c>
+      <x:c r="N16" s="36" t="str">
+        <x:f>IF(Hackathons!AA41="","",Hackathons!AA41)</x:f>
+        <x:v>Trophy</x:v>
+      </x:c>
+      <x:c r="O16" s="39" t="n">
+        <x:f>IF(Hackathons!AB41="","",Hackathons!AB41)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P16" s="40" t="str">
+        <x:f>IF(Hackathons!AC41="","",Hackathons!AC41)</x:f>
+      </x:c>
+      <x:c r="Q16" s="36" t="str">
+        <x:f>IF(Hackathons!AD41="","",Hackathons!AD41)</x:f>
+      </x:c>
+      <x:c r="R16" s="98" t="str">
+        <x:f>IF(Hackathons!AE41="","",Hackathons!AE41)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S16" s="98" t="str">
+        <x:f>IF(Hackathons!AF41="","",Hackathons!AF41)</x:f>
+        <x:v>Trophy, not cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="36" t="n">
+        <x:f>IF(Hackathons!A43="","",Hackathons!A43)</x:f>
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B17" s="36" t="str">
+        <x:f>Hackathons!B43</x:f>
+        <x:v>Nosana Hackathon 2025</x:v>
+      </x:c>
+      <x:c r="C17" s="36" t="str">
+        <x:f>IF(Hackathons!G43="","",Hackathons!G43)</x:f>
+        <x:v>1st Prize, $500 Nosana Cloud Credit</x:v>
+      </x:c>
+      <x:c r="D17" s="36" t="str">
+        <x:f>IF(Hackathons!Q43="","",Hackathons!Q43)</x:f>
+        <x:v>1st Prize</x:v>
+      </x:c>
+      <x:c r="E17" s="36" t="str">
+        <x:f>IF(Hackathons!R43="","",Hackathons!R43)</x:f>
+      </x:c>
+      <x:c r="F17" s="97" t="str">
+        <x:f>IF(Hackathons!S43="","",Hackathons!S43)</x:f>
+      </x:c>
+      <x:c r="G17" s="98" t="str">
+        <x:f>IF(Hackathons!T43="","",Hackathons!T43)</x:f>
+      </x:c>
+      <x:c r="H17" s="97" t="n">
+        <x:f>IF(Hackathons!U43="","",Hackathons!U43)</x:f>
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="I17" s="98" t="str">
+        <x:f>IF(Hackathons!V43="","",Hackathons!V43)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J17" s="99" t="str">
+        <x:f>IF(Hackathons!W43="","",Hackathons!W43)</x:f>
+      </x:c>
+      <x:c r="K17" s="97" t="str">
+        <x:f>IF(Hackathons!X43="","",Hackathons!X43)</x:f>
+      </x:c>
+      <x:c r="L17" s="98" t="str">
+        <x:f>IF(Hackathons!Y43="","",Hackathons!Y43)</x:f>
+      </x:c>
+      <x:c r="M17" s="36" t="str">
+        <x:f>IF(Hackathons!Z43="","",Hackathons!Z43)</x:f>
+        <x:v>Nosana Cloud credit</x:v>
+      </x:c>
+      <x:c r="N17" s="36" t="str">
+        <x:f>IF(Hackathons!AA43="","",Hackathons!AA43)</x:f>
+      </x:c>
+      <x:c r="O17" s="39" t="str">
+        <x:f>IF(Hackathons!AB43="","",Hackathons!AB43)</x:f>
+      </x:c>
+      <x:c r="P17" s="40" t="str">
+        <x:f>IF(Hackathons!AC43="","",Hackathons!AC43)</x:f>
+      </x:c>
+      <x:c r="Q17" s="36" t="str">
+        <x:f>IF(Hackathons!AD43="","",Hackathons!AD43)</x:f>
+      </x:c>
+      <x:c r="R17" s="98" t="str">
+        <x:f>IF(Hackathons!AE43="","",Hackathons!AE43)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S17" s="98" t="str">
+        <x:f>IF(Hackathons!AF43="","",Hackathons!AF43)</x:f>
+        <x:v>Cloud credit, not cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="36" t="n">
+        <x:f>IF(Hackathons!A51="","",Hackathons!A51)</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B18" s="36" t="str">
+        <x:f>Hackathons!B51</x:f>
+        <x:v>Agentfield Hackathon 2026</x:v>
+      </x:c>
+      <x:c r="C18" s="36" t="str">
+        <x:f>IF(Hackathons!G51="","",Hackathons!G51)</x:f>
+        <x:v>1st Prize (OpenRouter Credits $1000 USD)</x:v>
+      </x:c>
+      <x:c r="D18" s="36" t="str">
+        <x:f>IF(Hackathons!Q51="","",Hackathons!Q51)</x:f>
+        <x:v>1st Prize</x:v>
+      </x:c>
+      <x:c r="E18" s="36" t="str">
+        <x:f>IF(Hackathons!R51="","",Hackathons!R51)</x:f>
+      </x:c>
+      <x:c r="F18" s="97" t="str">
+        <x:f>IF(Hackathons!S51="","",Hackathons!S51)</x:f>
+      </x:c>
+      <x:c r="G18" s="98" t="str">
+        <x:f>IF(Hackathons!T51="","",Hackathons!T51)</x:f>
+      </x:c>
+      <x:c r="H18" s="97" t="n">
+        <x:f>IF(Hackathons!U51="","",Hackathons!U51)</x:f>
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="I18" s="98" t="str">
+        <x:f>IF(Hackathons!V51="","",Hackathons!V51)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J18" s="99" t="str">
+        <x:f>IF(Hackathons!W51="","",Hackathons!W51)</x:f>
+      </x:c>
+      <x:c r="K18" s="97" t="str">
+        <x:f>IF(Hackathons!X51="","",Hackathons!X51)</x:f>
+      </x:c>
+      <x:c r="L18" s="98" t="str">
+        <x:f>IF(Hackathons!Y51="","",Hackathons!Y51)</x:f>
+      </x:c>
+      <x:c r="M18" s="36" t="str">
+        <x:f>IF(Hackathons!Z51="","",Hackathons!Z51)</x:f>
+        <x:v>OpenRouter credits</x:v>
+      </x:c>
+      <x:c r="N18" s="36" t="str">
+        <x:f>IF(Hackathons!AA51="","",Hackathons!AA51)</x:f>
+      </x:c>
+      <x:c r="O18" s="39" t="str">
+        <x:f>IF(Hackathons!AB51="","",Hackathons!AB51)</x:f>
+      </x:c>
+      <x:c r="P18" s="40" t="str">
+        <x:f>IF(Hackathons!AC51="","",Hackathons!AC51)</x:f>
+      </x:c>
+      <x:c r="Q18" s="36" t="str">
+        <x:f>IF(Hackathons!AD51="","",Hackathons!AD51)</x:f>
+      </x:c>
+      <x:c r="R18" s="98" t="str">
+        <x:f>IF(Hackathons!AE51="","",Hackathons!AE51)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S18" s="98" t="str">
+        <x:f>IF(Hackathons!AF51="","",Hackathons!AF51)</x:f>
+        <x:v>API credits, not cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="36" t="n">
+        <x:f>IF(Hackathons!A53="","",Hackathons!A53)</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B19" s="36" t="str">
+        <x:f>Hackathons!B53</x:f>
+        <x:v>AgentForce Hackathon 2026</x:v>
+      </x:c>
+      <x:c r="C19" s="36" t="str">
+        <x:f>IF(Hackathons!G53="","",Hackathons!G53)</x:f>
+        <x:v>1st Prize (API Credits $500 USD)</x:v>
+      </x:c>
+      <x:c r="D19" s="36" t="str">
+        <x:f>IF(Hackathons!Q53="","",Hackathons!Q53)</x:f>
+        <x:v>1st Prize</x:v>
+      </x:c>
+      <x:c r="E19" s="36" t="str">
+        <x:f>IF(Hackathons!R53="","",Hackathons!R53)</x:f>
+      </x:c>
+      <x:c r="F19" s="97" t="str">
+        <x:f>IF(Hackathons!S53="","",Hackathons!S53)</x:f>
+      </x:c>
+      <x:c r="G19" s="98" t="str">
+        <x:f>IF(Hackathons!T53="","",Hackathons!T53)</x:f>
+      </x:c>
+      <x:c r="H19" s="97" t="n">
+        <x:f>IF(Hackathons!U53="","",Hackathons!U53)</x:f>
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="I19" s="98" t="str">
+        <x:f>IF(Hackathons!V53="","",Hackathons!V53)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J19" s="99" t="str">
+        <x:f>IF(Hackathons!W53="","",Hackathons!W53)</x:f>
+      </x:c>
+      <x:c r="K19" s="97" t="str">
+        <x:f>IF(Hackathons!X53="","",Hackathons!X53)</x:f>
+      </x:c>
+      <x:c r="L19" s="98" t="str">
+        <x:f>IF(Hackathons!Y53="","",Hackathons!Y53)</x:f>
+      </x:c>
+      <x:c r="M19" s="36" t="str">
+        <x:f>IF(Hackathons!Z53="","",Hackathons!Z53)</x:f>
+        <x:v>API credits</x:v>
+      </x:c>
+      <x:c r="N19" s="36" t="str">
+        <x:f>IF(Hackathons!AA53="","",Hackathons!AA53)</x:f>
+      </x:c>
+      <x:c r="O19" s="39" t="str">
+        <x:f>IF(Hackathons!AB53="","",Hackathons!AB53)</x:f>
+      </x:c>
+      <x:c r="P19" s="40" t="str">
+        <x:f>IF(Hackathons!AC53="","",Hackathons!AC53)</x:f>
+      </x:c>
+      <x:c r="Q19" s="36" t="str">
+        <x:f>IF(Hackathons!AD53="","",Hackathons!AD53)</x:f>
+      </x:c>
+      <x:c r="R19" s="98" t="str">
+        <x:f>IF(Hackathons!AE53="","",Hackathons!AE53)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S19" s="98" t="str">
+        <x:f>IF(Hackathons!AF53="","",Hackathons!AF53)</x:f>
+        <x:v>API credits, not cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="36" t="n">
+        <x:f>IF(Hackathons!A54="","",Hackathons!A54)</x:f>
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B20" s="36" t="str">
+        <x:f>Hackathons!B54</x:f>
+        <x:v>AgentForce Hackathon 2026</x:v>
+      </x:c>
+      <x:c r="C20" s="36" t="str">
+        <x:f>IF(Hackathons!G54="","",Hackathons!G54)</x:f>
+        <x:v>1st Prize (API Credits $500 USD)</x:v>
+      </x:c>
+      <x:c r="D20" s="36" t="str">
+        <x:f>IF(Hackathons!Q54="","",Hackathons!Q54)</x:f>
+        <x:v>1st Prize</x:v>
+      </x:c>
+      <x:c r="E20" s="36" t="str">
+        <x:f>IF(Hackathons!R54="","",Hackathons!R54)</x:f>
+      </x:c>
+      <x:c r="F20" s="97" t="str">
+        <x:f>IF(Hackathons!S54="","",Hackathons!S54)</x:f>
+      </x:c>
+      <x:c r="G20" s="98" t="str">
+        <x:f>IF(Hackathons!T54="","",Hackathons!T54)</x:f>
+      </x:c>
+      <x:c r="H20" s="97" t="n">
+        <x:f>IF(Hackathons!U54="","",Hackathons!U54)</x:f>
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="I20" s="98" t="str">
+        <x:f>IF(Hackathons!V54="","",Hackathons!V54)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J20" s="99" t="str">
+        <x:f>IF(Hackathons!W54="","",Hackathons!W54)</x:f>
+      </x:c>
+      <x:c r="K20" s="97" t="str">
+        <x:f>IF(Hackathons!X54="","",Hackathons!X54)</x:f>
+      </x:c>
+      <x:c r="L20" s="98" t="str">
+        <x:f>IF(Hackathons!Y54="","",Hackathons!Y54)</x:f>
+      </x:c>
+      <x:c r="M20" s="36" t="str">
+        <x:f>IF(Hackathons!Z54="","",Hackathons!Z54)</x:f>
+        <x:v>API credits</x:v>
+      </x:c>
+      <x:c r="N20" s="36" t="str">
+        <x:f>IF(Hackathons!AA54="","",Hackathons!AA54)</x:f>
+      </x:c>
+      <x:c r="O20" s="39" t="str">
+        <x:f>IF(Hackathons!AB54="","",Hackathons!AB54)</x:f>
+      </x:c>
+      <x:c r="P20" s="40" t="str">
+        <x:f>IF(Hackathons!AC54="","",Hackathons!AC54)</x:f>
+      </x:c>
+      <x:c r="Q20" s="36" t="str">
+        <x:f>IF(Hackathons!AD54="","",Hackathons!AD54)</x:f>
+      </x:c>
+      <x:c r="R20" s="98" t="str">
+        <x:f>IF(Hackathons!AE54="","",Hackathons!AE54)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S20" s="98" t="str">
+        <x:f>IF(Hackathons!AF54="","",Hackathons!AF54)</x:f>
+        <x:v>API credits, not cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="36" t="n">
+        <x:f>IF(Hackathons!A55="","",Hackathons!A55)</x:f>
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B21" s="36" t="str">
+        <x:f>Hackathons!B55</x:f>
+        <x:v>SUSS X Openclaw Hackathon 2026</x:v>
+      </x:c>
+      <x:c r="C21" s="36" t="str">
+        <x:f>IF(Hackathons!G55="","",Hackathons!G55)</x:f>
+        <x:v>1st Prize (Wavespeed AI Credits $150 USD)</x:v>
+      </x:c>
+      <x:c r="D21" s="36" t="str">
+        <x:f>IF(Hackathons!Q55="","",Hackathons!Q55)</x:f>
+        <x:v>1st Prize</x:v>
+      </x:c>
+      <x:c r="E21" s="36" t="str">
+        <x:f>IF(Hackathons!R55="","",Hackathons!R55)</x:f>
+      </x:c>
+      <x:c r="F21" s="97" t="str">
+        <x:f>IF(Hackathons!S55="","",Hackathons!S55)</x:f>
+      </x:c>
+      <x:c r="G21" s="98" t="str">
+        <x:f>IF(Hackathons!T55="","",Hackathons!T55)</x:f>
+      </x:c>
+      <x:c r="H21" s="97" t="n">
+        <x:f>IF(Hackathons!U55="","",Hackathons!U55)</x:f>
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="I21" s="98" t="str">
+        <x:f>IF(Hackathons!V55="","",Hackathons!V55)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J21" s="99" t="str">
+        <x:f>IF(Hackathons!W55="","",Hackathons!W55)</x:f>
+      </x:c>
+      <x:c r="K21" s="97" t="str">
+        <x:f>IF(Hackathons!X55="","",Hackathons!X55)</x:f>
+      </x:c>
+      <x:c r="L21" s="98" t="str">
+        <x:f>IF(Hackathons!Y55="","",Hackathons!Y55)</x:f>
+      </x:c>
+      <x:c r="M21" s="36" t="str">
+        <x:f>IF(Hackathons!Z55="","",Hackathons!Z55)</x:f>
+        <x:v>Wavespeed AI credits</x:v>
+      </x:c>
+      <x:c r="N21" s="36" t="str">
+        <x:f>IF(Hackathons!AA55="","",Hackathons!AA55)</x:f>
+      </x:c>
+      <x:c r="O21" s="39" t="str">
+        <x:f>IF(Hackathons!AB55="","",Hackathons!AB55)</x:f>
+      </x:c>
+      <x:c r="P21" s="40" t="str">
+        <x:f>IF(Hackathons!AC55="","",Hackathons!AC55)</x:f>
+      </x:c>
+      <x:c r="Q21" s="36" t="str">
+        <x:f>IF(Hackathons!AD55="","",Hackathons!AD55)</x:f>
+      </x:c>
+      <x:c r="R21" s="98" t="str">
+        <x:f>IF(Hackathons!AE55="","",Hackathons!AE55)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S21" s="98" t="str">
+        <x:f>IF(Hackathons!AF55="","",Hackathons!AF55)</x:f>
+        <x:v>API credits, not cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="36" t="n">
+        <x:f>IF(Hackathons!A58="","",Hackathons!A58)</x:f>
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B22" s="36" t="str">
+        <x:f>Hackathons!B58</x:f>
+        <x:v>Agora.io Voice AI Hackathon Singapore 2026</x:v>
+      </x:c>
+      <x:c r="C22" s="36" t="str">
+        <x:f>IF(Hackathons!G58="","",Hackathons!G58)</x:f>
+        <x:v>3rd Prize: S$300 Cash and S$385 worth of API Credits</x:v>
+      </x:c>
+      <x:c r="D22" s="36" t="str">
+        <x:f>IF(Hackathons!Q58="","",Hackathons!Q58)</x:f>
+        <x:v>3rd Prize</x:v>
+      </x:c>
+      <x:c r="E22" s="36" t="str">
+        <x:f>IF(Hackathons!R58="","",Hackathons!R58)</x:f>
+      </x:c>
+      <x:c r="F22" s="97" t="n">
+        <x:f>IF(Hackathons!S58="","",Hackathons!S58)</x:f>
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="G22" s="98" t="str">
+        <x:f>IF(Hackathons!T58="","",Hackathons!T58)</x:f>
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="H22" s="97" t="n">
+        <x:f>IF(Hackathons!U58="","",Hackathons!U58)</x:f>
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="I22" s="98" t="str">
+        <x:f>IF(Hackathons!V58="","",Hackathons!V58)</x:f>
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="J22" s="99" t="str">
+        <x:f>IF(Hackathons!W58="","",Hackathons!W58)</x:f>
+      </x:c>
+      <x:c r="K22" s="97" t="str">
+        <x:f>IF(Hackathons!X58="","",Hackathons!X58)</x:f>
+      </x:c>
+      <x:c r="L22" s="98" t="str">
+        <x:f>IF(Hackathons!Y58="","",Hackathons!Y58)</x:f>
+      </x:c>
+      <x:c r="M22" s="36" t="str">
+        <x:f>IF(Hackathons!Z58="","",Hackathons!Z58)</x:f>
+        <x:v>API credits</x:v>
+      </x:c>
+      <x:c r="N22" s="36" t="str">
+        <x:f>IF(Hackathons!AA58="","",Hackathons!AA58)</x:f>
+      </x:c>
+      <x:c r="O22" s="39" t="str">
+        <x:f>IF(Hackathons!AB58="","",Hackathons!AB58)</x:f>
+      </x:c>
+      <x:c r="P22" s="40" t="str">
+        <x:f>IF(Hackathons!AC58="","",Hackathons!AC58)</x:f>
+      </x:c>
+      <x:c r="Q22" s="36" t="str">
+        <x:f>IF(Hackathons!AD58="","",Hackathons!AD58)</x:f>
+      </x:c>
+      <x:c r="R22" s="98" t="str">
+        <x:f>IF(Hackathons!AE58="","",Hackathons!AE58)</x:f>
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="S22" s="98" t="str">
+        <x:f>IF(Hackathons!AF58="","",Hackathons!AF58)</x:f>
+        <x:v>Explicit cash; API credit value also tracked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="36" t="n">
+        <x:f>IF(Hackathons!A61="","",Hackathons!A61)</x:f>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B23" s="36" t="str">
+        <x:f>Hackathons!B61</x:f>
+        <x:v>Build Voice Agents with Speechmatics | TGB Buildathon 2026</x:v>
+      </x:c>
+      <x:c r="C23" s="36" t="str">
+        <x:f>IF(Hackathons!G61="","",Hackathons!G61)</x:f>
+        <x:v>2K USD Speechmatics Credits</x:v>
+      </x:c>
+      <x:c r="D23" s="36" t="str">
+        <x:f>IF(Hackathons!Q61="","",Hackathons!Q61)</x:f>
+        <x:v>Award</x:v>
+      </x:c>
+      <x:c r="E23" s="36" t="str">
+        <x:f>IF(Hackathons!R61="","",Hackathons!R61)</x:f>
+        <x:v>Speechmatics</x:v>
+      </x:c>
+      <x:c r="F23" s="97" t="str">
+        <x:f>IF(Hackathons!S61="","",Hackathons!S61)</x:f>
+      </x:c>
+      <x:c r="G23" s="98" t="str">
+        <x:f>IF(Hackathons!T61="","",Hackathons!T61)</x:f>
+      </x:c>
+      <x:c r="H23" s="97" t="n">
+        <x:f>IF(Hackathons!U61="","",Hackathons!U61)</x:f>
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="I23" s="98" t="str">
+        <x:f>IF(Hackathons!V61="","",Hackathons!V61)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J23" s="99" t="str">
+        <x:f>IF(Hackathons!W61="","",Hackathons!W61)</x:f>
+      </x:c>
+      <x:c r="K23" s="97" t="str">
+        <x:f>IF(Hackathons!X61="","",Hackathons!X61)</x:f>
+      </x:c>
+      <x:c r="L23" s="98" t="str">
+        <x:f>IF(Hackathons!Y61="","",Hackathons!Y61)</x:f>
+      </x:c>
+      <x:c r="M23" s="36" t="str">
+        <x:f>IF(Hackathons!Z61="","",Hackathons!Z61)</x:f>
+        <x:v>Speechmatics credits</x:v>
+      </x:c>
+      <x:c r="N23" s="36" t="str">
+        <x:f>IF(Hackathons!AA61="","",Hackathons!AA61)</x:f>
+      </x:c>
+      <x:c r="O23" s="39" t="str">
+        <x:f>IF(Hackathons!AB61="","",Hackathons!AB61)</x:f>
+      </x:c>
+      <x:c r="P23" s="40" t="str">
+        <x:f>IF(Hackathons!AC61="","",Hackathons!AC61)</x:f>
+      </x:c>
+      <x:c r="Q23" s="36" t="str">
+        <x:f>IF(Hackathons!AD61="","",Hackathons!AD61)</x:f>
+      </x:c>
+      <x:c r="R23" s="98" t="str">
+        <x:f>IF(Hackathons!AE61="","",Hackathons!AE61)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S23" s="98" t="str">
+        <x:f>IF(Hackathons!AF61="","",Hackathons!AF61)</x:f>
+        <x:v>USD-denominated credit value</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="36" t="n">
+        <x:f>IF(Hackathons!A62="","",Hackathons!A62)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B24" s="36" t="str">
+        <x:f>Hackathons!B62</x:f>
+        <x:v>Vercel Zero to Agent: Singapore (1 Hr Hackathon) 2026</x:v>
+      </x:c>
+      <x:c r="C24" s="36" t="str">
+        <x:f>IF(Hackathons!G62="","",Hackathons!G62)</x:f>
+        <x:v>v0 Sock</x:v>
+      </x:c>
+      <x:c r="D24" s="36" t="str">
+        <x:f>IF(Hackathons!Q62="","",Hackathons!Q62)</x:f>
+        <x:v>Award</x:v>
+      </x:c>
+      <x:c r="E24" s="36" t="str">
+        <x:f>IF(Hackathons!R62="","",Hackathons!R62)</x:f>
+        <x:v>v0</x:v>
+      </x:c>
+      <x:c r="F24" s="97" t="str">
+        <x:f>IF(Hackathons!S62="","",Hackathons!S62)</x:f>
+      </x:c>
+      <x:c r="G24" s="98" t="str">
+        <x:f>IF(Hackathons!T62="","",Hackathons!T62)</x:f>
+      </x:c>
+      <x:c r="H24" s="97" t="str">
+        <x:f>IF(Hackathons!U62="","",Hackathons!U62)</x:f>
+      </x:c>
+      <x:c r="I24" s="98" t="str">
+        <x:f>IF(Hackathons!V62="","",Hackathons!V62)</x:f>
+      </x:c>
+      <x:c r="J24" s="99" t="str">
+        <x:f>IF(Hackathons!W62="","",Hackathons!W62)</x:f>
+      </x:c>
+      <x:c r="K24" s="97" t="str">
+        <x:f>IF(Hackathons!X62="","",Hackathons!X62)</x:f>
+      </x:c>
+      <x:c r="L24" s="98" t="str">
+        <x:f>IF(Hackathons!Y62="","",Hackathons!Y62)</x:f>
+      </x:c>
+      <x:c r="M24" s="36" t="str">
+        <x:f>IF(Hackathons!Z62="","",Hackathons!Z62)</x:f>
+        <x:v>v0 Sock</x:v>
+      </x:c>
+      <x:c r="N24" s="36" t="str">
+        <x:f>IF(Hackathons!AA62="","",Hackathons!AA62)</x:f>
+        <x:v>v0 Sock</x:v>
+      </x:c>
+      <x:c r="O24" s="39" t="str">
+        <x:f>IF(Hackathons!AB62="","",Hackathons!AB62)</x:f>
+      </x:c>
+      <x:c r="P24" s="40" t="str">
+        <x:f>IF(Hackathons!AC62="","",Hackathons!AC62)</x:f>
+      </x:c>
+      <x:c r="Q24" s="36" t="str">
+        <x:f>IF(Hackathons!AD62="","",Hackathons!AD62)</x:f>
+      </x:c>
+      <x:c r="R24" s="98" t="str">
+        <x:f>IF(Hackathons!AE62="","",Hackathons!AE62)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S24" s="98" t="str">
+        <x:f>IF(Hackathons!AF62="","",Hackathons!AF62)</x:f>
+        <x:v>Physical item, not cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="36" t="n">
+        <x:f>IF(Hackathons!A67="","",Hackathons!A67)</x:f>
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="B25" s="36" t="str">
+        <x:f>Hackathons!B67</x:f>
+        <x:v>UCWS 2026 (Semi-Finals)</x:v>
+      </x:c>
+      <x:c r="C25" s="36" t="str">
+        <x:f>IF(Hackathons!G67="","",Hackathons!G67)</x:f>
+        <x:v>Top 20, 10K USD OpenAI Credits, 2K USD Gemini Cloud Credits</x:v>
+      </x:c>
+      <x:c r="D25" s="36" t="str">
+        <x:f>IF(Hackathons!Q67="","",Hackathons!Q67)</x:f>
+        <x:v>Top 20</x:v>
+      </x:c>
+      <x:c r="E25" s="36" t="str">
+        <x:f>IF(Hackathons!R67="","",Hackathons!R67)</x:f>
+      </x:c>
+      <x:c r="F25" s="97" t="str">
+        <x:f>IF(Hackathons!S67="","",Hackathons!S67)</x:f>
+      </x:c>
+      <x:c r="G25" s="98" t="str">
+        <x:f>IF(Hackathons!T67="","",Hackathons!T67)</x:f>
+      </x:c>
+      <x:c r="H25" s="97" t="n">
+        <x:f>IF(Hackathons!U67="","",Hackathons!U67)</x:f>
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="I25" s="98" t="str">
+        <x:f>IF(Hackathons!V67="","",Hackathons!V67)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J25" s="99" t="str">
+        <x:f>IF(Hackathons!W67="","",Hackathons!W67)</x:f>
+      </x:c>
+      <x:c r="K25" s="97" t="str">
+        <x:f>IF(Hackathons!X67="","",Hackathons!X67)</x:f>
+      </x:c>
+      <x:c r="L25" s="98" t="str">
+        <x:f>IF(Hackathons!Y67="","",Hackathons!Y67)</x:f>
+      </x:c>
+      <x:c r="M25" s="36" t="str">
+        <x:f>IF(Hackathons!Z67="","",Hackathons!Z67)</x:f>
+        <x:v>10K OpenAI credits; 2K Gemini Cloud credits</x:v>
+      </x:c>
+      <x:c r="N25" s="36" t="str">
+        <x:f>IF(Hackathons!AA67="","",Hackathons!AA67)</x:f>
+      </x:c>
+      <x:c r="O25" s="39" t="str">
+        <x:f>IF(Hackathons!AB67="","",Hackathons!AB67)</x:f>
+      </x:c>
+      <x:c r="P25" s="40" t="str">
+        <x:f>IF(Hackathons!AC67="","",Hackathons!AC67)</x:f>
+      </x:c>
+      <x:c r="Q25" s="36" t="str">
+        <x:f>IF(Hackathons!AD67="","",Hackathons!AD67)</x:f>
+      </x:c>
+      <x:c r="R25" s="98" t="str">
+        <x:f>IF(Hackathons!AE67="","",Hackathons!AE67)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S25" s="98" t="str">
+        <x:f>IF(Hackathons!AF67="","",Hackathons!AF67)</x:f>
+        <x:v>Credit value total combines two USD-denominated credits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="36" t="n">
+        <x:f>IF(Hackathons!A72="","",Hackathons!A72)</x:f>
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B26" s="36" t="str">
+        <x:f>Hackathons!B72</x:f>
+        <x:v>BUIDL_OPC_Hackathon_SG</x:v>
+      </x:c>
+      <x:c r="C26" s="36" t="str">
+        <x:f>IF(Hackathons!G72="","",Hackathons!G72)</x:f>
+        <x:v>4.5K USD AWS Credits</x:v>
+      </x:c>
+      <x:c r="D26" s="36" t="str">
+        <x:f>IF(Hackathons!Q72="","",Hackathons!Q72)</x:f>
+        <x:v>Award</x:v>
+      </x:c>
+      <x:c r="E26" s="36" t="str">
+        <x:f>IF(Hackathons!R72="","",Hackathons!R72)</x:f>
+        <x:v>AWS</x:v>
+      </x:c>
+      <x:c r="F26" s="97" t="str">
+        <x:f>IF(Hackathons!S72="","",Hackathons!S72)</x:f>
+      </x:c>
+      <x:c r="G26" s="98" t="str">
+        <x:f>IF(Hackathons!T72="","",Hackathons!T72)</x:f>
+      </x:c>
+      <x:c r="H26" s="97" t="n">
+        <x:f>IF(Hackathons!U72="","",Hackathons!U72)</x:f>
+        <x:v>4500</x:v>
+      </x:c>
+      <x:c r="I26" s="98" t="str">
+        <x:f>IF(Hackathons!V72="","",Hackathons!V72)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J26" s="99" t="str">
+        <x:f>IF(Hackathons!W72="","",Hackathons!W72)</x:f>
+      </x:c>
+      <x:c r="K26" s="97" t="str">
+        <x:f>IF(Hackathons!X72="","",Hackathons!X72)</x:f>
+      </x:c>
+      <x:c r="L26" s="98" t="str">
+        <x:f>IF(Hackathons!Y72="","",Hackathons!Y72)</x:f>
+      </x:c>
+      <x:c r="M26" s="36" t="str">
+        <x:f>IF(Hackathons!Z72="","",Hackathons!Z72)</x:f>
+        <x:v>AWS credits</x:v>
+      </x:c>
+      <x:c r="N26" s="36" t="str">
+        <x:f>IF(Hackathons!AA72="","",Hackathons!AA72)</x:f>
+      </x:c>
+      <x:c r="O26" s="39" t="str">
+        <x:f>IF(Hackathons!AB72="","",Hackathons!AB72)</x:f>
+      </x:c>
+      <x:c r="P26" s="40" t="str">
+        <x:f>IF(Hackathons!AC72="","",Hackathons!AC72)</x:f>
+      </x:c>
+      <x:c r="Q26" s="36" t="str">
+        <x:f>IF(Hackathons!AD72="","",Hackathons!AD72)</x:f>
+      </x:c>
+      <x:c r="R26" s="98" t="str">
+        <x:f>IF(Hackathons!AE72="","",Hackathons!AE72)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S26" s="98" t="str">
+        <x:f>IF(Hackathons!AF72="","",Hackathons!AF72)</x:f>
+        <x:v>USD-denominated credit value</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="36" t="n">
+        <x:f>IF(Hackathons!A76="","",Hackathons!A76)</x:f>
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B27" s="36" t="str">
+        <x:f>Hackathons!B76</x:f>
+        <x:v>One AI Hackathon 2026</x:v>
+      </x:c>
+      <x:c r="C27" s="36" t="str">
+        <x:f>IF(Hackathons!G76="","",Hackathons!G76)</x:f>
+        <x:v>Best Vertical Solution (Family Office Track), 2,000 Cybrdeck API credits (worth US$25)</x:v>
+      </x:c>
+      <x:c r="D27" s="36" t="str">
+        <x:f>IF(Hackathons!Q76="","",Hackathons!Q76)</x:f>
+        <x:v>Best Vertical Solution</x:v>
+      </x:c>
+      <x:c r="E27" s="36" t="str">
+        <x:f>IF(Hackathons!R76="","",Hackathons!R76)</x:f>
+        <x:v>Family Office Track</x:v>
+      </x:c>
+      <x:c r="F27" s="97" t="str">
+        <x:f>IF(Hackathons!S76="","",Hackathons!S76)</x:f>
+      </x:c>
+      <x:c r="G27" s="98" t="str">
+        <x:f>IF(Hackathons!T76="","",Hackathons!T76)</x:f>
+      </x:c>
+      <x:c r="H27" s="97" t="n">
+        <x:f>IF(Hackathons!U76="","",Hackathons!U76)</x:f>
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="I27" s="98" t="str">
+        <x:f>IF(Hackathons!V76="","",Hackathons!V76)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J27" s="99" t="str">
+        <x:f>IF(Hackathons!W76="","",Hackathons!W76)</x:f>
+      </x:c>
+      <x:c r="K27" s="97" t="str">
+        <x:f>IF(Hackathons!X76="","",Hackathons!X76)</x:f>
+      </x:c>
+      <x:c r="L27" s="98" t="str">
+        <x:f>IF(Hackathons!Y76="","",Hackathons!Y76)</x:f>
+      </x:c>
+      <x:c r="M27" s="36" t="str">
+        <x:f>IF(Hackathons!Z76="","",Hackathons!Z76)</x:f>
+        <x:v>2,000 Cybrdeck API credits</x:v>
+      </x:c>
+      <x:c r="N27" s="36" t="str">
+        <x:f>IF(Hackathons!AA76="","",Hackathons!AA76)</x:f>
+      </x:c>
+      <x:c r="O27" s="39" t="str">
+        <x:f>IF(Hackathons!AB76="","",Hackathons!AB76)</x:f>
+      </x:c>
+      <x:c r="P27" s="40" t="str">
+        <x:f>IF(Hackathons!AC76="","",Hackathons!AC76)</x:f>
+      </x:c>
+      <x:c r="Q27" s="36" t="str">
+        <x:f>IF(Hackathons!AD76="","",Hackathons!AD76)</x:f>
+      </x:c>
+      <x:c r="R27" s="98" t="str">
+        <x:f>IF(Hackathons!AE76="","",Hackathons!AE76)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S27" s="98" t="str">
+        <x:f>IF(Hackathons!AF76="","",Hackathons!AF76)</x:f>
+        <x:v>US$25 credit value, not cash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="36" t="n">
+        <x:f>IF(Hackathons!A80="","",Hackathons!A80)</x:f>
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="B28" s="36" t="str">
+        <x:f>Hackathons!B80</x:f>
+        <x:v>SG × SWK Friendship AI Business Design Hackathon</x:v>
+      </x:c>
+      <x:c r="C28" s="36" t="str">
+        <x:f>IF(Hackathons!G80="","",Hackathons!G80)</x:f>
+        <x:v>Trophy, First Runner Up, SG × Sarawak AI &amp; Design Hackathon 2026, 200 USD Kimi AI credits</x:v>
+      </x:c>
+      <x:c r="D28" s="36" t="str">
+        <x:f>IF(Hackathons!Q80="","",Hackathons!Q80)</x:f>
+        <x:v>First Runner Up</x:v>
+      </x:c>
+      <x:c r="E28" s="36" t="str">
+        <x:f>IF(Hackathons!R80="","",Hackathons!R80)</x:f>
+        <x:v>SG × Sarawak AI &amp; Design Hackathon 2026</x:v>
+      </x:c>
+      <x:c r="F28" s="97" t="str">
+        <x:f>IF(Hackathons!S80="","",Hackathons!S80)</x:f>
+      </x:c>
+      <x:c r="G28" s="98" t="str">
+        <x:f>IF(Hackathons!T80="","",Hackathons!T80)</x:f>
+      </x:c>
+      <x:c r="H28" s="97" t="n">
+        <x:f>IF(Hackathons!U80="","",Hackathons!U80)</x:f>
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I28" s="98" t="str">
+        <x:f>IF(Hackathons!V80="","",Hackathons!V80)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J28" s="99" t="str">
+        <x:f>IF(Hackathons!W80="","",Hackathons!W80)</x:f>
+      </x:c>
+      <x:c r="K28" s="97" t="str">
+        <x:f>IF(Hackathons!X80="","",Hackathons!X80)</x:f>
+      </x:c>
+      <x:c r="L28" s="98" t="str">
+        <x:f>IF(Hackathons!Y80="","",Hackathons!Y80)</x:f>
+      </x:c>
+      <x:c r="M28" s="36" t="str">
+        <x:f>IF(Hackathons!Z80="","",Hackathons!Z80)</x:f>
+        <x:v>Trophy; Kimi AI credits</x:v>
+      </x:c>
+      <x:c r="N28" s="36" t="str">
+        <x:f>IF(Hackathons!AA80="","",Hackathons!AA80)</x:f>
+        <x:v>Trophy</x:v>
+      </x:c>
+      <x:c r="O28" s="39" t="n">
+        <x:f>IF(Hackathons!AB80="","",Hackathons!AB80)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P28" s="40" t="str">
+        <x:f>IF(Hackathons!AC80="","",Hackathons!AC80)</x:f>
+      </x:c>
+      <x:c r="Q28" s="36" t="str">
+        <x:f>IF(Hackathons!AD80="","",Hackathons!AD80)</x:f>
+      </x:c>
+      <x:c r="R28" s="98" t="str">
+        <x:f>IF(Hackathons!AE80="","",Hackathons!AE80)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S28" s="98" t="str">
+        <x:f>IF(Hackathons!AF80="","",Hackathons!AF80)</x:f>
+        <x:v>Trophy excluded; credit value tracked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="36" t="n">
+        <x:f>IF(Hackathons!A81="","",Hackathons!A81)</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="B29" s="36" t="str">
+        <x:f>Hackathons!B81</x:f>
+        <x:v>GPT-6 Astra Hackathon: Singapore</x:v>
+      </x:c>
+      <x:c r="C29" s="36" t="str">
+        <x:f>IF(Hackathons!G81="","",Hackathons!G81)</x:f>
+        <x:v>Best use of GPT-Image-2.5, 5,000 USD OpenAI credits</x:v>
+      </x:c>
+      <x:c r="D29" s="36" t="str">
+        <x:f>IF(Hackathons!Q81="","",Hackathons!Q81)</x:f>
+        <x:v>Best Project</x:v>
+      </x:c>
+      <x:c r="E29" s="36" t="str">
+        <x:f>IF(Hackathons!R81="","",Hackathons!R81)</x:f>
+        <x:v>Best Use of GPT-Image-2.5</x:v>
+      </x:c>
+      <x:c r="F29" s="97" t="str">
+        <x:f>IF(Hackathons!S81="","",Hackathons!S81)</x:f>
+      </x:c>
+      <x:c r="G29" s="98" t="str">
+        <x:f>IF(Hackathons!T81="","",Hackathons!T81)</x:f>
+      </x:c>
+      <x:c r="H29" s="97" t="n">
+        <x:f>IF(Hackathons!U81="","",Hackathons!U81)</x:f>
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="I29" s="98" t="str">
+        <x:f>IF(Hackathons!V81="","",Hackathons!V81)</x:f>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J29" s="99" t="str">
+        <x:f>IF(Hackathons!W81="","",Hackathons!W81)</x:f>
+      </x:c>
+      <x:c r="K29" s="97" t="str">
+        <x:f>IF(Hackathons!X81="","",Hackathons!X81)</x:f>
+      </x:c>
+      <x:c r="L29" s="98" t="str">
+        <x:f>IF(Hackathons!Y81="","",Hackathons!Y81)</x:f>
+      </x:c>
+      <x:c r="M29" s="36" t="str">
+        <x:f>IF(Hackathons!Z81="","",Hackathons!Z81)</x:f>
+        <x:v>OpenAI credits</x:v>
+      </x:c>
+      <x:c r="N29" s="36" t="str">
+        <x:f>IF(Hackathons!AA81="","",Hackathons!AA81)</x:f>
+      </x:c>
+      <x:c r="O29" s="39" t="str">
+        <x:f>IF(Hackathons!AB81="","",Hackathons!AB81)</x:f>
+      </x:c>
+      <x:c r="P29" s="40" t="str">
+        <x:f>IF(Hackathons!AC81="","",Hackathons!AC81)</x:f>
+      </x:c>
+      <x:c r="Q29" s="36" t="str">
+        <x:f>IF(Hackathons!AD81="","",Hackathons!AD81)</x:f>
+      </x:c>
+      <x:c r="R29" s="98" t="str">
+        <x:f>IF(Hackathons!AE81="","",Hackathons!AE81)</x:f>
+        <x:v>Exclude</x:v>
+      </x:c>
+      <x:c r="S29" s="98" t="str">
+        <x:f>IF(Hackathons!AF81="","",Hackathons!AF81)</x:f>
+        <x:v>Credit value tracked</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:S1"/>
+    <x:mergeCell ref="A2:S2"/>
+    <x:mergeCell ref="A3:C3"/>
+    <x:mergeCell ref="D3:E3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7f5be77ed8d4f91"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Show dynamic prize money totals in detail view
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R412a67c1d73f4ddb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R7e608036e6544f79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R809ca3189425451b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Rd6fc6ff036414467"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R124a657e538a4d3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R71d217aecd414505"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R0441bb66b7f44a94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R1b3197785a3c4af9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R328ff04ba8bc4db6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R83c706e7409240bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="Raff842b5e0c94fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R688f47b25eef459c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2930,7 +2930,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="27">
+  <x:fills count="29">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -3062,6 +3062,16 @@
         <x:fgColor rgb="FFF3F6F9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -3126,7 +3136,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="107">
+  <x:cellXfs count="115">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3365,6 +3375,20 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="16" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="20" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="20" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="20" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -9420,10 +9444,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rbbb3a3ced68d4da4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R11329dca470543b8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R9cc7cdcca01d4159"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R7959174b22c14d3e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rbcd0254b458947d5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rdc95b2a17e624de0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rf5f8c46bf4374fcc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R1c25189e16c54152"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11001,12 +11025,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R924d8bbee39442ca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R33eefb0e748e46f4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R9ba917b27694442c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R8c85925d042e480e"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e9fee8640894264"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37fa3621bce54724"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11909,7 +11933,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b0235f68dc4d45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d7a373e70864afa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12805,6 +12829,26 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="E3" s="85"/>
+      <x:c r="F3" s="109" t="str">
+        <x:v>Cash-equivalent total (SGD)</x:v>
+      </x:c>
+      <x:c r="G3" s="109"/>
+      <x:c r="H3" s="109"/>
+      <x:c r="I3" s="114" t="n">
+        <x:f>SUMIFS(Hackathons!$S$2:$S$82,Hackathons!$T$2:$T$82,"SGD",Hackathons!$AE$2:$AE$82,"Yes")</x:f>
+        <x:v>2750</x:v>
+      </x:c>
+      <x:c r="J3" s="114"/>
+      <x:c r="L3" s="109" t="str">
+        <x:v>Cash-equivalent total (USD)</x:v>
+      </x:c>
+      <x:c r="M3" s="109"/>
+      <x:c r="N3" s="109"/>
+      <x:c r="O3" s="114" t="n">
+        <x:f>SUMIFS(Hackathons!$S$2:$S$82,Hackathons!$T$2:$T$82,"USD",Hackathons!$AE$2:$AE$82,"Yes")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P3" s="114"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="90" t="str">
@@ -14572,10 +14616,14 @@
     <x:mergeCell ref="A2:S2"/>
     <x:mergeCell ref="A3:C3"/>
     <x:mergeCell ref="D3:E3"/>
+    <x:mergeCell ref="F3:H3"/>
+    <x:mergeCell ref="I3:J3"/>
+    <x:mergeCell ref="L3:N3"/>
+    <x:mergeCell ref="O3:P3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7f5be77ed8d4f91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c47cef3f8e34d45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Include funding in prize value summary
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R0441bb66b7f44a94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R1b3197785a3c4af9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R328ff04ba8bc4db6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R83c706e7409240bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="Raff842b5e0c94fc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R688f47b25eef459c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rb0dc44d12c774e35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R38a5ac30b6974755"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R63d0098a306f4848"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R4c210b9cb61940ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R1cc5b506172b4377"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Rc20134a26691440f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2786,7 +2786,7 @@
     <x:numFmt numFmtId="200" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="25">
+  <x:fonts count="26">
     <x:font>
       <x:sz val="12"/>
       <x:color theme="1"/>
@@ -2929,8 +2929,13 @@
       <x:color rgb="FF17324D"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:sz val="12"/>
+      <x:color rgb="FF17324D"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="29">
+  <x:fills count="45">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -3072,6 +3077,86 @@
         <x:fgColor rgb="FFD9EAD3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -3136,7 +3221,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="115">
+  <x:cellXfs count="191">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3390,6 +3475,154 @@
     <x:xf numFmtId="200" fontId="20" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="20" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="20" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="20" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="20" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="20" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="20" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="25" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="25" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="20" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="20" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="25" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="25" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="20" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="20" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Hyperlink" xfId="1"/>
@@ -9444,10 +9677,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rbcd0254b458947d5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rdc95b2a17e624de0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rf5f8c46bf4374fcc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R1c25189e16c54152"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R5070ae83fdba46a8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rf6145fccf6464526"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rdc91e798dbe9420e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R2798f45ced464a17"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11025,12 +11258,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R9ba917b27694442c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R8c85925d042e480e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R737600c99c214822"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R9dbbb8d1857c4ce5"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37fa3621bce54724"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f41672e21ea4218"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11933,7 +12166,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d7a373e70864afa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d55760c47b541f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12606,7 +12839,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="61" t="str">
-        <x:v>Includes vouchers you chose to treat as cash-equivalent. Funding is intentionally excluded.</x:v>
+        <x:v>Includes vouchers you chose to treat as cash-equivalent. Funding is shown separately and included in the all-tracked totals below.</x:v>
       </x:c>
       <x:c r="B8" s="61"/>
       <x:c r="C8" s="61"/>
@@ -12728,13 +12961,26 @@
         <x:v>Known subscription value</x:v>
       </x:c>
     </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="64" t="str">
+        <x:v>Funding</x:v>
+      </x:c>
+      <x:c r="B17" s="64" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="C17" s="174" t="n">
+        <x:f>SUMIFS(Hackathons!$AC$2:$AC$82,Hackathons!$AD$2:$AD$82,B17)</x:f>
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="D17" s="64" t="str">
+        <x:v>Seed funding / grants</x:v>
+      </x:c>
+    </x:row>
     <x:row r="18">
-      <x:c r="A18" s="54" t="str">
-        <x:v>How to maintain this tab</x:v>
-      </x:c>
-      <x:c r="B18" s="54"/>
-      <x:c r="C18" s="54"/>
-      <x:c r="D18" s="54"/>
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
       <x:c r="E18" s="54"/>
       <x:c r="F18" s="54"/>
       <x:c r="G18" s="54"/>
@@ -12745,12 +12991,107 @@
       <x:c r="L18" s="54"/>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
-      <x:c r="A19" s="57" t="str">
-        <x:v>1. Update the yellow structured fields on Hackathons (columns S–Y and AE).  2. Use Cash-equivalent Treatment = Yes only for prizes you want counted as money.  3. Keep credit and subscription amounts in their original currencies; this dashboard deliberately does not convert currencies.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="22" customHeight="1"/>
-    <x:row r="21" ht="22" customHeight="1"/>
+      <x:c r="A19"/>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" s="178" t="str">
+        <x:v>All tracked monetary value</x:v>
+      </x:c>
+      <x:c r="B20" s="178" t="str">
+        <x:v>Currency</x:v>
+      </x:c>
+      <x:c r="C20" s="178" t="str">
+        <x:v>Amount</x:v>
+      </x:c>
+      <x:c r="D20" s="178" t="str">
+        <x:v>Includes</x:v>
+      </x:c>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
+      <x:c r="G20"/>
+      <x:c r="H20"/>
+      <x:c r="I20"/>
+      <x:c r="J20"/>
+      <x:c r="K20"/>
+      <x:c r="L20"/>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="181" t="str">
+        <x:v>All prize value</x:v>
+      </x:c>
+      <x:c r="B21" s="181" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="C21" s="185" t="n">
+        <x:f>SUMIFS(Hackathons!$S$2:$S$82,Hackathons!$T$2:$T$82,"SGD",Hackathons!$AE$2:$AE$82,"Yes")+SUMIFS(Hackathons!$U$2:$U$82,Hackathons!$V$2:$V$82,"SGD")+SUMIFS(Hackathons!$X$2:$X$82,Hackathons!$Y$2:$Y$82,"SGD")+SUMIFS(Hackathons!$AC$2:$AC$82,Hackathons!$AD$2:$AD$82,"SGD")</x:f>
+        <x:v>21135</x:v>
+      </x:c>
+      <x:c r="D21" s="181" t="str">
+        <x:v>Cash, credits, subscriptions, funding</x:v>
+      </x:c>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
+      <x:c r="H21"/>
+      <x:c r="I21"/>
+      <x:c r="J21"/>
+      <x:c r="K21"/>
+      <x:c r="L21"/>
+    </x:row>
+    <x:row r="22" ht="25" customHeight="1">
+      <x:c r="A22" s="181" t="str">
+        <x:v>All prize value</x:v>
+      </x:c>
+      <x:c r="B22" s="181" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="C22" s="185" t="n">
+        <x:f>SUMIFS(Hackathons!$S$2:$S$82,Hackathons!$T$2:$T$82,"USD",Hackathons!$AE$2:$AE$82,"Yes")+SUMIFS(Hackathons!$U$2:$U$82,Hackathons!$V$2:$V$82,"USD")+SUMIFS(Hackathons!$X$2:$X$82,Hackathons!$Y$2:$Y$82,"USD")+SUMIFS(Hackathons!$AC$2:$AC$82,Hackathons!$AD$2:$AD$82,"USD")</x:f>
+        <x:v>126414</x:v>
+      </x:c>
+      <x:c r="D22" s="181" t="str">
+        <x:v>Cash, credits, subscriptions, funding</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="25" customHeight="1">
+      <x:c r="A23" s="189" t="str">
+        <x:v>This combines money-like prizes, credits, subscriptions, and funding in the same currency. Trophies and physical assets are excluded because they have no recorded monetary value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24"/>
+      <x:c r="B24"/>
+      <x:c r="C24"/>
+      <x:c r="D24"/>
+      <x:c r="E24"/>
+      <x:c r="F24"/>
+      <x:c r="G24"/>
+      <x:c r="H24"/>
+      <x:c r="I24"/>
+      <x:c r="J24"/>
+      <x:c r="K24"/>
+      <x:c r="L24"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="190" t="str">
+        <x:v>How to maintain this tab</x:v>
+      </x:c>
+      <x:c r="B25" s="190"/>
+      <x:c r="C25" s="190"/>
+      <x:c r="D25" s="190"/>
+      <x:c r="E25" s="190"/>
+      <x:c r="F25" s="190"/>
+      <x:c r="G25" s="190"/>
+      <x:c r="H25" s="190"/>
+      <x:c r="I25" s="190"/>
+      <x:c r="J25" s="190"/>
+      <x:c r="K25" s="190"/>
+      <x:c r="L25" s="190"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="57" t="str">
+        <x:v>1. Update the yellow structured fields on Hackathons (columns S–Y and AE).  2. Record seed funding or grants in columns AC–AD.  3. Keep all values in their original currencies; this dashboard deliberately does not convert currencies.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:L1"/>
@@ -12774,7 +13115,9 @@
     <x:mergeCell ref="J8:K8"/>
     <x:mergeCell ref="A10:L10"/>
     <x:mergeCell ref="A18:L18"/>
-    <x:mergeCell ref="A19:L21"/>
+    <x:mergeCell ref="A23:L23"/>
+    <x:mergeCell ref="A25:L25"/>
+    <x:mergeCell ref="A26:L28"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -14623,7 +14966,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c47cef3f8e34d45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbc23ba9da984bb4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Standardize award summaries in prize details
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rb0dc44d12c774e35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R38a5ac30b6974755"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R63d0098a306f4848"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R4c210b9cb61940ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R1cc5b506172b4377"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Rc20134a26691440f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R9a70d0e706b34bc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R8703e043c74740f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R02a5fff09ec54696"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R40a1a6b6bd544efa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="Rc05e35a6d2f242b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R81a1cb0d3b544b30"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9677,10 +9677,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R5070ae83fdba46a8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rf6145fccf6464526"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rdc91e798dbe9420e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R2798f45ced464a17"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R0f570abde045437d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R61455f82b54b4990"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R302eef6afc894f03"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Ra8b66eacbb77463f"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11258,12 +11258,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R737600c99c214822"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R9dbbb8d1857c4ce5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Re264cfb16f194e64"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R0a98f61dcb194104"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f41672e21ea4218"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1057523a1334982"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12166,7 +12166,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d55760c47b541f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2931dda0bada466c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13132,7 +13132,7 @@
   <x:cols>
     <x:col min="1" max="1" width="7" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
@@ -13158,7 +13158,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="106" t="str">
-        <x:v>One row per currently classified award or prize record. Each value is linked to the Hackathons tab, so corrections there update this detail view automatically.</x:v>
+        <x:v>One row per currently classified award or prize record. The Award summary is standardized from the linked fields on Hackathons; the original raw text remains preserved there.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -13201,7 +13201,7 @@
         <x:v>Hackathon</x:v>
       </x:c>
       <x:c r="C4" s="90" t="str">
-        <x:v>Original award</x:v>
+        <x:v>Award summary</x:v>
       </x:c>
       <x:c r="D4" s="90" t="str">
         <x:v>Award type</x:v>
@@ -13262,8 +13262,8 @@
         <x:v>Education Technology Hackathon</x:v>
       </x:c>
       <x:c r="C5" s="36" t="str">
-        <x:f>IF(Hackathons!G2="","",Hackathons!G2)</x:f>
-        <x:v>First Place, 18k SGD seed Funding</x:v>
+        <x:f>D5&amp;IF(E5&lt;&gt;""," — "&amp;E5,"")&amp;IF(F5&lt;&gt;"",IF(M5&lt;&gt;"","","; "&amp;IF(G5="SGD","S$",IF(G5="USD","US$",G5&amp;" "))&amp;TEXT(F5,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H5&lt;&gt;"","; "&amp;IF(I5="SGD","S$",IF(I5="USD","US$",I5&amp;" "))&amp;TEXT(H5,"#,##0")&amp;" credits","")&amp;IF(J5&lt;&gt;"","; "&amp;TEXT(J5,"#,##0")&amp;" subscription(s)"&amp;IF(K5&lt;&gt;""," ("&amp;IF(L5="USD","US$",IF(L5="SGD","S$",L5&amp;" "))&amp;TEXT(K5,"#,##0")&amp;")",""),"")&amp;IF(M5&lt;&gt;"","; "&amp;M5,"")&amp;IF(O5&lt;&gt;"","; "&amp;TEXT(O5,"#,##0")&amp;" trophy/trophies","")&amp;IF(P5&lt;&gt;"","; "&amp;IF(Q5="SGD","S$",IF(Q5="USD","US$",Q5&amp;" "))&amp;TEXT(P5,"#,##0")&amp;" funding","")</x:f>
+        <x:v>1st Place; S$18,000 funding</x:v>
       </x:c>
       <x:c r="D5" s="36" t="str">
         <x:f>IF(Hackathons!Q2="","",Hackathons!Q2)</x:f>
@@ -13329,8 +13329,8 @@
         <x:v>DataDriven Hackathon 2016</x:v>
       </x:c>
       <x:c r="C6" s="36" t="str">
-        <x:f>IF(Hackathons!G4="","",Hackathons!G4)</x:f>
-        <x:v>*rated best project</x:v>
+        <x:f>D6&amp;IF(E6&lt;&gt;""," — "&amp;E6,"")&amp;IF(F6&lt;&gt;"",IF(M6&lt;&gt;"","","; "&amp;IF(G6="SGD","S$",IF(G6="USD","US$",G6&amp;" "))&amp;TEXT(F6,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H6&lt;&gt;"","; "&amp;IF(I6="SGD","S$",IF(I6="USD","US$",I6&amp;" "))&amp;TEXT(H6,"#,##0")&amp;" credits","")&amp;IF(J6&lt;&gt;"","; "&amp;TEXT(J6,"#,##0")&amp;" subscription(s)"&amp;IF(K6&lt;&gt;""," ("&amp;IF(L6="USD","US$",IF(L6="SGD","S$",L6&amp;" "))&amp;TEXT(K6,"#,##0")&amp;")",""),"")&amp;IF(M6&lt;&gt;"","; "&amp;M6,"")&amp;IF(O6&lt;&gt;"","; "&amp;TEXT(O6,"#,##0")&amp;" trophy/trophies","")&amp;IF(P6&lt;&gt;"","; "&amp;IF(Q6="SGD","S$",IF(Q6="USD","US$",Q6&amp;" "))&amp;TEXT(P6,"#,##0")&amp;" funding","")</x:f>
+        <x:v>Best Project — Rated best project</x:v>
       </x:c>
       <x:c r="D6" s="36" t="str">
         <x:f>IF(Hackathons!Q4="","",Hackathons!Q4)</x:f>
@@ -13395,8 +13395,8 @@
         <x:v>Fintech Festival Hackathon 2016</x:v>
       </x:c>
       <x:c r="C7" s="36" t="str">
-        <x:f>IF(Hackathons!G5="","",Hackathons!G5)</x:f>
-        <x:v>1st Place, Best Use of IBM Bluemix, US$100,000 IBM Bluemix Credits, SmartWatch</x:v>
+        <x:f>D7&amp;IF(E7&lt;&gt;""," — "&amp;E7,"")&amp;IF(F7&lt;&gt;"",IF(M7&lt;&gt;"","","; "&amp;IF(G7="SGD","S$",IF(G7="USD","US$",G7&amp;" "))&amp;TEXT(F7,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H7&lt;&gt;"","; "&amp;IF(I7="SGD","S$",IF(I7="USD","US$",I7&amp;" "))&amp;TEXT(H7,"#,##0")&amp;" credits","")&amp;IF(J7&lt;&gt;"","; "&amp;TEXT(J7,"#,##0")&amp;" subscription(s)"&amp;IF(K7&lt;&gt;""," ("&amp;IF(L7="USD","US$",IF(L7="SGD","S$",L7&amp;" "))&amp;TEXT(K7,"#,##0")&amp;")",""),"")&amp;IF(M7&lt;&gt;"","; "&amp;M7,"")&amp;IF(O7&lt;&gt;"","; "&amp;TEXT(O7,"#,##0")&amp;" trophy/trophies","")&amp;IF(P7&lt;&gt;"","; "&amp;IF(Q7="SGD","S$",IF(Q7="USD","US$",Q7&amp;" "))&amp;TEXT(P7,"#,##0")&amp;" funding","")</x:f>
+        <x:v>1st Place — Best Use of IBM Bluemix; US$100,000 credits; IBM Bluemix credits; SmartWatch</x:v>
       </x:c>
       <x:c r="D7" s="36" t="str">
         <x:f>IF(Hackathons!Q5="","",Hackathons!Q5)</x:f>
@@ -13465,8 +13465,8 @@
         <x:v>SO.IMPACT Bootcamp 2017</x:v>
       </x:c>
       <x:c r="C8" s="36" t="str">
-        <x:f>IF(Hackathons!G7="","",Hackathons!G7)</x:f>
-        <x:v>Shortlisted for top 10</x:v>
+        <x:f>D8&amp;IF(E8&lt;&gt;""," — "&amp;E8,"")&amp;IF(F8&lt;&gt;"",IF(M8&lt;&gt;"","","; "&amp;IF(G8="SGD","S$",IF(G8="USD","US$",G8&amp;" "))&amp;TEXT(F8,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H8&lt;&gt;"","; "&amp;IF(I8="SGD","S$",IF(I8="USD","US$",I8&amp;" "))&amp;TEXT(H8,"#,##0")&amp;" credits","")&amp;IF(J8&lt;&gt;"","; "&amp;TEXT(J8,"#,##0")&amp;" subscription(s)"&amp;IF(K8&lt;&gt;""," ("&amp;IF(L8="USD","US$",IF(L8="SGD","S$",L8&amp;" "))&amp;TEXT(K8,"#,##0")&amp;")",""),"")&amp;IF(M8&lt;&gt;"","; "&amp;M8,"")&amp;IF(O8&lt;&gt;"","; "&amp;TEXT(O8,"#,##0")&amp;" trophy/trophies","")&amp;IF(P8&lt;&gt;"","; "&amp;IF(Q8="SGD","S$",IF(Q8="USD","US$",Q8&amp;" "))&amp;TEXT(P8,"#,##0")&amp;" funding","")</x:f>
+        <x:v>Top 10</x:v>
       </x:c>
       <x:c r="D8" s="36" t="str">
         <x:f>IF(Hackathons!Q7="","",Hackathons!Q7)</x:f>
@@ -13530,8 +13530,8 @@
         <x:v>DataDriven Hackathon 2017</x:v>
       </x:c>
       <x:c r="C9" s="36" t="str">
-        <x:f>IF(Hackathons!G11="","",Hackathons!G11)</x:f>
-        <x:v>*rated best project </x:v>
+        <x:f>D9&amp;IF(E9&lt;&gt;""," — "&amp;E9,"")&amp;IF(F9&lt;&gt;"",IF(M9&lt;&gt;"","","; "&amp;IF(G9="SGD","S$",IF(G9="USD","US$",G9&amp;" "))&amp;TEXT(F9,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H9&lt;&gt;"","; "&amp;IF(I9="SGD","S$",IF(I9="USD","US$",I9&amp;" "))&amp;TEXT(H9,"#,##0")&amp;" credits","")&amp;IF(J9&lt;&gt;"","; "&amp;TEXT(J9,"#,##0")&amp;" subscription(s)"&amp;IF(K9&lt;&gt;""," ("&amp;IF(L9="USD","US$",IF(L9="SGD","S$",L9&amp;" "))&amp;TEXT(K9,"#,##0")&amp;")",""),"")&amp;IF(M9&lt;&gt;"","; "&amp;M9,"")&amp;IF(O9&lt;&gt;"","; "&amp;TEXT(O9,"#,##0")&amp;" trophy/trophies","")&amp;IF(P9&lt;&gt;"","; "&amp;IF(Q9="SGD","S$",IF(Q9="USD","US$",Q9&amp;" "))&amp;TEXT(P9,"#,##0")&amp;" funding","")</x:f>
+        <x:v>Best Project — Rated best project</x:v>
       </x:c>
       <x:c r="D9" s="36" t="str">
         <x:f>IF(Hackathons!Q11="","",Hackathons!Q11)</x:f>
@@ -13596,8 +13596,8 @@
         <x:v>#SPSEC SP Hackathon 2018</x:v>
       </x:c>
       <x:c r="C10" s="36" t="str">
-        <x:f>IF(Hackathons!G15="","",Hackathons!G15)</x:f>
-        <x:v>3rd Place, $100 Capitaland voucher</x:v>
+        <x:f>D10&amp;IF(E10&lt;&gt;""," — "&amp;E10,"")&amp;IF(F10&lt;&gt;"",IF(M10&lt;&gt;"","","; "&amp;IF(G10="SGD","S$",IF(G10="USD","US$",G10&amp;" "))&amp;TEXT(F10,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H10&lt;&gt;"","; "&amp;IF(I10="SGD","S$",IF(I10="USD","US$",I10&amp;" "))&amp;TEXT(H10,"#,##0")&amp;" credits","")&amp;IF(J10&lt;&gt;"","; "&amp;TEXT(J10,"#,##0")&amp;" subscription(s)"&amp;IF(K10&lt;&gt;""," ("&amp;IF(L10="USD","US$",IF(L10="SGD","S$",L10&amp;" "))&amp;TEXT(K10,"#,##0")&amp;")",""),"")&amp;IF(M10&lt;&gt;"","; "&amp;M10,"")&amp;IF(O10&lt;&gt;"","; "&amp;TEXT(O10,"#,##0")&amp;" trophy/trophies","")&amp;IF(P10&lt;&gt;"","; "&amp;IF(Q10="SGD","S$",IF(Q10="USD","US$",Q10&amp;" "))&amp;TEXT(P10,"#,##0")&amp;" funding","")</x:f>
+        <x:v>3rd Place; S$100 Capitaland voucher</x:v>
       </x:c>
       <x:c r="D10" s="36" t="str">
         <x:f>IF(Hackathons!Q15="","",Hackathons!Q15)</x:f>
@@ -13664,8 +13664,8 @@
         <x:v>#Mosque-Tech Challenge 2018</x:v>
       </x:c>
       <x:c r="C11" s="36" t="str">
-        <x:f>IF(Hackathons!G18="","",Hackathons!G18)</x:f>
-        <x:v>2nd Place, $600 cash</x:v>
+        <x:f>D11&amp;IF(E11&lt;&gt;""," — "&amp;E11,"")&amp;IF(F11&lt;&gt;"",IF(M11&lt;&gt;"","","; "&amp;IF(G11="SGD","S$",IF(G11="USD","US$",G11&amp;" "))&amp;TEXT(F11,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H11&lt;&gt;"","; "&amp;IF(I11="SGD","S$",IF(I11="USD","US$",I11&amp;" "))&amp;TEXT(H11,"#,##0")&amp;" credits","")&amp;IF(J11&lt;&gt;"","; "&amp;TEXT(J11,"#,##0")&amp;" subscription(s)"&amp;IF(K11&lt;&gt;""," ("&amp;IF(L11="USD","US$",IF(L11="SGD","S$",L11&amp;" "))&amp;TEXT(K11,"#,##0")&amp;")",""),"")&amp;IF(M11&lt;&gt;"","; "&amp;M11,"")&amp;IF(O11&lt;&gt;"","; "&amp;TEXT(O11,"#,##0")&amp;" trophy/trophies","")&amp;IF(P11&lt;&gt;"","; "&amp;IF(Q11="SGD","S$",IF(Q11="USD","US$",Q11&amp;" "))&amp;TEXT(P11,"#,##0")&amp;" funding","")</x:f>
+        <x:v>2nd Place; S$600 cash / voucher</x:v>
       </x:c>
       <x:c r="D11" s="36" t="str">
         <x:f>IF(Hackathons!Q18="","",Hackathons!Q18)</x:f>
@@ -13731,8 +13731,8 @@
         <x:v>#Mosque Hackathon 2019</x:v>
       </x:c>
       <x:c r="C12" s="36" t="str">
-        <x:f>IF(Hackathons!G26="","",Hackathons!G26)</x:f>
-        <x:v>3rd Place, $500 SGD cash</x:v>
+        <x:f>D12&amp;IF(E12&lt;&gt;""," — "&amp;E12,"")&amp;IF(F12&lt;&gt;"",IF(M12&lt;&gt;"","","; "&amp;IF(G12="SGD","S$",IF(G12="USD","US$",G12&amp;" "))&amp;TEXT(F12,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H12&lt;&gt;"","; "&amp;IF(I12="SGD","S$",IF(I12="USD","US$",I12&amp;" "))&amp;TEXT(H12,"#,##0")&amp;" credits","")&amp;IF(J12&lt;&gt;"","; "&amp;TEXT(J12,"#,##0")&amp;" subscription(s)"&amp;IF(K12&lt;&gt;""," ("&amp;IF(L12="USD","US$",IF(L12="SGD","S$",L12&amp;" "))&amp;TEXT(K12,"#,##0")&amp;")",""),"")&amp;IF(M12&lt;&gt;"","; "&amp;M12,"")&amp;IF(O12&lt;&gt;"","; "&amp;TEXT(O12,"#,##0")&amp;" trophy/trophies","")&amp;IF(P12&lt;&gt;"","; "&amp;IF(Q12="SGD","S$",IF(Q12="USD","US$",Q12&amp;" "))&amp;TEXT(P12,"#,##0")&amp;" funding","")</x:f>
+        <x:v>3rd Place; S$500 cash / voucher</x:v>
       </x:c>
       <x:c r="D12" s="36" t="str">
         <x:f>IF(Hackathons!Q26="","",Hackathons!Q26)</x:f>
@@ -13798,8 +13798,8 @@
         <x:v>ICP Ideathon 2023</x:v>
       </x:c>
       <x:c r="C13" s="36" t="str">
-        <x:f>IF(Hackathons!G34="","",Hackathons!G34)</x:f>
-        <x:v>3rd Prize (S$250 Cash)</x:v>
+        <x:f>D13&amp;IF(E13&lt;&gt;""," — "&amp;E13,"")&amp;IF(F13&lt;&gt;"",IF(M13&lt;&gt;"","","; "&amp;IF(G13="SGD","S$",IF(G13="USD","US$",G13&amp;" "))&amp;TEXT(F13,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H13&lt;&gt;"","; "&amp;IF(I13="SGD","S$",IF(I13="USD","US$",I13&amp;" "))&amp;TEXT(H13,"#,##0")&amp;" credits","")&amp;IF(J13&lt;&gt;"","; "&amp;TEXT(J13,"#,##0")&amp;" subscription(s)"&amp;IF(K13&lt;&gt;""," ("&amp;IF(L13="USD","US$",IF(L13="SGD","S$",L13&amp;" "))&amp;TEXT(K13,"#,##0")&amp;")",""),"")&amp;IF(M13&lt;&gt;"","; "&amp;M13,"")&amp;IF(O13&lt;&gt;"","; "&amp;TEXT(O13,"#,##0")&amp;" trophy/trophies","")&amp;IF(P13&lt;&gt;"","; "&amp;IF(Q13="SGD","S$",IF(Q13="USD","US$",Q13&amp;" "))&amp;TEXT(P13,"#,##0")&amp;" funding","")</x:f>
+        <x:v>3rd Prize; S$250 cash / voucher</x:v>
       </x:c>
       <x:c r="D13" s="36" t="str">
         <x:f>IF(Hackathons!Q34="","",Hackathons!Q34)</x:f>
@@ -13865,8 +13865,8 @@
         <x:v>Mosque Tech Challenge 2025</x:v>
       </x:c>
       <x:c r="C14" s="36" t="str">
-        <x:f>IF(Hackathons!G36="","",Hackathons!G36)</x:f>
-        <x:v>2nd Prize (S$1,000 Cash)</x:v>
+        <x:f>D14&amp;IF(E14&lt;&gt;""," — "&amp;E14,"")&amp;IF(F14&lt;&gt;"",IF(M14&lt;&gt;"","","; "&amp;IF(G14="SGD","S$",IF(G14="USD","US$",G14&amp;" "))&amp;TEXT(F14,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H14&lt;&gt;"","; "&amp;IF(I14="SGD","S$",IF(I14="USD","US$",I14&amp;" "))&amp;TEXT(H14,"#,##0")&amp;" credits","")&amp;IF(J14&lt;&gt;"","; "&amp;TEXT(J14,"#,##0")&amp;" subscription(s)"&amp;IF(K14&lt;&gt;""," ("&amp;IF(L14="USD","US$",IF(L14="SGD","S$",L14&amp;" "))&amp;TEXT(K14,"#,##0")&amp;")",""),"")&amp;IF(M14&lt;&gt;"","; "&amp;M14,"")&amp;IF(O14&lt;&gt;"","; "&amp;TEXT(O14,"#,##0")&amp;" trophy/trophies","")&amp;IF(P14&lt;&gt;"","; "&amp;IF(Q14="SGD","S$",IF(Q14="USD","US$",Q14&amp;" "))&amp;TEXT(P14,"#,##0")&amp;" funding","")</x:f>
+        <x:v>2nd Prize; S$1,000 cash / voucher</x:v>
       </x:c>
       <x:c r="D14" s="36" t="str">
         <x:f>IF(Hackathons!Q36="","",Hackathons!Q36)</x:f>
@@ -13932,8 +13932,8 @@
         <x:v>OOJU X Manus.AI Hackathon 2025</x:v>
       </x:c>
       <x:c r="C15" s="36" t="str">
-        <x:f>IF(Hackathons!G39="","",Hackathons!G39)</x:f>
-        <x:v>2nd Prize (Manus Pro Subscription)</x:v>
+        <x:f>D15&amp;IF(E15&lt;&gt;""," — "&amp;E15,"")&amp;IF(F15&lt;&gt;"",IF(M15&lt;&gt;"","","; "&amp;IF(G15="SGD","S$",IF(G15="USD","US$",G15&amp;" "))&amp;TEXT(F15,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H15&lt;&gt;"","; "&amp;IF(I15="SGD","S$",IF(I15="USD","US$",I15&amp;" "))&amp;TEXT(H15,"#,##0")&amp;" credits","")&amp;IF(J15&lt;&gt;"","; "&amp;TEXT(J15,"#,##0")&amp;" subscription(s)"&amp;IF(K15&lt;&gt;""," ("&amp;IF(L15="USD","US$",IF(L15="SGD","S$",L15&amp;" "))&amp;TEXT(K15,"#,##0")&amp;")",""),"")&amp;IF(M15&lt;&gt;"","; "&amp;M15,"")&amp;IF(O15&lt;&gt;"","; "&amp;TEXT(O15,"#,##0")&amp;" trophy/trophies","")&amp;IF(P15&lt;&gt;"","; "&amp;IF(Q15="SGD","S$",IF(Q15="USD","US$",Q15&amp;" "))&amp;TEXT(P15,"#,##0")&amp;" funding","")</x:f>
+        <x:v>2nd Prize; 1 subscription(s) (US$39); Manus Pro subscription</x:v>
       </x:c>
       <x:c r="D15" s="36" t="str">
         <x:f>IF(Hackathons!Q39="","",Hackathons!Q39)</x:f>
@@ -14001,8 +14001,8 @@
         <x:v>Sarawak AI Hackathon 2025</x:v>
       </x:c>
       <x:c r="C16" s="36" t="str">
-        <x:f>IF(Hackathons!G41="","",Hackathons!G41)</x:f>
-        <x:v>Throphy, Best Novel Hackathon Finisher</x:v>
+        <x:f>D16&amp;IF(E16&lt;&gt;""," — "&amp;E16,"")&amp;IF(F16&lt;&gt;"",IF(M16&lt;&gt;"","","; "&amp;IF(G16="SGD","S$",IF(G16="USD","US$",G16&amp;" "))&amp;TEXT(F16,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H16&lt;&gt;"","; "&amp;IF(I16="SGD","S$",IF(I16="USD","US$",I16&amp;" "))&amp;TEXT(H16,"#,##0")&amp;" credits","")&amp;IF(J16&lt;&gt;"","; "&amp;TEXT(J16,"#,##0")&amp;" subscription(s)"&amp;IF(K16&lt;&gt;""," ("&amp;IF(L16="USD","US$",IF(L16="SGD","S$",L16&amp;" "))&amp;TEXT(K16,"#,##0")&amp;")",""),"")&amp;IF(M16&lt;&gt;"","; "&amp;M16,"")&amp;IF(O16&lt;&gt;"","; "&amp;TEXT(O16,"#,##0")&amp;" trophy/trophies","")&amp;IF(P16&lt;&gt;"","; "&amp;IF(Q16="SGD","S$",IF(Q16="USD","US$",Q16&amp;" "))&amp;TEXT(P16,"#,##0")&amp;" funding","")</x:f>
+        <x:v>Best Finisher — Novel Hackathon; Trophy; 1 trophy/trophies</x:v>
       </x:c>
       <x:c r="D16" s="36" t="str">
         <x:f>IF(Hackathons!Q41="","",Hackathons!Q41)</x:f>
@@ -14070,8 +14070,8 @@
         <x:v>Nosana Hackathon 2025</x:v>
       </x:c>
       <x:c r="C17" s="36" t="str">
-        <x:f>IF(Hackathons!G43="","",Hackathons!G43)</x:f>
-        <x:v>1st Prize, $500 Nosana Cloud Credit</x:v>
+        <x:f>D17&amp;IF(E17&lt;&gt;""," — "&amp;E17,"")&amp;IF(F17&lt;&gt;"",IF(M17&lt;&gt;"","","; "&amp;IF(G17="SGD","S$",IF(G17="USD","US$",G17&amp;" "))&amp;TEXT(F17,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H17&lt;&gt;"","; "&amp;IF(I17="SGD","S$",IF(I17="USD","US$",I17&amp;" "))&amp;TEXT(H17,"#,##0")&amp;" credits","")&amp;IF(J17&lt;&gt;"","; "&amp;TEXT(J17,"#,##0")&amp;" subscription(s)"&amp;IF(K17&lt;&gt;""," ("&amp;IF(L17="USD","US$",IF(L17="SGD","S$",L17&amp;" "))&amp;TEXT(K17,"#,##0")&amp;")",""),"")&amp;IF(M17&lt;&gt;"","; "&amp;M17,"")&amp;IF(O17&lt;&gt;"","; "&amp;TEXT(O17,"#,##0")&amp;" trophy/trophies","")&amp;IF(P17&lt;&gt;"","; "&amp;IF(Q17="SGD","S$",IF(Q17="USD","US$",Q17&amp;" "))&amp;TEXT(P17,"#,##0")&amp;" funding","")</x:f>
+        <x:v>1st Prize; US$500 credits; Nosana Cloud credit</x:v>
       </x:c>
       <x:c r="D17" s="36" t="str">
         <x:f>IF(Hackathons!Q43="","",Hackathons!Q43)</x:f>
@@ -14138,8 +14138,8 @@
         <x:v>Agentfield Hackathon 2026</x:v>
       </x:c>
       <x:c r="C18" s="36" t="str">
-        <x:f>IF(Hackathons!G51="","",Hackathons!G51)</x:f>
-        <x:v>1st Prize (OpenRouter Credits $1000 USD)</x:v>
+        <x:f>D18&amp;IF(E18&lt;&gt;""," — "&amp;E18,"")&amp;IF(F18&lt;&gt;"",IF(M18&lt;&gt;"","","; "&amp;IF(G18="SGD","S$",IF(G18="USD","US$",G18&amp;" "))&amp;TEXT(F18,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H18&lt;&gt;"","; "&amp;IF(I18="SGD","S$",IF(I18="USD","US$",I18&amp;" "))&amp;TEXT(H18,"#,##0")&amp;" credits","")&amp;IF(J18&lt;&gt;"","; "&amp;TEXT(J18,"#,##0")&amp;" subscription(s)"&amp;IF(K18&lt;&gt;""," ("&amp;IF(L18="USD","US$",IF(L18="SGD","S$",L18&amp;" "))&amp;TEXT(K18,"#,##0")&amp;")",""),"")&amp;IF(M18&lt;&gt;"","; "&amp;M18,"")&amp;IF(O18&lt;&gt;"","; "&amp;TEXT(O18,"#,##0")&amp;" trophy/trophies","")&amp;IF(P18&lt;&gt;"","; "&amp;IF(Q18="SGD","S$",IF(Q18="USD","US$",Q18&amp;" "))&amp;TEXT(P18,"#,##0")&amp;" funding","")</x:f>
+        <x:v>1st Prize; US$1,000 credits; OpenRouter credits</x:v>
       </x:c>
       <x:c r="D18" s="36" t="str">
         <x:f>IF(Hackathons!Q51="","",Hackathons!Q51)</x:f>
@@ -14206,8 +14206,8 @@
         <x:v>AgentForce Hackathon 2026</x:v>
       </x:c>
       <x:c r="C19" s="36" t="str">
-        <x:f>IF(Hackathons!G53="","",Hackathons!G53)</x:f>
-        <x:v>1st Prize (API Credits $500 USD)</x:v>
+        <x:f>D19&amp;IF(E19&lt;&gt;""," — "&amp;E19,"")&amp;IF(F19&lt;&gt;"",IF(M19&lt;&gt;"","","; "&amp;IF(G19="SGD","S$",IF(G19="USD","US$",G19&amp;" "))&amp;TEXT(F19,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H19&lt;&gt;"","; "&amp;IF(I19="SGD","S$",IF(I19="USD","US$",I19&amp;" "))&amp;TEXT(H19,"#,##0")&amp;" credits","")&amp;IF(J19&lt;&gt;"","; "&amp;TEXT(J19,"#,##0")&amp;" subscription(s)"&amp;IF(K19&lt;&gt;""," ("&amp;IF(L19="USD","US$",IF(L19="SGD","S$",L19&amp;" "))&amp;TEXT(K19,"#,##0")&amp;")",""),"")&amp;IF(M19&lt;&gt;"","; "&amp;M19,"")&amp;IF(O19&lt;&gt;"","; "&amp;TEXT(O19,"#,##0")&amp;" trophy/trophies","")&amp;IF(P19&lt;&gt;"","; "&amp;IF(Q19="SGD","S$",IF(Q19="USD","US$",Q19&amp;" "))&amp;TEXT(P19,"#,##0")&amp;" funding","")</x:f>
+        <x:v>1st Prize; US$500 credits; API credits</x:v>
       </x:c>
       <x:c r="D19" s="36" t="str">
         <x:f>IF(Hackathons!Q53="","",Hackathons!Q53)</x:f>
@@ -14274,8 +14274,8 @@
         <x:v>AgentForce Hackathon 2026</x:v>
       </x:c>
       <x:c r="C20" s="36" t="str">
-        <x:f>IF(Hackathons!G54="","",Hackathons!G54)</x:f>
-        <x:v>1st Prize (API Credits $500 USD)</x:v>
+        <x:f>D20&amp;IF(E20&lt;&gt;""," — "&amp;E20,"")&amp;IF(F20&lt;&gt;"",IF(M20&lt;&gt;"","","; "&amp;IF(G20="SGD","S$",IF(G20="USD","US$",G20&amp;" "))&amp;TEXT(F20,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H20&lt;&gt;"","; "&amp;IF(I20="SGD","S$",IF(I20="USD","US$",I20&amp;" "))&amp;TEXT(H20,"#,##0")&amp;" credits","")&amp;IF(J20&lt;&gt;"","; "&amp;TEXT(J20,"#,##0")&amp;" subscription(s)"&amp;IF(K20&lt;&gt;""," ("&amp;IF(L20="USD","US$",IF(L20="SGD","S$",L20&amp;" "))&amp;TEXT(K20,"#,##0")&amp;")",""),"")&amp;IF(M20&lt;&gt;"","; "&amp;M20,"")&amp;IF(O20&lt;&gt;"","; "&amp;TEXT(O20,"#,##0")&amp;" trophy/trophies","")&amp;IF(P20&lt;&gt;"","; "&amp;IF(Q20="SGD","S$",IF(Q20="USD","US$",Q20&amp;" "))&amp;TEXT(P20,"#,##0")&amp;" funding","")</x:f>
+        <x:v>1st Prize; US$500 credits; API credits</x:v>
       </x:c>
       <x:c r="D20" s="36" t="str">
         <x:f>IF(Hackathons!Q54="","",Hackathons!Q54)</x:f>
@@ -14342,8 +14342,8 @@
         <x:v>SUSS X Openclaw Hackathon 2026</x:v>
       </x:c>
       <x:c r="C21" s="36" t="str">
-        <x:f>IF(Hackathons!G55="","",Hackathons!G55)</x:f>
-        <x:v>1st Prize (Wavespeed AI Credits $150 USD)</x:v>
+        <x:f>D21&amp;IF(E21&lt;&gt;""," — "&amp;E21,"")&amp;IF(F21&lt;&gt;"",IF(M21&lt;&gt;"","","; "&amp;IF(G21="SGD","S$",IF(G21="USD","US$",G21&amp;" "))&amp;TEXT(F21,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H21&lt;&gt;"","; "&amp;IF(I21="SGD","S$",IF(I21="USD","US$",I21&amp;" "))&amp;TEXT(H21,"#,##0")&amp;" credits","")&amp;IF(J21&lt;&gt;"","; "&amp;TEXT(J21,"#,##0")&amp;" subscription(s)"&amp;IF(K21&lt;&gt;""," ("&amp;IF(L21="USD","US$",IF(L21="SGD","S$",L21&amp;" "))&amp;TEXT(K21,"#,##0")&amp;")",""),"")&amp;IF(M21&lt;&gt;"","; "&amp;M21,"")&amp;IF(O21&lt;&gt;"","; "&amp;TEXT(O21,"#,##0")&amp;" trophy/trophies","")&amp;IF(P21&lt;&gt;"","; "&amp;IF(Q21="SGD","S$",IF(Q21="USD","US$",Q21&amp;" "))&amp;TEXT(P21,"#,##0")&amp;" funding","")</x:f>
+        <x:v>1st Prize; US$150 credits; Wavespeed AI credits</x:v>
       </x:c>
       <x:c r="D21" s="36" t="str">
         <x:f>IF(Hackathons!Q55="","",Hackathons!Q55)</x:f>
@@ -14410,8 +14410,8 @@
         <x:v>Agora.io Voice AI Hackathon Singapore 2026</x:v>
       </x:c>
       <x:c r="C22" s="36" t="str">
-        <x:f>IF(Hackathons!G58="","",Hackathons!G58)</x:f>
-        <x:v>3rd Prize: S$300 Cash and S$385 worth of API Credits</x:v>
+        <x:f>D22&amp;IF(E22&lt;&gt;""," — "&amp;E22,"")&amp;IF(F22&lt;&gt;"",IF(M22&lt;&gt;"","","; "&amp;IF(G22="SGD","S$",IF(G22="USD","US$",G22&amp;" "))&amp;TEXT(F22,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H22&lt;&gt;"","; "&amp;IF(I22="SGD","S$",IF(I22="USD","US$",I22&amp;" "))&amp;TEXT(H22,"#,##0")&amp;" credits","")&amp;IF(J22&lt;&gt;"","; "&amp;TEXT(J22,"#,##0")&amp;" subscription(s)"&amp;IF(K22&lt;&gt;""," ("&amp;IF(L22="USD","US$",IF(L22="SGD","S$",L22&amp;" "))&amp;TEXT(K22,"#,##0")&amp;")",""),"")&amp;IF(M22&lt;&gt;"","; "&amp;M22,"")&amp;IF(O22&lt;&gt;"","; "&amp;TEXT(O22,"#,##0")&amp;" trophy/trophies","")&amp;IF(P22&lt;&gt;"","; "&amp;IF(Q22="SGD","S$",IF(Q22="USD","US$",Q22&amp;" "))&amp;TEXT(P22,"#,##0")&amp;" funding","")</x:f>
+        <x:v>3rd Prize; S$385 credits; API credits</x:v>
       </x:c>
       <x:c r="D22" s="36" t="str">
         <x:f>IF(Hackathons!Q58="","",Hackathons!Q58)</x:f>
@@ -14480,8 +14480,8 @@
         <x:v>Build Voice Agents with Speechmatics | TGB Buildathon 2026</x:v>
       </x:c>
       <x:c r="C23" s="36" t="str">
-        <x:f>IF(Hackathons!G61="","",Hackathons!G61)</x:f>
-        <x:v>2K USD Speechmatics Credits</x:v>
+        <x:f>D23&amp;IF(E23&lt;&gt;""," — "&amp;E23,"")&amp;IF(F23&lt;&gt;"",IF(M23&lt;&gt;"","","; "&amp;IF(G23="SGD","S$",IF(G23="USD","US$",G23&amp;" "))&amp;TEXT(F23,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H23&lt;&gt;"","; "&amp;IF(I23="SGD","S$",IF(I23="USD","US$",I23&amp;" "))&amp;TEXT(H23,"#,##0")&amp;" credits","")&amp;IF(J23&lt;&gt;"","; "&amp;TEXT(J23,"#,##0")&amp;" subscription(s)"&amp;IF(K23&lt;&gt;""," ("&amp;IF(L23="USD","US$",IF(L23="SGD","S$",L23&amp;" "))&amp;TEXT(K23,"#,##0")&amp;")",""),"")&amp;IF(M23&lt;&gt;"","; "&amp;M23,"")&amp;IF(O23&lt;&gt;"","; "&amp;TEXT(O23,"#,##0")&amp;" trophy/trophies","")&amp;IF(P23&lt;&gt;"","; "&amp;IF(Q23="SGD","S$",IF(Q23="USD","US$",Q23&amp;" "))&amp;TEXT(P23,"#,##0")&amp;" funding","")</x:f>
+        <x:v>Award — Speechmatics; US$2,000 credits; Speechmatics credits</x:v>
       </x:c>
       <x:c r="D23" s="36" t="str">
         <x:f>IF(Hackathons!Q61="","",Hackathons!Q61)</x:f>
@@ -14549,8 +14549,8 @@
         <x:v>Vercel Zero to Agent: Singapore (1 Hr Hackathon) 2026</x:v>
       </x:c>
       <x:c r="C24" s="36" t="str">
-        <x:f>IF(Hackathons!G62="","",Hackathons!G62)</x:f>
-        <x:v>v0 Sock</x:v>
+        <x:f>D24&amp;IF(E24&lt;&gt;""," — "&amp;E24,"")&amp;IF(F24&lt;&gt;"",IF(M24&lt;&gt;"","","; "&amp;IF(G24="SGD","S$",IF(G24="USD","US$",G24&amp;" "))&amp;TEXT(F24,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H24&lt;&gt;"","; "&amp;IF(I24="SGD","S$",IF(I24="USD","US$",I24&amp;" "))&amp;TEXT(H24,"#,##0")&amp;" credits","")&amp;IF(J24&lt;&gt;"","; "&amp;TEXT(J24,"#,##0")&amp;" subscription(s)"&amp;IF(K24&lt;&gt;""," ("&amp;IF(L24="USD","US$",IF(L24="SGD","S$",L24&amp;" "))&amp;TEXT(K24,"#,##0")&amp;")",""),"")&amp;IF(M24&lt;&gt;"","; "&amp;M24,"")&amp;IF(O24&lt;&gt;"","; "&amp;TEXT(O24,"#,##0")&amp;" trophy/trophies","")&amp;IF(P24&lt;&gt;"","; "&amp;IF(Q24="SGD","S$",IF(Q24="USD","US$",Q24&amp;" "))&amp;TEXT(P24,"#,##0")&amp;" funding","")</x:f>
+        <x:v>Award — v0; v0 Sock</x:v>
       </x:c>
       <x:c r="D24" s="36" t="str">
         <x:f>IF(Hackathons!Q62="","",Hackathons!Q62)</x:f>
@@ -14617,8 +14617,8 @@
         <x:v>UCWS 2026 (Semi-Finals)</x:v>
       </x:c>
       <x:c r="C25" s="36" t="str">
-        <x:f>IF(Hackathons!G67="","",Hackathons!G67)</x:f>
-        <x:v>Top 20, 10K USD OpenAI Credits, 2K USD Gemini Cloud Credits</x:v>
+        <x:f>D25&amp;IF(E25&lt;&gt;""," — "&amp;E25,"")&amp;IF(F25&lt;&gt;"",IF(M25&lt;&gt;"","","; "&amp;IF(G25="SGD","S$",IF(G25="USD","US$",G25&amp;" "))&amp;TEXT(F25,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H25&lt;&gt;"","; "&amp;IF(I25="SGD","S$",IF(I25="USD","US$",I25&amp;" "))&amp;TEXT(H25,"#,##0")&amp;" credits","")&amp;IF(J25&lt;&gt;"","; "&amp;TEXT(J25,"#,##0")&amp;" subscription(s)"&amp;IF(K25&lt;&gt;""," ("&amp;IF(L25="USD","US$",IF(L25="SGD","S$",L25&amp;" "))&amp;TEXT(K25,"#,##0")&amp;")",""),"")&amp;IF(M25&lt;&gt;"","; "&amp;M25,"")&amp;IF(O25&lt;&gt;"","; "&amp;TEXT(O25,"#,##0")&amp;" trophy/trophies","")&amp;IF(P25&lt;&gt;"","; "&amp;IF(Q25="SGD","S$",IF(Q25="USD","US$",Q25&amp;" "))&amp;TEXT(P25,"#,##0")&amp;" funding","")</x:f>
+        <x:v>Top 20; US$12,000 credits; 10K OpenAI credits; 2K Gemini Cloud credits</x:v>
       </x:c>
       <x:c r="D25" s="36" t="str">
         <x:f>IF(Hackathons!Q67="","",Hackathons!Q67)</x:f>
@@ -14685,8 +14685,8 @@
         <x:v>BUIDL_OPC_Hackathon_SG</x:v>
       </x:c>
       <x:c r="C26" s="36" t="str">
-        <x:f>IF(Hackathons!G72="","",Hackathons!G72)</x:f>
-        <x:v>4.5K USD AWS Credits</x:v>
+        <x:f>D26&amp;IF(E26&lt;&gt;""," — "&amp;E26,"")&amp;IF(F26&lt;&gt;"",IF(M26&lt;&gt;"","","; "&amp;IF(G26="SGD","S$",IF(G26="USD","US$",G26&amp;" "))&amp;TEXT(F26,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H26&lt;&gt;"","; "&amp;IF(I26="SGD","S$",IF(I26="USD","US$",I26&amp;" "))&amp;TEXT(H26,"#,##0")&amp;" credits","")&amp;IF(J26&lt;&gt;"","; "&amp;TEXT(J26,"#,##0")&amp;" subscription(s)"&amp;IF(K26&lt;&gt;""," ("&amp;IF(L26="USD","US$",IF(L26="SGD","S$",L26&amp;" "))&amp;TEXT(K26,"#,##0")&amp;")",""),"")&amp;IF(M26&lt;&gt;"","; "&amp;M26,"")&amp;IF(O26&lt;&gt;"","; "&amp;TEXT(O26,"#,##0")&amp;" trophy/trophies","")&amp;IF(P26&lt;&gt;"","; "&amp;IF(Q26="SGD","S$",IF(Q26="USD","US$",Q26&amp;" "))&amp;TEXT(P26,"#,##0")&amp;" funding","")</x:f>
+        <x:v>Award — AWS; US$4,500 credits; AWS credits</x:v>
       </x:c>
       <x:c r="D26" s="36" t="str">
         <x:f>IF(Hackathons!Q72="","",Hackathons!Q72)</x:f>
@@ -14754,8 +14754,8 @@
         <x:v>One AI Hackathon 2026</x:v>
       </x:c>
       <x:c r="C27" s="36" t="str">
-        <x:f>IF(Hackathons!G76="","",Hackathons!G76)</x:f>
-        <x:v>Best Vertical Solution (Family Office Track), 2,000 Cybrdeck API credits (worth US$25)</x:v>
+        <x:f>D27&amp;IF(E27&lt;&gt;""," — "&amp;E27,"")&amp;IF(F27&lt;&gt;"",IF(M27&lt;&gt;"","","; "&amp;IF(G27="SGD","S$",IF(G27="USD","US$",G27&amp;" "))&amp;TEXT(F27,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H27&lt;&gt;"","; "&amp;IF(I27="SGD","S$",IF(I27="USD","US$",I27&amp;" "))&amp;TEXT(H27,"#,##0")&amp;" credits","")&amp;IF(J27&lt;&gt;"","; "&amp;TEXT(J27,"#,##0")&amp;" subscription(s)"&amp;IF(K27&lt;&gt;""," ("&amp;IF(L27="USD","US$",IF(L27="SGD","S$",L27&amp;" "))&amp;TEXT(K27,"#,##0")&amp;")",""),"")&amp;IF(M27&lt;&gt;"","; "&amp;M27,"")&amp;IF(O27&lt;&gt;"","; "&amp;TEXT(O27,"#,##0")&amp;" trophy/trophies","")&amp;IF(P27&lt;&gt;"","; "&amp;IF(Q27="SGD","S$",IF(Q27="USD","US$",Q27&amp;" "))&amp;TEXT(P27,"#,##0")&amp;" funding","")</x:f>
+        <x:v>Best Vertical Solution — Family Office Track; US$25 credits; 2,000 Cybrdeck API credits</x:v>
       </x:c>
       <x:c r="D27" s="36" t="str">
         <x:f>IF(Hackathons!Q76="","",Hackathons!Q76)</x:f>
@@ -14823,8 +14823,8 @@
         <x:v>SG × SWK Friendship AI Business Design Hackathon</x:v>
       </x:c>
       <x:c r="C28" s="36" t="str">
-        <x:f>IF(Hackathons!G80="","",Hackathons!G80)</x:f>
-        <x:v>Trophy, First Runner Up, SG × Sarawak AI &amp; Design Hackathon 2026, 200 USD Kimi AI credits</x:v>
+        <x:f>D28&amp;IF(E28&lt;&gt;""," — "&amp;E28,"")&amp;IF(F28&lt;&gt;"",IF(M28&lt;&gt;"","","; "&amp;IF(G28="SGD","S$",IF(G28="USD","US$",G28&amp;" "))&amp;TEXT(F28,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H28&lt;&gt;"","; "&amp;IF(I28="SGD","S$",IF(I28="USD","US$",I28&amp;" "))&amp;TEXT(H28,"#,##0")&amp;" credits","")&amp;IF(J28&lt;&gt;"","; "&amp;TEXT(J28,"#,##0")&amp;" subscription(s)"&amp;IF(K28&lt;&gt;""," ("&amp;IF(L28="USD","US$",IF(L28="SGD","S$",L28&amp;" "))&amp;TEXT(K28,"#,##0")&amp;")",""),"")&amp;IF(M28&lt;&gt;"","; "&amp;M28,"")&amp;IF(O28&lt;&gt;"","; "&amp;TEXT(O28,"#,##0")&amp;" trophy/trophies","")&amp;IF(P28&lt;&gt;"","; "&amp;IF(Q28="SGD","S$",IF(Q28="USD","US$",Q28&amp;" "))&amp;TEXT(P28,"#,##0")&amp;" funding","")</x:f>
+        <x:v>First Runner Up — SG × Sarawak AI &amp; Design Hackathon 2026; US$200 credits; Trophy; Kimi AI credits; 1 trophy/trophies</x:v>
       </x:c>
       <x:c r="D28" s="36" t="str">
         <x:f>IF(Hackathons!Q80="","",Hackathons!Q80)</x:f>
@@ -14894,8 +14894,8 @@
         <x:v>GPT-6 Astra Hackathon: Singapore</x:v>
       </x:c>
       <x:c r="C29" s="36" t="str">
-        <x:f>IF(Hackathons!G81="","",Hackathons!G81)</x:f>
-        <x:v>Best use of GPT-Image-2.5, 5,000 USD OpenAI credits</x:v>
+        <x:f>D29&amp;IF(E29&lt;&gt;""," — "&amp;E29,"")&amp;IF(F29&lt;&gt;"",IF(M29&lt;&gt;"","","; "&amp;IF(G29="SGD","S$",IF(G29="USD","US$",G29&amp;" "))&amp;TEXT(F29,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H29&lt;&gt;"","; "&amp;IF(I29="SGD","S$",IF(I29="USD","US$",I29&amp;" "))&amp;TEXT(H29,"#,##0")&amp;" credits","")&amp;IF(J29&lt;&gt;"","; "&amp;TEXT(J29,"#,##0")&amp;" subscription(s)"&amp;IF(K29&lt;&gt;""," ("&amp;IF(L29="USD","US$",IF(L29="SGD","S$",L29&amp;" "))&amp;TEXT(K29,"#,##0")&amp;")",""),"")&amp;IF(M29&lt;&gt;"","; "&amp;M29,"")&amp;IF(O29&lt;&gt;"","; "&amp;TEXT(O29,"#,##0")&amp;" trophy/trophies","")&amp;IF(P29&lt;&gt;"","; "&amp;IF(Q29="SGD","S$",IF(Q29="USD","US$",Q29&amp;" "))&amp;TEXT(P29,"#,##0")&amp;" funding","")</x:f>
+        <x:v>Best Project — Best Use of GPT-Image-2.5; US$5,000 credits; OpenAI credits</x:v>
       </x:c>
       <x:c r="D29" s="36" t="str">
         <x:f>IF(Hackathons!Q81="","",Hackathons!Q81)</x:f>
@@ -14966,7 +14966,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbc23ba9da984bb4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c7635549fdd4a93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Curate standardized award summaries
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R9a70d0e706b34bc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R8703e043c74740f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R02a5fff09ec54696"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R40a1a6b6bd544efa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="Rc05e35a6d2f242b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R81a1cb0d3b544b30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R0bea597d72b04c7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R085a953c905b4a7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R794b7a9eb2a64c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R07049fa541734a19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R78e6d45d68ab48e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R7ef7df85de984e89"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2935,7 +2935,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="45">
+  <x:fills count="47">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -3157,6 +3157,16 @@
         <x:fgColor rgb="FFFFF4CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF3F8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -3221,7 +3231,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="191">
+  <x:cellXfs count="199">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3623,6 +3633,24 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="17" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Hyperlink" xfId="1"/>
@@ -3936,6 +3964,7 @@
     <x:col min="30" max="30" width="18" hidden="0" customWidth="1"/>
     <x:col min="31" max="31" width="22" hidden="0" customWidth="1"/>
     <x:col min="32" max="32" width="32" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="58" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -4034,6 +4063,9 @@
       </x:c>
       <x:c r="AF1" s="26" t="str">
         <x:v>Review Note</x:v>
+      </x:c>
+      <x:c r="AG1" s="195" t="str">
+        <x:v>Award Summary</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -4110,6 +4142,9 @@
       </x:c>
       <x:c r="AF2" s="38" t="str">
         <x:v>Funding, not a cash prize</x:v>
+      </x:c>
+      <x:c r="AG2" s="198" t="str">
+        <x:v>1st Place — S$18,000 Seed Funding</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4177,6 +4212,7 @@
       <x:c r="AD3" s="36"/>
       <x:c r="AE3" s="38"/>
       <x:c r="AF3" s="38"/>
+      <x:c r="AG3" s="198"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4">
@@ -4251,6 +4287,9 @@
       <x:c r="AF4" s="38" t="str">
         <x:v>Recognition only</x:v>
       </x:c>
+      <x:c r="AG4" s="198" t="str">
+        <x:v>Best Project</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5">
@@ -4334,6 +4373,9 @@
       </x:c>
       <x:c r="AF5" s="38" t="str">
         <x:v>US$100,000 IBM Bluemix credit value</x:v>
+      </x:c>
+      <x:c r="AG5" s="198" t="str">
+        <x:v>1st Place — Best Use of IBM Bluemix — US$100,000 IBM Bluemix Credits — SmartWatch</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4401,6 +4443,7 @@
       <x:c r="AD6" s="36"/>
       <x:c r="AE6" s="38"/>
       <x:c r="AF6" s="38"/>
+      <x:c r="AG6" s="198"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7">
@@ -4472,6 +4515,9 @@
       </x:c>
       <x:c r="AF7" s="38" t="str">
         <x:v>Recognition only</x:v>
+      </x:c>
+      <x:c r="AG7" s="198" t="str">
+        <x:v>Top 10</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -4539,6 +4585,7 @@
       <x:c r="AD8" s="36"/>
       <x:c r="AE8" s="38"/>
       <x:c r="AF8" s="38"/>
+      <x:c r="AG8" s="198"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9">
@@ -4605,6 +4652,7 @@
       <x:c r="AD9" s="36"/>
       <x:c r="AE9" s="38"/>
       <x:c r="AF9" s="38"/>
+      <x:c r="AG9" s="198"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10">
@@ -4671,6 +4719,7 @@
       <x:c r="AD10" s="36"/>
       <x:c r="AE10" s="38"/>
       <x:c r="AF10" s="38"/>
+      <x:c r="AG10" s="198"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11">
@@ -4744,6 +4793,9 @@
       </x:c>
       <x:c r="AF11" s="38" t="str">
         <x:v>Recognition only</x:v>
+      </x:c>
+      <x:c r="AG11" s="198" t="str">
+        <x:v>Best Project</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -4811,6 +4863,7 @@
       <x:c r="AD12" s="36"/>
       <x:c r="AE12" s="38"/>
       <x:c r="AF12" s="38"/>
+      <x:c r="AG12" s="198"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13">
@@ -4877,6 +4930,7 @@
       <x:c r="AD13" s="36"/>
       <x:c r="AE13" s="38"/>
       <x:c r="AF13" s="38"/>
+      <x:c r="AG13" s="198"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14">
@@ -4943,6 +4997,7 @@
       <x:c r="AD14" s="36"/>
       <x:c r="AE14" s="38"/>
       <x:c r="AF14" s="38"/>
+      <x:c r="AG14" s="198"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15">
@@ -5020,6 +5075,9 @@
       </x:c>
       <x:c r="AF15" s="38" t="str">
         <x:v>Voucher counted as cash equivalent</x:v>
+      </x:c>
+      <x:c r="AG15" s="198" t="str">
+        <x:v>3rd Place — S$100 Capitaland Voucher</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -5087,6 +5145,7 @@
       <x:c r="AD16" s="36"/>
       <x:c r="AE16" s="38"/>
       <x:c r="AF16" s="38"/>
+      <x:c r="AG16" s="198"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17">
@@ -5153,6 +5212,7 @@
       <x:c r="AD17" s="36"/>
       <x:c r="AE17" s="38"/>
       <x:c r="AF17" s="38"/>
+      <x:c r="AG17" s="198"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18">
@@ -5228,6 +5288,9 @@
       </x:c>
       <x:c r="AF18" s="38" t="str">
         <x:v>Explicit cash</x:v>
+      </x:c>
+      <x:c r="AG18" s="198" t="str">
+        <x:v>2nd Place — S$600 Cash</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -5295,6 +5358,7 @@
       <x:c r="AD19" s="36"/>
       <x:c r="AE19" s="38"/>
       <x:c r="AF19" s="38"/>
+      <x:c r="AG19" s="198"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20">
@@ -5361,6 +5425,7 @@
       <x:c r="AD20" s="36"/>
       <x:c r="AE20" s="38"/>
       <x:c r="AF20" s="38"/>
+      <x:c r="AG20" s="198"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21">
@@ -5427,6 +5492,7 @@
       <x:c r="AD21" s="36"/>
       <x:c r="AE21" s="38"/>
       <x:c r="AF21" s="38"/>
+      <x:c r="AG21" s="198"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22">
@@ -5493,6 +5559,7 @@
       <x:c r="AD22" s="36"/>
       <x:c r="AE22" s="38"/>
       <x:c r="AF22" s="38"/>
+      <x:c r="AG22" s="198"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23">
@@ -5559,6 +5626,7 @@
       <x:c r="AD23" s="36"/>
       <x:c r="AE23" s="38"/>
       <x:c r="AF23" s="38"/>
+      <x:c r="AG23" s="198"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24">
@@ -5625,6 +5693,7 @@
       <x:c r="AD24" s="36"/>
       <x:c r="AE24" s="38"/>
       <x:c r="AF24" s="38"/>
+      <x:c r="AG24" s="198"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25">
@@ -5691,6 +5760,7 @@
       <x:c r="AD25" s="36"/>
       <x:c r="AE25" s="38"/>
       <x:c r="AF25" s="38"/>
+      <x:c r="AG25" s="198"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26">
@@ -5766,6 +5836,9 @@
       </x:c>
       <x:c r="AF26" s="38" t="str">
         <x:v>Explicit cash</x:v>
+      </x:c>
+      <x:c r="AG26" s="198" t="str">
+        <x:v>3rd Place — S$500 Cash</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -5833,6 +5906,7 @@
       <x:c r="AD27" s="36"/>
       <x:c r="AE27" s="38"/>
       <x:c r="AF27" s="38"/>
+      <x:c r="AG27" s="198"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28">
@@ -5899,6 +5973,7 @@
       <x:c r="AD28" s="36"/>
       <x:c r="AE28" s="38"/>
       <x:c r="AF28" s="38"/>
+      <x:c r="AG28" s="198"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29">
@@ -5965,6 +6040,7 @@
       <x:c r="AD29" s="36"/>
       <x:c r="AE29" s="38"/>
       <x:c r="AF29" s="38"/>
+      <x:c r="AG29" s="198"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30">
@@ -6031,6 +6107,7 @@
       <x:c r="AD30" s="36"/>
       <x:c r="AE30" s="38"/>
       <x:c r="AF30" s="38"/>
+      <x:c r="AG30" s="198"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31">
@@ -6097,6 +6174,7 @@
       <x:c r="AD31" s="36"/>
       <x:c r="AE31" s="38"/>
       <x:c r="AF31" s="38"/>
+      <x:c r="AG31" s="198"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32">
@@ -6163,6 +6241,7 @@
       <x:c r="AD32" s="36"/>
       <x:c r="AE32" s="38"/>
       <x:c r="AF32" s="38"/>
+      <x:c r="AG32" s="198"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33">
@@ -6227,6 +6306,7 @@
       <x:c r="AD33" s="36"/>
       <x:c r="AE33" s="38"/>
       <x:c r="AF33" s="38"/>
+      <x:c r="AG33" s="198"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34">
@@ -6278,7 +6358,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="Q34" s="36" t="str">
-        <x:v>3rd Prize</x:v>
+        <x:v>3rd Place</x:v>
       </x:c>
       <x:c r="R34" s="36"/>
       <x:c r="S34" s="37" t="n">
@@ -6302,6 +6382,9 @@
       </x:c>
       <x:c r="AF34" s="38" t="str">
         <x:v>Confirmed cash</x:v>
+      </x:c>
+      <x:c r="AG34" s="198" t="str">
+        <x:v>3rd Place — S$250 Cash</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -6369,6 +6452,7 @@
       <x:c r="AD35" s="36"/>
       <x:c r="AE35" s="38"/>
       <x:c r="AF35" s="38"/>
+      <x:c r="AG35" s="198"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36">
@@ -6420,7 +6504,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="Q36" s="36" t="str">
-        <x:v>2nd Prize</x:v>
+        <x:v>2nd Place</x:v>
       </x:c>
       <x:c r="R36" s="36"/>
       <x:c r="S36" s="37" t="n">
@@ -6444,6 +6528,9 @@
       </x:c>
       <x:c r="AF36" s="38" t="str">
         <x:v>Confirmed cash</x:v>
+      </x:c>
+      <x:c r="AG36" s="198" t="str">
+        <x:v>2nd Place — S$1,000 Cash</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -6511,6 +6598,7 @@
       <x:c r="AD37" s="36"/>
       <x:c r="AE37" s="38"/>
       <x:c r="AF37" s="38"/>
+      <x:c r="AG37" s="198"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38">
@@ -6577,6 +6665,7 @@
       <x:c r="AD38" s="36"/>
       <x:c r="AE38" s="38"/>
       <x:c r="AF38" s="38"/>
+      <x:c r="AG38" s="198"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39">
@@ -6656,6 +6745,9 @@
       </x:c>
       <x:c r="AF39" s="38" t="str">
         <x:v>US$39 monthly value at award period</x:v>
+      </x:c>
+      <x:c r="AG39" s="198" t="str">
+        <x:v>2nd Place — Manus Pro Subscription (US$39/month)</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -6723,6 +6815,7 @@
       <x:c r="AD40" s="36"/>
       <x:c r="AE40" s="38"/>
       <x:c r="AF40" s="38"/>
+      <x:c r="AG40" s="198"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41">
@@ -6799,6 +6892,9 @@
       </x:c>
       <x:c r="AF41" s="38" t="str">
         <x:v>Trophy, not cash</x:v>
+      </x:c>
+      <x:c r="AG41" s="198" t="str">
+        <x:v>Best Finisher — Novel Hackathon — Trophy</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -6863,6 +6959,7 @@
       <x:c r="AD42" s="36"/>
       <x:c r="AE42" s="38"/>
       <x:c r="AF42" s="38"/>
+      <x:c r="AG42" s="198"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43">
@@ -6940,6 +7037,9 @@
       </x:c>
       <x:c r="AF43" s="38" t="str">
         <x:v>Cloud credit, not cash</x:v>
+      </x:c>
+      <x:c r="AG43" s="198" t="str">
+        <x:v>1st Place — US$500 Nosana Cloud Credits</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -7007,6 +7107,7 @@
       <x:c r="AD44" s="36"/>
       <x:c r="AE44" s="38"/>
       <x:c r="AF44" s="38"/>
+      <x:c r="AG44" s="198"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45">
@@ -7073,6 +7174,7 @@
       <x:c r="AD45" s="36"/>
       <x:c r="AE45" s="38"/>
       <x:c r="AF45" s="38"/>
+      <x:c r="AG45" s="198"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46">
@@ -7139,6 +7241,7 @@
       <x:c r="AD46" s="36"/>
       <x:c r="AE46" s="38"/>
       <x:c r="AF46" s="38"/>
+      <x:c r="AG46" s="198"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47">
@@ -7205,6 +7308,7 @@
       <x:c r="AD47" s="36"/>
       <x:c r="AE47" s="38"/>
       <x:c r="AF47" s="38"/>
+      <x:c r="AG47" s="198"/>
     </x:row>
     <x:row r="48" ht="49.75" customHeight="1">
       <x:c r="A48">
@@ -7271,6 +7375,7 @@
       <x:c r="AD48" s="36"/>
       <x:c r="AE48" s="38"/>
       <x:c r="AF48" s="38"/>
+      <x:c r="AG48" s="198"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49">
@@ -7337,6 +7442,7 @@
       <x:c r="AD49" s="36"/>
       <x:c r="AE49" s="38"/>
       <x:c r="AF49" s="38"/>
+      <x:c r="AG49" s="198"/>
     </x:row>
     <x:row r="50" ht="34">
       <x:c r="A50">
@@ -7403,6 +7509,7 @@
       <x:c r="AD50" s="36"/>
       <x:c r="AE50" s="38"/>
       <x:c r="AF50" s="38"/>
+      <x:c r="AG50" s="198"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51">
@@ -7480,6 +7587,9 @@
       </x:c>
       <x:c r="AF51" s="38" t="str">
         <x:v>API credits, not cash</x:v>
+      </x:c>
+      <x:c r="AG51" s="198" t="str">
+        <x:v>1st Place — US$1,000 OpenRouter Credits</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -7547,6 +7657,7 @@
       <x:c r="AD52" s="36"/>
       <x:c r="AE52" s="38"/>
       <x:c r="AF52" s="38"/>
+      <x:c r="AG52" s="198"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53">
@@ -7625,6 +7736,9 @@
       <x:c r="AF53" s="38" t="str">
         <x:v>API credits, not cash</x:v>
       </x:c>
+      <x:c r="AG53" s="198" t="str">
+        <x:v>1st Place — US$500 API Credits</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54">
@@ -7703,6 +7817,9 @@
       <x:c r="AF54" s="38" t="str">
         <x:v>API credits, not cash</x:v>
       </x:c>
+      <x:c r="AG54" s="198" t="str">
+        <x:v>1st Place — US$500 API Credits</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="34">
       <x:c r="A55">
@@ -7780,6 +7897,9 @@
       </x:c>
       <x:c r="AF55" s="38" t="str">
         <x:v>API credits, not cash</x:v>
+      </x:c>
+      <x:c r="AG55" s="198" t="str">
+        <x:v>1st Place — US$150 Wavespeed AI Credits</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="17">
@@ -7847,6 +7967,7 @@
       <x:c r="AD56" s="36"/>
       <x:c r="AE56" s="38"/>
       <x:c r="AF56" s="38"/>
+      <x:c r="AG56" s="198"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57">
@@ -7913,6 +8034,7 @@
       <x:c r="AD57" s="36"/>
       <x:c r="AE57" s="38"/>
       <x:c r="AF57" s="38"/>
+      <x:c r="AG57" s="198"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58">
@@ -7994,6 +8116,9 @@
       </x:c>
       <x:c r="AF58" s="38" t="str">
         <x:v>Explicit cash; API credit value also tracked</x:v>
+      </x:c>
+      <x:c r="AG58" s="198" t="str">
+        <x:v>3rd Place — S$300 Cash + S$385 API Credits</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -8061,6 +8186,7 @@
       <x:c r="AD59" s="36"/>
       <x:c r="AE59" s="38"/>
       <x:c r="AF59" s="38"/>
+      <x:c r="AG59" s="198"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60">
@@ -8127,6 +8253,7 @@
       <x:c r="AD60" s="36"/>
       <x:c r="AE60" s="38"/>
       <x:c r="AF60" s="38"/>
+      <x:c r="AG60" s="198"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61">
@@ -8206,6 +8333,9 @@
       </x:c>
       <x:c r="AF61" s="38" t="str">
         <x:v>USD-denominated credit value</x:v>
+      </x:c>
+      <x:c r="AG61" s="198" t="str">
+        <x:v>Award — Speechmatics — US$2,000 Speechmatics Credits</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -8286,6 +8416,9 @@
       </x:c>
       <x:c r="AF62" s="38" t="str">
         <x:v>Physical item, not cash</x:v>
+      </x:c>
+      <x:c r="AG62" s="198" t="str">
+        <x:v>Award — v0 Sock</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -8353,6 +8486,7 @@
       <x:c r="AD63" s="36"/>
       <x:c r="AE63" s="38"/>
       <x:c r="AF63" s="38"/>
+      <x:c r="AG63" s="198"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64">
@@ -8419,6 +8553,7 @@
       <x:c r="AD64" s="36"/>
       <x:c r="AE64" s="38"/>
       <x:c r="AF64" s="38"/>
+      <x:c r="AG64" s="198"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65">
@@ -8485,6 +8620,7 @@
       <x:c r="AD65" s="36"/>
       <x:c r="AE65" s="38"/>
       <x:c r="AF65" s="38"/>
+      <x:c r="AG65" s="198"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66">
@@ -8551,6 +8687,7 @@
       <x:c r="AD66" s="36"/>
       <x:c r="AE66" s="38"/>
       <x:c r="AF66" s="38"/>
+      <x:c r="AG66" s="198"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67">
@@ -8628,6 +8765,9 @@
       </x:c>
       <x:c r="AF67" s="38" t="str">
         <x:v>Credit value total combines two USD-denominated credits</x:v>
+      </x:c>
+      <x:c r="AG67" s="198" t="str">
+        <x:v>Top 20 — US$12,000 Credits (OpenAI + Gemini Cloud)</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -8695,6 +8835,7 @@
       <x:c r="AD68" s="36"/>
       <x:c r="AE68" s="38"/>
       <x:c r="AF68" s="38"/>
+      <x:c r="AG68" s="198"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69">
@@ -8761,6 +8902,7 @@
       <x:c r="AD69" s="36"/>
       <x:c r="AE69" s="38"/>
       <x:c r="AF69" s="38"/>
+      <x:c r="AG69" s="198"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70">
@@ -8824,6 +8966,7 @@
       <x:c r="AD70" s="36"/>
       <x:c r="AE70" s="38"/>
       <x:c r="AF70" s="38"/>
+      <x:c r="AG70" s="198"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71">
@@ -8890,6 +9033,7 @@
       <x:c r="AD71" s="36"/>
       <x:c r="AE71" s="38"/>
       <x:c r="AF71" s="38"/>
+      <x:c r="AG71" s="198"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72">
@@ -8969,6 +9113,9 @@
       </x:c>
       <x:c r="AF72" s="38" t="str">
         <x:v>USD-denominated credit value</x:v>
+      </x:c>
+      <x:c r="AG72" s="198" t="str">
+        <x:v>Award — US$4,500 AWS Credits</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -9036,6 +9183,7 @@
       <x:c r="AD73" s="36"/>
       <x:c r="AE73" s="38"/>
       <x:c r="AF73" s="38"/>
+      <x:c r="AG73" s="198"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74">
@@ -9102,6 +9250,7 @@
       <x:c r="AD74" s="36"/>
       <x:c r="AE74" s="38"/>
       <x:c r="AF74" s="38"/>
+      <x:c r="AG74" s="198"/>
     </x:row>
     <x:row r="75" ht="34">
       <x:c r="A75">
@@ -9168,6 +9317,7 @@
       <x:c r="AD75" s="36"/>
       <x:c r="AE75" s="38"/>
       <x:c r="AF75" s="38"/>
+      <x:c r="AG75" s="198"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76">
@@ -9247,6 +9397,9 @@
       </x:c>
       <x:c r="AF76" s="38" t="str">
         <x:v>US$25 credit value, not cash</x:v>
+      </x:c>
+      <x:c r="AG76" s="198" t="str">
+        <x:v>Best Vertical Solution — Family Office Track — 2,000 Cybrdeck API Credits (US$25 value)</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -9314,6 +9467,7 @@
       <x:c r="AD77" s="36"/>
       <x:c r="AE77" s="38"/>
       <x:c r="AF77" s="38"/>
+      <x:c r="AG77" s="198"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78">
@@ -9380,6 +9534,7 @@
       <x:c r="AD78" s="36"/>
       <x:c r="AE78" s="38"/>
       <x:c r="AF78" s="38"/>
+      <x:c r="AG78" s="198"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79">
@@ -9446,6 +9601,7 @@
       <x:c r="AD79" s="36"/>
       <x:c r="AE79" s="38"/>
       <x:c r="AF79" s="38"/>
+      <x:c r="AG79" s="198"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" t="n">
@@ -9497,7 +9653,7 @@
         <x:v>https://luma.com/n0zkb5w0?tk=OBDQgW</x:v>
       </x:c>
       <x:c r="Q80" s="36" t="str">
-        <x:v>First Runner Up</x:v>
+        <x:v>First Runner-Up</x:v>
       </x:c>
       <x:c r="R80" s="36" t="str">
         <x:v>SG × Sarawak AI &amp; Design Hackathon 2026</x:v>
@@ -9529,6 +9685,9 @@
       </x:c>
       <x:c r="AF80" s="38" t="str">
         <x:v>Trophy excluded; credit value tracked</x:v>
+      </x:c>
+      <x:c r="AG80" s="198" t="str">
+        <x:v>First Runner-Up — SG × Sarawak AI &amp; Design Hackathon — US$200 Kimi AI Credits + Trophy</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -9609,6 +9768,9 @@
       </x:c>
       <x:c r="AF81" s="38" t="str">
         <x:v>Credit value tracked</x:v>
+      </x:c>
+      <x:c r="AG81" s="198" t="str">
+        <x:v>Best Project — Best Use of GPT-Image-2.5 — US$5,000 OpenAI Credits</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -9674,13 +9836,14 @@
       <x:c r="AD82" s="36"/>
       <x:c r="AE82" s="38"/>
       <x:c r="AF82" s="38"/>
+      <x:c r="AG82" s="198"/>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R0f570abde045437d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R61455f82b54b4990"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R302eef6afc894f03"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Ra8b66eacbb77463f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R27e30ceef8f54e31"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R621a569fdc794f82"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rf6436f694a7342d5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R0f731b896efd49b6"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11258,12 +11421,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Re264cfb16f194e64"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R0a98f61dcb194104"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rd70e071e6dbd49bd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R37aecd44f30641a3"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1057523a1334982"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R978dbdb592c142e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12166,7 +12329,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2931dda0bada466c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6859fb134c8a44f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13158,7 +13321,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="106" t="str">
-        <x:v>One row per currently classified award or prize record. The Award summary is standardized from the linked fields on Hackathons; the original raw text remains preserved there.</x:v>
+        <x:v>One row per currently classified award or prize record. Award Summary uses a curated, standardized format; the raw original award text remains preserved on Hackathons.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -13201,7 +13364,7 @@
         <x:v>Hackathon</x:v>
       </x:c>
       <x:c r="C4" s="90" t="str">
-        <x:v>Award summary</x:v>
+        <x:v>Award Summary</x:v>
       </x:c>
       <x:c r="D4" s="90" t="str">
         <x:v>Award type</x:v>
@@ -13262,8 +13425,8 @@
         <x:v>Education Technology Hackathon</x:v>
       </x:c>
       <x:c r="C5" s="36" t="str">
-        <x:f>D5&amp;IF(E5&lt;&gt;""," — "&amp;E5,"")&amp;IF(F5&lt;&gt;"",IF(M5&lt;&gt;"","","; "&amp;IF(G5="SGD","S$",IF(G5="USD","US$",G5&amp;" "))&amp;TEXT(F5,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H5&lt;&gt;"","; "&amp;IF(I5="SGD","S$",IF(I5="USD","US$",I5&amp;" "))&amp;TEXT(H5,"#,##0")&amp;" credits","")&amp;IF(J5&lt;&gt;"","; "&amp;TEXT(J5,"#,##0")&amp;" subscription(s)"&amp;IF(K5&lt;&gt;""," ("&amp;IF(L5="USD","US$",IF(L5="SGD","S$",L5&amp;" "))&amp;TEXT(K5,"#,##0")&amp;")",""),"")&amp;IF(M5&lt;&gt;"","; "&amp;M5,"")&amp;IF(O5&lt;&gt;"","; "&amp;TEXT(O5,"#,##0")&amp;" trophy/trophies","")&amp;IF(P5&lt;&gt;"","; "&amp;IF(Q5="SGD","S$",IF(Q5="USD","US$",Q5&amp;" "))&amp;TEXT(P5,"#,##0")&amp;" funding","")</x:f>
-        <x:v>1st Place; S$18,000 funding</x:v>
+        <x:f>Hackathons!AG2</x:f>
+        <x:v>1st Place — S$18,000 Seed Funding</x:v>
       </x:c>
       <x:c r="D5" s="36" t="str">
         <x:f>IF(Hackathons!Q2="","",Hackathons!Q2)</x:f>
@@ -13329,8 +13492,8 @@
         <x:v>DataDriven Hackathon 2016</x:v>
       </x:c>
       <x:c r="C6" s="36" t="str">
-        <x:f>D6&amp;IF(E6&lt;&gt;""," — "&amp;E6,"")&amp;IF(F6&lt;&gt;"",IF(M6&lt;&gt;"","","; "&amp;IF(G6="SGD","S$",IF(G6="USD","US$",G6&amp;" "))&amp;TEXT(F6,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H6&lt;&gt;"","; "&amp;IF(I6="SGD","S$",IF(I6="USD","US$",I6&amp;" "))&amp;TEXT(H6,"#,##0")&amp;" credits","")&amp;IF(J6&lt;&gt;"","; "&amp;TEXT(J6,"#,##0")&amp;" subscription(s)"&amp;IF(K6&lt;&gt;""," ("&amp;IF(L6="USD","US$",IF(L6="SGD","S$",L6&amp;" "))&amp;TEXT(K6,"#,##0")&amp;")",""),"")&amp;IF(M6&lt;&gt;"","; "&amp;M6,"")&amp;IF(O6&lt;&gt;"","; "&amp;TEXT(O6,"#,##0")&amp;" trophy/trophies","")&amp;IF(P6&lt;&gt;"","; "&amp;IF(Q6="SGD","S$",IF(Q6="USD","US$",Q6&amp;" "))&amp;TEXT(P6,"#,##0")&amp;" funding","")</x:f>
-        <x:v>Best Project — Rated best project</x:v>
+        <x:f>Hackathons!AG4</x:f>
+        <x:v>Best Project</x:v>
       </x:c>
       <x:c r="D6" s="36" t="str">
         <x:f>IF(Hackathons!Q4="","",Hackathons!Q4)</x:f>
@@ -13395,8 +13558,8 @@
         <x:v>Fintech Festival Hackathon 2016</x:v>
       </x:c>
       <x:c r="C7" s="36" t="str">
-        <x:f>D7&amp;IF(E7&lt;&gt;""," — "&amp;E7,"")&amp;IF(F7&lt;&gt;"",IF(M7&lt;&gt;"","","; "&amp;IF(G7="SGD","S$",IF(G7="USD","US$",G7&amp;" "))&amp;TEXT(F7,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H7&lt;&gt;"","; "&amp;IF(I7="SGD","S$",IF(I7="USD","US$",I7&amp;" "))&amp;TEXT(H7,"#,##0")&amp;" credits","")&amp;IF(J7&lt;&gt;"","; "&amp;TEXT(J7,"#,##0")&amp;" subscription(s)"&amp;IF(K7&lt;&gt;""," ("&amp;IF(L7="USD","US$",IF(L7="SGD","S$",L7&amp;" "))&amp;TEXT(K7,"#,##0")&amp;")",""),"")&amp;IF(M7&lt;&gt;"","; "&amp;M7,"")&amp;IF(O7&lt;&gt;"","; "&amp;TEXT(O7,"#,##0")&amp;" trophy/trophies","")&amp;IF(P7&lt;&gt;"","; "&amp;IF(Q7="SGD","S$",IF(Q7="USD","US$",Q7&amp;" "))&amp;TEXT(P7,"#,##0")&amp;" funding","")</x:f>
-        <x:v>1st Place — Best Use of IBM Bluemix; US$100,000 credits; IBM Bluemix credits; SmartWatch</x:v>
+        <x:f>Hackathons!AG5</x:f>
+        <x:v>1st Place — Best Use of IBM Bluemix — US$100,000 IBM Bluemix Credits — SmartWatch</x:v>
       </x:c>
       <x:c r="D7" s="36" t="str">
         <x:f>IF(Hackathons!Q5="","",Hackathons!Q5)</x:f>
@@ -13465,7 +13628,7 @@
         <x:v>SO.IMPACT Bootcamp 2017</x:v>
       </x:c>
       <x:c r="C8" s="36" t="str">
-        <x:f>D8&amp;IF(E8&lt;&gt;""," — "&amp;E8,"")&amp;IF(F8&lt;&gt;"",IF(M8&lt;&gt;"","","; "&amp;IF(G8="SGD","S$",IF(G8="USD","US$",G8&amp;" "))&amp;TEXT(F8,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H8&lt;&gt;"","; "&amp;IF(I8="SGD","S$",IF(I8="USD","US$",I8&amp;" "))&amp;TEXT(H8,"#,##0")&amp;" credits","")&amp;IF(J8&lt;&gt;"","; "&amp;TEXT(J8,"#,##0")&amp;" subscription(s)"&amp;IF(K8&lt;&gt;""," ("&amp;IF(L8="USD","US$",IF(L8="SGD","S$",L8&amp;" "))&amp;TEXT(K8,"#,##0")&amp;")",""),"")&amp;IF(M8&lt;&gt;"","; "&amp;M8,"")&amp;IF(O8&lt;&gt;"","; "&amp;TEXT(O8,"#,##0")&amp;" trophy/trophies","")&amp;IF(P8&lt;&gt;"","; "&amp;IF(Q8="SGD","S$",IF(Q8="USD","US$",Q8&amp;" "))&amp;TEXT(P8,"#,##0")&amp;" funding","")</x:f>
+        <x:f>Hackathons!AG7</x:f>
         <x:v>Top 10</x:v>
       </x:c>
       <x:c r="D8" s="36" t="str">
@@ -13530,8 +13693,8 @@
         <x:v>DataDriven Hackathon 2017</x:v>
       </x:c>
       <x:c r="C9" s="36" t="str">
-        <x:f>D9&amp;IF(E9&lt;&gt;""," — "&amp;E9,"")&amp;IF(F9&lt;&gt;"",IF(M9&lt;&gt;"","","; "&amp;IF(G9="SGD","S$",IF(G9="USD","US$",G9&amp;" "))&amp;TEXT(F9,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H9&lt;&gt;"","; "&amp;IF(I9="SGD","S$",IF(I9="USD","US$",I9&amp;" "))&amp;TEXT(H9,"#,##0")&amp;" credits","")&amp;IF(J9&lt;&gt;"","; "&amp;TEXT(J9,"#,##0")&amp;" subscription(s)"&amp;IF(K9&lt;&gt;""," ("&amp;IF(L9="USD","US$",IF(L9="SGD","S$",L9&amp;" "))&amp;TEXT(K9,"#,##0")&amp;")",""),"")&amp;IF(M9&lt;&gt;"","; "&amp;M9,"")&amp;IF(O9&lt;&gt;"","; "&amp;TEXT(O9,"#,##0")&amp;" trophy/trophies","")&amp;IF(P9&lt;&gt;"","; "&amp;IF(Q9="SGD","S$",IF(Q9="USD","US$",Q9&amp;" "))&amp;TEXT(P9,"#,##0")&amp;" funding","")</x:f>
-        <x:v>Best Project — Rated best project</x:v>
+        <x:f>Hackathons!AG11</x:f>
+        <x:v>Best Project</x:v>
       </x:c>
       <x:c r="D9" s="36" t="str">
         <x:f>IF(Hackathons!Q11="","",Hackathons!Q11)</x:f>
@@ -13596,8 +13759,8 @@
         <x:v>#SPSEC SP Hackathon 2018</x:v>
       </x:c>
       <x:c r="C10" s="36" t="str">
-        <x:f>D10&amp;IF(E10&lt;&gt;""," — "&amp;E10,"")&amp;IF(F10&lt;&gt;"",IF(M10&lt;&gt;"","","; "&amp;IF(G10="SGD","S$",IF(G10="USD","US$",G10&amp;" "))&amp;TEXT(F10,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H10&lt;&gt;"","; "&amp;IF(I10="SGD","S$",IF(I10="USD","US$",I10&amp;" "))&amp;TEXT(H10,"#,##0")&amp;" credits","")&amp;IF(J10&lt;&gt;"","; "&amp;TEXT(J10,"#,##0")&amp;" subscription(s)"&amp;IF(K10&lt;&gt;""," ("&amp;IF(L10="USD","US$",IF(L10="SGD","S$",L10&amp;" "))&amp;TEXT(K10,"#,##0")&amp;")",""),"")&amp;IF(M10&lt;&gt;"","; "&amp;M10,"")&amp;IF(O10&lt;&gt;"","; "&amp;TEXT(O10,"#,##0")&amp;" trophy/trophies","")&amp;IF(P10&lt;&gt;"","; "&amp;IF(Q10="SGD","S$",IF(Q10="USD","US$",Q10&amp;" "))&amp;TEXT(P10,"#,##0")&amp;" funding","")</x:f>
-        <x:v>3rd Place; S$100 Capitaland voucher</x:v>
+        <x:f>Hackathons!AG15</x:f>
+        <x:v>3rd Place — S$100 Capitaland Voucher</x:v>
       </x:c>
       <x:c r="D10" s="36" t="str">
         <x:f>IF(Hackathons!Q15="","",Hackathons!Q15)</x:f>
@@ -13664,8 +13827,8 @@
         <x:v>#Mosque-Tech Challenge 2018</x:v>
       </x:c>
       <x:c r="C11" s="36" t="str">
-        <x:f>D11&amp;IF(E11&lt;&gt;""," — "&amp;E11,"")&amp;IF(F11&lt;&gt;"",IF(M11&lt;&gt;"","","; "&amp;IF(G11="SGD","S$",IF(G11="USD","US$",G11&amp;" "))&amp;TEXT(F11,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H11&lt;&gt;"","; "&amp;IF(I11="SGD","S$",IF(I11="USD","US$",I11&amp;" "))&amp;TEXT(H11,"#,##0")&amp;" credits","")&amp;IF(J11&lt;&gt;"","; "&amp;TEXT(J11,"#,##0")&amp;" subscription(s)"&amp;IF(K11&lt;&gt;""," ("&amp;IF(L11="USD","US$",IF(L11="SGD","S$",L11&amp;" "))&amp;TEXT(K11,"#,##0")&amp;")",""),"")&amp;IF(M11&lt;&gt;"","; "&amp;M11,"")&amp;IF(O11&lt;&gt;"","; "&amp;TEXT(O11,"#,##0")&amp;" trophy/trophies","")&amp;IF(P11&lt;&gt;"","; "&amp;IF(Q11="SGD","S$",IF(Q11="USD","US$",Q11&amp;" "))&amp;TEXT(P11,"#,##0")&amp;" funding","")</x:f>
-        <x:v>2nd Place; S$600 cash / voucher</x:v>
+        <x:f>Hackathons!AG18</x:f>
+        <x:v>2nd Place — S$600 Cash</x:v>
       </x:c>
       <x:c r="D11" s="36" t="str">
         <x:f>IF(Hackathons!Q18="","",Hackathons!Q18)</x:f>
@@ -13731,8 +13894,8 @@
         <x:v>#Mosque Hackathon 2019</x:v>
       </x:c>
       <x:c r="C12" s="36" t="str">
-        <x:f>D12&amp;IF(E12&lt;&gt;""," — "&amp;E12,"")&amp;IF(F12&lt;&gt;"",IF(M12&lt;&gt;"","","; "&amp;IF(G12="SGD","S$",IF(G12="USD","US$",G12&amp;" "))&amp;TEXT(F12,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H12&lt;&gt;"","; "&amp;IF(I12="SGD","S$",IF(I12="USD","US$",I12&amp;" "))&amp;TEXT(H12,"#,##0")&amp;" credits","")&amp;IF(J12&lt;&gt;"","; "&amp;TEXT(J12,"#,##0")&amp;" subscription(s)"&amp;IF(K12&lt;&gt;""," ("&amp;IF(L12="USD","US$",IF(L12="SGD","S$",L12&amp;" "))&amp;TEXT(K12,"#,##0")&amp;")",""),"")&amp;IF(M12&lt;&gt;"","; "&amp;M12,"")&amp;IF(O12&lt;&gt;"","; "&amp;TEXT(O12,"#,##0")&amp;" trophy/trophies","")&amp;IF(P12&lt;&gt;"","; "&amp;IF(Q12="SGD","S$",IF(Q12="USD","US$",Q12&amp;" "))&amp;TEXT(P12,"#,##0")&amp;" funding","")</x:f>
-        <x:v>3rd Place; S$500 cash / voucher</x:v>
+        <x:f>Hackathons!AG26</x:f>
+        <x:v>3rd Place — S$500 Cash</x:v>
       </x:c>
       <x:c r="D12" s="36" t="str">
         <x:f>IF(Hackathons!Q26="","",Hackathons!Q26)</x:f>
@@ -13798,12 +13961,12 @@
         <x:v>ICP Ideathon 2023</x:v>
       </x:c>
       <x:c r="C13" s="36" t="str">
-        <x:f>D13&amp;IF(E13&lt;&gt;""," — "&amp;E13,"")&amp;IF(F13&lt;&gt;"",IF(M13&lt;&gt;"","","; "&amp;IF(G13="SGD","S$",IF(G13="USD","US$",G13&amp;" "))&amp;TEXT(F13,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H13&lt;&gt;"","; "&amp;IF(I13="SGD","S$",IF(I13="USD","US$",I13&amp;" "))&amp;TEXT(H13,"#,##0")&amp;" credits","")&amp;IF(J13&lt;&gt;"","; "&amp;TEXT(J13,"#,##0")&amp;" subscription(s)"&amp;IF(K13&lt;&gt;""," ("&amp;IF(L13="USD","US$",IF(L13="SGD","S$",L13&amp;" "))&amp;TEXT(K13,"#,##0")&amp;")",""),"")&amp;IF(M13&lt;&gt;"","; "&amp;M13,"")&amp;IF(O13&lt;&gt;"","; "&amp;TEXT(O13,"#,##0")&amp;" trophy/trophies","")&amp;IF(P13&lt;&gt;"","; "&amp;IF(Q13="SGD","S$",IF(Q13="USD","US$",Q13&amp;" "))&amp;TEXT(P13,"#,##0")&amp;" funding","")</x:f>
-        <x:v>3rd Prize; S$250 cash / voucher</x:v>
+        <x:f>Hackathons!AG34</x:f>
+        <x:v>3rd Place — S$250 Cash</x:v>
       </x:c>
       <x:c r="D13" s="36" t="str">
         <x:f>IF(Hackathons!Q34="","",Hackathons!Q34)</x:f>
-        <x:v>3rd Prize</x:v>
+        <x:v>3rd Place</x:v>
       </x:c>
       <x:c r="E13" s="36" t="str">
         <x:f>IF(Hackathons!R34="","",Hackathons!R34)</x:f>
@@ -13865,12 +14028,12 @@
         <x:v>Mosque Tech Challenge 2025</x:v>
       </x:c>
       <x:c r="C14" s="36" t="str">
-        <x:f>D14&amp;IF(E14&lt;&gt;""," — "&amp;E14,"")&amp;IF(F14&lt;&gt;"",IF(M14&lt;&gt;"","","; "&amp;IF(G14="SGD","S$",IF(G14="USD","US$",G14&amp;" "))&amp;TEXT(F14,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H14&lt;&gt;"","; "&amp;IF(I14="SGD","S$",IF(I14="USD","US$",I14&amp;" "))&amp;TEXT(H14,"#,##0")&amp;" credits","")&amp;IF(J14&lt;&gt;"","; "&amp;TEXT(J14,"#,##0")&amp;" subscription(s)"&amp;IF(K14&lt;&gt;""," ("&amp;IF(L14="USD","US$",IF(L14="SGD","S$",L14&amp;" "))&amp;TEXT(K14,"#,##0")&amp;")",""),"")&amp;IF(M14&lt;&gt;"","; "&amp;M14,"")&amp;IF(O14&lt;&gt;"","; "&amp;TEXT(O14,"#,##0")&amp;" trophy/trophies","")&amp;IF(P14&lt;&gt;"","; "&amp;IF(Q14="SGD","S$",IF(Q14="USD","US$",Q14&amp;" "))&amp;TEXT(P14,"#,##0")&amp;" funding","")</x:f>
-        <x:v>2nd Prize; S$1,000 cash / voucher</x:v>
+        <x:f>Hackathons!AG36</x:f>
+        <x:v>2nd Place — S$1,000 Cash</x:v>
       </x:c>
       <x:c r="D14" s="36" t="str">
         <x:f>IF(Hackathons!Q36="","",Hackathons!Q36)</x:f>
-        <x:v>2nd Prize</x:v>
+        <x:v>2nd Place</x:v>
       </x:c>
       <x:c r="E14" s="36" t="str">
         <x:f>IF(Hackathons!R36="","",Hackathons!R36)</x:f>
@@ -13932,8 +14095,8 @@
         <x:v>OOJU X Manus.AI Hackathon 2025</x:v>
       </x:c>
       <x:c r="C15" s="36" t="str">
-        <x:f>D15&amp;IF(E15&lt;&gt;""," — "&amp;E15,"")&amp;IF(F15&lt;&gt;"",IF(M15&lt;&gt;"","","; "&amp;IF(G15="SGD","S$",IF(G15="USD","US$",G15&amp;" "))&amp;TEXT(F15,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H15&lt;&gt;"","; "&amp;IF(I15="SGD","S$",IF(I15="USD","US$",I15&amp;" "))&amp;TEXT(H15,"#,##0")&amp;" credits","")&amp;IF(J15&lt;&gt;"","; "&amp;TEXT(J15,"#,##0")&amp;" subscription(s)"&amp;IF(K15&lt;&gt;""," ("&amp;IF(L15="USD","US$",IF(L15="SGD","S$",L15&amp;" "))&amp;TEXT(K15,"#,##0")&amp;")",""),"")&amp;IF(M15&lt;&gt;"","; "&amp;M15,"")&amp;IF(O15&lt;&gt;"","; "&amp;TEXT(O15,"#,##0")&amp;" trophy/trophies","")&amp;IF(P15&lt;&gt;"","; "&amp;IF(Q15="SGD","S$",IF(Q15="USD","US$",Q15&amp;" "))&amp;TEXT(P15,"#,##0")&amp;" funding","")</x:f>
-        <x:v>2nd Prize; 1 subscription(s) (US$39); Manus Pro subscription</x:v>
+        <x:f>Hackathons!AG39</x:f>
+        <x:v>2nd Place — Manus Pro Subscription (US$39/month)</x:v>
       </x:c>
       <x:c r="D15" s="36" t="str">
         <x:f>IF(Hackathons!Q39="","",Hackathons!Q39)</x:f>
@@ -14001,8 +14164,8 @@
         <x:v>Sarawak AI Hackathon 2025</x:v>
       </x:c>
       <x:c r="C16" s="36" t="str">
-        <x:f>D16&amp;IF(E16&lt;&gt;""," — "&amp;E16,"")&amp;IF(F16&lt;&gt;"",IF(M16&lt;&gt;"","","; "&amp;IF(G16="SGD","S$",IF(G16="USD","US$",G16&amp;" "))&amp;TEXT(F16,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H16&lt;&gt;"","; "&amp;IF(I16="SGD","S$",IF(I16="USD","US$",I16&amp;" "))&amp;TEXT(H16,"#,##0")&amp;" credits","")&amp;IF(J16&lt;&gt;"","; "&amp;TEXT(J16,"#,##0")&amp;" subscription(s)"&amp;IF(K16&lt;&gt;""," ("&amp;IF(L16="USD","US$",IF(L16="SGD","S$",L16&amp;" "))&amp;TEXT(K16,"#,##0")&amp;")",""),"")&amp;IF(M16&lt;&gt;"","; "&amp;M16,"")&amp;IF(O16&lt;&gt;"","; "&amp;TEXT(O16,"#,##0")&amp;" trophy/trophies","")&amp;IF(P16&lt;&gt;"","; "&amp;IF(Q16="SGD","S$",IF(Q16="USD","US$",Q16&amp;" "))&amp;TEXT(P16,"#,##0")&amp;" funding","")</x:f>
-        <x:v>Best Finisher — Novel Hackathon; Trophy; 1 trophy/trophies</x:v>
+        <x:f>Hackathons!AG41</x:f>
+        <x:v>Best Finisher — Novel Hackathon — Trophy</x:v>
       </x:c>
       <x:c r="D16" s="36" t="str">
         <x:f>IF(Hackathons!Q41="","",Hackathons!Q41)</x:f>
@@ -14070,8 +14233,8 @@
         <x:v>Nosana Hackathon 2025</x:v>
       </x:c>
       <x:c r="C17" s="36" t="str">
-        <x:f>D17&amp;IF(E17&lt;&gt;""," — "&amp;E17,"")&amp;IF(F17&lt;&gt;"",IF(M17&lt;&gt;"","","; "&amp;IF(G17="SGD","S$",IF(G17="USD","US$",G17&amp;" "))&amp;TEXT(F17,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H17&lt;&gt;"","; "&amp;IF(I17="SGD","S$",IF(I17="USD","US$",I17&amp;" "))&amp;TEXT(H17,"#,##0")&amp;" credits","")&amp;IF(J17&lt;&gt;"","; "&amp;TEXT(J17,"#,##0")&amp;" subscription(s)"&amp;IF(K17&lt;&gt;""," ("&amp;IF(L17="USD","US$",IF(L17="SGD","S$",L17&amp;" "))&amp;TEXT(K17,"#,##0")&amp;")",""),"")&amp;IF(M17&lt;&gt;"","; "&amp;M17,"")&amp;IF(O17&lt;&gt;"","; "&amp;TEXT(O17,"#,##0")&amp;" trophy/trophies","")&amp;IF(P17&lt;&gt;"","; "&amp;IF(Q17="SGD","S$",IF(Q17="USD","US$",Q17&amp;" "))&amp;TEXT(P17,"#,##0")&amp;" funding","")</x:f>
-        <x:v>1st Prize; US$500 credits; Nosana Cloud credit</x:v>
+        <x:f>Hackathons!AG43</x:f>
+        <x:v>1st Place — US$500 Nosana Cloud Credits</x:v>
       </x:c>
       <x:c r="D17" s="36" t="str">
         <x:f>IF(Hackathons!Q43="","",Hackathons!Q43)</x:f>
@@ -14138,8 +14301,8 @@
         <x:v>Agentfield Hackathon 2026</x:v>
       </x:c>
       <x:c r="C18" s="36" t="str">
-        <x:f>D18&amp;IF(E18&lt;&gt;""," — "&amp;E18,"")&amp;IF(F18&lt;&gt;"",IF(M18&lt;&gt;"","","; "&amp;IF(G18="SGD","S$",IF(G18="USD","US$",G18&amp;" "))&amp;TEXT(F18,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H18&lt;&gt;"","; "&amp;IF(I18="SGD","S$",IF(I18="USD","US$",I18&amp;" "))&amp;TEXT(H18,"#,##0")&amp;" credits","")&amp;IF(J18&lt;&gt;"","; "&amp;TEXT(J18,"#,##0")&amp;" subscription(s)"&amp;IF(K18&lt;&gt;""," ("&amp;IF(L18="USD","US$",IF(L18="SGD","S$",L18&amp;" "))&amp;TEXT(K18,"#,##0")&amp;")",""),"")&amp;IF(M18&lt;&gt;"","; "&amp;M18,"")&amp;IF(O18&lt;&gt;"","; "&amp;TEXT(O18,"#,##0")&amp;" trophy/trophies","")&amp;IF(P18&lt;&gt;"","; "&amp;IF(Q18="SGD","S$",IF(Q18="USD","US$",Q18&amp;" "))&amp;TEXT(P18,"#,##0")&amp;" funding","")</x:f>
-        <x:v>1st Prize; US$1,000 credits; OpenRouter credits</x:v>
+        <x:f>Hackathons!AG51</x:f>
+        <x:v>1st Place — US$1,000 OpenRouter Credits</x:v>
       </x:c>
       <x:c r="D18" s="36" t="str">
         <x:f>IF(Hackathons!Q51="","",Hackathons!Q51)</x:f>
@@ -14206,8 +14369,8 @@
         <x:v>AgentForce Hackathon 2026</x:v>
       </x:c>
       <x:c r="C19" s="36" t="str">
-        <x:f>D19&amp;IF(E19&lt;&gt;""," — "&amp;E19,"")&amp;IF(F19&lt;&gt;"",IF(M19&lt;&gt;"","","; "&amp;IF(G19="SGD","S$",IF(G19="USD","US$",G19&amp;" "))&amp;TEXT(F19,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H19&lt;&gt;"","; "&amp;IF(I19="SGD","S$",IF(I19="USD","US$",I19&amp;" "))&amp;TEXT(H19,"#,##0")&amp;" credits","")&amp;IF(J19&lt;&gt;"","; "&amp;TEXT(J19,"#,##0")&amp;" subscription(s)"&amp;IF(K19&lt;&gt;""," ("&amp;IF(L19="USD","US$",IF(L19="SGD","S$",L19&amp;" "))&amp;TEXT(K19,"#,##0")&amp;")",""),"")&amp;IF(M19&lt;&gt;"","; "&amp;M19,"")&amp;IF(O19&lt;&gt;"","; "&amp;TEXT(O19,"#,##0")&amp;" trophy/trophies","")&amp;IF(P19&lt;&gt;"","; "&amp;IF(Q19="SGD","S$",IF(Q19="USD","US$",Q19&amp;" "))&amp;TEXT(P19,"#,##0")&amp;" funding","")</x:f>
-        <x:v>1st Prize; US$500 credits; API credits</x:v>
+        <x:f>Hackathons!AG53</x:f>
+        <x:v>1st Place — US$500 API Credits</x:v>
       </x:c>
       <x:c r="D19" s="36" t="str">
         <x:f>IF(Hackathons!Q53="","",Hackathons!Q53)</x:f>
@@ -14274,8 +14437,8 @@
         <x:v>AgentForce Hackathon 2026</x:v>
       </x:c>
       <x:c r="C20" s="36" t="str">
-        <x:f>D20&amp;IF(E20&lt;&gt;""," — "&amp;E20,"")&amp;IF(F20&lt;&gt;"",IF(M20&lt;&gt;"","","; "&amp;IF(G20="SGD","S$",IF(G20="USD","US$",G20&amp;" "))&amp;TEXT(F20,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H20&lt;&gt;"","; "&amp;IF(I20="SGD","S$",IF(I20="USD","US$",I20&amp;" "))&amp;TEXT(H20,"#,##0")&amp;" credits","")&amp;IF(J20&lt;&gt;"","; "&amp;TEXT(J20,"#,##0")&amp;" subscription(s)"&amp;IF(K20&lt;&gt;""," ("&amp;IF(L20="USD","US$",IF(L20="SGD","S$",L20&amp;" "))&amp;TEXT(K20,"#,##0")&amp;")",""),"")&amp;IF(M20&lt;&gt;"","; "&amp;M20,"")&amp;IF(O20&lt;&gt;"","; "&amp;TEXT(O20,"#,##0")&amp;" trophy/trophies","")&amp;IF(P20&lt;&gt;"","; "&amp;IF(Q20="SGD","S$",IF(Q20="USD","US$",Q20&amp;" "))&amp;TEXT(P20,"#,##0")&amp;" funding","")</x:f>
-        <x:v>1st Prize; US$500 credits; API credits</x:v>
+        <x:f>Hackathons!AG54</x:f>
+        <x:v>1st Place — US$500 API Credits</x:v>
       </x:c>
       <x:c r="D20" s="36" t="str">
         <x:f>IF(Hackathons!Q54="","",Hackathons!Q54)</x:f>
@@ -14342,8 +14505,8 @@
         <x:v>SUSS X Openclaw Hackathon 2026</x:v>
       </x:c>
       <x:c r="C21" s="36" t="str">
-        <x:f>D21&amp;IF(E21&lt;&gt;""," — "&amp;E21,"")&amp;IF(F21&lt;&gt;"",IF(M21&lt;&gt;"","","; "&amp;IF(G21="SGD","S$",IF(G21="USD","US$",G21&amp;" "))&amp;TEXT(F21,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H21&lt;&gt;"","; "&amp;IF(I21="SGD","S$",IF(I21="USD","US$",I21&amp;" "))&amp;TEXT(H21,"#,##0")&amp;" credits","")&amp;IF(J21&lt;&gt;"","; "&amp;TEXT(J21,"#,##0")&amp;" subscription(s)"&amp;IF(K21&lt;&gt;""," ("&amp;IF(L21="USD","US$",IF(L21="SGD","S$",L21&amp;" "))&amp;TEXT(K21,"#,##0")&amp;")",""),"")&amp;IF(M21&lt;&gt;"","; "&amp;M21,"")&amp;IF(O21&lt;&gt;"","; "&amp;TEXT(O21,"#,##0")&amp;" trophy/trophies","")&amp;IF(P21&lt;&gt;"","; "&amp;IF(Q21="SGD","S$",IF(Q21="USD","US$",Q21&amp;" "))&amp;TEXT(P21,"#,##0")&amp;" funding","")</x:f>
-        <x:v>1st Prize; US$150 credits; Wavespeed AI credits</x:v>
+        <x:f>Hackathons!AG55</x:f>
+        <x:v>1st Place — US$150 Wavespeed AI Credits</x:v>
       </x:c>
       <x:c r="D21" s="36" t="str">
         <x:f>IF(Hackathons!Q55="","",Hackathons!Q55)</x:f>
@@ -14410,8 +14573,8 @@
         <x:v>Agora.io Voice AI Hackathon Singapore 2026</x:v>
       </x:c>
       <x:c r="C22" s="36" t="str">
-        <x:f>D22&amp;IF(E22&lt;&gt;""," — "&amp;E22,"")&amp;IF(F22&lt;&gt;"",IF(M22&lt;&gt;"","","; "&amp;IF(G22="SGD","S$",IF(G22="USD","US$",G22&amp;" "))&amp;TEXT(F22,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H22&lt;&gt;"","; "&amp;IF(I22="SGD","S$",IF(I22="USD","US$",I22&amp;" "))&amp;TEXT(H22,"#,##0")&amp;" credits","")&amp;IF(J22&lt;&gt;"","; "&amp;TEXT(J22,"#,##0")&amp;" subscription(s)"&amp;IF(K22&lt;&gt;""," ("&amp;IF(L22="USD","US$",IF(L22="SGD","S$",L22&amp;" "))&amp;TEXT(K22,"#,##0")&amp;")",""),"")&amp;IF(M22&lt;&gt;"","; "&amp;M22,"")&amp;IF(O22&lt;&gt;"","; "&amp;TEXT(O22,"#,##0")&amp;" trophy/trophies","")&amp;IF(P22&lt;&gt;"","; "&amp;IF(Q22="SGD","S$",IF(Q22="USD","US$",Q22&amp;" "))&amp;TEXT(P22,"#,##0")&amp;" funding","")</x:f>
-        <x:v>3rd Prize; S$385 credits; API credits</x:v>
+        <x:f>Hackathons!AG58</x:f>
+        <x:v>3rd Place — S$300 Cash + S$385 API Credits</x:v>
       </x:c>
       <x:c r="D22" s="36" t="str">
         <x:f>IF(Hackathons!Q58="","",Hackathons!Q58)</x:f>
@@ -14480,8 +14643,8 @@
         <x:v>Build Voice Agents with Speechmatics | TGB Buildathon 2026</x:v>
       </x:c>
       <x:c r="C23" s="36" t="str">
-        <x:f>D23&amp;IF(E23&lt;&gt;""," — "&amp;E23,"")&amp;IF(F23&lt;&gt;"",IF(M23&lt;&gt;"","","; "&amp;IF(G23="SGD","S$",IF(G23="USD","US$",G23&amp;" "))&amp;TEXT(F23,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H23&lt;&gt;"","; "&amp;IF(I23="SGD","S$",IF(I23="USD","US$",I23&amp;" "))&amp;TEXT(H23,"#,##0")&amp;" credits","")&amp;IF(J23&lt;&gt;"","; "&amp;TEXT(J23,"#,##0")&amp;" subscription(s)"&amp;IF(K23&lt;&gt;""," ("&amp;IF(L23="USD","US$",IF(L23="SGD","S$",L23&amp;" "))&amp;TEXT(K23,"#,##0")&amp;")",""),"")&amp;IF(M23&lt;&gt;"","; "&amp;M23,"")&amp;IF(O23&lt;&gt;"","; "&amp;TEXT(O23,"#,##0")&amp;" trophy/trophies","")&amp;IF(P23&lt;&gt;"","; "&amp;IF(Q23="SGD","S$",IF(Q23="USD","US$",Q23&amp;" "))&amp;TEXT(P23,"#,##0")&amp;" funding","")</x:f>
-        <x:v>Award — Speechmatics; US$2,000 credits; Speechmatics credits</x:v>
+        <x:f>Hackathons!AG61</x:f>
+        <x:v>Award — Speechmatics — US$2,000 Speechmatics Credits</x:v>
       </x:c>
       <x:c r="D23" s="36" t="str">
         <x:f>IF(Hackathons!Q61="","",Hackathons!Q61)</x:f>
@@ -14549,8 +14712,8 @@
         <x:v>Vercel Zero to Agent: Singapore (1 Hr Hackathon) 2026</x:v>
       </x:c>
       <x:c r="C24" s="36" t="str">
-        <x:f>D24&amp;IF(E24&lt;&gt;""," — "&amp;E24,"")&amp;IF(F24&lt;&gt;"",IF(M24&lt;&gt;"","","; "&amp;IF(G24="SGD","S$",IF(G24="USD","US$",G24&amp;" "))&amp;TEXT(F24,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H24&lt;&gt;"","; "&amp;IF(I24="SGD","S$",IF(I24="USD","US$",I24&amp;" "))&amp;TEXT(H24,"#,##0")&amp;" credits","")&amp;IF(J24&lt;&gt;"","; "&amp;TEXT(J24,"#,##0")&amp;" subscription(s)"&amp;IF(K24&lt;&gt;""," ("&amp;IF(L24="USD","US$",IF(L24="SGD","S$",L24&amp;" "))&amp;TEXT(K24,"#,##0")&amp;")",""),"")&amp;IF(M24&lt;&gt;"","; "&amp;M24,"")&amp;IF(O24&lt;&gt;"","; "&amp;TEXT(O24,"#,##0")&amp;" trophy/trophies","")&amp;IF(P24&lt;&gt;"","; "&amp;IF(Q24="SGD","S$",IF(Q24="USD","US$",Q24&amp;" "))&amp;TEXT(P24,"#,##0")&amp;" funding","")</x:f>
-        <x:v>Award — v0; v0 Sock</x:v>
+        <x:f>Hackathons!AG62</x:f>
+        <x:v>Award — v0 Sock</x:v>
       </x:c>
       <x:c r="D24" s="36" t="str">
         <x:f>IF(Hackathons!Q62="","",Hackathons!Q62)</x:f>
@@ -14617,8 +14780,8 @@
         <x:v>UCWS 2026 (Semi-Finals)</x:v>
       </x:c>
       <x:c r="C25" s="36" t="str">
-        <x:f>D25&amp;IF(E25&lt;&gt;""," — "&amp;E25,"")&amp;IF(F25&lt;&gt;"",IF(M25&lt;&gt;"","","; "&amp;IF(G25="SGD","S$",IF(G25="USD","US$",G25&amp;" "))&amp;TEXT(F25,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H25&lt;&gt;"","; "&amp;IF(I25="SGD","S$",IF(I25="USD","US$",I25&amp;" "))&amp;TEXT(H25,"#,##0")&amp;" credits","")&amp;IF(J25&lt;&gt;"","; "&amp;TEXT(J25,"#,##0")&amp;" subscription(s)"&amp;IF(K25&lt;&gt;""," ("&amp;IF(L25="USD","US$",IF(L25="SGD","S$",L25&amp;" "))&amp;TEXT(K25,"#,##0")&amp;")",""),"")&amp;IF(M25&lt;&gt;"","; "&amp;M25,"")&amp;IF(O25&lt;&gt;"","; "&amp;TEXT(O25,"#,##0")&amp;" trophy/trophies","")&amp;IF(P25&lt;&gt;"","; "&amp;IF(Q25="SGD","S$",IF(Q25="USD","US$",Q25&amp;" "))&amp;TEXT(P25,"#,##0")&amp;" funding","")</x:f>
-        <x:v>Top 20; US$12,000 credits; 10K OpenAI credits; 2K Gemini Cloud credits</x:v>
+        <x:f>Hackathons!AG67</x:f>
+        <x:v>Top 20 — US$12,000 Credits (OpenAI + Gemini Cloud)</x:v>
       </x:c>
       <x:c r="D25" s="36" t="str">
         <x:f>IF(Hackathons!Q67="","",Hackathons!Q67)</x:f>
@@ -14685,8 +14848,8 @@
         <x:v>BUIDL_OPC_Hackathon_SG</x:v>
       </x:c>
       <x:c r="C26" s="36" t="str">
-        <x:f>D26&amp;IF(E26&lt;&gt;""," — "&amp;E26,"")&amp;IF(F26&lt;&gt;"",IF(M26&lt;&gt;"","","; "&amp;IF(G26="SGD","S$",IF(G26="USD","US$",G26&amp;" "))&amp;TEXT(F26,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H26&lt;&gt;"","; "&amp;IF(I26="SGD","S$",IF(I26="USD","US$",I26&amp;" "))&amp;TEXT(H26,"#,##0")&amp;" credits","")&amp;IF(J26&lt;&gt;"","; "&amp;TEXT(J26,"#,##0")&amp;" subscription(s)"&amp;IF(K26&lt;&gt;""," ("&amp;IF(L26="USD","US$",IF(L26="SGD","S$",L26&amp;" "))&amp;TEXT(K26,"#,##0")&amp;")",""),"")&amp;IF(M26&lt;&gt;"","; "&amp;M26,"")&amp;IF(O26&lt;&gt;"","; "&amp;TEXT(O26,"#,##0")&amp;" trophy/trophies","")&amp;IF(P26&lt;&gt;"","; "&amp;IF(Q26="SGD","S$",IF(Q26="USD","US$",Q26&amp;" "))&amp;TEXT(P26,"#,##0")&amp;" funding","")</x:f>
-        <x:v>Award — AWS; US$4,500 credits; AWS credits</x:v>
+        <x:f>Hackathons!AG72</x:f>
+        <x:v>Award — US$4,500 AWS Credits</x:v>
       </x:c>
       <x:c r="D26" s="36" t="str">
         <x:f>IF(Hackathons!Q72="","",Hackathons!Q72)</x:f>
@@ -14754,8 +14917,8 @@
         <x:v>One AI Hackathon 2026</x:v>
       </x:c>
       <x:c r="C27" s="36" t="str">
-        <x:f>D27&amp;IF(E27&lt;&gt;""," — "&amp;E27,"")&amp;IF(F27&lt;&gt;"",IF(M27&lt;&gt;"","","; "&amp;IF(G27="SGD","S$",IF(G27="USD","US$",G27&amp;" "))&amp;TEXT(F27,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H27&lt;&gt;"","; "&amp;IF(I27="SGD","S$",IF(I27="USD","US$",I27&amp;" "))&amp;TEXT(H27,"#,##0")&amp;" credits","")&amp;IF(J27&lt;&gt;"","; "&amp;TEXT(J27,"#,##0")&amp;" subscription(s)"&amp;IF(K27&lt;&gt;""," ("&amp;IF(L27="USD","US$",IF(L27="SGD","S$",L27&amp;" "))&amp;TEXT(K27,"#,##0")&amp;")",""),"")&amp;IF(M27&lt;&gt;"","; "&amp;M27,"")&amp;IF(O27&lt;&gt;"","; "&amp;TEXT(O27,"#,##0")&amp;" trophy/trophies","")&amp;IF(P27&lt;&gt;"","; "&amp;IF(Q27="SGD","S$",IF(Q27="USD","US$",Q27&amp;" "))&amp;TEXT(P27,"#,##0")&amp;" funding","")</x:f>
-        <x:v>Best Vertical Solution — Family Office Track; US$25 credits; 2,000 Cybrdeck API credits</x:v>
+        <x:f>Hackathons!AG76</x:f>
+        <x:v>Best Vertical Solution — Family Office Track — 2,000 Cybrdeck API Credits (US$25 value)</x:v>
       </x:c>
       <x:c r="D27" s="36" t="str">
         <x:f>IF(Hackathons!Q76="","",Hackathons!Q76)</x:f>
@@ -14823,12 +14986,12 @@
         <x:v>SG × SWK Friendship AI Business Design Hackathon</x:v>
       </x:c>
       <x:c r="C28" s="36" t="str">
-        <x:f>D28&amp;IF(E28&lt;&gt;""," — "&amp;E28,"")&amp;IF(F28&lt;&gt;"",IF(M28&lt;&gt;"","","; "&amp;IF(G28="SGD","S$",IF(G28="USD","US$",G28&amp;" "))&amp;TEXT(F28,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H28&lt;&gt;"","; "&amp;IF(I28="SGD","S$",IF(I28="USD","US$",I28&amp;" "))&amp;TEXT(H28,"#,##0")&amp;" credits","")&amp;IF(J28&lt;&gt;"","; "&amp;TEXT(J28,"#,##0")&amp;" subscription(s)"&amp;IF(K28&lt;&gt;""," ("&amp;IF(L28="USD","US$",IF(L28="SGD","S$",L28&amp;" "))&amp;TEXT(K28,"#,##0")&amp;")",""),"")&amp;IF(M28&lt;&gt;"","; "&amp;M28,"")&amp;IF(O28&lt;&gt;"","; "&amp;TEXT(O28,"#,##0")&amp;" trophy/trophies","")&amp;IF(P28&lt;&gt;"","; "&amp;IF(Q28="SGD","S$",IF(Q28="USD","US$",Q28&amp;" "))&amp;TEXT(P28,"#,##0")&amp;" funding","")</x:f>
-        <x:v>First Runner Up — SG × Sarawak AI &amp; Design Hackathon 2026; US$200 credits; Trophy; Kimi AI credits; 1 trophy/trophies</x:v>
+        <x:f>Hackathons!AG80</x:f>
+        <x:v>First Runner-Up — SG × Sarawak AI &amp; Design Hackathon — US$200 Kimi AI Credits + Trophy</x:v>
       </x:c>
       <x:c r="D28" s="36" t="str">
         <x:f>IF(Hackathons!Q80="","",Hackathons!Q80)</x:f>
-        <x:v>First Runner Up</x:v>
+        <x:v>First Runner-Up</x:v>
       </x:c>
       <x:c r="E28" s="36" t="str">
         <x:f>IF(Hackathons!R80="","",Hackathons!R80)</x:f>
@@ -14894,8 +15057,8 @@
         <x:v>GPT-6 Astra Hackathon: Singapore</x:v>
       </x:c>
       <x:c r="C29" s="36" t="str">
-        <x:f>D29&amp;IF(E29&lt;&gt;""," — "&amp;E29,"")&amp;IF(F29&lt;&gt;"",IF(M29&lt;&gt;"","","; "&amp;IF(G29="SGD","S$",IF(G29="USD","US$",G29&amp;" "))&amp;TEXT(F29,"#,##0")&amp;" cash / voucher"),"")&amp;IF(H29&lt;&gt;"","; "&amp;IF(I29="SGD","S$",IF(I29="USD","US$",I29&amp;" "))&amp;TEXT(H29,"#,##0")&amp;" credits","")&amp;IF(J29&lt;&gt;"","; "&amp;TEXT(J29,"#,##0")&amp;" subscription(s)"&amp;IF(K29&lt;&gt;""," ("&amp;IF(L29="USD","US$",IF(L29="SGD","S$",L29&amp;" "))&amp;TEXT(K29,"#,##0")&amp;")",""),"")&amp;IF(M29&lt;&gt;"","; "&amp;M29,"")&amp;IF(O29&lt;&gt;"","; "&amp;TEXT(O29,"#,##0")&amp;" trophy/trophies","")&amp;IF(P29&lt;&gt;"","; "&amp;IF(Q29="SGD","S$",IF(Q29="USD","US$",Q29&amp;" "))&amp;TEXT(P29,"#,##0")&amp;" funding","")</x:f>
-        <x:v>Best Project — Best Use of GPT-Image-2.5; US$5,000 credits; OpenAI credits</x:v>
+        <x:f>Hackathons!AG81</x:f>
+        <x:v>Best Project — Best Use of GPT-Image-2.5 — US$5,000 OpenAI Credits</x:v>
       </x:c>
       <x:c r="D29" s="36" t="str">
         <x:f>IF(Hackathons!Q81="","",Hackathons!Q81)</x:f>
@@ -14966,7 +15129,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c7635549fdd4a93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1aef2d9be6946dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track prize-sharing team member counts
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R0bea597d72b04c7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R085a953c905b4a7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R794b7a9eb2a64c01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R07049fa541734a19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R78e6d45d68ab48e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R7ef7df85de984e89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R6e1cb2942a384ffe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R7aedc929a14942ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rce3807e131044f26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Re62de3c4c6474019"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R53d83a5c50b34802"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R2350369bc3714803"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2935,7 +2935,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="47">
+  <x:fills count="51">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -3167,6 +3167,26 @@
         <x:fgColor rgb="FFEAF3F8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F75B5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -3231,7 +3251,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="199">
+  <x:cellXfs count="214">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3651,6 +3671,39 @@
     <x:xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Hyperlink" xfId="1"/>
@@ -3965,6 +4018,7 @@
     <x:col min="31" max="31" width="22" hidden="0" customWidth="1"/>
     <x:col min="32" max="32" width="32" hidden="0" customWidth="1"/>
     <x:col min="33" max="33" width="58" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -4066,6 +4120,9 @@
       </x:c>
       <x:c r="AG1" s="195" t="str">
         <x:v>Award Summary</x:v>
+      </x:c>
+      <x:c r="AH1" s="203" t="str">
+        <x:v>Prize Sharing Team Members</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -4146,6 +4203,7 @@
       <x:c r="AG2" s="198" t="str">
         <x:v>1st Place — S$18,000 Seed Funding</x:v>
       </x:c>
+      <x:c r="AH2" s="206"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3">
@@ -4213,6 +4271,7 @@
       <x:c r="AE3" s="38"/>
       <x:c r="AF3" s="38"/>
       <x:c r="AG3" s="198"/>
+      <x:c r="AH3" s="206"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4">
@@ -4290,6 +4349,7 @@
       <x:c r="AG4" s="198" t="str">
         <x:v>Best Project</x:v>
       </x:c>
+      <x:c r="AH4" s="206"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5">
@@ -4377,6 +4437,7 @@
       <x:c r="AG5" s="198" t="str">
         <x:v>1st Place — Best Use of IBM Bluemix — US$100,000 IBM Bluemix Credits — SmartWatch</x:v>
       </x:c>
+      <x:c r="AH5" s="206"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6">
@@ -4444,6 +4505,7 @@
       <x:c r="AE6" s="38"/>
       <x:c r="AF6" s="38"/>
       <x:c r="AG6" s="198"/>
+      <x:c r="AH6" s="206"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7">
@@ -4519,6 +4581,7 @@
       <x:c r="AG7" s="198" t="str">
         <x:v>Top 10</x:v>
       </x:c>
+      <x:c r="AH7" s="206"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8">
@@ -4586,6 +4649,7 @@
       <x:c r="AE8" s="38"/>
       <x:c r="AF8" s="38"/>
       <x:c r="AG8" s="198"/>
+      <x:c r="AH8" s="206"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9">
@@ -4653,6 +4717,7 @@
       <x:c r="AE9" s="38"/>
       <x:c r="AF9" s="38"/>
       <x:c r="AG9" s="198"/>
+      <x:c r="AH9" s="206"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10">
@@ -4720,6 +4785,7 @@
       <x:c r="AE10" s="38"/>
       <x:c r="AF10" s="38"/>
       <x:c r="AG10" s="198"/>
+      <x:c r="AH10" s="206"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11">
@@ -4797,6 +4863,7 @@
       <x:c r="AG11" s="198" t="str">
         <x:v>Best Project</x:v>
       </x:c>
+      <x:c r="AH11" s="206"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12">
@@ -4864,6 +4931,7 @@
       <x:c r="AE12" s="38"/>
       <x:c r="AF12" s="38"/>
       <x:c r="AG12" s="198"/>
+      <x:c r="AH12" s="206"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13">
@@ -4931,6 +4999,7 @@
       <x:c r="AE13" s="38"/>
       <x:c r="AF13" s="38"/>
       <x:c r="AG13" s="198"/>
+      <x:c r="AH13" s="206"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14">
@@ -4998,6 +5067,7 @@
       <x:c r="AE14" s="38"/>
       <x:c r="AF14" s="38"/>
       <x:c r="AG14" s="198"/>
+      <x:c r="AH14" s="206"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15">
@@ -5079,6 +5149,7 @@
       <x:c r="AG15" s="198" t="str">
         <x:v>3rd Place — S$100 Capitaland Voucher</x:v>
       </x:c>
+      <x:c r="AH15" s="206"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16">
@@ -5146,6 +5217,7 @@
       <x:c r="AE16" s="38"/>
       <x:c r="AF16" s="38"/>
       <x:c r="AG16" s="198"/>
+      <x:c r="AH16" s="206"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17">
@@ -5213,6 +5285,7 @@
       <x:c r="AE17" s="38"/>
       <x:c r="AF17" s="38"/>
       <x:c r="AG17" s="198"/>
+      <x:c r="AH17" s="206"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18">
@@ -5292,6 +5365,7 @@
       <x:c r="AG18" s="198" t="str">
         <x:v>2nd Place — S$600 Cash</x:v>
       </x:c>
+      <x:c r="AH18" s="206"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19">
@@ -5359,6 +5433,7 @@
       <x:c r="AE19" s="38"/>
       <x:c r="AF19" s="38"/>
       <x:c r="AG19" s="198"/>
+      <x:c r="AH19" s="206"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20">
@@ -5426,6 +5501,7 @@
       <x:c r="AE20" s="38"/>
       <x:c r="AF20" s="38"/>
       <x:c r="AG20" s="198"/>
+      <x:c r="AH20" s="206"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21">
@@ -5493,6 +5569,7 @@
       <x:c r="AE21" s="38"/>
       <x:c r="AF21" s="38"/>
       <x:c r="AG21" s="198"/>
+      <x:c r="AH21" s="206"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22">
@@ -5560,6 +5637,7 @@
       <x:c r="AE22" s="38"/>
       <x:c r="AF22" s="38"/>
       <x:c r="AG22" s="198"/>
+      <x:c r="AH22" s="206"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23">
@@ -5627,6 +5705,7 @@
       <x:c r="AE23" s="38"/>
       <x:c r="AF23" s="38"/>
       <x:c r="AG23" s="198"/>
+      <x:c r="AH23" s="206"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24">
@@ -5694,6 +5773,7 @@
       <x:c r="AE24" s="38"/>
       <x:c r="AF24" s="38"/>
       <x:c r="AG24" s="198"/>
+      <x:c r="AH24" s="206"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25">
@@ -5761,6 +5841,7 @@
       <x:c r="AE25" s="38"/>
       <x:c r="AF25" s="38"/>
       <x:c r="AG25" s="198"/>
+      <x:c r="AH25" s="206"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26">
@@ -5840,6 +5921,7 @@
       <x:c r="AG26" s="198" t="str">
         <x:v>3rd Place — S$500 Cash</x:v>
       </x:c>
+      <x:c r="AH26" s="206"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27">
@@ -5907,6 +5989,7 @@
       <x:c r="AE27" s="38"/>
       <x:c r="AF27" s="38"/>
       <x:c r="AG27" s="198"/>
+      <x:c r="AH27" s="206"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28">
@@ -5974,6 +6057,7 @@
       <x:c r="AE28" s="38"/>
       <x:c r="AF28" s="38"/>
       <x:c r="AG28" s="198"/>
+      <x:c r="AH28" s="206"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29">
@@ -6041,6 +6125,7 @@
       <x:c r="AE29" s="38"/>
       <x:c r="AF29" s="38"/>
       <x:c r="AG29" s="198"/>
+      <x:c r="AH29" s="206"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30">
@@ -6108,6 +6193,7 @@
       <x:c r="AE30" s="38"/>
       <x:c r="AF30" s="38"/>
       <x:c r="AG30" s="198"/>
+      <x:c r="AH30" s="206"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31">
@@ -6175,6 +6261,7 @@
       <x:c r="AE31" s="38"/>
       <x:c r="AF31" s="38"/>
       <x:c r="AG31" s="198"/>
+      <x:c r="AH31" s="206"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32">
@@ -6242,6 +6329,7 @@
       <x:c r="AE32" s="38"/>
       <x:c r="AF32" s="38"/>
       <x:c r="AG32" s="198"/>
+      <x:c r="AH32" s="206"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33">
@@ -6307,6 +6395,7 @@
       <x:c r="AE33" s="38"/>
       <x:c r="AF33" s="38"/>
       <x:c r="AG33" s="198"/>
+      <x:c r="AH33" s="206"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34">
@@ -6386,6 +6475,7 @@
       <x:c r="AG34" s="198" t="str">
         <x:v>3rd Place — S$250 Cash</x:v>
       </x:c>
+      <x:c r="AH34" s="206"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35">
@@ -6453,6 +6543,7 @@
       <x:c r="AE35" s="38"/>
       <x:c r="AF35" s="38"/>
       <x:c r="AG35" s="198"/>
+      <x:c r="AH35" s="206"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36">
@@ -6532,6 +6623,7 @@
       <x:c r="AG36" s="198" t="str">
         <x:v>2nd Place — S$1,000 Cash</x:v>
       </x:c>
+      <x:c r="AH36" s="206"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37">
@@ -6599,6 +6691,7 @@
       <x:c r="AE37" s="38"/>
       <x:c r="AF37" s="38"/>
       <x:c r="AG37" s="198"/>
+      <x:c r="AH37" s="206"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38">
@@ -6666,6 +6759,7 @@
       <x:c r="AE38" s="38"/>
       <x:c r="AF38" s="38"/>
       <x:c r="AG38" s="198"/>
+      <x:c r="AH38" s="206"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39">
@@ -6749,6 +6843,7 @@
       <x:c r="AG39" s="198" t="str">
         <x:v>2nd Place — Manus Pro Subscription (US$39/month)</x:v>
       </x:c>
+      <x:c r="AH39" s="206"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40">
@@ -6816,6 +6911,7 @@
       <x:c r="AE40" s="38"/>
       <x:c r="AF40" s="38"/>
       <x:c r="AG40" s="198"/>
+      <x:c r="AH40" s="206"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41">
@@ -6896,6 +6992,7 @@
       <x:c r="AG41" s="198" t="str">
         <x:v>Best Finisher — Novel Hackathon — Trophy</x:v>
       </x:c>
+      <x:c r="AH41" s="206"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42">
@@ -6960,6 +7057,7 @@
       <x:c r="AE42" s="38"/>
       <x:c r="AF42" s="38"/>
       <x:c r="AG42" s="198"/>
+      <x:c r="AH42" s="206"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43">
@@ -7041,6 +7139,7 @@
       <x:c r="AG43" s="198" t="str">
         <x:v>1st Place — US$500 Nosana Cloud Credits</x:v>
       </x:c>
+      <x:c r="AH43" s="206"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44">
@@ -7108,6 +7207,7 @@
       <x:c r="AE44" s="38"/>
       <x:c r="AF44" s="38"/>
       <x:c r="AG44" s="198"/>
+      <x:c r="AH44" s="206"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45">
@@ -7175,6 +7275,7 @@
       <x:c r="AE45" s="38"/>
       <x:c r="AF45" s="38"/>
       <x:c r="AG45" s="198"/>
+      <x:c r="AH45" s="206"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46">
@@ -7242,6 +7343,7 @@
       <x:c r="AE46" s="38"/>
       <x:c r="AF46" s="38"/>
       <x:c r="AG46" s="198"/>
+      <x:c r="AH46" s="206"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47">
@@ -7309,6 +7411,7 @@
       <x:c r="AE47" s="38"/>
       <x:c r="AF47" s="38"/>
       <x:c r="AG47" s="198"/>
+      <x:c r="AH47" s="206"/>
     </x:row>
     <x:row r="48" ht="49.75" customHeight="1">
       <x:c r="A48">
@@ -7376,6 +7479,7 @@
       <x:c r="AE48" s="38"/>
       <x:c r="AF48" s="38"/>
       <x:c r="AG48" s="198"/>
+      <x:c r="AH48" s="206"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49">
@@ -7443,6 +7547,7 @@
       <x:c r="AE49" s="38"/>
       <x:c r="AF49" s="38"/>
       <x:c r="AG49" s="198"/>
+      <x:c r="AH49" s="206"/>
     </x:row>
     <x:row r="50" ht="34">
       <x:c r="A50">
@@ -7510,6 +7615,7 @@
       <x:c r="AE50" s="38"/>
       <x:c r="AF50" s="38"/>
       <x:c r="AG50" s="198"/>
+      <x:c r="AH50" s="206"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51">
@@ -7591,6 +7697,7 @@
       <x:c r="AG51" s="198" t="str">
         <x:v>1st Place — US$1,000 OpenRouter Credits</x:v>
       </x:c>
+      <x:c r="AH51" s="206"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52">
@@ -7658,6 +7765,7 @@
       <x:c r="AE52" s="38"/>
       <x:c r="AF52" s="38"/>
       <x:c r="AG52" s="198"/>
+      <x:c r="AH52" s="206"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53">
@@ -7739,6 +7847,7 @@
       <x:c r="AG53" s="198" t="str">
         <x:v>1st Place — US$500 API Credits</x:v>
       </x:c>
+      <x:c r="AH53" s="206"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54">
@@ -7820,6 +7929,7 @@
       <x:c r="AG54" s="198" t="str">
         <x:v>1st Place — US$500 API Credits</x:v>
       </x:c>
+      <x:c r="AH54" s="206"/>
     </x:row>
     <x:row r="55" ht="34">
       <x:c r="A55">
@@ -7901,6 +8011,7 @@
       <x:c r="AG55" s="198" t="str">
         <x:v>1st Place — US$150 Wavespeed AI Credits</x:v>
       </x:c>
+      <x:c r="AH55" s="206"/>
     </x:row>
     <x:row r="56" ht="17">
       <x:c r="A56">
@@ -7968,6 +8079,7 @@
       <x:c r="AE56" s="38"/>
       <x:c r="AF56" s="38"/>
       <x:c r="AG56" s="198"/>
+      <x:c r="AH56" s="206"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57">
@@ -8035,6 +8147,7 @@
       <x:c r="AE57" s="38"/>
       <x:c r="AF57" s="38"/>
       <x:c r="AG57" s="198"/>
+      <x:c r="AH57" s="206"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58">
@@ -8120,6 +8233,7 @@
       <x:c r="AG58" s="198" t="str">
         <x:v>3rd Place — S$300 Cash + S$385 API Credits</x:v>
       </x:c>
+      <x:c r="AH58" s="206"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59">
@@ -8187,6 +8301,7 @@
       <x:c r="AE59" s="38"/>
       <x:c r="AF59" s="38"/>
       <x:c r="AG59" s="198"/>
+      <x:c r="AH59" s="206"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60">
@@ -8254,6 +8369,7 @@
       <x:c r="AE60" s="38"/>
       <x:c r="AF60" s="38"/>
       <x:c r="AG60" s="198"/>
+      <x:c r="AH60" s="206"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61">
@@ -8337,6 +8453,7 @@
       <x:c r="AG61" s="198" t="str">
         <x:v>Award — Speechmatics — US$2,000 Speechmatics Credits</x:v>
       </x:c>
+      <x:c r="AH61" s="206"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62">
@@ -8420,6 +8537,7 @@
       <x:c r="AG62" s="198" t="str">
         <x:v>Award — v0 Sock</x:v>
       </x:c>
+      <x:c r="AH62" s="206"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63">
@@ -8487,6 +8605,7 @@
       <x:c r="AE63" s="38"/>
       <x:c r="AF63" s="38"/>
       <x:c r="AG63" s="198"/>
+      <x:c r="AH63" s="206"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64">
@@ -8554,6 +8673,7 @@
       <x:c r="AE64" s="38"/>
       <x:c r="AF64" s="38"/>
       <x:c r="AG64" s="198"/>
+      <x:c r="AH64" s="206"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65">
@@ -8621,6 +8741,7 @@
       <x:c r="AE65" s="38"/>
       <x:c r="AF65" s="38"/>
       <x:c r="AG65" s="198"/>
+      <x:c r="AH65" s="206"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66">
@@ -8688,6 +8809,7 @@
       <x:c r="AE66" s="38"/>
       <x:c r="AF66" s="38"/>
       <x:c r="AG66" s="198"/>
+      <x:c r="AH66" s="206"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67">
@@ -8769,6 +8891,7 @@
       <x:c r="AG67" s="198" t="str">
         <x:v>Top 20 — US$12,000 Credits (OpenAI + Gemini Cloud)</x:v>
       </x:c>
+      <x:c r="AH67" s="206"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68">
@@ -8836,6 +8959,7 @@
       <x:c r="AE68" s="38"/>
       <x:c r="AF68" s="38"/>
       <x:c r="AG68" s="198"/>
+      <x:c r="AH68" s="206"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69">
@@ -8903,6 +9027,7 @@
       <x:c r="AE69" s="38"/>
       <x:c r="AF69" s="38"/>
       <x:c r="AG69" s="198"/>
+      <x:c r="AH69" s="206"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70">
@@ -8967,6 +9092,7 @@
       <x:c r="AE70" s="38"/>
       <x:c r="AF70" s="38"/>
       <x:c r="AG70" s="198"/>
+      <x:c r="AH70" s="206"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71">
@@ -9034,6 +9160,7 @@
       <x:c r="AE71" s="38"/>
       <x:c r="AF71" s="38"/>
       <x:c r="AG71" s="198"/>
+      <x:c r="AH71" s="206"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72">
@@ -9117,6 +9244,7 @@
       <x:c r="AG72" s="198" t="str">
         <x:v>Award — US$4,500 AWS Credits</x:v>
       </x:c>
+      <x:c r="AH72" s="206"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73">
@@ -9184,6 +9312,7 @@
       <x:c r="AE73" s="38"/>
       <x:c r="AF73" s="38"/>
       <x:c r="AG73" s="198"/>
+      <x:c r="AH73" s="206"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74">
@@ -9251,6 +9380,7 @@
       <x:c r="AE74" s="38"/>
       <x:c r="AF74" s="38"/>
       <x:c r="AG74" s="198"/>
+      <x:c r="AH74" s="206"/>
     </x:row>
     <x:row r="75" ht="34">
       <x:c r="A75">
@@ -9318,6 +9448,7 @@
       <x:c r="AE75" s="38"/>
       <x:c r="AF75" s="38"/>
       <x:c r="AG75" s="198"/>
+      <x:c r="AH75" s="206"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76">
@@ -9401,6 +9532,7 @@
       <x:c r="AG76" s="198" t="str">
         <x:v>Best Vertical Solution — Family Office Track — 2,000 Cybrdeck API Credits (US$25 value)</x:v>
       </x:c>
+      <x:c r="AH76" s="206"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77">
@@ -9468,6 +9600,7 @@
       <x:c r="AE77" s="38"/>
       <x:c r="AF77" s="38"/>
       <x:c r="AG77" s="198"/>
+      <x:c r="AH77" s="206"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78">
@@ -9535,6 +9668,7 @@
       <x:c r="AE78" s="38"/>
       <x:c r="AF78" s="38"/>
       <x:c r="AG78" s="198"/>
+      <x:c r="AH78" s="206"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79">
@@ -9602,6 +9736,7 @@
       <x:c r="AE79" s="38"/>
       <x:c r="AF79" s="38"/>
       <x:c r="AG79" s="198"/>
+      <x:c r="AH79" s="206"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" t="n">
@@ -9689,6 +9824,7 @@
       <x:c r="AG80" s="198" t="str">
         <x:v>First Runner-Up — SG × Sarawak AI &amp; Design Hackathon — US$200 Kimi AI Credits + Trophy</x:v>
       </x:c>
+      <x:c r="AH80" s="206"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" t="n">
@@ -9772,6 +9908,7 @@
       <x:c r="AG81" s="198" t="str">
         <x:v>Best Project — Best Use of GPT-Image-2.5 — US$5,000 OpenAI Credits</x:v>
       </x:c>
+      <x:c r="AH81" s="206"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" t="n">
@@ -9837,13 +9974,14 @@
       <x:c r="AE82" s="38"/>
       <x:c r="AF82" s="38"/>
       <x:c r="AG82" s="198"/>
+      <x:c r="AH82" s="206"/>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R27e30ceef8f54e31"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R621a569fdc794f82"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rf6436f694a7342d5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R0f731b896efd49b6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R51f31ee7e26f4be9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R84401180a1f24449"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R642f9c0516584ef8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R7ec5528115b448ef"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11421,12 +11559,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rd70e071e6dbd49bd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R37aecd44f30641a3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rfda7e61034354180"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rcb19bfebc42047cd"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R978dbdb592c142e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R912d3e14b9604875"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12329,7 +12467,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6859fb134c8a44f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f85c45b37224e49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13312,16 +13450,17 @@
     <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="16" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="32" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="105" t="str">
+      <x:c r="A1" s="207" t="str">
         <x:v>Prize Money — Detailed Breakdown</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="106" t="str">
-        <x:v>One row per currently classified award or prize record. Award Summary uses a curated, standardized format; the raw original award text remains preserved on Hackathons.</x:v>
+        <x:v>One row per currently classified award or prize record. Award Summary uses a curated, standardized format; enter the number sharing a prize in Hackathons column AH.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -13414,6 +13553,9 @@
       <x:c r="S4" s="90" t="str">
         <x:v>Review note</x:v>
       </x:c>
+      <x:c r="T4" s="212" t="str">
+        <x:v>Prize Sharing Team Members</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="36" t="n">
@@ -13481,6 +13623,9 @@
         <x:f>IF(Hackathons!AF2="","",Hackathons!AF2)</x:f>
         <x:v>Funding, not a cash prize</x:v>
       </x:c>
+      <x:c r="T5" s="213" t="str">
+        <x:f>IF(Hackathons!AH2="","",Hackathons!AH2)</x:f>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="36" t="n">
@@ -13547,6 +13692,9 @@
         <x:f>IF(Hackathons!AF4="","",Hackathons!AF4)</x:f>
         <x:v>Recognition only</x:v>
       </x:c>
+      <x:c r="T6" s="213" t="str">
+        <x:f>IF(Hackathons!AH4="","",Hackathons!AH4)</x:f>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="36" t="n">
@@ -13617,6 +13765,9 @@
         <x:f>IF(Hackathons!AF5="","",Hackathons!AF5)</x:f>
         <x:v>US$100,000 IBM Bluemix credit value</x:v>
       </x:c>
+      <x:c r="T7" s="213" t="str">
+        <x:f>IF(Hackathons!AH5="","",Hackathons!AH5)</x:f>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="36" t="n">
@@ -13682,6 +13833,9 @@
         <x:f>IF(Hackathons!AF7="","",Hackathons!AF7)</x:f>
         <x:v>Recognition only</x:v>
       </x:c>
+      <x:c r="T8" s="213" t="str">
+        <x:f>IF(Hackathons!AH7="","",Hackathons!AH7)</x:f>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="36" t="n">
@@ -13748,6 +13902,9 @@
         <x:f>IF(Hackathons!AF11="","",Hackathons!AF11)</x:f>
         <x:v>Recognition only</x:v>
       </x:c>
+      <x:c r="T9" s="213" t="str">
+        <x:f>IF(Hackathons!AH11="","",Hackathons!AH11)</x:f>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="36" t="n">
@@ -13816,6 +13973,9 @@
         <x:f>IF(Hackathons!AF15="","",Hackathons!AF15)</x:f>
         <x:v>Voucher counted as cash equivalent</x:v>
       </x:c>
+      <x:c r="T10" s="213" t="str">
+        <x:f>IF(Hackathons!AH15="","",Hackathons!AH15)</x:f>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="36" t="n">
@@ -13883,6 +14043,9 @@
         <x:f>IF(Hackathons!AF18="","",Hackathons!AF18)</x:f>
         <x:v>Explicit cash</x:v>
       </x:c>
+      <x:c r="T11" s="213" t="str">
+        <x:f>IF(Hackathons!AH18="","",Hackathons!AH18)</x:f>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="36" t="n">
@@ -13949,6 +14112,9 @@
       <x:c r="S12" s="98" t="str">
         <x:f>IF(Hackathons!AF26="","",Hackathons!AF26)</x:f>
         <x:v>Explicit cash</x:v>
+      </x:c>
+      <x:c r="T12" s="213" t="str">
+        <x:f>IF(Hackathons!AH26="","",Hackathons!AH26)</x:f>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -14017,6 +14183,9 @@
         <x:f>IF(Hackathons!AF34="","",Hackathons!AF34)</x:f>
         <x:v>Confirmed cash</x:v>
       </x:c>
+      <x:c r="T13" s="213" t="str">
+        <x:f>IF(Hackathons!AH34="","",Hackathons!AH34)</x:f>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="36" t="n">
@@ -14084,6 +14253,9 @@
         <x:f>IF(Hackathons!AF36="","",Hackathons!AF36)</x:f>
         <x:v>Confirmed cash</x:v>
       </x:c>
+      <x:c r="T14" s="213" t="str">
+        <x:f>IF(Hackathons!AH36="","",Hackathons!AH36)</x:f>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="36" t="n">
@@ -14153,6 +14325,9 @@
         <x:f>IF(Hackathons!AF39="","",Hackathons!AF39)</x:f>
         <x:v>US$39 monthly value at award period</x:v>
       </x:c>
+      <x:c r="T15" s="213" t="str">
+        <x:f>IF(Hackathons!AH39="","",Hackathons!AH39)</x:f>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="36" t="n">
@@ -14222,6 +14397,9 @@
         <x:f>IF(Hackathons!AF41="","",Hackathons!AF41)</x:f>
         <x:v>Trophy, not cash</x:v>
       </x:c>
+      <x:c r="T16" s="213" t="str">
+        <x:f>IF(Hackathons!AH41="","",Hackathons!AH41)</x:f>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="36" t="n">
@@ -14290,6 +14468,9 @@
         <x:f>IF(Hackathons!AF43="","",Hackathons!AF43)</x:f>
         <x:v>Cloud credit, not cash</x:v>
       </x:c>
+      <x:c r="T17" s="213" t="str">
+        <x:f>IF(Hackathons!AH43="","",Hackathons!AH43)</x:f>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="36" t="n">
@@ -14358,6 +14539,9 @@
         <x:f>IF(Hackathons!AF51="","",Hackathons!AF51)</x:f>
         <x:v>API credits, not cash</x:v>
       </x:c>
+      <x:c r="T18" s="213" t="str">
+        <x:f>IF(Hackathons!AH51="","",Hackathons!AH51)</x:f>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="36" t="n">
@@ -14426,6 +14610,9 @@
         <x:f>IF(Hackathons!AF53="","",Hackathons!AF53)</x:f>
         <x:v>API credits, not cash</x:v>
       </x:c>
+      <x:c r="T19" s="213" t="str">
+        <x:f>IF(Hackathons!AH53="","",Hackathons!AH53)</x:f>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="36" t="n">
@@ -14494,6 +14681,9 @@
         <x:f>IF(Hackathons!AF54="","",Hackathons!AF54)</x:f>
         <x:v>API credits, not cash</x:v>
       </x:c>
+      <x:c r="T20" s="213" t="str">
+        <x:f>IF(Hackathons!AH54="","",Hackathons!AH54)</x:f>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="36" t="n">
@@ -14562,6 +14752,9 @@
         <x:f>IF(Hackathons!AF55="","",Hackathons!AF55)</x:f>
         <x:v>API credits, not cash</x:v>
       </x:c>
+      <x:c r="T21" s="213" t="str">
+        <x:f>IF(Hackathons!AH55="","",Hackathons!AH55)</x:f>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="36" t="n">
@@ -14632,6 +14825,9 @@
         <x:f>IF(Hackathons!AF58="","",Hackathons!AF58)</x:f>
         <x:v>Explicit cash; API credit value also tracked</x:v>
       </x:c>
+      <x:c r="T22" s="213" t="str">
+        <x:f>IF(Hackathons!AH58="","",Hackathons!AH58)</x:f>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="36" t="n">
@@ -14701,6 +14897,9 @@
         <x:f>IF(Hackathons!AF61="","",Hackathons!AF61)</x:f>
         <x:v>USD-denominated credit value</x:v>
       </x:c>
+      <x:c r="T23" s="213" t="str">
+        <x:f>IF(Hackathons!AH61="","",Hackathons!AH61)</x:f>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="36" t="n">
@@ -14769,6 +14968,9 @@
         <x:f>IF(Hackathons!AF62="","",Hackathons!AF62)</x:f>
         <x:v>Physical item, not cash</x:v>
       </x:c>
+      <x:c r="T24" s="213" t="str">
+        <x:f>IF(Hackathons!AH62="","",Hackathons!AH62)</x:f>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="36" t="n">
@@ -14837,6 +15039,9 @@
         <x:f>IF(Hackathons!AF67="","",Hackathons!AF67)</x:f>
         <x:v>Credit value total combines two USD-denominated credits</x:v>
       </x:c>
+      <x:c r="T25" s="213" t="str">
+        <x:f>IF(Hackathons!AH67="","",Hackathons!AH67)</x:f>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="36" t="n">
@@ -14906,6 +15111,9 @@
         <x:f>IF(Hackathons!AF72="","",Hackathons!AF72)</x:f>
         <x:v>USD-denominated credit value</x:v>
       </x:c>
+      <x:c r="T26" s="213" t="str">
+        <x:f>IF(Hackathons!AH72="","",Hackathons!AH72)</x:f>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="36" t="n">
@@ -14975,6 +15183,9 @@
         <x:f>IF(Hackathons!AF76="","",Hackathons!AF76)</x:f>
         <x:v>US$25 credit value, not cash</x:v>
       </x:c>
+      <x:c r="T27" s="213" t="str">
+        <x:f>IF(Hackathons!AH76="","",Hackathons!AH76)</x:f>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="36" t="n">
@@ -15046,6 +15257,9 @@
         <x:f>IF(Hackathons!AF80="","",Hackathons!AF80)</x:f>
         <x:v>Trophy excluded; credit value tracked</x:v>
       </x:c>
+      <x:c r="T28" s="213" t="str">
+        <x:f>IF(Hackathons!AH80="","",Hackathons!AH80)</x:f>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="36" t="n">
@@ -15115,21 +15329,24 @@
         <x:f>IF(Hackathons!AF81="","",Hackathons!AF81)</x:f>
         <x:v>Credit value tracked</x:v>
       </x:c>
+      <x:c r="T29" s="213" t="str">
+        <x:f>IF(Hackathons!AH81="","",Hackathons!AH81)</x:f>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:S1"/>
-    <x:mergeCell ref="A2:S2"/>
     <x:mergeCell ref="A3:C3"/>
     <x:mergeCell ref="D3:E3"/>
     <x:mergeCell ref="F3:H3"/>
     <x:mergeCell ref="I3:J3"/>
     <x:mergeCell ref="L3:N3"/>
     <x:mergeCell ref="O3:P3"/>
+    <x:mergeCell ref="A1:T1"/>
+    <x:mergeCell ref="A2:T2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1aef2d9be6946dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red2e66bf212a44db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Derive prize team counts from hackathon rosters
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R6e1cb2942a384ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R7aedc929a14942ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rce3807e131044f26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Re62de3c4c6474019"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R53d83a5c50b34802"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R2350369bc3714803"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R78055f633f7e4572"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rede65b37755745f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rb2d6e1ac63dc49a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R201f137145ff4a7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R3c2e97e6d4e84ad0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Rd026b830326e4d9b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3251,7 +3251,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="214">
+  <x:cellXfs count="215">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3704,6 +3704,9 @@
     <x:xf numFmtId="201" fontId="0" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Hyperlink" xfId="1"/>
@@ -4122,7 +4125,7 @@
         <x:v>Award Summary</x:v>
       </x:c>
       <x:c r="AH1" s="203" t="str">
-        <x:v>Prize Sharing Team Members</x:v>
+        <x:v>Hackathon Team Members</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -4203,7 +4206,10 @@
       <x:c r="AG2" s="198" t="str">
         <x:v>1st Place — S$18,000 Seed Funding</x:v>
       </x:c>
-      <x:c r="AH2" s="206"/>
+      <x:c r="AH2" s="214" t="n">
+        <x:f>IF(OR(J2="",J2="-"),"",LEN(J2)-LEN(SUBSTITUTE(J2,",",""))+1)</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3">
@@ -4271,7 +4277,10 @@
       <x:c r="AE3" s="38"/>
       <x:c r="AF3" s="38"/>
       <x:c r="AG3" s="198"/>
-      <x:c r="AH3" s="206"/>
+      <x:c r="AH3" s="214" t="n">
+        <x:f>IF(OR(J3="",J3="-"),"",LEN(J3)-LEN(SUBSTITUTE(J3,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4">
@@ -4349,7 +4358,10 @@
       <x:c r="AG4" s="198" t="str">
         <x:v>Best Project</x:v>
       </x:c>
-      <x:c r="AH4" s="206"/>
+      <x:c r="AH4" s="214" t="n">
+        <x:f>IF(OR(J4="",J4="-"),"",LEN(J4)-LEN(SUBSTITUTE(J4,",",""))+1)</x:f>
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5">
@@ -4437,7 +4449,10 @@
       <x:c r="AG5" s="198" t="str">
         <x:v>1st Place — Best Use of IBM Bluemix — US$100,000 IBM Bluemix Credits — SmartWatch</x:v>
       </x:c>
-      <x:c r="AH5" s="206"/>
+      <x:c r="AH5" s="214" t="n">
+        <x:f>IF(OR(J5="",J5="-"),"",LEN(J5)-LEN(SUBSTITUTE(J5,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6">
@@ -4505,7 +4520,10 @@
       <x:c r="AE6" s="38"/>
       <x:c r="AF6" s="38"/>
       <x:c r="AG6" s="198"/>
-      <x:c r="AH6" s="206"/>
+      <x:c r="AH6" s="214" t="n">
+        <x:f>IF(OR(J6="",J6="-"),"",LEN(J6)-LEN(SUBSTITUTE(J6,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7">
@@ -4581,7 +4599,10 @@
       <x:c r="AG7" s="198" t="str">
         <x:v>Top 10</x:v>
       </x:c>
-      <x:c r="AH7" s="206"/>
+      <x:c r="AH7" s="214" t="n">
+        <x:f>IF(OR(J7="",J7="-"),"",LEN(J7)-LEN(SUBSTITUTE(J7,",",""))+1)</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8">
@@ -4649,7 +4670,10 @@
       <x:c r="AE8" s="38"/>
       <x:c r="AF8" s="38"/>
       <x:c r="AG8" s="198"/>
-      <x:c r="AH8" s="206"/>
+      <x:c r="AH8" s="214" t="n">
+        <x:f>IF(OR(J8="",J8="-"),"",LEN(J8)-LEN(SUBSTITUTE(J8,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9">
@@ -4717,7 +4741,10 @@
       <x:c r="AE9" s="38"/>
       <x:c r="AF9" s="38"/>
       <x:c r="AG9" s="198"/>
-      <x:c r="AH9" s="206"/>
+      <x:c r="AH9" s="214" t="n">
+        <x:f>IF(OR(J9="",J9="-"),"",LEN(J9)-LEN(SUBSTITUTE(J9,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10">
@@ -4785,7 +4812,10 @@
       <x:c r="AE10" s="38"/>
       <x:c r="AF10" s="38"/>
       <x:c r="AG10" s="198"/>
-      <x:c r="AH10" s="206"/>
+      <x:c r="AH10" s="214" t="n">
+        <x:f>IF(OR(J10="",J10="-"),"",LEN(J10)-LEN(SUBSTITUTE(J10,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11">
@@ -4863,7 +4893,10 @@
       <x:c r="AG11" s="198" t="str">
         <x:v>Best Project</x:v>
       </x:c>
-      <x:c r="AH11" s="206"/>
+      <x:c r="AH11" s="214" t="n">
+        <x:f>IF(OR(J11="",J11="-"),"",LEN(J11)-LEN(SUBSTITUTE(J11,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12">
@@ -4931,7 +4964,10 @@
       <x:c r="AE12" s="38"/>
       <x:c r="AF12" s="38"/>
       <x:c r="AG12" s="198"/>
-      <x:c r="AH12" s="206"/>
+      <x:c r="AH12" s="214" t="n">
+        <x:f>IF(OR(J12="",J12="-"),"",LEN(J12)-LEN(SUBSTITUTE(J12,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13">
@@ -4999,7 +5035,10 @@
       <x:c r="AE13" s="38"/>
       <x:c r="AF13" s="38"/>
       <x:c r="AG13" s="198"/>
-      <x:c r="AH13" s="206"/>
+      <x:c r="AH13" s="214" t="n">
+        <x:f>IF(OR(J13="",J13="-"),"",LEN(J13)-LEN(SUBSTITUTE(J13,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14">
@@ -5067,7 +5106,10 @@
       <x:c r="AE14" s="38"/>
       <x:c r="AF14" s="38"/>
       <x:c r="AG14" s="198"/>
-      <x:c r="AH14" s="206"/>
+      <x:c r="AH14" s="214" t="n">
+        <x:f>IF(OR(J14="",J14="-"),"",LEN(J14)-LEN(SUBSTITUTE(J14,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15">
@@ -5149,7 +5191,10 @@
       <x:c r="AG15" s="198" t="str">
         <x:v>3rd Place — S$100 Capitaland Voucher</x:v>
       </x:c>
-      <x:c r="AH15" s="206"/>
+      <x:c r="AH15" s="214" t="n">
+        <x:f>IF(OR(J15="",J15="-"),"",LEN(J15)-LEN(SUBSTITUTE(J15,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16">
@@ -5217,7 +5262,10 @@
       <x:c r="AE16" s="38"/>
       <x:c r="AF16" s="38"/>
       <x:c r="AG16" s="198"/>
-      <x:c r="AH16" s="206"/>
+      <x:c r="AH16" s="214" t="n">
+        <x:f>IF(OR(J16="",J16="-"),"",LEN(J16)-LEN(SUBSTITUTE(J16,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17">
@@ -5285,7 +5333,10 @@
       <x:c r="AE17" s="38"/>
       <x:c r="AF17" s="38"/>
       <x:c r="AG17" s="198"/>
-      <x:c r="AH17" s="206"/>
+      <x:c r="AH17" s="214" t="n">
+        <x:f>IF(OR(J17="",J17="-"),"",LEN(J17)-LEN(SUBSTITUTE(J17,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18">
@@ -5365,7 +5416,10 @@
       <x:c r="AG18" s="198" t="str">
         <x:v>2nd Place — S$600 Cash</x:v>
       </x:c>
-      <x:c r="AH18" s="206"/>
+      <x:c r="AH18" s="214" t="n">
+        <x:f>IF(OR(J18="",J18="-"),"",LEN(J18)-LEN(SUBSTITUTE(J18,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19">
@@ -5433,7 +5487,10 @@
       <x:c r="AE19" s="38"/>
       <x:c r="AF19" s="38"/>
       <x:c r="AG19" s="198"/>
-      <x:c r="AH19" s="206"/>
+      <x:c r="AH19" s="214" t="n">
+        <x:f>IF(OR(J19="",J19="-"),"",LEN(J19)-LEN(SUBSTITUTE(J19,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20">
@@ -5501,7 +5558,10 @@
       <x:c r="AE20" s="38"/>
       <x:c r="AF20" s="38"/>
       <x:c r="AG20" s="198"/>
-      <x:c r="AH20" s="206"/>
+      <x:c r="AH20" s="214" t="n">
+        <x:f>IF(OR(J20="",J20="-"),"",LEN(J20)-LEN(SUBSTITUTE(J20,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21">
@@ -5569,7 +5629,10 @@
       <x:c r="AE21" s="38"/>
       <x:c r="AF21" s="38"/>
       <x:c r="AG21" s="198"/>
-      <x:c r="AH21" s="206"/>
+      <x:c r="AH21" s="214" t="n">
+        <x:f>IF(OR(J21="",J21="-"),"",LEN(J21)-LEN(SUBSTITUTE(J21,",",""))+1)</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22">
@@ -5637,7 +5700,10 @@
       <x:c r="AE22" s="38"/>
       <x:c r="AF22" s="38"/>
       <x:c r="AG22" s="198"/>
-      <x:c r="AH22" s="206"/>
+      <x:c r="AH22" s="214" t="n">
+        <x:f>IF(OR(J22="",J22="-"),"",LEN(J22)-LEN(SUBSTITUTE(J22,",",""))+1)</x:f>
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23">
@@ -5705,7 +5771,10 @@
       <x:c r="AE23" s="38"/>
       <x:c r="AF23" s="38"/>
       <x:c r="AG23" s="198"/>
-      <x:c r="AH23" s="206"/>
+      <x:c r="AH23" s="214" t="n">
+        <x:f>IF(OR(J23="",J23="-"),"",LEN(J23)-LEN(SUBSTITUTE(J23,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24">
@@ -5773,7 +5842,10 @@
       <x:c r="AE24" s="38"/>
       <x:c r="AF24" s="38"/>
       <x:c r="AG24" s="198"/>
-      <x:c r="AH24" s="206"/>
+      <x:c r="AH24" s="214" t="n">
+        <x:f>IF(OR(J24="",J24="-"),"",LEN(J24)-LEN(SUBSTITUTE(J24,",",""))+1)</x:f>
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25">
@@ -5841,7 +5913,10 @@
       <x:c r="AE25" s="38"/>
       <x:c r="AF25" s="38"/>
       <x:c r="AG25" s="198"/>
-      <x:c r="AH25" s="206"/>
+      <x:c r="AH25" s="214" t="n">
+        <x:f>IF(OR(J25="",J25="-"),"",LEN(J25)-LEN(SUBSTITUTE(J25,",",""))+1)</x:f>
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26">
@@ -5921,7 +5996,10 @@
       <x:c r="AG26" s="198" t="str">
         <x:v>3rd Place — S$500 Cash</x:v>
       </x:c>
-      <x:c r="AH26" s="206"/>
+      <x:c r="AH26" s="214" t="n">
+        <x:f>IF(OR(J26="",J26="-"),"",LEN(J26)-LEN(SUBSTITUTE(J26,",",""))+1)</x:f>
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27">
@@ -5989,7 +6067,10 @@
       <x:c r="AE27" s="38"/>
       <x:c r="AF27" s="38"/>
       <x:c r="AG27" s="198"/>
-      <x:c r="AH27" s="206"/>
+      <x:c r="AH27" s="214" t="n">
+        <x:f>IF(OR(J27="",J27="-"),"",LEN(J27)-LEN(SUBSTITUTE(J27,",",""))+1)</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28">
@@ -6057,7 +6138,10 @@
       <x:c r="AE28" s="38"/>
       <x:c r="AF28" s="38"/>
       <x:c r="AG28" s="198"/>
-      <x:c r="AH28" s="206"/>
+      <x:c r="AH28" s="214" t="n">
+        <x:f>IF(OR(J28="",J28="-"),"",LEN(J28)-LEN(SUBSTITUTE(J28,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29">
@@ -6125,7 +6209,10 @@
       <x:c r="AE29" s="38"/>
       <x:c r="AF29" s="38"/>
       <x:c r="AG29" s="198"/>
-      <x:c r="AH29" s="206"/>
+      <x:c r="AH29" s="214" t="n">
+        <x:f>IF(OR(J29="",J29="-"),"",LEN(J29)-LEN(SUBSTITUTE(J29,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30">
@@ -6193,7 +6280,10 @@
       <x:c r="AE30" s="38"/>
       <x:c r="AF30" s="38"/>
       <x:c r="AG30" s="198"/>
-      <x:c r="AH30" s="206"/>
+      <x:c r="AH30" s="214" t="n">
+        <x:f>IF(OR(J30="",J30="-"),"",LEN(J30)-LEN(SUBSTITUTE(J30,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31">
@@ -6261,7 +6351,10 @@
       <x:c r="AE31" s="38"/>
       <x:c r="AF31" s="38"/>
       <x:c r="AG31" s="198"/>
-      <x:c r="AH31" s="206"/>
+      <x:c r="AH31" s="214" t="n">
+        <x:f>IF(OR(J31="",J31="-"),"",LEN(J31)-LEN(SUBSTITUTE(J31,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32">
@@ -6329,7 +6422,10 @@
       <x:c r="AE32" s="38"/>
       <x:c r="AF32" s="38"/>
       <x:c r="AG32" s="198"/>
-      <x:c r="AH32" s="206"/>
+      <x:c r="AH32" s="214" t="n">
+        <x:f>IF(OR(J32="",J32="-"),"",LEN(J32)-LEN(SUBSTITUTE(J32,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33">
@@ -6395,7 +6491,10 @@
       <x:c r="AE33" s="38"/>
       <x:c r="AF33" s="38"/>
       <x:c r="AG33" s="198"/>
-      <x:c r="AH33" s="206"/>
+      <x:c r="AH33" s="214" t="n">
+        <x:f>IF(OR(J33="",J33="-"),"",LEN(J33)-LEN(SUBSTITUTE(J33,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34">
@@ -6475,7 +6574,10 @@
       <x:c r="AG34" s="198" t="str">
         <x:v>3rd Place — S$250 Cash</x:v>
       </x:c>
-      <x:c r="AH34" s="206"/>
+      <x:c r="AH34" s="214" t="n">
+        <x:f>IF(OR(J34="",J34="-"),"",LEN(J34)-LEN(SUBSTITUTE(J34,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35">
@@ -6543,7 +6645,10 @@
       <x:c r="AE35" s="38"/>
       <x:c r="AF35" s="38"/>
       <x:c r="AG35" s="198"/>
-      <x:c r="AH35" s="206"/>
+      <x:c r="AH35" s="214" t="n">
+        <x:f>IF(OR(J35="",J35="-"),"",LEN(J35)-LEN(SUBSTITUTE(J35,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36">
@@ -6623,7 +6728,10 @@
       <x:c r="AG36" s="198" t="str">
         <x:v>2nd Place — S$1,000 Cash</x:v>
       </x:c>
-      <x:c r="AH36" s="206"/>
+      <x:c r="AH36" s="214" t="n">
+        <x:f>IF(OR(J36="",J36="-"),"",LEN(J36)-LEN(SUBSTITUTE(J36,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37">
@@ -6691,7 +6799,10 @@
       <x:c r="AE37" s="38"/>
       <x:c r="AF37" s="38"/>
       <x:c r="AG37" s="198"/>
-      <x:c r="AH37" s="206"/>
+      <x:c r="AH37" s="214" t="n">
+        <x:f>IF(OR(J37="",J37="-"),"",LEN(J37)-LEN(SUBSTITUTE(J37,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38">
@@ -6759,7 +6870,10 @@
       <x:c r="AE38" s="38"/>
       <x:c r="AF38" s="38"/>
       <x:c r="AG38" s="198"/>
-      <x:c r="AH38" s="206"/>
+      <x:c r="AH38" s="214" t="n">
+        <x:f>IF(OR(J38="",J38="-"),"",LEN(J38)-LEN(SUBSTITUTE(J38,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39">
@@ -6843,7 +6957,10 @@
       <x:c r="AG39" s="198" t="str">
         <x:v>2nd Place — Manus Pro Subscription (US$39/month)</x:v>
       </x:c>
-      <x:c r="AH39" s="206"/>
+      <x:c r="AH39" s="214" t="n">
+        <x:f>IF(OR(J39="",J39="-"),"",LEN(J39)-LEN(SUBSTITUTE(J39,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40">
@@ -6911,7 +7028,10 @@
       <x:c r="AE40" s="38"/>
       <x:c r="AF40" s="38"/>
       <x:c r="AG40" s="198"/>
-      <x:c r="AH40" s="206"/>
+      <x:c r="AH40" s="214" t="n">
+        <x:f>IF(OR(J40="",J40="-"),"",LEN(J40)-LEN(SUBSTITUTE(J40,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41">
@@ -6992,7 +7112,10 @@
       <x:c r="AG41" s="198" t="str">
         <x:v>Best Finisher — Novel Hackathon — Trophy</x:v>
       </x:c>
-      <x:c r="AH41" s="206"/>
+      <x:c r="AH41" s="214" t="n">
+        <x:f>IF(OR(J41="",J41="-"),"",LEN(J41)-LEN(SUBSTITUTE(J41,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42">
@@ -7057,7 +7180,10 @@
       <x:c r="AE42" s="38"/>
       <x:c r="AF42" s="38"/>
       <x:c r="AG42" s="198"/>
-      <x:c r="AH42" s="206"/>
+      <x:c r="AH42" s="214" t="n">
+        <x:f>IF(OR(J42="",J42="-"),"",LEN(J42)-LEN(SUBSTITUTE(J42,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43">
@@ -7139,7 +7265,10 @@
       <x:c r="AG43" s="198" t="str">
         <x:v>1st Place — US$500 Nosana Cloud Credits</x:v>
       </x:c>
-      <x:c r="AH43" s="206"/>
+      <x:c r="AH43" s="214" t="n">
+        <x:f>IF(OR(J43="",J43="-"),"",LEN(J43)-LEN(SUBSTITUTE(J43,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44">
@@ -7207,7 +7336,10 @@
       <x:c r="AE44" s="38"/>
       <x:c r="AF44" s="38"/>
       <x:c r="AG44" s="198"/>
-      <x:c r="AH44" s="206"/>
+      <x:c r="AH44" s="214" t="n">
+        <x:f>IF(OR(J44="",J44="-"),"",LEN(J44)-LEN(SUBSTITUTE(J44,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45">
@@ -7275,7 +7407,10 @@
       <x:c r="AE45" s="38"/>
       <x:c r="AF45" s="38"/>
       <x:c r="AG45" s="198"/>
-      <x:c r="AH45" s="206"/>
+      <x:c r="AH45" s="214" t="n">
+        <x:f>IF(OR(J45="",J45="-"),"",LEN(J45)-LEN(SUBSTITUTE(J45,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46">
@@ -7343,7 +7478,10 @@
       <x:c r="AE46" s="38"/>
       <x:c r="AF46" s="38"/>
       <x:c r="AG46" s="198"/>
-      <x:c r="AH46" s="206"/>
+      <x:c r="AH46" s="214" t="n">
+        <x:f>IF(OR(J46="",J46="-"),"",LEN(J46)-LEN(SUBSTITUTE(J46,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47">
@@ -7411,7 +7549,10 @@
       <x:c r="AE47" s="38"/>
       <x:c r="AF47" s="38"/>
       <x:c r="AG47" s="198"/>
-      <x:c r="AH47" s="206"/>
+      <x:c r="AH47" s="214" t="n">
+        <x:f>IF(OR(J47="",J47="-"),"",LEN(J47)-LEN(SUBSTITUTE(J47,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="49.75" customHeight="1">
       <x:c r="A48">
@@ -7479,7 +7620,10 @@
       <x:c r="AE48" s="38"/>
       <x:c r="AF48" s="38"/>
       <x:c r="AG48" s="198"/>
-      <x:c r="AH48" s="206"/>
+      <x:c r="AH48" s="214" t="n">
+        <x:f>IF(OR(J48="",J48="-"),"",LEN(J48)-LEN(SUBSTITUTE(J48,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49">
@@ -7547,7 +7691,10 @@
       <x:c r="AE49" s="38"/>
       <x:c r="AF49" s="38"/>
       <x:c r="AG49" s="198"/>
-      <x:c r="AH49" s="206"/>
+      <x:c r="AH49" s="214" t="n">
+        <x:f>IF(OR(J49="",J49="-"),"",LEN(J49)-LEN(SUBSTITUTE(J49,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="34">
       <x:c r="A50">
@@ -7615,7 +7762,10 @@
       <x:c r="AE50" s="38"/>
       <x:c r="AF50" s="38"/>
       <x:c r="AG50" s="198"/>
-      <x:c r="AH50" s="206"/>
+      <x:c r="AH50" s="214" t="n">
+        <x:f>IF(OR(J50="",J50="-"),"",LEN(J50)-LEN(SUBSTITUTE(J50,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51">
@@ -7697,7 +7847,10 @@
       <x:c r="AG51" s="198" t="str">
         <x:v>1st Place — US$1,000 OpenRouter Credits</x:v>
       </x:c>
-      <x:c r="AH51" s="206"/>
+      <x:c r="AH51" s="214" t="n">
+        <x:f>IF(OR(J51="",J51="-"),"",LEN(J51)-LEN(SUBSTITUTE(J51,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52">
@@ -7765,7 +7918,10 @@
       <x:c r="AE52" s="38"/>
       <x:c r="AF52" s="38"/>
       <x:c r="AG52" s="198"/>
-      <x:c r="AH52" s="206"/>
+      <x:c r="AH52" s="214" t="n">
+        <x:f>IF(OR(J52="",J52="-"),"",LEN(J52)-LEN(SUBSTITUTE(J52,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53">
@@ -7847,7 +8003,10 @@
       <x:c r="AG53" s="198" t="str">
         <x:v>1st Place — US$500 API Credits</x:v>
       </x:c>
-      <x:c r="AH53" s="206"/>
+      <x:c r="AH53" s="214" t="n">
+        <x:f>IF(OR(J53="",J53="-"),"",LEN(J53)-LEN(SUBSTITUTE(J53,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54">
@@ -7929,7 +8088,10 @@
       <x:c r="AG54" s="198" t="str">
         <x:v>1st Place — US$500 API Credits</x:v>
       </x:c>
-      <x:c r="AH54" s="206"/>
+      <x:c r="AH54" s="214" t="n">
+        <x:f>IF(OR(J54="",J54="-"),"",LEN(J54)-LEN(SUBSTITUTE(J54,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="34">
       <x:c r="A55">
@@ -8011,7 +8173,10 @@
       <x:c r="AG55" s="198" t="str">
         <x:v>1st Place — US$150 Wavespeed AI Credits</x:v>
       </x:c>
-      <x:c r="AH55" s="206"/>
+      <x:c r="AH55" s="214" t="n">
+        <x:f>IF(OR(J55="",J55="-"),"",LEN(J55)-LEN(SUBSTITUTE(J55,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="17">
       <x:c r="A56">
@@ -8079,7 +8244,10 @@
       <x:c r="AE56" s="38"/>
       <x:c r="AF56" s="38"/>
       <x:c r="AG56" s="198"/>
-      <x:c r="AH56" s="206"/>
+      <x:c r="AH56" s="214" t="n">
+        <x:f>IF(OR(J56="",J56="-"),"",LEN(J56)-LEN(SUBSTITUTE(J56,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57">
@@ -8147,7 +8315,10 @@
       <x:c r="AE57" s="38"/>
       <x:c r="AF57" s="38"/>
       <x:c r="AG57" s="198"/>
-      <x:c r="AH57" s="206"/>
+      <x:c r="AH57" s="214" t="n">
+        <x:f>IF(OR(J57="",J57="-"),"",LEN(J57)-LEN(SUBSTITUTE(J57,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58">
@@ -8233,7 +8404,10 @@
       <x:c r="AG58" s="198" t="str">
         <x:v>3rd Place — S$300 Cash + S$385 API Credits</x:v>
       </x:c>
-      <x:c r="AH58" s="206"/>
+      <x:c r="AH58" s="214" t="n">
+        <x:f>IF(OR(J58="",J58="-"),"",LEN(J58)-LEN(SUBSTITUTE(J58,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59">
@@ -8301,7 +8475,10 @@
       <x:c r="AE59" s="38"/>
       <x:c r="AF59" s="38"/>
       <x:c r="AG59" s="198"/>
-      <x:c r="AH59" s="206"/>
+      <x:c r="AH59" s="214" t="n">
+        <x:f>IF(OR(J59="",J59="-"),"",LEN(J59)-LEN(SUBSTITUTE(J59,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60">
@@ -8369,7 +8546,10 @@
       <x:c r="AE60" s="38"/>
       <x:c r="AF60" s="38"/>
       <x:c r="AG60" s="198"/>
-      <x:c r="AH60" s="206"/>
+      <x:c r="AH60" s="214" t="n">
+        <x:f>IF(OR(J60="",J60="-"),"",LEN(J60)-LEN(SUBSTITUTE(J60,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61">
@@ -8453,7 +8633,10 @@
       <x:c r="AG61" s="198" t="str">
         <x:v>Award — Speechmatics — US$2,000 Speechmatics Credits</x:v>
       </x:c>
-      <x:c r="AH61" s="206"/>
+      <x:c r="AH61" s="214" t="n">
+        <x:f>IF(OR(J61="",J61="-"),"",LEN(J61)-LEN(SUBSTITUTE(J61,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62">
@@ -8537,7 +8720,10 @@
       <x:c r="AG62" s="198" t="str">
         <x:v>Award — v0 Sock</x:v>
       </x:c>
-      <x:c r="AH62" s="206"/>
+      <x:c r="AH62" s="214" t="n">
+        <x:f>IF(OR(J62="",J62="-"),"",LEN(J62)-LEN(SUBSTITUTE(J62,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63">
@@ -8605,7 +8791,10 @@
       <x:c r="AE63" s="38"/>
       <x:c r="AF63" s="38"/>
       <x:c r="AG63" s="198"/>
-      <x:c r="AH63" s="206"/>
+      <x:c r="AH63" s="214" t="n">
+        <x:f>IF(OR(J63="",J63="-"),"",LEN(J63)-LEN(SUBSTITUTE(J63,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64">
@@ -8673,7 +8862,10 @@
       <x:c r="AE64" s="38"/>
       <x:c r="AF64" s="38"/>
       <x:c r="AG64" s="198"/>
-      <x:c r="AH64" s="206"/>
+      <x:c r="AH64" s="214" t="n">
+        <x:f>IF(OR(J64="",J64="-"),"",LEN(J64)-LEN(SUBSTITUTE(J64,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65">
@@ -8741,7 +8933,10 @@
       <x:c r="AE65" s="38"/>
       <x:c r="AF65" s="38"/>
       <x:c r="AG65" s="198"/>
-      <x:c r="AH65" s="206"/>
+      <x:c r="AH65" s="214" t="n">
+        <x:f>IF(OR(J65="",J65="-"),"",LEN(J65)-LEN(SUBSTITUTE(J65,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66">
@@ -8809,7 +9004,10 @@
       <x:c r="AE66" s="38"/>
       <x:c r="AF66" s="38"/>
       <x:c r="AG66" s="198"/>
-      <x:c r="AH66" s="206"/>
+      <x:c r="AH66" s="214" t="n">
+        <x:f>IF(OR(J66="",J66="-"),"",LEN(J66)-LEN(SUBSTITUTE(J66,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67">
@@ -8891,7 +9089,10 @@
       <x:c r="AG67" s="198" t="str">
         <x:v>Top 20 — US$12,000 Credits (OpenAI + Gemini Cloud)</x:v>
       </x:c>
-      <x:c r="AH67" s="206"/>
+      <x:c r="AH67" s="214" t="n">
+        <x:f>IF(OR(J67="",J67="-"),"",LEN(J67)-LEN(SUBSTITUTE(J67,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68">
@@ -8959,7 +9160,10 @@
       <x:c r="AE68" s="38"/>
       <x:c r="AF68" s="38"/>
       <x:c r="AG68" s="198"/>
-      <x:c r="AH68" s="206"/>
+      <x:c r="AH68" s="214" t="n">
+        <x:f>IF(OR(J68="",J68="-"),"",LEN(J68)-LEN(SUBSTITUTE(J68,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69">
@@ -9027,7 +9231,10 @@
       <x:c r="AE69" s="38"/>
       <x:c r="AF69" s="38"/>
       <x:c r="AG69" s="198"/>
-      <x:c r="AH69" s="206"/>
+      <x:c r="AH69" s="214" t="n">
+        <x:f>IF(OR(J69="",J69="-"),"",LEN(J69)-LEN(SUBSTITUTE(J69,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70">
@@ -9092,7 +9299,10 @@
       <x:c r="AE70" s="38"/>
       <x:c r="AF70" s="38"/>
       <x:c r="AG70" s="198"/>
-      <x:c r="AH70" s="206"/>
+      <x:c r="AH70" s="214" t="n">
+        <x:f>IF(OR(J70="",J70="-"),"",LEN(J70)-LEN(SUBSTITUTE(J70,",",""))+1)</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71">
@@ -9160,7 +9370,10 @@
       <x:c r="AE71" s="38"/>
       <x:c r="AF71" s="38"/>
       <x:c r="AG71" s="198"/>
-      <x:c r="AH71" s="206"/>
+      <x:c r="AH71" s="214" t="n">
+        <x:f>IF(OR(J71="",J71="-"),"",LEN(J71)-LEN(SUBSTITUTE(J71,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72">
@@ -9244,7 +9457,10 @@
       <x:c r="AG72" s="198" t="str">
         <x:v>Award — US$4,500 AWS Credits</x:v>
       </x:c>
-      <x:c r="AH72" s="206"/>
+      <x:c r="AH72" s="214" t="n">
+        <x:f>IF(OR(J72="",J72="-"),"",LEN(J72)-LEN(SUBSTITUTE(J72,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73">
@@ -9312,7 +9528,10 @@
       <x:c r="AE73" s="38"/>
       <x:c r="AF73" s="38"/>
       <x:c r="AG73" s="198"/>
-      <x:c r="AH73" s="206"/>
+      <x:c r="AH73" s="214" t="n">
+        <x:f>IF(OR(J73="",J73="-"),"",LEN(J73)-LEN(SUBSTITUTE(J73,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74">
@@ -9380,7 +9599,10 @@
       <x:c r="AE74" s="38"/>
       <x:c r="AF74" s="38"/>
       <x:c r="AG74" s="198"/>
-      <x:c r="AH74" s="206"/>
+      <x:c r="AH74" s="214" t="n">
+        <x:f>IF(OR(J74="",J74="-"),"",LEN(J74)-LEN(SUBSTITUTE(J74,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="34">
       <x:c r="A75">
@@ -9448,7 +9670,10 @@
       <x:c r="AE75" s="38"/>
       <x:c r="AF75" s="38"/>
       <x:c r="AG75" s="198"/>
-      <x:c r="AH75" s="206"/>
+      <x:c r="AH75" s="214" t="n">
+        <x:f>IF(OR(J75="",J75="-"),"",LEN(J75)-LEN(SUBSTITUTE(J75,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76">
@@ -9532,7 +9757,10 @@
       <x:c r="AG76" s="198" t="str">
         <x:v>Best Vertical Solution — Family Office Track — 2,000 Cybrdeck API Credits (US$25 value)</x:v>
       </x:c>
-      <x:c r="AH76" s="206"/>
+      <x:c r="AH76" s="214" t="n">
+        <x:f>IF(OR(J76="",J76="-"),"",LEN(J76)-LEN(SUBSTITUTE(J76,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77">
@@ -9600,7 +9828,10 @@
       <x:c r="AE77" s="38"/>
       <x:c r="AF77" s="38"/>
       <x:c r="AG77" s="198"/>
-      <x:c r="AH77" s="206"/>
+      <x:c r="AH77" s="214" t="n">
+        <x:f>IF(OR(J77="",J77="-"),"",LEN(J77)-LEN(SUBSTITUTE(J77,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78">
@@ -9668,7 +9899,10 @@
       <x:c r="AE78" s="38"/>
       <x:c r="AF78" s="38"/>
       <x:c r="AG78" s="198"/>
-      <x:c r="AH78" s="206"/>
+      <x:c r="AH78" s="214" t="n">
+        <x:f>IF(OR(J78="",J78="-"),"",LEN(J78)-LEN(SUBSTITUTE(J78,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79">
@@ -9736,7 +9970,10 @@
       <x:c r="AE79" s="38"/>
       <x:c r="AF79" s="38"/>
       <x:c r="AG79" s="198"/>
-      <x:c r="AH79" s="206"/>
+      <x:c r="AH79" s="214" t="n">
+        <x:f>IF(OR(J79="",J79="-"),"",LEN(J79)-LEN(SUBSTITUTE(J79,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" t="n">
@@ -9824,7 +10061,10 @@
       <x:c r="AG80" s="198" t="str">
         <x:v>First Runner-Up — SG × Sarawak AI &amp; Design Hackathon — US$200 Kimi AI Credits + Trophy</x:v>
       </x:c>
-      <x:c r="AH80" s="206"/>
+      <x:c r="AH80" s="214" t="n">
+        <x:f>IF(OR(J80="",J80="-"),"",LEN(J80)-LEN(SUBSTITUTE(J80,",",""))+1)</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" t="n">
@@ -9908,7 +10148,10 @@
       <x:c r="AG81" s="198" t="str">
         <x:v>Best Project — Best Use of GPT-Image-2.5 — US$5,000 OpenAI Credits</x:v>
       </x:c>
-      <x:c r="AH81" s="206"/>
+      <x:c r="AH81" s="214" t="n">
+        <x:f>IF(OR(J81="",J81="-"),"",LEN(J81)-LEN(SUBSTITUTE(J81,",",""))+1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" t="n">
@@ -9974,14 +10217,17 @@
       <x:c r="AE82" s="38"/>
       <x:c r="AF82" s="38"/>
       <x:c r="AG82" s="198"/>
-      <x:c r="AH82" s="206"/>
+      <x:c r="AH82" s="214" t="n">
+        <x:f>IF(OR(J82="",J82="-"),"",LEN(J82)-LEN(SUBSTITUTE(J82,",",""))+1)</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R51f31ee7e26f4be9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R84401180a1f24449"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R642f9c0516584ef8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R7ec5528115b448ef"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R95b117621d5e4e86"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rfc1fc4a1196541f2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rff0609161e104161"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Ra7ea9f4d83704f6a"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11559,12 +11805,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rfda7e61034354180"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rcb19bfebc42047cd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rc287ada2c6d74343"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R621c89396f344127"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R912d3e14b9604875"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16e6b80f75fc4050"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12467,7 +12713,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f85c45b37224e49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c17cd1883c54546"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13460,7 +13706,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="106" t="str">
-        <x:v>One row per currently classified award or prize record. Award Summary uses a curated, standardized format; enter the number sharing a prize in Hackathons column AH.</x:v>
+        <x:v>One row per currently classified award or prize record. Award Summary uses a curated, standardized format; Hackathon Team Members is counted automatically from the comma-delimited Team Members roster.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -13554,7 +13800,7 @@
         <x:v>Review note</x:v>
       </x:c>
       <x:c r="T4" s="212" t="str">
-        <x:v>Prize Sharing Team Members</x:v>
+        <x:v>Hackathon Team Members</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -13623,8 +13869,9 @@
         <x:f>IF(Hackathons!AF2="","",Hackathons!AF2)</x:f>
         <x:v>Funding, not a cash prize</x:v>
       </x:c>
-      <x:c r="T5" s="213" t="str">
+      <x:c r="T5" s="213" t="n">
         <x:f>IF(Hackathons!AH2="","",Hackathons!AH2)</x:f>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -13692,8 +13939,9 @@
         <x:f>IF(Hackathons!AF4="","",Hackathons!AF4)</x:f>
         <x:v>Recognition only</x:v>
       </x:c>
-      <x:c r="T6" s="213" t="str">
+      <x:c r="T6" s="213" t="n">
         <x:f>IF(Hackathons!AH4="","",Hackathons!AH4)</x:f>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -13765,8 +14013,9 @@
         <x:f>IF(Hackathons!AF5="","",Hackathons!AF5)</x:f>
         <x:v>US$100,000 IBM Bluemix credit value</x:v>
       </x:c>
-      <x:c r="T7" s="213" t="str">
+      <x:c r="T7" s="213" t="n">
         <x:f>IF(Hackathons!AH5="","",Hackathons!AH5)</x:f>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -13833,8 +14082,9 @@
         <x:f>IF(Hackathons!AF7="","",Hackathons!AF7)</x:f>
         <x:v>Recognition only</x:v>
       </x:c>
-      <x:c r="T8" s="213" t="str">
+      <x:c r="T8" s="213" t="n">
         <x:f>IF(Hackathons!AH7="","",Hackathons!AH7)</x:f>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -13902,8 +14152,9 @@
         <x:f>IF(Hackathons!AF11="","",Hackathons!AF11)</x:f>
         <x:v>Recognition only</x:v>
       </x:c>
-      <x:c r="T9" s="213" t="str">
+      <x:c r="T9" s="213" t="n">
         <x:f>IF(Hackathons!AH11="","",Hackathons!AH11)</x:f>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -13973,8 +14224,9 @@
         <x:f>IF(Hackathons!AF15="","",Hackathons!AF15)</x:f>
         <x:v>Voucher counted as cash equivalent</x:v>
       </x:c>
-      <x:c r="T10" s="213" t="str">
+      <x:c r="T10" s="213" t="n">
         <x:f>IF(Hackathons!AH15="","",Hackathons!AH15)</x:f>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -14043,8 +14295,9 @@
         <x:f>IF(Hackathons!AF18="","",Hackathons!AF18)</x:f>
         <x:v>Explicit cash</x:v>
       </x:c>
-      <x:c r="T11" s="213" t="str">
+      <x:c r="T11" s="213" t="n">
         <x:f>IF(Hackathons!AH18="","",Hackathons!AH18)</x:f>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -14113,8 +14366,9 @@
         <x:f>IF(Hackathons!AF26="","",Hackathons!AF26)</x:f>
         <x:v>Explicit cash</x:v>
       </x:c>
-      <x:c r="T12" s="213" t="str">
+      <x:c r="T12" s="213" t="n">
         <x:f>IF(Hackathons!AH26="","",Hackathons!AH26)</x:f>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -14183,8 +14437,9 @@
         <x:f>IF(Hackathons!AF34="","",Hackathons!AF34)</x:f>
         <x:v>Confirmed cash</x:v>
       </x:c>
-      <x:c r="T13" s="213" t="str">
+      <x:c r="T13" s="213" t="n">
         <x:f>IF(Hackathons!AH34="","",Hackathons!AH34)</x:f>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -14253,8 +14508,9 @@
         <x:f>IF(Hackathons!AF36="","",Hackathons!AF36)</x:f>
         <x:v>Confirmed cash</x:v>
       </x:c>
-      <x:c r="T14" s="213" t="str">
+      <x:c r="T14" s="213" t="n">
         <x:f>IF(Hackathons!AH36="","",Hackathons!AH36)</x:f>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -14325,8 +14581,9 @@
         <x:f>IF(Hackathons!AF39="","",Hackathons!AF39)</x:f>
         <x:v>US$39 monthly value at award period</x:v>
       </x:c>
-      <x:c r="T15" s="213" t="str">
+      <x:c r="T15" s="213" t="n">
         <x:f>IF(Hackathons!AH39="","",Hackathons!AH39)</x:f>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -14397,8 +14654,9 @@
         <x:f>IF(Hackathons!AF41="","",Hackathons!AF41)</x:f>
         <x:v>Trophy, not cash</x:v>
       </x:c>
-      <x:c r="T16" s="213" t="str">
+      <x:c r="T16" s="213" t="n">
         <x:f>IF(Hackathons!AH41="","",Hackathons!AH41)</x:f>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -14468,8 +14726,9 @@
         <x:f>IF(Hackathons!AF43="","",Hackathons!AF43)</x:f>
         <x:v>Cloud credit, not cash</x:v>
       </x:c>
-      <x:c r="T17" s="213" t="str">
+      <x:c r="T17" s="213" t="n">
         <x:f>IF(Hackathons!AH43="","",Hackathons!AH43)</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -14539,8 +14798,9 @@
         <x:f>IF(Hackathons!AF51="","",Hackathons!AF51)</x:f>
         <x:v>API credits, not cash</x:v>
       </x:c>
-      <x:c r="T18" s="213" t="str">
+      <x:c r="T18" s="213" t="n">
         <x:f>IF(Hackathons!AH51="","",Hackathons!AH51)</x:f>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -14610,8 +14870,9 @@
         <x:f>IF(Hackathons!AF53="","",Hackathons!AF53)</x:f>
         <x:v>API credits, not cash</x:v>
       </x:c>
-      <x:c r="T19" s="213" t="str">
+      <x:c r="T19" s="213" t="n">
         <x:f>IF(Hackathons!AH53="","",Hackathons!AH53)</x:f>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -14681,8 +14942,9 @@
         <x:f>IF(Hackathons!AF54="","",Hackathons!AF54)</x:f>
         <x:v>API credits, not cash</x:v>
       </x:c>
-      <x:c r="T20" s="213" t="str">
+      <x:c r="T20" s="213" t="n">
         <x:f>IF(Hackathons!AH54="","",Hackathons!AH54)</x:f>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -14752,8 +15014,9 @@
         <x:f>IF(Hackathons!AF55="","",Hackathons!AF55)</x:f>
         <x:v>API credits, not cash</x:v>
       </x:c>
-      <x:c r="T21" s="213" t="str">
+      <x:c r="T21" s="213" t="n">
         <x:f>IF(Hackathons!AH55="","",Hackathons!AH55)</x:f>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -14825,8 +15088,9 @@
         <x:f>IF(Hackathons!AF58="","",Hackathons!AF58)</x:f>
         <x:v>Explicit cash; API credit value also tracked</x:v>
       </x:c>
-      <x:c r="T22" s="213" t="str">
+      <x:c r="T22" s="213" t="n">
         <x:f>IF(Hackathons!AH58="","",Hackathons!AH58)</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -14897,8 +15161,9 @@
         <x:f>IF(Hackathons!AF61="","",Hackathons!AF61)</x:f>
         <x:v>USD-denominated credit value</x:v>
       </x:c>
-      <x:c r="T23" s="213" t="str">
+      <x:c r="T23" s="213" t="n">
         <x:f>IF(Hackathons!AH61="","",Hackathons!AH61)</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -14968,8 +15233,9 @@
         <x:f>IF(Hackathons!AF62="","",Hackathons!AF62)</x:f>
         <x:v>Physical item, not cash</x:v>
       </x:c>
-      <x:c r="T24" s="213" t="str">
+      <x:c r="T24" s="213" t="n">
         <x:f>IF(Hackathons!AH62="","",Hackathons!AH62)</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -15039,8 +15305,9 @@
         <x:f>IF(Hackathons!AF67="","",Hackathons!AF67)</x:f>
         <x:v>Credit value total combines two USD-denominated credits</x:v>
       </x:c>
-      <x:c r="T25" s="213" t="str">
+      <x:c r="T25" s="213" t="n">
         <x:f>IF(Hackathons!AH67="","",Hackathons!AH67)</x:f>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -15111,8 +15378,9 @@
         <x:f>IF(Hackathons!AF72="","",Hackathons!AF72)</x:f>
         <x:v>USD-denominated credit value</x:v>
       </x:c>
-      <x:c r="T26" s="213" t="str">
+      <x:c r="T26" s="213" t="n">
         <x:f>IF(Hackathons!AH72="","",Hackathons!AH72)</x:f>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -15183,8 +15451,9 @@
         <x:f>IF(Hackathons!AF76="","",Hackathons!AF76)</x:f>
         <x:v>US$25 credit value, not cash</x:v>
       </x:c>
-      <x:c r="T27" s="213" t="str">
+      <x:c r="T27" s="213" t="n">
         <x:f>IF(Hackathons!AH76="","",Hackathons!AH76)</x:f>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -15257,8 +15526,9 @@
         <x:f>IF(Hackathons!AF80="","",Hackathons!AF80)</x:f>
         <x:v>Trophy excluded; credit value tracked</x:v>
       </x:c>
-      <x:c r="T28" s="213" t="str">
+      <x:c r="T28" s="213" t="n">
         <x:f>IF(Hackathons!AH80="","",Hackathons!AH80)</x:f>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -15329,8 +15599,9 @@
         <x:f>IF(Hackathons!AF81="","",Hackathons!AF81)</x:f>
         <x:v>Credit value tracked</x:v>
       </x:c>
-      <x:c r="T29" s="213" t="str">
+      <x:c r="T29" s="213" t="n">
         <x:f>IF(Hackathons!AH81="","",Hackathons!AH81)</x:f>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15346,7 +15617,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red2e66bf212a44db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bc88217540d4795"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct v0 hackathon award placement
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R78055f633f7e4572"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rede65b37755745f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rb2d6e1ac63dc49a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R201f137145ff4a7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R3c2e97e6d4e84ad0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Rd026b830326e4d9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Reb7c7f89b5ec4bec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R49c3aba8b997425e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rc381810b42d94889"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R4d932ad07d554cea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="Re20ea37a4651423a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R8767c55da7a94890"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1393,9 +1393,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">30/4/2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">v0 Sock</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Game</x:t>
@@ -8657,20 +8654,20 @@
       <x:c r="F62" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="G62" t="s">
+      <x:c r="G62" t="str">
+        <x:v>2nd Place — v0 Sock</x:v>
+      </x:c>
+      <x:c r="H62" t="s">
         <x:v>460</x:v>
       </x:c>
-      <x:c r="H62" t="s">
+      <x:c r="I62" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="I62" t="s">
-        <x:v>462</x:v>
       </x:c>
       <x:c r="J62" t="s">
         <x:v>309</x:v>
       </x:c>
       <x:c r="K62" t="s">
-        <x:v>463</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="L62" t="s">
         <x:v>25</x:v>
@@ -8685,10 +8682,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="P62" s="1" t="s">
-        <x:v>464</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="Q62" s="36" t="str">
-        <x:v>Award</x:v>
+        <x:v>2nd Place</x:v>
       </x:c>
       <x:c r="R62" s="36" t="str">
         <x:v>v0</x:v>
@@ -8718,7 +8715,7 @@
         <x:v>Physical item, not cash</x:v>
       </x:c>
       <x:c r="AG62" s="198" t="str">
-        <x:v>Award — v0 Sock</x:v>
+        <x:v>2nd Place — v0 Sock</x:v>
       </x:c>
       <x:c r="AH62" s="214" t="n">
         <x:f>IF(OR(J62="",J62="-"),"",LEN(J62)-LEN(SUBSTITUTE(J62,",",""))+1)</x:f>
@@ -8730,10 +8727,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="B63" t="s">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="C63" t="s">
         <x:v>465</x:v>
-      </x:c>
-      <x:c r="C63" t="s">
-        <x:v>466</x:v>
       </x:c>
       <x:c r="D63" s="5">
         <x:v>46085</x:v>
@@ -8742,7 +8739,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F63" t="s">
-        <x:v>467</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="G63" t="s">
         <x:v>25</x:v>
@@ -8751,13 +8748,13 @@
         <x:v>402</x:v>
       </x:c>
       <x:c r="I63" t="s">
-        <x:v>468</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="J63" t="s">
         <x:v>404</x:v>
       </x:c>
       <x:c r="K63" t="s">
-        <x:v>469</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="L63" t="s">
         <x:v>25</x:v>
@@ -8766,13 +8763,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N63" t="s">
+        <x:v>469</x:v>
+      </x:c>
+      <x:c r="O63" t="s">
         <x:v>470</x:v>
       </x:c>
-      <x:c r="O63" t="s">
+      <x:c r="P63" t="s">
         <x:v>471</x:v>
-      </x:c>
-      <x:c r="P63" t="s">
-        <x:v>472</x:v>
       </x:c>
       <x:c r="Q63" s="36"/>
       <x:c r="R63" s="36"/>
@@ -8801,7 +8798,7 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="B64" t="s">
-        <x:v>473</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="C64" t="s">
         <x:v>458</x:v>
@@ -8819,16 +8816,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H64" t="s">
-        <x:v>461</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="I64" t="s">
-        <x:v>474</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="J64" t="s">
         <x:v>309</x:v>
       </x:c>
       <x:c r="K64" t="s">
-        <x:v>475</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="L64" t="s">
         <x:v>25</x:v>
@@ -8840,10 +8837,10 @@
         <x:v>356</x:v>
       </x:c>
       <x:c r="O64" t="s">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="P64" t="s">
         <x:v>476</x:v>
-      </x:c>
-      <x:c r="P64" t="s">
-        <x:v>477</x:v>
       </x:c>
       <x:c r="Q64" s="36"/>
       <x:c r="R64" s="36"/>
@@ -8872,10 +8869,10 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="B65" t="s">
+        <x:v>477</x:v>
+      </x:c>
+      <x:c r="C65" t="s">
         <x:v>478</x:v>
-      </x:c>
-      <x:c r="C65" t="s">
-        <x:v>479</x:v>
       </x:c>
       <x:c r="D65" s="5">
         <x:v>46270</x:v>
@@ -8890,16 +8887,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H65" t="s">
-        <x:v>461</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="I65" t="s">
+        <x:v>479</x:v>
+      </x:c>
+      <x:c r="J65" t="s">
         <x:v>480</x:v>
       </x:c>
-      <x:c r="J65" t="s">
+      <x:c r="K65" t="s">
         <x:v>481</x:v>
-      </x:c>
-      <x:c r="K65" t="s">
-        <x:v>482</x:v>
       </x:c>
       <x:c r="L65" t="s">
         <x:v>25</x:v>
@@ -8911,10 +8908,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="O65" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="P65" t="s">
         <x:v>483</x:v>
-      </x:c>
-      <x:c r="P65" t="s">
-        <x:v>484</x:v>
       </x:c>
       <x:c r="Q65" s="36"/>
       <x:c r="R65" s="36"/>
@@ -8943,13 +8940,13 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B66" t="s">
+        <x:v>484</x:v>
+      </x:c>
+      <x:c r="C66" t="s">
         <x:v>485</x:v>
       </x:c>
-      <x:c r="C66" t="s">
+      <x:c r="D66" s="2" t="s">
         <x:v>486</x:v>
-      </x:c>
-      <x:c r="D66" s="2" t="s">
-        <x:v>487</x:v>
       </x:c>
       <x:c r="E66">
         <x:v>1</x:v>
@@ -8964,13 +8961,13 @@
         <x:v>376</x:v>
       </x:c>
       <x:c r="I66" t="s">
-        <x:v>488</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="J66" t="s">
         <x:v>309</x:v>
       </x:c>
       <x:c r="K66" t="s">
-        <x:v>489</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="L66" t="s">
         <x:v>25</x:v>
@@ -8979,13 +8976,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N66" t="s">
+        <x:v>489</x:v>
+      </x:c>
+      <x:c r="O66" t="s">
         <x:v>490</x:v>
       </x:c>
-      <x:c r="O66" t="s">
+      <x:c r="P66" t="s">
         <x:v>491</x:v>
-      </x:c>
-      <x:c r="P66" t="s">
-        <x:v>492</x:v>
       </x:c>
       <x:c r="Q66" s="36"/>
       <x:c r="R66" s="36"/>
@@ -9014,13 +9011,13 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B67" t="s">
+        <x:v>492</x:v>
+      </x:c>
+      <x:c r="C67" t="s">
         <x:v>493</x:v>
       </x:c>
-      <x:c r="C67" t="s">
+      <x:c r="D67" s="2" t="s">
         <x:v>494</x:v>
-      </x:c>
-      <x:c r="D67" s="2" t="s">
-        <x:v>495</x:v>
       </x:c>
       <x:c r="E67">
         <x:v>1</x:v>
@@ -9029,7 +9026,7 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="G67" t="s">
-        <x:v>496</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="H67" t="s">
         <x:v>402</x:v>
@@ -9038,10 +9035,10 @@
         <x:v>411</x:v>
       </x:c>
       <x:c r="J67" t="s">
+        <x:v>496</x:v>
+      </x:c>
+      <x:c r="K67" t="s">
         <x:v>497</x:v>
-      </x:c>
-      <x:c r="K67" t="s">
-        <x:v>498</x:v>
       </x:c>
       <x:c r="L67" t="s">
         <x:v>25</x:v>
@@ -9099,13 +9096,13 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B68" t="s">
-        <x:v>499</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="C68" t="s">
         <x:v>263</x:v>
       </x:c>
       <x:c r="D68" s="2" t="s">
-        <x:v>500</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="E68">
         <x:v>3</x:v>
@@ -9117,19 +9114,19 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H68" t="s">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="I68" t="s">
         <x:v>501</x:v>
       </x:c>
-      <x:c r="I68" t="s">
+      <x:c r="J68" t="s">
         <x:v>502</x:v>
       </x:c>
-      <x:c r="J68" t="s">
+      <x:c r="K68" t="s">
         <x:v>503</x:v>
       </x:c>
-      <x:c r="K68" t="s">
+      <x:c r="L68" t="s">
         <x:v>504</x:v>
-      </x:c>
-      <x:c r="L68" t="s">
-        <x:v>505</x:v>
       </x:c>
       <x:c r="M68" t="s">
         <x:v>26</x:v>
@@ -9138,7 +9135,7 @@
         <x:v>270</x:v>
       </x:c>
       <x:c r="O68" t="s">
-        <x:v>506</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="P68" t="s">
         <x:v>25</x:v>
@@ -9170,13 +9167,13 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B69" t="s">
+        <x:v>506</x:v>
+      </x:c>
+      <x:c r="C69" t="s">
+        <x:v>493</x:v>
+      </x:c>
+      <x:c r="D69" s="2" t="s">
         <x:v>507</x:v>
-      </x:c>
-      <x:c r="C69" t="s">
-        <x:v>494</x:v>
-      </x:c>
-      <x:c r="D69" s="2" t="s">
-        <x:v>508</x:v>
       </x:c>
       <x:c r="E69">
         <x:v>1</x:v>
@@ -9194,10 +9191,10 @@
         <x:v>411</x:v>
       </x:c>
       <x:c r="J69" t="s">
-        <x:v>497</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="K69" t="s">
-        <x:v>509</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="L69" t="s">
         <x:v>25</x:v>
@@ -9206,13 +9203,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N69" t="s">
+        <x:v>509</x:v>
+      </x:c>
+      <x:c r="O69" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="P69" t="s">
         <x:v>510</x:v>
-      </x:c>
-      <x:c r="O69" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="P69" t="s">
-        <x:v>511</x:v>
       </x:c>
       <x:c r="Q69" s="36"/>
       <x:c r="R69" s="36"/>
@@ -9241,13 +9238,13 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="B70" t="s">
+        <x:v>511</x:v>
+      </x:c>
+      <x:c r="C70" t="s">
         <x:v>512</x:v>
       </x:c>
-      <x:c r="C70" t="s">
+      <x:c r="D70" s="2" t="s">
         <x:v>513</x:v>
-      </x:c>
-      <x:c r="D70" s="2" t="s">
-        <x:v>514</x:v>
       </x:c>
       <x:c r="E70">
         <x:v>2</x:v>
@@ -9256,31 +9253,31 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="H70" t="s">
+        <x:v>514</x:v>
+      </x:c>
+      <x:c r="I70" t="s">
         <x:v>515</x:v>
       </x:c>
-      <x:c r="I70" t="s">
+      <x:c r="J70" t="s">
         <x:v>516</x:v>
       </x:c>
-      <x:c r="J70" t="s">
+      <x:c r="K70" t="s">
         <x:v>517</x:v>
       </x:c>
-      <x:c r="K70" t="s">
+      <x:c r="L70" t="s">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="M70" t="s">
         <x:v>518</x:v>
-      </x:c>
-      <x:c r="L70" t="s">
-        <x:v>513</x:v>
-      </x:c>
-      <x:c r="M70" t="s">
-        <x:v>519</x:v>
       </x:c>
       <x:c r="N70" t="s">
         <x:v>356</x:v>
       </x:c>
       <x:c r="O70" t="s">
+        <x:v>519</x:v>
+      </x:c>
+      <x:c r="P70" t="s">
         <x:v>520</x:v>
-      </x:c>
-      <x:c r="P70" t="s">
-        <x:v>521</x:v>
       </x:c>
       <x:c r="Q70" s="36"/>
       <x:c r="R70" s="36"/>
@@ -9309,13 +9306,13 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="B71" t="s">
+        <x:v>521</x:v>
+      </x:c>
+      <x:c r="C71" t="s">
         <x:v>522</x:v>
       </x:c>
-      <x:c r="C71" t="s">
+      <x:c r="D71" s="5" t="s">
         <x:v>523</x:v>
-      </x:c>
-      <x:c r="D71" s="5" t="s">
-        <x:v>524</x:v>
       </x:c>
       <x:c r="E71">
         <x:v>1</x:v>
@@ -9327,31 +9324,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H71" t="s">
-        <x:v>515</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="I71" t="s">
-        <x:v>525</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="J71" t="s">
         <x:v>309</x:v>
       </x:c>
       <x:c r="K71" t="s">
-        <x:v>526</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="L71" t="s">
-        <x:v>523</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="M71" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N71" t="s">
-        <x:v>490</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="O71" t="s">
+        <x:v>526</x:v>
+      </x:c>
+      <x:c r="P71" t="s">
         <x:v>527</x:v>
-      </x:c>
-      <x:c r="P71" t="s">
-        <x:v>528</x:v>
       </x:c>
       <x:c r="Q71" s="36"/>
       <x:c r="R71" s="36"/>
@@ -9380,10 +9377,10 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B72" t="s">
+        <x:v>528</x:v>
+      </x:c>
+      <x:c r="C72" t="s">
         <x:v>529</x:v>
-      </x:c>
-      <x:c r="C72" t="s">
-        <x:v>530</x:v>
       </x:c>
       <x:c r="D72" s="5">
         <x:v>46363</x:v>
@@ -9401,16 +9398,16 @@
         <x:v>238</x:v>
       </x:c>
       <x:c r="I72" t="s">
+        <x:v>530</x:v>
+      </x:c>
+      <x:c r="J72" t="s">
         <x:v>531</x:v>
       </x:c>
-      <x:c r="J72" t="s">
+      <x:c r="K72" t="s">
         <x:v>532</x:v>
       </x:c>
-      <x:c r="K72" t="s">
-        <x:v>533</x:v>
-      </x:c>
       <x:c r="L72" t="s">
-        <x:v>530</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="M72" t="s">
         <x:v>26</x:v>
@@ -9422,7 +9419,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="P72" t="s">
-        <x:v>534</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="Q72" s="36" t="str">
         <x:v>Award</x:v>
@@ -9467,13 +9464,13 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B73" t="s">
+        <x:v>534</x:v>
+      </x:c>
+      <x:c r="C73" t="s">
         <x:v>535</x:v>
       </x:c>
-      <x:c r="C73" t="s">
+      <x:c r="D73" s="2" t="s">
         <x:v>536</x:v>
-      </x:c>
-      <x:c r="D73" s="2" t="s">
-        <x:v>537</x:v>
       </x:c>
       <x:c r="E73">
         <x:v>1</x:v>
@@ -9485,31 +9482,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H73" t="s">
-        <x:v>461</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="I73" t="s">
-        <x:v>538</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="J73" t="s">
         <x:v>309</x:v>
       </x:c>
       <x:c r="K73" t="s">
-        <x:v>539</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="L73" t="s">
-        <x:v>536</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="M73" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N73" t="s">
+        <x:v>539</x:v>
+      </x:c>
+      <x:c r="O73" t="s">
         <x:v>540</x:v>
       </x:c>
-      <x:c r="O73" t="s">
+      <x:c r="P73" t="s">
         <x:v>541</x:v>
-      </x:c>
-      <x:c r="P73" t="s">
-        <x:v>542</x:v>
       </x:c>
       <x:c r="Q73" s="36"/>
       <x:c r="R73" s="36"/>
@@ -9538,13 +9535,13 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B74" t="s">
+        <x:v>542</x:v>
+      </x:c>
+      <x:c r="C74" t="s">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D74" s="2" t="s">
         <x:v>543</x:v>
-      </x:c>
-      <x:c r="C74" t="s">
-        <x:v>513</x:v>
-      </x:c>
-      <x:c r="D74" s="2" t="s">
-        <x:v>544</x:v>
       </x:c>
       <x:c r="E74">
         <x:v>10</x:v>
@@ -9556,31 +9553,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H74" t="s">
+        <x:v>544</x:v>
+      </x:c>
+      <x:c r="I74" t="s">
         <x:v>545</x:v>
-      </x:c>
-      <x:c r="I74" t="s">
-        <x:v>546</x:v>
       </x:c>
       <x:c r="J74" t="s">
         <x:v>309</x:v>
       </x:c>
       <x:c r="K74" t="s">
-        <x:v>547</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="L74" t="s">
-        <x:v>513</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="M74" t="s">
-        <x:v>519</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="N74" t="s">
         <x:v>356</x:v>
       </x:c>
       <x:c r="O74" t="s">
-        <x:v>548</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="P74" t="s">
-        <x:v>521</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="Q74" s="36"/>
       <x:c r="R74" s="36"/>
@@ -9609,10 +9606,10 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B75" s="12" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="C75" s="12" t="s">
         <x:v>549</x:v>
-      </x:c>
-      <x:c r="C75" s="12" t="s">
-        <x:v>550</x:v>
       </x:c>
       <x:c r="D75" s="5">
         <x:v>46150</x:v>
@@ -9627,19 +9624,19 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H75" s="12" t="s">
+        <x:v>549</x:v>
+      </x:c>
+      <x:c r="I75" s="14" t="s">
         <x:v>550</x:v>
-      </x:c>
-      <x:c r="I75" s="14" t="s">
-        <x:v>551</x:v>
       </x:c>
       <x:c r="J75" s="12" t="s">
         <x:v>309</x:v>
       </x:c>
       <x:c r="K75" s="12" t="s">
-        <x:v>552</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="L75" s="12" t="s">
-        <x:v>550</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="M75" s="12" t="s">
         <x:v>26</x:v>
@@ -9648,7 +9645,7 @@
         <x:v>270</x:v>
       </x:c>
       <x:c r="O75" t="s">
-        <x:v>553</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="P75" s="12" t="s">
         <x:v>25</x:v>
@@ -9680,13 +9677,13 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B76" s="12" t="s">
+        <x:v>553</x:v>
+      </x:c>
+      <x:c r="C76" s="12" t="s">
         <x:v>554</x:v>
       </x:c>
-      <x:c r="C76" s="12" t="s">
+      <x:c r="D76" s="13" t="s">
         <x:v>555</x:v>
-      </x:c>
-      <x:c r="D76" s="13" t="s">
-        <x:v>556</x:v>
       </x:c>
       <x:c r="E76">
         <x:v>1</x:v>
@@ -9698,31 +9695,31 @@
         <x:v>Best Vertical Solution (Family Office Track), 2,000 Cybrdeck API credits (worth US$25)</x:v>
       </x:c>
       <x:c r="H76" s="12" t="s">
+        <x:v>556</x:v>
+      </x:c>
+      <x:c r="I76" s="12" t="s">
         <x:v>557</x:v>
       </x:c>
-      <x:c r="I76" s="12" t="s">
+      <x:c r="J76" s="12" t="s">
         <x:v>558</x:v>
       </x:c>
-      <x:c r="J76" s="12" t="s">
+      <x:c r="K76" s="12" t="s">
         <x:v>559</x:v>
       </x:c>
-      <x:c r="K76" s="12" t="s">
-        <x:v>560</x:v>
-      </x:c>
       <x:c r="L76" s="12" t="s">
-        <x:v>555</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="M76" s="12" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N76" s="12" t="s">
+        <x:v>560</x:v>
+      </x:c>
+      <x:c r="O76" s="1" t="s">
         <x:v>561</x:v>
       </x:c>
-      <x:c r="O76" s="1" t="s">
+      <x:c r="P76" t="s">
         <x:v>562</x:v>
-      </x:c>
-      <x:c r="P76" t="s">
-        <x:v>563</x:v>
       </x:c>
       <x:c r="Q76" s="36" t="str">
         <x:v>Best Vertical Solution</x:v>
@@ -9767,13 +9764,13 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B77" t="s">
+        <x:v>563</x:v>
+      </x:c>
+      <x:c r="C77" t="s">
         <x:v>564</x:v>
       </x:c>
-      <x:c r="C77" t="s">
+      <x:c r="D77" t="s">
         <x:v>565</x:v>
-      </x:c>
-      <x:c r="D77" t="s">
-        <x:v>566</x:v>
       </x:c>
       <x:c r="E77">
         <x:v>1</x:v>
@@ -9785,31 +9782,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H77" t="s">
+        <x:v>566</x:v>
+      </x:c>
+      <x:c r="I77" t="s">
         <x:v>567</x:v>
-      </x:c>
-      <x:c r="I77" t="s">
-        <x:v>568</x:v>
       </x:c>
       <x:c r="J77" t="s">
         <x:v>309</x:v>
       </x:c>
       <x:c r="K77" t="s">
+        <x:v>568</x:v>
+      </x:c>
+      <x:c r="L77" t="s">
         <x:v>569</x:v>
-      </x:c>
-      <x:c r="L77" t="s">
-        <x:v>570</x:v>
       </x:c>
       <x:c r="M77" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N77" t="s">
+        <x:v>570</x:v>
+      </x:c>
+      <x:c r="O77" t="s">
         <x:v>571</x:v>
       </x:c>
-      <x:c r="O77" t="s">
+      <x:c r="P77" t="s">
         <x:v>572</x:v>
-      </x:c>
-      <x:c r="P77" t="s">
-        <x:v>573</x:v>
       </x:c>
       <x:c r="Q77" s="36"/>
       <x:c r="R77" s="36"/>
@@ -9838,13 +9835,13 @@
         <x:v>77</x:v>
       </x:c>
       <x:c r="B78" t="s">
+        <x:v>573</x:v>
+      </x:c>
+      <x:c r="C78" t="s">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D78" t="s">
         <x:v>574</x:v>
-      </x:c>
-      <x:c r="C78" t="s">
-        <x:v>513</x:v>
-      </x:c>
-      <x:c r="D78" t="s">
-        <x:v>575</x:v>
       </x:c>
       <x:c r="E78">
         <x:v>1</x:v>
@@ -9856,31 +9853,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H78" t="s">
+        <x:v>575</x:v>
+      </x:c>
+      <x:c r="I78" t="s">
         <x:v>576</x:v>
-      </x:c>
-      <x:c r="I78" t="s">
-        <x:v>577</x:v>
       </x:c>
       <x:c r="J78" t="s">
         <x:v>309</x:v>
       </x:c>
       <x:c r="K78" t="s">
-        <x:v>578</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="L78" t="s">
-        <x:v>513</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="M78" t="s">
-        <x:v>519</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="N78" t="s">
         <x:v>356</x:v>
       </x:c>
       <x:c r="O78" t="s">
-        <x:v>579</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="P78" t="s">
-        <x:v>521</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="Q78" s="36"/>
       <x:c r="R78" s="36"/>
@@ -9909,37 +9906,37 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="B79" t="s">
+        <x:v>579</x:v>
+      </x:c>
+      <x:c r="C79" t="s">
         <x:v>580</x:v>
       </x:c>
-      <x:c r="C79" t="s">
+      <x:c r="D79" t="s">
         <x:v>581</x:v>
-      </x:c>
-      <x:c r="D79" t="s">
-        <x:v>582</x:v>
       </x:c>
       <x:c r="E79">
         <x:v>4</x:v>
       </x:c>
       <x:c r="F79" t="s">
-        <x:v>467</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="G79" t="s">
         <x:v>25</x:v>
       </x:c>
       <x:c r="H79" t="s">
+        <x:v>582</x:v>
+      </x:c>
+      <x:c r="I79" t="s">
         <x:v>583</x:v>
       </x:c>
-      <x:c r="I79" t="s">
+      <x:c r="J79" t="s">
         <x:v>584</x:v>
       </x:c>
-      <x:c r="J79" t="s">
+      <x:c r="K79" t="s">
         <x:v>585</x:v>
       </x:c>
-      <x:c r="K79" t="s">
+      <x:c r="L79" t="s">
         <x:v>586</x:v>
-      </x:c>
-      <x:c r="L79" t="s">
-        <x:v>587</x:v>
       </x:c>
       <x:c r="M79" t="s">
         <x:v>26</x:v>
@@ -9948,10 +9945,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="O79" t="s">
+        <x:v>587</x:v>
+      </x:c>
+      <x:c r="P79" t="s">
         <x:v>588</x:v>
-      </x:c>
-      <x:c r="P79" t="s">
-        <x:v>589</x:v>
       </x:c>
       <x:c r="Q79" s="36"/>
       <x:c r="R79" s="36"/>
@@ -10224,10 +10221,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R95b117621d5e4e86"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rfc1fc4a1196541f2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rff0609161e104161"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Ra7ea9f4d83704f6a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R111a9b89060e430b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R62b5d75a144c4094"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Ra85ea0efba7b4665"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R09c9760ce8c24615"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -10250,7 +10247,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>590</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -10259,7 +10256,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="19" t="s">
-        <x:v>591</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="B2" s="19"/>
       <x:c r="C2" s="19"/>
@@ -10268,64 +10265,64 @@
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="11" t="s">
+        <x:v>591</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="s">
         <x:v>592</x:v>
       </x:c>
-      <x:c r="B4" s="11" t="s">
+      <x:c r="C4" s="11" t="s">
         <x:v>593</x:v>
       </x:c>
-      <x:c r="C4" s="11" t="s">
+      <x:c r="D4" s="11" t="s">
         <x:v>594</x:v>
       </x:c>
-      <x:c r="D4" s="11" t="s">
+      <x:c r="E4" s="11" t="s">
         <x:v>595</x:v>
-      </x:c>
-      <x:c r="E4" s="11" t="s">
-        <x:v>596</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="8" t="s">
+        <x:v>596</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="s">
         <x:v>597</x:v>
       </x:c>
-      <x:c r="B5" s="7" t="s">
+      <x:c r="C5" s="7" t="s">
         <x:v>598</x:v>
-      </x:c>
-      <x:c r="C5" s="7" t="s">
-        <x:v>599</x:v>
       </x:c>
       <x:c r="D5" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E5" s="10" t="s">
-        <x:v>600</x:v>
+        <x:v>599</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="8" t="s">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>601</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="s">
+      <x:c r="C6" s="7" t="s">
         <x:v>602</x:v>
-      </x:c>
-      <x:c r="C6" s="7" t="s">
-        <x:v>603</x:v>
       </x:c>
       <x:c r="D6" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="10" t="s">
-        <x:v>604</x:v>
+        <x:v>603</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="8" t="s">
+        <x:v>604</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
         <x:v>605</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="s">
+      <x:c r="C7" s="7" t="s">
         <x:v>606</x:v>
-      </x:c>
-      <x:c r="C7" s="7" t="s">
-        <x:v>607</x:v>
       </x:c>
       <x:c r="D7" s="9">
         <x:v>1</x:v>
@@ -10334,47 +10331,47 @@
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
       <x:c r="A8" s="8" t="s">
+        <x:v>607</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
         <x:v>608</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="s">
+      <x:c r="C8" s="7" t="s">
         <x:v>609</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="s">
-        <x:v>610</x:v>
       </x:c>
       <x:c r="D8" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E8" s="10" t="s">
-        <x:v>611</x:v>
+        <x:v>610</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" s="8" t="s">
+        <x:v>611</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
         <x:v>612</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="s">
-        <x:v>613</x:v>
-      </x:c>
       <x:c r="C9" s="7" t="s">
-        <x:v>603</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="D9" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="10" t="s">
-        <x:v>614</x:v>
+        <x:v>613</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
       <x:c r="A10" s="8" t="s">
+        <x:v>614</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="s">
         <x:v>615</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="s">
+      <x:c r="C10" s="7" t="s">
         <x:v>616</x:v>
-      </x:c>
-      <x:c r="C10" s="7" t="s">
-        <x:v>617</x:v>
       </x:c>
       <x:c r="D10" s="9">
         <x:v>1</x:v>
@@ -10383,47 +10380,47 @@
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
       <x:c r="A11" s="8" t="s">
+        <x:v>617</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="s">
         <x:v>618</x:v>
       </x:c>
-      <x:c r="B11" s="7" t="s">
+      <x:c r="C11" s="7" t="s">
         <x:v>619</x:v>
-      </x:c>
-      <x:c r="C11" s="7" t="s">
-        <x:v>620</x:v>
       </x:c>
       <x:c r="D11" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E11" s="10" t="s">
-        <x:v>621</x:v>
+        <x:v>620</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
       <x:c r="A12" s="8" t="s">
+        <x:v>621</x:v>
+      </x:c>
+      <x:c r="B12" s="7" t="s">
         <x:v>622</x:v>
       </x:c>
-      <x:c r="B12" s="7" t="s">
+      <x:c r="C12" s="7" t="s">
         <x:v>623</x:v>
-      </x:c>
-      <x:c r="C12" s="7" t="s">
-        <x:v>624</x:v>
       </x:c>
       <x:c r="D12" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E12" s="10" t="s">
-        <x:v>625</x:v>
+        <x:v>624</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
       <x:c r="A13" s="8" t="s">
+        <x:v>625</x:v>
+      </x:c>
+      <x:c r="B13" s="7" t="s">
         <x:v>626</x:v>
       </x:c>
-      <x:c r="B13" s="7" t="s">
+      <x:c r="C13" s="7" t="s">
         <x:v>627</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="s">
-        <x:v>628</x:v>
       </x:c>
       <x:c r="D13" s="9">
         <x:v>1</x:v>
@@ -10432,30 +10429,30 @@
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
       <x:c r="A14" s="8" t="s">
+        <x:v>628</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="s">
         <x:v>629</x:v>
       </x:c>
-      <x:c r="B14" s="7" t="s">
-        <x:v>630</x:v>
-      </x:c>
       <x:c r="C14" s="7" t="s">
-        <x:v>628</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="D14" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E14" s="10" t="s">
-        <x:v>631</x:v>
+        <x:v>630</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
       <x:c r="A15" s="8" t="s">
+        <x:v>631</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="s">
         <x:v>632</x:v>
       </x:c>
-      <x:c r="B15" s="7" t="s">
+      <x:c r="C15" s="7" t="s">
         <x:v>633</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="s">
-        <x:v>634</x:v>
       </x:c>
       <x:c r="D15" s="9">
         <x:v>1</x:v>
@@ -10464,30 +10461,30 @@
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
       <x:c r="A16" s="8" t="s">
+        <x:v>634</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="s">
         <x:v>635</x:v>
       </x:c>
-      <x:c r="B16" s="7" t="s">
+      <x:c r="C16" s="7" t="s">
         <x:v>636</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="s">
-        <x:v>637</x:v>
       </x:c>
       <x:c r="D16" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E16" s="10" t="s">
-        <x:v>638</x:v>
+        <x:v>637</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
       <x:c r="A17" s="8" t="s">
+        <x:v>638</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="s">
         <x:v>639</x:v>
       </x:c>
-      <x:c r="B17" s="7" t="s">
+      <x:c r="C17" s="7" t="s">
         <x:v>640</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="s">
-        <x:v>641</x:v>
       </x:c>
       <x:c r="D17" s="9">
         <x:v>1</x:v>
@@ -10496,47 +10493,47 @@
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
       <x:c r="A18" s="8" t="s">
+        <x:v>641</x:v>
+      </x:c>
+      <x:c r="B18" s="7" t="s">
         <x:v>642</x:v>
       </x:c>
-      <x:c r="B18" s="7" t="s">
+      <x:c r="C18" s="7" t="s">
         <x:v>643</x:v>
-      </x:c>
-      <x:c r="C18" s="7" t="s">
-        <x:v>644</x:v>
       </x:c>
       <x:c r="D18" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E18" s="10" t="s">
-        <x:v>645</x:v>
+        <x:v>644</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
       <x:c r="A19" s="8" t="s">
+        <x:v>645</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="s">
         <x:v>646</x:v>
       </x:c>
-      <x:c r="B19" s="7" t="s">
+      <x:c r="C19" s="7" t="s">
         <x:v>647</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="s">
-        <x:v>648</x:v>
       </x:c>
       <x:c r="D19" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E19" s="10" t="s">
-        <x:v>649</x:v>
+        <x:v>648</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28" customHeight="1">
       <x:c r="A20" s="8" t="s">
+        <x:v>649</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="s">
         <x:v>650</x:v>
       </x:c>
-      <x:c r="B20" s="7" t="s">
+      <x:c r="C20" s="7" t="s">
         <x:v>651</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>652</x:v>
       </x:c>
       <x:c r="D20" s="9">
         <x:v>1</x:v>
@@ -10545,10 +10542,10 @@
     </x:row>
     <x:row r="21" ht="28" customHeight="1">
       <x:c r="A21" s="8" t="s">
+        <x:v>652</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="s">
         <x:v>653</x:v>
-      </x:c>
-      <x:c r="B21" s="7" t="s">
-        <x:v>654</x:v>
       </x:c>
       <x:c r="C21" s="7" t="str">
         <x:v>#069, #071, #079</x:v>
@@ -10557,18 +10554,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E21" s="10" t="s">
-        <x:v>655</x:v>
+        <x:v>654</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
       <x:c r="A22" s="8" t="s">
+        <x:v>655</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="s">
         <x:v>656</x:v>
       </x:c>
-      <x:c r="B22" s="7" t="s">
+      <x:c r="C22" s="7" t="s">
         <x:v>657</x:v>
-      </x:c>
-      <x:c r="C22" s="7" t="s">
-        <x:v>658</x:v>
       </x:c>
       <x:c r="D22" s="9">
         <x:v>1</x:v>
@@ -10577,13 +10574,13 @@
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
       <x:c r="A23" s="8" t="s">
+        <x:v>658</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="s">
         <x:v>659</x:v>
       </x:c>
-      <x:c r="B23" s="7" t="s">
+      <x:c r="C23" s="7" t="s">
         <x:v>660</x:v>
-      </x:c>
-      <x:c r="C23" s="7" t="s">
-        <x:v>661</x:v>
       </x:c>
       <x:c r="D23" s="9">
         <x:v>1</x:v>
@@ -10592,10 +10589,10 @@
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
       <x:c r="A24" s="8" t="s">
+        <x:v>661</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="s">
         <x:v>662</x:v>
-      </x:c>
-      <x:c r="B24" s="7" t="s">
-        <x:v>663</x:v>
       </x:c>
       <x:c r="C24" s="7" t="str">
         <x:v>#054, #055, #056, #062, #066, #068, #075</x:v>
@@ -10604,12 +10601,12 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E24" s="10" t="s">
-        <x:v>664</x:v>
+        <x:v>663</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
       <x:c r="A25" s="8" t="s">
-        <x:v>665</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
         <x:v>Clement Lork</x:v>
@@ -10621,18 +10618,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E25" s="10" t="s">
-        <x:v>666</x:v>
+        <x:v>665</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="8" t="s">
+        <x:v>666</x:v>
+      </x:c>
+      <x:c r="B26" s="7" t="s">
         <x:v>667</x:v>
       </x:c>
-      <x:c r="B26" s="7" t="s">
-        <x:v>668</x:v>
-      </x:c>
       <x:c r="C26" s="7" t="s">
-        <x:v>607</x:v>
+        <x:v>606</x:v>
       </x:c>
       <x:c r="D26" s="9">
         <x:v>1</x:v>
@@ -10641,13 +10638,13 @@
     </x:row>
     <x:row r="27" ht="28" customHeight="1">
       <x:c r="A27" s="8" t="s">
+        <x:v>668</x:v>
+      </x:c>
+      <x:c r="B27" s="7" t="s">
         <x:v>669</x:v>
       </x:c>
-      <x:c r="B27" s="7" t="s">
+      <x:c r="C27" s="7" t="s">
         <x:v>670</x:v>
-      </x:c>
-      <x:c r="C27" s="7" t="s">
-        <x:v>671</x:v>
       </x:c>
       <x:c r="D27" s="9">
         <x:v>1</x:v>
@@ -10656,13 +10653,13 @@
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
       <x:c r="A28" s="8" t="s">
+        <x:v>671</x:v>
+      </x:c>
+      <x:c r="B28" s="7" t="s">
         <x:v>672</x:v>
       </x:c>
-      <x:c r="B28" s="7" t="s">
+      <x:c r="C28" s="7" t="s">
         <x:v>673</x:v>
-      </x:c>
-      <x:c r="C28" s="7" t="s">
-        <x:v>674</x:v>
       </x:c>
       <x:c r="D28" s="9">
         <x:v>2</x:v>
@@ -10671,13 +10668,13 @@
     </x:row>
     <x:row r="29" ht="28" customHeight="1">
       <x:c r="A29" s="8" t="s">
+        <x:v>674</x:v>
+      </x:c>
+      <x:c r="B29" s="7" t="s">
         <x:v>675</x:v>
       </x:c>
-      <x:c r="B29" s="7" t="s">
+      <x:c r="C29" s="7" t="s">
         <x:v>676</x:v>
-      </x:c>
-      <x:c r="C29" s="7" t="s">
-        <x:v>677</x:v>
       </x:c>
       <x:c r="D29" s="9">
         <x:v>4</x:v>
@@ -10686,13 +10683,13 @@
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
       <x:c r="A30" s="8" t="s">
+        <x:v>677</x:v>
+      </x:c>
+      <x:c r="B30" s="7" t="s">
         <x:v>678</x:v>
       </x:c>
-      <x:c r="B30" s="7" t="s">
-        <x:v>679</x:v>
-      </x:c>
       <x:c r="C30" s="7" t="s">
-        <x:v>671</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="D30" s="9">
         <x:v>1</x:v>
@@ -10701,47 +10698,47 @@
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="8" t="s">
+        <x:v>679</x:v>
+      </x:c>
+      <x:c r="B31" s="7" t="s">
         <x:v>680</x:v>
       </x:c>
-      <x:c r="B31" s="7" t="s">
-        <x:v>681</x:v>
-      </x:c>
       <x:c r="C31" s="7" t="s">
-        <x:v>620</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="D31" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E31" s="10" t="s">
-        <x:v>682</x:v>
+        <x:v>681</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="28" customHeight="1">
       <x:c r="A32" s="8" t="s">
+        <x:v>682</x:v>
+      </x:c>
+      <x:c r="B32" s="7" t="s">
         <x:v>683</x:v>
       </x:c>
-      <x:c r="B32" s="7" t="s">
+      <x:c r="C32" s="7" t="s">
         <x:v>684</x:v>
-      </x:c>
-      <x:c r="C32" s="7" t="s">
-        <x:v>685</x:v>
       </x:c>
       <x:c r="D32" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E32" s="10" t="s">
-        <x:v>686</x:v>
+        <x:v>685</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="8" t="s">
+        <x:v>686</x:v>
+      </x:c>
+      <x:c r="B33" s="7" t="s">
         <x:v>687</x:v>
       </x:c>
-      <x:c r="B33" s="7" t="s">
-        <x:v>688</x:v>
-      </x:c>
       <x:c r="C33" s="7" t="s">
-        <x:v>658</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="D33" s="9">
         <x:v>1</x:v>
@@ -10750,13 +10747,13 @@
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
       <x:c r="A34" s="8" t="s">
+        <x:v>688</x:v>
+      </x:c>
+      <x:c r="B34" s="7" t="s">
         <x:v>689</x:v>
       </x:c>
-      <x:c r="B34" s="7" t="s">
+      <x:c r="C34" s="7" t="s">
         <x:v>690</x:v>
-      </x:c>
-      <x:c r="C34" s="7" t="s">
-        <x:v>691</x:v>
       </x:c>
       <x:c r="D34" s="9">
         <x:v>1</x:v>
@@ -10765,47 +10762,47 @@
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
       <x:c r="A35" s="8" t="s">
+        <x:v>691</x:v>
+      </x:c>
+      <x:c r="B35" s="7" t="s">
         <x:v>692</x:v>
       </x:c>
-      <x:c r="B35" s="7" t="s">
+      <x:c r="C35" s="7" t="s">
         <x:v>693</x:v>
-      </x:c>
-      <x:c r="C35" s="7" t="s">
-        <x:v>694</x:v>
       </x:c>
       <x:c r="D35" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E35" s="10" t="s">
-        <x:v>695</x:v>
+        <x:v>694</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
       <x:c r="A36" s="8" t="s">
+        <x:v>695</x:v>
+      </x:c>
+      <x:c r="B36" s="7" t="s">
         <x:v>696</x:v>
       </x:c>
-      <x:c r="B36" s="7" t="s">
+      <x:c r="C36" s="7" t="s">
         <x:v>697</x:v>
-      </x:c>
-      <x:c r="C36" s="7" t="s">
-        <x:v>698</x:v>
       </x:c>
       <x:c r="D36" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E36" s="10" t="s">
-        <x:v>699</x:v>
+        <x:v>698</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
       <x:c r="A37" s="8" t="s">
+        <x:v>699</x:v>
+      </x:c>
+      <x:c r="B37" s="7" t="s">
         <x:v>700</x:v>
       </x:c>
-      <x:c r="B37" s="7" t="s">
+      <x:c r="C37" s="7" t="s">
         <x:v>701</x:v>
-      </x:c>
-      <x:c r="C37" s="7" t="s">
-        <x:v>702</x:v>
       </x:c>
       <x:c r="D37" s="9">
         <x:v>1</x:v>
@@ -10814,13 +10811,13 @@
     </x:row>
     <x:row r="38" ht="28" customHeight="1">
       <x:c r="A38" s="8" t="s">
+        <x:v>702</x:v>
+      </x:c>
+      <x:c r="B38" s="7" t="s">
         <x:v>703</x:v>
       </x:c>
-      <x:c r="B38" s="7" t="s">
-        <x:v>704</x:v>
-      </x:c>
       <x:c r="C38" s="7" t="s">
-        <x:v>641</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="D38" s="9">
         <x:v>1</x:v>
@@ -10829,13 +10826,13 @@
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
       <x:c r="A39" s="8" t="s">
+        <x:v>704</x:v>
+      </x:c>
+      <x:c r="B39" s="7" t="s">
         <x:v>705</x:v>
       </x:c>
-      <x:c r="B39" s="7" t="s">
+      <x:c r="C39" s="7" t="s">
         <x:v>706</x:v>
-      </x:c>
-      <x:c r="C39" s="7" t="s">
-        <x:v>707</x:v>
       </x:c>
       <x:c r="D39" s="9">
         <x:v>3</x:v>
@@ -10844,47 +10841,47 @@
     </x:row>
     <x:row r="40" ht="28" customHeight="1">
       <x:c r="A40" s="8" t="s">
+        <x:v>707</x:v>
+      </x:c>
+      <x:c r="B40" s="7" t="s">
         <x:v>708</x:v>
       </x:c>
-      <x:c r="B40" s="7" t="s">
+      <x:c r="C40" s="7" t="s">
         <x:v>709</x:v>
-      </x:c>
-      <x:c r="C40" s="7" t="s">
-        <x:v>710</x:v>
       </x:c>
       <x:c r="D40" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E40" s="10" t="s">
-        <x:v>711</x:v>
+        <x:v>710</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="8" t="s">
+        <x:v>711</x:v>
+      </x:c>
+      <x:c r="B41" s="7" t="s">
         <x:v>712</x:v>
       </x:c>
-      <x:c r="B41" s="7" t="s">
-        <x:v>713</x:v>
-      </x:c>
       <x:c r="C41" s="7" t="s">
-        <x:v>710</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="D41" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E41" s="10" t="s">
-        <x:v>714</x:v>
+        <x:v>713</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
       <x:c r="A42" s="8" t="s">
+        <x:v>714</x:v>
+      </x:c>
+      <x:c r="B42" s="7" t="s">
         <x:v>715</x:v>
       </x:c>
-      <x:c r="B42" s="7" t="s">
+      <x:c r="C42" s="7" t="s">
         <x:v>716</x:v>
-      </x:c>
-      <x:c r="C42" s="7" t="s">
-        <x:v>717</x:v>
       </x:c>
       <x:c r="D42" s="9">
         <x:v>1</x:v>
@@ -10893,10 +10890,10 @@
     </x:row>
     <x:row r="43" ht="28" customHeight="1">
       <x:c r="A43" s="8" t="s">
+        <x:v>717</x:v>
+      </x:c>
+      <x:c r="B43" s="7" t="s">
         <x:v>718</x:v>
-      </x:c>
-      <x:c r="B43" s="7" t="s">
-        <x:v>719</x:v>
       </x:c>
       <x:c r="C43" s="7" t="str">
         <x:v>#069, #079</x:v>
@@ -10908,30 +10905,30 @@
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="8" t="s">
+        <x:v>719</x:v>
+      </x:c>
+      <x:c r="B44" s="7" t="s">
         <x:v>720</x:v>
       </x:c>
-      <x:c r="B44" s="7" t="s">
-        <x:v>721</x:v>
-      </x:c>
       <x:c r="C44" s="7" t="s">
-        <x:v>674</x:v>
+        <x:v>673</x:v>
       </x:c>
       <x:c r="D44" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E44" s="10" t="s">
-        <x:v>722</x:v>
+        <x:v>721</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
       <x:c r="A45" s="8" t="s">
+        <x:v>722</x:v>
+      </x:c>
+      <x:c r="B45" s="7" t="s">
         <x:v>723</x:v>
       </x:c>
-      <x:c r="B45" s="7" t="s">
+      <x:c r="C45" s="7" t="s">
         <x:v>724</x:v>
-      </x:c>
-      <x:c r="C45" s="7" t="s">
-        <x:v>725</x:v>
       </x:c>
       <x:c r="D45" s="9">
         <x:v>1</x:v>
@@ -10940,13 +10937,13 @@
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
       <x:c r="A46" s="8" t="s">
+        <x:v>725</x:v>
+      </x:c>
+      <x:c r="B46" s="7" t="s">
         <x:v>726</x:v>
       </x:c>
-      <x:c r="B46" s="7" t="s">
-        <x:v>727</x:v>
-      </x:c>
       <x:c r="C46" s="7" t="s">
-        <x:v>691</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="D46" s="9">
         <x:v>1</x:v>
@@ -10955,47 +10952,47 @@
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
       <x:c r="A47" s="8" t="s">
+        <x:v>727</x:v>
+      </x:c>
+      <x:c r="B47" s="7" t="s">
         <x:v>728</x:v>
       </x:c>
-      <x:c r="B47" s="7" t="s">
-        <x:v>729</x:v>
-      </x:c>
       <x:c r="C47" s="7" t="s">
-        <x:v>603</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="D47" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E47" s="10" t="s">
-        <x:v>730</x:v>
+        <x:v>729</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
       <x:c r="A48" s="8" t="s">
+        <x:v>730</x:v>
+      </x:c>
+      <x:c r="B48" s="7" t="s">
         <x:v>731</x:v>
       </x:c>
-      <x:c r="B48" s="7" t="s">
+      <x:c r="C48" s="7" t="s">
         <x:v>732</x:v>
-      </x:c>
-      <x:c r="C48" s="7" t="s">
-        <x:v>733</x:v>
       </x:c>
       <x:c r="D48" s="9">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="10" t="s">
-        <x:v>734</x:v>
+        <x:v>733</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
       <x:c r="A49" s="8" t="s">
+        <x:v>734</x:v>
+      </x:c>
+      <x:c r="B49" s="7" t="s">
         <x:v>735</x:v>
       </x:c>
-      <x:c r="B49" s="7" t="s">
+      <x:c r="C49" s="7" t="s">
         <x:v>736</x:v>
-      </x:c>
-      <x:c r="C49" s="7" t="s">
-        <x:v>737</x:v>
       </x:c>
       <x:c r="D49" s="9">
         <x:v>1</x:v>
@@ -11004,13 +11001,13 @@
     </x:row>
     <x:row r="50" ht="28" customHeight="1">
       <x:c r="A50" s="8" t="s">
+        <x:v>737</x:v>
+      </x:c>
+      <x:c r="B50" s="7" t="s">
         <x:v>738</x:v>
       </x:c>
-      <x:c r="B50" s="7" t="s">
-        <x:v>739</x:v>
-      </x:c>
       <x:c r="C50" s="7" t="s">
-        <x:v>702</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="D50" s="9">
         <x:v>1</x:v>
@@ -11019,64 +11016,64 @@
     </x:row>
     <x:row r="51" ht="28" customHeight="1">
       <x:c r="A51" s="8" t="s">
+        <x:v>739</x:v>
+      </x:c>
+      <x:c r="B51" s="7" t="s">
         <x:v>740</x:v>
       </x:c>
-      <x:c r="B51" s="7" t="s">
+      <x:c r="C51" s="7" t="s">
         <x:v>741</x:v>
-      </x:c>
-      <x:c r="C51" s="7" t="s">
-        <x:v>742</x:v>
       </x:c>
       <x:c r="D51" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E51" s="10" t="s">
-        <x:v>743</x:v>
+        <x:v>742</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="28" customHeight="1">
       <x:c r="A52" s="8" t="s">
+        <x:v>743</x:v>
+      </x:c>
+      <x:c r="B52" s="7" t="s">
         <x:v>744</x:v>
       </x:c>
-      <x:c r="B52" s="7" t="s">
+      <x:c r="C52" s="7" t="s">
         <x:v>745</x:v>
-      </x:c>
-      <x:c r="C52" s="7" t="s">
-        <x:v>746</x:v>
       </x:c>
       <x:c r="D52" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E52" s="10" t="s">
-        <x:v>747</x:v>
+        <x:v>746</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="28" customHeight="1">
       <x:c r="A53" s="8" t="s">
+        <x:v>747</x:v>
+      </x:c>
+      <x:c r="B53" s="7" t="s">
         <x:v>748</x:v>
       </x:c>
-      <x:c r="B53" s="7" t="s">
+      <x:c r="C53" s="7" t="s">
         <x:v>749</x:v>
-      </x:c>
-      <x:c r="C53" s="7" t="s">
-        <x:v>750</x:v>
       </x:c>
       <x:c r="D53" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E53" s="10" t="s">
-        <x:v>751</x:v>
+        <x:v>750</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="28" customHeight="1">
       <x:c r="A54" s="8" t="s">
+        <x:v>751</x:v>
+      </x:c>
+      <x:c r="B54" s="7" t="s">
         <x:v>752</x:v>
       </x:c>
-      <x:c r="B54" s="7" t="s">
+      <x:c r="C54" s="7" t="s">
         <x:v>753</x:v>
-      </x:c>
-      <x:c r="C54" s="7" t="s">
-        <x:v>754</x:v>
       </x:c>
       <x:c r="D54" s="9">
         <x:v>1</x:v>
@@ -11085,81 +11082,81 @@
     </x:row>
     <x:row r="55" ht="28" customHeight="1">
       <x:c r="A55" s="8" t="s">
+        <x:v>754</x:v>
+      </x:c>
+      <x:c r="B55" s="7" t="s">
         <x:v>755</x:v>
       </x:c>
-      <x:c r="B55" s="7" t="s">
+      <x:c r="C55" s="7" t="s">
         <x:v>756</x:v>
-      </x:c>
-      <x:c r="C55" s="7" t="s">
-        <x:v>757</x:v>
       </x:c>
       <x:c r="D55" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E55" s="10" t="s">
-        <x:v>758</x:v>
+        <x:v>757</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="28" customHeight="1">
       <x:c r="A56" s="8" t="s">
+        <x:v>758</x:v>
+      </x:c>
+      <x:c r="B56" s="7" t="s">
         <x:v>759</x:v>
       </x:c>
-      <x:c r="B56" s="7" t="s">
+      <x:c r="C56" s="7" t="s">
         <x:v>760</x:v>
-      </x:c>
-      <x:c r="C56" s="7" t="s">
-        <x:v>761</x:v>
       </x:c>
       <x:c r="D56" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E56" s="10" t="s">
-        <x:v>762</x:v>
+        <x:v>761</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
       <x:c r="A57" s="8" t="s">
+        <x:v>762</x:v>
+      </x:c>
+      <x:c r="B57" s="7" t="s">
         <x:v>763</x:v>
       </x:c>
-      <x:c r="B57" s="7" t="s">
+      <x:c r="C57" s="7" t="s">
         <x:v>764</x:v>
-      </x:c>
-      <x:c r="C57" s="7" t="s">
-        <x:v>765</x:v>
       </x:c>
       <x:c r="D57" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E57" s="10" t="s">
-        <x:v>766</x:v>
+        <x:v>765</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
       <x:c r="A58" s="8" t="s">
+        <x:v>766</x:v>
+      </x:c>
+      <x:c r="B58" s="7" t="s">
         <x:v>767</x:v>
       </x:c>
-      <x:c r="B58" s="7" t="s">
+      <x:c r="C58" s="7" t="s">
         <x:v>768</x:v>
-      </x:c>
-      <x:c r="C58" s="7" t="s">
-        <x:v>769</x:v>
       </x:c>
       <x:c r="D58" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E58" s="10" t="s">
-        <x:v>770</x:v>
+        <x:v>769</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
       <x:c r="A59" s="8" t="s">
+        <x:v>770</x:v>
+      </x:c>
+      <x:c r="B59" s="7" t="s">
         <x:v>771</x:v>
       </x:c>
-      <x:c r="B59" s="7" t="s">
-        <x:v>772</x:v>
-      </x:c>
       <x:c r="C59" s="7" t="s">
-        <x:v>607</x:v>
+        <x:v>606</x:v>
       </x:c>
       <x:c r="D59" s="9">
         <x:v>1</x:v>
@@ -11168,13 +11165,13 @@
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
       <x:c r="A60" s="8" t="s">
+        <x:v>772</x:v>
+      </x:c>
+      <x:c r="B60" s="7" t="s">
         <x:v>773</x:v>
       </x:c>
-      <x:c r="B60" s="7" t="s">
-        <x:v>774</x:v>
-      </x:c>
       <x:c r="C60" s="7" t="s">
-        <x:v>644</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="D60" s="9">
         <x:v>1</x:v>
@@ -11183,13 +11180,13 @@
     </x:row>
     <x:row r="61" ht="28" customHeight="1">
       <x:c r="A61" s="8" t="s">
+        <x:v>774</x:v>
+      </x:c>
+      <x:c r="B61" s="7" t="s">
         <x:v>775</x:v>
       </x:c>
-      <x:c r="B61" s="7" t="s">
-        <x:v>776</x:v>
-      </x:c>
       <x:c r="C61" s="7" t="s">
-        <x:v>628</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="D61" s="9">
         <x:v>1</x:v>
@@ -11198,30 +11195,30 @@
     </x:row>
     <x:row r="62" ht="28" customHeight="1">
       <x:c r="A62" s="8" t="s">
+        <x:v>776</x:v>
+      </x:c>
+      <x:c r="B62" s="7" t="s">
         <x:v>777</x:v>
       </x:c>
-      <x:c r="B62" s="7" t="s">
-        <x:v>778</x:v>
-      </x:c>
       <x:c r="C62" s="7" t="s">
-        <x:v>634</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="D62" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E62" s="10" t="s">
-        <x:v>779</x:v>
+        <x:v>778</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="28" customHeight="1">
       <x:c r="A63" s="8" t="s">
+        <x:v>779</x:v>
+      </x:c>
+      <x:c r="B63" s="7" t="s">
         <x:v>780</x:v>
       </x:c>
-      <x:c r="B63" s="7" t="s">
-        <x:v>781</x:v>
-      </x:c>
       <x:c r="C63" s="7" t="s">
-        <x:v>628</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="D63" s="9">
         <x:v>1</x:v>
@@ -11230,13 +11227,13 @@
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
       <x:c r="A64" s="8" t="s">
+        <x:v>781</x:v>
+      </x:c>
+      <x:c r="B64" s="7" t="s">
         <x:v>782</x:v>
       </x:c>
-      <x:c r="B64" s="7" t="s">
+      <x:c r="C64" s="7" t="s">
         <x:v>783</x:v>
-      </x:c>
-      <x:c r="C64" s="7" t="s">
-        <x:v>784</x:v>
       </x:c>
       <x:c r="D64" s="9">
         <x:v>1</x:v>
@@ -11245,13 +11242,13 @@
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
       <x:c r="A65" s="8" t="s">
+        <x:v>784</x:v>
+      </x:c>
+      <x:c r="B65" s="7" t="s">
         <x:v>785</x:v>
       </x:c>
-      <x:c r="B65" s="7" t="s">
+      <x:c r="C65" s="7" t="s">
         <x:v>786</x:v>
-      </x:c>
-      <x:c r="C65" s="7" t="s">
-        <x:v>787</x:v>
       </x:c>
       <x:c r="D65" s="9">
         <x:v>1</x:v>
@@ -11260,13 +11257,13 @@
     </x:row>
     <x:row r="66" ht="28" customHeight="1">
       <x:c r="A66" s="8" t="s">
+        <x:v>787</x:v>
+      </x:c>
+      <x:c r="B66" s="7" t="s">
         <x:v>788</x:v>
       </x:c>
-      <x:c r="B66" s="7" t="s">
-        <x:v>789</x:v>
-      </x:c>
       <x:c r="C66" s="7" t="s">
-        <x:v>617</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="D66" s="9">
         <x:v>1</x:v>
@@ -11275,47 +11272,47 @@
     </x:row>
     <x:row r="67" ht="28" customHeight="1">
       <x:c r="A67" s="8" t="s">
+        <x:v>789</x:v>
+      </x:c>
+      <x:c r="B67" s="7" t="s">
         <x:v>790</x:v>
       </x:c>
-      <x:c r="B67" s="7" t="s">
-        <x:v>791</x:v>
-      </x:c>
       <x:c r="C67" s="7" t="s">
-        <x:v>769</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="D67" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E67" s="10" t="s">
-        <x:v>792</x:v>
+        <x:v>791</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="28" customHeight="1">
       <x:c r="A68" s="8" t="s">
+        <x:v>792</x:v>
+      </x:c>
+      <x:c r="B68" s="7" t="s">
         <x:v>793</x:v>
       </x:c>
-      <x:c r="B68" s="7" t="s">
-        <x:v>794</x:v>
-      </x:c>
       <x:c r="C68" s="7" t="s">
-        <x:v>644</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="D68" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E68" s="10" t="s">
-        <x:v>795</x:v>
+        <x:v>794</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
       <x:c r="A69" s="8" t="s">
+        <x:v>795</x:v>
+      </x:c>
+      <x:c r="B69" s="7" t="s">
         <x:v>796</x:v>
       </x:c>
-      <x:c r="B69" s="7" t="s">
-        <x:v>797</x:v>
-      </x:c>
       <x:c r="C69" s="7" t="s">
-        <x:v>624</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="D69" s="9">
         <x:v>1</x:v>
@@ -11324,13 +11321,13 @@
     </x:row>
     <x:row r="70" ht="28" customHeight="1">
       <x:c r="A70" s="8" t="s">
+        <x:v>797</x:v>
+      </x:c>
+      <x:c r="B70" s="7" t="s">
         <x:v>798</x:v>
       </x:c>
-      <x:c r="B70" s="7" t="s">
-        <x:v>799</x:v>
-      </x:c>
       <x:c r="C70" s="7" t="s">
-        <x:v>652</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="D70" s="9">
         <x:v>1</x:v>
@@ -11339,13 +11336,13 @@
     </x:row>
     <x:row r="71" ht="28" customHeight="1">
       <x:c r="A71" s="8" t="s">
+        <x:v>799</x:v>
+      </x:c>
+      <x:c r="B71" s="7" t="s">
         <x:v>800</x:v>
       </x:c>
-      <x:c r="B71" s="7" t="s">
+      <x:c r="C71" s="7" t="s">
         <x:v>801</x:v>
-      </x:c>
-      <x:c r="C71" s="7" t="s">
-        <x:v>802</x:v>
       </x:c>
       <x:c r="D71" s="9">
         <x:v>1</x:v>
@@ -11354,64 +11351,64 @@
     </x:row>
     <x:row r="72" ht="28" customHeight="1">
       <x:c r="A72" s="8" t="s">
+        <x:v>802</x:v>
+      </x:c>
+      <x:c r="B72" s="7" t="s">
         <x:v>803</x:v>
       </x:c>
-      <x:c r="B72" s="7" t="s">
+      <x:c r="C72" s="7" t="s">
         <x:v>804</x:v>
-      </x:c>
-      <x:c r="C72" s="7" t="s">
-        <x:v>805</x:v>
       </x:c>
       <x:c r="D72" s="9">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E72" s="10" t="s">
-        <x:v>806</x:v>
+        <x:v>805</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="28" customHeight="1">
       <x:c r="A73" s="8" t="s">
+        <x:v>806</x:v>
+      </x:c>
+      <x:c r="B73" s="7" t="s">
         <x:v>807</x:v>
       </x:c>
-      <x:c r="B73" s="7" t="s">
+      <x:c r="C73" s="7" t="s">
         <x:v>808</x:v>
-      </x:c>
-      <x:c r="C73" s="7" t="s">
-        <x:v>809</x:v>
       </x:c>
       <x:c r="D73" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E73" s="10" t="s">
-        <x:v>810</x:v>
+        <x:v>809</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="28" customHeight="1">
       <x:c r="A74" s="8" t="s">
+        <x:v>810</x:v>
+      </x:c>
+      <x:c r="B74" s="7" t="s">
         <x:v>811</x:v>
       </x:c>
-      <x:c r="B74" s="7" t="s">
-        <x:v>812</x:v>
-      </x:c>
       <x:c r="C74" s="7" t="s">
-        <x:v>610</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="D74" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E74" s="10" t="s">
-        <x:v>813</x:v>
+        <x:v>812</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="28" customHeight="1">
       <x:c r="A75" s="8" t="s">
+        <x:v>813</x:v>
+      </x:c>
+      <x:c r="B75" s="7" t="s">
         <x:v>814</x:v>
       </x:c>
-      <x:c r="B75" s="7" t="s">
-        <x:v>815</x:v>
-      </x:c>
       <x:c r="C75" s="7" t="s">
-        <x:v>725</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="D75" s="9">
         <x:v>1</x:v>
@@ -11420,64 +11417,64 @@
     </x:row>
     <x:row r="76" ht="28" customHeight="1">
       <x:c r="A76" s="8" t="s">
+        <x:v>815</x:v>
+      </x:c>
+      <x:c r="B76" s="7" t="s">
         <x:v>816</x:v>
       </x:c>
-      <x:c r="B76" s="7" t="s">
-        <x:v>817</x:v>
-      </x:c>
       <x:c r="C76" s="7" t="s">
-        <x:v>694</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="D76" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E76" s="10" t="s">
-        <x:v>818</x:v>
+        <x:v>817</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
       <x:c r="A77" s="8" t="s">
+        <x:v>818</x:v>
+      </x:c>
+      <x:c r="B77" s="7" t="s">
         <x:v>819</x:v>
       </x:c>
-      <x:c r="B77" s="7" t="s">
-        <x:v>820</x:v>
-      </x:c>
       <x:c r="C77" s="7" t="s">
-        <x:v>802</x:v>
+        <x:v>801</x:v>
       </x:c>
       <x:c r="D77" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E77" s="10" t="s">
-        <x:v>821</x:v>
+        <x:v>820</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
       <x:c r="A78" s="8" t="s">
+        <x:v>821</x:v>
+      </x:c>
+      <x:c r="B78" s="7" t="s">
         <x:v>822</x:v>
       </x:c>
-      <x:c r="B78" s="7" t="s">
-        <x:v>823</x:v>
-      </x:c>
       <x:c r="C78" s="7" t="s">
-        <x:v>599</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="D78" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E78" s="10" t="s">
-        <x:v>824</x:v>
+        <x:v>823</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="28" customHeight="1">
       <x:c r="A79" s="8" t="s">
+        <x:v>824</x:v>
+      </x:c>
+      <x:c r="B79" s="7" t="s">
         <x:v>825</x:v>
       </x:c>
-      <x:c r="B79" s="7" t="s">
-        <x:v>826</x:v>
-      </x:c>
       <x:c r="C79" s="7" t="s">
-        <x:v>694</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="D79" s="9">
         <x:v>1</x:v>
@@ -11486,24 +11483,24 @@
     </x:row>
     <x:row r="80" ht="28" customHeight="1">
       <x:c r="A80" s="8" t="s">
+        <x:v>826</x:v>
+      </x:c>
+      <x:c r="B80" s="7" t="s">
         <x:v>827</x:v>
       </x:c>
-      <x:c r="B80" s="7" t="s">
+      <x:c r="C80" s="7" t="s">
         <x:v>828</x:v>
-      </x:c>
-      <x:c r="C80" s="7" t="s">
-        <x:v>829</x:v>
       </x:c>
       <x:c r="D80" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E80" s="10" t="s">
-        <x:v>830</x:v>
+        <x:v>829</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="28" customHeight="1">
       <x:c r="A81" s="8" t="s">
-        <x:v>831</x:v>
+        <x:v>830</x:v>
       </x:c>
       <x:c r="B81" s="7" t="s">
         <x:v>171</x:v>
@@ -11515,35 +11512,35 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="E81" s="10" t="s">
-        <x:v>832</x:v>
+        <x:v>831</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="28" customHeight="1">
       <x:c r="A82" s="8" t="s">
+        <x:v>832</x:v>
+      </x:c>
+      <x:c r="B82" s="7" t="s">
         <x:v>833</x:v>
       </x:c>
-      <x:c r="B82" s="7" t="s">
+      <x:c r="C82" s="7" t="s">
         <x:v>834</x:v>
-      </x:c>
-      <x:c r="C82" s="7" t="s">
-        <x:v>835</x:v>
       </x:c>
       <x:c r="D82" s="9">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E82" s="10" t="s">
-        <x:v>836</x:v>
+        <x:v>835</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="28" customHeight="1">
       <x:c r="A83" s="8" t="s">
+        <x:v>836</x:v>
+      </x:c>
+      <x:c r="B83" s="7" t="s">
         <x:v>837</x:v>
       </x:c>
-      <x:c r="B83" s="7" t="s">
-        <x:v>838</x:v>
-      </x:c>
       <x:c r="C83" s="7" t="s">
-        <x:v>617</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="D83" s="9">
         <x:v>1</x:v>
@@ -11552,13 +11549,13 @@
     </x:row>
     <x:row r="84" ht="28" customHeight="1">
       <x:c r="A84" s="8" t="s">
+        <x:v>838</x:v>
+      </x:c>
+      <x:c r="B84" s="7" t="s">
         <x:v>839</x:v>
       </x:c>
-      <x:c r="B84" s="7" t="s">
+      <x:c r="C84" s="7" t="s">
         <x:v>840</x:v>
-      </x:c>
-      <x:c r="C84" s="7" t="s">
-        <x:v>841</x:v>
       </x:c>
       <x:c r="D84" s="9">
         <x:v>1</x:v>
@@ -11567,64 +11564,64 @@
     </x:row>
     <x:row r="85" ht="28" customHeight="1">
       <x:c r="A85" s="8" t="s">
+        <x:v>841</x:v>
+      </x:c>
+      <x:c r="B85" s="7" t="s">
         <x:v>842</x:v>
       </x:c>
-      <x:c r="B85" s="7" t="s">
-        <x:v>843</x:v>
-      </x:c>
       <x:c r="C85" s="7" t="s">
-        <x:v>620</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="D85" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E85" s="10" t="s">
-        <x:v>844</x:v>
+        <x:v>843</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="28" customHeight="1">
       <x:c r="A86" s="8" t="s">
+        <x:v>844</x:v>
+      </x:c>
+      <x:c r="B86" s="7" t="s">
         <x:v>845</x:v>
       </x:c>
-      <x:c r="B86" s="7" t="s">
+      <x:c r="C86" s="7" t="s">
         <x:v>846</x:v>
-      </x:c>
-      <x:c r="C86" s="7" t="s">
-        <x:v>847</x:v>
       </x:c>
       <x:c r="D86" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E86" s="10" t="s">
-        <x:v>848</x:v>
+        <x:v>847</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="28" customHeight="1">
       <x:c r="A87" s="8" t="s">
+        <x:v>848</x:v>
+      </x:c>
+      <x:c r="B87" s="7" t="s">
         <x:v>849</x:v>
       </x:c>
-      <x:c r="B87" s="7" t="s">
+      <x:c r="C87" s="7" t="s">
         <x:v>850</x:v>
-      </x:c>
-      <x:c r="C87" s="7" t="s">
-        <x:v>851</x:v>
       </x:c>
       <x:c r="D87" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E87" s="10" t="s">
-        <x:v>852</x:v>
+        <x:v>851</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="28" customHeight="1">
       <x:c r="A88" s="8" t="s">
+        <x:v>852</x:v>
+      </x:c>
+      <x:c r="B88" s="7" t="s">
         <x:v>853</x:v>
       </x:c>
-      <x:c r="B88" s="7" t="s">
-        <x:v>854</x:v>
-      </x:c>
       <x:c r="C88" s="7" t="s">
-        <x:v>725</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="D88" s="9">
         <x:v>1</x:v>
@@ -11633,13 +11630,13 @@
     </x:row>
     <x:row r="89" ht="28" customHeight="1">
       <x:c r="A89" s="8" t="s">
+        <x:v>854</x:v>
+      </x:c>
+      <x:c r="B89" s="7" t="s">
         <x:v>855</x:v>
       </x:c>
-      <x:c r="B89" s="7" t="s">
-        <x:v>856</x:v>
-      </x:c>
       <x:c r="C89" s="7" t="s">
-        <x:v>641</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="D89" s="9">
         <x:v>1</x:v>
@@ -11648,30 +11645,30 @@
     </x:row>
     <x:row r="90" ht="28" customHeight="1">
       <x:c r="A90" s="8" t="s">
+        <x:v>856</x:v>
+      </x:c>
+      <x:c r="B90" s="7" t="s">
         <x:v>857</x:v>
       </x:c>
-      <x:c r="B90" s="7" t="s">
-        <x:v>858</x:v>
-      </x:c>
       <x:c r="C90" s="7" t="s">
-        <x:v>769</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="D90" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E90" s="10" t="s">
-        <x:v>859</x:v>
+        <x:v>858</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="28" customHeight="1">
       <x:c r="A91" s="8" t="s">
+        <x:v>859</x:v>
+      </x:c>
+      <x:c r="B91" s="7" t="s">
         <x:v>860</x:v>
       </x:c>
-      <x:c r="B91" s="7" t="s">
+      <x:c r="C91" s="7" t="s">
         <x:v>861</x:v>
-      </x:c>
-      <x:c r="C91" s="7" t="s">
-        <x:v>862</x:v>
       </x:c>
       <x:c r="D91" s="9">
         <x:v>1</x:v>
@@ -11680,30 +11677,30 @@
     </x:row>
     <x:row r="92" ht="28" customHeight="1">
       <x:c r="A92" s="8" t="s">
+        <x:v>862</x:v>
+      </x:c>
+      <x:c r="B92" s="7" t="s">
         <x:v>863</x:v>
       </x:c>
-      <x:c r="B92" s="7" t="s">
+      <x:c r="C92" s="7" t="s">
         <x:v>864</x:v>
-      </x:c>
-      <x:c r="C92" s="7" t="s">
-        <x:v>865</x:v>
       </x:c>
       <x:c r="D92" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E92" s="10" t="s">
-        <x:v>866</x:v>
+        <x:v>865</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="28" customHeight="1">
       <x:c r="A93" s="8" t="s">
+        <x:v>866</x:v>
+      </x:c>
+      <x:c r="B93" s="7" t="s">
         <x:v>867</x:v>
       </x:c>
-      <x:c r="B93" s="7" t="s">
-        <x:v>868</x:v>
-      </x:c>
       <x:c r="C93" s="7" t="s">
-        <x:v>802</x:v>
+        <x:v>801</x:v>
       </x:c>
       <x:c r="D93" s="9">
         <x:v>1</x:v>
@@ -11712,30 +11709,30 @@
     </x:row>
     <x:row r="94" ht="28" customHeight="1">
       <x:c r="A94" s="8" t="s">
+        <x:v>868</x:v>
+      </x:c>
+      <x:c r="B94" s="7" t="s">
         <x:v>869</x:v>
       </x:c>
-      <x:c r="B94" s="7" t="s">
-        <x:v>870</x:v>
-      </x:c>
       <x:c r="C94" s="7" t="s">
-        <x:v>694</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="D94" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E94" s="10" t="s">
-        <x:v>871</x:v>
+        <x:v>870</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="28" customHeight="1">
       <x:c r="A95" s="8" t="s">
+        <x:v>871</x:v>
+      </x:c>
+      <x:c r="B95" s="7" t="s">
         <x:v>872</x:v>
       </x:c>
-      <x:c r="B95" s="7" t="s">
-        <x:v>873</x:v>
-      </x:c>
       <x:c r="C95" s="7" t="s">
-        <x:v>691</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="D95" s="9">
         <x:v>1</x:v>
@@ -11744,47 +11741,47 @@
     </x:row>
     <x:row r="96" ht="28" customHeight="1">
       <x:c r="A96" s="8" t="s">
+        <x:v>873</x:v>
+      </x:c>
+      <x:c r="B96" s="7" t="s">
         <x:v>874</x:v>
       </x:c>
-      <x:c r="B96" s="7" t="s">
+      <x:c r="C96" s="7" t="s">
         <x:v>875</x:v>
-      </x:c>
-      <x:c r="C96" s="7" t="s">
-        <x:v>876</x:v>
       </x:c>
       <x:c r="D96" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E96" s="10" t="s">
-        <x:v>877</x:v>
+        <x:v>876</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="28" customHeight="1">
       <x:c r="A97" s="8" t="s">
+        <x:v>877</x:v>
+      </x:c>
+      <x:c r="B97" s="7" t="s">
         <x:v>878</x:v>
       </x:c>
-      <x:c r="B97" s="7" t="s">
-        <x:v>879</x:v>
-      </x:c>
       <x:c r="C97" s="7" t="s">
-        <x:v>841</x:v>
+        <x:v>840</x:v>
       </x:c>
       <x:c r="D97" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E97" s="10" t="s">
-        <x:v>880</x:v>
+        <x:v>879</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="s">
+        <x:v>880</x:v>
+      </x:c>
+      <x:c r="B98" t="s">
         <x:v>881</x:v>
       </x:c>
-      <x:c r="B98" t="s">
+      <x:c r="C98" t="s">
         <x:v>882</x:v>
-      </x:c>
-      <x:c r="C98" t="s">
-        <x:v>883</x:v>
       </x:c>
       <x:c r="D98">
         <x:v>1</x:v>
@@ -11805,12 +11802,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rc287ada2c6d74343"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R621c89396f344127"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rcfc0873f932848e4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rb077957764054966"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16e6b80f75fc4050"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae04fc2996b24789"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11825,7 +11822,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>884</x:v>
+        <x:v>883</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -12713,7 +12710,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c17cd1883c54546"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R108db55027824cf1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12729,27 +12726,27 @@
   <x:sheetData>
     <x:row r="1" ht="34.75" customHeight="1">
       <x:c r="A1" s="20" t="s">
-        <x:v>885</x:v>
+        <x:v>884</x:v>
       </x:c>
       <x:c r="B1" s="20"/>
       <x:c r="C1" s="20"/>
     </x:row>
     <x:row r="2" ht="45.25" customHeight="1">
       <x:c r="A2" s="21" t="s">
-        <x:v>886</x:v>
+        <x:v>885</x:v>
       </x:c>
       <x:c r="B2" s="21"/>
       <x:c r="C2" s="21"/>
     </x:row>
     <x:row r="4" ht="29.25" customHeight="1">
       <x:c r="A4" s="15" t="s">
+        <x:v>886</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="s">
         <x:v>887</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="s">
+      <x:c r="C4" s="15" t="s">
         <x:v>888</x:v>
-      </x:c>
-      <x:c r="C4" s="15" t="s">
-        <x:v>889</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.75" customHeight="1">
@@ -12757,7 +12754,7 @@
         <x:v>307</x:v>
       </x:c>
       <x:c r="B5" s="16" t="s">
-        <x:v>890</x:v>
+        <x:v>889</x:v>
       </x:c>
       <x:c r="C5" s="17"/>
     </x:row>
@@ -12766,7 +12763,7 @@
         <x:v>169</x:v>
       </x:c>
       <x:c r="B6" s="16" t="s">
-        <x:v>891</x:v>
+        <x:v>890</x:v>
       </x:c>
       <x:c r="C6" s="17"/>
     </x:row>
@@ -12775,7 +12772,7 @@
         <x:v>376</x:v>
       </x:c>
       <x:c r="B7" s="16" t="s">
-        <x:v>892</x:v>
+        <x:v>891</x:v>
       </x:c>
       <x:c r="C7" s="17"/>
     </x:row>
@@ -12784,7 +12781,7 @@
         <x:v>451</x:v>
       </x:c>
       <x:c r="B8" s="16" t="s">
-        <x:v>892</x:v>
+        <x:v>891</x:v>
       </x:c>
       <x:c r="C8" s="17"/>
     </x:row>
@@ -12793,7 +12790,7 @@
         <x:v>344</x:v>
       </x:c>
       <x:c r="B9" s="16" t="s">
-        <x:v>893</x:v>
+        <x:v>892</x:v>
       </x:c>
       <x:c r="C9" s="17"/>
     </x:row>
@@ -12802,27 +12799,27 @@
         <x:v>365</x:v>
       </x:c>
       <x:c r="B10" s="16" t="s">
+        <x:v>893</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="s">
         <x:v>894</x:v>
-      </x:c>
-      <x:c r="C10" s="17" t="s">
-        <x:v>895</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.75" customHeight="1">
       <x:c r="A11" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="B11" s="16" t="s">
-        <x:v>892</x:v>
+        <x:v>891</x:v>
       </x:c>
       <x:c r="C11" s="17"/>
     </x:row>
     <x:row r="12" ht="26.75" customHeight="1">
       <x:c r="A12" s="16" t="s">
+        <x:v>896</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="s">
         <x:v>897</x:v>
-      </x:c>
-      <x:c r="B12" s="16" t="s">
-        <x:v>898</x:v>
       </x:c>
       <x:c r="C12" s="17"/>
     </x:row>
@@ -12831,25 +12828,25 @@
         <x:v>300</x:v>
       </x:c>
       <x:c r="B13" s="16" t="s">
-        <x:v>891</x:v>
+        <x:v>890</x:v>
       </x:c>
       <x:c r="C13" s="17"/>
     </x:row>
     <x:row r="14" ht="26.75" customHeight="1">
       <x:c r="A14" s="16" t="s">
+        <x:v>898</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="s">
         <x:v>899</x:v>
-      </x:c>
-      <x:c r="B14" s="16" t="s">
-        <x:v>900</x:v>
       </x:c>
       <x:c r="C14" s="17"/>
     </x:row>
     <x:row r="15" ht="26.75" customHeight="1">
       <x:c r="A15" s="16" t="s">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="s">
         <x:v>901</x:v>
-      </x:c>
-      <x:c r="B15" s="16" t="s">
-        <x:v>902</x:v>
       </x:c>
       <x:c r="C15" s="17"/>
     </x:row>
@@ -12858,7 +12855,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B16" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C16" s="17"/>
     </x:row>
@@ -12867,7 +12864,7 @@
         <x:v>197</x:v>
       </x:c>
       <x:c r="B17" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C17" s="17"/>
     </x:row>
@@ -12876,7 +12873,7 @@
         <x:v>402</x:v>
       </x:c>
       <x:c r="B18" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C18" s="17"/>
     </x:row>
@@ -12885,25 +12882,25 @@
         <x:v>257</x:v>
       </x:c>
       <x:c r="B19" s="16" t="s">
-        <x:v>890</x:v>
+        <x:v>889</x:v>
       </x:c>
       <x:c r="C19" s="17"/>
     </x:row>
     <x:row r="20" ht="26.75" customHeight="1">
       <x:c r="A20" s="16" t="s">
-        <x:v>557</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="B20" s="16" t="s">
-        <x:v>902</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C20" s="17"/>
     </x:row>
     <x:row r="21" ht="26.75" customHeight="1">
       <x:c r="A21" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="B21" s="16" t="s">
-        <x:v>902</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C21" s="17"/>
     </x:row>
@@ -12912,25 +12909,25 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="B22" s="16" t="s">
-        <x:v>902</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C22" s="17"/>
     </x:row>
     <x:row r="23" ht="26.75" customHeight="1">
       <x:c r="A23" s="16" t="s">
+        <x:v>904</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="s">
         <x:v>905</x:v>
-      </x:c>
-      <x:c r="B23" s="16" t="s">
-        <x:v>906</x:v>
       </x:c>
       <x:c r="C23" s="17"/>
     </x:row>
     <x:row r="24" ht="26.75" customHeight="1">
       <x:c r="A24" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="B24" s="16" t="s">
-        <x:v>890</x:v>
+        <x:v>889</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
     </x:row>
@@ -12939,36 +12936,36 @@
         <x:v>322</x:v>
       </x:c>
       <x:c r="B25" s="16" t="s">
-        <x:v>891</x:v>
+        <x:v>890</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
     </x:row>
     <x:row r="26" ht="26.75" customHeight="1">
       <x:c r="A26" s="16" t="s">
-        <x:v>461</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="B26" s="16" t="s">
-        <x:v>891</x:v>
+        <x:v>890</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
     </x:row>
     <x:row r="27" ht="26.75" customHeight="1">
       <x:c r="A27" s="16" t="s">
-        <x:v>550</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="B27" s="16" t="s">
-        <x:v>894</x:v>
+        <x:v>893</x:v>
       </x:c>
       <x:c r="C27" s="17" t="s">
-        <x:v>908</x:v>
+        <x:v>907</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="26.75" customHeight="1">
       <x:c r="A28" s="16" t="s">
-        <x:v>909</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="B28" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C28" s="17"/>
     </x:row>
@@ -12977,7 +12974,7 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B29" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C29" s="17"/>
     </x:row>
@@ -12986,7 +12983,7 @@
         <x:v>190</x:v>
       </x:c>
       <x:c r="B30" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C30" s="17"/>
     </x:row>
@@ -12995,25 +12992,25 @@
         <x:v>140</x:v>
       </x:c>
       <x:c r="B31" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C31" s="17"/>
     </x:row>
     <x:row r="32" ht="26.75" customHeight="1">
       <x:c r="A32" s="16" t="s">
-        <x:v>545</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="B32" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C32" s="17"/>
     </x:row>
     <x:row r="33" ht="26.75" customHeight="1">
       <x:c r="A33" s="16" t="s">
-        <x:v>910</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="B33" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C33" s="17"/>
     </x:row>
@@ -13022,16 +13019,16 @@
         <x:v>315</x:v>
       </x:c>
       <x:c r="B34" s="16" t="s">
-        <x:v>892</x:v>
+        <x:v>891</x:v>
       </x:c>
       <x:c r="C34" s="17"/>
     </x:row>
     <x:row r="35" ht="26.75" customHeight="1">
       <x:c r="A35" s="16" t="s">
-        <x:v>501</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="B35" s="16" t="s">
-        <x:v>891</x:v>
+        <x:v>890</x:v>
       </x:c>
       <x:c r="C35" s="17"/>
     </x:row>
@@ -13040,18 +13037,18 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B36" s="16" t="s">
+        <x:v>893</x:v>
+      </x:c>
+      <x:c r="C36" s="17" t="s">
         <x:v>894</x:v>
-      </x:c>
-      <x:c r="C36" s="17" t="s">
-        <x:v>895</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="26.75" customHeight="1">
       <x:c r="A37" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="B37" s="16" t="s">
-        <x:v>903</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="C37" s="17"/>
     </x:row>
@@ -13060,7 +13057,7 @@
         <x:v>176</x:v>
       </x:c>
       <x:c r="B38" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C38" s="17"/>
     </x:row>
@@ -13069,10 +13066,10 @@
         <x:v>238</x:v>
       </x:c>
       <x:c r="B39" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C39" s="17" t="s">
-        <x:v>912</x:v>
+        <x:v>911</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="26.75" customHeight="1">
@@ -13080,25 +13077,25 @@
         <x:v>441</x:v>
       </x:c>
       <x:c r="B40" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C40" s="17"/>
     </x:row>
     <x:row r="41" ht="26.75" customHeight="1">
       <x:c r="A41" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>912</x:v>
       </x:c>
       <x:c r="B41" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C41" s="17"/>
     </x:row>
     <x:row r="42" ht="26.75" customHeight="1">
       <x:c r="A42" s="16" t="s">
-        <x:v>914</x:v>
+        <x:v>913</x:v>
       </x:c>
       <x:c r="B42" s="16" t="s">
-        <x:v>902</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="C42" s="17"/>
     </x:row>
@@ -13107,10 +13104,10 @@
         <x:v>223</x:v>
       </x:c>
       <x:c r="B43" s="16" t="s">
+        <x:v>893</x:v>
+      </x:c>
+      <x:c r="C43" s="17" t="s">
         <x:v>894</x:v>
-      </x:c>
-      <x:c r="C43" s="17" t="s">
-        <x:v>895</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="26.75" customHeight="1">
@@ -13118,7 +13115,7 @@
         <x:v>181</x:v>
       </x:c>
       <x:c r="B44" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C44" s="17"/>
     </x:row>
@@ -13127,16 +13124,16 @@
         <x:v>161</x:v>
       </x:c>
       <x:c r="B45" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C45" s="17"/>
     </x:row>
     <x:row r="46" ht="26.75" customHeight="1">
       <x:c r="A46" s="16" t="s">
-        <x:v>915</x:v>
+        <x:v>914</x:v>
       </x:c>
       <x:c r="B46" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C46" s="17"/>
     </x:row>
@@ -13145,19 +13142,19 @@
         <x:v>155</x:v>
       </x:c>
       <x:c r="B47" s="16" t="s">
-        <x:v>893</x:v>
+        <x:v>892</x:v>
       </x:c>
       <x:c r="C47" s="17"/>
     </x:row>
     <x:row r="48" ht="26.75" customHeight="1">
       <x:c r="A48" s="16" t="s">
+        <x:v>915</x:v>
+      </x:c>
+      <x:c r="B48" s="16" t="s">
+        <x:v>893</x:v>
+      </x:c>
+      <x:c r="C48" s="17" t="s">
         <x:v>916</x:v>
-      </x:c>
-      <x:c r="B48" s="16" t="s">
-        <x:v>894</x:v>
-      </x:c>
-      <x:c r="C48" s="17" t="s">
-        <x:v>917</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="26.75" customHeight="1">
@@ -13165,7 +13162,7 @@
         <x:v>283</x:v>
       </x:c>
       <x:c r="B49" s="16" t="s">
-        <x:v>893</x:v>
+        <x:v>892</x:v>
       </x:c>
       <x:c r="C49" s="17"/>
     </x:row>
@@ -13174,16 +13171,16 @@
         <x:v>211</x:v>
       </x:c>
       <x:c r="B50" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C50" s="17"/>
     </x:row>
     <x:row r="51" ht="26.75" customHeight="1">
       <x:c r="A51" s="16" t="s">
-        <x:v>918</x:v>
+        <x:v>917</x:v>
       </x:c>
       <x:c r="B51" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C51" s="17"/>
     </x:row>
@@ -13192,38 +13189,38 @@
         <x:v>231</x:v>
       </x:c>
       <x:c r="B52" s="16" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="C52" s="17"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" t="s">
-        <x:v>567</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="B53" t="s">
         <x:v>376</x:v>
       </x:c>
       <x:c r="C53" t="s">
-        <x:v>919</x:v>
+        <x:v>918</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" t="s">
-        <x:v>576</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="B54" t="s">
-        <x:v>894</x:v>
+        <x:v>893</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" t="s">
-        <x:v>583</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="B55" t="s">
-        <x:v>892</x:v>
+        <x:v>891</x:v>
       </x:c>
       <x:c r="C55" t="s">
-        <x:v>920</x:v>
+        <x:v>919</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -15177,11 +15174,11 @@
       </x:c>
       <x:c r="C24" s="36" t="str">
         <x:f>Hackathons!AG62</x:f>
-        <x:v>Award — v0 Sock</x:v>
+        <x:v>2nd Place — v0 Sock</x:v>
       </x:c>
       <x:c r="D24" s="36" t="str">
         <x:f>IF(Hackathons!Q62="","",Hackathons!Q62)</x:f>
-        <x:v>Award</x:v>
+        <x:v>2nd Place</x:v>
       </x:c>
       <x:c r="E24" s="36" t="str">
         <x:f>IF(Hackathons!R62="","",Hackathons!R62)</x:f>
@@ -15617,7 +15614,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bc88217540d4795"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7a2ccdcf6574118"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine Cybrdeck award classification
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Reb7c7f89b5ec4bec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R49c3aba8b997425e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rc381810b42d94889"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R4d932ad07d554cea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="Re20ea37a4651423a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R8767c55da7a94890"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rb3e60a5ecbc34a7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rb69e45b2ba3d49b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R90438e500e9642a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R41b370a5656f41eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R7d8de5dfec2445bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Rc70b2f0ba1d84632"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9722,10 +9722,10 @@
         <x:v>562</x:v>
       </x:c>
       <x:c r="Q76" s="36" t="str">
-        <x:v>Best Vertical Solution</x:v>
+        <x:v>Best Project</x:v>
       </x:c>
       <x:c r="R76" s="36" t="str">
-        <x:v>Family Office Track</x:v>
+        <x:v>Best Vertical Solution: Family Office Track</x:v>
       </x:c>
       <x:c r="S76" s="37"/>
       <x:c r="T76" s="38"/>
@@ -9752,7 +9752,7 @@
         <x:v>US$25 credit value, not cash</x:v>
       </x:c>
       <x:c r="AG76" s="198" t="str">
-        <x:v>Best Vertical Solution — Family Office Track — 2,000 Cybrdeck API Credits (US$25 value)</x:v>
+        <x:v>Best Project — Best Vertical Solution: Family Office Track — 2,000 Cybrdeck API Credits (US$25 value)</x:v>
       </x:c>
       <x:c r="AH76" s="214" t="n">
         <x:f>IF(OR(J76="",J76="-"),"",LEN(J76)-LEN(SUBSTITUTE(J76,",",""))+1)</x:f>
@@ -10221,10 +10221,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R111a9b89060e430b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R62b5d75a144c4094"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Ra85ea0efba7b4665"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R09c9760ce8c24615"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R294db252d6914d32"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rd9cfaca261464761"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R6e4f983f59c04bfe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R45bca739c0314aa9"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11802,12 +11802,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rcfc0873f932848e4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rb077957764054966"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rfe43c39c2c2d4bc1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R8fcf8fb536bf41eb"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae04fc2996b24789"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0eb14a03b8d24582"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12710,7 +12710,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R108db55027824cf1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29a0808ee0b04ee7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15391,15 +15391,15 @@
       </x:c>
       <x:c r="C27" s="36" t="str">
         <x:f>Hackathons!AG76</x:f>
-        <x:v>Best Vertical Solution — Family Office Track — 2,000 Cybrdeck API Credits (US$25 value)</x:v>
+        <x:v>Best Project — Best Vertical Solution: Family Office Track — 2,000 Cybrdeck API Credits (US$25 value)</x:v>
       </x:c>
       <x:c r="D27" s="36" t="str">
         <x:f>IF(Hackathons!Q76="","",Hackathons!Q76)</x:f>
-        <x:v>Best Vertical Solution</x:v>
+        <x:v>Best Project</x:v>
       </x:c>
       <x:c r="E27" s="36" t="str">
         <x:f>IF(Hackathons!R76="","",Hackathons!R76)</x:f>
-        <x:v>Family Office Track</x:v>
+        <x:v>Best Vertical Solution: Family Office Track</x:v>
       </x:c>
       <x:c r="F27" s="97" t="str">
         <x:f>IF(Hackathons!S76="","",Hackathons!S76)</x:f>
@@ -15614,7 +15614,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7a2ccdcf6574118"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8231751892dd413c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct OPC hackathon placement
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rb3e60a5ecbc34a7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rb69e45b2ba3d49b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R90438e500e9642a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R41b370a5656f41eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R7d8de5dfec2445bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Rc70b2f0ba1d84632"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R20070750e37641d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rfec7f73e50b74be6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rbc5b98e953784fdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Rf690bc358ab24e3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R5820836089804009"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R0d9135182df14e07"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9392,7 +9392,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="G72" t="str">
-        <x:v>4.5K USD AWS Credits</x:v>
+        <x:v>Top 30 — US$4,500 AWS Credits</x:v>
       </x:c>
       <x:c r="H72" t="s">
         <x:v>238</x:v>
@@ -9422,7 +9422,7 @@
         <x:v>533</x:v>
       </x:c>
       <x:c r="Q72" s="36" t="str">
-        <x:v>Award</x:v>
+        <x:v>Top 30</x:v>
       </x:c>
       <x:c r="R72" s="36" t="str">
         <x:v>AWS</x:v>
@@ -9452,7 +9452,7 @@
         <x:v>USD-denominated credit value</x:v>
       </x:c>
       <x:c r="AG72" s="198" t="str">
-        <x:v>Award — US$4,500 AWS Credits</x:v>
+        <x:v>Top 30 — US$4,500 AWS Credits</x:v>
       </x:c>
       <x:c r="AH72" s="214" t="n">
         <x:f>IF(OR(J72="",J72="-"),"",LEN(J72)-LEN(SUBSTITUTE(J72,",",""))+1)</x:f>
@@ -10221,10 +10221,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R294db252d6914d32"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rd9cfaca261464761"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R6e4f983f59c04bfe"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R45bca739c0314aa9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Reea0356431dc41ee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R2526a6dfb8864afa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R31fe950834af401f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R3714db3a8ab24ef2"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11802,12 +11802,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rfe43c39c2c2d4bc1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R8fcf8fb536bf41eb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rc5add2e560e0445f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rbf49321d279b413c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0eb14a03b8d24582"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88c73f0343b54581"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12710,7 +12710,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29a0808ee0b04ee7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5aa252af49a645bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15318,11 +15318,11 @@
       </x:c>
       <x:c r="C26" s="36" t="str">
         <x:f>Hackathons!AG72</x:f>
-        <x:v>Award — US$4,500 AWS Credits</x:v>
+        <x:v>Top 30 — US$4,500 AWS Credits</x:v>
       </x:c>
       <x:c r="D26" s="36" t="str">
         <x:f>IF(Hackathons!Q72="","",Hackathons!Q72)</x:f>
-        <x:v>Award</x:v>
+        <x:v>Top 30</x:v>
       </x:c>
       <x:c r="E26" s="36" t="str">
         <x:f>IF(Hackathons!R72="","",Hackathons!R72)</x:f>
@@ -15614,7 +15614,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8231751892dd413c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R577881baf8f648ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine OPC and v0 award details
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rde0204323ae24e5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R71b5db9b247b4eb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R929fa21c3c7344a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R1e08a9633c6545e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R469fd6b52b6f4f8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Rdde87037e5cb4c6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R97cdd5c1e2044ad2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R5924662540ba40e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rd11ea0fa921b49a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Rb87d26190eae4e42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R3935d5d2783a42ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Rc678e916a0be4ef0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8678,7 +8678,7 @@
         <x:v>2nd Place</x:v>
       </x:c>
       <x:c r="R62" s="36" t="str">
-        <x:v>v0</x:v>
+        <x:v>v0 Sock</x:v>
       </x:c>
       <x:c r="S62" s="37"/>
       <x:c r="T62" s="38"/>
@@ -9414,9 +9414,7 @@
       <x:c r="Q72" s="36" t="str">
         <x:v>Top 30</x:v>
       </x:c>
-      <x:c r="R72" s="36" t="str">
-        <x:v>AWS</x:v>
-      </x:c>
+      <x:c r="R72" s="36"/>
       <x:c r="S72" s="37"/>
       <x:c r="T72" s="38"/>
       <x:c r="U72" s="37" t="n">
@@ -10211,10 +10209,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R158cedbdecf84b5b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R29da643633314cc8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R2587b3c26819437f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Rfb2140dc362a4116"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Raf0a946ee9524174"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R1cded7850b394676"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R5ded13067fd74a8e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R889ae99d32864598"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11792,12 +11790,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R79a7dc89000c49dd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R31f5a32fb27047de"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R5bec9333787d4df6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rf81095442d264c4b"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba4ede9654844f66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb88409eab1724c5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12700,7 +12698,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32137dba24ab4672"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6aa975881dfa40c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15103,7 +15101,7 @@
       </x:c>
       <x:c r="E23" s="36" t="str">
         <x:f>IF(Hackathons!R62="","",Hackathons!R62)</x:f>
-        <x:v>v0</x:v>
+        <x:v>v0 Sock</x:v>
       </x:c>
       <x:c r="F23" s="40" t="str">
         <x:f>IF(Hackathons!S62="","",Hackathons!S62)</x:f>
@@ -15247,7 +15245,6 @@
       </x:c>
       <x:c r="E25" s="36" t="str">
         <x:f>IF(Hackathons!R72="","",Hackathons!R72)</x:f>
-        <x:v>AWS</x:v>
       </x:c>
       <x:c r="F25" s="40" t="str">
         <x:f>IF(Hackathons!S72="","",Hackathons!S72)</x:f>
@@ -15557,7 +15554,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19f589c379564aee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8efb733ad37d42d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Rename Novel Hackathon finisher award
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R97cdd5c1e2044ad2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R5924662540ba40e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rd11ea0fa921b49a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Rb87d26190eae4e42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R3935d5d2783a42ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Rc678e916a0be4ef0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rc03a9f42bf804886"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rc940440fb3034e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R1e05a5bea69e488d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R6545c99eb3794940"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R25dd41e50fdf4ecd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Re2e051c4937e4720"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -907,9 +907,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Sep 6, 2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Throphy, Best Novel Hackathon Finisher</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Design</x:t>
@@ -7039,27 +7036,27 @@
       <x:c r="F41" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="G41" t="s">
+      <x:c r="G41" t="str">
+        <x:v>Novel Hackathon Finisher — Trophy</x:v>
+      </x:c>
+      <x:c r="H41" t="s">
         <x:v>298</x:v>
       </x:c>
-      <x:c r="H41" t="s">
+      <x:c r="J41" t="s">
         <x:v>299</x:v>
       </x:c>
-      <x:c r="J41" t="s">
+      <x:c r="K41" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="L41" t="s">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="K41" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="L41" t="s">
+      <x:c r="M41" t="s">
         <x:v>301</x:v>
       </x:c>
-      <x:c r="M41" t="s">
+      <x:c r="N41" t="s">
         <x:v>302</x:v>
       </x:c>
-      <x:c r="N41" t="s">
-        <x:v>303</x:v>
-      </x:c>
       <x:c r="O41" t="s">
         <x:v>25</x:v>
       </x:c>
@@ -7067,11 +7064,9 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="Q41" s="36" t="str">
-        <x:v>Best Finisher</x:v>
-      </x:c>
-      <x:c r="R41" s="36" t="str">
-        <x:v>Novel Hackathon</x:v>
-      </x:c>
+        <x:v>Novel Hackathon Finisher</x:v>
+      </x:c>
+      <x:c r="R41" s="36"/>
       <x:c r="S41" s="37"/>
       <x:c r="T41" s="38"/>
       <x:c r="U41" s="37"/>
@@ -7097,7 +7092,7 @@
         <x:v>Trophy, not cash</x:v>
       </x:c>
       <x:c r="AG41" s="198" t="str">
-        <x:v>Best Finisher — Novel Hackathon — Trophy</x:v>
+        <x:v>Novel Hackathon Finisher — Trophy</x:v>
       </x:c>
       <x:c r="AH41" s="214" t="n">
         <x:f>IF(OR(J41="",J41="-"),"",LEN(J41)-LEN(SUBSTITUTE(J41,",",""))+1)</x:f>
@@ -7109,10 +7104,10 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B42" t="s">
+        <x:v>303</x:v>
+      </x:c>
+      <x:c r="C42" t="s">
         <x:v>304</x:v>
-      </x:c>
-      <x:c r="C42" t="s">
-        <x:v>305</x:v>
       </x:c>
       <x:c r="D42" s="4">
         <x:v>45920</x:v>
@@ -7127,13 +7122,13 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H42" t="s">
+        <x:v>305</x:v>
+      </x:c>
+      <x:c r="I42" t="s">
         <x:v>306</x:v>
       </x:c>
-      <x:c r="I42" t="s">
+      <x:c r="J42" t="s">
         <x:v>307</x:v>
-      </x:c>
-      <x:c r="J42" t="s">
-        <x:v>308</x:v>
       </x:c>
       <x:c r="K42" t="s">
         <x:v>25</x:v>
@@ -7142,10 +7137,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N42" t="s">
+        <x:v>308</x:v>
+      </x:c>
+      <x:c r="O42" t="s">
         <x:v>309</x:v>
-      </x:c>
-      <x:c r="O42" t="s">
-        <x:v>310</x:v>
       </x:c>
       <x:c r="P42" t="s">
         <x:v>25</x:v>
@@ -7177,10 +7172,10 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="B43" t="s">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="C43" t="s">
         <x:v>311</x:v>
-      </x:c>
-      <x:c r="C43" t="s">
-        <x:v>312</x:v>
       </x:c>
       <x:c r="D43" s="4">
         <x:v>45930</x:v>
@@ -7192,31 +7187,31 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="G43" t="s">
+        <x:v>312</x:v>
+      </x:c>
+      <x:c r="H43" t="s">
         <x:v>313</x:v>
       </x:c>
-      <x:c r="H43" t="s">
+      <x:c r="I43" t="s">
         <x:v>314</x:v>
       </x:c>
-      <x:c r="I43" t="s">
+      <x:c r="J43" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K43" t="s">
         <x:v>315</x:v>
       </x:c>
-      <x:c r="J43" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K43" t="s">
-        <x:v>316</x:v>
-      </x:c>
       <x:c r="L43" t="s">
-        <x:v>312</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="M43" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N43" t="s">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="O43" t="s">
         <x:v>317</x:v>
-      </x:c>
-      <x:c r="O43" t="s">
-        <x:v>318</x:v>
       </x:c>
       <x:c r="P43" t="s">
         <x:v>25</x:v>
@@ -7262,10 +7257,10 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B44" t="s">
+        <x:v>318</x:v>
+      </x:c>
+      <x:c r="C44" t="s">
         <x:v>319</x:v>
-      </x:c>
-      <x:c r="C44" t="s">
-        <x:v>320</x:v>
       </x:c>
       <x:c r="D44" s="5">
         <x:v>45932</x:v>
@@ -7280,16 +7275,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H44" t="s">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="I44" t="s">
         <x:v>321</x:v>
       </x:c>
-      <x:c r="I44" t="s">
+      <x:c r="J44" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K44" t="s">
         <x:v>322</x:v>
-      </x:c>
-      <x:c r="J44" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K44" t="s">
-        <x:v>323</x:v>
       </x:c>
       <x:c r="L44" t="s">
         <x:v>25</x:v>
@@ -7333,13 +7328,13 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B45" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="C45" t="s">
         <x:v>324</x:v>
       </x:c>
-      <x:c r="C45" t="s">
+      <x:c r="D45" s="2" t="s">
         <x:v>325</x:v>
-      </x:c>
-      <x:c r="D45" s="2" t="s">
-        <x:v>326</x:v>
       </x:c>
       <x:c r="E45">
         <x:v>2</x:v>
@@ -7354,16 +7349,16 @@
         <x:v>264</x:v>
       </x:c>
       <x:c r="I45" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="J45" t="s">
         <x:v>327</x:v>
       </x:c>
-      <x:c r="J45" t="s">
+      <x:c r="K45" t="s">
         <x:v>328</x:v>
       </x:c>
-      <x:c r="K45" t="s">
+      <x:c r="L45" t="s">
         <x:v>329</x:v>
-      </x:c>
-      <x:c r="L45" t="s">
-        <x:v>330</x:v>
       </x:c>
       <x:c r="M45" t="s">
         <x:v>26</x:v>
@@ -7372,7 +7367,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="O45" t="s">
-        <x:v>331</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="P45" t="s">
         <x:v>25</x:v>
@@ -7404,10 +7399,10 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="B46" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="C46" t="s">
         <x:v>332</x:v>
-      </x:c>
-      <x:c r="C46" t="s">
-        <x:v>333</x:v>
       </x:c>
       <x:c r="D46" s="5">
         <x:v>45954</x:v>
@@ -7425,25 +7420,25 @@
         <x:v>264</x:v>
       </x:c>
       <x:c r="I46" t="s">
+        <x:v>333</x:v>
+      </x:c>
+      <x:c r="J46" t="s">
         <x:v>334</x:v>
       </x:c>
-      <x:c r="J46" t="s">
+      <x:c r="K46" t="s">
         <x:v>335</x:v>
       </x:c>
-      <x:c r="K46" t="s">
+      <x:c r="L46" t="s">
         <x:v>336</x:v>
-      </x:c>
-      <x:c r="L46" t="s">
-        <x:v>337</x:v>
       </x:c>
       <x:c r="M46" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N46" t="s">
+        <x:v>337</x:v>
+      </x:c>
+      <x:c r="O46" t="s">
         <x:v>338</x:v>
-      </x:c>
-      <x:c r="O46" t="s">
-        <x:v>339</x:v>
       </x:c>
       <x:c r="P46" t="s">
         <x:v>25</x:v>
@@ -7475,13 +7470,13 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="B47" t="s">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="C47" t="s">
         <x:v>340</x:v>
       </x:c>
-      <x:c r="C47" t="s">
+      <x:c r="D47" s="5" t="s">
         <x:v>341</x:v>
-      </x:c>
-      <x:c r="D47" s="5" t="s">
-        <x:v>342</x:v>
       </x:c>
       <x:c r="E47">
         <x:v>2.5</x:v>
@@ -7493,28 +7488,28 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H47" t="s">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="I47" t="s">
         <x:v>343</x:v>
       </x:c>
-      <x:c r="I47" t="s">
+      <x:c r="J47" t="s">
         <x:v>344</x:v>
       </x:c>
-      <x:c r="J47" t="s">
+      <x:c r="K47" t="s">
         <x:v>345</x:v>
       </x:c>
-      <x:c r="K47" t="s">
+      <x:c r="L47" t="s">
         <x:v>346</x:v>
-      </x:c>
-      <x:c r="L47" t="s">
-        <x:v>347</x:v>
       </x:c>
       <x:c r="M47" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N47" t="s">
+        <x:v>347</x:v>
+      </x:c>
+      <x:c r="O47" t="s">
         <x:v>348</x:v>
-      </x:c>
-      <x:c r="O47" t="s">
-        <x:v>349</x:v>
       </x:c>
       <x:c r="P47" t="s">
         <x:v>25</x:v>
@@ -7546,13 +7541,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="B48" t="s">
+        <x:v>349</x:v>
+      </x:c>
+      <x:c r="C48" t="s">
         <x:v>350</x:v>
       </x:c>
-      <x:c r="C48" t="s">
+      <x:c r="D48" s="2" t="s">
         <x:v>351</x:v>
-      </x:c>
-      <x:c r="D48" s="2" t="s">
-        <x:v>352</x:v>
       </x:c>
       <x:c r="E48">
         <x:v>2</x:v>
@@ -7567,25 +7562,25 @@
         <x:v>264</x:v>
       </x:c>
       <x:c r="I48" t="s">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="J48" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K48" t="s">
         <x:v>353</x:v>
       </x:c>
-      <x:c r="J48" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K48" t="s">
-        <x:v>354</x:v>
-      </x:c>
       <x:c r="L48" t="s">
-        <x:v>351</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="M48" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N48" t="s">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="O48" t="s">
         <x:v>355</x:v>
-      </x:c>
-      <x:c r="O48" t="s">
-        <x:v>356</x:v>
       </x:c>
       <x:c r="P48" t="s">
         <x:v>25</x:v>
@@ -7617,13 +7612,13 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B49" t="s">
+        <x:v>349</x:v>
+      </x:c>
+      <x:c r="C49" t="s">
         <x:v>350</x:v>
       </x:c>
-      <x:c r="C49" t="s">
+      <x:c r="D49" s="2" t="s">
         <x:v>351</x:v>
-      </x:c>
-      <x:c r="D49" s="2" t="s">
-        <x:v>352</x:v>
       </x:c>
       <x:c r="E49">
         <x:v>2</x:v>
@@ -7638,25 +7633,25 @@
         <x:v>264</x:v>
       </x:c>
       <x:c r="I49" t="s">
+        <x:v>356</x:v>
+      </x:c>
+      <x:c r="J49" t="s">
         <x:v>357</x:v>
       </x:c>
-      <x:c r="J49" t="s">
+      <x:c r="K49" t="s">
         <x:v>358</x:v>
       </x:c>
-      <x:c r="K49" t="s">
-        <x:v>359</x:v>
-      </x:c>
       <x:c r="L49" t="s">
-        <x:v>351</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="M49" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N49" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="O49" t="s">
-        <x:v>360</x:v>
+        <x:v>359</x:v>
       </x:c>
       <x:c r="P49" t="s">
         <x:v>25</x:v>
@@ -7688,13 +7683,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B50" t="s">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="C50" t="s">
         <x:v>361</x:v>
       </x:c>
-      <x:c r="C50" t="s">
+      <x:c r="D50" s="3" t="s">
         <x:v>362</x:v>
-      </x:c>
-      <x:c r="D50" s="3" t="s">
-        <x:v>363</x:v>
       </x:c>
       <x:c r="E50">
         <x:v>1</x:v>
@@ -7706,31 +7701,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H50" t="s">
+        <x:v>363</x:v>
+      </x:c>
+      <x:c r="I50" t="s">
         <x:v>364</x:v>
       </x:c>
-      <x:c r="I50" t="s">
+      <x:c r="J50" t="s">
         <x:v>365</x:v>
       </x:c>
-      <x:c r="J50" t="s">
+      <x:c r="K50" t="s">
         <x:v>366</x:v>
       </x:c>
-      <x:c r="K50" t="s">
+      <x:c r="L50" s="6" t="s">
         <x:v>367</x:v>
-      </x:c>
-      <x:c r="L50" s="6" t="s">
-        <x:v>368</x:v>
       </x:c>
       <x:c r="M50" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N50" t="s">
+        <x:v>368</x:v>
+      </x:c>
+      <x:c r="O50" t="s">
         <x:v>369</x:v>
       </x:c>
-      <x:c r="O50" t="s">
+      <x:c r="P50" t="s">
         <x:v>370</x:v>
-      </x:c>
-      <x:c r="P50" t="s">
-        <x:v>371</x:v>
       </x:c>
       <x:c r="Q50" s="36"/>
       <x:c r="R50" s="36"/>
@@ -7759,10 +7754,10 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="B51" t="s">
+        <x:v>371</x:v>
+      </x:c>
+      <x:c r="C51" t="s">
         <x:v>372</x:v>
-      </x:c>
-      <x:c r="C51" t="s">
-        <x:v>373</x:v>
       </x:c>
       <x:c r="D51" s="5">
         <x:v>46205</x:v>
@@ -7774,34 +7769,34 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="G51" t="s">
+        <x:v>373</x:v>
+      </x:c>
+      <x:c r="H51" t="s">
         <x:v>374</x:v>
       </x:c>
-      <x:c r="H51" t="s">
+      <x:c r="I51" t="s">
         <x:v>375</x:v>
       </x:c>
-      <x:c r="I51" t="s">
+      <x:c r="J51" t="s">
         <x:v>376</x:v>
       </x:c>
-      <x:c r="J51" t="s">
+      <x:c r="K51" t="s">
         <x:v>377</x:v>
       </x:c>
-      <x:c r="K51" t="s">
+      <x:c r="L51" t="s">
         <x:v>378</x:v>
-      </x:c>
-      <x:c r="L51" t="s">
-        <x:v>379</x:v>
       </x:c>
       <x:c r="M51" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N51" t="s">
-        <x:v>317</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="O51" t="s">
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="P51" t="s">
         <x:v>380</x:v>
-      </x:c>
-      <x:c r="P51" t="s">
-        <x:v>381</x:v>
       </x:c>
       <x:c r="Q51" s="36" t="str">
         <x:v>1st Prize</x:v>
@@ -7844,10 +7839,10 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="B52" t="s">
+        <x:v>371</x:v>
+      </x:c>
+      <x:c r="C52" t="s">
         <x:v>372</x:v>
-      </x:c>
-      <x:c r="C52" t="s">
-        <x:v>373</x:v>
       </x:c>
       <x:c r="D52" s="5">
         <x:v>46205</x:v>
@@ -7862,31 +7857,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H52" t="s">
-        <x:v>375</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="I52" t="s">
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="J52" t="s">
+        <x:v>376</x:v>
+      </x:c>
+      <x:c r="K52" t="s">
         <x:v>382</x:v>
       </x:c>
-      <x:c r="J52" t="s">
-        <x:v>377</x:v>
-      </x:c>
-      <x:c r="K52" t="s">
-        <x:v>383</x:v>
-      </x:c>
       <x:c r="L52" t="s">
-        <x:v>379</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="M52" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N52" t="s">
-        <x:v>317</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="O52" t="s">
-        <x:v>384</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="P52" t="s">
-        <x:v>381</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="Q52" s="36"/>
       <x:c r="R52" s="36"/>
@@ -7915,13 +7910,13 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="B53" t="s">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="C53" t="s">
+        <x:v>372</x:v>
+      </x:c>
+      <x:c r="D53" s="2" t="s">
         <x:v>385</x:v>
-      </x:c>
-      <x:c r="C53" t="s">
-        <x:v>373</x:v>
-      </x:c>
-      <x:c r="D53" s="2" t="s">
-        <x:v>386</x:v>
       </x:c>
       <x:c r="E53">
         <x:v>1</x:v>
@@ -7930,22 +7925,22 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="G53" t="s">
+        <x:v>386</x:v>
+      </x:c>
+      <x:c r="H53" t="s">
+        <x:v>374</x:v>
+      </x:c>
+      <x:c r="I53" t="s">
         <x:v>387</x:v>
       </x:c>
-      <x:c r="H53" t="s">
-        <x:v>375</x:v>
-      </x:c>
-      <x:c r="I53" t="s">
+      <x:c r="J53" t="s">
+        <x:v>365</x:v>
+      </x:c>
+      <x:c r="K53" t="s">
         <x:v>388</x:v>
       </x:c>
-      <x:c r="J53" t="s">
-        <x:v>366</x:v>
-      </x:c>
-      <x:c r="K53" t="s">
+      <x:c r="L53" t="s">
         <x:v>389</x:v>
-      </x:c>
-      <x:c r="L53" t="s">
-        <x:v>390</x:v>
       </x:c>
       <x:c r="M53" t="s">
         <x:v>26</x:v>
@@ -7954,10 +7949,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="O53" t="s">
+        <x:v>390</x:v>
+      </x:c>
+      <x:c r="P53" t="s">
         <x:v>391</x:v>
-      </x:c>
-      <x:c r="P53" t="s">
-        <x:v>392</x:v>
       </x:c>
       <x:c r="Q53" s="36" t="str">
         <x:v>1st Prize</x:v>
@@ -8000,13 +7995,13 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="B54" t="s">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="C54" t="s">
+        <x:v>372</x:v>
+      </x:c>
+      <x:c r="D54" s="2" t="s">
         <x:v>385</x:v>
-      </x:c>
-      <x:c r="C54" t="s">
-        <x:v>373</x:v>
-      </x:c>
-      <x:c r="D54" s="2" t="s">
-        <x:v>386</x:v>
       </x:c>
       <x:c r="E54">
         <x:v>1</x:v>
@@ -8015,22 +8010,22 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="G54" t="s">
-        <x:v>387</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="H54" t="s">
-        <x:v>375</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="I54" t="s">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="J54" t="s">
+        <x:v>365</x:v>
+      </x:c>
+      <x:c r="K54" t="s">
         <x:v>393</x:v>
       </x:c>
-      <x:c r="J54" t="s">
-        <x:v>366</x:v>
-      </x:c>
-      <x:c r="K54" t="s">
+      <x:c r="L54" t="s">
         <x:v>394</x:v>
-      </x:c>
-      <x:c r="L54" t="s">
-        <x:v>395</x:v>
       </x:c>
       <x:c r="M54" t="s">
         <x:v>26</x:v>
@@ -8039,10 +8034,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="O54" t="s">
-        <x:v>396</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="P54" t="s">
-        <x:v>392</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="Q54" s="36" t="str">
         <x:v>1st Prize</x:v>
@@ -8085,13 +8080,13 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="B55" t="s">
+        <x:v>396</x:v>
+      </x:c>
+      <x:c r="C55" s="6" t="s">
         <x:v>397</x:v>
       </x:c>
-      <x:c r="C55" s="6" t="s">
+      <x:c r="D55" s="2" t="s">
         <x:v>398</x:v>
-      </x:c>
-      <x:c r="D55" s="2" t="s">
-        <x:v>399</x:v>
       </x:c>
       <x:c r="E55">
         <x:v>1</x:v>
@@ -8100,19 +8095,19 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="G55" t="s">
+        <x:v>399</x:v>
+      </x:c>
+      <x:c r="H55" t="s">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="H55" t="s">
+      <x:c r="I55" s="6" t="s">
         <x:v>401</x:v>
       </x:c>
-      <x:c r="I55" s="6" t="s">
+      <x:c r="J55" t="s">
         <x:v>402</x:v>
       </x:c>
-      <x:c r="J55" t="s">
+      <x:c r="K55" t="s">
         <x:v>403</x:v>
-      </x:c>
-      <x:c r="K55" t="s">
-        <x:v>404</x:v>
       </x:c>
       <x:c r="L55" t="s">
         <x:v>25</x:v>
@@ -8121,13 +8116,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N55" t="s">
+        <x:v>404</x:v>
+      </x:c>
+      <x:c r="O55" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="P55" t="s">
         <x:v>405</x:v>
-      </x:c>
-      <x:c r="O55" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="P55" t="s">
-        <x:v>406</x:v>
       </x:c>
       <x:c r="Q55" s="36" t="str">
         <x:v>1st Prize</x:v>
@@ -8170,13 +8165,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="B56" t="s">
+        <x:v>406</x:v>
+      </x:c>
+      <x:c r="C56" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="C56" t="s">
+      <x:c r="D56" s="2" t="s">
         <x:v>408</x:v>
-      </x:c>
-      <x:c r="D56" s="2" t="s">
-        <x:v>409</x:v>
       </x:c>
       <x:c r="E56">
         <x:v>1</x:v>
@@ -8188,16 +8183,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H56" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="I56" s="6" t="s">
+        <x:v>409</x:v>
+      </x:c>
+      <x:c r="J56" t="s">
+        <x:v>402</x:v>
+      </x:c>
+      <x:c r="K56" t="s">
         <x:v>410</x:v>
-      </x:c>
-      <x:c r="J56" t="s">
-        <x:v>403</x:v>
-      </x:c>
-      <x:c r="K56" t="s">
-        <x:v>411</x:v>
       </x:c>
       <x:c r="L56" t="s">
         <x:v>25</x:v>
@@ -8212,7 +8207,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="P56" t="s">
-        <x:v>412</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="Q56" s="36"/>
       <x:c r="R56" s="36"/>
@@ -8241,10 +8236,10 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B57" t="s">
+        <x:v>412</x:v>
+      </x:c>
+      <x:c r="C57" t="s">
         <x:v>413</x:v>
-      </x:c>
-      <x:c r="C57" t="s">
-        <x:v>414</x:v>
       </x:c>
       <x:c r="D57" s="5">
         <x:v>46207</x:v>
@@ -8259,16 +8254,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H57" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="I57" t="s">
+        <x:v>414</x:v>
+      </x:c>
+      <x:c r="J57" t="s">
         <x:v>415</x:v>
       </x:c>
-      <x:c r="J57" t="s">
+      <x:c r="K57" t="s">
         <x:v>416</x:v>
-      </x:c>
-      <x:c r="K57" t="s">
-        <x:v>417</x:v>
       </x:c>
       <x:c r="L57" t="s">
         <x:v>25</x:v>
@@ -8280,10 +8275,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="O57" t="s">
+        <x:v>417</x:v>
+      </x:c>
+      <x:c r="P57" t="s">
         <x:v>418</x:v>
-      </x:c>
-      <x:c r="P57" t="s">
-        <x:v>419</x:v>
       </x:c>
       <x:c r="Q57" s="36"/>
       <x:c r="R57" s="36"/>
@@ -8312,10 +8307,10 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="B58" t="s">
+        <x:v>419</x:v>
+      </x:c>
+      <x:c r="C58" t="s">
         <x:v>420</x:v>
-      </x:c>
-      <x:c r="C58" t="s">
-        <x:v>421</x:v>
       </x:c>
       <x:c r="D58" s="5">
         <x:v>46299</x:v>
@@ -8330,16 +8325,16 @@
         <x:v>3rd Prize: S$300 Cash and S$385 worth of API Credits</x:v>
       </x:c>
       <x:c r="H58" t="s">
+        <x:v>421</x:v>
+      </x:c>
+      <x:c r="I58" t="s">
         <x:v>422</x:v>
       </x:c>
-      <x:c r="I58" t="s">
+      <x:c r="J58" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K58" t="s">
         <x:v>423</x:v>
-      </x:c>
-      <x:c r="J58" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K58" t="s">
-        <x:v>424</x:v>
       </x:c>
       <x:c r="L58" t="s">
         <x:v>25</x:v>
@@ -8348,13 +8343,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N58" t="s">
+        <x:v>424</x:v>
+      </x:c>
+      <x:c r="O58" t="s">
         <x:v>425</x:v>
       </x:c>
-      <x:c r="O58" t="s">
+      <x:c r="P58" t="s">
         <x:v>426</x:v>
-      </x:c>
-      <x:c r="P58" t="s">
-        <x:v>427</x:v>
       </x:c>
       <x:c r="Q58" s="36" t="str">
         <x:v>3rd Prize</x:v>
@@ -8401,13 +8396,13 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="B59" t="s">
+        <x:v>427</x:v>
+      </x:c>
+      <x:c r="C59" t="s">
         <x:v>428</x:v>
       </x:c>
-      <x:c r="C59" t="s">
+      <x:c r="D59" s="2" t="s">
         <x:v>429</x:v>
-      </x:c>
-      <x:c r="D59" s="2" t="s">
-        <x:v>430</x:v>
       </x:c>
       <x:c r="E59">
         <x:v>1</x:v>
@@ -8422,16 +8417,16 @@
         <x:v>139</x:v>
       </x:c>
       <x:c r="I59" t="s">
+        <x:v>430</x:v>
+      </x:c>
+      <x:c r="J59" t="s">
         <x:v>431</x:v>
       </x:c>
-      <x:c r="J59" t="s">
+      <x:c r="K59" t="s">
         <x:v>432</x:v>
       </x:c>
-      <x:c r="K59" t="s">
+      <x:c r="L59" t="s">
         <x:v>433</x:v>
-      </x:c>
-      <x:c r="L59" t="s">
-        <x:v>434</x:v>
       </x:c>
       <x:c r="M59" t="s">
         <x:v>26</x:v>
@@ -8440,10 +8435,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="O59" t="s">
+        <x:v>434</x:v>
+      </x:c>
+      <x:c r="P59" t="s">
         <x:v>435</x:v>
-      </x:c>
-      <x:c r="P59" t="s">
-        <x:v>436</x:v>
       </x:c>
       <x:c r="Q59" s="36"/>
       <x:c r="R59" s="36"/>
@@ -8472,13 +8467,13 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B60" t="s">
+        <x:v>436</x:v>
+      </x:c>
+      <x:c r="C60" t="s">
         <x:v>437</x:v>
       </x:c>
-      <x:c r="C60" t="s">
+      <x:c r="D60" s="2" t="s">
         <x:v>438</x:v>
-      </x:c>
-      <x:c r="D60" s="2" t="s">
-        <x:v>439</x:v>
       </x:c>
       <x:c r="E60">
         <x:v>1</x:v>
@@ -8490,16 +8485,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H60" t="s">
+        <x:v>439</x:v>
+      </x:c>
+      <x:c r="I60" t="s">
         <x:v>440</x:v>
       </x:c>
-      <x:c r="I60" t="s">
+      <x:c r="J60" t="s">
         <x:v>441</x:v>
       </x:c>
-      <x:c r="J60" t="s">
+      <x:c r="K60" t="s">
         <x:v>442</x:v>
-      </x:c>
-      <x:c r="K60" t="s">
-        <x:v>443</x:v>
       </x:c>
       <x:c r="L60" t="s">
         <x:v>25</x:v>
@@ -8508,13 +8503,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N60" t="s">
+        <x:v>443</x:v>
+      </x:c>
+      <x:c r="O60" t="s">
         <x:v>444</x:v>
       </x:c>
-      <x:c r="O60" t="s">
+      <x:c r="P60" t="s">
         <x:v>445</x:v>
-      </x:c>
-      <x:c r="P60" t="s">
-        <x:v>446</x:v>
       </x:c>
       <x:c r="Q60" s="36"/>
       <x:c r="R60" s="36"/>
@@ -8543,13 +8538,13 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="B61" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="C61" t="s">
         <x:v>447</x:v>
       </x:c>
-      <x:c r="C61" t="s">
+      <x:c r="D61" s="2" t="s">
         <x:v>448</x:v>
-      </x:c>
-      <x:c r="D61" s="2" t="s">
-        <x:v>449</x:v>
       </x:c>
       <x:c r="E61">
         <x:v>1</x:v>
@@ -8561,16 +8556,16 @@
         <x:v>2K USD Speechmatics Credits</x:v>
       </x:c>
       <x:c r="H61" t="s">
+        <x:v>449</x:v>
+      </x:c>
+      <x:c r="I61" t="s">
         <x:v>450</x:v>
       </x:c>
-      <x:c r="I61" t="s">
+      <x:c r="J61" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K61" t="s">
         <x:v>451</x:v>
-      </x:c>
-      <x:c r="J61" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K61" t="s">
-        <x:v>452</x:v>
       </x:c>
       <x:c r="L61" t="s">
         <x:v>25</x:v>
@@ -8579,13 +8574,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N61" t="s">
+        <x:v>452</x:v>
+      </x:c>
+      <x:c r="O61" t="s">
         <x:v>453</x:v>
       </x:c>
-      <x:c r="O61" t="s">
+      <x:c r="P61" s="1" t="s">
         <x:v>454</x:v>
-      </x:c>
-      <x:c r="P61" s="1" t="s">
-        <x:v>455</x:v>
       </x:c>
       <x:c r="Q61" s="36" t="str">
         <x:v>Award</x:v>
@@ -8630,13 +8625,13 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="B62" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="C62" t="s">
         <x:v>456</x:v>
       </x:c>
-      <x:c r="C62" t="s">
+      <x:c r="D62" s="2" t="s">
         <x:v>457</x:v>
-      </x:c>
-      <x:c r="D62" s="2" t="s">
-        <x:v>458</x:v>
       </x:c>
       <x:c r="E62">
         <x:v>1</x:v>
@@ -8648,16 +8643,16 @@
         <x:v>2nd Place — v0 Sock</x:v>
       </x:c>
       <x:c r="H62" t="s">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="I62" t="s">
         <x:v>459</x:v>
       </x:c>
-      <x:c r="I62" t="s">
+      <x:c r="J62" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K62" t="s">
         <x:v>460</x:v>
-      </x:c>
-      <x:c r="J62" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K62" t="s">
-        <x:v>461</x:v>
       </x:c>
       <x:c r="L62" t="s">
         <x:v>25</x:v>
@@ -8672,7 +8667,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="P62" s="1" t="s">
-        <x:v>462</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="Q62" s="36" t="str">
         <x:v>2nd Place</x:v>
@@ -8717,10 +8712,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="B63" t="s">
+        <x:v>462</x:v>
+      </x:c>
+      <x:c r="C63" t="s">
         <x:v>463</x:v>
-      </x:c>
-      <x:c r="C63" t="s">
-        <x:v>464</x:v>
       </x:c>
       <x:c r="D63" s="5">
         <x:v>46085</x:v>
@@ -8729,22 +8724,22 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F63" t="s">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="G63" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H63" t="s">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="I63" t="s">
         <x:v>465</x:v>
       </x:c>
-      <x:c r="G63" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="H63" t="s">
-        <x:v>401</x:v>
-      </x:c>
-      <x:c r="I63" t="s">
+      <x:c r="J63" t="s">
+        <x:v>402</x:v>
+      </x:c>
+      <x:c r="K63" t="s">
         <x:v>466</x:v>
-      </x:c>
-      <x:c r="J63" t="s">
-        <x:v>403</x:v>
-      </x:c>
-      <x:c r="K63" t="s">
-        <x:v>467</x:v>
       </x:c>
       <x:c r="L63" t="s">
         <x:v>25</x:v>
@@ -8753,13 +8748,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N63" t="s">
+        <x:v>467</x:v>
+      </x:c>
+      <x:c r="O63" t="s">
         <x:v>468</x:v>
       </x:c>
-      <x:c r="O63" t="s">
+      <x:c r="P63" t="s">
         <x:v>469</x:v>
-      </x:c>
-      <x:c r="P63" t="s">
-        <x:v>470</x:v>
       </x:c>
       <x:c r="Q63" s="36"/>
       <x:c r="R63" s="36"/>
@@ -8788,10 +8783,10 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="B64" t="s">
-        <x:v>471</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="C64" t="s">
-        <x:v>457</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="D64" s="5">
         <x:v>46116</x:v>
@@ -8806,16 +8801,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H64" t="s">
-        <x:v>459</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="I64" t="s">
+        <x:v>471</x:v>
+      </x:c>
+      <x:c r="J64" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K64" t="s">
         <x:v>472</x:v>
-      </x:c>
-      <x:c r="J64" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K64" t="s">
-        <x:v>473</x:v>
       </x:c>
       <x:c r="L64" t="s">
         <x:v>25</x:v>
@@ -8824,13 +8819,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N64" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="O64" t="s">
+        <x:v>473</x:v>
+      </x:c>
+      <x:c r="P64" t="s">
         <x:v>474</x:v>
-      </x:c>
-      <x:c r="P64" t="s">
-        <x:v>475</x:v>
       </x:c>
       <x:c r="Q64" s="36"/>
       <x:c r="R64" s="36"/>
@@ -8859,10 +8854,10 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="B65" t="s">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="C65" t="s">
         <x:v>476</x:v>
-      </x:c>
-      <x:c r="C65" t="s">
-        <x:v>477</x:v>
       </x:c>
       <x:c r="D65" s="5">
         <x:v>46270</x:v>
@@ -8877,16 +8872,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H65" t="s">
-        <x:v>459</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="I65" t="s">
+        <x:v>477</x:v>
+      </x:c>
+      <x:c r="J65" t="s">
         <x:v>478</x:v>
       </x:c>
-      <x:c r="J65" t="s">
+      <x:c r="K65" t="s">
         <x:v>479</x:v>
-      </x:c>
-      <x:c r="K65" t="s">
-        <x:v>480</x:v>
       </x:c>
       <x:c r="L65" t="s">
         <x:v>25</x:v>
@@ -8898,10 +8893,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="O65" t="s">
+        <x:v>480</x:v>
+      </x:c>
+      <x:c r="P65" t="s">
         <x:v>481</x:v>
-      </x:c>
-      <x:c r="P65" t="s">
-        <x:v>482</x:v>
       </x:c>
       <x:c r="Q65" s="36"/>
       <x:c r="R65" s="36"/>
@@ -8930,13 +8925,13 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B66" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="C66" t="s">
         <x:v>483</x:v>
       </x:c>
-      <x:c r="C66" t="s">
+      <x:c r="D66" s="2" t="s">
         <x:v>484</x:v>
-      </x:c>
-      <x:c r="D66" s="2" t="s">
-        <x:v>485</x:v>
       </x:c>
       <x:c r="E66">
         <x:v>1</x:v>
@@ -8948,16 +8943,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H66" t="s">
-        <x:v>375</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="I66" t="s">
+        <x:v>485</x:v>
+      </x:c>
+      <x:c r="J66" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K66" t="s">
         <x:v>486</x:v>
-      </x:c>
-      <x:c r="J66" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K66" t="s">
-        <x:v>487</x:v>
       </x:c>
       <x:c r="L66" t="s">
         <x:v>25</x:v>
@@ -8966,13 +8961,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N66" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="O66" t="s">
         <x:v>488</x:v>
       </x:c>
-      <x:c r="O66" t="s">
+      <x:c r="P66" t="s">
         <x:v>489</x:v>
-      </x:c>
-      <x:c r="P66" t="s">
-        <x:v>490</x:v>
       </x:c>
       <x:c r="Q66" s="36"/>
       <x:c r="R66" s="36"/>
@@ -9001,13 +8996,13 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B67" t="s">
+        <x:v>490</x:v>
+      </x:c>
+      <x:c r="C67" t="s">
         <x:v>491</x:v>
       </x:c>
-      <x:c r="C67" t="s">
+      <x:c r="D67" s="2" t="s">
         <x:v>492</x:v>
-      </x:c>
-      <x:c r="D67" s="2" t="s">
-        <x:v>493</x:v>
       </x:c>
       <x:c r="E67">
         <x:v>1</x:v>
@@ -9016,19 +9011,19 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="G67" t="s">
+        <x:v>493</x:v>
+      </x:c>
+      <x:c r="H67" t="s">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="I67" t="s">
+        <x:v>409</x:v>
+      </x:c>
+      <x:c r="J67" t="s">
         <x:v>494</x:v>
       </x:c>
-      <x:c r="H67" t="s">
-        <x:v>401</x:v>
-      </x:c>
-      <x:c r="I67" t="s">
-        <x:v>410</x:v>
-      </x:c>
-      <x:c r="J67" t="s">
+      <x:c r="K67" t="s">
         <x:v>495</x:v>
-      </x:c>
-      <x:c r="K67" t="s">
-        <x:v>496</x:v>
       </x:c>
       <x:c r="L67" t="s">
         <x:v>25</x:v>
@@ -9037,7 +9032,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N67" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="O67" t="s">
         <x:v>25</x:v>
@@ -9086,13 +9081,13 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B68" t="s">
-        <x:v>497</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="C68" t="s">
         <x:v>262</x:v>
       </x:c>
       <x:c r="D68" s="2" t="s">
-        <x:v>498</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="E68">
         <x:v>3</x:v>
@@ -9104,19 +9099,19 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H68" t="s">
+        <x:v>498</x:v>
+      </x:c>
+      <x:c r="I68" t="s">
         <x:v>499</x:v>
       </x:c>
-      <x:c r="I68" t="s">
+      <x:c r="J68" t="s">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="J68" t="s">
+      <x:c r="K68" t="s">
         <x:v>501</x:v>
       </x:c>
-      <x:c r="K68" t="s">
+      <x:c r="L68" t="s">
         <x:v>502</x:v>
-      </x:c>
-      <x:c r="L68" t="s">
-        <x:v>503</x:v>
       </x:c>
       <x:c r="M68" t="s">
         <x:v>26</x:v>
@@ -9125,7 +9120,7 @@
         <x:v>269</x:v>
       </x:c>
       <x:c r="O68" t="s">
-        <x:v>504</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="P68" t="s">
         <x:v>25</x:v>
@@ -9157,13 +9152,13 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B69" t="s">
+        <x:v>504</x:v>
+      </x:c>
+      <x:c r="C69" t="s">
+        <x:v>491</x:v>
+      </x:c>
+      <x:c r="D69" s="2" t="s">
         <x:v>505</x:v>
-      </x:c>
-      <x:c r="C69" t="s">
-        <x:v>492</x:v>
-      </x:c>
-      <x:c r="D69" s="2" t="s">
-        <x:v>506</x:v>
       </x:c>
       <x:c r="E69">
         <x:v>1</x:v>
@@ -9175,16 +9170,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H69" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="I69" t="s">
-        <x:v>410</x:v>
+        <x:v>409</x:v>
       </x:c>
       <x:c r="J69" t="s">
-        <x:v>495</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="K69" t="s">
-        <x:v>507</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="L69" t="s">
         <x:v>25</x:v>
@@ -9193,13 +9188,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="N69" t="s">
+        <x:v>507</x:v>
+      </x:c>
+      <x:c r="O69" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="P69" t="s">
         <x:v>508</x:v>
-      </x:c>
-      <x:c r="O69" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="P69" t="s">
-        <x:v>509</x:v>
       </x:c>
       <x:c r="Q69" s="36"/>
       <x:c r="R69" s="36"/>
@@ -9228,13 +9223,13 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="B70" t="s">
+        <x:v>509</x:v>
+      </x:c>
+      <x:c r="C70" t="s">
         <x:v>510</x:v>
       </x:c>
-      <x:c r="C70" t="s">
+      <x:c r="D70" s="2" t="s">
         <x:v>511</x:v>
-      </x:c>
-      <x:c r="D70" s="2" t="s">
-        <x:v>512</x:v>
       </x:c>
       <x:c r="E70">
         <x:v>2</x:v>
@@ -9243,31 +9238,31 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="H70" t="s">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="I70" t="s">
         <x:v>513</x:v>
       </x:c>
-      <x:c r="I70" t="s">
+      <x:c r="J70" t="s">
         <x:v>514</x:v>
       </x:c>
-      <x:c r="J70" t="s">
+      <x:c r="K70" t="s">
         <x:v>515</x:v>
       </x:c>
-      <x:c r="K70" t="s">
+      <x:c r="L70" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="M70" t="s">
         <x:v>516</x:v>
       </x:c>
-      <x:c r="L70" t="s">
-        <x:v>511</x:v>
-      </x:c>
-      <x:c r="M70" t="s">
+      <x:c r="N70" t="s">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="O70" t="s">
         <x:v>517</x:v>
       </x:c>
-      <x:c r="N70" t="s">
-        <x:v>355</x:v>
-      </x:c>
-      <x:c r="O70" t="s">
+      <x:c r="P70" t="s">
         <x:v>518</x:v>
-      </x:c>
-      <x:c r="P70" t="s">
-        <x:v>519</x:v>
       </x:c>
       <x:c r="Q70" s="36"/>
       <x:c r="R70" s="36"/>
@@ -9296,13 +9291,13 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="B71" t="s">
+        <x:v>519</x:v>
+      </x:c>
+      <x:c r="C71" t="s">
         <x:v>520</x:v>
       </x:c>
-      <x:c r="C71" t="s">
+      <x:c r="D71" s="5" t="s">
         <x:v>521</x:v>
-      </x:c>
-      <x:c r="D71" s="5" t="s">
-        <x:v>522</x:v>
       </x:c>
       <x:c r="E71">
         <x:v>1</x:v>
@@ -9314,31 +9309,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H71" t="s">
-        <x:v>513</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="I71" t="s">
+        <x:v>522</x:v>
+      </x:c>
+      <x:c r="J71" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K71" t="s">
         <x:v>523</x:v>
       </x:c>
-      <x:c r="J71" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K71" t="s">
-        <x:v>524</x:v>
-      </x:c>
       <x:c r="L71" t="s">
-        <x:v>521</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="M71" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N71" t="s">
-        <x:v>488</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="O71" t="s">
+        <x:v>524</x:v>
+      </x:c>
+      <x:c r="P71" t="s">
         <x:v>525</x:v>
-      </x:c>
-      <x:c r="P71" t="s">
-        <x:v>526</x:v>
       </x:c>
       <x:c r="Q71" s="36"/>
       <x:c r="R71" s="36"/>
@@ -9367,10 +9362,10 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B72" t="s">
+        <x:v>526</x:v>
+      </x:c>
+      <x:c r="C72" t="s">
         <x:v>527</x:v>
-      </x:c>
-      <x:c r="C72" t="s">
-        <x:v>528</x:v>
       </x:c>
       <x:c r="D72" s="5">
         <x:v>46363</x:v>
@@ -9388,16 +9383,16 @@
         <x:v>237</x:v>
       </x:c>
       <x:c r="I72" t="s">
+        <x:v>528</x:v>
+      </x:c>
+      <x:c r="J72" t="s">
         <x:v>529</x:v>
       </x:c>
-      <x:c r="J72" t="s">
+      <x:c r="K72" t="s">
         <x:v>530</x:v>
       </x:c>
-      <x:c r="K72" t="s">
-        <x:v>531</x:v>
-      </x:c>
       <x:c r="L72" t="s">
-        <x:v>528</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="M72" t="s">
         <x:v>26</x:v>
@@ -9409,7 +9404,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="P72" t="s">
-        <x:v>532</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="Q72" s="36" t="str">
         <x:v>Top 30</x:v>
@@ -9452,13 +9447,13 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B73" t="s">
+        <x:v>532</x:v>
+      </x:c>
+      <x:c r="C73" t="s">
         <x:v>533</x:v>
       </x:c>
-      <x:c r="C73" t="s">
+      <x:c r="D73" s="2" t="s">
         <x:v>534</x:v>
-      </x:c>
-      <x:c r="D73" s="2" t="s">
-        <x:v>535</x:v>
       </x:c>
       <x:c r="E73">
         <x:v>1</x:v>
@@ -9470,31 +9465,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H73" t="s">
-        <x:v>459</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="I73" t="s">
+        <x:v>535</x:v>
+      </x:c>
+      <x:c r="J73" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K73" t="s">
         <x:v>536</x:v>
       </x:c>
-      <x:c r="J73" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K73" t="s">
-        <x:v>537</x:v>
-      </x:c>
       <x:c r="L73" t="s">
-        <x:v>534</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="M73" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N73" t="s">
+        <x:v>537</x:v>
+      </x:c>
+      <x:c r="O73" t="s">
         <x:v>538</x:v>
       </x:c>
-      <x:c r="O73" t="s">
+      <x:c r="P73" t="s">
         <x:v>539</x:v>
-      </x:c>
-      <x:c r="P73" t="s">
-        <x:v>540</x:v>
       </x:c>
       <x:c r="Q73" s="36"/>
       <x:c r="R73" s="36"/>
@@ -9523,13 +9518,13 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B74" t="s">
+        <x:v>540</x:v>
+      </x:c>
+      <x:c r="C74" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="D74" s="2" t="s">
         <x:v>541</x:v>
-      </x:c>
-      <x:c r="C74" t="s">
-        <x:v>511</x:v>
-      </x:c>
-      <x:c r="D74" s="2" t="s">
-        <x:v>542</x:v>
       </x:c>
       <x:c r="E74">
         <x:v>10</x:v>
@@ -9541,31 +9536,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H74" t="s">
+        <x:v>542</x:v>
+      </x:c>
+      <x:c r="I74" t="s">
         <x:v>543</x:v>
       </x:c>
-      <x:c r="I74" t="s">
+      <x:c r="J74" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K74" t="s">
         <x:v>544</x:v>
       </x:c>
-      <x:c r="J74" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K74" t="s">
+      <x:c r="L74" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="M74" t="s">
+        <x:v>516</x:v>
+      </x:c>
+      <x:c r="N74" t="s">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="O74" t="s">
         <x:v>545</x:v>
       </x:c>
-      <x:c r="L74" t="s">
-        <x:v>511</x:v>
-      </x:c>
-      <x:c r="M74" t="s">
-        <x:v>517</x:v>
-      </x:c>
-      <x:c r="N74" t="s">
-        <x:v>355</x:v>
-      </x:c>
-      <x:c r="O74" t="s">
-        <x:v>546</x:v>
-      </x:c>
       <x:c r="P74" t="s">
-        <x:v>519</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="Q74" s="36"/>
       <x:c r="R74" s="36"/>
@@ -9594,10 +9589,10 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B75" s="12" t="s">
+        <x:v>546</x:v>
+      </x:c>
+      <x:c r="C75" s="12" t="s">
         <x:v>547</x:v>
-      </x:c>
-      <x:c r="C75" s="12" t="s">
-        <x:v>548</x:v>
       </x:c>
       <x:c r="D75" s="5">
         <x:v>46150</x:v>
@@ -9612,19 +9607,19 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H75" s="12" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="I75" s="14" t="s">
         <x:v>548</x:v>
       </x:c>
-      <x:c r="I75" s="14" t="s">
+      <x:c r="J75" s="12" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K75" s="12" t="s">
         <x:v>549</x:v>
       </x:c>
-      <x:c r="J75" s="12" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K75" s="12" t="s">
-        <x:v>550</x:v>
-      </x:c>
       <x:c r="L75" s="12" t="s">
-        <x:v>548</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="M75" s="12" t="s">
         <x:v>26</x:v>
@@ -9633,7 +9628,7 @@
         <x:v>269</x:v>
       </x:c>
       <x:c r="O75" t="s">
-        <x:v>551</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="P75" s="12" t="s">
         <x:v>25</x:v>
@@ -9665,13 +9660,13 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B76" s="12" t="s">
+        <x:v>551</x:v>
+      </x:c>
+      <x:c r="C76" s="12" t="s">
         <x:v>552</x:v>
       </x:c>
-      <x:c r="C76" s="12" t="s">
+      <x:c r="D76" s="13" t="s">
         <x:v>553</x:v>
-      </x:c>
-      <x:c r="D76" s="13" t="s">
-        <x:v>554</x:v>
       </x:c>
       <x:c r="E76">
         <x:v>1</x:v>
@@ -9683,31 +9678,31 @@
         <x:v>Best Vertical Solution (Family Office Track), 2,000 Cybrdeck API credits (worth US$25)</x:v>
       </x:c>
       <x:c r="H76" s="12" t="s">
+        <x:v>554</x:v>
+      </x:c>
+      <x:c r="I76" s="12" t="s">
         <x:v>555</x:v>
       </x:c>
-      <x:c r="I76" s="12" t="s">
+      <x:c r="J76" s="12" t="s">
         <x:v>556</x:v>
       </x:c>
-      <x:c r="J76" s="12" t="s">
+      <x:c r="K76" s="12" t="s">
         <x:v>557</x:v>
       </x:c>
-      <x:c r="K76" s="12" t="s">
-        <x:v>558</x:v>
-      </x:c>
       <x:c r="L76" s="12" t="s">
-        <x:v>553</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="M76" s="12" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N76" s="12" t="s">
+        <x:v>558</x:v>
+      </x:c>
+      <x:c r="O76" s="1" t="s">
         <x:v>559</x:v>
       </x:c>
-      <x:c r="O76" s="1" t="s">
+      <x:c r="P76" t="s">
         <x:v>560</x:v>
-      </x:c>
-      <x:c r="P76" t="s">
-        <x:v>561</x:v>
       </x:c>
       <x:c r="Q76" s="36" t="str">
         <x:v>Best Project</x:v>
@@ -9752,13 +9747,13 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B77" t="s">
+        <x:v>561</x:v>
+      </x:c>
+      <x:c r="C77" t="s">
         <x:v>562</x:v>
       </x:c>
-      <x:c r="C77" t="s">
+      <x:c r="D77" t="s">
         <x:v>563</x:v>
-      </x:c>
-      <x:c r="D77" t="s">
-        <x:v>564</x:v>
       </x:c>
       <x:c r="E77">
         <x:v>1</x:v>
@@ -9770,31 +9765,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H77" t="s">
+        <x:v>564</x:v>
+      </x:c>
+      <x:c r="I77" t="s">
         <x:v>565</x:v>
       </x:c>
-      <x:c r="I77" t="s">
+      <x:c r="J77" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K77" t="s">
         <x:v>566</x:v>
       </x:c>
-      <x:c r="J77" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K77" t="s">
+      <x:c r="L77" t="s">
         <x:v>567</x:v>
-      </x:c>
-      <x:c r="L77" t="s">
-        <x:v>568</x:v>
       </x:c>
       <x:c r="M77" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="N77" t="s">
+        <x:v>568</x:v>
+      </x:c>
+      <x:c r="O77" t="s">
         <x:v>569</x:v>
       </x:c>
-      <x:c r="O77" t="s">
+      <x:c r="P77" t="s">
         <x:v>570</x:v>
-      </x:c>
-      <x:c r="P77" t="s">
-        <x:v>571</x:v>
       </x:c>
       <x:c r="Q77" s="36"/>
       <x:c r="R77" s="36"/>
@@ -9823,13 +9818,13 @@
         <x:v>77</x:v>
       </x:c>
       <x:c r="B78" t="s">
+        <x:v>571</x:v>
+      </x:c>
+      <x:c r="C78" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="D78" t="s">
         <x:v>572</x:v>
-      </x:c>
-      <x:c r="C78" t="s">
-        <x:v>511</x:v>
-      </x:c>
-      <x:c r="D78" t="s">
-        <x:v>573</x:v>
       </x:c>
       <x:c r="E78">
         <x:v>1</x:v>
@@ -9841,31 +9836,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="H78" t="s">
+        <x:v>573</x:v>
+      </x:c>
+      <x:c r="I78" t="s">
         <x:v>574</x:v>
       </x:c>
-      <x:c r="I78" t="s">
+      <x:c r="J78" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="K78" t="s">
         <x:v>575</x:v>
       </x:c>
-      <x:c r="J78" t="s">
-        <x:v>308</x:v>
-      </x:c>
-      <x:c r="K78" t="s">
+      <x:c r="L78" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="M78" t="s">
+        <x:v>516</x:v>
+      </x:c>
+      <x:c r="N78" t="s">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="O78" t="s">
         <x:v>576</x:v>
       </x:c>
-      <x:c r="L78" t="s">
-        <x:v>511</x:v>
-      </x:c>
-      <x:c r="M78" t="s">
-        <x:v>517</x:v>
-      </x:c>
-      <x:c r="N78" t="s">
-        <x:v>355</x:v>
-      </x:c>
-      <x:c r="O78" t="s">
-        <x:v>577</x:v>
-      </x:c>
       <x:c r="P78" t="s">
-        <x:v>519</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="Q78" s="36"/>
       <x:c r="R78" s="36"/>
@@ -9894,37 +9889,37 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="B79" t="s">
+        <x:v>577</x:v>
+      </x:c>
+      <x:c r="C79" t="s">
         <x:v>578</x:v>
       </x:c>
-      <x:c r="C79" t="s">
+      <x:c r="D79" t="s">
         <x:v>579</x:v>
-      </x:c>
-      <x:c r="D79" t="s">
-        <x:v>580</x:v>
       </x:c>
       <x:c r="E79">
         <x:v>4</x:v>
       </x:c>
       <x:c r="F79" t="s">
-        <x:v>465</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="G79" t="s">
         <x:v>25</x:v>
       </x:c>
       <x:c r="H79" t="s">
+        <x:v>580</x:v>
+      </x:c>
+      <x:c r="I79" t="s">
         <x:v>581</x:v>
       </x:c>
-      <x:c r="I79" t="s">
+      <x:c r="J79" t="s">
         <x:v>582</x:v>
       </x:c>
-      <x:c r="J79" t="s">
+      <x:c r="K79" t="s">
         <x:v>583</x:v>
       </x:c>
-      <x:c r="K79" t="s">
+      <x:c r="L79" t="s">
         <x:v>584</x:v>
-      </x:c>
-      <x:c r="L79" t="s">
-        <x:v>585</x:v>
       </x:c>
       <x:c r="M79" t="s">
         <x:v>26</x:v>
@@ -9933,10 +9928,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="O79" t="s">
+        <x:v>585</x:v>
+      </x:c>
+      <x:c r="P79" t="s">
         <x:v>586</x:v>
-      </x:c>
-      <x:c r="P79" t="s">
-        <x:v>587</x:v>
       </x:c>
       <x:c r="Q79" s="36"/>
       <x:c r="R79" s="36"/>
@@ -10209,10 +10204,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Raf0a946ee9524174"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R1cded7850b394676"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R5ded13067fd74a8e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R889ae99d32864598"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R86400ab6245b46bb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R52d8145920914c09"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R91989bad373c4cad"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R2b2b25bbb7574864"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -10235,7 +10230,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>588</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -10244,7 +10239,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="19" t="s">
-        <x:v>589</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="B2" s="19"/>
       <x:c r="C2" s="19"/>
@@ -10253,64 +10248,64 @@
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="11" t="s">
+        <x:v>589</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="s">
         <x:v>590</x:v>
       </x:c>
-      <x:c r="B4" s="11" t="s">
+      <x:c r="C4" s="11" t="s">
         <x:v>591</x:v>
       </x:c>
-      <x:c r="C4" s="11" t="s">
+      <x:c r="D4" s="11" t="s">
         <x:v>592</x:v>
       </x:c>
-      <x:c r="D4" s="11" t="s">
+      <x:c r="E4" s="11" t="s">
         <x:v>593</x:v>
-      </x:c>
-      <x:c r="E4" s="11" t="s">
-        <x:v>594</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="8" t="s">
+        <x:v>594</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="s">
         <x:v>595</x:v>
       </x:c>
-      <x:c r="B5" s="7" t="s">
+      <x:c r="C5" s="7" t="s">
         <x:v>596</x:v>
-      </x:c>
-      <x:c r="C5" s="7" t="s">
-        <x:v>597</x:v>
       </x:c>
       <x:c r="D5" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E5" s="10" t="s">
-        <x:v>598</x:v>
+        <x:v>597</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="8" t="s">
+        <x:v>598</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>599</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="s">
+      <x:c r="C6" s="7" t="s">
         <x:v>600</x:v>
-      </x:c>
-      <x:c r="C6" s="7" t="s">
-        <x:v>601</x:v>
       </x:c>
       <x:c r="D6" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="10" t="s">
-        <x:v>602</x:v>
+        <x:v>601</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="8" t="s">
+        <x:v>602</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
         <x:v>603</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="s">
+      <x:c r="C7" s="7" t="s">
         <x:v>604</x:v>
-      </x:c>
-      <x:c r="C7" s="7" t="s">
-        <x:v>605</x:v>
       </x:c>
       <x:c r="D7" s="9">
         <x:v>1</x:v>
@@ -10319,47 +10314,47 @@
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
       <x:c r="A8" s="8" t="s">
+        <x:v>605</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
         <x:v>606</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="s">
+      <x:c r="C8" s="7" t="s">
         <x:v>607</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="s">
-        <x:v>608</x:v>
       </x:c>
       <x:c r="D8" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E8" s="10" t="s">
-        <x:v>609</x:v>
+        <x:v>608</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" s="8" t="s">
+        <x:v>609</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
         <x:v>610</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="s">
-        <x:v>611</x:v>
-      </x:c>
       <x:c r="C9" s="7" t="s">
-        <x:v>601</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="D9" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="10" t="s">
-        <x:v>612</x:v>
+        <x:v>611</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
       <x:c r="A10" s="8" t="s">
+        <x:v>612</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="s">
         <x:v>613</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="s">
+      <x:c r="C10" s="7" t="s">
         <x:v>614</x:v>
-      </x:c>
-      <x:c r="C10" s="7" t="s">
-        <x:v>615</x:v>
       </x:c>
       <x:c r="D10" s="9">
         <x:v>1</x:v>
@@ -10368,47 +10363,47 @@
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
       <x:c r="A11" s="8" t="s">
+        <x:v>615</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="s">
         <x:v>616</x:v>
       </x:c>
-      <x:c r="B11" s="7" t="s">
+      <x:c r="C11" s="7" t="s">
         <x:v>617</x:v>
-      </x:c>
-      <x:c r="C11" s="7" t="s">
-        <x:v>618</x:v>
       </x:c>
       <x:c r="D11" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E11" s="10" t="s">
-        <x:v>619</x:v>
+        <x:v>618</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
       <x:c r="A12" s="8" t="s">
+        <x:v>619</x:v>
+      </x:c>
+      <x:c r="B12" s="7" t="s">
         <x:v>620</x:v>
       </x:c>
-      <x:c r="B12" s="7" t="s">
+      <x:c r="C12" s="7" t="s">
         <x:v>621</x:v>
-      </x:c>
-      <x:c r="C12" s="7" t="s">
-        <x:v>622</x:v>
       </x:c>
       <x:c r="D12" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E12" s="10" t="s">
-        <x:v>623</x:v>
+        <x:v>622</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
       <x:c r="A13" s="8" t="s">
+        <x:v>623</x:v>
+      </x:c>
+      <x:c r="B13" s="7" t="s">
         <x:v>624</x:v>
       </x:c>
-      <x:c r="B13" s="7" t="s">
+      <x:c r="C13" s="7" t="s">
         <x:v>625</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="s">
-        <x:v>626</x:v>
       </x:c>
       <x:c r="D13" s="9">
         <x:v>1</x:v>
@@ -10417,30 +10412,30 @@
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
       <x:c r="A14" s="8" t="s">
+        <x:v>626</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="s">
         <x:v>627</x:v>
       </x:c>
-      <x:c r="B14" s="7" t="s">
-        <x:v>628</x:v>
-      </x:c>
       <x:c r="C14" s="7" t="s">
-        <x:v>626</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="D14" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E14" s="10" t="s">
-        <x:v>629</x:v>
+        <x:v>628</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
       <x:c r="A15" s="8" t="s">
+        <x:v>629</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="s">
         <x:v>630</x:v>
       </x:c>
-      <x:c r="B15" s="7" t="s">
+      <x:c r="C15" s="7" t="s">
         <x:v>631</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="s">
-        <x:v>632</x:v>
       </x:c>
       <x:c r="D15" s="9">
         <x:v>1</x:v>
@@ -10449,30 +10444,30 @@
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
       <x:c r="A16" s="8" t="s">
+        <x:v>632</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="s">
         <x:v>633</x:v>
       </x:c>
-      <x:c r="B16" s="7" t="s">
+      <x:c r="C16" s="7" t="s">
         <x:v>634</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="s">
-        <x:v>635</x:v>
       </x:c>
       <x:c r="D16" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E16" s="10" t="s">
-        <x:v>636</x:v>
+        <x:v>635</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
       <x:c r="A17" s="8" t="s">
+        <x:v>636</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="s">
         <x:v>637</x:v>
       </x:c>
-      <x:c r="B17" s="7" t="s">
+      <x:c r="C17" s="7" t="s">
         <x:v>638</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="s">
-        <x:v>639</x:v>
       </x:c>
       <x:c r="D17" s="9">
         <x:v>1</x:v>
@@ -10481,47 +10476,47 @@
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
       <x:c r="A18" s="8" t="s">
+        <x:v>639</x:v>
+      </x:c>
+      <x:c r="B18" s="7" t="s">
         <x:v>640</x:v>
       </x:c>
-      <x:c r="B18" s="7" t="s">
+      <x:c r="C18" s="7" t="s">
         <x:v>641</x:v>
-      </x:c>
-      <x:c r="C18" s="7" t="s">
-        <x:v>642</x:v>
       </x:c>
       <x:c r="D18" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E18" s="10" t="s">
-        <x:v>643</x:v>
+        <x:v>642</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
       <x:c r="A19" s="8" t="s">
+        <x:v>643</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="s">
         <x:v>644</x:v>
       </x:c>
-      <x:c r="B19" s="7" t="s">
+      <x:c r="C19" s="7" t="s">
         <x:v>645</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="s">
-        <x:v>646</x:v>
       </x:c>
       <x:c r="D19" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E19" s="10" t="s">
-        <x:v>647</x:v>
+        <x:v>646</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28" customHeight="1">
       <x:c r="A20" s="8" t="s">
+        <x:v>647</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="s">
         <x:v>648</x:v>
       </x:c>
-      <x:c r="B20" s="7" t="s">
+      <x:c r="C20" s="7" t="s">
         <x:v>649</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>650</x:v>
       </x:c>
       <x:c r="D20" s="9">
         <x:v>1</x:v>
@@ -10530,10 +10525,10 @@
     </x:row>
     <x:row r="21" ht="28" customHeight="1">
       <x:c r="A21" s="8" t="s">
+        <x:v>650</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="s">
         <x:v>651</x:v>
-      </x:c>
-      <x:c r="B21" s="7" t="s">
-        <x:v>652</x:v>
       </x:c>
       <x:c r="C21" s="7" t="str">
         <x:v>#069, #071, #079</x:v>
@@ -10542,18 +10537,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E21" s="10" t="s">
-        <x:v>653</x:v>
+        <x:v>652</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
       <x:c r="A22" s="8" t="s">
+        <x:v>653</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="s">
         <x:v>654</x:v>
       </x:c>
-      <x:c r="B22" s="7" t="s">
+      <x:c r="C22" s="7" t="s">
         <x:v>655</x:v>
-      </x:c>
-      <x:c r="C22" s="7" t="s">
-        <x:v>656</x:v>
       </x:c>
       <x:c r="D22" s="9">
         <x:v>1</x:v>
@@ -10562,13 +10557,13 @@
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
       <x:c r="A23" s="8" t="s">
+        <x:v>656</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="s">
         <x:v>657</x:v>
       </x:c>
-      <x:c r="B23" s="7" t="s">
+      <x:c r="C23" s="7" t="s">
         <x:v>658</x:v>
-      </x:c>
-      <x:c r="C23" s="7" t="s">
-        <x:v>659</x:v>
       </x:c>
       <x:c r="D23" s="9">
         <x:v>1</x:v>
@@ -10577,10 +10572,10 @@
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
       <x:c r="A24" s="8" t="s">
+        <x:v>659</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="s">
         <x:v>660</x:v>
-      </x:c>
-      <x:c r="B24" s="7" t="s">
-        <x:v>661</x:v>
       </x:c>
       <x:c r="C24" s="7" t="str">
         <x:v>#054, #055, #056, #062, #066, #068, #075</x:v>
@@ -10589,12 +10584,12 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E24" s="10" t="s">
-        <x:v>662</x:v>
+        <x:v>661</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
       <x:c r="A25" s="8" t="s">
-        <x:v>663</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
         <x:v>Clement Lork</x:v>
@@ -10606,18 +10601,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E25" s="10" t="s">
-        <x:v>664</x:v>
+        <x:v>663</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="8" t="s">
+        <x:v>664</x:v>
+      </x:c>
+      <x:c r="B26" s="7" t="s">
         <x:v>665</x:v>
       </x:c>
-      <x:c r="B26" s="7" t="s">
-        <x:v>666</x:v>
-      </x:c>
       <x:c r="C26" s="7" t="s">
-        <x:v>605</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="D26" s="9">
         <x:v>1</x:v>
@@ -10626,13 +10621,13 @@
     </x:row>
     <x:row r="27" ht="28" customHeight="1">
       <x:c r="A27" s="8" t="s">
+        <x:v>666</x:v>
+      </x:c>
+      <x:c r="B27" s="7" t="s">
         <x:v>667</x:v>
       </x:c>
-      <x:c r="B27" s="7" t="s">
+      <x:c r="C27" s="7" t="s">
         <x:v>668</x:v>
-      </x:c>
-      <x:c r="C27" s="7" t="s">
-        <x:v>669</x:v>
       </x:c>
       <x:c r="D27" s="9">
         <x:v>1</x:v>
@@ -10641,13 +10636,13 @@
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
       <x:c r="A28" s="8" t="s">
+        <x:v>669</x:v>
+      </x:c>
+      <x:c r="B28" s="7" t="s">
         <x:v>670</x:v>
       </x:c>
-      <x:c r="B28" s="7" t="s">
+      <x:c r="C28" s="7" t="s">
         <x:v>671</x:v>
-      </x:c>
-      <x:c r="C28" s="7" t="s">
-        <x:v>672</x:v>
       </x:c>
       <x:c r="D28" s="9">
         <x:v>2</x:v>
@@ -10656,13 +10651,13 @@
     </x:row>
     <x:row r="29" ht="28" customHeight="1">
       <x:c r="A29" s="8" t="s">
+        <x:v>672</x:v>
+      </x:c>
+      <x:c r="B29" s="7" t="s">
         <x:v>673</x:v>
       </x:c>
-      <x:c r="B29" s="7" t="s">
+      <x:c r="C29" s="7" t="s">
         <x:v>674</x:v>
-      </x:c>
-      <x:c r="C29" s="7" t="s">
-        <x:v>675</x:v>
       </x:c>
       <x:c r="D29" s="9">
         <x:v>4</x:v>
@@ -10671,13 +10666,13 @@
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
       <x:c r="A30" s="8" t="s">
+        <x:v>675</x:v>
+      </x:c>
+      <x:c r="B30" s="7" t="s">
         <x:v>676</x:v>
       </x:c>
-      <x:c r="B30" s="7" t="s">
-        <x:v>677</x:v>
-      </x:c>
       <x:c r="C30" s="7" t="s">
-        <x:v>669</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="D30" s="9">
         <x:v>1</x:v>
@@ -10686,47 +10681,47 @@
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="8" t="s">
+        <x:v>677</x:v>
+      </x:c>
+      <x:c r="B31" s="7" t="s">
         <x:v>678</x:v>
       </x:c>
-      <x:c r="B31" s="7" t="s">
-        <x:v>679</x:v>
-      </x:c>
       <x:c r="C31" s="7" t="s">
-        <x:v>618</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="D31" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E31" s="10" t="s">
-        <x:v>680</x:v>
+        <x:v>679</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="28" customHeight="1">
       <x:c r="A32" s="8" t="s">
+        <x:v>680</x:v>
+      </x:c>
+      <x:c r="B32" s="7" t="s">
         <x:v>681</x:v>
       </x:c>
-      <x:c r="B32" s="7" t="s">
+      <x:c r="C32" s="7" t="s">
         <x:v>682</x:v>
-      </x:c>
-      <x:c r="C32" s="7" t="s">
-        <x:v>683</x:v>
       </x:c>
       <x:c r="D32" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E32" s="10" t="s">
-        <x:v>684</x:v>
+        <x:v>683</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="8" t="s">
+        <x:v>684</x:v>
+      </x:c>
+      <x:c r="B33" s="7" t="s">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="B33" s="7" t="s">
-        <x:v>686</x:v>
-      </x:c>
       <x:c r="C33" s="7" t="s">
-        <x:v>656</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="D33" s="9">
         <x:v>1</x:v>
@@ -10735,13 +10730,13 @@
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
       <x:c r="A34" s="8" t="s">
+        <x:v>686</x:v>
+      </x:c>
+      <x:c r="B34" s="7" t="s">
         <x:v>687</x:v>
       </x:c>
-      <x:c r="B34" s="7" t="s">
+      <x:c r="C34" s="7" t="s">
         <x:v>688</x:v>
-      </x:c>
-      <x:c r="C34" s="7" t="s">
-        <x:v>689</x:v>
       </x:c>
       <x:c r="D34" s="9">
         <x:v>1</x:v>
@@ -10750,47 +10745,47 @@
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
       <x:c r="A35" s="8" t="s">
+        <x:v>689</x:v>
+      </x:c>
+      <x:c r="B35" s="7" t="s">
         <x:v>690</x:v>
       </x:c>
-      <x:c r="B35" s="7" t="s">
+      <x:c r="C35" s="7" t="s">
         <x:v>691</x:v>
-      </x:c>
-      <x:c r="C35" s="7" t="s">
-        <x:v>692</x:v>
       </x:c>
       <x:c r="D35" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E35" s="10" t="s">
-        <x:v>693</x:v>
+        <x:v>692</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
       <x:c r="A36" s="8" t="s">
+        <x:v>693</x:v>
+      </x:c>
+      <x:c r="B36" s="7" t="s">
         <x:v>694</x:v>
       </x:c>
-      <x:c r="B36" s="7" t="s">
+      <x:c r="C36" s="7" t="s">
         <x:v>695</x:v>
-      </x:c>
-      <x:c r="C36" s="7" t="s">
-        <x:v>696</x:v>
       </x:c>
       <x:c r="D36" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E36" s="10" t="s">
-        <x:v>697</x:v>
+        <x:v>696</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
       <x:c r="A37" s="8" t="s">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="B37" s="7" t="s">
         <x:v>698</x:v>
       </x:c>
-      <x:c r="B37" s="7" t="s">
+      <x:c r="C37" s="7" t="s">
         <x:v>699</x:v>
-      </x:c>
-      <x:c r="C37" s="7" t="s">
-        <x:v>700</x:v>
       </x:c>
       <x:c r="D37" s="9">
         <x:v>1</x:v>
@@ -10799,13 +10794,13 @@
     </x:row>
     <x:row r="38" ht="28" customHeight="1">
       <x:c r="A38" s="8" t="s">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="B38" s="7" t="s">
         <x:v>701</x:v>
       </x:c>
-      <x:c r="B38" s="7" t="s">
-        <x:v>702</x:v>
-      </x:c>
       <x:c r="C38" s="7" t="s">
-        <x:v>639</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="D38" s="9">
         <x:v>1</x:v>
@@ -10814,13 +10809,13 @@
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
       <x:c r="A39" s="8" t="s">
+        <x:v>702</x:v>
+      </x:c>
+      <x:c r="B39" s="7" t="s">
         <x:v>703</x:v>
       </x:c>
-      <x:c r="B39" s="7" t="s">
+      <x:c r="C39" s="7" t="s">
         <x:v>704</x:v>
-      </x:c>
-      <x:c r="C39" s="7" t="s">
-        <x:v>705</x:v>
       </x:c>
       <x:c r="D39" s="9">
         <x:v>3</x:v>
@@ -10829,47 +10824,47 @@
     </x:row>
     <x:row r="40" ht="28" customHeight="1">
       <x:c r="A40" s="8" t="s">
+        <x:v>705</x:v>
+      </x:c>
+      <x:c r="B40" s="7" t="s">
         <x:v>706</x:v>
       </x:c>
-      <x:c r="B40" s="7" t="s">
+      <x:c r="C40" s="7" t="s">
         <x:v>707</x:v>
-      </x:c>
-      <x:c r="C40" s="7" t="s">
-        <x:v>708</x:v>
       </x:c>
       <x:c r="D40" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E40" s="10" t="s">
-        <x:v>709</x:v>
+        <x:v>708</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="8" t="s">
+        <x:v>709</x:v>
+      </x:c>
+      <x:c r="B41" s="7" t="s">
         <x:v>710</x:v>
       </x:c>
-      <x:c r="B41" s="7" t="s">
-        <x:v>711</x:v>
-      </x:c>
       <x:c r="C41" s="7" t="s">
-        <x:v>708</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="D41" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E41" s="10" t="s">
-        <x:v>712</x:v>
+        <x:v>711</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
       <x:c r="A42" s="8" t="s">
+        <x:v>712</x:v>
+      </x:c>
+      <x:c r="B42" s="7" t="s">
         <x:v>713</x:v>
       </x:c>
-      <x:c r="B42" s="7" t="s">
+      <x:c r="C42" s="7" t="s">
         <x:v>714</x:v>
-      </x:c>
-      <x:c r="C42" s="7" t="s">
-        <x:v>715</x:v>
       </x:c>
       <x:c r="D42" s="9">
         <x:v>1</x:v>
@@ -10878,10 +10873,10 @@
     </x:row>
     <x:row r="43" ht="28" customHeight="1">
       <x:c r="A43" s="8" t="s">
+        <x:v>715</x:v>
+      </x:c>
+      <x:c r="B43" s="7" t="s">
         <x:v>716</x:v>
-      </x:c>
-      <x:c r="B43" s="7" t="s">
-        <x:v>717</x:v>
       </x:c>
       <x:c r="C43" s="7" t="str">
         <x:v>#069, #079</x:v>
@@ -10893,30 +10888,30 @@
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="8" t="s">
+        <x:v>717</x:v>
+      </x:c>
+      <x:c r="B44" s="7" t="s">
         <x:v>718</x:v>
       </x:c>
-      <x:c r="B44" s="7" t="s">
-        <x:v>719</x:v>
-      </x:c>
       <x:c r="C44" s="7" t="s">
-        <x:v>672</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="D44" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E44" s="10" t="s">
-        <x:v>720</x:v>
+        <x:v>719</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
       <x:c r="A45" s="8" t="s">
+        <x:v>720</x:v>
+      </x:c>
+      <x:c r="B45" s="7" t="s">
         <x:v>721</x:v>
       </x:c>
-      <x:c r="B45" s="7" t="s">
+      <x:c r="C45" s="7" t="s">
         <x:v>722</x:v>
-      </x:c>
-      <x:c r="C45" s="7" t="s">
-        <x:v>723</x:v>
       </x:c>
       <x:c r="D45" s="9">
         <x:v>1</x:v>
@@ -10925,13 +10920,13 @@
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
       <x:c r="A46" s="8" t="s">
+        <x:v>723</x:v>
+      </x:c>
+      <x:c r="B46" s="7" t="s">
         <x:v>724</x:v>
       </x:c>
-      <x:c r="B46" s="7" t="s">
-        <x:v>725</x:v>
-      </x:c>
       <x:c r="C46" s="7" t="s">
-        <x:v>689</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="D46" s="9">
         <x:v>1</x:v>
@@ -10940,47 +10935,47 @@
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
       <x:c r="A47" s="8" t="s">
+        <x:v>725</x:v>
+      </x:c>
+      <x:c r="B47" s="7" t="s">
         <x:v>726</x:v>
       </x:c>
-      <x:c r="B47" s="7" t="s">
-        <x:v>727</x:v>
-      </x:c>
       <x:c r="C47" s="7" t="s">
-        <x:v>601</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="D47" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E47" s="10" t="s">
-        <x:v>728</x:v>
+        <x:v>727</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
       <x:c r="A48" s="8" t="s">
+        <x:v>728</x:v>
+      </x:c>
+      <x:c r="B48" s="7" t="s">
         <x:v>729</x:v>
       </x:c>
-      <x:c r="B48" s="7" t="s">
+      <x:c r="C48" s="7" t="s">
         <x:v>730</x:v>
-      </x:c>
-      <x:c r="C48" s="7" t="s">
-        <x:v>731</x:v>
       </x:c>
       <x:c r="D48" s="9">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="10" t="s">
-        <x:v>732</x:v>
+        <x:v>731</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
       <x:c r="A49" s="8" t="s">
+        <x:v>732</x:v>
+      </x:c>
+      <x:c r="B49" s="7" t="s">
         <x:v>733</x:v>
       </x:c>
-      <x:c r="B49" s="7" t="s">
+      <x:c r="C49" s="7" t="s">
         <x:v>734</x:v>
-      </x:c>
-      <x:c r="C49" s="7" t="s">
-        <x:v>735</x:v>
       </x:c>
       <x:c r="D49" s="9">
         <x:v>1</x:v>
@@ -10989,13 +10984,13 @@
     </x:row>
     <x:row r="50" ht="28" customHeight="1">
       <x:c r="A50" s="8" t="s">
+        <x:v>735</x:v>
+      </x:c>
+      <x:c r="B50" s="7" t="s">
         <x:v>736</x:v>
       </x:c>
-      <x:c r="B50" s="7" t="s">
-        <x:v>737</x:v>
-      </x:c>
       <x:c r="C50" s="7" t="s">
-        <x:v>700</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="D50" s="9">
         <x:v>1</x:v>
@@ -11004,64 +10999,64 @@
     </x:row>
     <x:row r="51" ht="28" customHeight="1">
       <x:c r="A51" s="8" t="s">
+        <x:v>737</x:v>
+      </x:c>
+      <x:c r="B51" s="7" t="s">
         <x:v>738</x:v>
       </x:c>
-      <x:c r="B51" s="7" t="s">
+      <x:c r="C51" s="7" t="s">
         <x:v>739</x:v>
-      </x:c>
-      <x:c r="C51" s="7" t="s">
-        <x:v>740</x:v>
       </x:c>
       <x:c r="D51" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E51" s="10" t="s">
-        <x:v>741</x:v>
+        <x:v>740</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="28" customHeight="1">
       <x:c r="A52" s="8" t="s">
+        <x:v>741</x:v>
+      </x:c>
+      <x:c r="B52" s="7" t="s">
         <x:v>742</x:v>
       </x:c>
-      <x:c r="B52" s="7" t="s">
+      <x:c r="C52" s="7" t="s">
         <x:v>743</x:v>
-      </x:c>
-      <x:c r="C52" s="7" t="s">
-        <x:v>744</x:v>
       </x:c>
       <x:c r="D52" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E52" s="10" t="s">
-        <x:v>745</x:v>
+        <x:v>744</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="28" customHeight="1">
       <x:c r="A53" s="8" t="s">
+        <x:v>745</x:v>
+      </x:c>
+      <x:c r="B53" s="7" t="s">
         <x:v>746</x:v>
       </x:c>
-      <x:c r="B53" s="7" t="s">
+      <x:c r="C53" s="7" t="s">
         <x:v>747</x:v>
-      </x:c>
-      <x:c r="C53" s="7" t="s">
-        <x:v>748</x:v>
       </x:c>
       <x:c r="D53" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E53" s="10" t="s">
-        <x:v>749</x:v>
+        <x:v>748</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="28" customHeight="1">
       <x:c r="A54" s="8" t="s">
+        <x:v>749</x:v>
+      </x:c>
+      <x:c r="B54" s="7" t="s">
         <x:v>750</x:v>
       </x:c>
-      <x:c r="B54" s="7" t="s">
+      <x:c r="C54" s="7" t="s">
         <x:v>751</x:v>
-      </x:c>
-      <x:c r="C54" s="7" t="s">
-        <x:v>752</x:v>
       </x:c>
       <x:c r="D54" s="9">
         <x:v>1</x:v>
@@ -11070,81 +11065,81 @@
     </x:row>
     <x:row r="55" ht="28" customHeight="1">
       <x:c r="A55" s="8" t="s">
+        <x:v>752</x:v>
+      </x:c>
+      <x:c r="B55" s="7" t="s">
         <x:v>753</x:v>
       </x:c>
-      <x:c r="B55" s="7" t="s">
+      <x:c r="C55" s="7" t="s">
         <x:v>754</x:v>
-      </x:c>
-      <x:c r="C55" s="7" t="s">
-        <x:v>755</x:v>
       </x:c>
       <x:c r="D55" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E55" s="10" t="s">
-        <x:v>756</x:v>
+        <x:v>755</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="28" customHeight="1">
       <x:c r="A56" s="8" t="s">
+        <x:v>756</x:v>
+      </x:c>
+      <x:c r="B56" s="7" t="s">
         <x:v>757</x:v>
       </x:c>
-      <x:c r="B56" s="7" t="s">
+      <x:c r="C56" s="7" t="s">
         <x:v>758</x:v>
-      </x:c>
-      <x:c r="C56" s="7" t="s">
-        <x:v>759</x:v>
       </x:c>
       <x:c r="D56" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E56" s="10" t="s">
-        <x:v>760</x:v>
+        <x:v>759</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
       <x:c r="A57" s="8" t="s">
+        <x:v>760</x:v>
+      </x:c>
+      <x:c r="B57" s="7" t="s">
         <x:v>761</x:v>
       </x:c>
-      <x:c r="B57" s="7" t="s">
+      <x:c r="C57" s="7" t="s">
         <x:v>762</x:v>
-      </x:c>
-      <x:c r="C57" s="7" t="s">
-        <x:v>763</x:v>
       </x:c>
       <x:c r="D57" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E57" s="10" t="s">
-        <x:v>764</x:v>
+        <x:v>763</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
       <x:c r="A58" s="8" t="s">
+        <x:v>764</x:v>
+      </x:c>
+      <x:c r="B58" s="7" t="s">
         <x:v>765</x:v>
       </x:c>
-      <x:c r="B58" s="7" t="s">
+      <x:c r="C58" s="7" t="s">
         <x:v>766</x:v>
-      </x:c>
-      <x:c r="C58" s="7" t="s">
-        <x:v>767</x:v>
       </x:c>
       <x:c r="D58" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E58" s="10" t="s">
-        <x:v>768</x:v>
+        <x:v>767</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
       <x:c r="A59" s="8" t="s">
+        <x:v>768</x:v>
+      </x:c>
+      <x:c r="B59" s="7" t="s">
         <x:v>769</x:v>
       </x:c>
-      <x:c r="B59" s="7" t="s">
-        <x:v>770</x:v>
-      </x:c>
       <x:c r="C59" s="7" t="s">
-        <x:v>605</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="D59" s="9">
         <x:v>1</x:v>
@@ -11153,13 +11148,13 @@
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
       <x:c r="A60" s="8" t="s">
+        <x:v>770</x:v>
+      </x:c>
+      <x:c r="B60" s="7" t="s">
         <x:v>771</x:v>
       </x:c>
-      <x:c r="B60" s="7" t="s">
-        <x:v>772</x:v>
-      </x:c>
       <x:c r="C60" s="7" t="s">
-        <x:v>642</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="D60" s="9">
         <x:v>1</x:v>
@@ -11168,13 +11163,13 @@
     </x:row>
     <x:row r="61" ht="28" customHeight="1">
       <x:c r="A61" s="8" t="s">
+        <x:v>772</x:v>
+      </x:c>
+      <x:c r="B61" s="7" t="s">
         <x:v>773</x:v>
       </x:c>
-      <x:c r="B61" s="7" t="s">
-        <x:v>774</x:v>
-      </x:c>
       <x:c r="C61" s="7" t="s">
-        <x:v>626</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="D61" s="9">
         <x:v>1</x:v>
@@ -11183,30 +11178,30 @@
     </x:row>
     <x:row r="62" ht="28" customHeight="1">
       <x:c r="A62" s="8" t="s">
+        <x:v>774</x:v>
+      </x:c>
+      <x:c r="B62" s="7" t="s">
         <x:v>775</x:v>
       </x:c>
-      <x:c r="B62" s="7" t="s">
-        <x:v>776</x:v>
-      </x:c>
       <x:c r="C62" s="7" t="s">
-        <x:v>632</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="D62" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E62" s="10" t="s">
-        <x:v>777</x:v>
+        <x:v>776</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="28" customHeight="1">
       <x:c r="A63" s="8" t="s">
+        <x:v>777</x:v>
+      </x:c>
+      <x:c r="B63" s="7" t="s">
         <x:v>778</x:v>
       </x:c>
-      <x:c r="B63" s="7" t="s">
-        <x:v>779</x:v>
-      </x:c>
       <x:c r="C63" s="7" t="s">
-        <x:v>626</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="D63" s="9">
         <x:v>1</x:v>
@@ -11215,13 +11210,13 @@
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
       <x:c r="A64" s="8" t="s">
+        <x:v>779</x:v>
+      </x:c>
+      <x:c r="B64" s="7" t="s">
         <x:v>780</x:v>
       </x:c>
-      <x:c r="B64" s="7" t="s">
+      <x:c r="C64" s="7" t="s">
         <x:v>781</x:v>
-      </x:c>
-      <x:c r="C64" s="7" t="s">
-        <x:v>782</x:v>
       </x:c>
       <x:c r="D64" s="9">
         <x:v>1</x:v>
@@ -11230,13 +11225,13 @@
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
       <x:c r="A65" s="8" t="s">
+        <x:v>782</x:v>
+      </x:c>
+      <x:c r="B65" s="7" t="s">
         <x:v>783</x:v>
       </x:c>
-      <x:c r="B65" s="7" t="s">
+      <x:c r="C65" s="7" t="s">
         <x:v>784</x:v>
-      </x:c>
-      <x:c r="C65" s="7" t="s">
-        <x:v>785</x:v>
       </x:c>
       <x:c r="D65" s="9">
         <x:v>1</x:v>
@@ -11245,13 +11240,13 @@
     </x:row>
     <x:row r="66" ht="28" customHeight="1">
       <x:c r="A66" s="8" t="s">
+        <x:v>785</x:v>
+      </x:c>
+      <x:c r="B66" s="7" t="s">
         <x:v>786</x:v>
       </x:c>
-      <x:c r="B66" s="7" t="s">
-        <x:v>787</x:v>
-      </x:c>
       <x:c r="C66" s="7" t="s">
-        <x:v>615</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="D66" s="9">
         <x:v>1</x:v>
@@ -11260,47 +11255,47 @@
     </x:row>
     <x:row r="67" ht="28" customHeight="1">
       <x:c r="A67" s="8" t="s">
+        <x:v>787</x:v>
+      </x:c>
+      <x:c r="B67" s="7" t="s">
         <x:v>788</x:v>
       </x:c>
-      <x:c r="B67" s="7" t="s">
-        <x:v>789</x:v>
-      </x:c>
       <x:c r="C67" s="7" t="s">
-        <x:v>767</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="D67" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E67" s="10" t="s">
-        <x:v>790</x:v>
+        <x:v>789</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="28" customHeight="1">
       <x:c r="A68" s="8" t="s">
+        <x:v>790</x:v>
+      </x:c>
+      <x:c r="B68" s="7" t="s">
         <x:v>791</x:v>
       </x:c>
-      <x:c r="B68" s="7" t="s">
-        <x:v>792</x:v>
-      </x:c>
       <x:c r="C68" s="7" t="s">
-        <x:v>642</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="D68" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E68" s="10" t="s">
-        <x:v>793</x:v>
+        <x:v>792</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
       <x:c r="A69" s="8" t="s">
+        <x:v>793</x:v>
+      </x:c>
+      <x:c r="B69" s="7" t="s">
         <x:v>794</x:v>
       </x:c>
-      <x:c r="B69" s="7" t="s">
-        <x:v>795</x:v>
-      </x:c>
       <x:c r="C69" s="7" t="s">
-        <x:v>622</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="D69" s="9">
         <x:v>1</x:v>
@@ -11309,13 +11304,13 @@
     </x:row>
     <x:row r="70" ht="28" customHeight="1">
       <x:c r="A70" s="8" t="s">
+        <x:v>795</x:v>
+      </x:c>
+      <x:c r="B70" s="7" t="s">
         <x:v>796</x:v>
       </x:c>
-      <x:c r="B70" s="7" t="s">
-        <x:v>797</x:v>
-      </x:c>
       <x:c r="C70" s="7" t="s">
-        <x:v>650</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="D70" s="9">
         <x:v>1</x:v>
@@ -11324,13 +11319,13 @@
     </x:row>
     <x:row r="71" ht="28" customHeight="1">
       <x:c r="A71" s="8" t="s">
+        <x:v>797</x:v>
+      </x:c>
+      <x:c r="B71" s="7" t="s">
         <x:v>798</x:v>
       </x:c>
-      <x:c r="B71" s="7" t="s">
+      <x:c r="C71" s="7" t="s">
         <x:v>799</x:v>
-      </x:c>
-      <x:c r="C71" s="7" t="s">
-        <x:v>800</x:v>
       </x:c>
       <x:c r="D71" s="9">
         <x:v>1</x:v>
@@ -11339,64 +11334,64 @@
     </x:row>
     <x:row r="72" ht="28" customHeight="1">
       <x:c r="A72" s="8" t="s">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="B72" s="7" t="s">
         <x:v>801</x:v>
       </x:c>
-      <x:c r="B72" s="7" t="s">
+      <x:c r="C72" s="7" t="s">
         <x:v>802</x:v>
-      </x:c>
-      <x:c r="C72" s="7" t="s">
-        <x:v>803</x:v>
       </x:c>
       <x:c r="D72" s="9">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E72" s="10" t="s">
-        <x:v>804</x:v>
+        <x:v>803</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="28" customHeight="1">
       <x:c r="A73" s="8" t="s">
+        <x:v>804</x:v>
+      </x:c>
+      <x:c r="B73" s="7" t="s">
         <x:v>805</x:v>
       </x:c>
-      <x:c r="B73" s="7" t="s">
+      <x:c r="C73" s="7" t="s">
         <x:v>806</x:v>
-      </x:c>
-      <x:c r="C73" s="7" t="s">
-        <x:v>807</x:v>
       </x:c>
       <x:c r="D73" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E73" s="10" t="s">
-        <x:v>808</x:v>
+        <x:v>807</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="28" customHeight="1">
       <x:c r="A74" s="8" t="s">
+        <x:v>808</x:v>
+      </x:c>
+      <x:c r="B74" s="7" t="s">
         <x:v>809</x:v>
       </x:c>
-      <x:c r="B74" s="7" t="s">
-        <x:v>810</x:v>
-      </x:c>
       <x:c r="C74" s="7" t="s">
-        <x:v>608</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="D74" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E74" s="10" t="s">
-        <x:v>811</x:v>
+        <x:v>810</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="28" customHeight="1">
       <x:c r="A75" s="8" t="s">
+        <x:v>811</x:v>
+      </x:c>
+      <x:c r="B75" s="7" t="s">
         <x:v>812</x:v>
       </x:c>
-      <x:c r="B75" s="7" t="s">
-        <x:v>813</x:v>
-      </x:c>
       <x:c r="C75" s="7" t="s">
-        <x:v>723</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="D75" s="9">
         <x:v>1</x:v>
@@ -11405,64 +11400,64 @@
     </x:row>
     <x:row r="76" ht="28" customHeight="1">
       <x:c r="A76" s="8" t="s">
+        <x:v>813</x:v>
+      </x:c>
+      <x:c r="B76" s="7" t="s">
         <x:v>814</x:v>
       </x:c>
-      <x:c r="B76" s="7" t="s">
-        <x:v>815</x:v>
-      </x:c>
       <x:c r="C76" s="7" t="s">
-        <x:v>692</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="D76" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E76" s="10" t="s">
-        <x:v>816</x:v>
+        <x:v>815</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
       <x:c r="A77" s="8" t="s">
+        <x:v>816</x:v>
+      </x:c>
+      <x:c r="B77" s="7" t="s">
         <x:v>817</x:v>
       </x:c>
-      <x:c r="B77" s="7" t="s">
-        <x:v>818</x:v>
-      </x:c>
       <x:c r="C77" s="7" t="s">
-        <x:v>800</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="D77" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E77" s="10" t="s">
-        <x:v>819</x:v>
+        <x:v>818</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
       <x:c r="A78" s="8" t="s">
+        <x:v>819</x:v>
+      </x:c>
+      <x:c r="B78" s="7" t="s">
         <x:v>820</x:v>
       </x:c>
-      <x:c r="B78" s="7" t="s">
-        <x:v>821</x:v>
-      </x:c>
       <x:c r="C78" s="7" t="s">
-        <x:v>597</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="D78" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E78" s="10" t="s">
-        <x:v>822</x:v>
+        <x:v>821</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="28" customHeight="1">
       <x:c r="A79" s="8" t="s">
+        <x:v>822</x:v>
+      </x:c>
+      <x:c r="B79" s="7" t="s">
         <x:v>823</x:v>
       </x:c>
-      <x:c r="B79" s="7" t="s">
-        <x:v>824</x:v>
-      </x:c>
       <x:c r="C79" s="7" t="s">
-        <x:v>692</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="D79" s="9">
         <x:v>1</x:v>
@@ -11471,24 +11466,24 @@
     </x:row>
     <x:row r="80" ht="28" customHeight="1">
       <x:c r="A80" s="8" t="s">
+        <x:v>824</x:v>
+      </x:c>
+      <x:c r="B80" s="7" t="s">
         <x:v>825</x:v>
       </x:c>
-      <x:c r="B80" s="7" t="s">
+      <x:c r="C80" s="7" t="s">
         <x:v>826</x:v>
-      </x:c>
-      <x:c r="C80" s="7" t="s">
-        <x:v>827</x:v>
       </x:c>
       <x:c r="D80" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E80" s="10" t="s">
-        <x:v>828</x:v>
+        <x:v>827</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="28" customHeight="1">
       <x:c r="A81" s="8" t="s">
-        <x:v>829</x:v>
+        <x:v>828</x:v>
       </x:c>
       <x:c r="B81" s="7" t="s">
         <x:v>170</x:v>
@@ -11500,35 +11495,35 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="E81" s="10" t="s">
-        <x:v>830</x:v>
+        <x:v>829</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="28" customHeight="1">
       <x:c r="A82" s="8" t="s">
+        <x:v>830</x:v>
+      </x:c>
+      <x:c r="B82" s="7" t="s">
         <x:v>831</x:v>
       </x:c>
-      <x:c r="B82" s="7" t="s">
+      <x:c r="C82" s="7" t="s">
         <x:v>832</x:v>
-      </x:c>
-      <x:c r="C82" s="7" t="s">
-        <x:v>833</x:v>
       </x:c>
       <x:c r="D82" s="9">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E82" s="10" t="s">
-        <x:v>834</x:v>
+        <x:v>833</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="28" customHeight="1">
       <x:c r="A83" s="8" t="s">
+        <x:v>834</x:v>
+      </x:c>
+      <x:c r="B83" s="7" t="s">
         <x:v>835</x:v>
       </x:c>
-      <x:c r="B83" s="7" t="s">
-        <x:v>836</x:v>
-      </x:c>
       <x:c r="C83" s="7" t="s">
-        <x:v>615</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="D83" s="9">
         <x:v>1</x:v>
@@ -11537,13 +11532,13 @@
     </x:row>
     <x:row r="84" ht="28" customHeight="1">
       <x:c r="A84" s="8" t="s">
+        <x:v>836</x:v>
+      </x:c>
+      <x:c r="B84" s="7" t="s">
         <x:v>837</x:v>
       </x:c>
-      <x:c r="B84" s="7" t="s">
+      <x:c r="C84" s="7" t="s">
         <x:v>838</x:v>
-      </x:c>
-      <x:c r="C84" s="7" t="s">
-        <x:v>839</x:v>
       </x:c>
       <x:c r="D84" s="9">
         <x:v>1</x:v>
@@ -11552,64 +11547,64 @@
     </x:row>
     <x:row r="85" ht="28" customHeight="1">
       <x:c r="A85" s="8" t="s">
+        <x:v>839</x:v>
+      </x:c>
+      <x:c r="B85" s="7" t="s">
         <x:v>840</x:v>
       </x:c>
-      <x:c r="B85" s="7" t="s">
-        <x:v>841</x:v>
-      </x:c>
       <x:c r="C85" s="7" t="s">
-        <x:v>618</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="D85" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E85" s="10" t="s">
-        <x:v>842</x:v>
+        <x:v>841</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="28" customHeight="1">
       <x:c r="A86" s="8" t="s">
+        <x:v>842</x:v>
+      </x:c>
+      <x:c r="B86" s="7" t="s">
         <x:v>843</x:v>
       </x:c>
-      <x:c r="B86" s="7" t="s">
+      <x:c r="C86" s="7" t="s">
         <x:v>844</x:v>
-      </x:c>
-      <x:c r="C86" s="7" t="s">
-        <x:v>845</x:v>
       </x:c>
       <x:c r="D86" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E86" s="10" t="s">
-        <x:v>846</x:v>
+        <x:v>845</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="28" customHeight="1">
       <x:c r="A87" s="8" t="s">
+        <x:v>846</x:v>
+      </x:c>
+      <x:c r="B87" s="7" t="s">
         <x:v>847</x:v>
       </x:c>
-      <x:c r="B87" s="7" t="s">
+      <x:c r="C87" s="7" t="s">
         <x:v>848</x:v>
-      </x:c>
-      <x:c r="C87" s="7" t="s">
-        <x:v>849</x:v>
       </x:c>
       <x:c r="D87" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E87" s="10" t="s">
-        <x:v>850</x:v>
+        <x:v>849</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="28" customHeight="1">
       <x:c r="A88" s="8" t="s">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="B88" s="7" t="s">
         <x:v>851</x:v>
       </x:c>
-      <x:c r="B88" s="7" t="s">
-        <x:v>852</x:v>
-      </x:c>
       <x:c r="C88" s="7" t="s">
-        <x:v>723</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="D88" s="9">
         <x:v>1</x:v>
@@ -11618,13 +11613,13 @@
     </x:row>
     <x:row r="89" ht="28" customHeight="1">
       <x:c r="A89" s="8" t="s">
+        <x:v>852</x:v>
+      </x:c>
+      <x:c r="B89" s="7" t="s">
         <x:v>853</x:v>
       </x:c>
-      <x:c r="B89" s="7" t="s">
-        <x:v>854</x:v>
-      </x:c>
       <x:c r="C89" s="7" t="s">
-        <x:v>639</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="D89" s="9">
         <x:v>1</x:v>
@@ -11633,30 +11628,30 @@
     </x:row>
     <x:row r="90" ht="28" customHeight="1">
       <x:c r="A90" s="8" t="s">
+        <x:v>854</x:v>
+      </x:c>
+      <x:c r="B90" s="7" t="s">
         <x:v>855</x:v>
       </x:c>
-      <x:c r="B90" s="7" t="s">
-        <x:v>856</x:v>
-      </x:c>
       <x:c r="C90" s="7" t="s">
-        <x:v>767</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="D90" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E90" s="10" t="s">
-        <x:v>857</x:v>
+        <x:v>856</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="28" customHeight="1">
       <x:c r="A91" s="8" t="s">
+        <x:v>857</x:v>
+      </x:c>
+      <x:c r="B91" s="7" t="s">
         <x:v>858</x:v>
       </x:c>
-      <x:c r="B91" s="7" t="s">
+      <x:c r="C91" s="7" t="s">
         <x:v>859</x:v>
-      </x:c>
-      <x:c r="C91" s="7" t="s">
-        <x:v>860</x:v>
       </x:c>
       <x:c r="D91" s="9">
         <x:v>1</x:v>
@@ -11665,30 +11660,30 @@
     </x:row>
     <x:row r="92" ht="28" customHeight="1">
       <x:c r="A92" s="8" t="s">
+        <x:v>860</x:v>
+      </x:c>
+      <x:c r="B92" s="7" t="s">
         <x:v>861</x:v>
       </x:c>
-      <x:c r="B92" s="7" t="s">
+      <x:c r="C92" s="7" t="s">
         <x:v>862</x:v>
-      </x:c>
-      <x:c r="C92" s="7" t="s">
-        <x:v>863</x:v>
       </x:c>
       <x:c r="D92" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E92" s="10" t="s">
-        <x:v>864</x:v>
+        <x:v>863</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="28" customHeight="1">
       <x:c r="A93" s="8" t="s">
+        <x:v>864</x:v>
+      </x:c>
+      <x:c r="B93" s="7" t="s">
         <x:v>865</x:v>
       </x:c>
-      <x:c r="B93" s="7" t="s">
-        <x:v>866</x:v>
-      </x:c>
       <x:c r="C93" s="7" t="s">
-        <x:v>800</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="D93" s="9">
         <x:v>1</x:v>
@@ -11697,30 +11692,30 @@
     </x:row>
     <x:row r="94" ht="28" customHeight="1">
       <x:c r="A94" s="8" t="s">
+        <x:v>866</x:v>
+      </x:c>
+      <x:c r="B94" s="7" t="s">
         <x:v>867</x:v>
       </x:c>
-      <x:c r="B94" s="7" t="s">
-        <x:v>868</x:v>
-      </x:c>
       <x:c r="C94" s="7" t="s">
-        <x:v>692</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="D94" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E94" s="10" t="s">
-        <x:v>869</x:v>
+        <x:v>868</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="28" customHeight="1">
       <x:c r="A95" s="8" t="s">
+        <x:v>869</x:v>
+      </x:c>
+      <x:c r="B95" s="7" t="s">
         <x:v>870</x:v>
       </x:c>
-      <x:c r="B95" s="7" t="s">
-        <x:v>871</x:v>
-      </x:c>
       <x:c r="C95" s="7" t="s">
-        <x:v>689</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="D95" s="9">
         <x:v>1</x:v>
@@ -11729,47 +11724,47 @@
     </x:row>
     <x:row r="96" ht="28" customHeight="1">
       <x:c r="A96" s="8" t="s">
+        <x:v>871</x:v>
+      </x:c>
+      <x:c r="B96" s="7" t="s">
         <x:v>872</x:v>
       </x:c>
-      <x:c r="B96" s="7" t="s">
+      <x:c r="C96" s="7" t="s">
         <x:v>873</x:v>
-      </x:c>
-      <x:c r="C96" s="7" t="s">
-        <x:v>874</x:v>
       </x:c>
       <x:c r="D96" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E96" s="10" t="s">
-        <x:v>875</x:v>
+        <x:v>874</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="28" customHeight="1">
       <x:c r="A97" s="8" t="s">
+        <x:v>875</x:v>
+      </x:c>
+      <x:c r="B97" s="7" t="s">
         <x:v>876</x:v>
       </x:c>
-      <x:c r="B97" s="7" t="s">
-        <x:v>877</x:v>
-      </x:c>
       <x:c r="C97" s="7" t="s">
-        <x:v>839</x:v>
+        <x:v>838</x:v>
       </x:c>
       <x:c r="D97" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E97" s="10" t="s">
-        <x:v>878</x:v>
+        <x:v>877</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="s">
+        <x:v>878</x:v>
+      </x:c>
+      <x:c r="B98" t="s">
         <x:v>879</x:v>
       </x:c>
-      <x:c r="B98" t="s">
+      <x:c r="C98" t="s">
         <x:v>880</x:v>
-      </x:c>
-      <x:c r="C98" t="s">
-        <x:v>881</x:v>
       </x:c>
       <x:c r="D98">
         <x:v>1</x:v>
@@ -11790,12 +11785,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R5bec9333787d4df6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rf81095442d264c4b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rd71cdaf2c33e4e78"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R72925ea18c0c4378"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb88409eab1724c5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce7a530232d8479b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11810,7 +11805,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>882</x:v>
+        <x:v>881</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -12698,7 +12693,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6aa975881dfa40c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd97109cda8264351"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12714,35 +12709,35 @@
   <x:sheetData>
     <x:row r="1" ht="34.75" customHeight="1">
       <x:c r="A1" s="20" t="s">
-        <x:v>883</x:v>
+        <x:v>882</x:v>
       </x:c>
       <x:c r="B1" s="20"/>
       <x:c r="C1" s="20"/>
     </x:row>
     <x:row r="2" ht="45.25" customHeight="1">
       <x:c r="A2" s="21" t="s">
-        <x:v>884</x:v>
+        <x:v>883</x:v>
       </x:c>
       <x:c r="B2" s="21"/>
       <x:c r="C2" s="21"/>
     </x:row>
     <x:row r="4" ht="29.25" customHeight="1">
       <x:c r="A4" s="15" t="s">
+        <x:v>884</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="s">
         <x:v>885</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="s">
+      <x:c r="C4" s="15" t="s">
         <x:v>886</x:v>
-      </x:c>
-      <x:c r="C4" s="15" t="s">
-        <x:v>887</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.75" customHeight="1">
       <x:c r="A5" s="16" t="s">
-        <x:v>306</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="B5" s="16" t="s">
-        <x:v>888</x:v>
+        <x:v>887</x:v>
       </x:c>
       <x:c r="C5" s="17"/>
     </x:row>
@@ -12751,90 +12746,90 @@
         <x:v>168</x:v>
       </x:c>
       <x:c r="B6" s="16" t="s">
-        <x:v>889</x:v>
+        <x:v>888</x:v>
       </x:c>
       <x:c r="C6" s="17"/>
     </x:row>
     <x:row r="7" ht="26.75" customHeight="1">
       <x:c r="A7" s="16" t="s">
-        <x:v>375</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="B7" s="16" t="s">
-        <x:v>890</x:v>
+        <x:v>889</x:v>
       </x:c>
       <x:c r="C7" s="17"/>
     </x:row>
     <x:row r="8" ht="26.75" customHeight="1">
       <x:c r="A8" s="16" t="s">
-        <x:v>450</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="B8" s="16" t="s">
-        <x:v>890</x:v>
+        <x:v>889</x:v>
       </x:c>
       <x:c r="C8" s="17"/>
     </x:row>
     <x:row r="9" ht="26.75" customHeight="1">
       <x:c r="A9" s="16" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B9" s="16" t="s">
-        <x:v>891</x:v>
+        <x:v>890</x:v>
       </x:c>
       <x:c r="C9" s="17"/>
     </x:row>
     <x:row r="10" ht="26.75" customHeight="1">
       <x:c r="A10" s="16" t="s">
-        <x:v>364</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="B10" s="16" t="s">
+        <x:v>891</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="s">
         <x:v>892</x:v>
-      </x:c>
-      <x:c r="C10" s="17" t="s">
-        <x:v>893</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.75" customHeight="1">
       <x:c r="A11" s="16" t="s">
-        <x:v>894</x:v>
+        <x:v>893</x:v>
       </x:c>
       <x:c r="B11" s="16" t="s">
-        <x:v>890</x:v>
+        <x:v>889</x:v>
       </x:c>
       <x:c r="C11" s="17"/>
     </x:row>
     <x:row r="12" ht="26.75" customHeight="1">
       <x:c r="A12" s="16" t="s">
+        <x:v>894</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="s">
         <x:v>895</x:v>
-      </x:c>
-      <x:c r="B12" s="16" t="s">
-        <x:v>896</x:v>
       </x:c>
       <x:c r="C12" s="17"/>
     </x:row>
     <x:row r="13" ht="26.75" customHeight="1">
       <x:c r="A13" s="16" t="s">
-        <x:v>299</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="B13" s="16" t="s">
-        <x:v>889</x:v>
+        <x:v>888</x:v>
       </x:c>
       <x:c r="C13" s="17"/>
     </x:row>
     <x:row r="14" ht="26.75" customHeight="1">
       <x:c r="A14" s="16" t="s">
+        <x:v>896</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="s">
         <x:v>897</x:v>
-      </x:c>
-      <x:c r="B14" s="16" t="s">
-        <x:v>898</x:v>
       </x:c>
       <x:c r="C14" s="17"/>
     </x:row>
     <x:row r="15" ht="26.75" customHeight="1">
       <x:c r="A15" s="16" t="s">
+        <x:v>898</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="s">
         <x:v>899</x:v>
-      </x:c>
-      <x:c r="B15" s="16" t="s">
-        <x:v>900</x:v>
       </x:c>
       <x:c r="C15" s="17"/>
     </x:row>
@@ -12843,7 +12838,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B16" s="16" t="s">
-        <x:v>901</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C16" s="17"/>
     </x:row>
@@ -12852,16 +12847,16 @@
         <x:v>196</x:v>
       </x:c>
       <x:c r="B17" s="16" t="s">
-        <x:v>901</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C17" s="17"/>
     </x:row>
     <x:row r="18" ht="26.75" customHeight="1">
       <x:c r="A18" s="16" t="s">
-        <x:v>401</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="B18" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C18" s="17"/>
     </x:row>
@@ -12870,25 +12865,25 @@
         <x:v>256</x:v>
       </x:c>
       <x:c r="B19" s="16" t="s">
-        <x:v>888</x:v>
+        <x:v>887</x:v>
       </x:c>
       <x:c r="C19" s="17"/>
     </x:row>
     <x:row r="20" ht="26.75" customHeight="1">
       <x:c r="A20" s="16" t="s">
-        <x:v>555</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="B20" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C20" s="17"/>
     </x:row>
     <x:row r="21" ht="26.75" customHeight="1">
       <x:c r="A21" s="16" t="s">
-        <x:v>902</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="B21" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C21" s="17"/>
     </x:row>
@@ -12897,63 +12892,63 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="B22" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C22" s="17"/>
     </x:row>
     <x:row r="23" ht="26.75" customHeight="1">
       <x:c r="A23" s="16" t="s">
+        <x:v>902</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="s">
         <x:v>903</x:v>
-      </x:c>
-      <x:c r="B23" s="16" t="s">
-        <x:v>904</x:v>
       </x:c>
       <x:c r="C23" s="17"/>
     </x:row>
     <x:row r="24" ht="26.75" customHeight="1">
       <x:c r="A24" s="16" t="s">
-        <x:v>905</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="B24" s="16" t="s">
-        <x:v>888</x:v>
+        <x:v>887</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
     </x:row>
     <x:row r="25" ht="26.75" customHeight="1">
       <x:c r="A25" s="16" t="s">
-        <x:v>321</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="B25" s="16" t="s">
-        <x:v>889</x:v>
+        <x:v>888</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
     </x:row>
     <x:row r="26" ht="26.75" customHeight="1">
       <x:c r="A26" s="16" t="s">
-        <x:v>459</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="B26" s="16" t="s">
-        <x:v>889</x:v>
+        <x:v>888</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
     </x:row>
     <x:row r="27" ht="26.75" customHeight="1">
       <x:c r="A27" s="16" t="s">
-        <x:v>548</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="B27" s="16" t="s">
-        <x:v>892</x:v>
+        <x:v>891</x:v>
       </x:c>
       <x:c r="C27" s="17" t="s">
-        <x:v>906</x:v>
+        <x:v>905</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="26.75" customHeight="1">
       <x:c r="A28" s="16" t="s">
-        <x:v>907</x:v>
+        <x:v>906</x:v>
       </x:c>
       <x:c r="B28" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C28" s="17"/>
     </x:row>
@@ -12962,7 +12957,7 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B29" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C29" s="17"/>
     </x:row>
@@ -12971,7 +12966,7 @@
         <x:v>189</x:v>
       </x:c>
       <x:c r="B30" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C30" s="17"/>
     </x:row>
@@ -12980,43 +12975,43 @@
         <x:v>139</x:v>
       </x:c>
       <x:c r="B31" s="16" t="s">
-        <x:v>901</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C31" s="17"/>
     </x:row>
     <x:row r="32" ht="26.75" customHeight="1">
       <x:c r="A32" s="16" t="s">
-        <x:v>543</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="B32" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C32" s="17"/>
     </x:row>
     <x:row r="33" ht="26.75" customHeight="1">
       <x:c r="A33" s="16" t="s">
-        <x:v>908</x:v>
+        <x:v>907</x:v>
       </x:c>
       <x:c r="B33" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C33" s="17"/>
     </x:row>
     <x:row r="34" ht="26.75" customHeight="1">
       <x:c r="A34" s="16" t="s">
-        <x:v>314</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="B34" s="16" t="s">
-        <x:v>890</x:v>
+        <x:v>889</x:v>
       </x:c>
       <x:c r="C34" s="17"/>
     </x:row>
     <x:row r="35" ht="26.75" customHeight="1">
       <x:c r="A35" s="16" t="s">
-        <x:v>499</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="B35" s="16" t="s">
-        <x:v>889</x:v>
+        <x:v>888</x:v>
       </x:c>
       <x:c r="C35" s="17"/>
     </x:row>
@@ -13025,18 +13020,18 @@
         <x:v>264</x:v>
       </x:c>
       <x:c r="B36" s="16" t="s">
+        <x:v>891</x:v>
+      </x:c>
+      <x:c r="C36" s="17" t="s">
         <x:v>892</x:v>
-      </x:c>
-      <x:c r="C36" s="17" t="s">
-        <x:v>893</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="26.75" customHeight="1">
       <x:c r="A37" s="16" t="s">
-        <x:v>909</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="B37" s="16" t="s">
-        <x:v>901</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C37" s="17"/>
     </x:row>
@@ -13045,7 +13040,7 @@
         <x:v>175</x:v>
       </x:c>
       <x:c r="B38" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C38" s="17"/>
     </x:row>
@@ -13054,36 +13049,36 @@
         <x:v>237</x:v>
       </x:c>
       <x:c r="B39" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C39" s="17" t="s">
-        <x:v>910</x:v>
+        <x:v>909</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="26.75" customHeight="1">
       <x:c r="A40" s="16" t="s">
-        <x:v>440</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="B40" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C40" s="17"/>
     </x:row>
     <x:row r="41" ht="26.75" customHeight="1">
       <x:c r="A41" s="16" t="s">
-        <x:v>911</x:v>
+        <x:v>910</x:v>
       </x:c>
       <x:c r="B41" s="16" t="s">
-        <x:v>896</x:v>
+        <x:v>895</x:v>
       </x:c>
       <x:c r="C41" s="17"/>
     </x:row>
     <x:row r="42" ht="26.75" customHeight="1">
       <x:c r="A42" s="16" t="s">
-        <x:v>912</x:v>
+        <x:v>911</x:v>
       </x:c>
       <x:c r="B42" s="16" t="s">
-        <x:v>900</x:v>
+        <x:v>899</x:v>
       </x:c>
       <x:c r="C42" s="17"/>
     </x:row>
@@ -13092,10 +13087,10 @@
         <x:v>222</x:v>
       </x:c>
       <x:c r="B43" s="16" t="s">
+        <x:v>891</x:v>
+      </x:c>
+      <x:c r="C43" s="17" t="s">
         <x:v>892</x:v>
-      </x:c>
-      <x:c r="C43" s="17" t="s">
-        <x:v>893</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="26.75" customHeight="1">
@@ -13103,7 +13098,7 @@
         <x:v>180</x:v>
       </x:c>
       <x:c r="B44" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C44" s="17"/>
     </x:row>
@@ -13112,16 +13107,16 @@
         <x:v>160</x:v>
       </x:c>
       <x:c r="B45" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C45" s="17"/>
     </x:row>
     <x:row r="46" ht="26.75" customHeight="1">
       <x:c r="A46" s="16" t="s">
-        <x:v>913</x:v>
+        <x:v>912</x:v>
       </x:c>
       <x:c r="B46" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C46" s="17"/>
     </x:row>
@@ -13130,19 +13125,19 @@
         <x:v>154</x:v>
       </x:c>
       <x:c r="B47" s="16" t="s">
-        <x:v>891</x:v>
+        <x:v>890</x:v>
       </x:c>
       <x:c r="C47" s="17"/>
     </x:row>
     <x:row r="48" ht="26.75" customHeight="1">
       <x:c r="A48" s="16" t="s">
+        <x:v>913</x:v>
+      </x:c>
+      <x:c r="B48" s="16" t="s">
+        <x:v>891</x:v>
+      </x:c>
+      <x:c r="C48" s="17" t="s">
         <x:v>914</x:v>
-      </x:c>
-      <x:c r="B48" s="16" t="s">
-        <x:v>892</x:v>
-      </x:c>
-      <x:c r="C48" s="17" t="s">
-        <x:v>915</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="26.75" customHeight="1">
@@ -13150,7 +13145,7 @@
         <x:v>282</x:v>
       </x:c>
       <x:c r="B49" s="16" t="s">
-        <x:v>891</x:v>
+        <x:v>890</x:v>
       </x:c>
       <x:c r="C49" s="17"/>
     </x:row>
@@ -13159,16 +13154,16 @@
         <x:v>210</x:v>
       </x:c>
       <x:c r="B50" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C50" s="17"/>
     </x:row>
     <x:row r="51" ht="26.75" customHeight="1">
       <x:c r="A51" s="16" t="s">
-        <x:v>916</x:v>
+        <x:v>915</x:v>
       </x:c>
       <x:c r="B51" s="16" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
       <x:c r="C51" s="17"/>
     </x:row>
@@ -13177,38 +13172,38 @@
         <x:v>230</x:v>
       </x:c>
       <x:c r="B52" s="16" t="s">
-        <x:v>904</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="C52" s="17"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" t="s">
-        <x:v>565</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="B53" t="s">
-        <x:v>375</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="C53" t="s">
-        <x:v>917</x:v>
+        <x:v>916</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" t="s">
-        <x:v>574</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="B54" t="s">
-        <x:v>892</x:v>
+        <x:v>891</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" t="s">
-        <x:v>581</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="B55" t="s">
-        <x:v>890</x:v>
+        <x:v>889</x:v>
       </x:c>
       <x:c r="C55" t="s">
-        <x:v>918</x:v>
+        <x:v>917</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -14513,15 +14508,14 @@
       </x:c>
       <x:c r="C15" s="36" t="str">
         <x:f>Hackathons!AG41</x:f>
-        <x:v>Best Finisher — Novel Hackathon — Trophy</x:v>
+        <x:v>Novel Hackathon Finisher — Trophy</x:v>
       </x:c>
       <x:c r="D15" s="36" t="str">
         <x:f>IF(Hackathons!Q41="","",Hackathons!Q41)</x:f>
-        <x:v>Best Finisher</x:v>
+        <x:v>Novel Hackathon Finisher</x:v>
       </x:c>
       <x:c r="E15" s="36" t="str">
         <x:f>IF(Hackathons!R41="","",Hackathons!R41)</x:f>
-        <x:v>Novel Hackathon</x:v>
       </x:c>
       <x:c r="F15" s="40" t="str">
         <x:f>IF(Hackathons!S41="","",Hackathons!S41)</x:f>
@@ -15554,7 +15548,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8efb733ad37d42d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b1d9ca2e714246"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add assets section to prize summary
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rc03a9f42bf804886"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rc940440fb3034e88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R1e05a5bea69e488d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R6545c99eb3794940"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R25dd41e50fdf4ecd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Re2e051c4937e4720"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rf238c05ba69445bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R1d06d2f5703e4d03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R6683e971badc4a42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R52425019153b4f6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="Rad213280c05d4694"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R182772dca728419f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2777,7 +2777,7 @@
     <x:numFmt numFmtId="200" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="26">
+  <x:fonts count="27">
     <x:font>
       <x:sz val="12"/>
       <x:color theme="1"/>
@@ -2925,8 +2925,13 @@
       <x:color rgb="FF17324D"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF17324D"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="51">
+  <x:fills count="57">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -3178,6 +3183,36 @@
         <x:fgColor rgb="FF2F75B5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F75B5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6F9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -3242,7 +3277,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="215">
+  <x:cellXfs count="237">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3698,6 +3733,46 @@
     <x:xf numFmtId="201" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="20" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="20" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="20" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Hyperlink" xfId="1"/>
@@ -10204,10 +10279,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R86400ab6245b46bb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R52d8145920914c09"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R91989bad373c4cad"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R2b2b25bbb7574864"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rde8d257df8e44b99"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R7ae426f112fb48a3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rd4ee5f9c6e3f4090"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Re4c28be0b7d54f2f"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11785,12 +11860,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rd71cdaf2c33e4e78"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R72925ea18c0c4378"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rbb54174f33834ce8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rf632eb84daf94dc2"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce7a530232d8479b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2a57f04891e4b57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12693,7 +12768,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd97109cda8264351"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dc8382e978c415c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13412,6 +13487,13 @@
       <x:c r="D11" s="63" t="str">
         <x:v>How it is calculated</x:v>
       </x:c>
+      <x:c r="H11" s="217" t="str">
+        <x:v>Assets Collected</x:v>
+      </x:c>
+      <x:c r="I11" s="217"/>
+      <x:c r="J11" s="217"/>
+      <x:c r="K11" s="217"/>
+      <x:c r="L11" s="217"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="64" t="str">
@@ -13427,6 +13509,16 @@
       <x:c r="D12" s="64" t="str">
         <x:v>Cash and vouchers marked Yes</x:v>
       </x:c>
+      <x:c r="H12" s="220" t="str">
+        <x:v>Recorded asset entries</x:v>
+      </x:c>
+      <x:c r="I12" s="220"/>
+      <x:c r="J12" s="225" t="n">
+        <x:f>COUNTIFS(Hackathons!$AA$2:$AA$82,"&lt;&gt;")</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K12" s="225"/>
+      <x:c r="L12" s="225"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="64" t="str">
@@ -13442,6 +13534,16 @@
       <x:c r="D13" s="64" t="str">
         <x:v>Cash and vouchers marked Yes</x:v>
       </x:c>
+      <x:c r="H13" s="220" t="str">
+        <x:v>Trophies collected</x:v>
+      </x:c>
+      <x:c r="I13" s="220"/>
+      <x:c r="J13" s="225" t="n">
+        <x:f>SUM(Hackathons!$AB$2:$AB$82)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K13" s="225"/>
+      <x:c r="L13" s="225"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="64" t="str">
@@ -13457,6 +13559,13 @@
       <x:c r="D14" s="64" t="str">
         <x:v>Non-cash product / API credits</x:v>
       </x:c>
+      <x:c r="H14" s="228" t="str">
+        <x:v>Recorded items</x:v>
+      </x:c>
+      <x:c r="I14" s="228"/>
+      <x:c r="J14" s="228"/>
+      <x:c r="K14" s="228"/>
+      <x:c r="L14" s="228"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="64" t="str">
@@ -13472,6 +13581,14 @@
       <x:c r="D15" s="64" t="str">
         <x:v>Non-cash product / API credits</x:v>
       </x:c>
+      <x:c r="H15" s="232" t="str">
+        <x:f>IF(COUNTIFS(Hackathons!$AA$2:$AA$82,"&lt;&gt;")=0,"None recorded",TEXTJOIN(", ",TRUE,Hackathons!$AA$2:$AA$82))</x:f>
+        <x:v>SmartWatch, Trophy, v0 Sock, Trophy</x:v>
+      </x:c>
+      <x:c r="I15" s="232"/>
+      <x:c r="J15" s="232"/>
+      <x:c r="K15" s="232"/>
+      <x:c r="L15" s="232"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="64" t="str">
@@ -13487,6 +13604,11 @@
       <x:c r="D16" s="64" t="str">
         <x:v>Known subscription value</x:v>
       </x:c>
+      <x:c r="H16" s="232"/>
+      <x:c r="I16" s="232"/>
+      <x:c r="J16" s="232"/>
+      <x:c r="K16" s="232"/>
+      <x:c r="L16" s="232"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="64" t="str">
@@ -13502,6 +13624,13 @@
       <x:c r="D17" s="64" t="str">
         <x:v>Seed funding / grants</x:v>
       </x:c>
+      <x:c r="H17" s="236" t="str">
+        <x:v>Assets remain outside monetary totals until a value is recorded.</x:v>
+      </x:c>
+      <x:c r="I17" s="236"/>
+      <x:c r="J17" s="236"/>
+      <x:c r="K17" s="236"/>
+      <x:c r="L17" s="236"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18"/>
@@ -13645,6 +13774,14 @@
     <x:mergeCell ref="A23:L23"/>
     <x:mergeCell ref="A25:L25"/>
     <x:mergeCell ref="A26:L28"/>
+    <x:mergeCell ref="H11:L11"/>
+    <x:mergeCell ref="H12:I12"/>
+    <x:mergeCell ref="J12:L12"/>
+    <x:mergeCell ref="H13:I13"/>
+    <x:mergeCell ref="J13:L13"/>
+    <x:mergeCell ref="H14:L14"/>
+    <x:mergeCell ref="H15:L16"/>
+    <x:mergeCell ref="H17:L17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -15548,7 +15685,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b1d9ca2e714246"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd18374b675244252"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Itemize hackathon assets in prize summary
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rf238c05ba69445bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R1d06d2f5703e4d03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R6683e971badc4a42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R52425019153b4f6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="Rad213280c05d4694"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R182772dca728419f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rf135fa4f44854e05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R61c23c1ff2c04d6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R0dd743f5d41149b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R5df50614081843e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R997cb46670624eba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R1165191221944385"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2931,7 +2931,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="57">
+  <x:fills count="69">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -3213,6 +3213,66 @@
         <x:fgColor rgb="FFF3F6F9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F75B5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6F9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F75B5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6F9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -3277,7 +3337,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="237">
+  <x:cellXfs count="285">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3773,6 +3833,98 @@
     <x:xf numFmtId="0" fontId="19" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="58" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="20" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="20" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="20" fillId="59" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="26" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="20" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="20" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="20" fillId="65" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="26" fillId="67" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Hyperlink" xfId="1"/>
@@ -10279,10 +10431,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rde8d257df8e44b99"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R7ae426f112fb48a3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rd4ee5f9c6e3f4090"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Re4c28be0b7d54f2f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R198af3399e6d4de7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rc77cade870934880"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rcbfa9e64a57944a3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R63c6082c30954a82"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11860,12 +12012,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rbb54174f33834ce8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rf632eb84daf94dc2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R68a460aa87ea4276"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rd102277c625f458c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2a57f04891e4b57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6adebb72bfec420d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12768,7 +12920,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dc8382e978c415c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44413633340d4248"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13334,9 +13486,9 @@
     <x:col min="5" max="5" width="4" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="4" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="4" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="4" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="4" hidden="0" customWidth="1"/>
   </x:cols>
@@ -13487,13 +13639,13 @@
       <x:c r="D11" s="63" t="str">
         <x:v>How it is calculated</x:v>
       </x:c>
-      <x:c r="H11" s="217" t="str">
+      <x:c r="H11" s="263" t="str">
         <x:v>Assets Collected</x:v>
       </x:c>
-      <x:c r="I11" s="217"/>
-      <x:c r="J11" s="217"/>
-      <x:c r="K11" s="217"/>
-      <x:c r="L11" s="217"/>
+      <x:c r="I11" s="263"/>
+      <x:c r="J11" s="263"/>
+      <x:c r="K11" s="263"/>
+      <x:c r="L11" s="263"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="64" t="str">
@@ -13509,16 +13661,16 @@
       <x:c r="D12" s="64" t="str">
         <x:v>Cash and vouchers marked Yes</x:v>
       </x:c>
-      <x:c r="H12" s="220" t="str">
+      <x:c r="H12" s="266" t="str">
         <x:v>Recorded asset entries</x:v>
       </x:c>
-      <x:c r="I12" s="220"/>
-      <x:c r="J12" s="225" t="n">
+      <x:c r="I12" s="266"/>
+      <x:c r="J12" s="271" t="n">
         <x:f>COUNTIFS(Hackathons!$AA$2:$AA$82,"&lt;&gt;")</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="K12" s="225"/>
-      <x:c r="L12" s="225"/>
+      <x:c r="K12" s="271"/>
+      <x:c r="L12" s="271"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="64" t="str">
@@ -13534,16 +13686,16 @@
       <x:c r="D13" s="64" t="str">
         <x:v>Cash and vouchers marked Yes</x:v>
       </x:c>
-      <x:c r="H13" s="220" t="str">
+      <x:c r="H13" s="266" t="str">
         <x:v>Trophies collected</x:v>
       </x:c>
-      <x:c r="I13" s="220"/>
-      <x:c r="J13" s="225" t="n">
+      <x:c r="I13" s="266"/>
+      <x:c r="J13" s="271" t="n">
         <x:f>SUM(Hackathons!$AB$2:$AB$82)</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K13" s="225"/>
-      <x:c r="L13" s="225"/>
+      <x:c r="K13" s="271"/>
+      <x:c r="L13" s="271"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="64" t="str">
@@ -13559,15 +13711,19 @@
       <x:c r="D14" s="64" t="str">
         <x:v>Non-cash product / API credits</x:v>
       </x:c>
-      <x:c r="H14" s="228" t="str">
-        <x:v>Recorded items</x:v>
-      </x:c>
-      <x:c r="I14" s="228"/>
-      <x:c r="J14" s="228"/>
-      <x:c r="K14" s="228"/>
-      <x:c r="L14" s="228"/>
-    </x:row>
-    <x:row r="15">
+      <x:c r="H14" s="275" t="str">
+        <x:v>Hackathon</x:v>
+      </x:c>
+      <x:c r="I14" s="275" t="str">
+        <x:v>Item</x:v>
+      </x:c>
+      <x:c r="J14" s="275" t="str">
+        <x:v>Trophies</x:v>
+      </x:c>
+      <x:c r="K14"/>
+      <x:c r="L14"/>
+    </x:row>
+    <x:row r="15" ht="36" customHeight="1">
       <x:c r="A15" s="64" t="str">
         <x:v>Credits</x:v>
       </x:c>
@@ -13581,16 +13737,21 @@
       <x:c r="D15" s="64" t="str">
         <x:v>Non-cash product / API credits</x:v>
       </x:c>
-      <x:c r="H15" s="232" t="str">
-        <x:f>IF(COUNTIFS(Hackathons!$AA$2:$AA$82,"&lt;&gt;")=0,"None recorded",TEXTJOIN(", ",TRUE,Hackathons!$AA$2:$AA$82))</x:f>
-        <x:v>SmartWatch, Trophy, v0 Sock, Trophy</x:v>
-      </x:c>
-      <x:c r="I15" s="232"/>
-      <x:c r="J15" s="232"/>
-      <x:c r="K15" s="232"/>
-      <x:c r="L15" s="232"/>
-    </x:row>
-    <x:row r="16">
+      <x:c r="H15" s="279" t="str">
+        <x:f>Hackathons!B5</x:f>
+        <x:v>Fintech Festival Hackathon 2016</x:v>
+      </x:c>
+      <x:c r="I15" s="279" t="str">
+        <x:f>Hackathons!AA5</x:f>
+        <x:v>SmartWatch</x:v>
+      </x:c>
+      <x:c r="J15" s="280" t="str">
+        <x:f>IF(Hackathons!AB5="","",Hackathons!AB5)</x:f>
+      </x:c>
+      <x:c r="K15"/>
+      <x:c r="L15"/>
+    </x:row>
+    <x:row r="16" ht="36" customHeight="1">
       <x:c r="A16" s="64" t="str">
         <x:v>Subscriptions</x:v>
       </x:c>
@@ -13604,13 +13765,22 @@
       <x:c r="D16" s="64" t="str">
         <x:v>Known subscription value</x:v>
       </x:c>
-      <x:c r="H16" s="232"/>
-      <x:c r="I16" s="232"/>
-      <x:c r="J16" s="232"/>
-      <x:c r="K16" s="232"/>
-      <x:c r="L16" s="232"/>
-    </x:row>
-    <x:row r="17">
+      <x:c r="H16" s="279" t="str">
+        <x:f>Hackathons!B41</x:f>
+        <x:v>Sarawak AI Hackathon 2025</x:v>
+      </x:c>
+      <x:c r="I16" s="279" t="str">
+        <x:f>Hackathons!AA41</x:f>
+        <x:v>Trophy</x:v>
+      </x:c>
+      <x:c r="J16" s="280" t="n">
+        <x:f>IF(Hackathons!AB41="","",Hackathons!AB41)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K16"/>
+      <x:c r="L16"/>
+    </x:row>
+    <x:row r="17" ht="36" customHeight="1">
       <x:c r="A17" s="64" t="str">
         <x:v>Funding</x:v>
       </x:c>
@@ -13624,15 +13794,21 @@
       <x:c r="D17" s="64" t="str">
         <x:v>Seed funding / grants</x:v>
       </x:c>
-      <x:c r="H17" s="236" t="str">
-        <x:v>Assets remain outside monetary totals until a value is recorded.</x:v>
-      </x:c>
-      <x:c r="I17" s="236"/>
-      <x:c r="J17" s="236"/>
-      <x:c r="K17" s="236"/>
-      <x:c r="L17" s="236"/>
-    </x:row>
-    <x:row r="18">
+      <x:c r="H17" s="279" t="str">
+        <x:f>Hackathons!B62</x:f>
+        <x:v>Vercel Zero to Agent: Singapore (1 Hr Hackathon) 2026</x:v>
+      </x:c>
+      <x:c r="I17" s="279" t="str">
+        <x:f>Hackathons!AA62</x:f>
+        <x:v>v0 Sock</x:v>
+      </x:c>
+      <x:c r="J17" s="280" t="str">
+        <x:f>IF(Hackathons!AB62="","",Hackathons!AB62)</x:f>
+      </x:c>
+      <x:c r="K17"/>
+      <x:c r="L17"/>
+    </x:row>
+    <x:row r="18" ht="36" customHeight="1">
       <x:c r="A18"/>
       <x:c r="B18"/>
       <x:c r="C18"/>
@@ -13640,14 +13816,30 @@
       <x:c r="E18" s="54"/>
       <x:c r="F18" s="54"/>
       <x:c r="G18" s="54"/>
-      <x:c r="H18" s="54"/>
-      <x:c r="I18" s="54"/>
-      <x:c r="J18" s="54"/>
-      <x:c r="K18" s="54"/>
-      <x:c r="L18" s="54"/>
+      <x:c r="H18" s="279" t="str">
+        <x:f>Hackathons!B80</x:f>
+        <x:v>SG × SWK Friendship AI Business Design Hackathon</x:v>
+      </x:c>
+      <x:c r="I18" s="279" t="str">
+        <x:f>Hackathons!AA80</x:f>
+        <x:v>Trophy</x:v>
+      </x:c>
+      <x:c r="J18" s="280" t="n">
+        <x:f>IF(Hackathons!AB80="","",Hackathons!AB80)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K18"/>
+      <x:c r="L18"/>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19"/>
+      <x:c r="H19" s="284" t="str">
+        <x:v>Assets remain outside monetary totals until a value is recorded.</x:v>
+      </x:c>
+      <x:c r="I19" s="284"/>
+      <x:c r="J19" s="284"/>
+      <x:c r="K19" s="284"/>
+      <x:c r="L19" s="284"/>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="A20" s="178" t="str">
@@ -13770,7 +13962,6 @@
     <x:mergeCell ref="H8:I8"/>
     <x:mergeCell ref="J8:K8"/>
     <x:mergeCell ref="A10:L10"/>
-    <x:mergeCell ref="A18:L18"/>
     <x:mergeCell ref="A23:L23"/>
     <x:mergeCell ref="A25:L25"/>
     <x:mergeCell ref="A26:L28"/>
@@ -13779,9 +13970,7 @@
     <x:mergeCell ref="J12:L12"/>
     <x:mergeCell ref="H13:I13"/>
     <x:mergeCell ref="J13:L13"/>
-    <x:mergeCell ref="H14:L14"/>
-    <x:mergeCell ref="H15:L16"/>
-    <x:mergeCell ref="H17:L17"/>
+    <x:mergeCell ref="H19:L19"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -15685,7 +15874,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd18374b675244252"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76e527c299364fad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add individual prize share normalization
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rf135fa4f44854e05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R61c23c1ff2c04d6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R0dd743f5d41149b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R5df50614081843e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R997cb46670624eba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R1165191221944385"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rc485fa41ca204210"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R1554981277e046ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rf960998e65714767"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R1cf4ef5148e74746"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="Rb5065535bfc446a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Rac4bfb2a84204a19"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2931,7 +2931,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="69">
+  <x:fills count="75">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -3273,6 +3273,36 @@
         <x:fgColor rgb="FFF3F6F9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F75B5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -3337,7 +3367,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="285">
+  <x:cellXfs count="310">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3923,6 +3953,63 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="19" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="21" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="20" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -3985,9 +4072,9 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="PrizeDetailsTable" displayName="PrizeDetailsTable" ref="A4:T28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:T28"/>
-  <x:tableColumns count="20">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="PrizeDetailsTable" displayName="PrizeDetailsTable" ref="A4:X28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:X28"/>
+  <x:tableColumns count="24">
     <x:tableColumn id="1" name="#"/>
     <x:tableColumn id="2" name="Hackathon"/>
     <x:tableColumn id="3" name="Award Summary"/>
@@ -4008,6 +4095,10 @@
     <x:tableColumn id="18" name="Money counted?"/>
     <x:tableColumn id="19" name="Review note"/>
     <x:tableColumn id="20" name="Hackathon Team Members"/>
+    <x:tableColumn id="21" name="Individual Share: Cash"/>
+    <x:tableColumn id="22" name="Individual Share: Credits"/>
+    <x:tableColumn id="23" name="Individual Share: Subscription"/>
+    <x:tableColumn id="24" name="Individual Share: Funding"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -10431,10 +10522,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R198af3399e6d4de7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rc77cade870934880"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rcbfa9e64a57944a3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R63c6082c30954a82"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rae5a31463bf04317"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R422df4d78f76447c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R2798de959e1a4b69"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Rc45f7bfefc0c462a"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12012,12 +12103,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R68a460aa87ea4276"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rd102277c625f458c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Ref9db53484204246"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R82ba7a1bdd55433b"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6adebb72bfec420d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2268f2d8566d4c86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12920,7 +13011,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44413633340d4248"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf356bad273264ec5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13939,6 +14030,202 @@
       <x:c r="A26" s="57" t="str">
         <x:v>1. Update the yellow structured fields on Hackathons (columns S–Y and AE).  2. Record seed funding or grants in columns AC–AD.  3. Keep all values in their original currencies; this dashboard deliberately does not convert currencies.</x:v>
       </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="294" t="str">
+        <x:v>Individual Share (Equal Split)</x:v>
+      </x:c>
+      <x:c r="B30" s="294"/>
+      <x:c r="C30" s="294"/>
+      <x:c r="D30" s="294"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="298" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="B31" s="298" t="str">
+        <x:v>Currency</x:v>
+      </x:c>
+      <x:c r="C31" s="298" t="str">
+        <x:v>Individual amount</x:v>
+      </x:c>
+      <x:c r="D31" s="298" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="300" t="str">
+        <x:v>Cash-equivalent prizes</x:v>
+      </x:c>
+      <x:c r="B32" s="300" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="C32" s="303" t="n">
+        <x:f>SUMIFS('Prize Details'!$U$5:$U$28,'Prize Details'!$G$5:$G$28,B32)</x:f>
+        <x:v>1008.3333333333333</x:v>
+      </x:c>
+      <x:c r="D32" s="300" t="str">
+        <x:v>Team prize ÷ team members</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="300" t="str">
+        <x:v>Cash-equivalent prizes</x:v>
+      </x:c>
+      <x:c r="B33" s="300" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="C33" s="303" t="n">
+        <x:f>SUMIFS('Prize Details'!$U$5:$U$28,'Prize Details'!$G$5:$G$28,B33)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D33" s="300" t="str">
+        <x:v>Team prize ÷ team members</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="300" t="str">
+        <x:v>Credits</x:v>
+      </x:c>
+      <x:c r="B34" s="300" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="C34" s="303" t="n">
+        <x:f>SUMIFS('Prize Details'!$V$5:$V$28,'Prize Details'!$I$5:$I$28,B34)</x:f>
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="D34" s="300" t="str">
+        <x:v>Team credits ÷ team members</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="300" t="str">
+        <x:v>Credits</x:v>
+      </x:c>
+      <x:c r="B35" s="300" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="C35" s="303" t="n">
+        <x:f>SUMIFS('Prize Details'!$V$5:$V$28,'Prize Details'!$I$5:$I$28,B35)</x:f>
+        <x:v>39045.833333333336</x:v>
+      </x:c>
+      <x:c r="D35" s="300" t="str">
+        <x:v>Team credits ÷ team members</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="300" t="str">
+        <x:v>Subscriptions</x:v>
+      </x:c>
+      <x:c r="B36" s="300" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="C36" s="303" t="n">
+        <x:f>SUMIFS('Prize Details'!$W$5:$W$28,'Prize Details'!$L$5:$L$28,B36)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D36" s="300" t="str">
+        <x:v>Team subscription value ÷ team members</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="300" t="str">
+        <x:v>Subscriptions</x:v>
+      </x:c>
+      <x:c r="B37" s="300" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="C37" s="303" t="n">
+        <x:f>SUMIFS('Prize Details'!$W$5:$W$28,'Prize Details'!$L$5:$L$28,B37)</x:f>
+        <x:v>9.75</x:v>
+      </x:c>
+      <x:c r="D37" s="300" t="str">
+        <x:v>Team subscription value ÷ team members</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="300" t="str">
+        <x:v>Funding</x:v>
+      </x:c>
+      <x:c r="B38" s="300" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="C38" s="303" t="n">
+        <x:f>SUMIFS('Prize Details'!$X$5:$X$28,'Prize Details'!$Q$5:$Q$28,B38)</x:f>
+        <x:v>3600</x:v>
+      </x:c>
+      <x:c r="D38" s="300" t="str">
+        <x:v>Team funding ÷ team members</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="300" t="str">
+        <x:v>Funding</x:v>
+      </x:c>
+      <x:c r="B39" s="300" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="C39" s="303" t="n">
+        <x:f>SUMIFS('Prize Details'!$X$5:$X$28,'Prize Details'!$Q$5:$Q$28,B39)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D39" s="300" t="str">
+        <x:v>Team funding ÷ team members</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="294" t="str">
+        <x:v>Your Total Tracked Value</x:v>
+      </x:c>
+      <x:c r="B41" s="294"/>
+      <x:c r="C41" s="294"/>
+      <x:c r="D41" s="294"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="300" t="str">
+        <x:v>Individual value</x:v>
+      </x:c>
+      <x:c r="B42" s="300" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="C42" s="305" t="n">
+        <x:f>SUM(C32,C34,C36,C38)</x:f>
+        <x:v>4993.333333333333</x:v>
+      </x:c>
+      <x:c r="D42" s="300" t="str">
+        <x:v>Cash, credits, subscriptions, funding</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="300" t="str">
+        <x:v>Individual value</x:v>
+      </x:c>
+      <x:c r="B43" s="300" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="C43" s="305" t="n">
+        <x:f>SUM(C33,C35,C37,C39)</x:f>
+        <x:v>39055.583333333336</x:v>
+      </x:c>
+      <x:c r="D43" s="300" t="str">
+        <x:v>Cash, credits, subscriptions, funding</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="24" customHeight="1">
+      <x:c r="A45" s="309" t="str">
+        <x:v>Individual values assume an equal split across comma-delimited team members. Assets and trophies are excluded from these monetary totals.</x:v>
+      </x:c>
+      <x:c r="B45" s="309"/>
+      <x:c r="C45" s="309"/>
+      <x:c r="D45" s="309"/>
+      <x:c r="E45" s="309"/>
+      <x:c r="F45" s="309"/>
+      <x:c r="G45" s="309"/>
+      <x:c r="H45" s="309"/>
+      <x:c r="I45" s="309"/>
+      <x:c r="J45" s="309"/>
+      <x:c r="K45" s="309"/>
+      <x:c r="L45" s="309"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -13971,6 +14258,9 @@
     <x:mergeCell ref="H13:I13"/>
     <x:mergeCell ref="J13:L13"/>
     <x:mergeCell ref="H19:L19"/>
+    <x:mergeCell ref="A30:D30"/>
+    <x:mergeCell ref="A41:D41"/>
+    <x:mergeCell ref="A45:L45"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -14002,17 +14292,21 @@
     <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="16" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="32" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="20" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="20" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="20" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="20" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="207" t="str">
+      <x:c r="A1" s="285" t="str">
         <x:v>Prize Money — Detailed Breakdown</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="106" t="str">
-        <x:v>One row per currently classified award or prize record. Award Summary uses a curated, standardized format; Hackathon Team Members is counted automatically from the comma-delimited Team Members roster.</x:v>
+        <x:v>Team totals are shown first. Individual Share assumes an equal split across the comma-delimited Hackathon Team Members roster.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -14108,6 +14402,18 @@
       <x:c r="T4" s="36" t="str">
         <x:v>Hackathon Team Members</x:v>
       </x:c>
+      <x:c r="U4" s="36" t="str">
+        <x:v>Individual Share: Cash</x:v>
+      </x:c>
+      <x:c r="V4" s="36" t="str">
+        <x:v>Individual Share: Credits</x:v>
+      </x:c>
+      <x:c r="W4" s="36" t="str">
+        <x:v>Individual Share: Subscription</x:v>
+      </x:c>
+      <x:c r="X4" s="36" t="str">
+        <x:v>Individual Share: Funding</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="36" t="n">
@@ -14179,6 +14485,19 @@
         <x:f>IF(Hackathons!AH2="","",Hackathons!AH2)</x:f>
         <x:v>5</x:v>
       </x:c>
+      <x:c r="U5" s="291" t="str">
+        <x:f>IF(OR(F5="",T5=""),"",F5/T5)</x:f>
+      </x:c>
+      <x:c r="V5" s="291" t="str">
+        <x:f>IF(OR(H5="",T5=""),"",H5/T5)</x:f>
+      </x:c>
+      <x:c r="W5" s="291" t="str">
+        <x:f>IF(OR(K5="",T5=""),"",K5/T5)</x:f>
+      </x:c>
+      <x:c r="X5" s="291" t="n">
+        <x:f>IF(OR(P5="",T5=""),"",P5/T5)</x:f>
+        <x:v>3600</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="36" t="n">
@@ -14249,6 +14568,18 @@
         <x:f>IF(Hackathons!AH4="","",Hackathons!AH4)</x:f>
         <x:v>6</x:v>
       </x:c>
+      <x:c r="U6" s="291" t="str">
+        <x:f>IF(OR(F6="",T6=""),"",F6/T6)</x:f>
+      </x:c>
+      <x:c r="V6" s="291" t="str">
+        <x:f>IF(OR(H6="",T6=""),"",H6/T6)</x:f>
+      </x:c>
+      <x:c r="W6" s="291" t="str">
+        <x:f>IF(OR(K6="",T6=""),"",K6/T6)</x:f>
+      </x:c>
+      <x:c r="X6" s="291" t="str">
+        <x:f>IF(OR(P6="",T6=""),"",P6/T6)</x:f>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="36" t="n">
@@ -14323,6 +14654,19 @@
         <x:f>IF(Hackathons!AH5="","",Hackathons!AH5)</x:f>
         <x:v>4</x:v>
       </x:c>
+      <x:c r="U7" s="291" t="str">
+        <x:f>IF(OR(F7="",T7=""),"",F7/T7)</x:f>
+      </x:c>
+      <x:c r="V7" s="291" t="n">
+        <x:f>IF(OR(H7="",T7=""),"",H7/T7)</x:f>
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="W7" s="291" t="str">
+        <x:f>IF(OR(K7="",T7=""),"",K7/T7)</x:f>
+      </x:c>
+      <x:c r="X7" s="291" t="str">
+        <x:f>IF(OR(P7="",T7=""),"",P7/T7)</x:f>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="36" t="n">
@@ -14393,6 +14737,18 @@
         <x:f>IF(Hackathons!AH11="","",Hackathons!AH11)</x:f>
         <x:v>3</x:v>
       </x:c>
+      <x:c r="U8" s="291" t="str">
+        <x:f>IF(OR(F8="",T8=""),"",F8/T8)</x:f>
+      </x:c>
+      <x:c r="V8" s="291" t="str">
+        <x:f>IF(OR(H8="",T8=""),"",H8/T8)</x:f>
+      </x:c>
+      <x:c r="W8" s="291" t="str">
+        <x:f>IF(OR(K8="",T8=""),"",K8/T8)</x:f>
+      </x:c>
+      <x:c r="X8" s="291" t="str">
+        <x:f>IF(OR(P8="",T8=""),"",P8/T8)</x:f>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="36" t="n">
@@ -14465,6 +14821,19 @@
         <x:f>IF(Hackathons!AH15="","",Hackathons!AH15)</x:f>
         <x:v>2</x:v>
       </x:c>
+      <x:c r="U9" s="291" t="n">
+        <x:f>IF(OR(F9="",T9=""),"",F9/T9)</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="V9" s="291" t="str">
+        <x:f>IF(OR(H9="",T9=""),"",H9/T9)</x:f>
+      </x:c>
+      <x:c r="W9" s="291" t="str">
+        <x:f>IF(OR(K9="",T9=""),"",K9/T9)</x:f>
+      </x:c>
+      <x:c r="X9" s="291" t="str">
+        <x:f>IF(OR(P9="",T9=""),"",P9/T9)</x:f>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="36" t="n">
@@ -14536,6 +14905,19 @@
         <x:f>IF(Hackathons!AH18="","",Hackathons!AH18)</x:f>
         <x:v>3</x:v>
       </x:c>
+      <x:c r="U10" s="291" t="n">
+        <x:f>IF(OR(F10="",T10=""),"",F10/T10)</x:f>
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="V10" s="291" t="str">
+        <x:f>IF(OR(H10="",T10=""),"",H10/T10)</x:f>
+      </x:c>
+      <x:c r="W10" s="291" t="str">
+        <x:f>IF(OR(K10="",T10=""),"",K10/T10)</x:f>
+      </x:c>
+      <x:c r="X10" s="291" t="str">
+        <x:f>IF(OR(P10="",T10=""),"",P10/T10)</x:f>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="36" t="n">
@@ -14606,6 +14988,19 @@
       <x:c r="T11" s="39" t="n">
         <x:f>IF(Hackathons!AH26="","",Hackathons!AH26)</x:f>
         <x:v>6</x:v>
+      </x:c>
+      <x:c r="U11" s="291" t="n">
+        <x:f>IF(OR(F11="",T11=""),"",F11/T11)</x:f>
+        <x:v>83.33333333333333</x:v>
+      </x:c>
+      <x:c r="V11" s="291" t="str">
+        <x:f>IF(OR(H11="",T11=""),"",H11/T11)</x:f>
+      </x:c>
+      <x:c r="W11" s="291" t="str">
+        <x:f>IF(OR(K11="",T11=""),"",K11/T11)</x:f>
+      </x:c>
+      <x:c r="X11" s="291" t="str">
+        <x:f>IF(OR(P11="",T11=""),"",P11/T11)</x:f>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -14678,6 +15073,19 @@
         <x:f>IF(Hackathons!AH34="","",Hackathons!AH34)</x:f>
         <x:v>2</x:v>
       </x:c>
+      <x:c r="U12" s="291" t="n">
+        <x:f>IF(OR(F12="",T12=""),"",F12/T12)</x:f>
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="V12" s="291" t="str">
+        <x:f>IF(OR(H12="",T12=""),"",H12/T12)</x:f>
+      </x:c>
+      <x:c r="W12" s="291" t="str">
+        <x:f>IF(OR(K12="",T12=""),"",K12/T12)</x:f>
+      </x:c>
+      <x:c r="X12" s="291" t="str">
+        <x:f>IF(OR(P12="",T12=""),"",P12/T12)</x:f>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="36" t="n">
@@ -14749,6 +15157,19 @@
         <x:f>IF(Hackathons!AH36="","",Hackathons!AH36)</x:f>
         <x:v>4</x:v>
       </x:c>
+      <x:c r="U13" s="291" t="n">
+        <x:f>IF(OR(F13="",T13=""),"",F13/T13)</x:f>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="V13" s="291" t="str">
+        <x:f>IF(OR(H13="",T13=""),"",H13/T13)</x:f>
+      </x:c>
+      <x:c r="W13" s="291" t="str">
+        <x:f>IF(OR(K13="",T13=""),"",K13/T13)</x:f>
+      </x:c>
+      <x:c r="X13" s="291" t="str">
+        <x:f>IF(OR(P13="",T13=""),"",P13/T13)</x:f>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="36" t="n">
@@ -14822,6 +15243,19 @@
         <x:f>IF(Hackathons!AH39="","",Hackathons!AH39)</x:f>
         <x:v>4</x:v>
       </x:c>
+      <x:c r="U14" s="291" t="str">
+        <x:f>IF(OR(F14="",T14=""),"",F14/T14)</x:f>
+      </x:c>
+      <x:c r="V14" s="291" t="str">
+        <x:f>IF(OR(H14="",T14=""),"",H14/T14)</x:f>
+      </x:c>
+      <x:c r="W14" s="291" t="n">
+        <x:f>IF(OR(K14="",T14=""),"",K14/T14)</x:f>
+        <x:v>9.75</x:v>
+      </x:c>
+      <x:c r="X14" s="291" t="str">
+        <x:f>IF(OR(P14="",T14=""),"",P14/T14)</x:f>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="36" t="n">
@@ -14894,6 +15328,18 @@
         <x:f>IF(Hackathons!AH41="","",Hackathons!AH41)</x:f>
         <x:v>2</x:v>
       </x:c>
+      <x:c r="U15" s="291" t="str">
+        <x:f>IF(OR(F15="",T15=""),"",F15/T15)</x:f>
+      </x:c>
+      <x:c r="V15" s="291" t="str">
+        <x:f>IF(OR(H15="",T15=""),"",H15/T15)</x:f>
+      </x:c>
+      <x:c r="W15" s="291" t="str">
+        <x:f>IF(OR(K15="",T15=""),"",K15/T15)</x:f>
+      </x:c>
+      <x:c r="X15" s="291" t="str">
+        <x:f>IF(OR(P15="",T15=""),"",P15/T15)</x:f>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="36" t="n">
@@ -14966,6 +15412,19 @@
         <x:f>IF(Hackathons!AH43="","",Hackathons!AH43)</x:f>
         <x:v>1</x:v>
       </x:c>
+      <x:c r="U16" s="291" t="str">
+        <x:f>IF(OR(F16="",T16=""),"",F16/T16)</x:f>
+      </x:c>
+      <x:c r="V16" s="291" t="n">
+        <x:f>IF(OR(H16="",T16=""),"",H16/T16)</x:f>
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="W16" s="291" t="str">
+        <x:f>IF(OR(K16="",T16=""),"",K16/T16)</x:f>
+      </x:c>
+      <x:c r="X16" s="291" t="str">
+        <x:f>IF(OR(P16="",T16=""),"",P16/T16)</x:f>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="36" t="n">
@@ -15038,6 +15497,19 @@
         <x:f>IF(Hackathons!AH51="","",Hackathons!AH51)</x:f>
         <x:v>3</x:v>
       </x:c>
+      <x:c r="U17" s="291" t="str">
+        <x:f>IF(OR(F17="",T17=""),"",F17/T17)</x:f>
+      </x:c>
+      <x:c r="V17" s="291" t="n">
+        <x:f>IF(OR(H17="",T17=""),"",H17/T17)</x:f>
+        <x:v>333.3333333333333</x:v>
+      </x:c>
+      <x:c r="W17" s="291" t="str">
+        <x:f>IF(OR(K17="",T17=""),"",K17/T17)</x:f>
+      </x:c>
+      <x:c r="X17" s="291" t="str">
+        <x:f>IF(OR(P17="",T17=""),"",P17/T17)</x:f>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="36" t="n">
@@ -15110,6 +15582,19 @@
         <x:f>IF(Hackathons!AH53="","",Hackathons!AH53)</x:f>
         <x:v>3</x:v>
       </x:c>
+      <x:c r="U18" s="291" t="str">
+        <x:f>IF(OR(F18="",T18=""),"",F18/T18)</x:f>
+      </x:c>
+      <x:c r="V18" s="291" t="n">
+        <x:f>IF(OR(H18="",T18=""),"",H18/T18)</x:f>
+        <x:v>166.66666666666666</x:v>
+      </x:c>
+      <x:c r="W18" s="291" t="str">
+        <x:f>IF(OR(K18="",T18=""),"",K18/T18)</x:f>
+      </x:c>
+      <x:c r="X18" s="291" t="str">
+        <x:f>IF(OR(P18="",T18=""),"",P18/T18)</x:f>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="36" t="n">
@@ -15182,6 +15667,19 @@
         <x:f>IF(Hackathons!AH54="","",Hackathons!AH54)</x:f>
         <x:v>3</x:v>
       </x:c>
+      <x:c r="U19" s="291" t="str">
+        <x:f>IF(OR(F19="",T19=""),"",F19/T19)</x:f>
+      </x:c>
+      <x:c r="V19" s="291" t="n">
+        <x:f>IF(OR(H19="",T19=""),"",H19/T19)</x:f>
+        <x:v>166.66666666666666</x:v>
+      </x:c>
+      <x:c r="W19" s="291" t="str">
+        <x:f>IF(OR(K19="",T19=""),"",K19/T19)</x:f>
+      </x:c>
+      <x:c r="X19" s="291" t="str">
+        <x:f>IF(OR(P19="",T19=""),"",P19/T19)</x:f>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="36" t="n">
@@ -15254,6 +15752,19 @@
         <x:f>IF(Hackathons!AH55="","",Hackathons!AH55)</x:f>
         <x:v>3</x:v>
       </x:c>
+      <x:c r="U20" s="291" t="str">
+        <x:f>IF(OR(F20="",T20=""),"",F20/T20)</x:f>
+      </x:c>
+      <x:c r="V20" s="291" t="n">
+        <x:f>IF(OR(H20="",T20=""),"",H20/T20)</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="W20" s="291" t="str">
+        <x:f>IF(OR(K20="",T20=""),"",K20/T20)</x:f>
+      </x:c>
+      <x:c r="X20" s="291" t="str">
+        <x:f>IF(OR(P20="",T20=""),"",P20/T20)</x:f>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="36" t="n">
@@ -15328,6 +15839,20 @@
         <x:f>IF(Hackathons!AH58="","",Hackathons!AH58)</x:f>
         <x:v>1</x:v>
       </x:c>
+      <x:c r="U21" s="291" t="n">
+        <x:f>IF(OR(F21="",T21=""),"",F21/T21)</x:f>
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="V21" s="291" t="n">
+        <x:f>IF(OR(H21="",T21=""),"",H21/T21)</x:f>
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="W21" s="291" t="str">
+        <x:f>IF(OR(K21="",T21=""),"",K21/T21)</x:f>
+      </x:c>
+      <x:c r="X21" s="291" t="str">
+        <x:f>IF(OR(P21="",T21=""),"",P21/T21)</x:f>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="36" t="n">
@@ -15401,6 +15926,19 @@
         <x:f>IF(Hackathons!AH61="","",Hackathons!AH61)</x:f>
         <x:v>1</x:v>
       </x:c>
+      <x:c r="U22" s="291" t="str">
+        <x:f>IF(OR(F22="",T22=""),"",F22/T22)</x:f>
+      </x:c>
+      <x:c r="V22" s="291" t="n">
+        <x:f>IF(OR(H22="",T22=""),"",H22/T22)</x:f>
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="W22" s="291" t="str">
+        <x:f>IF(OR(K22="",T22=""),"",K22/T22)</x:f>
+      </x:c>
+      <x:c r="X22" s="291" t="str">
+        <x:f>IF(OR(P22="",T22=""),"",P22/T22)</x:f>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="36" t="n">
@@ -15473,6 +16011,18 @@
         <x:f>IF(Hackathons!AH62="","",Hackathons!AH62)</x:f>
         <x:v>1</x:v>
       </x:c>
+      <x:c r="U23" s="291" t="str">
+        <x:f>IF(OR(F23="",T23=""),"",F23/T23)</x:f>
+      </x:c>
+      <x:c r="V23" s="291" t="str">
+        <x:f>IF(OR(H23="",T23=""),"",H23/T23)</x:f>
+      </x:c>
+      <x:c r="W23" s="291" t="str">
+        <x:f>IF(OR(K23="",T23=""),"",K23/T23)</x:f>
+      </x:c>
+      <x:c r="X23" s="291" t="str">
+        <x:f>IF(OR(P23="",T23=""),"",P23/T23)</x:f>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="36" t="n">
@@ -15545,6 +16095,19 @@
         <x:f>IF(Hackathons!AH67="","",Hackathons!AH67)</x:f>
         <x:v>2</x:v>
       </x:c>
+      <x:c r="U24" s="291" t="str">
+        <x:f>IF(OR(F24="",T24=""),"",F24/T24)</x:f>
+      </x:c>
+      <x:c r="V24" s="291" t="n">
+        <x:f>IF(OR(H24="",T24=""),"",H24/T24)</x:f>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="W24" s="291" t="str">
+        <x:f>IF(OR(K24="",T24=""),"",K24/T24)</x:f>
+      </x:c>
+      <x:c r="X24" s="291" t="str">
+        <x:f>IF(OR(P24="",T24=""),"",P24/T24)</x:f>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="36" t="n">
@@ -15617,6 +16180,19 @@
         <x:f>IF(Hackathons!AH72="","",Hackathons!AH72)</x:f>
         <x:v>2</x:v>
       </x:c>
+      <x:c r="U25" s="291" t="str">
+        <x:f>IF(OR(F25="",T25=""),"",F25/T25)</x:f>
+      </x:c>
+      <x:c r="V25" s="291" t="n">
+        <x:f>IF(OR(H25="",T25=""),"",H25/T25)</x:f>
+        <x:v>2250</x:v>
+      </x:c>
+      <x:c r="W25" s="291" t="str">
+        <x:f>IF(OR(K25="",T25=""),"",K25/T25)</x:f>
+      </x:c>
+      <x:c r="X25" s="291" t="str">
+        <x:f>IF(OR(P25="",T25=""),"",P25/T25)</x:f>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="36" t="n">
@@ -15690,6 +16266,19 @@
         <x:f>IF(Hackathons!AH76="","",Hackathons!AH76)</x:f>
         <x:v>2</x:v>
       </x:c>
+      <x:c r="U26" s="291" t="str">
+        <x:f>IF(OR(F26="",T26=""),"",F26/T26)</x:f>
+      </x:c>
+      <x:c r="V26" s="291" t="n">
+        <x:f>IF(OR(H26="",T26=""),"",H26/T26)</x:f>
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="W26" s="291" t="str">
+        <x:f>IF(OR(K26="",T26=""),"",K26/T26)</x:f>
+      </x:c>
+      <x:c r="X26" s="291" t="str">
+        <x:f>IF(OR(P26="",T26=""),"",P26/T26)</x:f>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="36" t="n">
@@ -15765,6 +16354,19 @@
         <x:f>IF(Hackathons!AH80="","",Hackathons!AH80)</x:f>
         <x:v>3</x:v>
       </x:c>
+      <x:c r="U27" s="291" t="str">
+        <x:f>IF(OR(F27="",T27=""),"",F27/T27)</x:f>
+      </x:c>
+      <x:c r="V27" s="291" t="n">
+        <x:f>IF(OR(H27="",T27=""),"",H27/T27)</x:f>
+        <x:v>66.66666666666667</x:v>
+      </x:c>
+      <x:c r="W27" s="291" t="str">
+        <x:f>IF(OR(K27="",T27=""),"",K27/T27)</x:f>
+      </x:c>
+      <x:c r="X27" s="291" t="str">
+        <x:f>IF(OR(P27="",T27=""),"",P27/T27)</x:f>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="36" t="n">
@@ -15837,6 +16439,19 @@
       <x:c r="T28" s="39" t="n">
         <x:f>IF(Hackathons!AH81="","",Hackathons!AH81)</x:f>
         <x:v>2</x:v>
+      </x:c>
+      <x:c r="U28" s="291" t="str">
+        <x:f>IF(OR(F28="",T28=""),"",F28/T28)</x:f>
+      </x:c>
+      <x:c r="V28" s="291" t="n">
+        <x:f>IF(OR(H28="",T28=""),"",H28/T28)</x:f>
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="W28" s="291" t="str">
+        <x:f>IF(OR(K28="",T28=""),"",K28/T28)</x:f>
+      </x:c>
+      <x:c r="X28" s="291" t="str">
+        <x:f>IF(OR(P28="",T28=""),"",P28/T28)</x:f>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -15869,12 +16484,12 @@
     <x:mergeCell ref="I3:J3"/>
     <x:mergeCell ref="L3:N3"/>
     <x:mergeCell ref="O3:P3"/>
-    <x:mergeCell ref="A1:T1"/>
-    <x:mergeCell ref="A2:T2"/>
+    <x:mergeCell ref="A1:X1"/>
+    <x:mergeCell ref="A2:X2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76e527c299364fad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d81d6b4bd0e435b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Separate team and individual prize calculations
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rc485fa41ca204210"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R1554981277e046ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rf960998e65714767"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R1cf4ef5148e74746"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="Rb5065535bfc446a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Rac4bfb2a84204a19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R5086a9bf30184a1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R342cd8104a854545"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R4f9f37ef8c3449a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R3ed4ac851b0541b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R3d686e817b3e42ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R69fc5980797f411e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2931,7 +2931,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="75">
+  <x:fills count="83">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -3303,6 +3303,46 @@
         <x:fgColor rgb="FFFFF4CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -3367,7 +3407,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="310">
+  <x:cellXfs count="333">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4011,6 +4051,55 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="19" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="20" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="20" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="20" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="79" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="20" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -4078,27 +4167,27 @@
     <x:tableColumn id="1" name="#"/>
     <x:tableColumn id="2" name="Hackathon"/>
     <x:tableColumn id="3" name="Award Summary"/>
-    <x:tableColumn id="4" name="Award type"/>
-    <x:tableColumn id="5" name="Additional info"/>
-    <x:tableColumn id="6" name="Cash-equivalent amount"/>
-    <x:tableColumn id="7" name="Cash currency"/>
-    <x:tableColumn id="8" name="Credit amount"/>
-    <x:tableColumn id="9" name="Credit currency / units"/>
-    <x:tableColumn id="10" name="Subscription count"/>
-    <x:tableColumn id="11" name="Subscription amount"/>
-    <x:tableColumn id="12" name="Subscription currency"/>
-    <x:tableColumn id="13" name="Other non-cash prize"/>
-    <x:tableColumn id="14" name="Physical asset"/>
-    <x:tableColumn id="15" name="Trophy count"/>
-    <x:tableColumn id="16" name="Funding amount"/>
-    <x:tableColumn id="17" name="Funding currency"/>
-    <x:tableColumn id="18" name="Money counted?"/>
-    <x:tableColumn id="19" name="Review note"/>
-    <x:tableColumn id="20" name="Hackathon Team Members"/>
-    <x:tableColumn id="21" name="Individual Share: Cash"/>
-    <x:tableColumn id="22" name="Individual Share: Credits"/>
-    <x:tableColumn id="23" name="Individual Share: Subscription"/>
-    <x:tableColumn id="24" name="Individual Share: Funding"/>
+    <x:tableColumn id="4" name="Award Type"/>
+    <x:tableColumn id="5" name="Additional Info"/>
+    <x:tableColumn id="6" name="Hackathon Team Members"/>
+    <x:tableColumn id="7" name="Team Cash"/>
+    <x:tableColumn id="8" name="Cash Currency"/>
+    <x:tableColumn id="9" name="Individual Cash"/>
+    <x:tableColumn id="10" name="Team Credits"/>
+    <x:tableColumn id="11" name="Credit Currency / Units"/>
+    <x:tableColumn id="12" name="Individual Credits"/>
+    <x:tableColumn id="13" name="Subscription Count"/>
+    <x:tableColumn id="14" name="Team Subscription Value"/>
+    <x:tableColumn id="15" name="Subscription Currency"/>
+    <x:tableColumn id="16" name="Individual Subscription Value"/>
+    <x:tableColumn id="17" name="Team Funding"/>
+    <x:tableColumn id="18" name="Funding Currency"/>
+    <x:tableColumn id="19" name="Individual Funding"/>
+    <x:tableColumn id="20" name="Other Non-cash Prize"/>
+    <x:tableColumn id="21" name="Physical Asset"/>
+    <x:tableColumn id="22" name="Trophy Count"/>
+    <x:tableColumn id="23" name="Money Counted?"/>
+    <x:tableColumn id="24" name="Review Note"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -10522,10 +10611,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rae5a31463bf04317"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="R422df4d78f76447c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R2798de959e1a4b69"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Rc45f7bfefc0c462a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R7d42d3f8c83f45ef"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Ra45910a294814618"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R94bef50221ac4675"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R8e17481ca8ce412b"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12103,12 +12192,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Ref9db53484204246"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R82ba7a1bdd55433b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rf30cf03179bb42d1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R9288beee155f4f8c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2268f2d8566d4c86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3ed47fb0b6a48bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13011,7 +13100,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf356bad273264ec5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R032838a9ec4d4766"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13580,8 +13669,8 @@
     <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="4" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="4" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -13948,11 +14037,13 @@
       <x:c r="E20"/>
       <x:c r="F20"/>
       <x:c r="G20"/>
-      <x:c r="H20"/>
-      <x:c r="I20"/>
-      <x:c r="J20"/>
-      <x:c r="K20"/>
-      <x:c r="L20"/>
+      <x:c r="H20" s="330" t="str">
+        <x:v>Individual Total (Equal Split)</x:v>
+      </x:c>
+      <x:c r="I20" s="330"/>
+      <x:c r="J20" s="330"/>
+      <x:c r="K20" s="330"/>
+      <x:c r="L20" s="330"/>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="A21" s="181" t="str">
@@ -13970,11 +14061,18 @@
       </x:c>
       <x:c r="E21"/>
       <x:c r="F21"/>
-      <x:c r="H21"/>
-      <x:c r="I21"/>
-      <x:c r="J21"/>
-      <x:c r="K21"/>
-      <x:c r="L21"/>
+      <x:c r="H21" s="331" t="str">
+        <x:v>Individual tracked value</x:v>
+      </x:c>
+      <x:c r="I21" s="331"/>
+      <x:c r="J21" s="331" t="str">
+        <x:v>SGD</x:v>
+      </x:c>
+      <x:c r="K21" s="332" t="n">
+        <x:f>SUMIFS('Prize Details'!$I$5:$I$28,'Prize Details'!$H$5:$H$28,J21)+SUMIFS('Prize Details'!$L$5:$L$28,'Prize Details'!$K$5:$K$28,J21)+SUMIFS('Prize Details'!$P$5:$P$28,'Prize Details'!$O$5:$O$28,J21)+SUMIFS('Prize Details'!$S$5:$S$28,'Prize Details'!$R$5:$R$28,J21)</x:f>
+        <x:v>4993.333333333333</x:v>
+      </x:c>
+      <x:c r="L21" s="332"/>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
       <x:c r="A22" s="181" t="str">
@@ -13990,6 +14088,16 @@
       <x:c r="D22" s="181" t="str">
         <x:v>Cash, credits, subscriptions, funding</x:v>
       </x:c>
+      <x:c r="H22" s="331"/>
+      <x:c r="I22" s="331"/>
+      <x:c r="J22" s="331" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="K22" s="332" t="n">
+        <x:f>SUMIFS('Prize Details'!$I$5:$I$28,'Prize Details'!$H$5:$H$28,J22)+SUMIFS('Prize Details'!$L$5:$L$28,'Prize Details'!$K$5:$K$28,J22)+SUMIFS('Prize Details'!$P$5:$P$28,'Prize Details'!$O$5:$O$28,J22)+SUMIFS('Prize Details'!$S$5:$S$28,'Prize Details'!$R$5:$R$28,J22)</x:f>
+        <x:v>39055.583333333336</x:v>
+      </x:c>
+      <x:c r="L22" s="332"/>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
       <x:c r="A23" s="189" t="str">
@@ -14028,204 +14136,100 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="57" t="str">
-        <x:v>1. Update the yellow structured fields on Hackathons (columns S–Y and AE).  2. Record seed funding or grants in columns AC–AD.  3. Keep all values in their original currencies; this dashboard deliberately does not convert currencies.</x:v>
+        <x:v>1. Update the yellow structured fields on Hackathons (columns S–Y and AE).  2. Record seed funding or grants in columns AC–AD.  3. Individual totals are calculated from Prize Details using the hackathon team roster.  4. Keep all values in their original currencies; this dashboard does not convert currencies.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="294" t="str">
-        <x:v>Individual Share (Equal Split)</x:v>
-      </x:c>
-      <x:c r="B30" s="294"/>
-      <x:c r="C30" s="294"/>
-      <x:c r="D30" s="294"/>
+      <x:c r="A30"/>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="298" t="str">
-        <x:v>Category</x:v>
-      </x:c>
-      <x:c r="B31" s="298" t="str">
-        <x:v>Currency</x:v>
-      </x:c>
-      <x:c r="C31" s="298" t="str">
-        <x:v>Individual amount</x:v>
-      </x:c>
-      <x:c r="D31" s="298" t="str">
-        <x:v>Method</x:v>
-      </x:c>
+      <x:c r="A31"/>
+      <x:c r="B31"/>
+      <x:c r="C31"/>
+      <x:c r="D31"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="300" t="str">
-        <x:v>Cash-equivalent prizes</x:v>
-      </x:c>
-      <x:c r="B32" s="300" t="str">
-        <x:v>SGD</x:v>
-      </x:c>
-      <x:c r="C32" s="303" t="n">
-        <x:f>SUMIFS('Prize Details'!$U$5:$U$28,'Prize Details'!$G$5:$G$28,B32)</x:f>
-        <x:v>1008.3333333333333</x:v>
-      </x:c>
-      <x:c r="D32" s="300" t="str">
-        <x:v>Team prize ÷ team members</x:v>
-      </x:c>
+      <x:c r="A32"/>
+      <x:c r="B32"/>
+      <x:c r="C32"/>
+      <x:c r="D32"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="300" t="str">
-        <x:v>Cash-equivalent prizes</x:v>
-      </x:c>
-      <x:c r="B33" s="300" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="C33" s="303" t="n">
-        <x:f>SUMIFS('Prize Details'!$U$5:$U$28,'Prize Details'!$G$5:$G$28,B33)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D33" s="300" t="str">
-        <x:v>Team prize ÷ team members</x:v>
-      </x:c>
+      <x:c r="A33"/>
+      <x:c r="B33"/>
+      <x:c r="C33"/>
+      <x:c r="D33"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="300" t="str">
-        <x:v>Credits</x:v>
-      </x:c>
-      <x:c r="B34" s="300" t="str">
-        <x:v>SGD</x:v>
-      </x:c>
-      <x:c r="C34" s="303" t="n">
-        <x:f>SUMIFS('Prize Details'!$V$5:$V$28,'Prize Details'!$I$5:$I$28,B34)</x:f>
-        <x:v>385</x:v>
-      </x:c>
-      <x:c r="D34" s="300" t="str">
-        <x:v>Team credits ÷ team members</x:v>
-      </x:c>
+      <x:c r="A34"/>
+      <x:c r="B34"/>
+      <x:c r="C34"/>
+      <x:c r="D34"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="300" t="str">
-        <x:v>Credits</x:v>
-      </x:c>
-      <x:c r="B35" s="300" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="C35" s="303" t="n">
-        <x:f>SUMIFS('Prize Details'!$V$5:$V$28,'Prize Details'!$I$5:$I$28,B35)</x:f>
-        <x:v>39045.833333333336</x:v>
-      </x:c>
-      <x:c r="D35" s="300" t="str">
-        <x:v>Team credits ÷ team members</x:v>
-      </x:c>
+      <x:c r="A35"/>
+      <x:c r="B35"/>
+      <x:c r="C35"/>
+      <x:c r="D35"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="300" t="str">
-        <x:v>Subscriptions</x:v>
-      </x:c>
-      <x:c r="B36" s="300" t="str">
-        <x:v>SGD</x:v>
-      </x:c>
-      <x:c r="C36" s="303" t="n">
-        <x:f>SUMIFS('Prize Details'!$W$5:$W$28,'Prize Details'!$L$5:$L$28,B36)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D36" s="300" t="str">
-        <x:v>Team subscription value ÷ team members</x:v>
-      </x:c>
+      <x:c r="A36"/>
+      <x:c r="B36"/>
+      <x:c r="C36"/>
+      <x:c r="D36"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="300" t="str">
-        <x:v>Subscriptions</x:v>
-      </x:c>
-      <x:c r="B37" s="300" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="C37" s="303" t="n">
-        <x:f>SUMIFS('Prize Details'!$W$5:$W$28,'Prize Details'!$L$5:$L$28,B37)</x:f>
-        <x:v>9.75</x:v>
-      </x:c>
-      <x:c r="D37" s="300" t="str">
-        <x:v>Team subscription value ÷ team members</x:v>
-      </x:c>
+      <x:c r="A37"/>
+      <x:c r="B37"/>
+      <x:c r="C37"/>
+      <x:c r="D37"/>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="300" t="str">
-        <x:v>Funding</x:v>
-      </x:c>
-      <x:c r="B38" s="300" t="str">
-        <x:v>SGD</x:v>
-      </x:c>
-      <x:c r="C38" s="303" t="n">
-        <x:f>SUMIFS('Prize Details'!$X$5:$X$28,'Prize Details'!$Q$5:$Q$28,B38)</x:f>
-        <x:v>3600</x:v>
-      </x:c>
-      <x:c r="D38" s="300" t="str">
-        <x:v>Team funding ÷ team members</x:v>
-      </x:c>
+      <x:c r="A38"/>
+      <x:c r="B38"/>
+      <x:c r="C38"/>
+      <x:c r="D38"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="300" t="str">
-        <x:v>Funding</x:v>
-      </x:c>
-      <x:c r="B39" s="300" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="C39" s="303" t="n">
-        <x:f>SUMIFS('Prize Details'!$X$5:$X$28,'Prize Details'!$Q$5:$Q$28,B39)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D39" s="300" t="str">
-        <x:v>Team funding ÷ team members</x:v>
-      </x:c>
+      <x:c r="A39"/>
+      <x:c r="B39"/>
+      <x:c r="C39"/>
+      <x:c r="D39"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="294" t="str">
-        <x:v>Your Total Tracked Value</x:v>
-      </x:c>
-      <x:c r="B41" s="294"/>
-      <x:c r="C41" s="294"/>
-      <x:c r="D41" s="294"/>
+      <x:c r="A41"/>
+      <x:c r="B41"/>
+      <x:c r="C41"/>
+      <x:c r="D41"/>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="300" t="str">
-        <x:v>Individual value</x:v>
-      </x:c>
-      <x:c r="B42" s="300" t="str">
-        <x:v>SGD</x:v>
-      </x:c>
-      <x:c r="C42" s="305" t="n">
-        <x:f>SUM(C32,C34,C36,C38)</x:f>
-        <x:v>4993.333333333333</x:v>
-      </x:c>
-      <x:c r="D42" s="300" t="str">
-        <x:v>Cash, credits, subscriptions, funding</x:v>
-      </x:c>
+      <x:c r="A42"/>
+      <x:c r="B42"/>
+      <x:c r="C42"/>
+      <x:c r="D42"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="300" t="str">
-        <x:v>Individual value</x:v>
-      </x:c>
-      <x:c r="B43" s="300" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="C43" s="305" t="n">
-        <x:f>SUM(C33,C35,C37,C39)</x:f>
-        <x:v>39055.583333333336</x:v>
-      </x:c>
-      <x:c r="D43" s="300" t="str">
-        <x:v>Cash, credits, subscriptions, funding</x:v>
-      </x:c>
+      <x:c r="A43"/>
+      <x:c r="B43"/>
+      <x:c r="C43"/>
+      <x:c r="D43"/>
     </x:row>
     <x:row r="45" ht="24" customHeight="1">
-      <x:c r="A45" s="309" t="str">
-        <x:v>Individual values assume an equal split across comma-delimited team members. Assets and trophies are excluded from these monetary totals.</x:v>
-      </x:c>
-      <x:c r="B45" s="309"/>
-      <x:c r="C45" s="309"/>
-      <x:c r="D45" s="309"/>
-      <x:c r="E45" s="309"/>
-      <x:c r="F45" s="309"/>
-      <x:c r="G45" s="309"/>
-      <x:c r="H45" s="309"/>
-      <x:c r="I45" s="309"/>
-      <x:c r="J45" s="309"/>
-      <x:c r="K45" s="309"/>
-      <x:c r="L45" s="309"/>
+      <x:c r="A45"/>
+      <x:c r="B45"/>
+      <x:c r="C45"/>
+      <x:c r="D45"/>
+      <x:c r="E45"/>
+      <x:c r="F45"/>
+      <x:c r="G45"/>
+      <x:c r="H45"/>
+      <x:c r="I45"/>
+      <x:c r="J45"/>
+      <x:c r="K45"/>
+      <x:c r="L45"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -14258,9 +14262,10 @@
     <x:mergeCell ref="H13:I13"/>
     <x:mergeCell ref="J13:L13"/>
     <x:mergeCell ref="H19:L19"/>
-    <x:mergeCell ref="A30:D30"/>
-    <x:mergeCell ref="A41:D41"/>
-    <x:mergeCell ref="A45:L45"/>
+    <x:mergeCell ref="H20:L20"/>
+    <x:mergeCell ref="H21:I22"/>
+    <x:mergeCell ref="K21:L21"/>
+    <x:mergeCell ref="K22:L22"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -14276,37 +14281,37 @@
     <x:col min="1" max="1" width="7" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="32" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="14" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="16" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="32" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="22" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="16" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="18" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="32" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="20" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="20" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="20" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="20" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="14" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="16" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="32" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="285" t="str">
-        <x:v>Prize Money — Detailed Breakdown</x:v>
+      <x:c r="A1" s="325" t="str">
+        <x:v>Prize Details — Team Totals and Individual Share</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="106" t="str">
-        <x:v>Team totals are shown first. Individual Share assumes an equal split across the comma-delimited Hackathon Team Members roster.</x:v>
+        <x:v>Individual Share = Team total ÷ Hackathon Team Members. Currencies remain separate and all values are linked to Hackathons.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -14352,67 +14357,67 @@
         <x:v>Award Summary</x:v>
       </x:c>
       <x:c r="D4" s="36" t="str">
-        <x:v>Award type</x:v>
+        <x:v>Award Type</x:v>
       </x:c>
       <x:c r="E4" s="36" t="str">
-        <x:v>Additional info</x:v>
+        <x:v>Additional Info</x:v>
       </x:c>
       <x:c r="F4" s="36" t="str">
-        <x:v>Cash-equivalent amount</x:v>
+        <x:v>Hackathon Team Members</x:v>
       </x:c>
       <x:c r="G4" s="36" t="str">
-        <x:v>Cash currency</x:v>
+        <x:v>Team Cash</x:v>
       </x:c>
       <x:c r="H4" s="36" t="str">
-        <x:v>Credit amount</x:v>
+        <x:v>Cash Currency</x:v>
       </x:c>
       <x:c r="I4" s="36" t="str">
-        <x:v>Credit currency / units</x:v>
+        <x:v>Individual Cash</x:v>
       </x:c>
       <x:c r="J4" s="36" t="str">
-        <x:v>Subscription count</x:v>
+        <x:v>Team Credits</x:v>
       </x:c>
       <x:c r="K4" s="36" t="str">
-        <x:v>Subscription amount</x:v>
+        <x:v>Credit Currency / Units</x:v>
       </x:c>
       <x:c r="L4" s="36" t="str">
-        <x:v>Subscription currency</x:v>
+        <x:v>Individual Credits</x:v>
       </x:c>
       <x:c r="M4" s="36" t="str">
-        <x:v>Other non-cash prize</x:v>
+        <x:v>Subscription Count</x:v>
       </x:c>
       <x:c r="N4" s="36" t="str">
-        <x:v>Physical asset</x:v>
+        <x:v>Team Subscription Value</x:v>
       </x:c>
       <x:c r="O4" s="36" t="str">
-        <x:v>Trophy count</x:v>
+        <x:v>Subscription Currency</x:v>
       </x:c>
       <x:c r="P4" s="36" t="str">
-        <x:v>Funding amount</x:v>
+        <x:v>Individual Subscription Value</x:v>
       </x:c>
       <x:c r="Q4" s="36" t="str">
-        <x:v>Funding currency</x:v>
+        <x:v>Team Funding</x:v>
       </x:c>
       <x:c r="R4" s="36" t="str">
-        <x:v>Money counted?</x:v>
+        <x:v>Funding Currency</x:v>
       </x:c>
       <x:c r="S4" s="36" t="str">
-        <x:v>Review note</x:v>
+        <x:v>Individual Funding</x:v>
       </x:c>
       <x:c r="T4" s="36" t="str">
-        <x:v>Hackathon Team Members</x:v>
+        <x:v>Other Non-cash Prize</x:v>
       </x:c>
       <x:c r="U4" s="36" t="str">
-        <x:v>Individual Share: Cash</x:v>
+        <x:v>Physical Asset</x:v>
       </x:c>
       <x:c r="V4" s="36" t="str">
-        <x:v>Individual Share: Credits</x:v>
+        <x:v>Trophy Count</x:v>
       </x:c>
       <x:c r="W4" s="36" t="str">
-        <x:v>Individual Share: Subscription</x:v>
+        <x:v>Money Counted?</x:v>
       </x:c>
       <x:c r="X4" s="36" t="str">
-        <x:v>Individual Share: Funding</x:v>
+        <x:v>Review Note</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -14435,68 +14440,68 @@
       <x:c r="E5" s="36" t="str">
         <x:f>IF(Hackathons!R2="","",Hackathons!R2)</x:f>
       </x:c>
-      <x:c r="F5" s="40" t="str">
+      <x:c r="F5" s="36" t="n">
+        <x:f>IF(Hackathons!AH2="","",Hackathons!AH2)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G5" s="40" t="str">
         <x:f>IF(Hackathons!S2="","",Hackathons!S2)</x:f>
       </x:c>
-      <x:c r="G5" s="36" t="str">
+      <x:c r="H5" s="36" t="str">
         <x:f>IF(Hackathons!T2="","",Hackathons!T2)</x:f>
       </x:c>
-      <x:c r="H5" s="40" t="str">
+      <x:c r="I5" s="329" t="str">
+        <x:f>IF(OR(G5="",F5=""),"",G5/F5)</x:f>
+      </x:c>
+      <x:c r="J5" s="40" t="str">
         <x:f>IF(Hackathons!U2="","",Hackathons!U2)</x:f>
       </x:c>
-      <x:c r="I5" s="36" t="str">
+      <x:c r="K5" s="36" t="str">
         <x:f>IF(Hackathons!V2="","",Hackathons!V2)</x:f>
       </x:c>
-      <x:c r="J5" s="39" t="str">
+      <x:c r="L5" s="329" t="str">
+        <x:f>IF(OR(J5="",F5=""),"",J5/F5)</x:f>
+      </x:c>
+      <x:c r="M5" s="39" t="str">
         <x:f>IF(Hackathons!W2="","",Hackathons!W2)</x:f>
       </x:c>
-      <x:c r="K5" s="40" t="str">
+      <x:c r="N5" s="40" t="str">
         <x:f>IF(Hackathons!X2="","",Hackathons!X2)</x:f>
       </x:c>
-      <x:c r="L5" s="36" t="str">
+      <x:c r="O5" s="36" t="str">
         <x:f>IF(Hackathons!Y2="","",Hackathons!Y2)</x:f>
       </x:c>
-      <x:c r="M5" s="36" t="str">
-        <x:f>IF(Hackathons!Z2="","",Hackathons!Z2)</x:f>
-      </x:c>
-      <x:c r="N5" s="36" t="str">
-        <x:f>IF(Hackathons!AA2="","",Hackathons!AA2)</x:f>
-      </x:c>
-      <x:c r="O5" s="39" t="str">
-        <x:f>IF(Hackathons!AB2="","",Hackathons!AB2)</x:f>
-      </x:c>
-      <x:c r="P5" s="40" t="n">
+      <x:c r="P5" s="329" t="str">
+        <x:f>IF(OR(N5="",F5=""),"",N5/F5)</x:f>
+      </x:c>
+      <x:c r="Q5" s="40" t="n">
         <x:f>IF(Hackathons!AC2="","",Hackathons!AC2)</x:f>
         <x:v>18000</x:v>
       </x:c>
-      <x:c r="Q5" s="36" t="str">
+      <x:c r="R5" s="36" t="str">
         <x:f>IF(Hackathons!AD2="","",Hackathons!AD2)</x:f>
         <x:v>SGD</x:v>
       </x:c>
-      <x:c r="R5" s="36" t="str">
+      <x:c r="S5" s="329" t="n">
+        <x:f>IF(OR(Q5="",F5=""),"",Q5/F5)</x:f>
+        <x:v>3600</x:v>
+      </x:c>
+      <x:c r="T5" s="36" t="str">
+        <x:f>IF(Hackathons!Z2="","",Hackathons!Z2)</x:f>
+      </x:c>
+      <x:c r="U5" s="36" t="str">
+        <x:f>IF(Hackathons!AA2="","",Hackathons!AA2)</x:f>
+      </x:c>
+      <x:c r="V5" s="39" t="str">
+        <x:f>IF(Hackathons!AB2="","",Hackathons!AB2)</x:f>
+      </x:c>
+      <x:c r="W5" s="36" t="str">
         <x:f>IF(Hackathons!AE2="","",Hackathons!AE2)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S5" s="36" t="str">
+      <x:c r="X5" s="36" t="str">
         <x:f>IF(Hackathons!AF2="","",Hackathons!AF2)</x:f>
         <x:v>Funding, not a cash prize</x:v>
-      </x:c>
-      <x:c r="T5" s="39" t="n">
-        <x:f>IF(Hackathons!AH2="","",Hackathons!AH2)</x:f>
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="U5" s="291" t="str">
-        <x:f>IF(OR(F5="",T5=""),"",F5/T5)</x:f>
-      </x:c>
-      <x:c r="V5" s="291" t="str">
-        <x:f>IF(OR(H5="",T5=""),"",H5/T5)</x:f>
-      </x:c>
-      <x:c r="W5" s="291" t="str">
-        <x:f>IF(OR(K5="",T5=""),"",K5/T5)</x:f>
-      </x:c>
-      <x:c r="X5" s="291" t="n">
-        <x:f>IF(OR(P5="",T5=""),"",P5/T5)</x:f>
-        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -14520,65 +14525,65 @@
         <x:f>IF(Hackathons!R4="","",Hackathons!R4)</x:f>
         <x:v>Rated best project</x:v>
       </x:c>
-      <x:c r="F6" s="40" t="str">
+      <x:c r="F6" s="36" t="n">
+        <x:f>IF(Hackathons!AH4="","",Hackathons!AH4)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G6" s="40" t="str">
         <x:f>IF(Hackathons!S4="","",Hackathons!S4)</x:f>
       </x:c>
-      <x:c r="G6" s="36" t="str">
+      <x:c r="H6" s="36" t="str">
         <x:f>IF(Hackathons!T4="","",Hackathons!T4)</x:f>
       </x:c>
-      <x:c r="H6" s="40" t="str">
+      <x:c r="I6" s="329" t="str">
+        <x:f>IF(OR(G6="",F6=""),"",G6/F6)</x:f>
+      </x:c>
+      <x:c r="J6" s="40" t="str">
         <x:f>IF(Hackathons!U4="","",Hackathons!U4)</x:f>
       </x:c>
-      <x:c r="I6" s="36" t="str">
+      <x:c r="K6" s="36" t="str">
         <x:f>IF(Hackathons!V4="","",Hackathons!V4)</x:f>
       </x:c>
-      <x:c r="J6" s="39" t="str">
+      <x:c r="L6" s="329" t="str">
+        <x:f>IF(OR(J6="",F6=""),"",J6/F6)</x:f>
+      </x:c>
+      <x:c r="M6" s="39" t="str">
         <x:f>IF(Hackathons!W4="","",Hackathons!W4)</x:f>
       </x:c>
-      <x:c r="K6" s="40" t="str">
+      <x:c r="N6" s="40" t="str">
         <x:f>IF(Hackathons!X4="","",Hackathons!X4)</x:f>
       </x:c>
-      <x:c r="L6" s="36" t="str">
+      <x:c r="O6" s="36" t="str">
         <x:f>IF(Hackathons!Y4="","",Hackathons!Y4)</x:f>
       </x:c>
-      <x:c r="M6" s="36" t="str">
+      <x:c r="P6" s="329" t="str">
+        <x:f>IF(OR(N6="",F6=""),"",N6/F6)</x:f>
+      </x:c>
+      <x:c r="Q6" s="40" t="str">
+        <x:f>IF(Hackathons!AC4="","",Hackathons!AC4)</x:f>
+      </x:c>
+      <x:c r="R6" s="36" t="str">
+        <x:f>IF(Hackathons!AD4="","",Hackathons!AD4)</x:f>
+      </x:c>
+      <x:c r="S6" s="329" t="str">
+        <x:f>IF(OR(Q6="",F6=""),"",Q6/F6)</x:f>
+      </x:c>
+      <x:c r="T6" s="36" t="str">
         <x:f>IF(Hackathons!Z4="","",Hackathons!Z4)</x:f>
       </x:c>
-      <x:c r="N6" s="36" t="str">
+      <x:c r="U6" s="36" t="str">
         <x:f>IF(Hackathons!AA4="","",Hackathons!AA4)</x:f>
       </x:c>
-      <x:c r="O6" s="39" t="str">
+      <x:c r="V6" s="39" t="str">
         <x:f>IF(Hackathons!AB4="","",Hackathons!AB4)</x:f>
       </x:c>
-      <x:c r="P6" s="40" t="str">
-        <x:f>IF(Hackathons!AC4="","",Hackathons!AC4)</x:f>
-      </x:c>
-      <x:c r="Q6" s="36" t="str">
-        <x:f>IF(Hackathons!AD4="","",Hackathons!AD4)</x:f>
-      </x:c>
-      <x:c r="R6" s="36" t="str">
+      <x:c r="W6" s="36" t="str">
         <x:f>IF(Hackathons!AE4="","",Hackathons!AE4)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S6" s="36" t="str">
+      <x:c r="X6" s="36" t="str">
         <x:f>IF(Hackathons!AF4="","",Hackathons!AF4)</x:f>
         <x:v>Recognition only</x:v>
-      </x:c>
-      <x:c r="T6" s="39" t="n">
-        <x:f>IF(Hackathons!AH4="","",Hackathons!AH4)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="U6" s="291" t="str">
-        <x:f>IF(OR(F6="",T6=""),"",F6/T6)</x:f>
-      </x:c>
-      <x:c r="V6" s="291" t="str">
-        <x:f>IF(OR(H6="",T6=""),"",H6/T6)</x:f>
-      </x:c>
-      <x:c r="W6" s="291" t="str">
-        <x:f>IF(OR(K6="",T6=""),"",K6/T6)</x:f>
-      </x:c>
-      <x:c r="X6" s="291" t="str">
-        <x:f>IF(OR(P6="",T6=""),"",P6/T6)</x:f>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -14602,70 +14607,70 @@
         <x:f>IF(Hackathons!R5="","",Hackathons!R5)</x:f>
         <x:v>Best Use of IBM Bluemix</x:v>
       </x:c>
-      <x:c r="F7" s="40" t="str">
+      <x:c r="F7" s="36" t="n">
+        <x:f>IF(Hackathons!AH5="","",Hackathons!AH5)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G7" s="40" t="str">
         <x:f>IF(Hackathons!S5="","",Hackathons!S5)</x:f>
       </x:c>
-      <x:c r="G7" s="36" t="str">
+      <x:c r="H7" s="36" t="str">
         <x:f>IF(Hackathons!T5="","",Hackathons!T5)</x:f>
       </x:c>
-      <x:c r="H7" s="40" t="n">
+      <x:c r="I7" s="329" t="str">
+        <x:f>IF(OR(G7="",F7=""),"",G7/F7)</x:f>
+      </x:c>
+      <x:c r="J7" s="40" t="n">
         <x:f>IF(Hackathons!U5="","",Hackathons!U5)</x:f>
         <x:v>100000</x:v>
       </x:c>
-      <x:c r="I7" s="36" t="str">
+      <x:c r="K7" s="36" t="str">
         <x:f>IF(Hackathons!V5="","",Hackathons!V5)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="J7" s="39" t="str">
+      <x:c r="L7" s="329" t="n">
+        <x:f>IF(OR(J7="",F7=""),"",J7/F7)</x:f>
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="M7" s="39" t="str">
         <x:f>IF(Hackathons!W5="","",Hackathons!W5)</x:f>
       </x:c>
-      <x:c r="K7" s="40" t="str">
+      <x:c r="N7" s="40" t="str">
         <x:f>IF(Hackathons!X5="","",Hackathons!X5)</x:f>
       </x:c>
-      <x:c r="L7" s="36" t="str">
+      <x:c r="O7" s="36" t="str">
         <x:f>IF(Hackathons!Y5="","",Hackathons!Y5)</x:f>
       </x:c>
-      <x:c r="M7" s="36" t="str">
+      <x:c r="P7" s="329" t="str">
+        <x:f>IF(OR(N7="",F7=""),"",N7/F7)</x:f>
+      </x:c>
+      <x:c r="Q7" s="40" t="str">
+        <x:f>IF(Hackathons!AC5="","",Hackathons!AC5)</x:f>
+      </x:c>
+      <x:c r="R7" s="36" t="str">
+        <x:f>IF(Hackathons!AD5="","",Hackathons!AD5)</x:f>
+      </x:c>
+      <x:c r="S7" s="329" t="str">
+        <x:f>IF(OR(Q7="",F7=""),"",Q7/F7)</x:f>
+      </x:c>
+      <x:c r="T7" s="36" t="str">
         <x:f>IF(Hackathons!Z5="","",Hackathons!Z5)</x:f>
         <x:v>IBM Bluemix credits; SmartWatch</x:v>
       </x:c>
-      <x:c r="N7" s="36" t="str">
+      <x:c r="U7" s="36" t="str">
         <x:f>IF(Hackathons!AA5="","",Hackathons!AA5)</x:f>
         <x:v>SmartWatch</x:v>
       </x:c>
-      <x:c r="O7" s="39" t="str">
+      <x:c r="V7" s="39" t="str">
         <x:f>IF(Hackathons!AB5="","",Hackathons!AB5)</x:f>
       </x:c>
-      <x:c r="P7" s="40" t="str">
-        <x:f>IF(Hackathons!AC5="","",Hackathons!AC5)</x:f>
-      </x:c>
-      <x:c r="Q7" s="36" t="str">
-        <x:f>IF(Hackathons!AD5="","",Hackathons!AD5)</x:f>
-      </x:c>
-      <x:c r="R7" s="36" t="str">
+      <x:c r="W7" s="36" t="str">
         <x:f>IF(Hackathons!AE5="","",Hackathons!AE5)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S7" s="36" t="str">
+      <x:c r="X7" s="36" t="str">
         <x:f>IF(Hackathons!AF5="","",Hackathons!AF5)</x:f>
         <x:v>US$100,000 IBM Bluemix credit value</x:v>
-      </x:c>
-      <x:c r="T7" s="39" t="n">
-        <x:f>IF(Hackathons!AH5="","",Hackathons!AH5)</x:f>
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="U7" s="291" t="str">
-        <x:f>IF(OR(F7="",T7=""),"",F7/T7)</x:f>
-      </x:c>
-      <x:c r="V7" s="291" t="n">
-        <x:f>IF(OR(H7="",T7=""),"",H7/T7)</x:f>
-        <x:v>25000</x:v>
-      </x:c>
-      <x:c r="W7" s="291" t="str">
-        <x:f>IF(OR(K7="",T7=""),"",K7/T7)</x:f>
-      </x:c>
-      <x:c r="X7" s="291" t="str">
-        <x:f>IF(OR(P7="",T7=""),"",P7/T7)</x:f>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -14689,65 +14694,65 @@
         <x:f>IF(Hackathons!R11="","",Hackathons!R11)</x:f>
         <x:v>Rated best project</x:v>
       </x:c>
-      <x:c r="F8" s="40" t="str">
+      <x:c r="F8" s="36" t="n">
+        <x:f>IF(Hackathons!AH11="","",Hackathons!AH11)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G8" s="40" t="str">
         <x:f>IF(Hackathons!S11="","",Hackathons!S11)</x:f>
       </x:c>
-      <x:c r="G8" s="36" t="str">
+      <x:c r="H8" s="36" t="str">
         <x:f>IF(Hackathons!T11="","",Hackathons!T11)</x:f>
       </x:c>
-      <x:c r="H8" s="40" t="str">
+      <x:c r="I8" s="329" t="str">
+        <x:f>IF(OR(G8="",F8=""),"",G8/F8)</x:f>
+      </x:c>
+      <x:c r="J8" s="40" t="str">
         <x:f>IF(Hackathons!U11="","",Hackathons!U11)</x:f>
       </x:c>
-      <x:c r="I8" s="36" t="str">
+      <x:c r="K8" s="36" t="str">
         <x:f>IF(Hackathons!V11="","",Hackathons!V11)</x:f>
       </x:c>
-      <x:c r="J8" s="39" t="str">
+      <x:c r="L8" s="329" t="str">
+        <x:f>IF(OR(J8="",F8=""),"",J8/F8)</x:f>
+      </x:c>
+      <x:c r="M8" s="39" t="str">
         <x:f>IF(Hackathons!W11="","",Hackathons!W11)</x:f>
       </x:c>
-      <x:c r="K8" s="40" t="str">
+      <x:c r="N8" s="40" t="str">
         <x:f>IF(Hackathons!X11="","",Hackathons!X11)</x:f>
       </x:c>
-      <x:c r="L8" s="36" t="str">
+      <x:c r="O8" s="36" t="str">
         <x:f>IF(Hackathons!Y11="","",Hackathons!Y11)</x:f>
       </x:c>
-      <x:c r="M8" s="36" t="str">
+      <x:c r="P8" s="329" t="str">
+        <x:f>IF(OR(N8="",F8=""),"",N8/F8)</x:f>
+      </x:c>
+      <x:c r="Q8" s="40" t="str">
+        <x:f>IF(Hackathons!AC11="","",Hackathons!AC11)</x:f>
+      </x:c>
+      <x:c r="R8" s="36" t="str">
+        <x:f>IF(Hackathons!AD11="","",Hackathons!AD11)</x:f>
+      </x:c>
+      <x:c r="S8" s="329" t="str">
+        <x:f>IF(OR(Q8="",F8=""),"",Q8/F8)</x:f>
+      </x:c>
+      <x:c r="T8" s="36" t="str">
         <x:f>IF(Hackathons!Z11="","",Hackathons!Z11)</x:f>
       </x:c>
-      <x:c r="N8" s="36" t="str">
+      <x:c r="U8" s="36" t="str">
         <x:f>IF(Hackathons!AA11="","",Hackathons!AA11)</x:f>
       </x:c>
-      <x:c r="O8" s="39" t="str">
+      <x:c r="V8" s="39" t="str">
         <x:f>IF(Hackathons!AB11="","",Hackathons!AB11)</x:f>
       </x:c>
-      <x:c r="P8" s="40" t="str">
-        <x:f>IF(Hackathons!AC11="","",Hackathons!AC11)</x:f>
-      </x:c>
-      <x:c r="Q8" s="36" t="str">
-        <x:f>IF(Hackathons!AD11="","",Hackathons!AD11)</x:f>
-      </x:c>
-      <x:c r="R8" s="36" t="str">
+      <x:c r="W8" s="36" t="str">
         <x:f>IF(Hackathons!AE11="","",Hackathons!AE11)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S8" s="36" t="str">
+      <x:c r="X8" s="36" t="str">
         <x:f>IF(Hackathons!AF11="","",Hackathons!AF11)</x:f>
         <x:v>Recognition only</x:v>
-      </x:c>
-      <x:c r="T8" s="39" t="n">
-        <x:f>IF(Hackathons!AH11="","",Hackathons!AH11)</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="U8" s="291" t="str">
-        <x:f>IF(OR(F8="",T8=""),"",F8/T8)</x:f>
-      </x:c>
-      <x:c r="V8" s="291" t="str">
-        <x:f>IF(OR(H8="",T8=""),"",H8/T8)</x:f>
-      </x:c>
-      <x:c r="W8" s="291" t="str">
-        <x:f>IF(OR(K8="",T8=""),"",K8/T8)</x:f>
-      </x:c>
-      <x:c r="X8" s="291" t="str">
-        <x:f>IF(OR(P8="",T8=""),"",P8/T8)</x:f>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -14770,69 +14775,69 @@
       <x:c r="E9" s="36" t="str">
         <x:f>IF(Hackathons!R15="","",Hackathons!R15)</x:f>
       </x:c>
-      <x:c r="F9" s="40" t="n">
+      <x:c r="F9" s="36" t="n">
+        <x:f>IF(Hackathons!AH15="","",Hackathons!AH15)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G9" s="40" t="n">
         <x:f>IF(Hackathons!S15="","",Hackathons!S15)</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="G9" s="36" t="str">
+      <x:c r="H9" s="36" t="str">
         <x:f>IF(Hackathons!T15="","",Hackathons!T15)</x:f>
         <x:v>SGD</x:v>
       </x:c>
-      <x:c r="H9" s="40" t="str">
+      <x:c r="I9" s="329" t="n">
+        <x:f>IF(OR(G9="",F9=""),"",G9/F9)</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="J9" s="40" t="str">
         <x:f>IF(Hackathons!U15="","",Hackathons!U15)</x:f>
       </x:c>
-      <x:c r="I9" s="36" t="str">
+      <x:c r="K9" s="36" t="str">
         <x:f>IF(Hackathons!V15="","",Hackathons!V15)</x:f>
       </x:c>
-      <x:c r="J9" s="39" t="str">
+      <x:c r="L9" s="329" t="str">
+        <x:f>IF(OR(J9="",F9=""),"",J9/F9)</x:f>
+      </x:c>
+      <x:c r="M9" s="39" t="str">
         <x:f>IF(Hackathons!W15="","",Hackathons!W15)</x:f>
       </x:c>
-      <x:c r="K9" s="40" t="str">
+      <x:c r="N9" s="40" t="str">
         <x:f>IF(Hackathons!X15="","",Hackathons!X15)</x:f>
       </x:c>
-      <x:c r="L9" s="36" t="str">
+      <x:c r="O9" s="36" t="str">
         <x:f>IF(Hackathons!Y15="","",Hackathons!Y15)</x:f>
       </x:c>
-      <x:c r="M9" s="36" t="str">
+      <x:c r="P9" s="329" t="str">
+        <x:f>IF(OR(N9="",F9=""),"",N9/F9)</x:f>
+      </x:c>
+      <x:c r="Q9" s="40" t="str">
+        <x:f>IF(Hackathons!AC15="","",Hackathons!AC15)</x:f>
+      </x:c>
+      <x:c r="R9" s="36" t="str">
+        <x:f>IF(Hackathons!AD15="","",Hackathons!AD15)</x:f>
+      </x:c>
+      <x:c r="S9" s="329" t="str">
+        <x:f>IF(OR(Q9="",F9=""),"",Q9/F9)</x:f>
+      </x:c>
+      <x:c r="T9" s="36" t="str">
         <x:f>IF(Hackathons!Z15="","",Hackathons!Z15)</x:f>
         <x:v>S$100 Capitaland voucher</x:v>
       </x:c>
-      <x:c r="N9" s="36" t="str">
+      <x:c r="U9" s="36" t="str">
         <x:f>IF(Hackathons!AA15="","",Hackathons!AA15)</x:f>
       </x:c>
-      <x:c r="O9" s="39" t="str">
+      <x:c r="V9" s="39" t="str">
         <x:f>IF(Hackathons!AB15="","",Hackathons!AB15)</x:f>
       </x:c>
-      <x:c r="P9" s="40" t="str">
-        <x:f>IF(Hackathons!AC15="","",Hackathons!AC15)</x:f>
-      </x:c>
-      <x:c r="Q9" s="36" t="str">
-        <x:f>IF(Hackathons!AD15="","",Hackathons!AD15)</x:f>
-      </x:c>
-      <x:c r="R9" s="36" t="str">
+      <x:c r="W9" s="36" t="str">
         <x:f>IF(Hackathons!AE15="","",Hackathons!AE15)</x:f>
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="S9" s="36" t="str">
+      <x:c r="X9" s="36" t="str">
         <x:f>IF(Hackathons!AF15="","",Hackathons!AF15)</x:f>
         <x:v>Voucher counted as cash equivalent</x:v>
-      </x:c>
-      <x:c r="T9" s="39" t="n">
-        <x:f>IF(Hackathons!AH15="","",Hackathons!AH15)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="U9" s="291" t="n">
-        <x:f>IF(OR(F9="",T9=""),"",F9/T9)</x:f>
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="V9" s="291" t="str">
-        <x:f>IF(OR(H9="",T9=""),"",H9/T9)</x:f>
-      </x:c>
-      <x:c r="W9" s="291" t="str">
-        <x:f>IF(OR(K9="",T9=""),"",K9/T9)</x:f>
-      </x:c>
-      <x:c r="X9" s="291" t="str">
-        <x:f>IF(OR(P9="",T9=""),"",P9/T9)</x:f>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -14855,68 +14860,68 @@
       <x:c r="E10" s="36" t="str">
         <x:f>IF(Hackathons!R18="","",Hackathons!R18)</x:f>
       </x:c>
-      <x:c r="F10" s="40" t="n">
+      <x:c r="F10" s="36" t="n">
+        <x:f>IF(Hackathons!AH18="","",Hackathons!AH18)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G10" s="40" t="n">
         <x:f>IF(Hackathons!S18="","",Hackathons!S18)</x:f>
         <x:v>600</x:v>
       </x:c>
-      <x:c r="G10" s="36" t="str">
+      <x:c r="H10" s="36" t="str">
         <x:f>IF(Hackathons!T18="","",Hackathons!T18)</x:f>
         <x:v>SGD</x:v>
       </x:c>
-      <x:c r="H10" s="40" t="str">
+      <x:c r="I10" s="329" t="n">
+        <x:f>IF(OR(G10="",F10=""),"",G10/F10)</x:f>
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="J10" s="40" t="str">
         <x:f>IF(Hackathons!U18="","",Hackathons!U18)</x:f>
       </x:c>
-      <x:c r="I10" s="36" t="str">
+      <x:c r="K10" s="36" t="str">
         <x:f>IF(Hackathons!V18="","",Hackathons!V18)</x:f>
       </x:c>
-      <x:c r="J10" s="39" t="str">
+      <x:c r="L10" s="329" t="str">
+        <x:f>IF(OR(J10="",F10=""),"",J10/F10)</x:f>
+      </x:c>
+      <x:c r="M10" s="39" t="str">
         <x:f>IF(Hackathons!W18="","",Hackathons!W18)</x:f>
       </x:c>
-      <x:c r="K10" s="40" t="str">
+      <x:c r="N10" s="40" t="str">
         <x:f>IF(Hackathons!X18="","",Hackathons!X18)</x:f>
       </x:c>
-      <x:c r="L10" s="36" t="str">
+      <x:c r="O10" s="36" t="str">
         <x:f>IF(Hackathons!Y18="","",Hackathons!Y18)</x:f>
       </x:c>
-      <x:c r="M10" s="36" t="str">
+      <x:c r="P10" s="329" t="str">
+        <x:f>IF(OR(N10="",F10=""),"",N10/F10)</x:f>
+      </x:c>
+      <x:c r="Q10" s="40" t="str">
+        <x:f>IF(Hackathons!AC18="","",Hackathons!AC18)</x:f>
+      </x:c>
+      <x:c r="R10" s="36" t="str">
+        <x:f>IF(Hackathons!AD18="","",Hackathons!AD18)</x:f>
+      </x:c>
+      <x:c r="S10" s="329" t="str">
+        <x:f>IF(OR(Q10="",F10=""),"",Q10/F10)</x:f>
+      </x:c>
+      <x:c r="T10" s="36" t="str">
         <x:f>IF(Hackathons!Z18="","",Hackathons!Z18)</x:f>
       </x:c>
-      <x:c r="N10" s="36" t="str">
+      <x:c r="U10" s="36" t="str">
         <x:f>IF(Hackathons!AA18="","",Hackathons!AA18)</x:f>
       </x:c>
-      <x:c r="O10" s="39" t="str">
+      <x:c r="V10" s="39" t="str">
         <x:f>IF(Hackathons!AB18="","",Hackathons!AB18)</x:f>
       </x:c>
-      <x:c r="P10" s="40" t="str">
-        <x:f>IF(Hackathons!AC18="","",Hackathons!AC18)</x:f>
-      </x:c>
-      <x:c r="Q10" s="36" t="str">
-        <x:f>IF(Hackathons!AD18="","",Hackathons!AD18)</x:f>
-      </x:c>
-      <x:c r="R10" s="36" t="str">
+      <x:c r="W10" s="36" t="str">
         <x:f>IF(Hackathons!AE18="","",Hackathons!AE18)</x:f>
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="S10" s="36" t="str">
+      <x:c r="X10" s="36" t="str">
         <x:f>IF(Hackathons!AF18="","",Hackathons!AF18)</x:f>
         <x:v>Explicit cash</x:v>
-      </x:c>
-      <x:c r="T10" s="39" t="n">
-        <x:f>IF(Hackathons!AH18="","",Hackathons!AH18)</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="U10" s="291" t="n">
-        <x:f>IF(OR(F10="",T10=""),"",F10/T10)</x:f>
-        <x:v>200</x:v>
-      </x:c>
-      <x:c r="V10" s="291" t="str">
-        <x:f>IF(OR(H10="",T10=""),"",H10/T10)</x:f>
-      </x:c>
-      <x:c r="W10" s="291" t="str">
-        <x:f>IF(OR(K10="",T10=""),"",K10/T10)</x:f>
-      </x:c>
-      <x:c r="X10" s="291" t="str">
-        <x:f>IF(OR(P10="",T10=""),"",P10/T10)</x:f>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -14939,68 +14944,68 @@
       <x:c r="E11" s="36" t="str">
         <x:f>IF(Hackathons!R26="","",Hackathons!R26)</x:f>
       </x:c>
-      <x:c r="F11" s="40" t="n">
+      <x:c r="F11" s="36" t="n">
+        <x:f>IF(Hackathons!AH26="","",Hackathons!AH26)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G11" s="40" t="n">
         <x:f>IF(Hackathons!S26="","",Hackathons!S26)</x:f>
         <x:v>500</x:v>
       </x:c>
-      <x:c r="G11" s="36" t="str">
+      <x:c r="H11" s="36" t="str">
         <x:f>IF(Hackathons!T26="","",Hackathons!T26)</x:f>
         <x:v>SGD</x:v>
       </x:c>
-      <x:c r="H11" s="40" t="str">
+      <x:c r="I11" s="329" t="n">
+        <x:f>IF(OR(G11="",F11=""),"",G11/F11)</x:f>
+        <x:v>83.33333333333333</x:v>
+      </x:c>
+      <x:c r="J11" s="40" t="str">
         <x:f>IF(Hackathons!U26="","",Hackathons!U26)</x:f>
       </x:c>
-      <x:c r="I11" s="36" t="str">
+      <x:c r="K11" s="36" t="str">
         <x:f>IF(Hackathons!V26="","",Hackathons!V26)</x:f>
       </x:c>
-      <x:c r="J11" s="39" t="str">
+      <x:c r="L11" s="329" t="str">
+        <x:f>IF(OR(J11="",F11=""),"",J11/F11)</x:f>
+      </x:c>
+      <x:c r="M11" s="39" t="str">
         <x:f>IF(Hackathons!W26="","",Hackathons!W26)</x:f>
       </x:c>
-      <x:c r="K11" s="40" t="str">
+      <x:c r="N11" s="40" t="str">
         <x:f>IF(Hackathons!X26="","",Hackathons!X26)</x:f>
       </x:c>
-      <x:c r="L11" s="36" t="str">
+      <x:c r="O11" s="36" t="str">
         <x:f>IF(Hackathons!Y26="","",Hackathons!Y26)</x:f>
       </x:c>
-      <x:c r="M11" s="36" t="str">
+      <x:c r="P11" s="329" t="str">
+        <x:f>IF(OR(N11="",F11=""),"",N11/F11)</x:f>
+      </x:c>
+      <x:c r="Q11" s="40" t="str">
+        <x:f>IF(Hackathons!AC26="","",Hackathons!AC26)</x:f>
+      </x:c>
+      <x:c r="R11" s="36" t="str">
+        <x:f>IF(Hackathons!AD26="","",Hackathons!AD26)</x:f>
+      </x:c>
+      <x:c r="S11" s="329" t="str">
+        <x:f>IF(OR(Q11="",F11=""),"",Q11/F11)</x:f>
+      </x:c>
+      <x:c r="T11" s="36" t="str">
         <x:f>IF(Hackathons!Z26="","",Hackathons!Z26)</x:f>
       </x:c>
-      <x:c r="N11" s="36" t="str">
+      <x:c r="U11" s="36" t="str">
         <x:f>IF(Hackathons!AA26="","",Hackathons!AA26)</x:f>
       </x:c>
-      <x:c r="O11" s="39" t="str">
+      <x:c r="V11" s="39" t="str">
         <x:f>IF(Hackathons!AB26="","",Hackathons!AB26)</x:f>
       </x:c>
-      <x:c r="P11" s="40" t="str">
-        <x:f>IF(Hackathons!AC26="","",Hackathons!AC26)</x:f>
-      </x:c>
-      <x:c r="Q11" s="36" t="str">
-        <x:f>IF(Hackathons!AD26="","",Hackathons!AD26)</x:f>
-      </x:c>
-      <x:c r="R11" s="36" t="str">
+      <x:c r="W11" s="36" t="str">
         <x:f>IF(Hackathons!AE26="","",Hackathons!AE26)</x:f>
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="S11" s="36" t="str">
+      <x:c r="X11" s="36" t="str">
         <x:f>IF(Hackathons!AF26="","",Hackathons!AF26)</x:f>
         <x:v>Explicit cash</x:v>
-      </x:c>
-      <x:c r="T11" s="39" t="n">
-        <x:f>IF(Hackathons!AH26="","",Hackathons!AH26)</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="U11" s="291" t="n">
-        <x:f>IF(OR(F11="",T11=""),"",F11/T11)</x:f>
-        <x:v>83.33333333333333</x:v>
-      </x:c>
-      <x:c r="V11" s="291" t="str">
-        <x:f>IF(OR(H11="",T11=""),"",H11/T11)</x:f>
-      </x:c>
-      <x:c r="W11" s="291" t="str">
-        <x:f>IF(OR(K11="",T11=""),"",K11/T11)</x:f>
-      </x:c>
-      <x:c r="X11" s="291" t="str">
-        <x:f>IF(OR(P11="",T11=""),"",P11/T11)</x:f>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -15023,68 +15028,68 @@
       <x:c r="E12" s="36" t="str">
         <x:f>IF(Hackathons!R34="","",Hackathons!R34)</x:f>
       </x:c>
-      <x:c r="F12" s="40" t="n">
+      <x:c r="F12" s="36" t="n">
+        <x:f>IF(Hackathons!AH34="","",Hackathons!AH34)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G12" s="40" t="n">
         <x:f>IF(Hackathons!S34="","",Hackathons!S34)</x:f>
         <x:v>250</x:v>
       </x:c>
-      <x:c r="G12" s="36" t="str">
+      <x:c r="H12" s="36" t="str">
         <x:f>IF(Hackathons!T34="","",Hackathons!T34)</x:f>
         <x:v>SGD</x:v>
       </x:c>
-      <x:c r="H12" s="40" t="str">
+      <x:c r="I12" s="329" t="n">
+        <x:f>IF(OR(G12="",F12=""),"",G12/F12)</x:f>
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="J12" s="40" t="str">
         <x:f>IF(Hackathons!U34="","",Hackathons!U34)</x:f>
       </x:c>
-      <x:c r="I12" s="36" t="str">
+      <x:c r="K12" s="36" t="str">
         <x:f>IF(Hackathons!V34="","",Hackathons!V34)</x:f>
       </x:c>
-      <x:c r="J12" s="39" t="str">
+      <x:c r="L12" s="329" t="str">
+        <x:f>IF(OR(J12="",F12=""),"",J12/F12)</x:f>
+      </x:c>
+      <x:c r="M12" s="39" t="str">
         <x:f>IF(Hackathons!W34="","",Hackathons!W34)</x:f>
       </x:c>
-      <x:c r="K12" s="40" t="str">
+      <x:c r="N12" s="40" t="str">
         <x:f>IF(Hackathons!X34="","",Hackathons!X34)</x:f>
       </x:c>
-      <x:c r="L12" s="36" t="str">
+      <x:c r="O12" s="36" t="str">
         <x:f>IF(Hackathons!Y34="","",Hackathons!Y34)</x:f>
       </x:c>
-      <x:c r="M12" s="36" t="str">
+      <x:c r="P12" s="329" t="str">
+        <x:f>IF(OR(N12="",F12=""),"",N12/F12)</x:f>
+      </x:c>
+      <x:c r="Q12" s="40" t="str">
+        <x:f>IF(Hackathons!AC34="","",Hackathons!AC34)</x:f>
+      </x:c>
+      <x:c r="R12" s="36" t="str">
+        <x:f>IF(Hackathons!AD34="","",Hackathons!AD34)</x:f>
+      </x:c>
+      <x:c r="S12" s="329" t="str">
+        <x:f>IF(OR(Q12="",F12=""),"",Q12/F12)</x:f>
+      </x:c>
+      <x:c r="T12" s="36" t="str">
         <x:f>IF(Hackathons!Z34="","",Hackathons!Z34)</x:f>
       </x:c>
-      <x:c r="N12" s="36" t="str">
+      <x:c r="U12" s="36" t="str">
         <x:f>IF(Hackathons!AA34="","",Hackathons!AA34)</x:f>
       </x:c>
-      <x:c r="O12" s="39" t="str">
+      <x:c r="V12" s="39" t="str">
         <x:f>IF(Hackathons!AB34="","",Hackathons!AB34)</x:f>
       </x:c>
-      <x:c r="P12" s="40" t="str">
-        <x:f>IF(Hackathons!AC34="","",Hackathons!AC34)</x:f>
-      </x:c>
-      <x:c r="Q12" s="36" t="str">
-        <x:f>IF(Hackathons!AD34="","",Hackathons!AD34)</x:f>
-      </x:c>
-      <x:c r="R12" s="36" t="str">
+      <x:c r="W12" s="36" t="str">
         <x:f>IF(Hackathons!AE34="","",Hackathons!AE34)</x:f>
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="S12" s="36" t="str">
+      <x:c r="X12" s="36" t="str">
         <x:f>IF(Hackathons!AF34="","",Hackathons!AF34)</x:f>
         <x:v>Confirmed cash</x:v>
-      </x:c>
-      <x:c r="T12" s="39" t="n">
-        <x:f>IF(Hackathons!AH34="","",Hackathons!AH34)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="U12" s="291" t="n">
-        <x:f>IF(OR(F12="",T12=""),"",F12/T12)</x:f>
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="V12" s="291" t="str">
-        <x:f>IF(OR(H12="",T12=""),"",H12/T12)</x:f>
-      </x:c>
-      <x:c r="W12" s="291" t="str">
-        <x:f>IF(OR(K12="",T12=""),"",K12/T12)</x:f>
-      </x:c>
-      <x:c r="X12" s="291" t="str">
-        <x:f>IF(OR(P12="",T12=""),"",P12/T12)</x:f>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -15107,68 +15112,68 @@
       <x:c r="E13" s="36" t="str">
         <x:f>IF(Hackathons!R36="","",Hackathons!R36)</x:f>
       </x:c>
-      <x:c r="F13" s="40" t="n">
+      <x:c r="F13" s="36" t="n">
+        <x:f>IF(Hackathons!AH36="","",Hackathons!AH36)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G13" s="40" t="n">
         <x:f>IF(Hackathons!S36="","",Hackathons!S36)</x:f>
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="G13" s="36" t="str">
+      <x:c r="H13" s="36" t="str">
         <x:f>IF(Hackathons!T36="","",Hackathons!T36)</x:f>
         <x:v>SGD</x:v>
       </x:c>
-      <x:c r="H13" s="40" t="str">
+      <x:c r="I13" s="329" t="n">
+        <x:f>IF(OR(G13="",F13=""),"",G13/F13)</x:f>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="J13" s="40" t="str">
         <x:f>IF(Hackathons!U36="","",Hackathons!U36)</x:f>
       </x:c>
-      <x:c r="I13" s="36" t="str">
+      <x:c r="K13" s="36" t="str">
         <x:f>IF(Hackathons!V36="","",Hackathons!V36)</x:f>
       </x:c>
-      <x:c r="J13" s="39" t="str">
+      <x:c r="L13" s="329" t="str">
+        <x:f>IF(OR(J13="",F13=""),"",J13/F13)</x:f>
+      </x:c>
+      <x:c r="M13" s="39" t="str">
         <x:f>IF(Hackathons!W36="","",Hackathons!W36)</x:f>
       </x:c>
-      <x:c r="K13" s="40" t="str">
+      <x:c r="N13" s="40" t="str">
         <x:f>IF(Hackathons!X36="","",Hackathons!X36)</x:f>
       </x:c>
-      <x:c r="L13" s="36" t="str">
+      <x:c r="O13" s="36" t="str">
         <x:f>IF(Hackathons!Y36="","",Hackathons!Y36)</x:f>
       </x:c>
-      <x:c r="M13" s="36" t="str">
+      <x:c r="P13" s="329" t="str">
+        <x:f>IF(OR(N13="",F13=""),"",N13/F13)</x:f>
+      </x:c>
+      <x:c r="Q13" s="40" t="str">
+        <x:f>IF(Hackathons!AC36="","",Hackathons!AC36)</x:f>
+      </x:c>
+      <x:c r="R13" s="36" t="str">
+        <x:f>IF(Hackathons!AD36="","",Hackathons!AD36)</x:f>
+      </x:c>
+      <x:c r="S13" s="329" t="str">
+        <x:f>IF(OR(Q13="",F13=""),"",Q13/F13)</x:f>
+      </x:c>
+      <x:c r="T13" s="36" t="str">
         <x:f>IF(Hackathons!Z36="","",Hackathons!Z36)</x:f>
       </x:c>
-      <x:c r="N13" s="36" t="str">
+      <x:c r="U13" s="36" t="str">
         <x:f>IF(Hackathons!AA36="","",Hackathons!AA36)</x:f>
       </x:c>
-      <x:c r="O13" s="39" t="str">
+      <x:c r="V13" s="39" t="str">
         <x:f>IF(Hackathons!AB36="","",Hackathons!AB36)</x:f>
       </x:c>
-      <x:c r="P13" s="40" t="str">
-        <x:f>IF(Hackathons!AC36="","",Hackathons!AC36)</x:f>
-      </x:c>
-      <x:c r="Q13" s="36" t="str">
-        <x:f>IF(Hackathons!AD36="","",Hackathons!AD36)</x:f>
-      </x:c>
-      <x:c r="R13" s="36" t="str">
+      <x:c r="W13" s="36" t="str">
         <x:f>IF(Hackathons!AE36="","",Hackathons!AE36)</x:f>
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="S13" s="36" t="str">
+      <x:c r="X13" s="36" t="str">
         <x:f>IF(Hackathons!AF36="","",Hackathons!AF36)</x:f>
         <x:v>Confirmed cash</x:v>
-      </x:c>
-      <x:c r="T13" s="39" t="n">
-        <x:f>IF(Hackathons!AH36="","",Hackathons!AH36)</x:f>
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="U13" s="291" t="n">
-        <x:f>IF(OR(F13="",T13=""),"",F13/T13)</x:f>
-        <x:v>250</x:v>
-      </x:c>
-      <x:c r="V13" s="291" t="str">
-        <x:f>IF(OR(H13="",T13=""),"",H13/T13)</x:f>
-      </x:c>
-      <x:c r="W13" s="291" t="str">
-        <x:f>IF(OR(K13="",T13=""),"",K13/T13)</x:f>
-      </x:c>
-      <x:c r="X13" s="291" t="str">
-        <x:f>IF(OR(P13="",T13=""),"",P13/T13)</x:f>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -15191,70 +15196,70 @@
       <x:c r="E14" s="36" t="str">
         <x:f>IF(Hackathons!R39="","",Hackathons!R39)</x:f>
       </x:c>
-      <x:c r="F14" s="40" t="str">
+      <x:c r="F14" s="36" t="n">
+        <x:f>IF(Hackathons!AH39="","",Hackathons!AH39)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G14" s="40" t="str">
         <x:f>IF(Hackathons!S39="","",Hackathons!S39)</x:f>
       </x:c>
-      <x:c r="G14" s="36" t="str">
+      <x:c r="H14" s="36" t="str">
         <x:f>IF(Hackathons!T39="","",Hackathons!T39)</x:f>
       </x:c>
-      <x:c r="H14" s="40" t="str">
+      <x:c r="I14" s="329" t="str">
+        <x:f>IF(OR(G14="",F14=""),"",G14/F14)</x:f>
+      </x:c>
+      <x:c r="J14" s="40" t="str">
         <x:f>IF(Hackathons!U39="","",Hackathons!U39)</x:f>
       </x:c>
-      <x:c r="I14" s="36" t="str">
+      <x:c r="K14" s="36" t="str">
         <x:f>IF(Hackathons!V39="","",Hackathons!V39)</x:f>
       </x:c>
-      <x:c r="J14" s="39" t="n">
+      <x:c r="L14" s="329" t="str">
+        <x:f>IF(OR(J14="",F14=""),"",J14/F14)</x:f>
+      </x:c>
+      <x:c r="M14" s="39" t="n">
         <x:f>IF(Hackathons!W39="","",Hackathons!W39)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K14" s="40" t="n">
+      <x:c r="N14" s="40" t="n">
         <x:f>IF(Hackathons!X39="","",Hackathons!X39)</x:f>
         <x:v>39</x:v>
       </x:c>
-      <x:c r="L14" s="36" t="str">
+      <x:c r="O14" s="36" t="str">
         <x:f>IF(Hackathons!Y39="","",Hackathons!Y39)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="M14" s="36" t="str">
+      <x:c r="P14" s="329" t="n">
+        <x:f>IF(OR(N14="",F14=""),"",N14/F14)</x:f>
+        <x:v>9.75</x:v>
+      </x:c>
+      <x:c r="Q14" s="40" t="str">
+        <x:f>IF(Hackathons!AC39="","",Hackathons!AC39)</x:f>
+      </x:c>
+      <x:c r="R14" s="36" t="str">
+        <x:f>IF(Hackathons!AD39="","",Hackathons!AD39)</x:f>
+      </x:c>
+      <x:c r="S14" s="329" t="str">
+        <x:f>IF(OR(Q14="",F14=""),"",Q14/F14)</x:f>
+      </x:c>
+      <x:c r="T14" s="36" t="str">
         <x:f>IF(Hackathons!Z39="","",Hackathons!Z39)</x:f>
         <x:v>Manus Pro subscription</x:v>
       </x:c>
-      <x:c r="N14" s="36" t="str">
+      <x:c r="U14" s="36" t="str">
         <x:f>IF(Hackathons!AA39="","",Hackathons!AA39)</x:f>
       </x:c>
-      <x:c r="O14" s="39" t="str">
+      <x:c r="V14" s="39" t="str">
         <x:f>IF(Hackathons!AB39="","",Hackathons!AB39)</x:f>
       </x:c>
-      <x:c r="P14" s="40" t="str">
-        <x:f>IF(Hackathons!AC39="","",Hackathons!AC39)</x:f>
-      </x:c>
-      <x:c r="Q14" s="36" t="str">
-        <x:f>IF(Hackathons!AD39="","",Hackathons!AD39)</x:f>
-      </x:c>
-      <x:c r="R14" s="36" t="str">
+      <x:c r="W14" s="36" t="str">
         <x:f>IF(Hackathons!AE39="","",Hackathons!AE39)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S14" s="36" t="str">
+      <x:c r="X14" s="36" t="str">
         <x:f>IF(Hackathons!AF39="","",Hackathons!AF39)</x:f>
         <x:v>US$39 monthly value at award period</x:v>
-      </x:c>
-      <x:c r="T14" s="39" t="n">
-        <x:f>IF(Hackathons!AH39="","",Hackathons!AH39)</x:f>
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="U14" s="291" t="str">
-        <x:f>IF(OR(F14="",T14=""),"",F14/T14)</x:f>
-      </x:c>
-      <x:c r="V14" s="291" t="str">
-        <x:f>IF(OR(H14="",T14=""),"",H14/T14)</x:f>
-      </x:c>
-      <x:c r="W14" s="291" t="n">
-        <x:f>IF(OR(K14="",T14=""),"",K14/T14)</x:f>
-        <x:v>9.75</x:v>
-      </x:c>
-      <x:c r="X14" s="291" t="str">
-        <x:f>IF(OR(P14="",T14=""),"",P14/T14)</x:f>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -15277,68 +15282,68 @@
       <x:c r="E15" s="36" t="str">
         <x:f>IF(Hackathons!R41="","",Hackathons!R41)</x:f>
       </x:c>
-      <x:c r="F15" s="40" t="str">
+      <x:c r="F15" s="36" t="n">
+        <x:f>IF(Hackathons!AH41="","",Hackathons!AH41)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G15" s="40" t="str">
         <x:f>IF(Hackathons!S41="","",Hackathons!S41)</x:f>
       </x:c>
-      <x:c r="G15" s="36" t="str">
+      <x:c r="H15" s="36" t="str">
         <x:f>IF(Hackathons!T41="","",Hackathons!T41)</x:f>
       </x:c>
-      <x:c r="H15" s="40" t="str">
+      <x:c r="I15" s="329" t="str">
+        <x:f>IF(OR(G15="",F15=""),"",G15/F15)</x:f>
+      </x:c>
+      <x:c r="J15" s="40" t="str">
         <x:f>IF(Hackathons!U41="","",Hackathons!U41)</x:f>
       </x:c>
-      <x:c r="I15" s="36" t="str">
+      <x:c r="K15" s="36" t="str">
         <x:f>IF(Hackathons!V41="","",Hackathons!V41)</x:f>
       </x:c>
-      <x:c r="J15" s="39" t="str">
+      <x:c r="L15" s="329" t="str">
+        <x:f>IF(OR(J15="",F15=""),"",J15/F15)</x:f>
+      </x:c>
+      <x:c r="M15" s="39" t="str">
         <x:f>IF(Hackathons!W41="","",Hackathons!W41)</x:f>
       </x:c>
-      <x:c r="K15" s="40" t="str">
+      <x:c r="N15" s="40" t="str">
         <x:f>IF(Hackathons!X41="","",Hackathons!X41)</x:f>
       </x:c>
-      <x:c r="L15" s="36" t="str">
+      <x:c r="O15" s="36" t="str">
         <x:f>IF(Hackathons!Y41="","",Hackathons!Y41)</x:f>
       </x:c>
-      <x:c r="M15" s="36" t="str">
+      <x:c r="P15" s="329" t="str">
+        <x:f>IF(OR(N15="",F15=""),"",N15/F15)</x:f>
+      </x:c>
+      <x:c r="Q15" s="40" t="str">
+        <x:f>IF(Hackathons!AC41="","",Hackathons!AC41)</x:f>
+      </x:c>
+      <x:c r="R15" s="36" t="str">
+        <x:f>IF(Hackathons!AD41="","",Hackathons!AD41)</x:f>
+      </x:c>
+      <x:c r="S15" s="329" t="str">
+        <x:f>IF(OR(Q15="",F15=""),"",Q15/F15)</x:f>
+      </x:c>
+      <x:c r="T15" s="36" t="str">
         <x:f>IF(Hackathons!Z41="","",Hackathons!Z41)</x:f>
         <x:v>Trophy</x:v>
       </x:c>
-      <x:c r="N15" s="36" t="str">
+      <x:c r="U15" s="36" t="str">
         <x:f>IF(Hackathons!AA41="","",Hackathons!AA41)</x:f>
         <x:v>Trophy</x:v>
       </x:c>
-      <x:c r="O15" s="39" t="n">
+      <x:c r="V15" s="39" t="n">
         <x:f>IF(Hackathons!AB41="","",Hackathons!AB41)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="P15" s="40" t="str">
-        <x:f>IF(Hackathons!AC41="","",Hackathons!AC41)</x:f>
-      </x:c>
-      <x:c r="Q15" s="36" t="str">
-        <x:f>IF(Hackathons!AD41="","",Hackathons!AD41)</x:f>
-      </x:c>
-      <x:c r="R15" s="36" t="str">
+      <x:c r="W15" s="36" t="str">
         <x:f>IF(Hackathons!AE41="","",Hackathons!AE41)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S15" s="36" t="str">
+      <x:c r="X15" s="36" t="str">
         <x:f>IF(Hackathons!AF41="","",Hackathons!AF41)</x:f>
         <x:v>Trophy, not cash</x:v>
-      </x:c>
-      <x:c r="T15" s="39" t="n">
-        <x:f>IF(Hackathons!AH41="","",Hackathons!AH41)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="U15" s="291" t="str">
-        <x:f>IF(OR(F15="",T15=""),"",F15/T15)</x:f>
-      </x:c>
-      <x:c r="V15" s="291" t="str">
-        <x:f>IF(OR(H15="",T15=""),"",H15/T15)</x:f>
-      </x:c>
-      <x:c r="W15" s="291" t="str">
-        <x:f>IF(OR(K15="",T15=""),"",K15/T15)</x:f>
-      </x:c>
-      <x:c r="X15" s="291" t="str">
-        <x:f>IF(OR(P15="",T15=""),"",P15/T15)</x:f>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -15361,69 +15366,69 @@
       <x:c r="E16" s="36" t="str">
         <x:f>IF(Hackathons!R43="","",Hackathons!R43)</x:f>
       </x:c>
-      <x:c r="F16" s="40" t="str">
+      <x:c r="F16" s="36" t="n">
+        <x:f>IF(Hackathons!AH43="","",Hackathons!AH43)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G16" s="40" t="str">
         <x:f>IF(Hackathons!S43="","",Hackathons!S43)</x:f>
       </x:c>
-      <x:c r="G16" s="36" t="str">
+      <x:c r="H16" s="36" t="str">
         <x:f>IF(Hackathons!T43="","",Hackathons!T43)</x:f>
       </x:c>
-      <x:c r="H16" s="40" t="n">
+      <x:c r="I16" s="329" t="str">
+        <x:f>IF(OR(G16="",F16=""),"",G16/F16)</x:f>
+      </x:c>
+      <x:c r="J16" s="40" t="n">
         <x:f>IF(Hackathons!U43="","",Hackathons!U43)</x:f>
         <x:v>500</x:v>
       </x:c>
-      <x:c r="I16" s="36" t="str">
+      <x:c r="K16" s="36" t="str">
         <x:f>IF(Hackathons!V43="","",Hackathons!V43)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="J16" s="39" t="str">
+      <x:c r="L16" s="329" t="n">
+        <x:f>IF(OR(J16="",F16=""),"",J16/F16)</x:f>
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="M16" s="39" t="str">
         <x:f>IF(Hackathons!W43="","",Hackathons!W43)</x:f>
       </x:c>
-      <x:c r="K16" s="40" t="str">
+      <x:c r="N16" s="40" t="str">
         <x:f>IF(Hackathons!X43="","",Hackathons!X43)</x:f>
       </x:c>
-      <x:c r="L16" s="36" t="str">
+      <x:c r="O16" s="36" t="str">
         <x:f>IF(Hackathons!Y43="","",Hackathons!Y43)</x:f>
       </x:c>
-      <x:c r="M16" s="36" t="str">
+      <x:c r="P16" s="329" t="str">
+        <x:f>IF(OR(N16="",F16=""),"",N16/F16)</x:f>
+      </x:c>
+      <x:c r="Q16" s="40" t="str">
+        <x:f>IF(Hackathons!AC43="","",Hackathons!AC43)</x:f>
+      </x:c>
+      <x:c r="R16" s="36" t="str">
+        <x:f>IF(Hackathons!AD43="","",Hackathons!AD43)</x:f>
+      </x:c>
+      <x:c r="S16" s="329" t="str">
+        <x:f>IF(OR(Q16="",F16=""),"",Q16/F16)</x:f>
+      </x:c>
+      <x:c r="T16" s="36" t="str">
         <x:f>IF(Hackathons!Z43="","",Hackathons!Z43)</x:f>
         <x:v>Nosana Cloud credit</x:v>
       </x:c>
-      <x:c r="N16" s="36" t="str">
+      <x:c r="U16" s="36" t="str">
         <x:f>IF(Hackathons!AA43="","",Hackathons!AA43)</x:f>
       </x:c>
-      <x:c r="O16" s="39" t="str">
+      <x:c r="V16" s="39" t="str">
         <x:f>IF(Hackathons!AB43="","",Hackathons!AB43)</x:f>
       </x:c>
-      <x:c r="P16" s="40" t="str">
-        <x:f>IF(Hackathons!AC43="","",Hackathons!AC43)</x:f>
-      </x:c>
-      <x:c r="Q16" s="36" t="str">
-        <x:f>IF(Hackathons!AD43="","",Hackathons!AD43)</x:f>
-      </x:c>
-      <x:c r="R16" s="36" t="str">
+      <x:c r="W16" s="36" t="str">
         <x:f>IF(Hackathons!AE43="","",Hackathons!AE43)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S16" s="36" t="str">
+      <x:c r="X16" s="36" t="str">
         <x:f>IF(Hackathons!AF43="","",Hackathons!AF43)</x:f>
         <x:v>Cloud credit, not cash</x:v>
-      </x:c>
-      <x:c r="T16" s="39" t="n">
-        <x:f>IF(Hackathons!AH43="","",Hackathons!AH43)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U16" s="291" t="str">
-        <x:f>IF(OR(F16="",T16=""),"",F16/T16)</x:f>
-      </x:c>
-      <x:c r="V16" s="291" t="n">
-        <x:f>IF(OR(H16="",T16=""),"",H16/T16)</x:f>
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="W16" s="291" t="str">
-        <x:f>IF(OR(K16="",T16=""),"",K16/T16)</x:f>
-      </x:c>
-      <x:c r="X16" s="291" t="str">
-        <x:f>IF(OR(P16="",T16=""),"",P16/T16)</x:f>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -15446,69 +15451,69 @@
       <x:c r="E17" s="36" t="str">
         <x:f>IF(Hackathons!R51="","",Hackathons!R51)</x:f>
       </x:c>
-      <x:c r="F17" s="40" t="str">
+      <x:c r="F17" s="36" t="n">
+        <x:f>IF(Hackathons!AH51="","",Hackathons!AH51)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G17" s="40" t="str">
         <x:f>IF(Hackathons!S51="","",Hackathons!S51)</x:f>
       </x:c>
-      <x:c r="G17" s="36" t="str">
+      <x:c r="H17" s="36" t="str">
         <x:f>IF(Hackathons!T51="","",Hackathons!T51)</x:f>
       </x:c>
-      <x:c r="H17" s="40" t="n">
+      <x:c r="I17" s="329" t="str">
+        <x:f>IF(OR(G17="",F17=""),"",G17/F17)</x:f>
+      </x:c>
+      <x:c r="J17" s="40" t="n">
         <x:f>IF(Hackathons!U51="","",Hackathons!U51)</x:f>
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="I17" s="36" t="str">
+      <x:c r="K17" s="36" t="str">
         <x:f>IF(Hackathons!V51="","",Hackathons!V51)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="J17" s="39" t="str">
+      <x:c r="L17" s="329" t="n">
+        <x:f>IF(OR(J17="",F17=""),"",J17/F17)</x:f>
+        <x:v>333.3333333333333</x:v>
+      </x:c>
+      <x:c r="M17" s="39" t="str">
         <x:f>IF(Hackathons!W51="","",Hackathons!W51)</x:f>
       </x:c>
-      <x:c r="K17" s="40" t="str">
+      <x:c r="N17" s="40" t="str">
         <x:f>IF(Hackathons!X51="","",Hackathons!X51)</x:f>
       </x:c>
-      <x:c r="L17" s="36" t="str">
+      <x:c r="O17" s="36" t="str">
         <x:f>IF(Hackathons!Y51="","",Hackathons!Y51)</x:f>
       </x:c>
-      <x:c r="M17" s="36" t="str">
+      <x:c r="P17" s="329" t="str">
+        <x:f>IF(OR(N17="",F17=""),"",N17/F17)</x:f>
+      </x:c>
+      <x:c r="Q17" s="40" t="str">
+        <x:f>IF(Hackathons!AC51="","",Hackathons!AC51)</x:f>
+      </x:c>
+      <x:c r="R17" s="36" t="str">
+        <x:f>IF(Hackathons!AD51="","",Hackathons!AD51)</x:f>
+      </x:c>
+      <x:c r="S17" s="329" t="str">
+        <x:f>IF(OR(Q17="",F17=""),"",Q17/F17)</x:f>
+      </x:c>
+      <x:c r="T17" s="36" t="str">
         <x:f>IF(Hackathons!Z51="","",Hackathons!Z51)</x:f>
         <x:v>OpenRouter credits</x:v>
       </x:c>
-      <x:c r="N17" s="36" t="str">
+      <x:c r="U17" s="36" t="str">
         <x:f>IF(Hackathons!AA51="","",Hackathons!AA51)</x:f>
       </x:c>
-      <x:c r="O17" s="39" t="str">
+      <x:c r="V17" s="39" t="str">
         <x:f>IF(Hackathons!AB51="","",Hackathons!AB51)</x:f>
       </x:c>
-      <x:c r="P17" s="40" t="str">
-        <x:f>IF(Hackathons!AC51="","",Hackathons!AC51)</x:f>
-      </x:c>
-      <x:c r="Q17" s="36" t="str">
-        <x:f>IF(Hackathons!AD51="","",Hackathons!AD51)</x:f>
-      </x:c>
-      <x:c r="R17" s="36" t="str">
+      <x:c r="W17" s="36" t="str">
         <x:f>IF(Hackathons!AE51="","",Hackathons!AE51)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S17" s="36" t="str">
+      <x:c r="X17" s="36" t="str">
         <x:f>IF(Hackathons!AF51="","",Hackathons!AF51)</x:f>
         <x:v>API credits, not cash</x:v>
-      </x:c>
-      <x:c r="T17" s="39" t="n">
-        <x:f>IF(Hackathons!AH51="","",Hackathons!AH51)</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="U17" s="291" t="str">
-        <x:f>IF(OR(F17="",T17=""),"",F17/T17)</x:f>
-      </x:c>
-      <x:c r="V17" s="291" t="n">
-        <x:f>IF(OR(H17="",T17=""),"",H17/T17)</x:f>
-        <x:v>333.3333333333333</x:v>
-      </x:c>
-      <x:c r="W17" s="291" t="str">
-        <x:f>IF(OR(K17="",T17=""),"",K17/T17)</x:f>
-      </x:c>
-      <x:c r="X17" s="291" t="str">
-        <x:f>IF(OR(P17="",T17=""),"",P17/T17)</x:f>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -15531,69 +15536,69 @@
       <x:c r="E18" s="36" t="str">
         <x:f>IF(Hackathons!R53="","",Hackathons!R53)</x:f>
       </x:c>
-      <x:c r="F18" s="40" t="str">
+      <x:c r="F18" s="36" t="n">
+        <x:f>IF(Hackathons!AH53="","",Hackathons!AH53)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G18" s="40" t="str">
         <x:f>IF(Hackathons!S53="","",Hackathons!S53)</x:f>
       </x:c>
-      <x:c r="G18" s="36" t="str">
+      <x:c r="H18" s="36" t="str">
         <x:f>IF(Hackathons!T53="","",Hackathons!T53)</x:f>
       </x:c>
-      <x:c r="H18" s="40" t="n">
+      <x:c r="I18" s="329" t="str">
+        <x:f>IF(OR(G18="",F18=""),"",G18/F18)</x:f>
+      </x:c>
+      <x:c r="J18" s="40" t="n">
         <x:f>IF(Hackathons!U53="","",Hackathons!U53)</x:f>
         <x:v>500</x:v>
       </x:c>
-      <x:c r="I18" s="36" t="str">
+      <x:c r="K18" s="36" t="str">
         <x:f>IF(Hackathons!V53="","",Hackathons!V53)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="J18" s="39" t="str">
+      <x:c r="L18" s="329" t="n">
+        <x:f>IF(OR(J18="",F18=""),"",J18/F18)</x:f>
+        <x:v>166.66666666666666</x:v>
+      </x:c>
+      <x:c r="M18" s="39" t="str">
         <x:f>IF(Hackathons!W53="","",Hackathons!W53)</x:f>
       </x:c>
-      <x:c r="K18" s="40" t="str">
+      <x:c r="N18" s="40" t="str">
         <x:f>IF(Hackathons!X53="","",Hackathons!X53)</x:f>
       </x:c>
-      <x:c r="L18" s="36" t="str">
+      <x:c r="O18" s="36" t="str">
         <x:f>IF(Hackathons!Y53="","",Hackathons!Y53)</x:f>
       </x:c>
-      <x:c r="M18" s="36" t="str">
+      <x:c r="P18" s="329" t="str">
+        <x:f>IF(OR(N18="",F18=""),"",N18/F18)</x:f>
+      </x:c>
+      <x:c r="Q18" s="40" t="str">
+        <x:f>IF(Hackathons!AC53="","",Hackathons!AC53)</x:f>
+      </x:c>
+      <x:c r="R18" s="36" t="str">
+        <x:f>IF(Hackathons!AD53="","",Hackathons!AD53)</x:f>
+      </x:c>
+      <x:c r="S18" s="329" t="str">
+        <x:f>IF(OR(Q18="",F18=""),"",Q18/F18)</x:f>
+      </x:c>
+      <x:c r="T18" s="36" t="str">
         <x:f>IF(Hackathons!Z53="","",Hackathons!Z53)</x:f>
         <x:v>API credits</x:v>
       </x:c>
-      <x:c r="N18" s="36" t="str">
+      <x:c r="U18" s="36" t="str">
         <x:f>IF(Hackathons!AA53="","",Hackathons!AA53)</x:f>
       </x:c>
-      <x:c r="O18" s="39" t="str">
+      <x:c r="V18" s="39" t="str">
         <x:f>IF(Hackathons!AB53="","",Hackathons!AB53)</x:f>
       </x:c>
-      <x:c r="P18" s="40" t="str">
-        <x:f>IF(Hackathons!AC53="","",Hackathons!AC53)</x:f>
-      </x:c>
-      <x:c r="Q18" s="36" t="str">
-        <x:f>IF(Hackathons!AD53="","",Hackathons!AD53)</x:f>
-      </x:c>
-      <x:c r="R18" s="36" t="str">
+      <x:c r="W18" s="36" t="str">
         <x:f>IF(Hackathons!AE53="","",Hackathons!AE53)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S18" s="36" t="str">
+      <x:c r="X18" s="36" t="str">
         <x:f>IF(Hackathons!AF53="","",Hackathons!AF53)</x:f>
         <x:v>API credits, not cash</x:v>
-      </x:c>
-      <x:c r="T18" s="39" t="n">
-        <x:f>IF(Hackathons!AH53="","",Hackathons!AH53)</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="U18" s="291" t="str">
-        <x:f>IF(OR(F18="",T18=""),"",F18/T18)</x:f>
-      </x:c>
-      <x:c r="V18" s="291" t="n">
-        <x:f>IF(OR(H18="",T18=""),"",H18/T18)</x:f>
-        <x:v>166.66666666666666</x:v>
-      </x:c>
-      <x:c r="W18" s="291" t="str">
-        <x:f>IF(OR(K18="",T18=""),"",K18/T18)</x:f>
-      </x:c>
-      <x:c r="X18" s="291" t="str">
-        <x:f>IF(OR(P18="",T18=""),"",P18/T18)</x:f>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -15616,69 +15621,69 @@
       <x:c r="E19" s="36" t="str">
         <x:f>IF(Hackathons!R54="","",Hackathons!R54)</x:f>
       </x:c>
-      <x:c r="F19" s="40" t="str">
+      <x:c r="F19" s="36" t="n">
+        <x:f>IF(Hackathons!AH54="","",Hackathons!AH54)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G19" s="40" t="str">
         <x:f>IF(Hackathons!S54="","",Hackathons!S54)</x:f>
       </x:c>
-      <x:c r="G19" s="36" t="str">
+      <x:c r="H19" s="36" t="str">
         <x:f>IF(Hackathons!T54="","",Hackathons!T54)</x:f>
       </x:c>
-      <x:c r="H19" s="40" t="n">
+      <x:c r="I19" s="329" t="str">
+        <x:f>IF(OR(G19="",F19=""),"",G19/F19)</x:f>
+      </x:c>
+      <x:c r="J19" s="40" t="n">
         <x:f>IF(Hackathons!U54="","",Hackathons!U54)</x:f>
         <x:v>500</x:v>
       </x:c>
-      <x:c r="I19" s="36" t="str">
+      <x:c r="K19" s="36" t="str">
         <x:f>IF(Hackathons!V54="","",Hackathons!V54)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="J19" s="39" t="str">
+      <x:c r="L19" s="329" t="n">
+        <x:f>IF(OR(J19="",F19=""),"",J19/F19)</x:f>
+        <x:v>166.66666666666666</x:v>
+      </x:c>
+      <x:c r="M19" s="39" t="str">
         <x:f>IF(Hackathons!W54="","",Hackathons!W54)</x:f>
       </x:c>
-      <x:c r="K19" s="40" t="str">
+      <x:c r="N19" s="40" t="str">
         <x:f>IF(Hackathons!X54="","",Hackathons!X54)</x:f>
       </x:c>
-      <x:c r="L19" s="36" t="str">
+      <x:c r="O19" s="36" t="str">
         <x:f>IF(Hackathons!Y54="","",Hackathons!Y54)</x:f>
       </x:c>
-      <x:c r="M19" s="36" t="str">
+      <x:c r="P19" s="329" t="str">
+        <x:f>IF(OR(N19="",F19=""),"",N19/F19)</x:f>
+      </x:c>
+      <x:c r="Q19" s="40" t="str">
+        <x:f>IF(Hackathons!AC54="","",Hackathons!AC54)</x:f>
+      </x:c>
+      <x:c r="R19" s="36" t="str">
+        <x:f>IF(Hackathons!AD54="","",Hackathons!AD54)</x:f>
+      </x:c>
+      <x:c r="S19" s="329" t="str">
+        <x:f>IF(OR(Q19="",F19=""),"",Q19/F19)</x:f>
+      </x:c>
+      <x:c r="T19" s="36" t="str">
         <x:f>IF(Hackathons!Z54="","",Hackathons!Z54)</x:f>
         <x:v>API credits</x:v>
       </x:c>
-      <x:c r="N19" s="36" t="str">
+      <x:c r="U19" s="36" t="str">
         <x:f>IF(Hackathons!AA54="","",Hackathons!AA54)</x:f>
       </x:c>
-      <x:c r="O19" s="39" t="str">
+      <x:c r="V19" s="39" t="str">
         <x:f>IF(Hackathons!AB54="","",Hackathons!AB54)</x:f>
       </x:c>
-      <x:c r="P19" s="40" t="str">
-        <x:f>IF(Hackathons!AC54="","",Hackathons!AC54)</x:f>
-      </x:c>
-      <x:c r="Q19" s="36" t="str">
-        <x:f>IF(Hackathons!AD54="","",Hackathons!AD54)</x:f>
-      </x:c>
-      <x:c r="R19" s="36" t="str">
+      <x:c r="W19" s="36" t="str">
         <x:f>IF(Hackathons!AE54="","",Hackathons!AE54)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S19" s="36" t="str">
+      <x:c r="X19" s="36" t="str">
         <x:f>IF(Hackathons!AF54="","",Hackathons!AF54)</x:f>
         <x:v>API credits, not cash</x:v>
-      </x:c>
-      <x:c r="T19" s="39" t="n">
-        <x:f>IF(Hackathons!AH54="","",Hackathons!AH54)</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="U19" s="291" t="str">
-        <x:f>IF(OR(F19="",T19=""),"",F19/T19)</x:f>
-      </x:c>
-      <x:c r="V19" s="291" t="n">
-        <x:f>IF(OR(H19="",T19=""),"",H19/T19)</x:f>
-        <x:v>166.66666666666666</x:v>
-      </x:c>
-      <x:c r="W19" s="291" t="str">
-        <x:f>IF(OR(K19="",T19=""),"",K19/T19)</x:f>
-      </x:c>
-      <x:c r="X19" s="291" t="str">
-        <x:f>IF(OR(P19="",T19=""),"",P19/T19)</x:f>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -15701,69 +15706,69 @@
       <x:c r="E20" s="36" t="str">
         <x:f>IF(Hackathons!R55="","",Hackathons!R55)</x:f>
       </x:c>
-      <x:c r="F20" s="40" t="str">
+      <x:c r="F20" s="36" t="n">
+        <x:f>IF(Hackathons!AH55="","",Hackathons!AH55)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G20" s="40" t="str">
         <x:f>IF(Hackathons!S55="","",Hackathons!S55)</x:f>
       </x:c>
-      <x:c r="G20" s="36" t="str">
+      <x:c r="H20" s="36" t="str">
         <x:f>IF(Hackathons!T55="","",Hackathons!T55)</x:f>
       </x:c>
-      <x:c r="H20" s="40" t="n">
+      <x:c r="I20" s="329" t="str">
+        <x:f>IF(OR(G20="",F20=""),"",G20/F20)</x:f>
+      </x:c>
+      <x:c r="J20" s="40" t="n">
         <x:f>IF(Hackathons!U55="","",Hackathons!U55)</x:f>
         <x:v>150</x:v>
       </x:c>
-      <x:c r="I20" s="36" t="str">
+      <x:c r="K20" s="36" t="str">
         <x:f>IF(Hackathons!V55="","",Hackathons!V55)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="J20" s="39" t="str">
+      <x:c r="L20" s="329" t="n">
+        <x:f>IF(OR(J20="",F20=""),"",J20/F20)</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="M20" s="39" t="str">
         <x:f>IF(Hackathons!W55="","",Hackathons!W55)</x:f>
       </x:c>
-      <x:c r="K20" s="40" t="str">
+      <x:c r="N20" s="40" t="str">
         <x:f>IF(Hackathons!X55="","",Hackathons!X55)</x:f>
       </x:c>
-      <x:c r="L20" s="36" t="str">
+      <x:c r="O20" s="36" t="str">
         <x:f>IF(Hackathons!Y55="","",Hackathons!Y55)</x:f>
       </x:c>
-      <x:c r="M20" s="36" t="str">
+      <x:c r="P20" s="329" t="str">
+        <x:f>IF(OR(N20="",F20=""),"",N20/F20)</x:f>
+      </x:c>
+      <x:c r="Q20" s="40" t="str">
+        <x:f>IF(Hackathons!AC55="","",Hackathons!AC55)</x:f>
+      </x:c>
+      <x:c r="R20" s="36" t="str">
+        <x:f>IF(Hackathons!AD55="","",Hackathons!AD55)</x:f>
+      </x:c>
+      <x:c r="S20" s="329" t="str">
+        <x:f>IF(OR(Q20="",F20=""),"",Q20/F20)</x:f>
+      </x:c>
+      <x:c r="T20" s="36" t="str">
         <x:f>IF(Hackathons!Z55="","",Hackathons!Z55)</x:f>
         <x:v>Wavespeed AI credits</x:v>
       </x:c>
-      <x:c r="N20" s="36" t="str">
+      <x:c r="U20" s="36" t="str">
         <x:f>IF(Hackathons!AA55="","",Hackathons!AA55)</x:f>
       </x:c>
-      <x:c r="O20" s="39" t="str">
+      <x:c r="V20" s="39" t="str">
         <x:f>IF(Hackathons!AB55="","",Hackathons!AB55)</x:f>
       </x:c>
-      <x:c r="P20" s="40" t="str">
-        <x:f>IF(Hackathons!AC55="","",Hackathons!AC55)</x:f>
-      </x:c>
-      <x:c r="Q20" s="36" t="str">
-        <x:f>IF(Hackathons!AD55="","",Hackathons!AD55)</x:f>
-      </x:c>
-      <x:c r="R20" s="36" t="str">
+      <x:c r="W20" s="36" t="str">
         <x:f>IF(Hackathons!AE55="","",Hackathons!AE55)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S20" s="36" t="str">
+      <x:c r="X20" s="36" t="str">
         <x:f>IF(Hackathons!AF55="","",Hackathons!AF55)</x:f>
         <x:v>API credits, not cash</x:v>
-      </x:c>
-      <x:c r="T20" s="39" t="n">
-        <x:f>IF(Hackathons!AH55="","",Hackathons!AH55)</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="U20" s="291" t="str">
-        <x:f>IF(OR(F20="",T20=""),"",F20/T20)</x:f>
-      </x:c>
-      <x:c r="V20" s="291" t="n">
-        <x:f>IF(OR(H20="",T20=""),"",H20/T20)</x:f>
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="W20" s="291" t="str">
-        <x:f>IF(OR(K20="",T20=""),"",K20/T20)</x:f>
-      </x:c>
-      <x:c r="X20" s="291" t="str">
-        <x:f>IF(OR(P20="",T20=""),"",P20/T20)</x:f>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -15786,72 +15791,72 @@
       <x:c r="E21" s="36" t="str">
         <x:f>IF(Hackathons!R58="","",Hackathons!R58)</x:f>
       </x:c>
-      <x:c r="F21" s="40" t="n">
+      <x:c r="F21" s="36" t="n">
+        <x:f>IF(Hackathons!AH58="","",Hackathons!AH58)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G21" s="40" t="n">
         <x:f>IF(Hackathons!S58="","",Hackathons!S58)</x:f>
         <x:v>300</x:v>
       </x:c>
-      <x:c r="G21" s="36" t="str">
+      <x:c r="H21" s="36" t="str">
         <x:f>IF(Hackathons!T58="","",Hackathons!T58)</x:f>
         <x:v>SGD</x:v>
       </x:c>
-      <x:c r="H21" s="40" t="n">
+      <x:c r="I21" s="329" t="n">
+        <x:f>IF(OR(G21="",F21=""),"",G21/F21)</x:f>
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="J21" s="40" t="n">
         <x:f>IF(Hackathons!U58="","",Hackathons!U58)</x:f>
         <x:v>385</x:v>
       </x:c>
-      <x:c r="I21" s="36" t="str">
+      <x:c r="K21" s="36" t="str">
         <x:f>IF(Hackathons!V58="","",Hackathons!V58)</x:f>
         <x:v>SGD</x:v>
       </x:c>
-      <x:c r="J21" s="39" t="str">
+      <x:c r="L21" s="329" t="n">
+        <x:f>IF(OR(J21="",F21=""),"",J21/F21)</x:f>
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="M21" s="39" t="str">
         <x:f>IF(Hackathons!W58="","",Hackathons!W58)</x:f>
       </x:c>
-      <x:c r="K21" s="40" t="str">
+      <x:c r="N21" s="40" t="str">
         <x:f>IF(Hackathons!X58="","",Hackathons!X58)</x:f>
       </x:c>
-      <x:c r="L21" s="36" t="str">
+      <x:c r="O21" s="36" t="str">
         <x:f>IF(Hackathons!Y58="","",Hackathons!Y58)</x:f>
       </x:c>
-      <x:c r="M21" s="36" t="str">
+      <x:c r="P21" s="329" t="str">
+        <x:f>IF(OR(N21="",F21=""),"",N21/F21)</x:f>
+      </x:c>
+      <x:c r="Q21" s="40" t="str">
+        <x:f>IF(Hackathons!AC58="","",Hackathons!AC58)</x:f>
+      </x:c>
+      <x:c r="R21" s="36" t="str">
+        <x:f>IF(Hackathons!AD58="","",Hackathons!AD58)</x:f>
+      </x:c>
+      <x:c r="S21" s="329" t="str">
+        <x:f>IF(OR(Q21="",F21=""),"",Q21/F21)</x:f>
+      </x:c>
+      <x:c r="T21" s="36" t="str">
         <x:f>IF(Hackathons!Z58="","",Hackathons!Z58)</x:f>
         <x:v>API credits</x:v>
       </x:c>
-      <x:c r="N21" s="36" t="str">
+      <x:c r="U21" s="36" t="str">
         <x:f>IF(Hackathons!AA58="","",Hackathons!AA58)</x:f>
       </x:c>
-      <x:c r="O21" s="39" t="str">
+      <x:c r="V21" s="39" t="str">
         <x:f>IF(Hackathons!AB58="","",Hackathons!AB58)</x:f>
       </x:c>
-      <x:c r="P21" s="40" t="str">
-        <x:f>IF(Hackathons!AC58="","",Hackathons!AC58)</x:f>
-      </x:c>
-      <x:c r="Q21" s="36" t="str">
-        <x:f>IF(Hackathons!AD58="","",Hackathons!AD58)</x:f>
-      </x:c>
-      <x:c r="R21" s="36" t="str">
+      <x:c r="W21" s="36" t="str">
         <x:f>IF(Hackathons!AE58="","",Hackathons!AE58)</x:f>
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="S21" s="36" t="str">
+      <x:c r="X21" s="36" t="str">
         <x:f>IF(Hackathons!AF58="","",Hackathons!AF58)</x:f>
         <x:v>Explicit cash; API credit value also tracked</x:v>
-      </x:c>
-      <x:c r="T21" s="39" t="n">
-        <x:f>IF(Hackathons!AH58="","",Hackathons!AH58)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U21" s="291" t="n">
-        <x:f>IF(OR(F21="",T21=""),"",F21/T21)</x:f>
-        <x:v>300</x:v>
-      </x:c>
-      <x:c r="V21" s="291" t="n">
-        <x:f>IF(OR(H21="",T21=""),"",H21/T21)</x:f>
-        <x:v>385</x:v>
-      </x:c>
-      <x:c r="W21" s="291" t="str">
-        <x:f>IF(OR(K21="",T21=""),"",K21/T21)</x:f>
-      </x:c>
-      <x:c r="X21" s="291" t="str">
-        <x:f>IF(OR(P21="",T21=""),"",P21/T21)</x:f>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -15875,69 +15880,69 @@
         <x:f>IF(Hackathons!R61="","",Hackathons!R61)</x:f>
         <x:v>Speechmatics</x:v>
       </x:c>
-      <x:c r="F22" s="40" t="str">
+      <x:c r="F22" s="36" t="n">
+        <x:f>IF(Hackathons!AH61="","",Hackathons!AH61)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G22" s="40" t="str">
         <x:f>IF(Hackathons!S61="","",Hackathons!S61)</x:f>
       </x:c>
-      <x:c r="G22" s="36" t="str">
+      <x:c r="H22" s="36" t="str">
         <x:f>IF(Hackathons!T61="","",Hackathons!T61)</x:f>
       </x:c>
-      <x:c r="H22" s="40" t="n">
+      <x:c r="I22" s="329" t="str">
+        <x:f>IF(OR(G22="",F22=""),"",G22/F22)</x:f>
+      </x:c>
+      <x:c r="J22" s="40" t="n">
         <x:f>IF(Hackathons!U61="","",Hackathons!U61)</x:f>
         <x:v>2000</x:v>
       </x:c>
-      <x:c r="I22" s="36" t="str">
+      <x:c r="K22" s="36" t="str">
         <x:f>IF(Hackathons!V61="","",Hackathons!V61)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="J22" s="39" t="str">
+      <x:c r="L22" s="329" t="n">
+        <x:f>IF(OR(J22="",F22=""),"",J22/F22)</x:f>
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="M22" s="39" t="str">
         <x:f>IF(Hackathons!W61="","",Hackathons!W61)</x:f>
       </x:c>
-      <x:c r="K22" s="40" t="str">
+      <x:c r="N22" s="40" t="str">
         <x:f>IF(Hackathons!X61="","",Hackathons!X61)</x:f>
       </x:c>
-      <x:c r="L22" s="36" t="str">
+      <x:c r="O22" s="36" t="str">
         <x:f>IF(Hackathons!Y61="","",Hackathons!Y61)</x:f>
       </x:c>
-      <x:c r="M22" s="36" t="str">
+      <x:c r="P22" s="329" t="str">
+        <x:f>IF(OR(N22="",F22=""),"",N22/F22)</x:f>
+      </x:c>
+      <x:c r="Q22" s="40" t="str">
+        <x:f>IF(Hackathons!AC61="","",Hackathons!AC61)</x:f>
+      </x:c>
+      <x:c r="R22" s="36" t="str">
+        <x:f>IF(Hackathons!AD61="","",Hackathons!AD61)</x:f>
+      </x:c>
+      <x:c r="S22" s="329" t="str">
+        <x:f>IF(OR(Q22="",F22=""),"",Q22/F22)</x:f>
+      </x:c>
+      <x:c r="T22" s="36" t="str">
         <x:f>IF(Hackathons!Z61="","",Hackathons!Z61)</x:f>
         <x:v>Speechmatics credits</x:v>
       </x:c>
-      <x:c r="N22" s="36" t="str">
+      <x:c r="U22" s="36" t="str">
         <x:f>IF(Hackathons!AA61="","",Hackathons!AA61)</x:f>
       </x:c>
-      <x:c r="O22" s="39" t="str">
+      <x:c r="V22" s="39" t="str">
         <x:f>IF(Hackathons!AB61="","",Hackathons!AB61)</x:f>
       </x:c>
-      <x:c r="P22" s="40" t="str">
-        <x:f>IF(Hackathons!AC61="","",Hackathons!AC61)</x:f>
-      </x:c>
-      <x:c r="Q22" s="36" t="str">
-        <x:f>IF(Hackathons!AD61="","",Hackathons!AD61)</x:f>
-      </x:c>
-      <x:c r="R22" s="36" t="str">
+      <x:c r="W22" s="36" t="str">
         <x:f>IF(Hackathons!AE61="","",Hackathons!AE61)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S22" s="36" t="str">
+      <x:c r="X22" s="36" t="str">
         <x:f>IF(Hackathons!AF61="","",Hackathons!AF61)</x:f>
         <x:v>USD-denominated credit value</x:v>
-      </x:c>
-      <x:c r="T22" s="39" t="n">
-        <x:f>IF(Hackathons!AH61="","",Hackathons!AH61)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U22" s="291" t="str">
-        <x:f>IF(OR(F22="",T22=""),"",F22/T22)</x:f>
-      </x:c>
-      <x:c r="V22" s="291" t="n">
-        <x:f>IF(OR(H22="",T22=""),"",H22/T22)</x:f>
-        <x:v>2000</x:v>
-      </x:c>
-      <x:c r="W22" s="291" t="str">
-        <x:f>IF(OR(K22="",T22=""),"",K22/T22)</x:f>
-      </x:c>
-      <x:c r="X22" s="291" t="str">
-        <x:f>IF(OR(P22="",T22=""),"",P22/T22)</x:f>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -15961,67 +15966,67 @@
         <x:f>IF(Hackathons!R62="","",Hackathons!R62)</x:f>
         <x:v>v0 Sock</x:v>
       </x:c>
-      <x:c r="F23" s="40" t="str">
+      <x:c r="F23" s="36" t="n">
+        <x:f>IF(Hackathons!AH62="","",Hackathons!AH62)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G23" s="40" t="str">
         <x:f>IF(Hackathons!S62="","",Hackathons!S62)</x:f>
       </x:c>
-      <x:c r="G23" s="36" t="str">
+      <x:c r="H23" s="36" t="str">
         <x:f>IF(Hackathons!T62="","",Hackathons!T62)</x:f>
       </x:c>
-      <x:c r="H23" s="40" t="str">
+      <x:c r="I23" s="329" t="str">
+        <x:f>IF(OR(G23="",F23=""),"",G23/F23)</x:f>
+      </x:c>
+      <x:c r="J23" s="40" t="str">
         <x:f>IF(Hackathons!U62="","",Hackathons!U62)</x:f>
       </x:c>
-      <x:c r="I23" s="36" t="str">
+      <x:c r="K23" s="36" t="str">
         <x:f>IF(Hackathons!V62="","",Hackathons!V62)</x:f>
       </x:c>
-      <x:c r="J23" s="39" t="str">
+      <x:c r="L23" s="329" t="str">
+        <x:f>IF(OR(J23="",F23=""),"",J23/F23)</x:f>
+      </x:c>
+      <x:c r="M23" s="39" t="str">
         <x:f>IF(Hackathons!W62="","",Hackathons!W62)</x:f>
       </x:c>
-      <x:c r="K23" s="40" t="str">
+      <x:c r="N23" s="40" t="str">
         <x:f>IF(Hackathons!X62="","",Hackathons!X62)</x:f>
       </x:c>
-      <x:c r="L23" s="36" t="str">
+      <x:c r="O23" s="36" t="str">
         <x:f>IF(Hackathons!Y62="","",Hackathons!Y62)</x:f>
       </x:c>
-      <x:c r="M23" s="36" t="str">
+      <x:c r="P23" s="329" t="str">
+        <x:f>IF(OR(N23="",F23=""),"",N23/F23)</x:f>
+      </x:c>
+      <x:c r="Q23" s="40" t="str">
+        <x:f>IF(Hackathons!AC62="","",Hackathons!AC62)</x:f>
+      </x:c>
+      <x:c r="R23" s="36" t="str">
+        <x:f>IF(Hackathons!AD62="","",Hackathons!AD62)</x:f>
+      </x:c>
+      <x:c r="S23" s="329" t="str">
+        <x:f>IF(OR(Q23="",F23=""),"",Q23/F23)</x:f>
+      </x:c>
+      <x:c r="T23" s="36" t="str">
         <x:f>IF(Hackathons!Z62="","",Hackathons!Z62)</x:f>
         <x:v>v0 Sock</x:v>
       </x:c>
-      <x:c r="N23" s="36" t="str">
+      <x:c r="U23" s="36" t="str">
         <x:f>IF(Hackathons!AA62="","",Hackathons!AA62)</x:f>
         <x:v>v0 Sock</x:v>
       </x:c>
-      <x:c r="O23" s="39" t="str">
+      <x:c r="V23" s="39" t="str">
         <x:f>IF(Hackathons!AB62="","",Hackathons!AB62)</x:f>
       </x:c>
-      <x:c r="P23" s="40" t="str">
-        <x:f>IF(Hackathons!AC62="","",Hackathons!AC62)</x:f>
-      </x:c>
-      <x:c r="Q23" s="36" t="str">
-        <x:f>IF(Hackathons!AD62="","",Hackathons!AD62)</x:f>
-      </x:c>
-      <x:c r="R23" s="36" t="str">
+      <x:c r="W23" s="36" t="str">
         <x:f>IF(Hackathons!AE62="","",Hackathons!AE62)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S23" s="36" t="str">
+      <x:c r="X23" s="36" t="str">
         <x:f>IF(Hackathons!AF62="","",Hackathons!AF62)</x:f>
         <x:v>Physical item, not cash</x:v>
-      </x:c>
-      <x:c r="T23" s="39" t="n">
-        <x:f>IF(Hackathons!AH62="","",Hackathons!AH62)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U23" s="291" t="str">
-        <x:f>IF(OR(F23="",T23=""),"",F23/T23)</x:f>
-      </x:c>
-      <x:c r="V23" s="291" t="str">
-        <x:f>IF(OR(H23="",T23=""),"",H23/T23)</x:f>
-      </x:c>
-      <x:c r="W23" s="291" t="str">
-        <x:f>IF(OR(K23="",T23=""),"",K23/T23)</x:f>
-      </x:c>
-      <x:c r="X23" s="291" t="str">
-        <x:f>IF(OR(P23="",T23=""),"",P23/T23)</x:f>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -16044,69 +16049,69 @@
       <x:c r="E24" s="36" t="str">
         <x:f>IF(Hackathons!R67="","",Hackathons!R67)</x:f>
       </x:c>
-      <x:c r="F24" s="40" t="str">
+      <x:c r="F24" s="36" t="n">
+        <x:f>IF(Hackathons!AH67="","",Hackathons!AH67)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G24" s="40" t="str">
         <x:f>IF(Hackathons!S67="","",Hackathons!S67)</x:f>
       </x:c>
-      <x:c r="G24" s="36" t="str">
+      <x:c r="H24" s="36" t="str">
         <x:f>IF(Hackathons!T67="","",Hackathons!T67)</x:f>
       </x:c>
-      <x:c r="H24" s="40" t="n">
+      <x:c r="I24" s="329" t="str">
+        <x:f>IF(OR(G24="",F24=""),"",G24/F24)</x:f>
+      </x:c>
+      <x:c r="J24" s="40" t="n">
         <x:f>IF(Hackathons!U67="","",Hackathons!U67)</x:f>
         <x:v>12000</x:v>
       </x:c>
-      <x:c r="I24" s="36" t="str">
+      <x:c r="K24" s="36" t="str">
         <x:f>IF(Hackathons!V67="","",Hackathons!V67)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="J24" s="39" t="str">
+      <x:c r="L24" s="329" t="n">
+        <x:f>IF(OR(J24="",F24=""),"",J24/F24)</x:f>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="M24" s="39" t="str">
         <x:f>IF(Hackathons!W67="","",Hackathons!W67)</x:f>
       </x:c>
-      <x:c r="K24" s="40" t="str">
+      <x:c r="N24" s="40" t="str">
         <x:f>IF(Hackathons!X67="","",Hackathons!X67)</x:f>
       </x:c>
-      <x:c r="L24" s="36" t="str">
+      <x:c r="O24" s="36" t="str">
         <x:f>IF(Hackathons!Y67="","",Hackathons!Y67)</x:f>
       </x:c>
-      <x:c r="M24" s="36" t="str">
+      <x:c r="P24" s="329" t="str">
+        <x:f>IF(OR(N24="",F24=""),"",N24/F24)</x:f>
+      </x:c>
+      <x:c r="Q24" s="40" t="str">
+        <x:f>IF(Hackathons!AC67="","",Hackathons!AC67)</x:f>
+      </x:c>
+      <x:c r="R24" s="36" t="str">
+        <x:f>IF(Hackathons!AD67="","",Hackathons!AD67)</x:f>
+      </x:c>
+      <x:c r="S24" s="329" t="str">
+        <x:f>IF(OR(Q24="",F24=""),"",Q24/F24)</x:f>
+      </x:c>
+      <x:c r="T24" s="36" t="str">
         <x:f>IF(Hackathons!Z67="","",Hackathons!Z67)</x:f>
         <x:v>10K OpenAI credits; 2K Gemini Cloud credits</x:v>
       </x:c>
-      <x:c r="N24" s="36" t="str">
+      <x:c r="U24" s="36" t="str">
         <x:f>IF(Hackathons!AA67="","",Hackathons!AA67)</x:f>
       </x:c>
-      <x:c r="O24" s="39" t="str">
+      <x:c r="V24" s="39" t="str">
         <x:f>IF(Hackathons!AB67="","",Hackathons!AB67)</x:f>
       </x:c>
-      <x:c r="P24" s="40" t="str">
-        <x:f>IF(Hackathons!AC67="","",Hackathons!AC67)</x:f>
-      </x:c>
-      <x:c r="Q24" s="36" t="str">
-        <x:f>IF(Hackathons!AD67="","",Hackathons!AD67)</x:f>
-      </x:c>
-      <x:c r="R24" s="36" t="str">
+      <x:c r="W24" s="36" t="str">
         <x:f>IF(Hackathons!AE67="","",Hackathons!AE67)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S24" s="36" t="str">
+      <x:c r="X24" s="36" t="str">
         <x:f>IF(Hackathons!AF67="","",Hackathons!AF67)</x:f>
         <x:v>Credit value total combines two USD-denominated credits</x:v>
-      </x:c>
-      <x:c r="T24" s="39" t="n">
-        <x:f>IF(Hackathons!AH67="","",Hackathons!AH67)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="U24" s="291" t="str">
-        <x:f>IF(OR(F24="",T24=""),"",F24/T24)</x:f>
-      </x:c>
-      <x:c r="V24" s="291" t="n">
-        <x:f>IF(OR(H24="",T24=""),"",H24/T24)</x:f>
-        <x:v>6000</x:v>
-      </x:c>
-      <x:c r="W24" s="291" t="str">
-        <x:f>IF(OR(K24="",T24=""),"",K24/T24)</x:f>
-      </x:c>
-      <x:c r="X24" s="291" t="str">
-        <x:f>IF(OR(P24="",T24=""),"",P24/T24)</x:f>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -16129,69 +16134,69 @@
       <x:c r="E25" s="36" t="str">
         <x:f>IF(Hackathons!R72="","",Hackathons!R72)</x:f>
       </x:c>
-      <x:c r="F25" s="40" t="str">
+      <x:c r="F25" s="36" t="n">
+        <x:f>IF(Hackathons!AH72="","",Hackathons!AH72)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G25" s="40" t="str">
         <x:f>IF(Hackathons!S72="","",Hackathons!S72)</x:f>
       </x:c>
-      <x:c r="G25" s="36" t="str">
+      <x:c r="H25" s="36" t="str">
         <x:f>IF(Hackathons!T72="","",Hackathons!T72)</x:f>
       </x:c>
-      <x:c r="H25" s="40" t="n">
+      <x:c r="I25" s="329" t="str">
+        <x:f>IF(OR(G25="",F25=""),"",G25/F25)</x:f>
+      </x:c>
+      <x:c r="J25" s="40" t="n">
         <x:f>IF(Hackathons!U72="","",Hackathons!U72)</x:f>
         <x:v>4500</x:v>
       </x:c>
-      <x:c r="I25" s="36" t="str">
+      <x:c r="K25" s="36" t="str">
         <x:f>IF(Hackathons!V72="","",Hackathons!V72)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="J25" s="39" t="str">
+      <x:c r="L25" s="329" t="n">
+        <x:f>IF(OR(J25="",F25=""),"",J25/F25)</x:f>
+        <x:v>2250</x:v>
+      </x:c>
+      <x:c r="M25" s="39" t="str">
         <x:f>IF(Hackathons!W72="","",Hackathons!W72)</x:f>
       </x:c>
-      <x:c r="K25" s="40" t="str">
+      <x:c r="N25" s="40" t="str">
         <x:f>IF(Hackathons!X72="","",Hackathons!X72)</x:f>
       </x:c>
-      <x:c r="L25" s="36" t="str">
+      <x:c r="O25" s="36" t="str">
         <x:f>IF(Hackathons!Y72="","",Hackathons!Y72)</x:f>
       </x:c>
-      <x:c r="M25" s="36" t="str">
+      <x:c r="P25" s="329" t="str">
+        <x:f>IF(OR(N25="",F25=""),"",N25/F25)</x:f>
+      </x:c>
+      <x:c r="Q25" s="40" t="str">
+        <x:f>IF(Hackathons!AC72="","",Hackathons!AC72)</x:f>
+      </x:c>
+      <x:c r="R25" s="36" t="str">
+        <x:f>IF(Hackathons!AD72="","",Hackathons!AD72)</x:f>
+      </x:c>
+      <x:c r="S25" s="329" t="str">
+        <x:f>IF(OR(Q25="",F25=""),"",Q25/F25)</x:f>
+      </x:c>
+      <x:c r="T25" s="36" t="str">
         <x:f>IF(Hackathons!Z72="","",Hackathons!Z72)</x:f>
         <x:v>AWS credits</x:v>
       </x:c>
-      <x:c r="N25" s="36" t="str">
+      <x:c r="U25" s="36" t="str">
         <x:f>IF(Hackathons!AA72="","",Hackathons!AA72)</x:f>
       </x:c>
-      <x:c r="O25" s="39" t="str">
+      <x:c r="V25" s="39" t="str">
         <x:f>IF(Hackathons!AB72="","",Hackathons!AB72)</x:f>
       </x:c>
-      <x:c r="P25" s="40" t="str">
-        <x:f>IF(Hackathons!AC72="","",Hackathons!AC72)</x:f>
-      </x:c>
-      <x:c r="Q25" s="36" t="str">
-        <x:f>IF(Hackathons!AD72="","",Hackathons!AD72)</x:f>
-      </x:c>
-      <x:c r="R25" s="36" t="str">
+      <x:c r="W25" s="36" t="str">
         <x:f>IF(Hackathons!AE72="","",Hackathons!AE72)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S25" s="36" t="str">
+      <x:c r="X25" s="36" t="str">
         <x:f>IF(Hackathons!AF72="","",Hackathons!AF72)</x:f>
         <x:v>USD-denominated credit value</x:v>
-      </x:c>
-      <x:c r="T25" s="39" t="n">
-        <x:f>IF(Hackathons!AH72="","",Hackathons!AH72)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="U25" s="291" t="str">
-        <x:f>IF(OR(F25="",T25=""),"",F25/T25)</x:f>
-      </x:c>
-      <x:c r="V25" s="291" t="n">
-        <x:f>IF(OR(H25="",T25=""),"",H25/T25)</x:f>
-        <x:v>2250</x:v>
-      </x:c>
-      <x:c r="W25" s="291" t="str">
-        <x:f>IF(OR(K25="",T25=""),"",K25/T25)</x:f>
-      </x:c>
-      <x:c r="X25" s="291" t="str">
-        <x:f>IF(OR(P25="",T25=""),"",P25/T25)</x:f>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -16215,69 +16220,69 @@
         <x:f>IF(Hackathons!R76="","",Hackathons!R76)</x:f>
         <x:v>Best Vertical Solution: Family Office Track</x:v>
       </x:c>
-      <x:c r="F26" s="40" t="str">
+      <x:c r="F26" s="36" t="n">
+        <x:f>IF(Hackathons!AH76="","",Hackathons!AH76)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G26" s="40" t="str">
         <x:f>IF(Hackathons!S76="","",Hackathons!S76)</x:f>
       </x:c>
-      <x:c r="G26" s="36" t="str">
+      <x:c r="H26" s="36" t="str">
         <x:f>IF(Hackathons!T76="","",Hackathons!T76)</x:f>
       </x:c>
-      <x:c r="H26" s="40" t="n">
+      <x:c r="I26" s="329" t="str">
+        <x:f>IF(OR(G26="",F26=""),"",G26/F26)</x:f>
+      </x:c>
+      <x:c r="J26" s="40" t="n">
         <x:f>IF(Hackathons!U76="","",Hackathons!U76)</x:f>
         <x:v>25</x:v>
       </x:c>
-      <x:c r="I26" s="36" t="str">
+      <x:c r="K26" s="36" t="str">
         <x:f>IF(Hackathons!V76="","",Hackathons!V76)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="J26" s="39" t="str">
+      <x:c r="L26" s="329" t="n">
+        <x:f>IF(OR(J26="",F26=""),"",J26/F26)</x:f>
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="M26" s="39" t="str">
         <x:f>IF(Hackathons!W76="","",Hackathons!W76)</x:f>
       </x:c>
-      <x:c r="K26" s="40" t="str">
+      <x:c r="N26" s="40" t="str">
         <x:f>IF(Hackathons!X76="","",Hackathons!X76)</x:f>
       </x:c>
-      <x:c r="L26" s="36" t="str">
+      <x:c r="O26" s="36" t="str">
         <x:f>IF(Hackathons!Y76="","",Hackathons!Y76)</x:f>
       </x:c>
-      <x:c r="M26" s="36" t="str">
+      <x:c r="P26" s="329" t="str">
+        <x:f>IF(OR(N26="",F26=""),"",N26/F26)</x:f>
+      </x:c>
+      <x:c r="Q26" s="40" t="str">
+        <x:f>IF(Hackathons!AC76="","",Hackathons!AC76)</x:f>
+      </x:c>
+      <x:c r="R26" s="36" t="str">
+        <x:f>IF(Hackathons!AD76="","",Hackathons!AD76)</x:f>
+      </x:c>
+      <x:c r="S26" s="329" t="str">
+        <x:f>IF(OR(Q26="",F26=""),"",Q26/F26)</x:f>
+      </x:c>
+      <x:c r="T26" s="36" t="str">
         <x:f>IF(Hackathons!Z76="","",Hackathons!Z76)</x:f>
         <x:v>2,000 Cybrdeck API credits</x:v>
       </x:c>
-      <x:c r="N26" s="36" t="str">
+      <x:c r="U26" s="36" t="str">
         <x:f>IF(Hackathons!AA76="","",Hackathons!AA76)</x:f>
       </x:c>
-      <x:c r="O26" s="39" t="str">
+      <x:c r="V26" s="39" t="str">
         <x:f>IF(Hackathons!AB76="","",Hackathons!AB76)</x:f>
       </x:c>
-      <x:c r="P26" s="40" t="str">
-        <x:f>IF(Hackathons!AC76="","",Hackathons!AC76)</x:f>
-      </x:c>
-      <x:c r="Q26" s="36" t="str">
-        <x:f>IF(Hackathons!AD76="","",Hackathons!AD76)</x:f>
-      </x:c>
-      <x:c r="R26" s="36" t="str">
+      <x:c r="W26" s="36" t="str">
         <x:f>IF(Hackathons!AE76="","",Hackathons!AE76)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S26" s="36" t="str">
+      <x:c r="X26" s="36" t="str">
         <x:f>IF(Hackathons!AF76="","",Hackathons!AF76)</x:f>
         <x:v>US$25 credit value, not cash</x:v>
-      </x:c>
-      <x:c r="T26" s="39" t="n">
-        <x:f>IF(Hackathons!AH76="","",Hackathons!AH76)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="U26" s="291" t="str">
-        <x:f>IF(OR(F26="",T26=""),"",F26/T26)</x:f>
-      </x:c>
-      <x:c r="V26" s="291" t="n">
-        <x:f>IF(OR(H26="",T26=""),"",H26/T26)</x:f>
-        <x:v>12.5</x:v>
-      </x:c>
-      <x:c r="W26" s="291" t="str">
-        <x:f>IF(OR(K26="",T26=""),"",K26/T26)</x:f>
-      </x:c>
-      <x:c r="X26" s="291" t="str">
-        <x:f>IF(OR(P26="",T26=""),"",P26/T26)</x:f>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -16301,71 +16306,71 @@
         <x:f>IF(Hackathons!R80="","",Hackathons!R80)</x:f>
         <x:v>SG × Sarawak AI &amp; Design Hackathon 2026</x:v>
       </x:c>
-      <x:c r="F27" s="40" t="str">
+      <x:c r="F27" s="36" t="n">
+        <x:f>IF(Hackathons!AH80="","",Hackathons!AH80)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G27" s="40" t="str">
         <x:f>IF(Hackathons!S80="","",Hackathons!S80)</x:f>
       </x:c>
-      <x:c r="G27" s="36" t="str">
+      <x:c r="H27" s="36" t="str">
         <x:f>IF(Hackathons!T80="","",Hackathons!T80)</x:f>
       </x:c>
-      <x:c r="H27" s="40" t="n">
+      <x:c r="I27" s="329" t="str">
+        <x:f>IF(OR(G27="",F27=""),"",G27/F27)</x:f>
+      </x:c>
+      <x:c r="J27" s="40" t="n">
         <x:f>IF(Hackathons!U80="","",Hackathons!U80)</x:f>
         <x:v>200</x:v>
       </x:c>
-      <x:c r="I27" s="36" t="str">
+      <x:c r="K27" s="36" t="str">
         <x:f>IF(Hackathons!V80="","",Hackathons!V80)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="J27" s="39" t="str">
+      <x:c r="L27" s="329" t="n">
+        <x:f>IF(OR(J27="",F27=""),"",J27/F27)</x:f>
+        <x:v>66.66666666666667</x:v>
+      </x:c>
+      <x:c r="M27" s="39" t="str">
         <x:f>IF(Hackathons!W80="","",Hackathons!W80)</x:f>
       </x:c>
-      <x:c r="K27" s="40" t="str">
+      <x:c r="N27" s="40" t="str">
         <x:f>IF(Hackathons!X80="","",Hackathons!X80)</x:f>
       </x:c>
-      <x:c r="L27" s="36" t="str">
+      <x:c r="O27" s="36" t="str">
         <x:f>IF(Hackathons!Y80="","",Hackathons!Y80)</x:f>
       </x:c>
-      <x:c r="M27" s="36" t="str">
+      <x:c r="P27" s="329" t="str">
+        <x:f>IF(OR(N27="",F27=""),"",N27/F27)</x:f>
+      </x:c>
+      <x:c r="Q27" s="40" t="str">
+        <x:f>IF(Hackathons!AC80="","",Hackathons!AC80)</x:f>
+      </x:c>
+      <x:c r="R27" s="36" t="str">
+        <x:f>IF(Hackathons!AD80="","",Hackathons!AD80)</x:f>
+      </x:c>
+      <x:c r="S27" s="329" t="str">
+        <x:f>IF(OR(Q27="",F27=""),"",Q27/F27)</x:f>
+      </x:c>
+      <x:c r="T27" s="36" t="str">
         <x:f>IF(Hackathons!Z80="","",Hackathons!Z80)</x:f>
         <x:v>Trophy; Kimi AI credits</x:v>
       </x:c>
-      <x:c r="N27" s="36" t="str">
+      <x:c r="U27" s="36" t="str">
         <x:f>IF(Hackathons!AA80="","",Hackathons!AA80)</x:f>
         <x:v>Trophy</x:v>
       </x:c>
-      <x:c r="O27" s="39" t="n">
+      <x:c r="V27" s="39" t="n">
         <x:f>IF(Hackathons!AB80="","",Hackathons!AB80)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="P27" s="40" t="str">
-        <x:f>IF(Hackathons!AC80="","",Hackathons!AC80)</x:f>
-      </x:c>
-      <x:c r="Q27" s="36" t="str">
-        <x:f>IF(Hackathons!AD80="","",Hackathons!AD80)</x:f>
-      </x:c>
-      <x:c r="R27" s="36" t="str">
+      <x:c r="W27" s="36" t="str">
         <x:f>IF(Hackathons!AE80="","",Hackathons!AE80)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S27" s="36" t="str">
+      <x:c r="X27" s="36" t="str">
         <x:f>IF(Hackathons!AF80="","",Hackathons!AF80)</x:f>
         <x:v>Trophy excluded; credit value tracked</x:v>
-      </x:c>
-      <x:c r="T27" s="39" t="n">
-        <x:f>IF(Hackathons!AH80="","",Hackathons!AH80)</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="U27" s="291" t="str">
-        <x:f>IF(OR(F27="",T27=""),"",F27/T27)</x:f>
-      </x:c>
-      <x:c r="V27" s="291" t="n">
-        <x:f>IF(OR(H27="",T27=""),"",H27/T27)</x:f>
-        <x:v>66.66666666666667</x:v>
-      </x:c>
-      <x:c r="W27" s="291" t="str">
-        <x:f>IF(OR(K27="",T27=""),"",K27/T27)</x:f>
-      </x:c>
-      <x:c r="X27" s="291" t="str">
-        <x:f>IF(OR(P27="",T27=""),"",P27/T27)</x:f>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -16389,69 +16394,69 @@
         <x:f>IF(Hackathons!R81="","",Hackathons!R81)</x:f>
         <x:v>Best Use of GPT-Image-2.5</x:v>
       </x:c>
-      <x:c r="F28" s="40" t="str">
+      <x:c r="F28" s="36" t="n">
+        <x:f>IF(Hackathons!AH81="","",Hackathons!AH81)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G28" s="40" t="str">
         <x:f>IF(Hackathons!S81="","",Hackathons!S81)</x:f>
       </x:c>
-      <x:c r="G28" s="36" t="str">
+      <x:c r="H28" s="36" t="str">
         <x:f>IF(Hackathons!T81="","",Hackathons!T81)</x:f>
       </x:c>
-      <x:c r="H28" s="40" t="n">
+      <x:c r="I28" s="329" t="str">
+        <x:f>IF(OR(G28="",F28=""),"",G28/F28)</x:f>
+      </x:c>
+      <x:c r="J28" s="40" t="n">
         <x:f>IF(Hackathons!U81="","",Hackathons!U81)</x:f>
         <x:v>5000</x:v>
       </x:c>
-      <x:c r="I28" s="36" t="str">
+      <x:c r="K28" s="36" t="str">
         <x:f>IF(Hackathons!V81="","",Hackathons!V81)</x:f>
         <x:v>USD</x:v>
       </x:c>
-      <x:c r="J28" s="39" t="str">
+      <x:c r="L28" s="329" t="n">
+        <x:f>IF(OR(J28="",F28=""),"",J28/F28)</x:f>
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="M28" s="39" t="str">
         <x:f>IF(Hackathons!W81="","",Hackathons!W81)</x:f>
       </x:c>
-      <x:c r="K28" s="40" t="str">
+      <x:c r="N28" s="40" t="str">
         <x:f>IF(Hackathons!X81="","",Hackathons!X81)</x:f>
       </x:c>
-      <x:c r="L28" s="36" t="str">
+      <x:c r="O28" s="36" t="str">
         <x:f>IF(Hackathons!Y81="","",Hackathons!Y81)</x:f>
       </x:c>
-      <x:c r="M28" s="36" t="str">
+      <x:c r="P28" s="329" t="str">
+        <x:f>IF(OR(N28="",F28=""),"",N28/F28)</x:f>
+      </x:c>
+      <x:c r="Q28" s="40" t="str">
+        <x:f>IF(Hackathons!AC81="","",Hackathons!AC81)</x:f>
+      </x:c>
+      <x:c r="R28" s="36" t="str">
+        <x:f>IF(Hackathons!AD81="","",Hackathons!AD81)</x:f>
+      </x:c>
+      <x:c r="S28" s="329" t="str">
+        <x:f>IF(OR(Q28="",F28=""),"",Q28/F28)</x:f>
+      </x:c>
+      <x:c r="T28" s="36" t="str">
         <x:f>IF(Hackathons!Z81="","",Hackathons!Z81)</x:f>
         <x:v>OpenAI credits</x:v>
       </x:c>
-      <x:c r="N28" s="36" t="str">
+      <x:c r="U28" s="36" t="str">
         <x:f>IF(Hackathons!AA81="","",Hackathons!AA81)</x:f>
       </x:c>
-      <x:c r="O28" s="39" t="str">
+      <x:c r="V28" s="39" t="str">
         <x:f>IF(Hackathons!AB81="","",Hackathons!AB81)</x:f>
       </x:c>
-      <x:c r="P28" s="40" t="str">
-        <x:f>IF(Hackathons!AC81="","",Hackathons!AC81)</x:f>
-      </x:c>
-      <x:c r="Q28" s="36" t="str">
-        <x:f>IF(Hackathons!AD81="","",Hackathons!AD81)</x:f>
-      </x:c>
-      <x:c r="R28" s="36" t="str">
+      <x:c r="W28" s="36" t="str">
         <x:f>IF(Hackathons!AE81="","",Hackathons!AE81)</x:f>
         <x:v>Exclude</x:v>
       </x:c>
-      <x:c r="S28" s="36" t="str">
+      <x:c r="X28" s="36" t="str">
         <x:f>IF(Hackathons!AF81="","",Hackathons!AF81)</x:f>
         <x:v>Credit value tracked</x:v>
-      </x:c>
-      <x:c r="T28" s="39" t="n">
-        <x:f>IF(Hackathons!AH81="","",Hackathons!AH81)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="U28" s="291" t="str">
-        <x:f>IF(OR(F28="",T28=""),"",F28/T28)</x:f>
-      </x:c>
-      <x:c r="V28" s="291" t="n">
-        <x:f>IF(OR(H28="",T28=""),"",H28/T28)</x:f>
-        <x:v>2500</x:v>
-      </x:c>
-      <x:c r="W28" s="291" t="str">
-        <x:f>IF(OR(K28="",T28=""),"",K28/T28)</x:f>
-      </x:c>
-      <x:c r="X28" s="291" t="str">
-        <x:f>IF(OR(P28="",T28=""),"",P28/T28)</x:f>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -16489,7 +16494,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d81d6b4bd0e435b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe6832ab8fa04574"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update Malcolm and Benjamin profiles for hackathon 82
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Re72da61c7dad482a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R486fec5c24a94426"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rb170c662b6d84d75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Red41e681a88243a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R1c9cf0af29df4e56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="Rf7c2e01acc31425d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R76d29f1f4a0e4656"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R0a1d1a34c8a14bfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R9f1fb4a151954edd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Ree2f052f15194a9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R6d162ff07e28483c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R9b35692b604646fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11489,7 +11489,7 @@
         <x:v>A 1-vs-1 fitness challenge app with AI-recommended rewards and Reap agentic payments tied to participants’ progress.</x:v>
       </x:c>
       <x:c r="J83" s="64" t="str">
-        <x:v>sayyid, malcolm, ben</x:v>
+        <x:v>sayyid, malcolm, Benjamin</x:v>
       </x:c>
       <x:c r="K83" s="64" t="str">
         <x:v>FitStake</x:v>
@@ -11541,10 +11541,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R6f38b84034494ad6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Re814593afa1c484a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="Rccbd3b8030fb44e8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R899dac60bcd74ecc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rae8b2e67944c4b45"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Ra1c9aa60b5c744e5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R8357c51be1ab4fb5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Rdfe66792bd1a45bb"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -13120,14 +13120,16 @@
       <x:c r="D99" s="9" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E99" s="10"/>
+      <x:c r="E99" s="10" t="str">
+        <x:v>https://www.linkedin.com/in/malcolm-t-804840113/</x:v>
+      </x:c>
     </x:row>
     <x:row r="100" ht="28" customHeight="1">
       <x:c r="A100" t="str">
         <x:v>P096</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>ben</x:v>
+        <x:v>Benjamin</x:v>
       </x:c>
       <x:c r="C100" t="str">
         <x:v>#082</x:v>
@@ -13135,7 +13137,9 @@
       <x:c r="D100" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E100"/>
+      <x:c r="E100" t="str">
+        <x:v>https://www.linkedin.com/in/sedilix/</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -13155,12 +13159,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rc565807ee679498e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R71fad2f457c8464b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rd0175f6f22c64cb5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R35e005e11b034f1f"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R135a4d7c01274a6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R528d3d039cf94be0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14142,7 +14146,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f2186b6f4834ffc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdf6a527acac44fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17704,7 +17708,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f7da744c5a14c47"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf87eb2df18404f6d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Improve hackathon insights, archive artwork, and interactive exhibits
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R76d29f1f4a0e4656"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R0a1d1a34c8a14bfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R9f1fb4a151954edd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="Ree2f052f15194a9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="R6d162ff07e28483c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R9b35692b604646fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R25fece26f46847ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rdbd7b65706734ef6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R33f6e60656bc4cb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Map" sheetId="4" r:id="R8212702754f649f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Money" sheetId="5" r:id="Rb26454f442d8450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prize Details" sheetId="6" r:id="R4b7d63b711a749d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -847,9 +847,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Singapore X Sarawak</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sarawak</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Makeramai Makerspace, Kuching, Sarawak, Malaysia</x:t>
@@ -8224,11 +8221,11 @@
       <x:c r="L41" t="s">
         <x:v>277</x:v>
       </x:c>
-      <x:c r="M41" t="s">
+      <x:c r="M41" t="str">
+        <x:v>Malaysia</x:v>
+      </x:c>
+      <x:c r="N41" t="s">
         <x:v>278</x:v>
-      </x:c>
-      <x:c r="N41" t="s">
-        <x:v>279</x:v>
       </x:c>
       <x:c r="O41" t="s">
         <x:v>8</x:v>
@@ -8281,10 +8278,10 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B42" t="s">
+        <x:v>279</x:v>
+      </x:c>
+      <x:c r="C42" t="s">
         <x:v>280</x:v>
-      </x:c>
-      <x:c r="C42" t="s">
-        <x:v>281</x:v>
       </x:c>
       <x:c r="D42" s="4">
         <x:v>45920</x:v>
@@ -8299,13 +8296,13 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H42" t="s">
+        <x:v>281</x:v>
+      </x:c>
+      <x:c r="I42" t="s">
         <x:v>282</x:v>
       </x:c>
-      <x:c r="I42" t="s">
+      <x:c r="J42" t="s">
         <x:v>283</x:v>
-      </x:c>
-      <x:c r="J42" t="s">
-        <x:v>284</x:v>
       </x:c>
       <x:c r="K42" t="s">
         <x:v>8</x:v>
@@ -8314,10 +8311,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="N42" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="O42" t="s">
         <x:v>285</x:v>
-      </x:c>
-      <x:c r="O42" t="s">
-        <x:v>286</x:v>
       </x:c>
       <x:c r="P42" t="s">
         <x:v>8</x:v>
@@ -8350,10 +8347,10 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="B43" t="s">
+        <x:v>286</x:v>
+      </x:c>
+      <x:c r="C43" t="s">
         <x:v>287</x:v>
-      </x:c>
-      <x:c r="C43" t="s">
-        <x:v>288</x:v>
       </x:c>
       <x:c r="D43" s="4">
         <x:v>45930</x:v>
@@ -8368,28 +8365,28 @@
         <x:v>1st Place — US$500 Nosana Cloud Credits</x:v>
       </x:c>
       <x:c r="H43" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="I43" t="s">
         <x:v>289</x:v>
       </x:c>
-      <x:c r="I43" t="s">
+      <x:c r="J43" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K43" t="s">
         <x:v>290</x:v>
       </x:c>
-      <x:c r="J43" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K43" t="s">
-        <x:v>291</x:v>
-      </x:c>
       <x:c r="L43" t="s">
-        <x:v>288</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="M43" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="N43" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="O43" t="s">
         <x:v>292</x:v>
-      </x:c>
-      <x:c r="O43" t="s">
-        <x:v>293</x:v>
       </x:c>
       <x:c r="P43" t="s">
         <x:v>8</x:v>
@@ -8439,10 +8436,10 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B44" t="s">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="C44" t="s">
         <x:v>294</x:v>
-      </x:c>
-      <x:c r="C44" t="s">
-        <x:v>295</x:v>
       </x:c>
       <x:c r="D44" s="5">
         <x:v>45932</x:v>
@@ -8457,16 +8454,16 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H44" t="s">
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="I44" t="s">
         <x:v>296</x:v>
       </x:c>
-      <x:c r="I44" t="s">
+      <x:c r="J44" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K44" t="s">
         <x:v>297</x:v>
-      </x:c>
-      <x:c r="J44" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K44" t="s">
-        <x:v>298</x:v>
       </x:c>
       <x:c r="L44" t="s">
         <x:v>8</x:v>
@@ -8511,13 +8508,13 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B45" t="s">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="C45" t="s">
         <x:v>299</x:v>
       </x:c>
-      <x:c r="C45" t="s">
+      <x:c r="D45" s="2" t="s">
         <x:v>300</x:v>
-      </x:c>
-      <x:c r="D45" s="2" t="s">
-        <x:v>301</x:v>
       </x:c>
       <x:c r="E45">
         <x:v>2</x:v>
@@ -8532,16 +8529,16 @@
         <x:v>242</x:v>
       </x:c>
       <x:c r="I45" t="s">
+        <x:v>301</x:v>
+      </x:c>
+      <x:c r="J45" t="s">
         <x:v>302</x:v>
       </x:c>
-      <x:c r="J45" t="s">
+      <x:c r="K45" t="s">
         <x:v>303</x:v>
       </x:c>
-      <x:c r="K45" t="s">
+      <x:c r="L45" t="s">
         <x:v>304</x:v>
-      </x:c>
-      <x:c r="L45" t="s">
-        <x:v>305</x:v>
       </x:c>
       <x:c r="M45" t="s">
         <x:v>9</x:v>
@@ -8550,7 +8547,7 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="O45" t="s">
-        <x:v>306</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="P45" t="s">
         <x:v>8</x:v>
@@ -8583,10 +8580,10 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="B46" t="s">
+        <x:v>306</x:v>
+      </x:c>
+      <x:c r="C46" t="s">
         <x:v>307</x:v>
-      </x:c>
-      <x:c r="C46" t="s">
-        <x:v>308</x:v>
       </x:c>
       <x:c r="D46" s="5">
         <x:v>45954</x:v>
@@ -8604,25 +8601,25 @@
         <x:v>242</x:v>
       </x:c>
       <x:c r="I46" t="s">
+        <x:v>308</x:v>
+      </x:c>
+      <x:c r="J46" t="s">
         <x:v>309</x:v>
       </x:c>
-      <x:c r="J46" t="s">
+      <x:c r="K46" t="s">
         <x:v>310</x:v>
       </x:c>
-      <x:c r="K46" t="s">
+      <x:c r="L46" t="s">
         <x:v>311</x:v>
-      </x:c>
-      <x:c r="L46" t="s">
-        <x:v>312</x:v>
       </x:c>
       <x:c r="M46" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="N46" t="s">
+        <x:v>312</x:v>
+      </x:c>
+      <x:c r="O46" t="s">
         <x:v>313</x:v>
-      </x:c>
-      <x:c r="O46" t="s">
-        <x:v>314</x:v>
       </x:c>
       <x:c r="P46" t="s">
         <x:v>8</x:v>
@@ -8655,13 +8652,13 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="B47" t="s">
+        <x:v>314</x:v>
+      </x:c>
+      <x:c r="C47" t="s">
         <x:v>315</x:v>
       </x:c>
-      <x:c r="C47" t="s">
+      <x:c r="D47" s="5" t="s">
         <x:v>316</x:v>
-      </x:c>
-      <x:c r="D47" s="5" t="s">
-        <x:v>317</x:v>
       </x:c>
       <x:c r="E47">
         <x:v>2.5</x:v>
@@ -8673,28 +8670,28 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H47" t="s">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="I47" t="s">
         <x:v>318</x:v>
       </x:c>
-      <x:c r="I47" t="s">
+      <x:c r="J47" t="s">
         <x:v>319</x:v>
       </x:c>
-      <x:c r="J47" t="s">
+      <x:c r="K47" t="s">
         <x:v>320</x:v>
       </x:c>
-      <x:c r="K47" t="s">
+      <x:c r="L47" t="s">
         <x:v>321</x:v>
-      </x:c>
-      <x:c r="L47" t="s">
-        <x:v>322</x:v>
       </x:c>
       <x:c r="M47" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="N47" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="O47" t="s">
         <x:v>323</x:v>
-      </x:c>
-      <x:c r="O47" t="s">
-        <x:v>324</x:v>
       </x:c>
       <x:c r="P47" t="s">
         <x:v>8</x:v>
@@ -8727,13 +8724,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="B48" t="s">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="C48" t="s">
         <x:v>325</x:v>
       </x:c>
-      <x:c r="C48" t="s">
+      <x:c r="D48" s="2" t="s">
         <x:v>326</x:v>
-      </x:c>
-      <x:c r="D48" s="2" t="s">
-        <x:v>327</x:v>
       </x:c>
       <x:c r="E48">
         <x:v>2</x:v>
@@ -8748,25 +8745,25 @@
         <x:v>242</x:v>
       </x:c>
       <x:c r="I48" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="J48" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K48" t="s">
         <x:v>328</x:v>
       </x:c>
-      <x:c r="J48" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K48" t="s">
-        <x:v>329</x:v>
-      </x:c>
       <x:c r="L48" t="s">
-        <x:v>326</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="M48" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="N48" t="s">
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="O48" t="s">
         <x:v>330</x:v>
-      </x:c>
-      <x:c r="O48" t="s">
-        <x:v>331</x:v>
       </x:c>
       <x:c r="P48" t="s">
         <x:v>8</x:v>
@@ -8799,13 +8796,13 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B49" t="s">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="C49" t="s">
         <x:v>325</x:v>
       </x:c>
-      <x:c r="C49" t="s">
+      <x:c r="D49" s="2" t="s">
         <x:v>326</x:v>
-      </x:c>
-      <x:c r="D49" s="2" t="s">
-        <x:v>327</x:v>
       </x:c>
       <x:c r="E49">
         <x:v>2</x:v>
@@ -8820,25 +8817,25 @@
         <x:v>242</x:v>
       </x:c>
       <x:c r="I49" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="J49" t="s">
         <x:v>332</x:v>
       </x:c>
-      <x:c r="J49" t="s">
+      <x:c r="K49" t="s">
         <x:v>333</x:v>
       </x:c>
-      <x:c r="K49" t="s">
-        <x:v>334</x:v>
-      </x:c>
       <x:c r="L49" t="s">
-        <x:v>326</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="M49" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="N49" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="O49" t="s">
-        <x:v>335</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="P49" t="s">
         <x:v>8</x:v>
@@ -8871,13 +8868,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B50" t="s">
+        <x:v>335</x:v>
+      </x:c>
+      <x:c r="C50" t="s">
         <x:v>336</x:v>
       </x:c>
-      <x:c r="C50" t="s">
+      <x:c r="D50" s="3" t="s">
         <x:v>337</x:v>
-      </x:c>
-      <x:c r="D50" s="3" t="s">
-        <x:v>338</x:v>
       </x:c>
       <x:c r="E50">
         <x:v>1</x:v>
@@ -8889,31 +8886,31 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H50" t="s">
+        <x:v>338</x:v>
+      </x:c>
+      <x:c r="I50" t="s">
         <x:v>339</x:v>
       </x:c>
-      <x:c r="I50" t="s">
+      <x:c r="J50" t="s">
         <x:v>340</x:v>
       </x:c>
-      <x:c r="J50" t="s">
+      <x:c r="K50" t="s">
         <x:v>341</x:v>
       </x:c>
-      <x:c r="K50" t="s">
+      <x:c r="L50" s="6" t="s">
         <x:v>342</x:v>
-      </x:c>
-      <x:c r="L50" s="6" t="s">
-        <x:v>343</x:v>
       </x:c>
       <x:c r="M50" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="N50" t="s">
+        <x:v>343</x:v>
+      </x:c>
+      <x:c r="O50" t="s">
         <x:v>344</x:v>
       </x:c>
-      <x:c r="O50" t="s">
+      <x:c r="P50" t="s">
         <x:v>345</x:v>
-      </x:c>
-      <x:c r="P50" t="s">
-        <x:v>346</x:v>
       </x:c>
       <x:c r="Q50" s="36"/>
       <x:c r="R50" s="36"/>
@@ -8943,10 +8940,10 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="B51" t="s">
+        <x:v>346</x:v>
+      </x:c>
+      <x:c r="C51" t="s">
         <x:v>347</x:v>
-      </x:c>
-      <x:c r="C51" t="s">
-        <x:v>348</x:v>
       </x:c>
       <x:c r="D51" s="5">
         <x:v>46205</x:v>
@@ -8961,31 +8958,31 @@
         <x:v>1st Place — US$1,000 OpenRouter Credits</x:v>
       </x:c>
       <x:c r="H51" t="s">
+        <x:v>348</x:v>
+      </x:c>
+      <x:c r="I51" t="s">
         <x:v>349</x:v>
       </x:c>
-      <x:c r="I51" t="s">
+      <x:c r="J51" t="s">
         <x:v>350</x:v>
       </x:c>
-      <x:c r="J51" t="s">
+      <x:c r="K51" t="s">
         <x:v>351</x:v>
       </x:c>
-      <x:c r="K51" t="s">
+      <x:c r="L51" t="s">
         <x:v>352</x:v>
-      </x:c>
-      <x:c r="L51" t="s">
-        <x:v>353</x:v>
       </x:c>
       <x:c r="M51" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="N51" t="s">
-        <x:v>292</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="O51" t="s">
+        <x:v>353</x:v>
+      </x:c>
+      <x:c r="P51" t="s">
         <x:v>354</x:v>
-      </x:c>
-      <x:c r="P51" t="s">
-        <x:v>355</x:v>
       </x:c>
       <x:c r="Q51" s="36" t="str">
         <x:v>1st Prize</x:v>
@@ -9032,10 +9029,10 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="B52" t="s">
+        <x:v>346</x:v>
+      </x:c>
+      <x:c r="C52" t="s">
         <x:v>347</x:v>
-      </x:c>
-      <x:c r="C52" t="s">
-        <x:v>348</x:v>
       </x:c>
       <x:c r="D52" s="5">
         <x:v>46205</x:v>
@@ -9050,31 +9047,31 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H52" t="s">
-        <x:v>349</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="I52" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="J52" t="s">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="K52" t="s">
         <x:v>356</x:v>
       </x:c>
-      <x:c r="J52" t="s">
-        <x:v>351</x:v>
-      </x:c>
-      <x:c r="K52" t="s">
-        <x:v>357</x:v>
-      </x:c>
       <x:c r="L52" t="s">
-        <x:v>353</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="M52" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="N52" t="s">
-        <x:v>292</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="O52" t="s">
-        <x:v>358</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="P52" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="Q52" s="36"/>
       <x:c r="R52" s="36"/>
@@ -9104,13 +9101,13 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="B53" t="s">
+        <x:v>358</x:v>
+      </x:c>
+      <x:c r="C53" t="s">
+        <x:v>347</x:v>
+      </x:c>
+      <x:c r="D53" s="2" t="s">
         <x:v>359</x:v>
-      </x:c>
-      <x:c r="C53" t="s">
-        <x:v>348</x:v>
-      </x:c>
-      <x:c r="D53" s="2" t="s">
-        <x:v>360</x:v>
       </x:c>
       <x:c r="E53">
         <x:v>1</x:v>
@@ -9122,19 +9119,19 @@
         <x:v>1st Place — US$500 API Credits</x:v>
       </x:c>
       <x:c r="H53" t="s">
-        <x:v>349</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="I53" t="s">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="J53" t="s">
+        <x:v>340</x:v>
+      </x:c>
+      <x:c r="K53" t="s">
         <x:v>361</x:v>
       </x:c>
-      <x:c r="J53" t="s">
-        <x:v>341</x:v>
-      </x:c>
-      <x:c r="K53" t="s">
+      <x:c r="L53" t="s">
         <x:v>362</x:v>
-      </x:c>
-      <x:c r="L53" t="s">
-        <x:v>363</x:v>
       </x:c>
       <x:c r="M53" t="s">
         <x:v>9</x:v>
@@ -9143,10 +9140,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="O53" t="s">
+        <x:v>363</x:v>
+      </x:c>
+      <x:c r="P53" t="s">
         <x:v>364</x:v>
-      </x:c>
-      <x:c r="P53" t="s">
-        <x:v>365</x:v>
       </x:c>
       <x:c r="Q53" s="36" t="str">
         <x:v>1st Prize</x:v>
@@ -9193,13 +9190,13 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="B54" t="s">
+        <x:v>358</x:v>
+      </x:c>
+      <x:c r="C54" t="s">
+        <x:v>347</x:v>
+      </x:c>
+      <x:c r="D54" s="2" t="s">
         <x:v>359</x:v>
-      </x:c>
-      <x:c r="C54" t="s">
-        <x:v>348</x:v>
-      </x:c>
-      <x:c r="D54" s="2" t="s">
-        <x:v>360</x:v>
       </x:c>
       <x:c r="E54">
         <x:v>1</x:v>
@@ -9211,19 +9208,19 @@
         <x:v>1st Place — US$500 API Credits</x:v>
       </x:c>
       <x:c r="H54" t="s">
-        <x:v>349</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="I54" t="s">
+        <x:v>365</x:v>
+      </x:c>
+      <x:c r="J54" t="s">
+        <x:v>340</x:v>
+      </x:c>
+      <x:c r="K54" t="s">
         <x:v>366</x:v>
       </x:c>
-      <x:c r="J54" t="s">
-        <x:v>341</x:v>
-      </x:c>
-      <x:c r="K54" t="s">
+      <x:c r="L54" t="s">
         <x:v>367</x:v>
-      </x:c>
-      <x:c r="L54" t="s">
-        <x:v>368</x:v>
       </x:c>
       <x:c r="M54" t="s">
         <x:v>9</x:v>
@@ -9232,10 +9229,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="O54" t="s">
-        <x:v>369</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="P54" t="s">
-        <x:v>365</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="Q54" s="36" t="str">
         <x:v>1st Prize</x:v>
@@ -9282,13 +9279,13 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="B55" t="s">
+        <x:v>369</x:v>
+      </x:c>
+      <x:c r="C55" s="6" t="s">
         <x:v>370</x:v>
       </x:c>
-      <x:c r="C55" s="6" t="s">
+      <x:c r="D55" s="2" t="s">
         <x:v>371</x:v>
-      </x:c>
-      <x:c r="D55" s="2" t="s">
-        <x:v>372</x:v>
       </x:c>
       <x:c r="E55">
         <x:v>1</x:v>
@@ -9300,16 +9297,16 @@
         <x:v>1st Place — US$150 Wavespeed AI Credits</x:v>
       </x:c>
       <x:c r="H55" t="s">
+        <x:v>372</x:v>
+      </x:c>
+      <x:c r="I55" s="6" t="s">
         <x:v>373</x:v>
       </x:c>
-      <x:c r="I55" s="6" t="s">
+      <x:c r="J55" t="s">
         <x:v>374</x:v>
       </x:c>
-      <x:c r="J55" t="s">
+      <x:c r="K55" t="s">
         <x:v>375</x:v>
-      </x:c>
-      <x:c r="K55" t="s">
-        <x:v>376</x:v>
       </x:c>
       <x:c r="L55" t="s">
         <x:v>8</x:v>
@@ -9318,13 +9315,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="N55" t="s">
-        <x:v>377</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="O55" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="P55" t="s">
-        <x:v>378</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="Q55" s="36" t="str">
         <x:v>1st Prize</x:v>
@@ -9371,13 +9368,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="B56" t="s">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="C56" t="s">
         <x:v>379</x:v>
       </x:c>
-      <x:c r="C56" t="s">
+      <x:c r="D56" s="2" t="s">
         <x:v>380</x:v>
-      </x:c>
-      <x:c r="D56" s="2" t="s">
-        <x:v>381</x:v>
       </x:c>
       <x:c r="E56">
         <x:v>1</x:v>
@@ -9389,16 +9386,16 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H56" t="s">
-        <x:v>373</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="I56" s="6" t="s">
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="J56" t="s">
+        <x:v>374</x:v>
+      </x:c>
+      <x:c r="K56" t="s">
         <x:v>382</x:v>
-      </x:c>
-      <x:c r="J56" t="s">
-        <x:v>375</x:v>
-      </x:c>
-      <x:c r="K56" t="s">
-        <x:v>383</x:v>
       </x:c>
       <x:c r="L56" t="s">
         <x:v>8</x:v>
@@ -9413,7 +9410,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="P56" t="s">
-        <x:v>384</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="Q56" s="36"/>
       <x:c r="R56" s="36"/>
@@ -9443,10 +9440,10 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B57" t="s">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="C57" t="s">
         <x:v>385</x:v>
-      </x:c>
-      <x:c r="C57" t="s">
-        <x:v>386</x:v>
       </x:c>
       <x:c r="D57" s="5">
         <x:v>46207</x:v>
@@ -9461,16 +9458,16 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H57" t="s">
-        <x:v>373</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="I57" t="s">
+        <x:v>386</x:v>
+      </x:c>
+      <x:c r="J57" t="s">
         <x:v>387</x:v>
       </x:c>
-      <x:c r="J57" t="s">
+      <x:c r="K57" t="s">
         <x:v>388</x:v>
-      </x:c>
-      <x:c r="K57" t="s">
-        <x:v>389</x:v>
       </x:c>
       <x:c r="L57" t="s">
         <x:v>8</x:v>
@@ -9482,10 +9479,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="O57" t="s">
+        <x:v>389</x:v>
+      </x:c>
+      <x:c r="P57" t="s">
         <x:v>390</x:v>
-      </x:c>
-      <x:c r="P57" t="s">
-        <x:v>391</x:v>
       </x:c>
       <x:c r="Q57" s="36"/>
       <x:c r="R57" s="36"/>
@@ -9515,10 +9512,10 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="B58" t="s">
+        <x:v>391</x:v>
+      </x:c>
+      <x:c r="C58" t="s">
         <x:v>392</x:v>
-      </x:c>
-      <x:c r="C58" t="s">
-        <x:v>393</x:v>
       </x:c>
       <x:c r="D58" s="5">
         <x:v>46299</x:v>
@@ -9533,16 +9530,16 @@
         <x:v>3rd Place — S$300 Cash + S$385 API Credits</x:v>
       </x:c>
       <x:c r="H58" t="s">
+        <x:v>393</x:v>
+      </x:c>
+      <x:c r="I58" t="s">
         <x:v>394</x:v>
       </x:c>
-      <x:c r="I58" t="s">
+      <x:c r="J58" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K58" t="s">
         <x:v>395</x:v>
-      </x:c>
-      <x:c r="J58" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K58" t="s">
-        <x:v>396</x:v>
       </x:c>
       <x:c r="L58" t="s">
         <x:v>8</x:v>
@@ -9551,13 +9548,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="N58" t="s">
+        <x:v>396</x:v>
+      </x:c>
+      <x:c r="O58" t="s">
         <x:v>397</x:v>
       </x:c>
-      <x:c r="O58" t="s">
+      <x:c r="P58" t="s">
         <x:v>398</x:v>
-      </x:c>
-      <x:c r="P58" t="s">
-        <x:v>399</x:v>
       </x:c>
       <x:c r="Q58" s="36" t="str">
         <x:v>3rd Prize</x:v>
@@ -9608,13 +9605,13 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="B59" t="s">
+        <x:v>399</x:v>
+      </x:c>
+      <x:c r="C59" t="s">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="C59" t="s">
+      <x:c r="D59" s="2" t="s">
         <x:v>401</x:v>
-      </x:c>
-      <x:c r="D59" s="2" t="s">
-        <x:v>402</x:v>
       </x:c>
       <x:c r="E59">
         <x:v>1</x:v>
@@ -9629,16 +9626,16 @@
         <x:v>118</x:v>
       </x:c>
       <x:c r="I59" t="s">
+        <x:v>402</x:v>
+      </x:c>
+      <x:c r="J59" t="s">
         <x:v>403</x:v>
       </x:c>
-      <x:c r="J59" t="s">
+      <x:c r="K59" t="s">
         <x:v>404</x:v>
       </x:c>
-      <x:c r="K59" t="s">
+      <x:c r="L59" t="s">
         <x:v>405</x:v>
-      </x:c>
-      <x:c r="L59" t="s">
-        <x:v>406</x:v>
       </x:c>
       <x:c r="M59" t="s">
         <x:v>9</x:v>
@@ -9647,10 +9644,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="O59" t="s">
+        <x:v>406</x:v>
+      </x:c>
+      <x:c r="P59" t="s">
         <x:v>407</x:v>
-      </x:c>
-      <x:c r="P59" t="s">
-        <x:v>408</x:v>
       </x:c>
       <x:c r="Q59" s="36"/>
       <x:c r="R59" s="36"/>
@@ -9680,13 +9677,13 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B60" t="s">
+        <x:v>408</x:v>
+      </x:c>
+      <x:c r="C60" t="s">
         <x:v>409</x:v>
       </x:c>
-      <x:c r="C60" t="s">
+      <x:c r="D60" s="2" t="s">
         <x:v>410</x:v>
-      </x:c>
-      <x:c r="D60" s="2" t="s">
-        <x:v>411</x:v>
       </x:c>
       <x:c r="E60">
         <x:v>1</x:v>
@@ -9698,16 +9695,16 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H60" t="s">
+        <x:v>411</x:v>
+      </x:c>
+      <x:c r="I60" t="s">
         <x:v>412</x:v>
       </x:c>
-      <x:c r="I60" t="s">
+      <x:c r="J60" t="s">
         <x:v>413</x:v>
       </x:c>
-      <x:c r="J60" t="s">
+      <x:c r="K60" t="s">
         <x:v>414</x:v>
-      </x:c>
-      <x:c r="K60" t="s">
-        <x:v>415</x:v>
       </x:c>
       <x:c r="L60" t="s">
         <x:v>8</x:v>
@@ -9716,13 +9713,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="N60" t="s">
+        <x:v>415</x:v>
+      </x:c>
+      <x:c r="O60" t="s">
         <x:v>416</x:v>
       </x:c>
-      <x:c r="O60" t="s">
+      <x:c r="P60" t="s">
         <x:v>417</x:v>
-      </x:c>
-      <x:c r="P60" t="s">
-        <x:v>418</x:v>
       </x:c>
       <x:c r="Q60" s="36"/>
       <x:c r="R60" s="36"/>
@@ -9752,13 +9749,13 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="B61" t="s">
+        <x:v>418</x:v>
+      </x:c>
+      <x:c r="C61" t="s">
         <x:v>419</x:v>
       </x:c>
-      <x:c r="C61" t="s">
+      <x:c r="D61" s="2" t="s">
         <x:v>420</x:v>
-      </x:c>
-      <x:c r="D61" s="2" t="s">
-        <x:v>421</x:v>
       </x:c>
       <x:c r="E61">
         <x:v>1</x:v>
@@ -9770,16 +9767,16 @@
         <x:v>Award — Speechmatics — US$2,000 Speechmatics Credits</x:v>
       </x:c>
       <x:c r="H61" t="s">
+        <x:v>421</x:v>
+      </x:c>
+      <x:c r="I61" t="s">
         <x:v>422</x:v>
       </x:c>
-      <x:c r="I61" t="s">
+      <x:c r="J61" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K61" t="s">
         <x:v>423</x:v>
-      </x:c>
-      <x:c r="J61" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K61" t="s">
-        <x:v>424</x:v>
       </x:c>
       <x:c r="L61" t="s">
         <x:v>8</x:v>
@@ -9788,13 +9785,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="N61" t="s">
+        <x:v>424</x:v>
+      </x:c>
+      <x:c r="O61" t="s">
         <x:v>425</x:v>
       </x:c>
-      <x:c r="O61" t="s">
+      <x:c r="P61" s="1" t="s">
         <x:v>426</x:v>
-      </x:c>
-      <x:c r="P61" s="1" t="s">
-        <x:v>427</x:v>
       </x:c>
       <x:c r="Q61" s="36" t="str">
         <x:v>Award</x:v>
@@ -9843,13 +9840,13 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="B62" t="s">
+        <x:v>427</x:v>
+      </x:c>
+      <x:c r="C62" t="s">
         <x:v>428</x:v>
       </x:c>
-      <x:c r="C62" t="s">
+      <x:c r="D62" s="2" t="s">
         <x:v>429</x:v>
-      </x:c>
-      <x:c r="D62" s="2" t="s">
-        <x:v>430</x:v>
       </x:c>
       <x:c r="E62">
         <x:v>1</x:v>
@@ -9861,16 +9858,16 @@
         <x:v>2nd Place — v0 Sock</x:v>
       </x:c>
       <x:c r="H62" t="s">
+        <x:v>430</x:v>
+      </x:c>
+      <x:c r="I62" t="s">
         <x:v>431</x:v>
       </x:c>
-      <x:c r="I62" t="s">
+      <x:c r="J62" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K62" t="s">
         <x:v>432</x:v>
-      </x:c>
-      <x:c r="J62" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K62" t="s">
-        <x:v>433</x:v>
       </x:c>
       <x:c r="L62" t="s">
         <x:v>8</x:v>
@@ -9885,7 +9882,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="P62" s="1" t="s">
-        <x:v>434</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="Q62" s="36" t="str">
         <x:v>2nd Place</x:v>
@@ -9934,10 +9931,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="B63" t="s">
+        <x:v>434</x:v>
+      </x:c>
+      <x:c r="C63" t="s">
         <x:v>435</x:v>
-      </x:c>
-      <x:c r="C63" t="s">
-        <x:v>436</x:v>
       </x:c>
       <x:c r="D63" s="5">
         <x:v>46085</x:v>
@@ -9946,22 +9943,22 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F63" t="s">
-        <x:v>437</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="G63" t="str">
         <x:v>-</x:v>
       </x:c>
       <x:c r="H63" t="s">
-        <x:v>373</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="I63" t="s">
+        <x:v>437</x:v>
+      </x:c>
+      <x:c r="J63" t="s">
+        <x:v>374</x:v>
+      </x:c>
+      <x:c r="K63" t="s">
         <x:v>438</x:v>
-      </x:c>
-      <x:c r="J63" t="s">
-        <x:v>375</x:v>
-      </x:c>
-      <x:c r="K63" t="s">
-        <x:v>439</x:v>
       </x:c>
       <x:c r="L63" t="s">
         <x:v>8</x:v>
@@ -9970,13 +9967,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="N63" t="s">
+        <x:v>439</x:v>
+      </x:c>
+      <x:c r="O63" t="s">
         <x:v>440</x:v>
       </x:c>
-      <x:c r="O63" t="s">
+      <x:c r="P63" t="s">
         <x:v>441</x:v>
-      </x:c>
-      <x:c r="P63" t="s">
-        <x:v>442</x:v>
       </x:c>
       <x:c r="Q63" s="36"/>
       <x:c r="R63" s="36"/>
@@ -10006,10 +10003,10 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="B64" t="s">
-        <x:v>443</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="C64" t="s">
-        <x:v>429</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="D64" s="5">
         <x:v>46116</x:v>
@@ -10024,16 +10021,16 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H64" t="s">
-        <x:v>431</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="I64" t="s">
+        <x:v>443</x:v>
+      </x:c>
+      <x:c r="J64" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K64" t="s">
         <x:v>444</x:v>
-      </x:c>
-      <x:c r="J64" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K64" t="s">
-        <x:v>445</x:v>
       </x:c>
       <x:c r="L64" t="s">
         <x:v>8</x:v>
@@ -10042,13 +10039,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="N64" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="O64" t="s">
+        <x:v>445</x:v>
+      </x:c>
+      <x:c r="P64" t="s">
         <x:v>446</x:v>
-      </x:c>
-      <x:c r="P64" t="s">
-        <x:v>447</x:v>
       </x:c>
       <x:c r="Q64" s="36"/>
       <x:c r="R64" s="36"/>
@@ -10078,10 +10075,10 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="B65" t="s">
+        <x:v>447</x:v>
+      </x:c>
+      <x:c r="C65" t="s">
         <x:v>448</x:v>
-      </x:c>
-      <x:c r="C65" t="s">
-        <x:v>449</x:v>
       </x:c>
       <x:c r="D65" s="5">
         <x:v>46270</x:v>
@@ -10096,16 +10093,16 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H65" t="s">
-        <x:v>431</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="I65" t="s">
+        <x:v>449</x:v>
+      </x:c>
+      <x:c r="J65" t="s">
         <x:v>450</x:v>
       </x:c>
-      <x:c r="J65" t="s">
+      <x:c r="K65" t="s">
         <x:v>451</x:v>
-      </x:c>
-      <x:c r="K65" t="s">
-        <x:v>452</x:v>
       </x:c>
       <x:c r="L65" t="s">
         <x:v>8</x:v>
@@ -10117,10 +10114,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="O65" t="s">
+        <x:v>452</x:v>
+      </x:c>
+      <x:c r="P65" t="s">
         <x:v>453</x:v>
-      </x:c>
-      <x:c r="P65" t="s">
-        <x:v>454</x:v>
       </x:c>
       <x:c r="Q65" s="36"/>
       <x:c r="R65" s="36"/>
@@ -10150,13 +10147,13 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B66" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="C66" t="s">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="C66" t="s">
+      <x:c r="D66" s="2" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="D66" s="2" t="s">
-        <x:v>457</x:v>
       </x:c>
       <x:c r="E66">
         <x:v>1</x:v>
@@ -10168,16 +10165,16 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H66" t="s">
-        <x:v>349</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="I66" t="s">
+        <x:v>457</x:v>
+      </x:c>
+      <x:c r="J66" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K66" t="s">
         <x:v>458</x:v>
-      </x:c>
-      <x:c r="J66" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K66" t="s">
-        <x:v>459</x:v>
       </x:c>
       <x:c r="L66" t="s">
         <x:v>8</x:v>
@@ -10186,13 +10183,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="N66" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="O66" t="s">
         <x:v>460</x:v>
       </x:c>
-      <x:c r="O66" t="s">
+      <x:c r="P66" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="P66" t="s">
-        <x:v>462</x:v>
       </x:c>
       <x:c r="Q66" s="36"/>
       <x:c r="R66" s="36"/>
@@ -10222,13 +10219,13 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B67" t="s">
+        <x:v>462</x:v>
+      </x:c>
+      <x:c r="C67" t="s">
         <x:v>463</x:v>
       </x:c>
-      <x:c r="C67" t="s">
+      <x:c r="D67" s="2" t="s">
         <x:v>464</x:v>
-      </x:c>
-      <x:c r="D67" s="2" t="s">
-        <x:v>465</x:v>
       </x:c>
       <x:c r="E67">
         <x:v>1</x:v>
@@ -10240,16 +10237,16 @@
         <x:v>Top 20 — US$12,000 Credits (OpenAI + Gemini Cloud)</x:v>
       </x:c>
       <x:c r="H67" t="s">
-        <x:v>373</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="I67" t="s">
-        <x:v>382</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="J67" t="s">
+        <x:v>465</x:v>
+      </x:c>
+      <x:c r="K67" t="s">
         <x:v>466</x:v>
-      </x:c>
-      <x:c r="K67" t="s">
-        <x:v>467</x:v>
       </x:c>
       <x:c r="L67" t="s">
         <x:v>8</x:v>
@@ -10258,7 +10255,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="N67" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="O67" t="s">
         <x:v>8</x:v>
@@ -10311,13 +10308,13 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B68" t="s">
-        <x:v>468</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="C68" t="s">
         <x:v>240</x:v>
       </x:c>
       <x:c r="D68" s="2" t="s">
-        <x:v>469</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="E68">
         <x:v>3</x:v>
@@ -10329,19 +10326,19 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H68" t="s">
+        <x:v>469</x:v>
+      </x:c>
+      <x:c r="I68" t="s">
         <x:v>470</x:v>
       </x:c>
-      <x:c r="I68" t="s">
+      <x:c r="J68" t="s">
         <x:v>471</x:v>
       </x:c>
-      <x:c r="J68" t="s">
+      <x:c r="K68" t="s">
         <x:v>472</x:v>
       </x:c>
-      <x:c r="K68" t="s">
+      <x:c r="L68" t="s">
         <x:v>473</x:v>
-      </x:c>
-      <x:c r="L68" t="s">
-        <x:v>474</x:v>
       </x:c>
       <x:c r="M68" t="s">
         <x:v>9</x:v>
@@ -10350,7 +10347,7 @@
         <x:v>247</x:v>
       </x:c>
       <x:c r="O68" t="s">
-        <x:v>475</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="P68" t="s">
         <x:v>8</x:v>
@@ -10383,13 +10380,13 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B69" t="s">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="C69" t="s">
+        <x:v>463</x:v>
+      </x:c>
+      <x:c r="D69" s="2" t="s">
         <x:v>476</x:v>
-      </x:c>
-      <x:c r="C69" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="D69" s="2" t="s">
-        <x:v>477</x:v>
       </x:c>
       <x:c r="E69">
         <x:v>1</x:v>
@@ -10401,16 +10398,16 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H69" t="s">
-        <x:v>373</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="I69" t="s">
-        <x:v>382</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="J69" t="s">
-        <x:v>466</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="K69" t="s">
-        <x:v>478</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="L69" t="s">
         <x:v>8</x:v>
@@ -10419,13 +10416,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="N69" t="s">
-        <x:v>479</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="O69" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="P69" t="s">
-        <x:v>480</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="Q69" s="36"/>
       <x:c r="R69" s="36"/>
@@ -10455,13 +10452,13 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="B70" t="s">
+        <x:v>480</x:v>
+      </x:c>
+      <x:c r="C70" t="s">
         <x:v>481</x:v>
       </x:c>
-      <x:c r="C70" t="s">
+      <x:c r="D70" s="2" t="s">
         <x:v>482</x:v>
-      </x:c>
-      <x:c r="D70" s="2" t="s">
-        <x:v>483</x:v>
       </x:c>
       <x:c r="E70">
         <x:v>2</x:v>
@@ -10471,31 +10468,31 @@
       </x:c>
       <x:c r="G70"/>
       <x:c r="H70" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="I70" t="s">
         <x:v>484</x:v>
       </x:c>
-      <x:c r="I70" t="s">
+      <x:c r="J70" t="s">
         <x:v>485</x:v>
       </x:c>
-      <x:c r="J70" t="s">
+      <x:c r="K70" t="s">
         <x:v>486</x:v>
       </x:c>
-      <x:c r="K70" t="s">
+      <x:c r="L70" t="s">
+        <x:v>481</x:v>
+      </x:c>
+      <x:c r="M70" t="s">
         <x:v>487</x:v>
       </x:c>
-      <x:c r="L70" t="s">
-        <x:v>482</x:v>
-      </x:c>
-      <x:c r="M70" t="s">
+      <x:c r="N70" t="s">
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="O70" t="s">
         <x:v>488</x:v>
       </x:c>
-      <x:c r="N70" t="s">
-        <x:v>330</x:v>
-      </x:c>
-      <x:c r="O70" t="s">
+      <x:c r="P70" t="s">
         <x:v>489</x:v>
-      </x:c>
-      <x:c r="P70" t="s">
-        <x:v>490</x:v>
       </x:c>
       <x:c r="Q70" s="36"/>
       <x:c r="R70" s="36"/>
@@ -10525,13 +10522,13 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="B71" t="s">
+        <x:v>490</x:v>
+      </x:c>
+      <x:c r="C71" t="s">
         <x:v>491</x:v>
       </x:c>
-      <x:c r="C71" t="s">
+      <x:c r="D71" s="5" t="s">
         <x:v>492</x:v>
-      </x:c>
-      <x:c r="D71" s="5" t="s">
-        <x:v>493</x:v>
       </x:c>
       <x:c r="E71">
         <x:v>1</x:v>
@@ -10543,31 +10540,31 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H71" t="s">
-        <x:v>484</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="I71" t="s">
+        <x:v>493</x:v>
+      </x:c>
+      <x:c r="J71" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K71" t="s">
         <x:v>494</x:v>
       </x:c>
-      <x:c r="J71" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K71" t="s">
-        <x:v>495</x:v>
-      </x:c>
       <x:c r="L71" t="s">
-        <x:v>492</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="M71" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="N71" t="s">
-        <x:v>460</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="O71" t="s">
+        <x:v>495</x:v>
+      </x:c>
+      <x:c r="P71" t="s">
         <x:v>496</x:v>
-      </x:c>
-      <x:c r="P71" t="s">
-        <x:v>497</x:v>
       </x:c>
       <x:c r="Q71" s="36"/>
       <x:c r="R71" s="36"/>
@@ -10597,10 +10594,10 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B72" t="s">
+        <x:v>497</x:v>
+      </x:c>
+      <x:c r="C72" t="s">
         <x:v>498</x:v>
-      </x:c>
-      <x:c r="C72" t="s">
-        <x:v>499</x:v>
       </x:c>
       <x:c r="D72" s="5">
         <x:v>46363</x:v>
@@ -10618,16 +10615,16 @@
         <x:v>215</x:v>
       </x:c>
       <x:c r="I72" t="s">
+        <x:v>499</x:v>
+      </x:c>
+      <x:c r="J72" t="s">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="J72" t="s">
+      <x:c r="K72" t="s">
         <x:v>501</x:v>
       </x:c>
-      <x:c r="K72" t="s">
-        <x:v>502</x:v>
-      </x:c>
       <x:c r="L72" t="s">
-        <x:v>499</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="M72" t="s">
         <x:v>9</x:v>
@@ -10639,7 +10636,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="P72" t="s">
-        <x:v>503</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="Q72" s="36" t="str">
         <x:v>Top 30</x:v>
@@ -10686,13 +10683,13 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B73" t="s">
+        <x:v>503</x:v>
+      </x:c>
+      <x:c r="C73" t="s">
         <x:v>504</x:v>
       </x:c>
-      <x:c r="C73" t="s">
+      <x:c r="D73" s="2" t="s">
         <x:v>505</x:v>
-      </x:c>
-      <x:c r="D73" s="2" t="s">
-        <x:v>506</x:v>
       </x:c>
       <x:c r="E73">
         <x:v>1</x:v>
@@ -10704,31 +10701,31 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H73" t="s">
-        <x:v>431</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="I73" t="s">
+        <x:v>506</x:v>
+      </x:c>
+      <x:c r="J73" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K73" t="s">
         <x:v>507</x:v>
       </x:c>
-      <x:c r="J73" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K73" t="s">
-        <x:v>508</x:v>
-      </x:c>
       <x:c r="L73" t="s">
-        <x:v>505</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="M73" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="N73" t="s">
+        <x:v>508</x:v>
+      </x:c>
+      <x:c r="O73" t="s">
         <x:v>509</x:v>
       </x:c>
-      <x:c r="O73" t="s">
+      <x:c r="P73" t="s">
         <x:v>510</x:v>
-      </x:c>
-      <x:c r="P73" t="s">
-        <x:v>511</x:v>
       </x:c>
       <x:c r="Q73" s="36"/>
       <x:c r="R73" s="36"/>
@@ -10758,13 +10755,13 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B74" t="s">
+        <x:v>511</x:v>
+      </x:c>
+      <x:c r="C74" t="s">
+        <x:v>481</x:v>
+      </x:c>
+      <x:c r="D74" s="2" t="s">
         <x:v>512</x:v>
-      </x:c>
-      <x:c r="C74" t="s">
-        <x:v>482</x:v>
-      </x:c>
-      <x:c r="D74" s="2" t="s">
-        <x:v>513</x:v>
       </x:c>
       <x:c r="E74">
         <x:v>10</x:v>
@@ -10776,31 +10773,31 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H74" t="s">
+        <x:v>513</x:v>
+      </x:c>
+      <x:c r="I74" t="s">
         <x:v>514</x:v>
       </x:c>
-      <x:c r="I74" t="s">
+      <x:c r="J74" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K74" t="s">
         <x:v>515</x:v>
       </x:c>
-      <x:c r="J74" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K74" t="s">
+      <x:c r="L74" t="s">
+        <x:v>481</x:v>
+      </x:c>
+      <x:c r="M74" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="N74" t="s">
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="O74" t="s">
         <x:v>516</x:v>
       </x:c>
-      <x:c r="L74" t="s">
-        <x:v>482</x:v>
-      </x:c>
-      <x:c r="M74" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="N74" t="s">
-        <x:v>330</x:v>
-      </x:c>
-      <x:c r="O74" t="s">
-        <x:v>517</x:v>
-      </x:c>
       <x:c r="P74" t="s">
-        <x:v>490</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="Q74" s="36"/>
       <x:c r="R74" s="36"/>
@@ -10830,10 +10827,10 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B75" s="12" t="s">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="C75" s="12" t="s">
         <x:v>518</x:v>
-      </x:c>
-      <x:c r="C75" s="12" t="s">
-        <x:v>519</x:v>
       </x:c>
       <x:c r="D75" s="5">
         <x:v>46150</x:v>
@@ -10848,19 +10845,19 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H75" s="12" t="s">
+        <x:v>518</x:v>
+      </x:c>
+      <x:c r="I75" s="14" t="s">
         <x:v>519</x:v>
       </x:c>
-      <x:c r="I75" s="14" t="s">
+      <x:c r="J75" s="12" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K75" s="12" t="s">
         <x:v>520</x:v>
       </x:c>
-      <x:c r="J75" s="12" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K75" s="12" t="s">
-        <x:v>521</x:v>
-      </x:c>
       <x:c r="L75" s="12" t="s">
-        <x:v>519</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="M75" s="12" t="s">
         <x:v>9</x:v>
@@ -10869,7 +10866,7 @@
         <x:v>247</x:v>
       </x:c>
       <x:c r="O75" t="s">
-        <x:v>522</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="P75" s="12" t="s">
         <x:v>8</x:v>
@@ -10902,13 +10899,13 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B76" s="12" t="s">
+        <x:v>522</x:v>
+      </x:c>
+      <x:c r="C76" s="12" t="s">
         <x:v>523</x:v>
       </x:c>
-      <x:c r="C76" s="12" t="s">
+      <x:c r="D76" s="13" t="s">
         <x:v>524</x:v>
-      </x:c>
-      <x:c r="D76" s="13" t="s">
-        <x:v>525</x:v>
       </x:c>
       <x:c r="E76">
         <x:v>1</x:v>
@@ -10920,31 +10917,31 @@
         <x:v>Best Project — Best Vertical Solution: Family Office Track — 2,000 Cybrdeck API Credits Each (US$25 value)</x:v>
       </x:c>
       <x:c r="H76" s="12" t="s">
+        <x:v>525</x:v>
+      </x:c>
+      <x:c r="I76" s="12" t="s">
         <x:v>526</x:v>
       </x:c>
-      <x:c r="I76" s="12" t="s">
+      <x:c r="J76" s="12" t="s">
         <x:v>527</x:v>
       </x:c>
-      <x:c r="J76" s="12" t="s">
+      <x:c r="K76" s="12" t="s">
         <x:v>528</x:v>
       </x:c>
-      <x:c r="K76" s="12" t="s">
-        <x:v>529</x:v>
-      </x:c>
       <x:c r="L76" s="12" t="s">
-        <x:v>524</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="M76" s="12" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="N76" s="12" t="s">
+        <x:v>529</x:v>
+      </x:c>
+      <x:c r="O76" s="1" t="s">
         <x:v>530</x:v>
       </x:c>
-      <x:c r="O76" s="1" t="s">
+      <x:c r="P76" t="s">
         <x:v>531</x:v>
-      </x:c>
-      <x:c r="P76" t="s">
-        <x:v>532</x:v>
       </x:c>
       <x:c r="Q76" s="36" t="str">
         <x:v>Best Project</x:v>
@@ -10993,13 +10990,13 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B77" t="s">
+        <x:v>532</x:v>
+      </x:c>
+      <x:c r="C77" t="s">
         <x:v>533</x:v>
       </x:c>
-      <x:c r="C77" t="s">
+      <x:c r="D77" t="s">
         <x:v>534</x:v>
-      </x:c>
-      <x:c r="D77" t="s">
-        <x:v>535</x:v>
       </x:c>
       <x:c r="E77">
         <x:v>1</x:v>
@@ -11011,31 +11008,31 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H77" t="s">
+        <x:v>535</x:v>
+      </x:c>
+      <x:c r="I77" t="s">
         <x:v>536</x:v>
       </x:c>
-      <x:c r="I77" t="s">
+      <x:c r="J77" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K77" t="s">
         <x:v>537</x:v>
       </x:c>
-      <x:c r="J77" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K77" t="s">
+      <x:c r="L77" t="s">
         <x:v>538</x:v>
-      </x:c>
-      <x:c r="L77" t="s">
-        <x:v>539</x:v>
       </x:c>
       <x:c r="M77" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="N77" t="s">
+        <x:v>539</x:v>
+      </x:c>
+      <x:c r="O77" t="s">
         <x:v>540</x:v>
       </x:c>
-      <x:c r="O77" t="s">
+      <x:c r="P77" t="s">
         <x:v>541</x:v>
-      </x:c>
-      <x:c r="P77" t="s">
-        <x:v>542</x:v>
       </x:c>
       <x:c r="Q77" s="36"/>
       <x:c r="R77" s="36"/>
@@ -11065,13 +11062,13 @@
         <x:v>77</x:v>
       </x:c>
       <x:c r="B78" t="s">
+        <x:v>542</x:v>
+      </x:c>
+      <x:c r="C78" t="s">
+        <x:v>481</x:v>
+      </x:c>
+      <x:c r="D78" t="s">
         <x:v>543</x:v>
-      </x:c>
-      <x:c r="C78" t="s">
-        <x:v>482</x:v>
-      </x:c>
-      <x:c r="D78" t="s">
-        <x:v>544</x:v>
       </x:c>
       <x:c r="E78">
         <x:v>1</x:v>
@@ -11083,31 +11080,31 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="H78" t="s">
+        <x:v>544</x:v>
+      </x:c>
+      <x:c r="I78" t="s">
         <x:v>545</x:v>
       </x:c>
-      <x:c r="I78" t="s">
+      <x:c r="J78" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="K78" t="s">
         <x:v>546</x:v>
       </x:c>
-      <x:c r="J78" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="K78" t="s">
+      <x:c r="L78" t="s">
+        <x:v>481</x:v>
+      </x:c>
+      <x:c r="M78" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="N78" t="s">
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="O78" t="s">
         <x:v>547</x:v>
       </x:c>
-      <x:c r="L78" t="s">
-        <x:v>482</x:v>
-      </x:c>
-      <x:c r="M78" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="N78" t="s">
-        <x:v>330</x:v>
-      </x:c>
-      <x:c r="O78" t="s">
-        <x:v>548</x:v>
-      </x:c>
       <x:c r="P78" t="s">
-        <x:v>490</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="Q78" s="36"/>
       <x:c r="R78" s="36"/>
@@ -11137,37 +11134,37 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="B79" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="C79" t="s">
         <x:v>549</x:v>
       </x:c>
-      <x:c r="C79" t="s">
+      <x:c r="D79" t="s">
         <x:v>550</x:v>
-      </x:c>
-      <x:c r="D79" t="s">
-        <x:v>551</x:v>
       </x:c>
       <x:c r="E79">
         <x:v>4</x:v>
       </x:c>
       <x:c r="F79" t="s">
-        <x:v>437</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="G79" t="str">
         <x:v>-</x:v>
       </x:c>
       <x:c r="H79" t="s">
+        <x:v>551</x:v>
+      </x:c>
+      <x:c r="I79" t="s">
         <x:v>552</x:v>
       </x:c>
-      <x:c r="I79" t="s">
+      <x:c r="J79" t="s">
         <x:v>553</x:v>
       </x:c>
-      <x:c r="J79" t="s">
+      <x:c r="K79" t="s">
         <x:v>554</x:v>
       </x:c>
-      <x:c r="K79" t="s">
+      <x:c r="L79" t="s">
         <x:v>555</x:v>
-      </x:c>
-      <x:c r="L79" t="s">
-        <x:v>556</x:v>
       </x:c>
       <x:c r="M79" t="s">
         <x:v>9</x:v>
@@ -11176,10 +11173,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="O79" t="s">
+        <x:v>556</x:v>
+      </x:c>
+      <x:c r="P79" t="s">
         <x:v>557</x:v>
-      </x:c>
-      <x:c r="P79" t="s">
-        <x:v>558</x:v>
       </x:c>
       <x:c r="Q79" s="36"/>
       <x:c r="R79" s="36"/>
@@ -11541,10 +11538,10 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rae8b2e67944c4b45"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Ra1c9aa60b5c744e5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R8357c51be1ab4fb5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="Rdfe66792bd1a45bb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R8a655a4498524652"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rafa1682aa70d40de"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="R7c15874e500a47e5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="R1d95719619e342dd"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11567,7 +11564,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>559</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -11576,7 +11573,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="19" t="s">
-        <x:v>560</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="B2" s="19"/>
       <x:c r="C2" s="19"/>
@@ -11585,64 +11582,64 @@
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="11" t="s">
+        <x:v>560</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="s">
         <x:v>561</x:v>
       </x:c>
-      <x:c r="B4" s="11" t="s">
+      <x:c r="C4" s="11" t="s">
         <x:v>562</x:v>
       </x:c>
-      <x:c r="C4" s="11" t="s">
+      <x:c r="D4" s="11" t="s">
         <x:v>563</x:v>
       </x:c>
-      <x:c r="D4" s="11" t="s">
+      <x:c r="E4" s="11" t="s">
         <x:v>564</x:v>
-      </x:c>
-      <x:c r="E4" s="11" t="s">
-        <x:v>565</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="8" t="s">
+        <x:v>565</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="s">
         <x:v>566</x:v>
       </x:c>
-      <x:c r="B5" s="7" t="s">
+      <x:c r="C5" s="7" t="s">
         <x:v>567</x:v>
-      </x:c>
-      <x:c r="C5" s="7" t="s">
-        <x:v>568</x:v>
       </x:c>
       <x:c r="D5" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E5" s="10" t="s">
-        <x:v>569</x:v>
+        <x:v>568</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="8" t="s">
+        <x:v>569</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>570</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="s">
+      <x:c r="C6" s="7" t="s">
         <x:v>571</x:v>
-      </x:c>
-      <x:c r="C6" s="7" t="s">
-        <x:v>572</x:v>
       </x:c>
       <x:c r="D6" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="10" t="s">
-        <x:v>573</x:v>
+        <x:v>572</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="8" t="s">
+        <x:v>573</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
         <x:v>574</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="s">
+      <x:c r="C7" s="7" t="s">
         <x:v>575</x:v>
-      </x:c>
-      <x:c r="C7" s="7" t="s">
-        <x:v>576</x:v>
       </x:c>
       <x:c r="D7" s="9">
         <x:v>1</x:v>
@@ -11651,47 +11648,47 @@
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
       <x:c r="A8" s="8" t="s">
+        <x:v>576</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
         <x:v>577</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="s">
+      <x:c r="C8" s="7" t="s">
         <x:v>578</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="s">
-        <x:v>579</x:v>
       </x:c>
       <x:c r="D8" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E8" s="10" t="s">
-        <x:v>580</x:v>
+        <x:v>579</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" s="8" t="s">
+        <x:v>580</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
         <x:v>581</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="s">
-        <x:v>582</x:v>
-      </x:c>
       <x:c r="C9" s="7" t="s">
-        <x:v>572</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="D9" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="10" t="s">
-        <x:v>583</x:v>
+        <x:v>582</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
       <x:c r="A10" s="8" t="s">
+        <x:v>583</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="s">
         <x:v>584</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="s">
+      <x:c r="C10" s="7" t="s">
         <x:v>585</x:v>
-      </x:c>
-      <x:c r="C10" s="7" t="s">
-        <x:v>586</x:v>
       </x:c>
       <x:c r="D10" s="9">
         <x:v>1</x:v>
@@ -11700,47 +11697,47 @@
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
       <x:c r="A11" s="8" t="s">
+        <x:v>586</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="s">
         <x:v>587</x:v>
       </x:c>
-      <x:c r="B11" s="7" t="s">
+      <x:c r="C11" s="7" t="s">
         <x:v>588</x:v>
-      </x:c>
-      <x:c r="C11" s="7" t="s">
-        <x:v>589</x:v>
       </x:c>
       <x:c r="D11" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E11" s="10" t="s">
-        <x:v>590</x:v>
+        <x:v>589</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
       <x:c r="A12" s="8" t="s">
+        <x:v>590</x:v>
+      </x:c>
+      <x:c r="B12" s="7" t="s">
         <x:v>591</x:v>
       </x:c>
-      <x:c r="B12" s="7" t="s">
+      <x:c r="C12" s="7" t="s">
         <x:v>592</x:v>
-      </x:c>
-      <x:c r="C12" s="7" t="s">
-        <x:v>593</x:v>
       </x:c>
       <x:c r="D12" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E12" s="10" t="s">
-        <x:v>594</x:v>
+        <x:v>593</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
       <x:c r="A13" s="8" t="s">
+        <x:v>594</x:v>
+      </x:c>
+      <x:c r="B13" s="7" t="s">
         <x:v>595</x:v>
       </x:c>
-      <x:c r="B13" s="7" t="s">
+      <x:c r="C13" s="7" t="s">
         <x:v>596</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="s">
-        <x:v>597</x:v>
       </x:c>
       <x:c r="D13" s="9">
         <x:v>1</x:v>
@@ -11749,30 +11746,30 @@
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
       <x:c r="A14" s="8" t="s">
+        <x:v>597</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="s">
         <x:v>598</x:v>
       </x:c>
-      <x:c r="B14" s="7" t="s">
-        <x:v>599</x:v>
-      </x:c>
       <x:c r="C14" s="7" t="s">
-        <x:v>597</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="D14" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E14" s="10" t="s">
-        <x:v>600</x:v>
+        <x:v>599</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28" customHeight="1">
       <x:c r="A15" s="8" t="s">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="s">
         <x:v>601</x:v>
       </x:c>
-      <x:c r="B15" s="7" t="s">
+      <x:c r="C15" s="7" t="s">
         <x:v>602</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="s">
-        <x:v>603</x:v>
       </x:c>
       <x:c r="D15" s="9">
         <x:v>1</x:v>
@@ -11781,30 +11778,30 @@
     </x:row>
     <x:row r="16" ht="28" customHeight="1">
       <x:c r="A16" s="8" t="s">
+        <x:v>603</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="s">
         <x:v>604</x:v>
       </x:c>
-      <x:c r="B16" s="7" t="s">
+      <x:c r="C16" s="7" t="s">
         <x:v>605</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="s">
-        <x:v>606</x:v>
       </x:c>
       <x:c r="D16" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E16" s="10" t="s">
-        <x:v>607</x:v>
+        <x:v>606</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
       <x:c r="A17" s="8" t="s">
+        <x:v>607</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="s">
         <x:v>608</x:v>
       </x:c>
-      <x:c r="B17" s="7" t="s">
+      <x:c r="C17" s="7" t="s">
         <x:v>609</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="s">
-        <x:v>610</x:v>
       </x:c>
       <x:c r="D17" s="9">
         <x:v>1</x:v>
@@ -11813,47 +11810,47 @@
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
       <x:c r="A18" s="8" t="s">
+        <x:v>610</x:v>
+      </x:c>
+      <x:c r="B18" s="7" t="s">
         <x:v>611</x:v>
       </x:c>
-      <x:c r="B18" s="7" t="s">
+      <x:c r="C18" s="7" t="s">
         <x:v>612</x:v>
-      </x:c>
-      <x:c r="C18" s="7" t="s">
-        <x:v>613</x:v>
       </x:c>
       <x:c r="D18" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E18" s="10" t="s">
-        <x:v>614</x:v>
+        <x:v>613</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
       <x:c r="A19" s="8" t="s">
+        <x:v>614</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="s">
         <x:v>615</x:v>
       </x:c>
-      <x:c r="B19" s="7" t="s">
+      <x:c r="C19" s="7" t="s">
         <x:v>616</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="s">
-        <x:v>617</x:v>
       </x:c>
       <x:c r="D19" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E19" s="10" t="s">
-        <x:v>618</x:v>
+        <x:v>617</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28" customHeight="1">
       <x:c r="A20" s="8" t="s">
+        <x:v>618</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="s">
         <x:v>619</x:v>
       </x:c>
-      <x:c r="B20" s="7" t="s">
+      <x:c r="C20" s="7" t="s">
         <x:v>620</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>621</x:v>
       </x:c>
       <x:c r="D20" s="9">
         <x:v>1</x:v>
@@ -11862,10 +11859,10 @@
     </x:row>
     <x:row r="21" ht="28" customHeight="1">
       <x:c r="A21" s="8" t="s">
+        <x:v>621</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="s">
         <x:v>622</x:v>
-      </x:c>
-      <x:c r="B21" s="7" t="s">
-        <x:v>623</x:v>
       </x:c>
       <x:c r="C21" s="7" t="str">
         <x:v>#069, #071, #079</x:v>
@@ -11874,18 +11871,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E21" s="10" t="s">
-        <x:v>624</x:v>
+        <x:v>623</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
       <x:c r="A22" s="8" t="s">
+        <x:v>624</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="s">
         <x:v>625</x:v>
       </x:c>
-      <x:c r="B22" s="7" t="s">
+      <x:c r="C22" s="7" t="s">
         <x:v>626</x:v>
-      </x:c>
-      <x:c r="C22" s="7" t="s">
-        <x:v>627</x:v>
       </x:c>
       <x:c r="D22" s="9">
         <x:v>1</x:v>
@@ -11894,13 +11891,13 @@
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
       <x:c r="A23" s="8" t="s">
+        <x:v>627</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="s">
         <x:v>628</x:v>
       </x:c>
-      <x:c r="B23" s="7" t="s">
+      <x:c r="C23" s="7" t="s">
         <x:v>629</x:v>
-      </x:c>
-      <x:c r="C23" s="7" t="s">
-        <x:v>630</x:v>
       </x:c>
       <x:c r="D23" s="9">
         <x:v>1</x:v>
@@ -11909,10 +11906,10 @@
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
       <x:c r="A24" s="8" t="s">
+        <x:v>630</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="s">
         <x:v>631</x:v>
-      </x:c>
-      <x:c r="B24" s="7" t="s">
-        <x:v>632</x:v>
       </x:c>
       <x:c r="C24" s="7" t="str">
         <x:v>#054, #055, #056, #062, #066, #068, #075</x:v>
@@ -11921,12 +11918,12 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E24" s="10" t="s">
-        <x:v>633</x:v>
+        <x:v>632</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
       <x:c r="A25" s="8" t="s">
-        <x:v>634</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
         <x:v>Clement Lork</x:v>
@@ -11938,18 +11935,18 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E25" s="10" t="s">
-        <x:v>635</x:v>
+        <x:v>634</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="28" customHeight="1">
       <x:c r="A26" s="8" t="s">
+        <x:v>635</x:v>
+      </x:c>
+      <x:c r="B26" s="7" t="s">
         <x:v>636</x:v>
       </x:c>
-      <x:c r="B26" s="7" t="s">
-        <x:v>637</x:v>
-      </x:c>
       <x:c r="C26" s="7" t="s">
-        <x:v>576</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="D26" s="9">
         <x:v>1</x:v>
@@ -11958,13 +11955,13 @@
     </x:row>
     <x:row r="27" ht="28" customHeight="1">
       <x:c r="A27" s="8" t="s">
+        <x:v>637</x:v>
+      </x:c>
+      <x:c r="B27" s="7" t="s">
         <x:v>638</x:v>
       </x:c>
-      <x:c r="B27" s="7" t="s">
+      <x:c r="C27" s="7" t="s">
         <x:v>639</x:v>
-      </x:c>
-      <x:c r="C27" s="7" t="s">
-        <x:v>640</x:v>
       </x:c>
       <x:c r="D27" s="9">
         <x:v>1</x:v>
@@ -11973,13 +11970,13 @@
     </x:row>
     <x:row r="28" ht="28" customHeight="1">
       <x:c r="A28" s="8" t="s">
+        <x:v>640</x:v>
+      </x:c>
+      <x:c r="B28" s="7" t="s">
         <x:v>641</x:v>
       </x:c>
-      <x:c r="B28" s="7" t="s">
+      <x:c r="C28" s="7" t="s">
         <x:v>642</x:v>
-      </x:c>
-      <x:c r="C28" s="7" t="s">
-        <x:v>643</x:v>
       </x:c>
       <x:c r="D28" s="9">
         <x:v>2</x:v>
@@ -11988,13 +11985,13 @@
     </x:row>
     <x:row r="29" ht="28" customHeight="1">
       <x:c r="A29" s="8" t="s">
+        <x:v>643</x:v>
+      </x:c>
+      <x:c r="B29" s="7" t="s">
         <x:v>644</x:v>
       </x:c>
-      <x:c r="B29" s="7" t="s">
+      <x:c r="C29" s="7" t="s">
         <x:v>645</x:v>
-      </x:c>
-      <x:c r="C29" s="7" t="s">
-        <x:v>646</x:v>
       </x:c>
       <x:c r="D29" s="9">
         <x:v>4</x:v>
@@ -12003,13 +12000,13 @@
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
       <x:c r="A30" s="8" t="s">
+        <x:v>646</x:v>
+      </x:c>
+      <x:c r="B30" s="7" t="s">
         <x:v>647</x:v>
       </x:c>
-      <x:c r="B30" s="7" t="s">
-        <x:v>648</x:v>
-      </x:c>
       <x:c r="C30" s="7" t="s">
-        <x:v>640</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="D30" s="9">
         <x:v>1</x:v>
@@ -12018,47 +12015,47 @@
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="8" t="s">
+        <x:v>648</x:v>
+      </x:c>
+      <x:c r="B31" s="7" t="s">
         <x:v>649</x:v>
       </x:c>
-      <x:c r="B31" s="7" t="s">
-        <x:v>650</x:v>
-      </x:c>
       <x:c r="C31" s="7" t="s">
-        <x:v>589</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="D31" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E31" s="10" t="s">
-        <x:v>651</x:v>
+        <x:v>650</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="28" customHeight="1">
       <x:c r="A32" s="8" t="s">
+        <x:v>651</x:v>
+      </x:c>
+      <x:c r="B32" s="7" t="s">
         <x:v>652</x:v>
       </x:c>
-      <x:c r="B32" s="7" t="s">
+      <x:c r="C32" s="7" t="s">
         <x:v>653</x:v>
-      </x:c>
-      <x:c r="C32" s="7" t="s">
-        <x:v>654</x:v>
       </x:c>
       <x:c r="D32" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E32" s="10" t="s">
-        <x:v>655</x:v>
+        <x:v>654</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="8" t="s">
+        <x:v>655</x:v>
+      </x:c>
+      <x:c r="B33" s="7" t="s">
         <x:v>656</x:v>
       </x:c>
-      <x:c r="B33" s="7" t="s">
-        <x:v>657</x:v>
-      </x:c>
       <x:c r="C33" s="7" t="s">
-        <x:v>627</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="D33" s="9">
         <x:v>1</x:v>
@@ -12067,13 +12064,13 @@
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
       <x:c r="A34" s="8" t="s">
+        <x:v>657</x:v>
+      </x:c>
+      <x:c r="B34" s="7" t="s">
         <x:v>658</x:v>
       </x:c>
-      <x:c r="B34" s="7" t="s">
+      <x:c r="C34" s="7" t="s">
         <x:v>659</x:v>
-      </x:c>
-      <x:c r="C34" s="7" t="s">
-        <x:v>660</x:v>
       </x:c>
       <x:c r="D34" s="9">
         <x:v>1</x:v>
@@ -12082,47 +12079,47 @@
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
       <x:c r="A35" s="8" t="s">
+        <x:v>660</x:v>
+      </x:c>
+      <x:c r="B35" s="7" t="s">
         <x:v>661</x:v>
       </x:c>
-      <x:c r="B35" s="7" t="s">
+      <x:c r="C35" s="7" t="s">
         <x:v>662</x:v>
-      </x:c>
-      <x:c r="C35" s="7" t="s">
-        <x:v>663</x:v>
       </x:c>
       <x:c r="D35" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E35" s="10" t="s">
-        <x:v>664</x:v>
+        <x:v>663</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
       <x:c r="A36" s="8" t="s">
+        <x:v>664</x:v>
+      </x:c>
+      <x:c r="B36" s="7" t="s">
         <x:v>665</x:v>
       </x:c>
-      <x:c r="B36" s="7" t="s">
+      <x:c r="C36" s="7" t="s">
         <x:v>666</x:v>
-      </x:c>
-      <x:c r="C36" s="7" t="s">
-        <x:v>667</x:v>
       </x:c>
       <x:c r="D36" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E36" s="10" t="s">
-        <x:v>668</x:v>
+        <x:v>667</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
       <x:c r="A37" s="8" t="s">
+        <x:v>668</x:v>
+      </x:c>
+      <x:c r="B37" s="7" t="s">
         <x:v>669</x:v>
       </x:c>
-      <x:c r="B37" s="7" t="s">
+      <x:c r="C37" s="7" t="s">
         <x:v>670</x:v>
-      </x:c>
-      <x:c r="C37" s="7" t="s">
-        <x:v>671</x:v>
       </x:c>
       <x:c r="D37" s="9">
         <x:v>1</x:v>
@@ -12131,13 +12128,13 @@
     </x:row>
     <x:row r="38" ht="28" customHeight="1">
       <x:c r="A38" s="8" t="s">
+        <x:v>671</x:v>
+      </x:c>
+      <x:c r="B38" s="7" t="s">
         <x:v>672</x:v>
       </x:c>
-      <x:c r="B38" s="7" t="s">
-        <x:v>673</x:v>
-      </x:c>
       <x:c r="C38" s="7" t="s">
-        <x:v>610</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="D38" s="9">
         <x:v>1</x:v>
@@ -12146,13 +12143,13 @@
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
       <x:c r="A39" s="8" t="s">
+        <x:v>673</x:v>
+      </x:c>
+      <x:c r="B39" s="7" t="s">
         <x:v>674</x:v>
       </x:c>
-      <x:c r="B39" s="7" t="s">
+      <x:c r="C39" s="7" t="s">
         <x:v>675</x:v>
-      </x:c>
-      <x:c r="C39" s="7" t="s">
-        <x:v>676</x:v>
       </x:c>
       <x:c r="D39" s="9">
         <x:v>3</x:v>
@@ -12161,47 +12158,47 @@
     </x:row>
     <x:row r="40" ht="28" customHeight="1">
       <x:c r="A40" s="8" t="s">
+        <x:v>676</x:v>
+      </x:c>
+      <x:c r="B40" s="7" t="s">
         <x:v>677</x:v>
       </x:c>
-      <x:c r="B40" s="7" t="s">
+      <x:c r="C40" s="7" t="s">
         <x:v>678</x:v>
-      </x:c>
-      <x:c r="C40" s="7" t="s">
-        <x:v>679</x:v>
       </x:c>
       <x:c r="D40" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E40" s="10" t="s">
-        <x:v>680</x:v>
+        <x:v>679</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28" customHeight="1">
       <x:c r="A41" s="8" t="s">
+        <x:v>680</x:v>
+      </x:c>
+      <x:c r="B41" s="7" t="s">
         <x:v>681</x:v>
       </x:c>
-      <x:c r="B41" s="7" t="s">
-        <x:v>682</x:v>
-      </x:c>
       <x:c r="C41" s="7" t="s">
-        <x:v>679</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="D41" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E41" s="10" t="s">
-        <x:v>683</x:v>
+        <x:v>682</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="28" customHeight="1">
       <x:c r="A42" s="8" t="s">
+        <x:v>683</x:v>
+      </x:c>
+      <x:c r="B42" s="7" t="s">
         <x:v>684</x:v>
       </x:c>
-      <x:c r="B42" s="7" t="s">
+      <x:c r="C42" s="7" t="s">
         <x:v>685</x:v>
-      </x:c>
-      <x:c r="C42" s="7" t="s">
-        <x:v>686</x:v>
       </x:c>
       <x:c r="D42" s="9">
         <x:v>1</x:v>
@@ -12210,10 +12207,10 @@
     </x:row>
     <x:row r="43" ht="28" customHeight="1">
       <x:c r="A43" s="8" t="s">
+        <x:v>686</x:v>
+      </x:c>
+      <x:c r="B43" s="7" t="s">
         <x:v>687</x:v>
-      </x:c>
-      <x:c r="B43" s="7" t="s">
-        <x:v>688</x:v>
       </x:c>
       <x:c r="C43" s="7" t="str">
         <x:v>#069, #079</x:v>
@@ -12225,30 +12222,30 @@
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="8" t="s">
+        <x:v>688</x:v>
+      </x:c>
+      <x:c r="B44" s="7" t="s">
         <x:v>689</x:v>
       </x:c>
-      <x:c r="B44" s="7" t="s">
-        <x:v>690</x:v>
-      </x:c>
       <x:c r="C44" s="7" t="s">
-        <x:v>643</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="D44" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E44" s="10" t="s">
-        <x:v>691</x:v>
+        <x:v>690</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
       <x:c r="A45" s="8" t="s">
+        <x:v>691</x:v>
+      </x:c>
+      <x:c r="B45" s="7" t="s">
         <x:v>692</x:v>
       </x:c>
-      <x:c r="B45" s="7" t="s">
+      <x:c r="C45" s="7" t="s">
         <x:v>693</x:v>
-      </x:c>
-      <x:c r="C45" s="7" t="s">
-        <x:v>694</x:v>
       </x:c>
       <x:c r="D45" s="9">
         <x:v>1</x:v>
@@ -12257,13 +12254,13 @@
     </x:row>
     <x:row r="46" ht="28" customHeight="1">
       <x:c r="A46" s="8" t="s">
+        <x:v>694</x:v>
+      </x:c>
+      <x:c r="B46" s="7" t="s">
         <x:v>695</x:v>
       </x:c>
-      <x:c r="B46" s="7" t="s">
-        <x:v>696</x:v>
-      </x:c>
       <x:c r="C46" s="7" t="s">
-        <x:v>660</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="D46" s="9">
         <x:v>1</x:v>
@@ -12272,47 +12269,47 @@
     </x:row>
     <x:row r="47" ht="28" customHeight="1">
       <x:c r="A47" s="8" t="s">
+        <x:v>696</x:v>
+      </x:c>
+      <x:c r="B47" s="7" t="s">
         <x:v>697</x:v>
       </x:c>
-      <x:c r="B47" s="7" t="s">
-        <x:v>698</x:v>
-      </x:c>
       <x:c r="C47" s="7" t="s">
-        <x:v>572</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="D47" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E47" s="10" t="s">
-        <x:v>699</x:v>
+        <x:v>698</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="28" customHeight="1">
       <x:c r="A48" s="8" t="s">
+        <x:v>699</x:v>
+      </x:c>
+      <x:c r="B48" s="7" t="s">
         <x:v>700</x:v>
       </x:c>
-      <x:c r="B48" s="7" t="s">
+      <x:c r="C48" s="7" t="s">
         <x:v>701</x:v>
-      </x:c>
-      <x:c r="C48" s="7" t="s">
-        <x:v>702</x:v>
       </x:c>
       <x:c r="D48" s="9">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E48" s="10" t="s">
-        <x:v>703</x:v>
+        <x:v>702</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="28" customHeight="1">
       <x:c r="A49" s="8" t="s">
+        <x:v>703</x:v>
+      </x:c>
+      <x:c r="B49" s="7" t="s">
         <x:v>704</x:v>
       </x:c>
-      <x:c r="B49" s="7" t="s">
+      <x:c r="C49" s="7" t="s">
         <x:v>705</x:v>
-      </x:c>
-      <x:c r="C49" s="7" t="s">
-        <x:v>706</x:v>
       </x:c>
       <x:c r="D49" s="9">
         <x:v>1</x:v>
@@ -12321,13 +12318,13 @@
     </x:row>
     <x:row r="50" ht="28" customHeight="1">
       <x:c r="A50" s="8" t="s">
+        <x:v>706</x:v>
+      </x:c>
+      <x:c r="B50" s="7" t="s">
         <x:v>707</x:v>
       </x:c>
-      <x:c r="B50" s="7" t="s">
-        <x:v>708</x:v>
-      </x:c>
       <x:c r="C50" s="7" t="s">
-        <x:v>671</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="D50" s="9">
         <x:v>1</x:v>
@@ -12336,64 +12333,64 @@
     </x:row>
     <x:row r="51" ht="28" customHeight="1">
       <x:c r="A51" s="8" t="s">
+        <x:v>708</x:v>
+      </x:c>
+      <x:c r="B51" s="7" t="s">
         <x:v>709</x:v>
       </x:c>
-      <x:c r="B51" s="7" t="s">
+      <x:c r="C51" s="7" t="s">
         <x:v>710</x:v>
-      </x:c>
-      <x:c r="C51" s="7" t="s">
-        <x:v>711</x:v>
       </x:c>
       <x:c r="D51" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E51" s="10" t="s">
-        <x:v>712</x:v>
+        <x:v>711</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="28" customHeight="1">
       <x:c r="A52" s="8" t="s">
+        <x:v>712</x:v>
+      </x:c>
+      <x:c r="B52" s="7" t="s">
         <x:v>713</x:v>
       </x:c>
-      <x:c r="B52" s="7" t="s">
+      <x:c r="C52" s="7" t="s">
         <x:v>714</x:v>
-      </x:c>
-      <x:c r="C52" s="7" t="s">
-        <x:v>715</x:v>
       </x:c>
       <x:c r="D52" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E52" s="10" t="s">
-        <x:v>716</x:v>
+        <x:v>715</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="28" customHeight="1">
       <x:c r="A53" s="8" t="s">
+        <x:v>716</x:v>
+      </x:c>
+      <x:c r="B53" s="7" t="s">
         <x:v>717</x:v>
       </x:c>
-      <x:c r="B53" s="7" t="s">
+      <x:c r="C53" s="7" t="s">
         <x:v>718</x:v>
-      </x:c>
-      <x:c r="C53" s="7" t="s">
-        <x:v>719</x:v>
       </x:c>
       <x:c r="D53" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E53" s="10" t="s">
-        <x:v>720</x:v>
+        <x:v>719</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="28" customHeight="1">
       <x:c r="A54" s="8" t="s">
+        <x:v>720</x:v>
+      </x:c>
+      <x:c r="B54" s="7" t="s">
         <x:v>721</x:v>
       </x:c>
-      <x:c r="B54" s="7" t="s">
+      <x:c r="C54" s="7" t="s">
         <x:v>722</x:v>
-      </x:c>
-      <x:c r="C54" s="7" t="s">
-        <x:v>723</x:v>
       </x:c>
       <x:c r="D54" s="9">
         <x:v>1</x:v>
@@ -12402,81 +12399,81 @@
     </x:row>
     <x:row r="55" ht="28" customHeight="1">
       <x:c r="A55" s="8" t="s">
+        <x:v>723</x:v>
+      </x:c>
+      <x:c r="B55" s="7" t="s">
         <x:v>724</x:v>
       </x:c>
-      <x:c r="B55" s="7" t="s">
+      <x:c r="C55" s="7" t="s">
         <x:v>725</x:v>
-      </x:c>
-      <x:c r="C55" s="7" t="s">
-        <x:v>726</x:v>
       </x:c>
       <x:c r="D55" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E55" s="10" t="s">
-        <x:v>727</x:v>
+        <x:v>726</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="28" customHeight="1">
       <x:c r="A56" s="8" t="s">
+        <x:v>727</x:v>
+      </x:c>
+      <x:c r="B56" s="7" t="s">
         <x:v>728</x:v>
       </x:c>
-      <x:c r="B56" s="7" t="s">
+      <x:c r="C56" s="7" t="s">
         <x:v>729</x:v>
-      </x:c>
-      <x:c r="C56" s="7" t="s">
-        <x:v>730</x:v>
       </x:c>
       <x:c r="D56" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E56" s="10" t="s">
-        <x:v>731</x:v>
+        <x:v>730</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="28" customHeight="1">
       <x:c r="A57" s="8" t="s">
+        <x:v>731</x:v>
+      </x:c>
+      <x:c r="B57" s="7" t="s">
         <x:v>732</x:v>
       </x:c>
-      <x:c r="B57" s="7" t="s">
+      <x:c r="C57" s="7" t="s">
         <x:v>733</x:v>
-      </x:c>
-      <x:c r="C57" s="7" t="s">
-        <x:v>734</x:v>
       </x:c>
       <x:c r="D57" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E57" s="10" t="s">
-        <x:v>735</x:v>
+        <x:v>734</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
       <x:c r="A58" s="8" t="s">
+        <x:v>735</x:v>
+      </x:c>
+      <x:c r="B58" s="7" t="s">
         <x:v>736</x:v>
       </x:c>
-      <x:c r="B58" s="7" t="s">
+      <x:c r="C58" s="7" t="s">
         <x:v>737</x:v>
-      </x:c>
-      <x:c r="C58" s="7" t="s">
-        <x:v>738</x:v>
       </x:c>
       <x:c r="D58" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E58" s="10" t="s">
-        <x:v>739</x:v>
+        <x:v>738</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="28" customHeight="1">
       <x:c r="A59" s="8" t="s">
+        <x:v>739</x:v>
+      </x:c>
+      <x:c r="B59" s="7" t="s">
         <x:v>740</x:v>
       </x:c>
-      <x:c r="B59" s="7" t="s">
-        <x:v>741</x:v>
-      </x:c>
       <x:c r="C59" s="7" t="s">
-        <x:v>576</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="D59" s="9">
         <x:v>1</x:v>
@@ -12485,13 +12482,13 @@
     </x:row>
     <x:row r="60" ht="28" customHeight="1">
       <x:c r="A60" s="8" t="s">
+        <x:v>741</x:v>
+      </x:c>
+      <x:c r="B60" s="7" t="s">
         <x:v>742</x:v>
       </x:c>
-      <x:c r="B60" s="7" t="s">
-        <x:v>743</x:v>
-      </x:c>
       <x:c r="C60" s="7" t="s">
-        <x:v>613</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="D60" s="9">
         <x:v>1</x:v>
@@ -12500,13 +12497,13 @@
     </x:row>
     <x:row r="61" ht="28" customHeight="1">
       <x:c r="A61" s="8" t="s">
+        <x:v>743</x:v>
+      </x:c>
+      <x:c r="B61" s="7" t="s">
         <x:v>744</x:v>
       </x:c>
-      <x:c r="B61" s="7" t="s">
-        <x:v>745</x:v>
-      </x:c>
       <x:c r="C61" s="7" t="s">
-        <x:v>597</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="D61" s="9">
         <x:v>1</x:v>
@@ -12515,30 +12512,30 @@
     </x:row>
     <x:row r="62" ht="28" customHeight="1">
       <x:c r="A62" s="8" t="s">
+        <x:v>745</x:v>
+      </x:c>
+      <x:c r="B62" s="7" t="s">
         <x:v>746</x:v>
       </x:c>
-      <x:c r="B62" s="7" t="s">
-        <x:v>747</x:v>
-      </x:c>
       <x:c r="C62" s="7" t="s">
-        <x:v>603</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="D62" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E62" s="10" t="s">
-        <x:v>748</x:v>
+        <x:v>747</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="28" customHeight="1">
       <x:c r="A63" s="8" t="s">
+        <x:v>748</x:v>
+      </x:c>
+      <x:c r="B63" s="7" t="s">
         <x:v>749</x:v>
       </x:c>
-      <x:c r="B63" s="7" t="s">
-        <x:v>750</x:v>
-      </x:c>
       <x:c r="C63" s="7" t="s">
-        <x:v>597</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="D63" s="9">
         <x:v>1</x:v>
@@ -12547,13 +12544,13 @@
     </x:row>
     <x:row r="64" ht="28" customHeight="1">
       <x:c r="A64" s="8" t="s">
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="B64" s="7" t="s">
         <x:v>751</x:v>
       </x:c>
-      <x:c r="B64" s="7" t="s">
+      <x:c r="C64" s="7" t="s">
         <x:v>752</x:v>
-      </x:c>
-      <x:c r="C64" s="7" t="s">
-        <x:v>753</x:v>
       </x:c>
       <x:c r="D64" s="9">
         <x:v>1</x:v>
@@ -12562,13 +12559,13 @@
     </x:row>
     <x:row r="65" ht="28" customHeight="1">
       <x:c r="A65" s="8" t="s">
+        <x:v>753</x:v>
+      </x:c>
+      <x:c r="B65" s="7" t="s">
         <x:v>754</x:v>
       </x:c>
-      <x:c r="B65" s="7" t="s">
+      <x:c r="C65" s="7" t="s">
         <x:v>755</x:v>
-      </x:c>
-      <x:c r="C65" s="7" t="s">
-        <x:v>756</x:v>
       </x:c>
       <x:c r="D65" s="9">
         <x:v>1</x:v>
@@ -12577,13 +12574,13 @@
     </x:row>
     <x:row r="66" ht="28" customHeight="1">
       <x:c r="A66" s="8" t="s">
+        <x:v>756</x:v>
+      </x:c>
+      <x:c r="B66" s="7" t="s">
         <x:v>757</x:v>
       </x:c>
-      <x:c r="B66" s="7" t="s">
-        <x:v>758</x:v>
-      </x:c>
       <x:c r="C66" s="7" t="s">
-        <x:v>586</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="D66" s="9">
         <x:v>1</x:v>
@@ -12592,47 +12589,47 @@
     </x:row>
     <x:row r="67" ht="28" customHeight="1">
       <x:c r="A67" s="8" t="s">
+        <x:v>758</x:v>
+      </x:c>
+      <x:c r="B67" s="7" t="s">
         <x:v>759</x:v>
       </x:c>
-      <x:c r="B67" s="7" t="s">
-        <x:v>760</x:v>
-      </x:c>
       <x:c r="C67" s="7" t="s">
-        <x:v>738</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="D67" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E67" s="10" t="s">
-        <x:v>761</x:v>
+        <x:v>760</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="28" customHeight="1">
       <x:c r="A68" s="8" t="s">
+        <x:v>761</x:v>
+      </x:c>
+      <x:c r="B68" s="7" t="s">
         <x:v>762</x:v>
       </x:c>
-      <x:c r="B68" s="7" t="s">
-        <x:v>763</x:v>
-      </x:c>
       <x:c r="C68" s="7" t="s">
-        <x:v>613</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="D68" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E68" s="10" t="s">
-        <x:v>764</x:v>
+        <x:v>763</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="28" customHeight="1">
       <x:c r="A69" s="8" t="s">
+        <x:v>764</x:v>
+      </x:c>
+      <x:c r="B69" s="7" t="s">
         <x:v>765</x:v>
       </x:c>
-      <x:c r="B69" s="7" t="s">
-        <x:v>766</x:v>
-      </x:c>
       <x:c r="C69" s="7" t="s">
-        <x:v>593</x:v>
+        <x:v>592</x:v>
       </x:c>
       <x:c r="D69" s="9">
         <x:v>1</x:v>
@@ -12641,13 +12638,13 @@
     </x:row>
     <x:row r="70" ht="28" customHeight="1">
       <x:c r="A70" s="8" t="s">
+        <x:v>766</x:v>
+      </x:c>
+      <x:c r="B70" s="7" t="s">
         <x:v>767</x:v>
       </x:c>
-      <x:c r="B70" s="7" t="s">
-        <x:v>768</x:v>
-      </x:c>
       <x:c r="C70" s="7" t="s">
-        <x:v>621</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="D70" s="9">
         <x:v>1</x:v>
@@ -12656,13 +12653,13 @@
     </x:row>
     <x:row r="71" ht="28" customHeight="1">
       <x:c r="A71" s="8" t="s">
+        <x:v>768</x:v>
+      </x:c>
+      <x:c r="B71" s="7" t="s">
         <x:v>769</x:v>
       </x:c>
-      <x:c r="B71" s="7" t="s">
+      <x:c r="C71" s="7" t="s">
         <x:v>770</x:v>
-      </x:c>
-      <x:c r="C71" s="7" t="s">
-        <x:v>771</x:v>
       </x:c>
       <x:c r="D71" s="9">
         <x:v>1</x:v>
@@ -12671,64 +12668,64 @@
     </x:row>
     <x:row r="72" ht="28" customHeight="1">
       <x:c r="A72" s="8" t="s">
+        <x:v>771</x:v>
+      </x:c>
+      <x:c r="B72" s="7" t="s">
         <x:v>772</x:v>
       </x:c>
-      <x:c r="B72" s="7" t="s">
+      <x:c r="C72" s="7" t="s">
         <x:v>773</x:v>
-      </x:c>
-      <x:c r="C72" s="7" t="s">
-        <x:v>774</x:v>
       </x:c>
       <x:c r="D72" s="9">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E72" s="10" t="s">
-        <x:v>775</x:v>
+        <x:v>774</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="28" customHeight="1">
       <x:c r="A73" s="8" t="s">
+        <x:v>775</x:v>
+      </x:c>
+      <x:c r="B73" s="7" t="s">
         <x:v>776</x:v>
       </x:c>
-      <x:c r="B73" s="7" t="s">
+      <x:c r="C73" s="7" t="s">
         <x:v>777</x:v>
-      </x:c>
-      <x:c r="C73" s="7" t="s">
-        <x:v>778</x:v>
       </x:c>
       <x:c r="D73" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E73" s="10" t="s">
-        <x:v>779</x:v>
+        <x:v>778</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="28" customHeight="1">
       <x:c r="A74" s="8" t="s">
+        <x:v>779</x:v>
+      </x:c>
+      <x:c r="B74" s="7" t="s">
         <x:v>780</x:v>
       </x:c>
-      <x:c r="B74" s="7" t="s">
-        <x:v>781</x:v>
-      </x:c>
       <x:c r="C74" s="7" t="s">
-        <x:v>579</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="D74" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E74" s="10" t="s">
-        <x:v>782</x:v>
+        <x:v>781</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="28" customHeight="1">
       <x:c r="A75" s="8" t="s">
+        <x:v>782</x:v>
+      </x:c>
+      <x:c r="B75" s="7" t="s">
         <x:v>783</x:v>
       </x:c>
-      <x:c r="B75" s="7" t="s">
-        <x:v>784</x:v>
-      </x:c>
       <x:c r="C75" s="7" t="s">
-        <x:v>694</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="D75" s="9">
         <x:v>1</x:v>
@@ -12737,64 +12734,64 @@
     </x:row>
     <x:row r="76" ht="28" customHeight="1">
       <x:c r="A76" s="8" t="s">
+        <x:v>784</x:v>
+      </x:c>
+      <x:c r="B76" s="7" t="s">
         <x:v>785</x:v>
       </x:c>
-      <x:c r="B76" s="7" t="s">
-        <x:v>786</x:v>
-      </x:c>
       <x:c r="C76" s="7" t="s">
-        <x:v>663</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="D76" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E76" s="10" t="s">
-        <x:v>787</x:v>
+        <x:v>786</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
       <x:c r="A77" s="8" t="s">
+        <x:v>787</x:v>
+      </x:c>
+      <x:c r="B77" s="7" t="s">
         <x:v>788</x:v>
       </x:c>
-      <x:c r="B77" s="7" t="s">
-        <x:v>789</x:v>
-      </x:c>
       <x:c r="C77" s="7" t="s">
-        <x:v>771</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="D77" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E77" s="10" t="s">
-        <x:v>790</x:v>
+        <x:v>789</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
       <x:c r="A78" s="8" t="s">
+        <x:v>790</x:v>
+      </x:c>
+      <x:c r="B78" s="7" t="s">
         <x:v>791</x:v>
       </x:c>
-      <x:c r="B78" s="7" t="s">
-        <x:v>792</x:v>
-      </x:c>
       <x:c r="C78" s="7" t="s">
-        <x:v>568</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="D78" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E78" s="10" t="s">
-        <x:v>793</x:v>
+        <x:v>792</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="28" customHeight="1">
       <x:c r="A79" s="8" t="s">
+        <x:v>793</x:v>
+      </x:c>
+      <x:c r="B79" s="7" t="s">
         <x:v>794</x:v>
       </x:c>
-      <x:c r="B79" s="7" t="s">
-        <x:v>795</x:v>
-      </x:c>
       <x:c r="C79" s="7" t="s">
-        <x:v>663</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="D79" s="9">
         <x:v>1</x:v>
@@ -12803,24 +12800,24 @@
     </x:row>
     <x:row r="80" ht="28" customHeight="1">
       <x:c r="A80" s="8" t="s">
+        <x:v>795</x:v>
+      </x:c>
+      <x:c r="B80" s="7" t="s">
         <x:v>796</x:v>
       </x:c>
-      <x:c r="B80" s="7" t="s">
+      <x:c r="C80" s="7" t="s">
         <x:v>797</x:v>
-      </x:c>
-      <x:c r="C80" s="7" t="s">
-        <x:v>798</x:v>
       </x:c>
       <x:c r="D80" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E80" s="10" t="s">
-        <x:v>799</x:v>
+        <x:v>798</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="28" customHeight="1">
       <x:c r="A81" s="8" t="s">
-        <x:v>800</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="B81" s="7" t="s">
         <x:v>149</x:v>
@@ -12832,35 +12829,35 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E81" s="10" t="s">
-        <x:v>801</x:v>
+        <x:v>800</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="28" customHeight="1">
       <x:c r="A82" s="8" t="s">
+        <x:v>801</x:v>
+      </x:c>
+      <x:c r="B82" s="7" t="s">
         <x:v>802</x:v>
       </x:c>
-      <x:c r="B82" s="7" t="s">
+      <x:c r="C82" s="7" t="s">
         <x:v>803</x:v>
-      </x:c>
-      <x:c r="C82" s="7" t="s">
-        <x:v>804</x:v>
       </x:c>
       <x:c r="D82" s="9">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E82" s="10" t="s">
-        <x:v>805</x:v>
+        <x:v>804</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="28" customHeight="1">
       <x:c r="A83" s="8" t="s">
+        <x:v>805</x:v>
+      </x:c>
+      <x:c r="B83" s="7" t="s">
         <x:v>806</x:v>
       </x:c>
-      <x:c r="B83" s="7" t="s">
-        <x:v>807</x:v>
-      </x:c>
       <x:c r="C83" s="7" t="s">
-        <x:v>586</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="D83" s="9">
         <x:v>1</x:v>
@@ -12869,13 +12866,13 @@
     </x:row>
     <x:row r="84" ht="28" customHeight="1">
       <x:c r="A84" s="8" t="s">
+        <x:v>807</x:v>
+      </x:c>
+      <x:c r="B84" s="7" t="s">
         <x:v>808</x:v>
       </x:c>
-      <x:c r="B84" s="7" t="s">
+      <x:c r="C84" s="7" t="s">
         <x:v>809</x:v>
-      </x:c>
-      <x:c r="C84" s="7" t="s">
-        <x:v>810</x:v>
       </x:c>
       <x:c r="D84" s="9">
         <x:v>1</x:v>
@@ -12884,64 +12881,64 @@
     </x:row>
     <x:row r="85" ht="28" customHeight="1">
       <x:c r="A85" s="8" t="s">
+        <x:v>810</x:v>
+      </x:c>
+      <x:c r="B85" s="7" t="s">
         <x:v>811</x:v>
       </x:c>
-      <x:c r="B85" s="7" t="s">
-        <x:v>812</x:v>
-      </x:c>
       <x:c r="C85" s="7" t="s">
-        <x:v>589</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="D85" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E85" s="10" t="s">
-        <x:v>813</x:v>
+        <x:v>812</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="28" customHeight="1">
       <x:c r="A86" s="8" t="s">
+        <x:v>813</x:v>
+      </x:c>
+      <x:c r="B86" s="7" t="s">
         <x:v>814</x:v>
       </x:c>
-      <x:c r="B86" s="7" t="s">
+      <x:c r="C86" s="7" t="s">
         <x:v>815</x:v>
-      </x:c>
-      <x:c r="C86" s="7" t="s">
-        <x:v>816</x:v>
       </x:c>
       <x:c r="D86" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E86" s="10" t="s">
-        <x:v>817</x:v>
+        <x:v>816</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="28" customHeight="1">
       <x:c r="A87" s="8" t="s">
+        <x:v>817</x:v>
+      </x:c>
+      <x:c r="B87" s="7" t="s">
         <x:v>818</x:v>
       </x:c>
-      <x:c r="B87" s="7" t="s">
+      <x:c r="C87" s="7" t="s">
         <x:v>819</x:v>
-      </x:c>
-      <x:c r="C87" s="7" t="s">
-        <x:v>820</x:v>
       </x:c>
       <x:c r="D87" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E87" s="10" t="s">
-        <x:v>821</x:v>
+        <x:v>820</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="28" customHeight="1">
       <x:c r="A88" s="8" t="s">
+        <x:v>821</x:v>
+      </x:c>
+      <x:c r="B88" s="7" t="s">
         <x:v>822</x:v>
       </x:c>
-      <x:c r="B88" s="7" t="s">
-        <x:v>823</x:v>
-      </x:c>
       <x:c r="C88" s="7" t="s">
-        <x:v>694</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="D88" s="9">
         <x:v>1</x:v>
@@ -12950,13 +12947,13 @@
     </x:row>
     <x:row r="89" ht="28" customHeight="1">
       <x:c r="A89" s="8" t="s">
+        <x:v>823</x:v>
+      </x:c>
+      <x:c r="B89" s="7" t="s">
         <x:v>824</x:v>
       </x:c>
-      <x:c r="B89" s="7" t="s">
-        <x:v>825</x:v>
-      </x:c>
       <x:c r="C89" s="7" t="s">
-        <x:v>610</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="D89" s="9">
         <x:v>1</x:v>
@@ -12965,30 +12962,30 @@
     </x:row>
     <x:row r="90" ht="28" customHeight="1">
       <x:c r="A90" s="8" t="s">
+        <x:v>825</x:v>
+      </x:c>
+      <x:c r="B90" s="7" t="s">
         <x:v>826</x:v>
       </x:c>
-      <x:c r="B90" s="7" t="s">
-        <x:v>827</x:v>
-      </x:c>
       <x:c r="C90" s="7" t="s">
-        <x:v>738</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="D90" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E90" s="10" t="s">
-        <x:v>828</x:v>
+        <x:v>827</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="28" customHeight="1">
       <x:c r="A91" s="8" t="s">
+        <x:v>828</x:v>
+      </x:c>
+      <x:c r="B91" s="7" t="s">
         <x:v>829</x:v>
       </x:c>
-      <x:c r="B91" s="7" t="s">
+      <x:c r="C91" s="7" t="s">
         <x:v>830</x:v>
-      </x:c>
-      <x:c r="C91" s="7" t="s">
-        <x:v>831</x:v>
       </x:c>
       <x:c r="D91" s="9">
         <x:v>1</x:v>
@@ -12997,30 +12994,30 @@
     </x:row>
     <x:row r="92" ht="28" customHeight="1">
       <x:c r="A92" s="8" t="s">
+        <x:v>831</x:v>
+      </x:c>
+      <x:c r="B92" s="7" t="s">
         <x:v>832</x:v>
       </x:c>
-      <x:c r="B92" s="7" t="s">
+      <x:c r="C92" s="7" t="s">
         <x:v>833</x:v>
-      </x:c>
-      <x:c r="C92" s="7" t="s">
-        <x:v>834</x:v>
       </x:c>
       <x:c r="D92" s="9">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E92" s="10" t="s">
-        <x:v>835</x:v>
+        <x:v>834</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="28" customHeight="1">
       <x:c r="A93" s="8" t="s">
+        <x:v>835</x:v>
+      </x:c>
+      <x:c r="B93" s="7" t="s">
         <x:v>836</x:v>
       </x:c>
-      <x:c r="B93" s="7" t="s">
-        <x:v>837</x:v>
-      </x:c>
       <x:c r="C93" s="7" t="s">
-        <x:v>771</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="D93" s="9">
         <x:v>1</x:v>
@@ -13029,30 +13026,30 @@
     </x:row>
     <x:row r="94" ht="28" customHeight="1">
       <x:c r="A94" s="8" t="s">
+        <x:v>837</x:v>
+      </x:c>
+      <x:c r="B94" s="7" t="s">
         <x:v>838</x:v>
       </x:c>
-      <x:c r="B94" s="7" t="s">
-        <x:v>839</x:v>
-      </x:c>
       <x:c r="C94" s="7" t="s">
-        <x:v>663</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="D94" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E94" s="10" t="s">
-        <x:v>840</x:v>
+        <x:v>839</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="28" customHeight="1">
       <x:c r="A95" s="8" t="s">
+        <x:v>840</x:v>
+      </x:c>
+      <x:c r="B95" s="7" t="s">
         <x:v>841</x:v>
       </x:c>
-      <x:c r="B95" s="7" t="s">
-        <x:v>842</x:v>
-      </x:c>
       <x:c r="C95" s="7" t="s">
-        <x:v>660</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="D95" s="9">
         <x:v>1</x:v>
@@ -13061,47 +13058,47 @@
     </x:row>
     <x:row r="96" ht="28" customHeight="1">
       <x:c r="A96" s="8" t="s">
+        <x:v>842</x:v>
+      </x:c>
+      <x:c r="B96" s="7" t="s">
         <x:v>843</x:v>
       </x:c>
-      <x:c r="B96" s="7" t="s">
+      <x:c r="C96" s="7" t="s">
         <x:v>844</x:v>
-      </x:c>
-      <x:c r="C96" s="7" t="s">
-        <x:v>845</x:v>
       </x:c>
       <x:c r="D96" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E96" s="10" t="s">
-        <x:v>846</x:v>
+        <x:v>845</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="28" customHeight="1">
       <x:c r="A97" s="8" t="s">
+        <x:v>846</x:v>
+      </x:c>
+      <x:c r="B97" s="7" t="s">
         <x:v>847</x:v>
       </x:c>
-      <x:c r="B97" s="7" t="s">
-        <x:v>848</x:v>
-      </x:c>
       <x:c r="C97" s="7" t="s">
-        <x:v>810</x:v>
+        <x:v>809</x:v>
       </x:c>
       <x:c r="D97" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E97" s="10" t="s">
-        <x:v>849</x:v>
+        <x:v>848</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="s">
+        <x:v>849</x:v>
+      </x:c>
+      <x:c r="B98" t="s">
         <x:v>850</x:v>
       </x:c>
-      <x:c r="B98" t="s">
+      <x:c r="C98" t="s">
         <x:v>851</x:v>
-      </x:c>
-      <x:c r="C98" t="s">
-        <x:v>852</x:v>
       </x:c>
       <x:c r="D98">
         <x:v>1</x:v>
@@ -13159,12 +13156,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rd0175f6f22c64cb5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R35e005e11b034f1f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rbfb833ef596343da"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R717c473891914bca"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R528d3d039cf94be0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea3758034d724ae6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13179,7 +13176,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="18" t="s">
-        <x:v>853</x:v>
+        <x:v>852</x:v>
       </x:c>
       <x:c r="B1" s="18"/>
       <x:c r="C1" s="18"/>
@@ -14146,7 +14143,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdf6a527acac44fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd953f1fd33354830"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14162,35 +14159,35 @@
   <x:sheetData>
     <x:row r="1" ht="34.75" customHeight="1">
       <x:c r="A1" s="20" t="s">
-        <x:v>854</x:v>
+        <x:v>853</x:v>
       </x:c>
       <x:c r="B1" s="20"/>
       <x:c r="C1" s="20"/>
     </x:row>
     <x:row r="2" ht="45.25" customHeight="1">
       <x:c r="A2" s="21" t="s">
-        <x:v>855</x:v>
+        <x:v>854</x:v>
       </x:c>
       <x:c r="B2" s="21"/>
       <x:c r="C2" s="21"/>
     </x:row>
     <x:row r="4" ht="29.25" customHeight="1">
       <x:c r="A4" s="15" t="s">
+        <x:v>855</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="s">
         <x:v>856</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="s">
+      <x:c r="C4" s="15" t="s">
         <x:v>857</x:v>
-      </x:c>
-      <x:c r="C4" s="15" t="s">
-        <x:v>858</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.75" customHeight="1">
       <x:c r="A5" s="16" t="s">
-        <x:v>282</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="B5" s="16" t="s">
-        <x:v>859</x:v>
+        <x:v>858</x:v>
       </x:c>
       <x:c r="C5" s="17"/>
     </x:row>
@@ -14199,63 +14196,63 @@
         <x:v>147</x:v>
       </x:c>
       <x:c r="B6" s="16" t="s">
-        <x:v>860</x:v>
+        <x:v>859</x:v>
       </x:c>
       <x:c r="C6" s="17"/>
     </x:row>
     <x:row r="7" ht="26.75" customHeight="1">
       <x:c r="A7" s="16" t="s">
-        <x:v>349</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="B7" s="16" t="s">
-        <x:v>861</x:v>
+        <x:v>860</x:v>
       </x:c>
       <x:c r="C7" s="17"/>
     </x:row>
     <x:row r="8" ht="26.75" customHeight="1">
       <x:c r="A8" s="16" t="s">
-        <x:v>422</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="B8" s="16" t="s">
-        <x:v>861</x:v>
+        <x:v>860</x:v>
       </x:c>
       <x:c r="C8" s="17"/>
     </x:row>
     <x:row r="9" ht="26.75" customHeight="1">
       <x:c r="A9" s="16" t="s">
-        <x:v>318</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="B9" s="16" t="s">
-        <x:v>862</x:v>
+        <x:v>861</x:v>
       </x:c>
       <x:c r="C9" s="17"/>
     </x:row>
     <x:row r="10" ht="26.75" customHeight="1">
       <x:c r="A10" s="16" t="s">
-        <x:v>339</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="B10" s="16" t="s">
+        <x:v>862</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="s">
         <x:v>863</x:v>
-      </x:c>
-      <x:c r="C10" s="17" t="s">
-        <x:v>864</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.75" customHeight="1">
       <x:c r="A11" s="16" t="s">
-        <x:v>865</x:v>
+        <x:v>864</x:v>
       </x:c>
       <x:c r="B11" s="16" t="s">
-        <x:v>861</x:v>
+        <x:v>860</x:v>
       </x:c>
       <x:c r="C11" s="17"/>
     </x:row>
     <x:row r="12" ht="26.75" customHeight="1">
       <x:c r="A12" s="16" t="s">
+        <x:v>865</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="s">
         <x:v>866</x:v>
-      </x:c>
-      <x:c r="B12" s="16" t="s">
-        <x:v>867</x:v>
       </x:c>
       <x:c r="C12" s="17"/>
     </x:row>
@@ -14264,25 +14261,25 @@
         <x:v>275</x:v>
       </x:c>
       <x:c r="B13" s="16" t="s">
-        <x:v>860</x:v>
+        <x:v>859</x:v>
       </x:c>
       <x:c r="C13" s="17"/>
     </x:row>
     <x:row r="14" ht="26.75" customHeight="1">
       <x:c r="A14" s="16" t="s">
+        <x:v>867</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="s">
         <x:v>868</x:v>
-      </x:c>
-      <x:c r="B14" s="16" t="s">
-        <x:v>869</x:v>
       </x:c>
       <x:c r="C14" s="17"/>
     </x:row>
     <x:row r="15" ht="26.75" customHeight="1">
       <x:c r="A15" s="16" t="s">
+        <x:v>869</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="s">
         <x:v>870</x:v>
-      </x:c>
-      <x:c r="B15" s="16" t="s">
-        <x:v>871</x:v>
       </x:c>
       <x:c r="C15" s="17"/>
     </x:row>
@@ -14291,7 +14288,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B16" s="16" t="s">
-        <x:v>872</x:v>
+        <x:v>871</x:v>
       </x:c>
       <x:c r="C16" s="17"/>
     </x:row>
@@ -14300,16 +14297,16 @@
         <x:v>174</x:v>
       </x:c>
       <x:c r="B17" s="16" t="s">
-        <x:v>872</x:v>
+        <x:v>871</x:v>
       </x:c>
       <x:c r="C17" s="17"/>
     </x:row>
     <x:row r="18" ht="26.75" customHeight="1">
       <x:c r="A18" s="16" t="s">
-        <x:v>373</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="B18" s="16" t="s">
-        <x:v>867</x:v>
+        <x:v>866</x:v>
       </x:c>
       <x:c r="C18" s="17"/>
     </x:row>
@@ -14318,25 +14315,25 @@
         <x:v>234</x:v>
       </x:c>
       <x:c r="B19" s="16" t="s">
-        <x:v>859</x:v>
+        <x:v>858</x:v>
       </x:c>
       <x:c r="C19" s="17"/>
     </x:row>
     <x:row r="20" ht="26.75" customHeight="1">
       <x:c r="A20" s="16" t="s">
-        <x:v>526</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="B20" s="16" t="s">
-        <x:v>871</x:v>
+        <x:v>870</x:v>
       </x:c>
       <x:c r="C20" s="17"/>
     </x:row>
     <x:row r="21" ht="26.75" customHeight="1">
       <x:c r="A21" s="16" t="s">
-        <x:v>873</x:v>
+        <x:v>872</x:v>
       </x:c>
       <x:c r="B21" s="16" t="s">
-        <x:v>871</x:v>
+        <x:v>870</x:v>
       </x:c>
       <x:c r="C21" s="17"/>
     </x:row>
@@ -14345,63 +14342,63 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B22" s="16" t="s">
-        <x:v>871</x:v>
+        <x:v>870</x:v>
       </x:c>
       <x:c r="C22" s="17"/>
     </x:row>
     <x:row r="23" ht="26.75" customHeight="1">
       <x:c r="A23" s="16" t="s">
+        <x:v>873</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="s">
         <x:v>874</x:v>
-      </x:c>
-      <x:c r="B23" s="16" t="s">
-        <x:v>875</x:v>
       </x:c>
       <x:c r="C23" s="17"/>
     </x:row>
     <x:row r="24" ht="26.75" customHeight="1">
       <x:c r="A24" s="16" t="s">
-        <x:v>876</x:v>
+        <x:v>875</x:v>
       </x:c>
       <x:c r="B24" s="16" t="s">
-        <x:v>859</x:v>
+        <x:v>858</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
     </x:row>
     <x:row r="25" ht="26.75" customHeight="1">
       <x:c r="A25" s="16" t="s">
-        <x:v>296</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B25" s="16" t="s">
-        <x:v>860</x:v>
+        <x:v>859</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
     </x:row>
     <x:row r="26" ht="26.75" customHeight="1">
       <x:c r="A26" s="16" t="s">
-        <x:v>431</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="B26" s="16" t="s">
-        <x:v>860</x:v>
+        <x:v>859</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
     </x:row>
     <x:row r="27" ht="26.75" customHeight="1">
       <x:c r="A27" s="16" t="s">
-        <x:v>519</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="B27" s="16" t="s">
-        <x:v>863</x:v>
+        <x:v>862</x:v>
       </x:c>
       <x:c r="C27" s="17" t="s">
-        <x:v>877</x:v>
+        <x:v>876</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="26.75" customHeight="1">
       <x:c r="A28" s="16" t="s">
-        <x:v>878</x:v>
+        <x:v>877</x:v>
       </x:c>
       <x:c r="B28" s="16" t="s">
-        <x:v>875</x:v>
+        <x:v>874</x:v>
       </x:c>
       <x:c r="C28" s="17"/>
     </x:row>
@@ -14410,7 +14407,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="B29" s="16" t="s">
-        <x:v>875</x:v>
+        <x:v>874</x:v>
       </x:c>
       <x:c r="C29" s="17"/>
     </x:row>
@@ -14419,7 +14416,7 @@
         <x:v>167</x:v>
       </x:c>
       <x:c r="B30" s="16" t="s">
-        <x:v>875</x:v>
+        <x:v>874</x:v>
       </x:c>
       <x:c r="C30" s="17"/>
     </x:row>
@@ -14428,43 +14425,43 @@
         <x:v>118</x:v>
       </x:c>
       <x:c r="B31" s="16" t="s">
-        <x:v>872</x:v>
+        <x:v>871</x:v>
       </x:c>
       <x:c r="C31" s="17"/>
     </x:row>
     <x:row r="32" ht="26.75" customHeight="1">
       <x:c r="A32" s="16" t="s">
-        <x:v>514</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="B32" s="16" t="s">
-        <x:v>867</x:v>
+        <x:v>866</x:v>
       </x:c>
       <x:c r="C32" s="17"/>
     </x:row>
     <x:row r="33" ht="26.75" customHeight="1">
       <x:c r="A33" s="16" t="s">
-        <x:v>879</x:v>
+        <x:v>878</x:v>
       </x:c>
       <x:c r="B33" s="16" t="s">
-        <x:v>867</x:v>
+        <x:v>866</x:v>
       </x:c>
       <x:c r="C33" s="17"/>
     </x:row>
     <x:row r="34" ht="26.75" customHeight="1">
       <x:c r="A34" s="16" t="s">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="B34" s="16" t="s">
-        <x:v>861</x:v>
+        <x:v>860</x:v>
       </x:c>
       <x:c r="C34" s="17"/>
     </x:row>
     <x:row r="35" ht="26.75" customHeight="1">
       <x:c r="A35" s="16" t="s">
-        <x:v>470</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="B35" s="16" t="s">
-        <x:v>860</x:v>
+        <x:v>859</x:v>
       </x:c>
       <x:c r="C35" s="17"/>
     </x:row>
@@ -14473,18 +14470,18 @@
         <x:v>242</x:v>
       </x:c>
       <x:c r="B36" s="16" t="s">
+        <x:v>862</x:v>
+      </x:c>
+      <x:c r="C36" s="17" t="s">
         <x:v>863</x:v>
-      </x:c>
-      <x:c r="C36" s="17" t="s">
-        <x:v>864</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="26.75" customHeight="1">
       <x:c r="A37" s="16" t="s">
-        <x:v>880</x:v>
+        <x:v>879</x:v>
       </x:c>
       <x:c r="B37" s="16" t="s">
-        <x:v>872</x:v>
+        <x:v>871</x:v>
       </x:c>
       <x:c r="C37" s="17"/>
     </x:row>
@@ -14493,7 +14490,7 @@
         <x:v>154</x:v>
       </x:c>
       <x:c r="B38" s="16" t="s">
-        <x:v>869</x:v>
+        <x:v>868</x:v>
       </x:c>
       <x:c r="C38" s="17"/>
     </x:row>
@@ -14502,36 +14499,36 @@
         <x:v>215</x:v>
       </x:c>
       <x:c r="B39" s="16" t="s">
-        <x:v>867</x:v>
+        <x:v>866</x:v>
       </x:c>
       <x:c r="C39" s="17" t="s">
-        <x:v>881</x:v>
+        <x:v>880</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="26.75" customHeight="1">
       <x:c r="A40" s="16" t="s">
-        <x:v>412</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="B40" s="16" t="s">
-        <x:v>867</x:v>
+        <x:v>866</x:v>
       </x:c>
       <x:c r="C40" s="17"/>
     </x:row>
     <x:row r="41" ht="26.75" customHeight="1">
       <x:c r="A41" s="16" t="s">
-        <x:v>882</x:v>
+        <x:v>881</x:v>
       </x:c>
       <x:c r="B41" s="16" t="s">
-        <x:v>867</x:v>
+        <x:v>866</x:v>
       </x:c>
       <x:c r="C41" s="17"/>
     </x:row>
     <x:row r="42" ht="26.75" customHeight="1">
       <x:c r="A42" s="16" t="s">
-        <x:v>883</x:v>
+        <x:v>882</x:v>
       </x:c>
       <x:c r="B42" s="16" t="s">
-        <x:v>871</x:v>
+        <x:v>870</x:v>
       </x:c>
       <x:c r="C42" s="17"/>
     </x:row>
@@ -14540,10 +14537,10 @@
         <x:v>200</x:v>
       </x:c>
       <x:c r="B43" s="16" t="s">
+        <x:v>862</x:v>
+      </x:c>
+      <x:c r="C43" s="17" t="s">
         <x:v>863</x:v>
-      </x:c>
-      <x:c r="C43" s="17" t="s">
-        <x:v>864</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="26.75" customHeight="1">
@@ -14551,7 +14548,7 @@
         <x:v>159</x:v>
       </x:c>
       <x:c r="B44" s="16" t="s">
-        <x:v>869</x:v>
+        <x:v>868</x:v>
       </x:c>
       <x:c r="C44" s="17"/>
     </x:row>
@@ -14560,16 +14557,16 @@
         <x:v>139</x:v>
       </x:c>
       <x:c r="B45" s="16" t="s">
-        <x:v>869</x:v>
+        <x:v>868</x:v>
       </x:c>
       <x:c r="C45" s="17"/>
     </x:row>
     <x:row r="46" ht="26.75" customHeight="1">
       <x:c r="A46" s="16" t="s">
-        <x:v>884</x:v>
+        <x:v>883</x:v>
       </x:c>
       <x:c r="B46" s="16" t="s">
-        <x:v>869</x:v>
+        <x:v>868</x:v>
       </x:c>
       <x:c r="C46" s="17"/>
     </x:row>
@@ -14578,19 +14575,19 @@
         <x:v>133</x:v>
       </x:c>
       <x:c r="B47" s="16" t="s">
-        <x:v>862</x:v>
+        <x:v>861</x:v>
       </x:c>
       <x:c r="C47" s="17"/>
     </x:row>
     <x:row r="48" ht="26.75" customHeight="1">
       <x:c r="A48" s="16" t="s">
+        <x:v>884</x:v>
+      </x:c>
+      <x:c r="B48" s="16" t="s">
+        <x:v>862</x:v>
+      </x:c>
+      <x:c r="C48" s="17" t="s">
         <x:v>885</x:v>
-      </x:c>
-      <x:c r="B48" s="16" t="s">
-        <x:v>863</x:v>
-      </x:c>
-      <x:c r="C48" s="17" t="s">
-        <x:v>886</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="26.75" customHeight="1">
@@ -14598,7 +14595,7 @@
         <x:v>259</x:v>
       </x:c>
       <x:c r="B49" s="16" t="s">
-        <x:v>862</x:v>
+        <x:v>861</x:v>
       </x:c>
       <x:c r="C49" s="17"/>
     </x:row>
@@ -14607,16 +14604,16 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="B50" s="16" t="s">
-        <x:v>869</x:v>
+        <x:v>868</x:v>
       </x:c>
       <x:c r="C50" s="17"/>
     </x:row>
     <x:row r="51" ht="26.75" customHeight="1">
       <x:c r="A51" s="16" t="s">
-        <x:v>887</x:v>
+        <x:v>886</x:v>
       </x:c>
       <x:c r="B51" s="16" t="s">
-        <x:v>869</x:v>
+        <x:v>868</x:v>
       </x:c>
       <x:c r="C51" s="17"/>
     </x:row>
@@ -14625,38 +14622,38 @@
         <x:v>208</x:v>
       </x:c>
       <x:c r="B52" s="16" t="s">
-        <x:v>875</x:v>
+        <x:v>874</x:v>
       </x:c>
       <x:c r="C52" s="17"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" t="s">
-        <x:v>536</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="B53" t="s">
-        <x:v>349</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="C53" t="s">
-        <x:v>888</x:v>
+        <x:v>887</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" t="s">
-        <x:v>545</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="B54" t="s">
-        <x:v>863</x:v>
+        <x:v>862</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" t="s">
-        <x:v>552</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="B55" t="s">
-        <x:v>861</x:v>
+        <x:v>860</x:v>
       </x:c>
       <x:c r="C55" t="s">
-        <x:v>889</x:v>
+        <x:v>888</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -17708,7 +17705,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf87eb2df18404f6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R722b769d16d04474"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update project exhibits, 3D artwork, links, and certificates
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -5112,6 +5112,7 @@
     <x:col min="33" max="33" width="58" hidden="0" customWidth="1"/>
     <x:col min="34" max="34" width="20" hidden="0" customWidth="1"/>
     <x:col min="35" max="35" width="20" hidden="0" customWidth="1"/>
+    <x:col min="36" max="36" width="70" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -5219,6 +5220,9 @@
       </x:c>
       <x:c r="AI1" s="532" t="str">
         <x:v>Prize Split</x:v>
+      </x:c>
+      <x:c r="AJ1" s="532" t="str">
+        <x:v>Project URL</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -10516,6 +10520,9 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AI70" s="493"/>
+      <x:c r="AJ70" s="64" t="str">
+        <x:v>https://public-apps-sayyidkhan.zocomputer.io/zorder/</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71">
@@ -10588,6 +10595,9 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI71" s="493"/>
+      <x:c r="AJ71" s="64" t="str">
+        <x:v>https://public-apps-sayyidkhan.zocomputer.io/relationship-mapper/</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72">
@@ -10749,6 +10759,9 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI73" s="493"/>
+      <x:c r="AJ73" s="64" t="str">
+        <x:v>https://alien-homecoming.lovable.app/</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74">
@@ -10983,6 +10996,9 @@
       </x:c>
       <x:c r="AI76" s="493" t="str">
         <x:v>Per Team Member</x:v>
+      </x:c>
+      <x:c r="AJ76" s="64" t="str">
+        <x:v>https://gr-atlas.vercel.app/</x:v>
       </x:c>
     </x:row>
     <x:row r="77">

</xml_diff>

<commit_message>
Update hackathon source links and refine interactive project exhibits
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -5268,8 +5268,10 @@
       <x:c r="N2" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="O2" t="s">
-        <x:v>8</x:v>
+      <x:c r="O2" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/sayyidkhan/xueyiyi</x:t>
+        </x:is>
       </x:c>
       <x:c r="P2" t="s">
         <x:v>8</x:v>
@@ -5355,8 +5357,10 @@
       <x:c r="N3" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="O3" t="s">
-        <x:v>8</x:v>
+      <x:c r="O3" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/sayyidkhan/xueyiyi</x:t>
+        </x:is>
       </x:c>
       <x:c r="P3" t="s">
         <x:v>8</x:v>
@@ -6196,8 +6200,10 @@
       <x:c r="N14" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="O14" t="s">
-        <x:v>8</x:v>
+      <x:c r="O14" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/sayyidkhan/test-app-net-worth-evaluator</x:t>
+        </x:is>
       </x:c>
       <x:c r="P14" t="s">
         <x:v>8</x:v>
@@ -6357,8 +6363,10 @@
       <x:c r="N16" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="O16" t="s">
-        <x:v>8</x:v>
+      <x:c r="O16" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/sayyidkhan/unesco-weatherguru</x:t>
+        </x:is>
       </x:c>
       <x:c r="P16" t="s">
         <x:v>8</x:v>
@@ -6501,8 +6509,10 @@
       <x:c r="N18" t="s">
         <x:v>114</x:v>
       </x:c>
-      <x:c r="O18" t="s">
-        <x:v>8</x:v>
+      <x:c r="O18" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/sayyidkhan/goldigloo</x:t>
+        </x:is>
       </x:c>
       <x:c r="P18" t="s">
         <x:v>8</x:v>
@@ -6588,8 +6598,10 @@
       <x:c r="N19" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="O19" t="s">
-        <x:v>8</x:v>
+      <x:c r="O19" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/sayyidkhan/checker-app</x:t>
+        </x:is>
       </x:c>
       <x:c r="P19" t="s">
         <x:v>8</x:v>
@@ -6660,8 +6672,10 @@
       <x:c r="N20" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="O20" t="s">
-        <x:v>8</x:v>
+      <x:c r="O20" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/sayyidkhan/fasight</x:t>
+        </x:is>
       </x:c>
       <x:c r="P20" t="s">
         <x:v>8</x:v>
@@ -6948,8 +6962,10 @@
       <x:c r="N24" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="O24" t="s">
-        <x:v>8</x:v>
+      <x:c r="O24" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/sayyidkhan/pestoverflow</x:t>
+        </x:is>
       </x:c>
       <x:c r="P24" t="s">
         <x:v>8</x:v>
@@ -7020,8 +7036,10 @@
       <x:c r="N25" t="s">
         <x:v>163</x:v>
       </x:c>
-      <x:c r="O25" t="s">
-        <x:v>8</x:v>
+      <x:c r="O25" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/sayyidkhan/my-next-gym</x:t>
+        </x:is>
       </x:c>
       <x:c r="P25" t="s">
         <x:v>8</x:v>
@@ -7092,8 +7110,10 @@
       <x:c r="N26" t="s">
         <x:v>165</x:v>
       </x:c>
-      <x:c r="O26" t="s">
-        <x:v>8</x:v>
+      <x:c r="O26" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/sayyidkhan/neurosurge</x:t>
+        </x:is>
       </x:c>
       <x:c r="P26" t="s">
         <x:v>8</x:v>
@@ -7179,8 +7199,10 @@
       <x:c r="N27" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="O27" t="s">
-        <x:v>8</x:v>
+      <x:c r="O27" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/sayyidkhan/amigo</x:t>
+        </x:is>
       </x:c>
       <x:c r="P27" t="s">
         <x:v>8</x:v>
@@ -7539,8 +7561,10 @@
       <x:c r="N32" t="s">
         <x:v>206</x:v>
       </x:c>
-      <x:c r="O32" t="s">
-        <x:v>8</x:v>
+      <x:c r="O32" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/sayyidkhan/growthguru</x:t>
+        </x:is>
       </x:c>
       <x:c r="P32" t="s">
         <x:v>8</x:v>

</xml_diff>

<commit_message>
Correct Uncle Dustin project name and refine PestOverflow alert animation
</commit_message>
<xml_diff>
--- a/data/Hackathon CV.xlsx
+++ b/data/Hackathon CV.xlsx
@@ -7405,8 +7405,10 @@
       <x:c r="J30" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="K30" t="s">
-        <x:v>162</x:v>
+      <x:c r="K30" t="inlineStr">
+        <x:is>
+          <x:t>Uncle Dustin</x:t>
+        </x:is>
       </x:c>
       <x:c r="L30" t="s">
         <x:v>8</x:v>

</xml_diff>